<commit_message>
📰 뉴스 데이터 2026-06-24_09:04
</commit_message>
<xml_diff>
--- a/data/SCM_물류_브리핑.xlsx
+++ b/data/SCM_물류_브리핑.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J34"/>
+  <dimension ref="A1:J64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2082,6 +2082,1442 @@
       </c>
       <c r="J34" s="4" t="inlineStr"/>
     </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>['26년 6월] 물류 Market Intelligence 리포트</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>5월 SCFI 종합지수가 17.9% 상승했으며, 미주 및 유럽 항로 운임이 급등하여 물류비 부담이 가중되고 있으며, 7월 미국 관세 정책 변경 가능성 및 BAF 조정 전 선적 수요가 주요 원인으로 분석된다.</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>주요 항로의 해상 운임이 급등하여 우리 회사의 물류 비용에 즉각적인 영향을 미치며, 7월 미국 관세 정책 변경 가능성으로 인한 선적 수요 증가는 추가적인 운송 지연을 야기할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>해상 운임 상승에 따른 물류비 예산 재검토 및 운송 계획 조정, 7월 미국 관세 정책 변화에 대한 대비책 마련.</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>cello</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cello-square.com/kr/marketupdates/view-2241.do</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>RSK-006</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>항만 혼잡에 340만TEU 발묶여…공급망 압박 심화</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>전 세계 주요 항만에서 약 340만 TEU 규모의 컨테이너선 운항 능력이 항만 혼잡으로 발이 묶여 글로벌 해상 물류망의 병목 현상이 심화되고 있으며, 이는 선복 부족과 운항 지연을 가중시키고 있다.</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>전 세계적인 항만 혼잡으로 인한 대규모 선복 능력 손실은 해상 운송 지연 및 선복 부족을 심화시켜 우리 회사의 생산 및 물류 계획에 직접적인 차질을 초래할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>주요 항로의 운송 지연 현황 면밀히 모니터링, 재고 수준 및 안전 재고량 점검, 대체 운송 경로 또는 운송 방식 검토, 운송 파트너와 긴밀한 소통.</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>oceanpress</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oceanpress.co.kr/news/article.html?no=30418</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>RSK-007</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 다시 긴장…운임 올라도 해운업계 표정 복잡</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협의 지정학적 불확실성이 다시 커지면서 유조선 및 LNG 운반선 운임 상승 가능성이 제기되고, 전쟁 위험 보험료 증가 등 해운업계의 실적 변동성이 확대되고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협의 긴장 고조는 중동발 원자재 및 에너지 운송에 직접적인 영향을 미치며, 해상 운임 및 보험료 상승으로 이어져 당사의 물류 비용에 즉각적인 부담을 줄 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>중동 항로 이용 시 대체 운송 경로 및 선사 옵션을 긴급 검토하고, 전쟁 위험 보험료 변동에 따른 비용 증가를 예측하여 예산을 조정해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>ZDNet korea</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>https://zdnet.co.kr/view/?no=20260623064540</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>RSK-008</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>[해양통신] 지중해 노선 스팟운임 프리미엄 1,500달러 돌파</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>아시아-지중해 항로의 컨테이너 스팟 운임이 아시아-북유럽 항로 대비 FEU당 1,500달러 이상의 프리미엄을 기록하며 급등하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>아시아-지중해 항로의 스팟 운임 급등은 해당 항로를 이용하는 당사의 운송 비용에 즉각적인 부담을 주며, 운송 계획 및 예산에 직접적인 영향을 미칩니다.</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>지중해 항로 운송 계획이 있다면 즉시 운임 변동을 확인하고, 대체 운송 방안 또는 장기 계약 협상 가능성을 검토하여 비용 상승에 대비해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>oceanpress.co.kr</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>https://oceanpress.co.kr/news/article.html?no=30405</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>RSK-009</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>뉴스스페이스</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>미중 무역 전쟁이 반도체, 클라우드 등 첨단 기술 분야로 확대되며 희토류 및 고성능 소재 공급망에 제약이 발생하고 있으며, 이는 한국 기업에 기회와 리스크를 동시에 제공한다.</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>미중 무역 갈등 심화와 희토류 등 핵심 소재 공급망 제약은 배터리/전자부품 제조에 필수적인 원자재 조달에 직접적인 위험을 초래할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>핵심 원자재(희토류, 고성능 소재)의 재고 수준 점검, 대체 공급처 발굴 및 다변화 전략 수립, 지정학적 리스크에 따른 공급망 시나리오 분석 및 비상 계획 수립.</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>뉴스스페이스</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>https://newsspace.kr/news/article.html?no=14451</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>RSK-010</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>중국 자원 무기화에…韓 ‘탈중국 공급망’ 전략적 파트너로 - 이투데이</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>중국 정부가 미국 방산·희토류 기업을 제재하며 자원 무기화를 가속화하는 가운데, 포스코·LS 등 한국 기업들이 비중국 공급망 구축을 위한 전략적 파트너십을 모색하고 있다.</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>중국의 자원 무기화는 배터리/전자부품 제조에 필수적인 희토류 등 핵심 원자재의 공급 안정성에 직접적인 위협이 되므로, 탈중국 공급망 구축이 시급하다.</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>핵심 원자재(희토류 등)의 공급망 다변화 전략 가속화, 비중국 공급처 발굴 및 계약 추진, 국내외 전략적 파트너십 강화 검토.</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>이투데이</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>https://www.etoday.co.kr/news/view/2595984</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>RSK-011</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>‘비용 효율 → 안보 생존’ … 재편되는 국제 에너지 시장-국민일보</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>미국-이란 전쟁은 글로벌 에너지 시장의 판도를 흔들어 에너지 및 원자재 공급망이 지정학적 리스크에 취약해지면서 '비용 효율'에서 '안보 생존'으로 패러다임이 재편되고 있다.</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>중동 지정학적 리스크로 인한 에너지 및 원자재 공급망 불안정성 증가는 배터리/전자부품 제조에 필수적인 원자재 조달 및 물류 비용에 직접적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>에너지 및 원자재 공급망의 지정학적 리스크 평가 강화, 공급망 다변화 및 비상 계획 재검토, 에너지 효율 개선 및 대체 에너지원 활용 방안 모색.</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>국민일보</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>https://kmib.co.kr/article/view.asp?arcid=1782117710&amp;code=11151100&amp;sid1=eco</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>RSK-012</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>미국-이란 전쟁: 물류 인프라 현황 및 대안 업데이트</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>미국-이란 전쟁 상황 관련 중동 지역 해상 및 항공 물류 인프라 현황을 업데이트했으며, 현재까지 주요 항만 및 공항의 가동에 전일 대비 변동사항은 없다고 밝혔다.</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>중동 지역의 지정학적 리스크는 주요 해상 운송로에 영향을 줄 수 있으므로 지속적인 모니터링이 필요하나, 현재까지 물류 인프라에 직접적인 변동은 없다.</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>중동 지역 정세 및 해상 운송로 상황 지속 모니터링.</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>cello</t>
+        </is>
+      </c>
+      <c r="I42" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cello-square.com/kr/marketupdates/view-2174.do</t>
+        </is>
+      </c>
+      <c r="J42" s="3" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>멕시코, 미국 최대 교역국 유지하는 한편 트럼프 USMCA 연장에 의문 제기</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>멕시코가 미국 최대 교역국 지위를 유지하는 가운데, 트럼프 전 대통령이 미국-멕시코-캐나다 무역협정(USMCA) 갱신에 의문을 제기하여 향후 북미 무역 정책 변화 가능성이 제기되었다.</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>USMCA 갱신 불확실성은 북미 지역 무역 환경에 변화를 가져와 관세 및 공급망 전략에 영향을 미칠 수 있으므로 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>북미 무역 정책 변화 동향 지속 모니터링 및 잠재적 관세 영향 분석 준비.</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>cello</t>
+        </is>
+      </c>
+      <c r="I43" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cello-square.com/kr/marketupdates/view-2243.do</t>
+        </is>
+      </c>
+      <c r="J43" s="3" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>물류 담당자를 위한 금주의 물류 소식 (‘26년 6월 2주차)</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>6월 13일 이탈리아 전역에서 항공 부문 파업이 예정되어 EasyJet 항공편 및 일부 공항의 운항 차질이 예상되었으며, 국내선 및 유럽 역내 노선의 결항 및 지연 가능성이 높았다.</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>이탈리아 항공 부문 파업은 유럽 내 항공 운송에 지연을 초래할 수 있으며, 우리 회사의 유럽향 긴급 물량 운송에 영향을 미칠 수 있으므로 모니터링이 필요하다. (과거 시점이지만, 유사 상황 대비 차원)</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>이탈리아 및 유럽 내 항공 운송 계획 점검 및 대체 운송 방안 고려 (향후 유사 상황 발생 시).</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>cello</t>
+        </is>
+      </c>
+      <c r="I44" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cello-square.com/kr/marketupdates/view-2238.do</t>
+        </is>
+      </c>
+      <c r="J44" s="3" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>보더랜드 멕시코: 우버 프레이트, 이른 성수기 및 강력한 멕시코 수요 전망</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>우버 프레이트는 2026년 하반기 미국-멕시코 공급망에서 화물 시장이 더욱 타이트해지고 성수기가 조기에 시작될 것으로 전망하며, 멕시코 수요가 강세를 보일 것으로 예상했다.</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>미국-멕시코 국경 운송 시장의 타이트함과 조기 성수기 도래는 해당 지역 물류 비용 상승 및 운송 지연을 야기할 수 있으므로 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>미국-멕시코 국경 운송 수요 및 공급 상황 지속 모니터링, 운송 파트너와 사전 협의를 통한 운송 계획 수립.</t>
+        </is>
+      </c>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>cello</t>
+        </is>
+      </c>
+      <c r="I45" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cello-square.com/kr/marketupdates/view-2236.do</t>
+        </is>
+      </c>
+      <c r="J45" s="3" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>오만 외무 “이란 측과 통항료 없는 호르무즈 안전 통과 재확인”</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>오만 외무장관이 이란 측과 호르무즈 해협의 국제법 준수 및 통항료 없는 안전 통항 보장을 재확인하여 중동 해상 운송로의 안정성 유지 노력을 밝혔다.</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협의 안전 통항 재확인은 중동 지역 해상 운송의 불확실성을 일부 완화하지만, 지정학적 리스크는 여전히 존재하므로 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>중동 지역 정세 및 해상 운송로 상황 지속 모니터링.</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>kita</t>
+        </is>
+      </c>
+      <c r="I46" s="3" t="inlineStr">
+        <is>
+          <t>https://www.kita.net/shippers/board/newsView.do?morgueCode=2&amp;dataCls=B&amp;dataSeq=8132</t>
+        </is>
+      </c>
+      <c r="J46" s="3" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>Transpacific: Ripe for new non-alliance services</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence 분석에 따르면 아시아-북미 서안 항로의 높은 스팟 운임이 새로운 비동맹 서비스의 출현을 촉진할 수 있는 환경을 조성하고 있다.</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>태평양 항로의 시장 역학 변화는 장기적으로 운임 및 서비스 옵션에 영향을 줄 수 있으므로, 잠재적인 시장 변화를 모니터링할 필요가 있다.</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>태평양 항로의 신규 서비스 동향 및 운임 변화 추이 지속 모니터링.</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I47" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/393-transpacific-ripe-for-new-non-alliance-services</t>
+        </is>
+      </c>
+      <c r="J47" s="3" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>Decoding Gemini’s Mediterranean Surge</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>Gemini Cooperation이 컨테이너 선박을 재배치하며 지중해 항로에 변화를 주고 있으며, 이는 동서 컨테이너 선박 배치에 영향을 미칩니다.</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>특정 해운 동맹의 선박 재배치는 지중해 항로의 선복량 및 스케줄에 변화를 줄 수 있어, 해당 지역을 이용하는 운송 계획에 잠재적 영향을 미칠 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>지중해 항로 이용 시 Gemini Cooperation의 서비스 변화를 주시하고, 필요시 다른 선사 옵션을 검토해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I48" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/392-decoding-gemini-s-mediterranean-surge</t>
+        </is>
+      </c>
+      <c r="J48" s="3" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>Q1 EBIT drops to USD 1.35bn in 2026 (so far)</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>2026년 1분기 해운 선사들의 EBIT가 13.5억 달러로 하락하며 어려운 재정 상황에 직면했음을 보여줍니다.</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>선사들의 수익성 악화는 향후 운임 정책이나 서비스 수준에 영향을 줄 수 있으므로, 장기적인 운송 계약 및 비용 관점에서 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>주요 계약 선사들의 재무 건전성을 지속적으로 모니터링하고, 운임 협상 시 참고 자료로 활용해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I49" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/389-q1-ebit-drops-to-usd-1-35bn-in-2026-so-far</t>
+        </is>
+      </c>
+      <c r="J49" s="3" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>20260624 경제·물류 주요뉴스</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>콜롬비아산 중질유 원유가 약 4년 11개월 만에 도입되었고, 호르무즈 해협 통항이 재개되는 분위기 속에 국제유가가 하락했습니다.</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>콜롬비아 원유 도입 및 호르무즈 해협 통항 재개는 국제유가 안정화에 긍정적이나, 유가 변동성은 지속되므로 추이를 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>유가 변동에 따른 연료 할증료 변화를 주시하고, 운송 계약 시 유가 연동 조항을 검토해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H50" s="3" t="inlineStr">
+        <is>
+          <t>SURFF</t>
+        </is>
+      </c>
+      <c r="I50" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260624-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J50" s="3" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>20260623 경제·물류 주요뉴스</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>미-이란 협상 진전으로 국제유가가 급락하고 호르무즈 해협 개방 분위기가 조성되어 공급 불안이 완화되고 있으며, 무역 구조 변화로 원화 약세가 나타나고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>국제유가 하락 및 호르무즈 해협 안정화는 긍정적이나, 원화 약세는 수입 물류비용 증가로 이어질 수 있어 종합적인 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="inlineStr">
+        <is>
+          <t>유가 및 환율 변동 추이를 지속적으로 모니터링하고, 환율 변동에 대비한 헤지 전략 또는 계약 조건 검토를 고려해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H51" s="3" t="inlineStr">
+        <is>
+          <t>SURFF</t>
+        </is>
+      </c>
+      <c r="I51" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260623-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J51" s="3" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>20260622 경제·물류 주요뉴스</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>인도네시아발 신규 항로가 확대되고 있으며, HMM은 운임 하락, 공급 증가, 관세 변수, 중동발 비용 부담 등 다양한 도전 과제에 직면해 있고, 남미 동안 및 미 서안 컨테이너 운임이 언급되었습니다.</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>인도네시아 신규 항로 확대는 긍정적이나, 전반적인 운임 하락 추세와 HMM의 전략적 과제는 향후 해상 운송 시장의 불안정성을 시사하므로 지속적인 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>주요 항로의 운임 변동을 주시하고, 장기 운송 계약 시 유연성을 확보하는 방안을 검토해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="inlineStr">
+        <is>
+          <t>SURFF</t>
+        </is>
+      </c>
+      <c r="I52" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260622-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J52" s="3" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>[글로벌 워치]트럼프 '오일 패권' 확장 전략 통하나…베네수엘라 원유 수출 2배 급증</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>트럼프 전 대통령이 주도한 베네수엘라 에너지 부문 제재 완화 조치로 베네수엘라의 원유 수출량이 전년 대비 2배 이상 급증했습니다.</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>베네수엘라 원유 수출 증가는 국제 유가 안정화에 기여할 수 있으나, 향후 미국 정책 변화에 따라 다시 변동될 수 있으므로 지속적인 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>국제 유가 동향을 지속적으로 모니터링하고, 유가 변동에 따른 물류비 영향 시나리오를 검토해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>이비엔(EBN)뉴스센터</t>
+        </is>
+      </c>
+      <c r="I53" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebn.co.kr/news/articleView.html?idxno=1713536</t>
+        </is>
+      </c>
+      <c r="J53" s="3" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>[호르무즈 개방] 반도체업 , 소재 가격부담 완화…'헬륨' 공급망 안정화 &lt; 기업포커스 &lt; ICT &lt; 산업 &lt; 기사본문 - 신아일보</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>미국과 이란 간 종전 합의로 중동 카타르산 수입 비중이 높은 반도체 핵심소재 헬륨의 공급망이 안정화될 것으로 예상되어 국내 반도체 업계가 환영하고 있다.</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>반도체 핵심소재인 헬륨 공급망 안정화는 간접적으로 전자부품 제조에 긍정적 영향을 줄 수 있으나, 당사의 직접적인 헬륨 사용 여부 및 비중을 확인해야 한다.</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>헬륨 등 반도체 관련 가스 및 소재의 당사 사용 현황 및 공급망 안정화 효과 분석.</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="inlineStr">
+        <is>
+          <t>신아일보</t>
+        </is>
+      </c>
+      <c r="I54" s="3" t="inlineStr">
+        <is>
+          <t>https://www.shinailbo.co.kr/news/articleView.html?idxno=5032326</t>
+        </is>
+      </c>
+      <c r="J54" s="3" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 물류난에 발 묶인 중고차…'폐차 수출' 사실상 전멸</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협의 지정학적 긴장으로 국내 중고차 수출 시장이 물류난을 겪었으나, 미-이란 종전 합의 후 일부 선박이 해협을 빠져나오며 상황이 개선될 조짐을 보인다.</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협은 주요 해상 운송로이므로, 긴장 완화는 해상 운임 및 운송 지연 리스크 감소에 긍정적이나, 중고차 산업에 대한 직접적인 영향은 제한적이다.</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 통과 선박 스케줄 및 해상 운임 동향 지속 모니터링.</t>
+        </is>
+      </c>
+      <c r="H55" s="3" t="inlineStr">
+        <is>
+          <t>뉴스핌</t>
+        </is>
+      </c>
+      <c r="I55" s="3" t="inlineStr">
+        <is>
+          <t>https://www.newspim.com/news/view/20260623000857</t>
+        </is>
+      </c>
+      <c r="J55" s="3" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>미·이란 종전 기대감에 항공유 가격 급락…"8월 유류할증료 추가 인하 전망" - 파이낸셜뉴스</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>미국과 이란의 종전 합의로 국제유가가 하향 안정세로 돌아서면서, 항공 유류할증료가 8월에 추가 인하될 가능성이 커져 물류비 부담 완화가 기대된다.</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>국제유가 하락 및 항공 유류할증료 인하는 항공 운송 비용 절감으로 이어져 당사의 물류비 부담을 완화할 수 있으므로 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr">
+        <is>
+          <t>항공 운임 및 유류할증료 변동 추이 모니터링, 물류비 절감 방안 검토.</t>
+        </is>
+      </c>
+      <c r="H56" s="3" t="inlineStr">
+        <is>
+          <t>파이낸셜뉴스</t>
+        </is>
+      </c>
+      <c r="I56" s="3" t="inlineStr">
+        <is>
+          <t>https://fnnews.com/news/202606230531012212</t>
+        </is>
+      </c>
+      <c r="J56" s="3" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>캐세이카고, 화물 10.5% 증가한 15만t</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr">
+        <is>
+          <t>캐세이카고의 5월 항공화물 운송량이 전년 대비 10.5% 증가했으며, 평균 적재율도 소폭 상승하여 항공 화물 수요 증가 추세를 보였다.</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>특정 항공사의 실적 증가 소식으로, 우리 회사의 물류 운영에 직접적인 영향은 미미하며 참고 수준이다.</t>
+        </is>
+      </c>
+      <c r="G57" s="4" t="n"/>
+      <c r="H57" s="4" t="inlineStr">
+        <is>
+          <t>cargonews</t>
+        </is>
+      </c>
+      <c r="I57" s="4" t="inlineStr">
+        <is>
+          <t>https://www.cargonews.co.kr/news/articleView.html?idxno=60394</t>
+        </is>
+      </c>
+      <c r="J57" s="4" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>States and Supporting Partners Join IATA’s Alliance to Expand CORSIA Carbon Credit Supply</t>
+        </is>
+      </c>
+      <c r="E58" s="4" t="inlineStr">
+        <is>
+          <t>IATA가 국제 항공 탄소 상쇄 및 감축 제도(CORSIA)의 탄소 배출권 공급 확대를 위한 연합에 더 많은 국가 및 파트너들이 참여했다고 발표했다.</t>
+        </is>
+      </c>
+      <c r="F58" s="4" t="inlineStr">
+        <is>
+          <t>항공 산업의 장기적인 탄소 감축 노력의 일환으로, 우리 회사의 물류 운영에 당장 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G58" s="4" t="n"/>
+      <c r="H58" s="4" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I58" s="4" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-23-states-supporting-partners-join-iata-alliance-expand-corsia-carbon-credit-supply/</t>
+        </is>
+      </c>
+      <c r="J58" s="4" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>Brazil’s Opportunity to Be a SAF Powerhouse</t>
+        </is>
+      </c>
+      <c r="E59" s="4" t="inlineStr">
+        <is>
+          <t>IATA는 브라질이 지속 가능한 항공 연료(SAF) 생산의 핵심 국가가 될 잠재력이 있음을 강조하며, 항공 운송의 탈탄소화에 기여할 수 있다고 밝혔다.</t>
+        </is>
+      </c>
+      <c r="F59" s="4" t="inlineStr">
+        <is>
+          <t>항공 산업의 장기적인 친환경 연료 전환 노력의 일환으로, 우리 회사의 물류 운영에 당장 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G59" s="4" t="n"/>
+      <c r="H59" s="4" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I59" s="4" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-08-brazil-opportunity-saf-powerhouse/</t>
+        </is>
+      </c>
+      <c r="J59" s="4" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>여수광양항, 벌크선 LNG 벙커링·원료 하역 동시 수행</t>
+        </is>
+      </c>
+      <c r="E60" s="4" t="inlineStr">
+        <is>
+          <t>여수광양항이 9만 톤급 벌크선에 LNG 벙커링과 원료 하역 작업을 동시에 성공적으로 수행하며, LNG 벙커링 상용화 시장 진입의 전환점을 마련했다.</t>
+        </is>
+      </c>
+      <c r="F60" s="4" t="inlineStr">
+        <is>
+          <t>특정 항만의 친환경 선박 연료 공급 인프라 확충 소식으로, 우리 회사의 컨테이너 물류 운영에 당장 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G60" s="4" t="n"/>
+      <c r="H60" s="4" t="inlineStr">
+        <is>
+          <t>ksg</t>
+        </is>
+      </c>
+      <c r="I60" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksg.co.kr/news/main_newsView.jsp?pNum=147478</t>
+        </is>
+      </c>
+      <c r="J60" s="4" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>2026-Q1: NAEC Ports Consolidate Market Share</t>
+        </is>
+      </c>
+      <c r="E61" s="4" t="inlineStr">
+        <is>
+          <t>2026년 1분기 북미 동부 해안(NAEC) 항만의 총 물동량과 수입 물동량이 감소했음에도 불구하고 시장 점유율을 공고히 했습니다.</t>
+        </is>
+      </c>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>북미 동부 항만의 물동량 감소는 당사 물류 운영에 직접적인 영향을 미치기보다는 전반적인 시장 동향을 파악하는 참고 자료입니다.</t>
+        </is>
+      </c>
+      <c r="G61" s="4" t="n"/>
+      <c r="H61" s="4" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I61" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/391-2026-q1-naec-ports-consolidate-market-share</t>
+        </is>
+      </c>
+      <c r="J61" s="4" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>Global Schedule Reliability for April 2026 the Highest of the Year</t>
+        </is>
+      </c>
+      <c r="E62" s="4" t="inlineStr">
+        <is>
+          <t>2026년 4월 전 세계 해상 운송 스케줄 신뢰도가 연중 최고치를 기록하며 정시 운항 성능이 개선되었음을 나타냅니다.</t>
+        </is>
+      </c>
+      <c r="F62" s="4" t="inlineStr">
+        <is>
+          <t>전반적인 해상 운송 스케줄 신뢰도 개선은 긍정적인 신호이나, 특정 항로나 당사 운송에 미치는 즉각적인 영향은 미미합니다.</t>
+        </is>
+      </c>
+      <c r="G62" s="4" t="n"/>
+      <c r="H62" s="4" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I62" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/390-global-schedule-reliability-for-april-2026-the-highest-of-the-year</t>
+        </is>
+      </c>
+      <c r="J62" s="4" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t>부산항 신항 셔틀버스, 탑승 수요 맞춤형 운행체제로 개편</t>
+        </is>
+      </c>
+      <c r="E63" s="4" t="inlineStr">
+        <is>
+          <t>부산항 신항이 항만 근로자 출퇴근 시간 단축을 위해 셔틀버스 운행 체제를 수요 맞춤형으로 개편하고 스마트 버스 서비스를 제공합니다.</t>
+        </is>
+      </c>
+      <c r="F63" s="4" t="inlineStr">
+        <is>
+          <t>부산항 신항 내부 셔틀버스 시스템 개선은 항만 근로자 편의 증진에 기여하지만, 당사의 컨테이너 운송 및 물류 흐름에 직접적인 영향은 없습니다.</t>
+        </is>
+      </c>
+      <c r="G63" s="4" t="n"/>
+      <c r="H63" s="4" t="inlineStr">
+        <is>
+          <t>shippingnewsnet.com</t>
+        </is>
+      </c>
+      <c r="I63" s="4" t="inlineStr">
+        <is>
+          <t>https://www.shippingnewsnet.com/news/articleView.html?idxno=70858</t>
+        </is>
+      </c>
+      <c r="J63" s="4" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t>씨메스로보틱스 / ‘물류·제조 대형 수주 잇달아’ 피지컬 AI 기반 로봇 자동화 사업 가속</t>
+        </is>
+      </c>
+      <c r="E64" s="4" t="inlineStr">
+        <is>
+          <t>씨메스로보틱스가 물류 및 제조 현장에서 피지컬 AI 기반 로봇 자동화 사업을 확대하며 대형 수주를 잇달아 확보하고, 1분기 사상 최대 매출을 달성했습니다.</t>
+        </is>
+      </c>
+      <c r="F64" s="4" t="inlineStr">
+        <is>
+          <t>물류 자동화 기술 발전 소식은 장기적인 관점에서 물류 효율성 개선에 참고가 되지만, 당사의 현재 물류 운영에 직접적인 영향은 없습니다.</t>
+        </is>
+      </c>
+      <c r="G64" s="4" t="n"/>
+      <c r="H64" s="4" t="inlineStr">
+        <is>
+          <t>ulogistics.co.kr</t>
+        </is>
+      </c>
+      <c r="I64" s="4" t="inlineStr">
+        <is>
+          <t>http://www.ulogistics.co.kr/test/board.php?board=all2&amp;command=body&amp;no=5202</t>
+        </is>
+      </c>
+      <c r="J64" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2094,7 +3530,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2198,6 +3634,49 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>3121.69</v>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>+136 (+4.6%)</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>+881 (+39.3%)</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>3747</v>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>+398 (+11.9%)</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>+940 (+33.5%)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2210,7 +3689,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2446,6 +3925,251 @@
       </c>
       <c r="I6" s="6" t="inlineStr"/>
     </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>RSK-006</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>['26년 6월] 물류 Market Intelligence 리포트</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr"/>
+      <c r="G7" s="6" t="inlineStr"/>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>해상 운임 상승에 따른 물류비 예산 재검토 및 운송 계획 조정, 7월 미국 관세 정책 변화에 대한 대비책 마련.</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>RSK-007</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>항만 혼잡에 340만TEU 발묶여…공급망 압박 심화</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr"/>
+      <c r="G8" s="6" t="inlineStr"/>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>주요 항로의 운송 지연 현황 면밀히 모니터링, 재고 수준 및 안전 재고량 점검, 대체 운송 경로 또는 운송 방식 검토, 운송 파트너와 긴밀한 소통.</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>RSK-008</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈 다시 긴장…운임 올라도 해운업계 표정 복잡</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr"/>
+      <c r="G9" s="6" t="inlineStr"/>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>중동 항로 이용 시 대체 운송 경로 및 선사 옵션을 긴급 검토하고, 전쟁 위험 보험료 변동에 따른 비용 증가를 예측하여 예산을 조정해야 합니다.</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>RSK-009</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>[해양통신] 지중해 노선 스팟운임 프리미엄 1,500달러 돌파</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr"/>
+      <c r="G10" s="6" t="inlineStr"/>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>지중해 항로 운송 계획이 있다면 즉시 운임 변동을 확인하고, 대체 운송 방안 또는 장기 계약 협상 가능성을 검토하여 비용 상승에 대비해야 합니다.</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>RSK-010</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>뉴스스페이스</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr"/>
+      <c r="G11" s="6" t="inlineStr"/>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>핵심 원자재(희토류, 고성능 소재)의 재고 수준 점검, 대체 공급처 발굴 및 다변화 전략 수립, 지정학적 리스크에 따른 공급망 시나리오 분석 및 비상 계획 수립.</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>RSK-011</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>중국 자원 무기화에…韓 ‘탈중국 공급망’ 전략적 파트너로 - 이투데이</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr"/>
+      <c r="G12" s="6" t="inlineStr"/>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>핵심 원자재(희토류 등)의 공급망 다변화 전략 가속화, 비중국 공급처 발굴 및 계약 추진, 국내외 전략적 파트너십 강화 검토.</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>RSK-012</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>‘비용 효율 → 안보 생존’ … 재편되는 국제 에너지 시장-국민일보</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr"/>
+      <c r="G13" s="6" t="inlineStr"/>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>에너지 및 원자재 공급망의 지정학적 리스크 평가 강화, 공급망 다변화 및 비상 계획 재검토, 에너지 효율 개선 및 대체 에너지원 활용 방안 모색.</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
📰 뉴스 데이터 2026-06-24_19:35
</commit_message>
<xml_diff>
--- a/data/SCM_물류_브리핑.xlsx
+++ b/data/SCM_물류_브리핑.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J64"/>
+  <dimension ref="A1:J82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3517,6 +3517,866 @@
         </is>
       </c>
       <c r="J64" s="4" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>[2026.6.24.] 중동 전쟁 관련 유가 및 물류 동향</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>중동 전쟁 장기화로 인해 유가 변동성이 커지고 물류 동향에 불확실성이 증가하고 있어, 해상 및 항공 운임 상승 압력이 지속될 수 있다.</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>중동 전쟁은 주요 해상 운송 경로에 영향을 미치고 유가 상승을 유발하여 해상 및 항공 운임에 직접적인 상승 압력을 가하므로, 물류비용 및 운송 스케줄에 즉각적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>유가 및 운임 변동 추이를 면밀히 주시하고, 물류 파트너사와 운임 계약 조건 재검토, 대체 운송 경로 및 모드 활용 가능성 검토.</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>kotra</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>https://dream.kotra.or.kr/kotranews/cms/news/actionKotraBoardDetail.do?SITE_NO=3&amp;MENU_ID=70&amp;CONTENTS_NO=1&amp;pNttSn=242390</t>
+        </is>
+      </c>
+      <c r="J65" s="2" t="inlineStr">
+        <is>
+          <t>RSK-013</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>亞 - 유럽 수출항로, 4월 ‘컨’ 물동량 12% 증가...6개월 연속 플러스</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>4월 아시아-유럽 수출항로의 컨테이너 물동량이 전년 동월 대비 12% 증가하여 6개월 연속 상승세를 기록했으며, 이는 역대 최고치이다.</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>아시아-유럽 항로의 물동량 급증은 해당 항로의 선박 공간 부족 및 항만 적체를 유발하여 운송 지연과 운임 상승 압력으로 이어질 수 있으므로 즉각적인 대응이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>아시아-유럽 항로의 선박 공간 확보 현황 및 운임 변동을 면밀히 주시하고, 물류 파트너사와 긴밀히 협력하여 선적 계획을 조정하며, 필요시 대체 운송 옵션(예: 항공 운송)을 검토.</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>shippingnews</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>https://www.shippingnewsnet.com/news/articleView.html?idxno=70878</t>
+        </is>
+      </c>
+      <c r="J66" s="2" t="inlineStr">
+        <is>
+          <t>RSK-014</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>WMES 2026 Speech - Stuart Fox, IATA's Director Flight and Operations</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="inlineStr">
+        <is>
+          <t>IATA는 항공기 인도 지연, 엔진 수명 단축, 예비 부품 확보의 어려움 등 항공 산업이 직면한 공급망 문제를 지적하며, 이는 항공 운송의 안정성에 영향을 미칠 수 있음을 시사했다.</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t>항공기 부품 공급망 문제는 항공 화물 운송 능력 및 스케줄에 간접적인 영향을 미칠 수 있으므로, 항공 운송 안정성 측면에서 추이를 모니터링할 필요가 있다.</t>
+        </is>
+      </c>
+      <c r="G67" s="3" t="inlineStr">
+        <is>
+          <t>항공 운송 파트너사의 서비스 안정성 및 스케줄 준수율 변화를 주시하고, 필요시 대체 운송 옵션을 검토.</t>
+        </is>
+      </c>
+      <c r="H67" s="3" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I67" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-speeches/06-24-wmes-2026-speech-stuart-fox-iata-director-flight-operations/</t>
+        </is>
+      </c>
+      <c r="J67" s="3" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>한국 화주사, 하청 물류기업의 탄소 인증서를 검증해야 한다</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="inlineStr">
+        <is>
+          <t>국내 물류 공급망에서 하청 물류기업의 탄소 배출량 산정 및 인증서 검증 필요성이 제기되며, 화주사의 공급망 탄소 관리 책임이 강화될 것으로 예상된다.</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
+          <t>향후 물류 파트너사 선정 및 계약 시 탄소 배출량 관리 역량이 중요한 평가 요소가 될 수 있으며, 우리 회사의 ESG 경영 목표 달성과도 연관된다.</t>
+        </is>
+      </c>
+      <c r="G68" s="3" t="inlineStr">
+        <is>
+          <t>물류 파트너사들의 탄소 배출량 관리 현황 및 인증서 보유 여부를 파악하고, 장기적인 공급망 탄소 관리 전략 수립을 검토.</t>
+        </is>
+      </c>
+      <c r="H68" s="3" t="inlineStr">
+        <is>
+          <t>kita</t>
+        </is>
+      </c>
+      <c r="I68" s="3" t="inlineStr">
+        <is>
+          <t>https://www.kita.net/shippers/board/newsView.do?morgueCode=2&amp;dataCls=A&amp;dataSeq=2524</t>
+        </is>
+      </c>
+      <c r="J68" s="3" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>‘공급망 위기시대의 역설’ 해운·선원 안보적 가치 재조명</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="inlineStr">
+        <is>
+          <t>중동 전쟁 장기화 등 지정학적 위기로 인해 공급망 단절 우려가 커지면서, 전시 및 비상시 전략물자 조달을 위한 경제안보선대 구축과 전략해기사 양성의 필요성이 강조되고 있다.</t>
+        </is>
+      </c>
+      <c r="F69" s="3" t="inlineStr">
+        <is>
+          <t>지정학적 리스크가 해운 공급망 안정성에 미치는 영향이 커지고 있으며, 이는 장기적으로 운송 경로 및 비용에 영향을 줄 수 있으므로 관련 정책 변화를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G69" s="3" t="inlineStr">
+        <is>
+          <t>지정학적 리스크에 따른 해운 정책 변화 및 공급망 안정화 노력에 대한 정보를 지속적으로 파악하고, 비상시 공급망 대응 계획에 반영할 요소를 검토.</t>
+        </is>
+      </c>
+      <c r="H69" s="3" t="inlineStr">
+        <is>
+          <t>ksg</t>
+        </is>
+      </c>
+      <c r="I69" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ksg.co.kr/news/main_newsView.jsp?pNum=147482</t>
+        </is>
+      </c>
+      <c r="J69" s="3" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>Tracking True Vessel Delay</t>
+        </is>
+      </c>
+      <c r="E70" s="3" t="inlineStr">
+        <is>
+          <t>해운사들이 운송 지연을 줄이기 위해 선박 스케줄에 여유 시간을 추가하는 '스케줄 버퍼링'을 늘리고 있으며, 이는 실제 운송 시간과 정시성 지표에 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="F70" s="3" t="inlineStr">
+        <is>
+          <t>해운사들의 스케줄 버퍼링 증가는 겉으로는 정시성을 높이는 것처럼 보일 수 있으나, 실제 운송 시간 증가로 이어질 수 있어 운송 리드타임 관리에 영향을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="G70" s="3" t="inlineStr">
+        <is>
+          <t>해상 운송 파트너사의 정시성 지표와 실제 운송 리드타임을 비교 분석하고, 운송 스케줄 변경 가능성에 대비하여 재고 수준 및 생산 계획을 검토.</t>
+        </is>
+      </c>
+      <c r="H70" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I70" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/394-tracking-true-vessel-delay</t>
+        </is>
+      </c>
+      <c r="J70" s="3" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>Transpacific: Ripe for new non-alliance services</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="inlineStr">
+        <is>
+          <t>태평양 횡단 항로에서 비동맹 컨테이너 선박 용량의 점유율과 스팟 운임 간의 관계를 분석한 결과, 새로운 비동맹 서비스의 출현 가능성이 높아지고 있다.</t>
+        </is>
+      </c>
+      <c r="F71" s="3" t="inlineStr">
+        <is>
+          <t>새로운 비동맹 서비스의 등장은 태평양 횡단 항로의 운송 용량과 경쟁 환경에 변화를 가져와 운임 및 서비스 옵션에 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G71" s="3" t="inlineStr">
+        <is>
+          <t>태평양 횡단 항로의 신규 서비스 동향을 주시하고, 운송 파트너사 포트폴리오 및 계약 조건에 미칠 영향을 분석.</t>
+        </is>
+      </c>
+      <c r="H71" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I71" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/393-transpacific-ripe-for-new-non-alliance-services</t>
+        </is>
+      </c>
+      <c r="J71" s="3" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>Global Schedule Reliability for April 2026 the Highest of the Year</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
+          <t>2026년 4월 글로벌 선박 스케줄 정시성이 올해 최고치를 기록했으며, 이는 해상 운송의 안정성이 다소 개선되었음을 나타낸다.</t>
+        </is>
+      </c>
+      <c r="F72" s="3" t="inlineStr">
+        <is>
+          <t>글로벌 선박 스케줄 정시성 개선은 해상 운송의 예측 가능성을 높여 물류 계획 수립에 긍정적이나, 지속적인 개선 여부를 모니터링하여 안정적인 공급망 운영에 활용해야 한다.</t>
+        </is>
+      </c>
+      <c r="G72" s="3" t="inlineStr">
+        <is>
+          <t>해상 운송 파트너사의 정시성 지표를 지속적으로 확인하고, 개선 추세가 유지될 경우 재고 관리 및 생산 계획 최적화에 반영할 가능성을 검토.</t>
+        </is>
+      </c>
+      <c r="H72" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I72" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/390-global-schedule-reliability-for-april-2026-the-highest-of-the-year</t>
+        </is>
+      </c>
+      <c r="J72" s="3" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>미중, 희토류 이어 구리 전쟁?…기술 패권경쟁 새 전선 부각</t>
+        </is>
+      </c>
+      <c r="E73" s="3" t="inlineStr">
+        <is>
+          <t>미중 기술 패권 경쟁이 희토류에 이어 구리로 확전될 조짐을 보이며, 이는 배터리 및 전자부품 제조에 필수적인 핵심 원자재 공급망에 새로운 지정학적 리스크를 부각시키고 있다.</t>
+        </is>
+      </c>
+      <c r="F73" s="3" t="inlineStr">
+        <is>
+          <t>구리는 배터리 및 전자부품 제조에 필수적인 원자재이므로, 미중 간 구리 관련 무역 분쟁 발생 시 원자재 수급 및 가격에 직접적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G73" s="3" t="inlineStr">
+        <is>
+          <t>구리 등 핵심 원자재의 글로벌 공급망 동향 및 미중 무역 정책 변화를 지속적으로 모니터링하고, 필요시 대체 공급처 확보 방안을 검토해야 한다.</t>
+        </is>
+      </c>
+      <c r="H73" s="3" t="inlineStr">
+        <is>
+          <t>연합뉴스</t>
+        </is>
+      </c>
+      <c r="I73" s="3" t="inlineStr">
+        <is>
+          <t>https://yna.co.kr/view/AKR20260624085400009</t>
+        </is>
+      </c>
+      <c r="J73" s="3" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>中, 美 국방부 블랙리스트에 맞불…미국 기업 수십 곳 무역 제한</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="inlineStr">
+        <is>
+          <t>중국이 미국 국방부의 중국 기업 블랙리스트 확대에 대응하여 미국 기업 수십 곳에 대한 무역 제한 조치를 발표했으며, 이는 중국산 이중용도 품목의 수출 통제도 포함한다.</t>
+        </is>
+      </c>
+      <c r="F74" s="3" t="inlineStr">
+        <is>
+          <t>미중 무역 분쟁 심화는 우리의 공급망 내 미국 기업 또는 중국산 이중용도 품목을 사용하는 협력사에 영향을 미쳐 물류 및 생산 계획에 간접적인 위험을 초래할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G74" s="3" t="inlineStr">
+        <is>
+          <t>공급망 내 미국 기업 및 중국산 이중용도 품목 사용 여부를 파악하고, 관련 규제 변화에 대한 모니터링을 강화하여 잠재적 리스크에 대비해야 한다.</t>
+        </is>
+      </c>
+      <c r="H74" s="3" t="inlineStr">
+        <is>
+          <t>헬로티 HelloT</t>
+        </is>
+      </c>
+      <c r="I74" s="3" t="inlineStr">
+        <is>
+          <t>https://hellot.net/news/article.html?no=113358</t>
+        </is>
+      </c>
+      <c r="J74" s="3" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>중국 희토류 규제 위반 혐의, 대련서 묶여버린 일본 전기설비업체 직원들</t>
+        </is>
+      </c>
+      <c r="E75" s="3" t="inlineStr">
+        <is>
+          <t>중국 세관 당국이 희토류 관련 수출 규제 위반 및 밀수 혐의로 일본 전기설비업체 직원 2명을 구금했으며, 이는 중국의 희토류 수출 통제 강화 기조를 보여준다.</t>
+        </is>
+      </c>
+      <c r="F75" s="3" t="inlineStr">
+        <is>
+          <t>중국의 희토류 수출 규제 강화는 배터리 및 전자부품 생산에 필요한 희토류 원자재의 수급 안정성에 영향을 미칠 수 있으며, 관련 무역 리스크를 증가시킨다.</t>
+        </is>
+      </c>
+      <c r="G75" s="3" t="inlineStr">
+        <is>
+          <t>희토류를 사용하는 부품이 있는지 확인하고, 중국의 희토류 수출 정책 및 통관 절차 변화를 면밀히 모니터링하며, 필요시 공급망 다변화 방안을 검토해야 한다.</t>
+        </is>
+      </c>
+      <c r="H75" s="3" t="inlineStr">
+        <is>
+          <t>인사이트</t>
+        </is>
+      </c>
+      <c r="I75" s="3" t="inlineStr">
+        <is>
+          <t>https://insight.co.kr/news/560017</t>
+        </is>
+      </c>
+      <c r="J75" s="3" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>[2026 기후경쟁력포럼] 'AI데이터센터·반도체·배터리' 한국 지탱하는 산업에 불어오는 친환경 요구, 탈탄소 전력이 미래 경쟁력 가른다</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="inlineStr">
+        <is>
+          <t>AI 데이터센터, 반도체, 배터리 등 한국의 주요 산업에서 탈탄소 전력 사용 및 친환경 요구가 강화되고 있으며, 이는 미래 경쟁력을 좌우할 핵심 요소로 부상하고 있다.</t>
+        </is>
+      </c>
+      <c r="F76" s="3" t="inlineStr">
+        <is>
+          <t>배터리/전자부품 제조기업으로서 친환경 및 탈탄소 요구는 장기적인 생산 및 물류 운영 전략, 공급망 관리, ESG 경영에 중요한 영향을 미치므로 지속적인 관심이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G76" s="3" t="inlineStr">
+        <is>
+          <t>친환경 에너지 전환 및 탄소 배출 저감 목표를 수립하고, 공급망 전반에 걸쳐 ESG 요소를 통합하는 전략을 검토해야 한다.</t>
+        </is>
+      </c>
+      <c r="H76" s="3" t="inlineStr">
+        <is>
+          <t>허프포스트코리아</t>
+        </is>
+      </c>
+      <c r="I76" s="3" t="inlineStr">
+        <is>
+          <t>https://huffingtonpost.kr/article/258207</t>
+        </is>
+      </c>
+      <c r="J76" s="3" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>EU 코발트 규제 강화에 업계 반발…핵심광물 자립 전략 흔들리나</t>
+        </is>
+      </c>
+      <c r="E77" s="3" t="inlineStr">
+        <is>
+          <t>EU의 코발트 분진 규제 강화가 역내 정제·재활용 기반을 약화시켜 핵심광물 공급망 전략에 영향을 미칠 수 있다는 우려가 제기되었다. 이는 배터리 생산에 필수적인 코발트의 조달 및 가공 방식에 변화를 요구할 수 있다.</t>
+        </is>
+      </c>
+      <c r="F77" s="3" t="inlineStr">
+        <is>
+          <t>EU의 코발트 규제 강화는 배터리 핵심 원자재 조달 및 가공 방식에 영향을 미쳐 향후 공급망 전략 재검토가 필요할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G77" s="3" t="inlineStr">
+        <is>
+          <t>EU의 코발트 규제 동향을 지속적으로 모니터링하고, 공급망 내 코발트 조달 및 가공 파트너사와의 협력 방안을 검토.</t>
+        </is>
+      </c>
+      <c r="H77" s="3" t="inlineStr">
+        <is>
+          <t>더구루</t>
+        </is>
+      </c>
+      <c r="I77" s="3" t="inlineStr">
+        <is>
+          <t>https://theguru.co.kr/news/article.html?no=103408</t>
+        </is>
+      </c>
+      <c r="J77" s="3" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 재개방에도 국제유가 70달러 유지 전망 : 한국 조선업 플랜트 사업에 기회 오나</t>
+        </is>
+      </c>
+      <c r="E78" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 재개방에도 불구하고 기뢰, 항만시설 훼손 등으로 국제유가가 배럴당 70달러대를 유지할 것으로 전망되어 물류비용에 지속적인 영향을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="F78" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 상황과 국제유가 전망은 해상 및 항공 운임의 유류할증료에 직접적인 영향을 미치므로 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G78" s="3" t="inlineStr">
+        <is>
+          <t>국제유가 및 해상/항공 운임 동향을 면밀히 모니터링하고, 유류할증료 변동에 따른 물류비 예산 영향을 분석.</t>
+        </is>
+      </c>
+      <c r="H78" s="3" t="inlineStr">
+        <is>
+          <t>허핑턴포스트코리아</t>
+        </is>
+      </c>
+      <c r="I78" s="3" t="inlineStr">
+        <is>
+          <t>https://www.huffingtonpost.kr/article/258200</t>
+        </is>
+      </c>
+      <c r="J78" s="3" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C79" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D79" s="4" t="inlineStr">
+        <is>
+          <t>삼성·SK, 수도권 넘어 호남·충청으로…AI 반도체 영토 넓힌다</t>
+        </is>
+      </c>
+      <c r="E79" s="4" t="inlineStr">
+        <is>
+          <t>삼성전자와 SK하이닉스가 AI 반도체 수요 폭증에 대응하여 수도권을 넘어 호남·충청 지역으로 생산기지를 확대하고 있으며, 이는 고대역폭 메모리(HBM) 및 첨단 패키징 수요 증가에 따른 전략적 움직임이다.</t>
+        </is>
+      </c>
+      <c r="F79" s="4" t="inlineStr">
+        <is>
+          <t>주요 고객사의 생산기지 확장은 장기적으로 우리의 물류 네트워크 및 공급 전략에 영향을 미칠 수 있으나, 당장 직접적인 운영 변화는 없다.</t>
+        </is>
+      </c>
+      <c r="G79" s="4" t="inlineStr">
+        <is>
+          <t>고객사 생산기지 확장 계획을 모니터링하고, 향후 물류 거점 및 공급망 전략에 미칠 영향을 검토한다.</t>
+        </is>
+      </c>
+      <c r="H79" s="4" t="inlineStr">
+        <is>
+          <t>뉴스핌</t>
+        </is>
+      </c>
+      <c r="I79" s="4" t="inlineStr">
+        <is>
+          <t>https://www.newspim.com/news/view/20260624000586</t>
+        </is>
+      </c>
+      <c r="J79" s="4" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="inlineStr">
+        <is>
+          <t>“K-배터리, 반도체 버금가는 전략산업”…세제지원 실효성 촉구</t>
+        </is>
+      </c>
+      <c r="E80" s="4" t="inlineStr">
+        <is>
+          <t>K-배터리 산업이 반도체에 버금가는 전략산업으로 부상하며 적자 기업도 혜택을 볼 수 있는 세제지원 체계가 필요하다는 주장이 제기되었다. 이는 배터리 산업의 경쟁력 강화 및 투자 유치와 관련이 있다.</t>
+        </is>
+      </c>
+      <c r="F80" s="4" t="inlineStr">
+        <is>
+          <t>세제지원 논의는 장기적인 산업 경쟁력에 영향을 미치지만, 당장 우리 물류 운영에 직접적인 변화를 요구하지는 않는다.</t>
+        </is>
+      </c>
+      <c r="G80" s="4" t="n"/>
+      <c r="H80" s="4" t="inlineStr">
+        <is>
+          <t>전자신문</t>
+        </is>
+      </c>
+      <c r="I80" s="4" t="inlineStr">
+        <is>
+          <t>https://etnews.com/20260624000346</t>
+        </is>
+      </c>
+      <c r="J80" s="4" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C81" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D81" s="4" t="inlineStr">
+        <is>
+          <t>미 재무 "동맹도 미국 시장접근엔 의무 수반" | 연합뉴스</t>
+        </is>
+      </c>
+      <c r="E81" s="4" t="inlineStr">
+        <is>
+          <t>미국 재무장관이 동맹국들도 미국 시장 접근 시 의무가 수반됨을 강조하며, 적대 세력의 공급망 차단에 대비한 경제 회복력 구축을 촉구했다.</t>
+        </is>
+      </c>
+      <c r="F81" s="4" t="inlineStr">
+        <is>
+          <t>고위 관계자의 일반적인 무역 정책 발언으로, 당장 우리 물류 운영에 직접적인 영향을 미치지 않는다.</t>
+        </is>
+      </c>
+      <c r="G81" s="4" t="n"/>
+      <c r="H81" s="4" t="inlineStr">
+        <is>
+          <t>연합뉴스</t>
+        </is>
+      </c>
+      <c r="I81" s="4" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20260624091800009</t>
+        </is>
+      </c>
+      <c r="J81" s="4" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B82" s="4" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C82" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D82" s="4" t="inlineStr">
+        <is>
+          <t>[호르무즈 개방] 반도체업 , 소재 가격부담 완화…'헬륨' 공급망 안정화</t>
+        </is>
+      </c>
+      <c r="E82" s="4" t="inlineStr">
+        <is>
+          <t>미국과 이란 간 종전 합의로 호르무즈 해협이 개방되면서 반도체 핵심소재인 헬륨의 공급망이 안정화될 것으로 기대된다.</t>
+        </is>
+      </c>
+      <c r="F82" s="4" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 개방은 긍정적이나, 해당 뉴스는 반도체 산업의 헬륨 공급망에 초점을 맞춰 배터리/전자부품 물류에 직접적인 영향은 미미하다.</t>
+        </is>
+      </c>
+      <c r="G82" s="4" t="n"/>
+      <c r="H82" s="4" t="inlineStr">
+        <is>
+          <t>신아일보</t>
+        </is>
+      </c>
+      <c r="I82" s="4" t="inlineStr">
+        <is>
+          <t>https://www.shinailbo.co.kr/news/articleView.html?idxno=5032326</t>
+        </is>
+      </c>
+      <c r="J82" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
@@ -3689,7 +4549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4170,6 +5030,76 @@
       </c>
       <c r="I13" s="6" t="inlineStr"/>
     </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>RSK-013</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>[2026.6.24.] 중동 전쟁 관련 유가 및 물류 동향</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr"/>
+      <c r="G14" s="6" t="inlineStr"/>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>유가 및 운임 변동 추이를 면밀히 주시하고, 물류 파트너사와 운임 계약 조건 재검토, 대체 운송 경로 및 모드 활용 가능성 검토.</t>
+        </is>
+      </c>
+      <c r="I14" s="6" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>RSK-014</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>亞 - 유럽 수출항로, 4월 ‘컨’ 물동량 12% 증가...6개월 연속 플러스</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr"/>
+      <c r="G15" s="6" t="inlineStr"/>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>아시아-유럽 항로의 선박 공간 확보 현황 및 운임 변동을 면밀히 주시하고, 물류 파트너사와 긴밀히 협력하여 선적 계획을 조정하며, 필요시 대체 운송 옵션(예: 항공 운송)을 검토.</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
📰 뉴스 데이터 2026-06-25_09:09
</commit_message>
<xml_diff>
--- a/data/SCM_물류_브리핑.xlsx
+++ b/data/SCM_물류_브리핑.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J82"/>
+  <dimension ref="A1:J110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4378,6 +4378,1322 @@
       </c>
       <c r="J82" s="4" t="inlineStr"/>
     </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 폐쇄로 화물 192조원어치 고립</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 폐쇄로 1,200척의 화물선과 약 1,250억 달러 상당의 화물이 고립되었으며, 이는 중동발 물류에 치명적인 영향을 미칠 수 있는 심각한 상황입니다.</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협은 주요 원유 및 가스 수송로이며, 폐쇄 시 물류 운영에 직접적인 차질과 유가 및 운임 급등을 야기할 수 있어 즉각적인 대응 계획이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>중동 항로 이용 시 대체 경로 및 운송 수단 검토, 비상 계획 수립 및 관련 부서와 비상 상황 대응 시나리오 공유.</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="inlineStr">
+        <is>
+          <t>연합뉴스</t>
+        </is>
+      </c>
+      <c r="I83" s="2" t="inlineStr">
+        <is>
+          <t>https://yna.co.kr/view/AKR20260624074300009</t>
+        </is>
+      </c>
+      <c r="J83" s="2" t="inlineStr">
+        <is>
+          <t>RSK-015</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>EU산 배터리 현지화 요구 강세&amp;hellip;韓 배터리 소재, 유럽 거점 효과 본다 [배터리레이다]</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>유럽연합(EU)이 '메이드 인 유럽' 기조를 강화하며 배터리 현지화 요구가 강해지고 있어, 국내 배터리 소재 기업들이 유럽 내 거점 확보를 통해 수혜를 볼 수 있다는 전망이 나온다.</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>EU의 현지화 요구는 유럽 시장 공급을 위한 생산 및 물류 전략에 직접적인 영향을 미치며, 현지 생산 또는 소재 공급망 재편을 고려해야 할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>EU 시장 공급을 위한 현지 생산 및 소재 조달 전략을 재검토하고, 유럽 내 물류 거점 및 공급망 최적화 방안을 수립.</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>디지털데일리</t>
+        </is>
+      </c>
+      <c r="I84" s="2" t="inlineStr">
+        <is>
+          <t>https://ddaily.co.kr/page/view/2026062413521879081</t>
+        </is>
+      </c>
+      <c r="J84" s="2" t="inlineStr">
+        <is>
+          <t>RSK-016</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>CPSC Mandatory eFiling Takes Effect July 8; TPEB Rates Surge ~10% as Peak Season Demand Outpaces Capacity</t>
+        </is>
+      </c>
+      <c r="E85" s="3" t="inlineStr">
+        <is>
+          <t>미국 CPSC의 의무 전자신고가 7월 8일 발효되며, 피크 시즌 수요가 공급을 초과하면서 태평양 횡단 동향(TPEB) 운임이 약 10% 급등하고 있다. 또한, 미국 세관국경보호국(CBP)은 강제 노동 관련 통합 지침을 발표했다.</t>
+        </is>
+      </c>
+      <c r="F85" s="3" t="inlineStr">
+        <is>
+          <t>TPEB 운임 상승은 물류비 증가로 이어질 수 있으며, CPSC 전자신고 및 강제 노동 지침은 향후 통관 및 공급망 관리에 영향을 줄 수 있어 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G85" s="3" t="inlineStr">
+        <is>
+          <t>TPEB 운임 추이 모니터링 및 CPSC 전자신고, 강제 노동 지침 관련 내부 프로세스 검토 준비.</t>
+        </is>
+      </c>
+      <c r="H85" s="3" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I85" s="3" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/june-18-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J85" s="3" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t>DOJ Appeals CIT's IEEPA Refund Injunction as CAPE Phase 2 Targets June 29; TPEB Rates Surge 30% Into Peak</t>
+        </is>
+      </c>
+      <c r="E86" s="3" t="inlineStr">
+        <is>
+          <t>법무부가 국제무역법원(CIT)의 IEEPA 환불 명령에 항소했으며, CAPE 2단계가 6월 29일 시행될 예정이고, 피크 시즌 진입으로 태평양 횡단 동향(TPEB) 운임이 30% 급등했다.</t>
+        </is>
+      </c>
+      <c r="F86" s="3" t="inlineStr">
+        <is>
+          <t>TPEB 운임의 급격한 상승은 물류비에 직접적인 영향을 미치며, 관세 환불 및 통관 관련 정책 변화는 향후 수입 절차에 영향을 줄 수 있어 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G86" s="3" t="inlineStr">
+        <is>
+          <t>TPEB 운임 상승에 따른 물류비 예산 검토 및 대체 운송 방안 고려. 관세 관련 정책 변화에 대한 정보 수집.</t>
+        </is>
+      </c>
+      <c r="H86" s="3" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I86" s="3" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/june-11-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J86" s="3" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="inlineStr">
+        <is>
+          <t>U.S. Appeals CIT's IEEPA Refund Order to Federal Circuit; TPEB Rates Rise as Peak Season Demand Tightens Capacity</t>
+        </is>
+      </c>
+      <c r="E87" s="3" t="inlineStr">
+        <is>
+          <t>미국이 국제무역법원(CIT)의 IEEPA 환불 명령에 연방항소법원에 항소했으며, 트럼프 대통령은 세관 집행 개혁 행정명령에 서명하여 수입자 기록(IOR) 요건 강화 및 공개 의무 확대를 지시했다. 또한, 피크 시즌 수요로 태평양 횡단 동향(TPEB) 운임이 상승하고 있다.</t>
+        </is>
+      </c>
+      <c r="F87" s="3" t="inlineStr">
+        <is>
+          <t>TPEB 운임 상승은 물류비에 영향을 미치며, 세관 집행 개혁 및 IOR 요건 강화는 향후 미국 수출입 통관 절차에 직접적인 영향을 줄 수 있어 지속적인 모니터링과 대비가 필요하다.</t>
+        </is>
+      </c>
+      <c r="G87" s="3" t="inlineStr">
+        <is>
+          <t>TPEB 운임 추이 모니터링 및 미국 세관 규제 변화에 대한 정보 수집 및 내부 프로세스 영향 분석 준비.</t>
+        </is>
+      </c>
+      <c r="H87" s="3" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I87" s="3" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/june-3-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J87" s="3" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="inlineStr">
+        <is>
+          <t>Section 232 Duties Reduced to 15% for Taiwanese Goods, Retroactive to May 1; China Air Rates Spike on Supply Contraction and Month-End Demand</t>
+        </is>
+      </c>
+      <c r="E88" s="3" t="inlineStr">
+        <is>
+          <t>대만산 특정 품목에 대한 232조 관세가 5월 1일부로 소급 적용되어 15%로 인하되었으며, 공급 감소와 월말 수요로 인해 중국발 항공 운임이 급등했다.</t>
+        </is>
+      </c>
+      <c r="F88" s="3" t="inlineStr">
+        <is>
+          <t>중국발 항공 운임 급등은 항공 운송을 이용하는 우리 회사의 물류비에 직접적인 영향을 미칠 수 있으며, 대만 관세 인하는 관련 부품 조달 시 참고할 수 있는 정보이다.</t>
+        </is>
+      </c>
+      <c r="G88" s="3" t="inlineStr">
+        <is>
+          <t>중국발 항공 운임 추이 모니터링 및 항공 운송 비용 증가에 대비한 예산 검토.</t>
+        </is>
+      </c>
+      <c r="H88" s="3" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I88" s="3" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/may-28-2026-cit-rejects-governments-stay-request/</t>
+        </is>
+      </c>
+      <c r="J88" s="3" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>한국 화주사, 하청 물류기업의 탄소 인증서를 검증해야 한다</t>
+        </is>
+      </c>
+      <c r="E89" s="3" t="inlineStr">
+        <is>
+          <t>국내 물류 공급망에서 하청 물류기업의 배출량 산정 방식과 탄소 인증서 검증 필요성이 제기되며, 화주사의 공급망 탄소 관리 책임이 강조되고 있다.</t>
+        </is>
+      </c>
+      <c r="F89" s="3" t="inlineStr">
+        <is>
+          <t>공급망 탄소 관리 책임이 화주사로 확대될 가능성이 있으며, 이는 향후 물류 파트너 선정 및 운영 프로세스에 영향을 미칠 수 있어 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G89" s="3" t="inlineStr">
+        <is>
+          <t>공급망 탄소 배출량 관리 및 하청 물류기업의 탄소 인증서 검증 요구에 대비하여 정보 수집 및 내부 검토 시작.</t>
+        </is>
+      </c>
+      <c r="H89" s="3" t="inlineStr">
+        <is>
+          <t>kita</t>
+        </is>
+      </c>
+      <c r="I89" s="3" t="inlineStr">
+        <is>
+          <t>https://www.kita.net/shippers/board/newsView.do?morgueCode=2&amp;dataCls=A&amp;dataSeq=2524</t>
+        </is>
+      </c>
+      <c r="J89" s="3" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="inlineStr">
+        <is>
+          <t>Tracking True Vessel Delay</t>
+        </is>
+      </c>
+      <c r="E90" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence는 선박 스케줄 버퍼링과 조기 입항 간의 관계를 분석하며, 선사들이 운송 시간을 늘리는 스케줄 버퍼링에 점점 더 의존하고 있다고 밝혔다.</t>
+        </is>
+      </c>
+      <c r="F90" s="3" t="inlineStr">
+        <is>
+          <t>선사들의 스케줄 버퍼링 증가는 실제 운송 시간 증가로 이어져 우리 회사의 해상 운송 리드 타임 및 재고 계획에 영향을 미칠 수 있으므로 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G90" s="3" t="inlineStr">
+        <is>
+          <t>해상 운송 리드 타임 변화 추이 모니터링 및 재고 계획에 미칠 영향 분석.</t>
+        </is>
+      </c>
+      <c r="H90" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I90" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/394-tracking-true-vessel-delay</t>
+        </is>
+      </c>
+      <c r="J90" s="3" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 통항 완화 조짐 및 유가 하락</t>
+        </is>
+      </c>
+      <c r="E91" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 통항 관련 불확실성이 완화되는 조짐이 보이며, 한국 선박 일부가 해협을 통과하고 이란이 통행료를 받지 않겠다고 통보하는 등 상황 변화로 국제유가가 하락했습니다.</t>
+        </is>
+      </c>
+      <c r="F91" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협의 상황 완화는 긍정적이나, 중동 정세는 여전히 변동성이 크므로 유가 및 물류비에 미칠 영향을 지속적으로 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G91" s="3" t="inlineStr">
+        <is>
+          <t>중동 항로 이용 시 선박 스케줄 및 운임 변동 가능성 지속 모니터링, 유가 추이 분석을 통한 물류비 예측.</t>
+        </is>
+      </c>
+      <c r="H91" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I91" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260625-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J91" s="3" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="inlineStr">
+        <is>
+          <t>종전 후속 협상에도 해상운임 고공행진...해운사 실적 개선 기대</t>
+        </is>
+      </c>
+      <c r="E92" s="3" t="inlineStr">
+        <is>
+          <t>미국과 이란의 종전 협상에도 불구하고 호르무즈 해협 관련 불확실성으로 글로벌 해상운임 상승세가 지속되고 있으며, 이는 해운사 실적 개선으로 이어질 전망입니다.</t>
+        </is>
+      </c>
+      <c r="F92" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협의 지정학적 불확실성이 해상운임 상승을 지속시키고 있어, 물류비 증가에 대한 대비와 추이 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G92" s="3" t="inlineStr">
+        <is>
+          <t>주요 항로 운임 변동 추이 모니터링 및 장기 계약 조건 재검토, 운임 상승에 대비한 예산 계획 수립.</t>
+        </is>
+      </c>
+      <c r="H92" s="3" t="inlineStr">
+        <is>
+          <t>뉴스핌</t>
+        </is>
+      </c>
+      <c r="I92" s="3" t="inlineStr">
+        <is>
+          <t>https://www.newspim.com/news/view/20260624000803</t>
+        </is>
+      </c>
+      <c r="J92" s="3" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>글로벌 컨테이너 시장, 예측 불가능한 '수요 파동' 중심 구조로 재편</t>
+        </is>
+      </c>
+      <c r="E93" s="3" t="inlineStr">
+        <is>
+          <t>글로벌 컨테이너 시장이 전통적인 성수기·비수기 사이클에서 벗어나 예측하기 어려운 '수요 파동' 중심 구조로 재편되고 있다는 분석이 나왔습니다.</t>
+        </is>
+      </c>
+      <c r="F93" s="3" t="inlineStr">
+        <is>
+          <t>시장 예측 불확실성 증가는 물류 계획 수립 및 선복 확보에 어려움을 줄 수 있으므로, 장기적인 관점에서 시장 동향을 모니터링하고 유연한 전략을 준비해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G93" s="3" t="inlineStr">
+        <is>
+          <t>시장 동향 분석 강화, 공급망 유연성 확보 방안 검토, 다양한 운송 옵션 확보.</t>
+        </is>
+      </c>
+      <c r="H93" s="3" t="inlineStr">
+        <is>
+          <t>해양통신</t>
+        </is>
+      </c>
+      <c r="I93" s="3" t="inlineStr">
+        <is>
+          <t>https://oceanpress.co.kr/news/article.html?no=30423</t>
+        </is>
+      </c>
+      <c r="J93" s="3" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>인도네시아 신규 항로 확대 및 남미/미서안 컨테이너 운임 상승</t>
+        </is>
+      </c>
+      <c r="E94" s="3" t="inlineStr">
+        <is>
+          <t>인도네시아발 신규 항로가 확대되고 선복 교환 등으로 물류 네트워크가 강화되는 가운데, 남미 동안 및 미 서안 컨테이너 운임이 상승했습니다.</t>
+        </is>
+      </c>
+      <c r="F94" s="3" t="inlineStr">
+        <is>
+          <t>특정 항로의 운임 상승은 해당 지역으로의 물류비 증가를 야기할 수 있으며, 신규 항로 확대는 장기적인 물류 효율성 개선 가능성을 제공하므로 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G94" s="3" t="inlineStr">
+        <is>
+          <t>해당 항로 이용 시 운임 변동 추이 모니터링 및 운송 계획에 반영, 인도네시아 신규 항로 활용 가능성 검토.</t>
+        </is>
+      </c>
+      <c r="H94" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I94" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260622-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J94" s="3" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B95" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="inlineStr">
+        <is>
+          <t>Logistics Cybersecurity Statistics 2026: Supply Chain Disruption</t>
+        </is>
+      </c>
+      <c r="E95" s="3" t="inlineStr">
+        <is>
+          <t>2026년 물류 사이버보안 통계는 공급망 침해, 랜섬웨어, 제3자 리스크, 클라우드 노출 및 운영 중단 위험에 대한 정보를 제공하며, 물류 공급망의 사이버 보안 취약성을 강조한다.</t>
+        </is>
+      </c>
+      <c r="F95" s="3" t="inlineStr">
+        <is>
+          <t>물류 공급망의 사이버 보안 위협은 우리 회사의 운영 중단 및 데이터 유출 리스크를 증가시킬 수 있으므로 지속적인 모니터링과 대비가 필요하다.</t>
+        </is>
+      </c>
+      <c r="G95" s="3" t="inlineStr">
+        <is>
+          <t>공급망 전반의 사이버 보안 취약점 점검 및 강화 방안 검토.</t>
+        </is>
+      </c>
+      <c r="H95" s="3" t="inlineStr">
+        <is>
+          <t>deepstrike.io</t>
+        </is>
+      </c>
+      <c r="I95" s="3" t="inlineStr">
+        <is>
+          <t>https://deepstrike.io/blog/logistics-cybersecurity-statistics</t>
+        </is>
+      </c>
+      <c r="J95" s="3" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="inlineStr">
+        <is>
+          <t>How Nissan turned a compliance database into a supply chain resilience engine</t>
+        </is>
+      </c>
+      <c r="E96" s="3" t="inlineStr">
+        <is>
+          <t>닛산이 규제 준수 데이터베이스를 활용하여 공급망 탄력성 엔진을 구축, 미국 관세, 반도체 부족, 사이버 교란 등의 위험을 완화하고 경쟁 우위를 확보했다.</t>
+        </is>
+      </c>
+      <c r="F96" s="3" t="inlineStr">
+        <is>
+          <t>다른 기업의 공급망 탄력성 강화 사례는 우리 회사의 공급망 관리 전략 개선에 참고할 만하며, 특히 관세 및 부품 부족 대응에 시사하는 바가 크다.</t>
+        </is>
+      </c>
+      <c r="G96" s="3" t="inlineStr">
+        <is>
+          <t>공급망 데이터 활용을 통한 리스크 관리 및 탄력성 강화 방안 연구.</t>
+        </is>
+      </c>
+      <c r="H96" s="3" t="inlineStr">
+        <is>
+          <t>news.google.com</t>
+        </is>
+      </c>
+      <c r="I96" s="3" t="inlineStr">
+        <is>
+          <t>https://news.google.com/read/CBMiwgJBVV95cUxOaXlJLTNyMjh5bW4zdlRYMElpX0MtZV9mZGh0LU9HUHJQbHpqY3NyZmdGQjlVd29ZWDNwVGF3MEpUSDVIRFBXd2p5cDQxX0RoM01uTXlibGkxRHNyeDJCVFIyU2IyM2l3OVNraXVDbUp1NEh0WlZWYW1XRWNOeVpHajVTaHI0d29fNEdnaGhiOUNLSG9tZk1hcnRkZzRURDU4MS1iUTJWRTJISnNSalBoNEhNVHlvZWpmNVZNZXNhVlEtbDVKa2YzMlptdDBTT1k2TW1WSnNRZHlyYkxCRm5VNjBrYUozckgtMC0yMGxxa2NLU0JRZDA1RnhjOHhUYU5EcUxZNnU1dW9qS29SUXpBMklnQ3lTNVVjTHMzcTJvSVdiMWF5VTdKZkFqdEVtUWhIb0s2OFpJYnJudmpON3ln?hl=en-US&amp;gl=US&amp;ceid=US%3Aen</t>
+        </is>
+      </c>
+      <c r="J96" s="3" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B97" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C97" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="inlineStr">
+        <is>
+          <t>미중, 희토류 이어 구리 전쟁?…기술 패권경쟁 새 전선 부각</t>
+        </is>
+      </c>
+      <c r="E97" s="3" t="inlineStr">
+        <is>
+          <t>미중 기술 패권 경쟁이 희토류에 이어 구리로 확대될 조짐을 보이며, 구리 공급망의 지정학적 리스크가 부각되고 있다.</t>
+        </is>
+      </c>
+      <c r="F97" s="3" t="inlineStr">
+        <is>
+          <t>구리는 배터리 및 전자부품의 핵심 원자재로, 미중 갈등 심화 시 공급망 불안정 및 가격 변동성 증가 가능성이 있어 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G97" s="3" t="inlineStr">
+        <is>
+          <t>주요 원자재인 구리의 글로벌 공급망 동향 및 미중 정책 변화를 면밀히 주시하고, 대체 공급처 확보 가능성을 검토.</t>
+        </is>
+      </c>
+      <c r="H97" s="3" t="inlineStr">
+        <is>
+          <t>연합뉴스</t>
+        </is>
+      </c>
+      <c r="I97" s="3" t="inlineStr">
+        <is>
+          <t>https://yna.co.kr/view/AKR20260624085400009</t>
+        </is>
+      </c>
+      <c r="J97" s="3" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B98" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D98" s="3" t="inlineStr">
+        <is>
+          <t>[2026 기후경쟁력포럼] 'AI데이터센터·반도체·배터리' 한국 지탱하는 산업에 불어오는 친환경 요구, 탈탄소 전력이 미래 경쟁력 가른다</t>
+        </is>
+      </c>
+      <c r="E98" s="3" t="inlineStr">
+        <is>
+          <t>배터리 산업을 포함한 주요 산업에서 탈탄소 전력 사용 등 친환경 요구가 강화되고 있으며, 이는 미래 경쟁력을 좌우할 핵심 요소로 부상하고 있다.</t>
+        </is>
+      </c>
+      <c r="F98" s="3" t="inlineStr">
+        <is>
+          <t>탈탄소 전력 사용 요구는 생산 및 물류 운영의 에너지 전환 및 탄소 배출량 관리에 대한 장기적인 전략 수립에 영향을 미칠 수 있으므로 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G98" s="3" t="inlineStr">
+        <is>
+          <t>장기적인 탄소 중립 목표 달성을 위한 에너지 전환 계획 및 친환경 물류 솔루션 도입 가능성을 검토.</t>
+        </is>
+      </c>
+      <c r="H98" s="3" t="inlineStr">
+        <is>
+          <t>허핑턴포스트코리아</t>
+        </is>
+      </c>
+      <c r="I98" s="3" t="inlineStr">
+        <is>
+          <t>https://huffingtonpost.kr/article/258207</t>
+        </is>
+      </c>
+      <c r="J98" s="3" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B99" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C99" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D99" s="3" t="inlineStr">
+        <is>
+          <t>미 재무 "동맹도 미국 시장접근엔 의무 수반"</t>
+        </is>
+      </c>
+      <c r="E99" s="3" t="inlineStr">
+        <is>
+          <t>미국 재무장관이 동맹국들도 미국 시장 접근 시 공급망 회복력 구축 의무를 수반해야 한다고 강조하며, 향후 무역 파트너국들에 대한 새로운 요구사항이 발생할 수 있음을 시사했다.</t>
+        </is>
+      </c>
+      <c r="F99" s="3" t="inlineStr">
+        <is>
+          <t>미국의 공급망 회복력 구축 요구는 향후 대미 수출입 규제나 공급망 실사 강화로 이어질 수 있어 관련 정책 변화를 주시해야 한다.</t>
+        </is>
+      </c>
+      <c r="G99" s="3" t="inlineStr">
+        <is>
+          <t>대미 수출입 관련 잠재적 규제 변화를 모니터링하고, 공급망 실사 및 리스크 관리 체계를 강화할 방안을 검토.</t>
+        </is>
+      </c>
+      <c r="H99" s="3" t="inlineStr">
+        <is>
+          <t>연합뉴스</t>
+        </is>
+      </c>
+      <c r="I99" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20260624091800009</t>
+        </is>
+      </c>
+      <c r="J99" s="3" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B100" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C100" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D100" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 재개방에도 국제유가 70달러 유지 전망 : 한국 조선업 플랜트 사업에 기회 오나</t>
+        </is>
+      </c>
+      <c r="E100" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 재개방에도 불구하고 국제유가가 배럴당 70달러 선을 유지할 것으로 전망되며, 이는 원유 수송 지연 및 중동 석유시설 재가동 문제와 연관되어 있다.</t>
+        </is>
+      </c>
+      <c r="F100" s="3" t="inlineStr">
+        <is>
+          <t>국제유가 변동은 해상 및 항공 운임에 직접적인 영향을 미쳐 물류비 상승 요인이 될 수 있으므로 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G100" s="3" t="inlineStr">
+        <is>
+          <t>유가 변동에 따른 운송비 변화를 예측하고, 운송 계약 시 유류할증료 조건 등을 면밀히 검토.</t>
+        </is>
+      </c>
+      <c r="H100" s="3" t="inlineStr">
+        <is>
+          <t>허핑턴포스트코리아</t>
+        </is>
+      </c>
+      <c r="I100" s="3" t="inlineStr">
+        <is>
+          <t>https://huffingtonpost.kr/article/258200</t>
+        </is>
+      </c>
+      <c r="J100" s="3" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B101" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C101" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D101" s="3" t="inlineStr">
+        <is>
+          <t>대전 생필품·개인서비스요금 상승세 지속…고환율·유가·기상 여건 영향</t>
+        </is>
+      </c>
+      <c r="E101" s="3" t="inlineStr">
+        <is>
+          <t>고환율과 국제유가 상승이 대전 지역 물가 상승의 주요 요인으로 지목되었으며, 이는 물류비용 증가로 이어질 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="F101" s="3" t="inlineStr">
+        <is>
+          <t>국제유가 상승과 고환율은 해상/항공 운임 및 전반적인 물류비용 상승으로 이어져 SCM 본부의 물류 예산 및 운영에 지속적인 영향을 미칠 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G101" s="3" t="inlineStr">
+        <is>
+          <t>유가 및 환율 변동 추이를 지속적으로 모니터링하고, 운송 계약 조건 재검토 및 비용 절감 방안을 모색해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H101" s="3" t="inlineStr">
+        <is>
+          <t>굿모닝충청</t>
+        </is>
+      </c>
+      <c r="I101" s="3" t="inlineStr">
+        <is>
+          <t>https://www.goodmorningcc.com/news/articleView.html?idxno=447979</t>
+        </is>
+      </c>
+      <c r="J101" s="3" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B102" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C102" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D102" s="4" t="inlineStr">
+        <is>
+          <t>세바, HAN-ORD 주3편 정기 전세편 운항</t>
+        </is>
+      </c>
+      <c r="E102" s="4" t="inlineStr">
+        <is>
+          <t>세바로지스틱스가 베트남 하노이(HAN)와 미국 시카고(ORD) 간 주 3회 정기 전세편 운항을 시작하여 아시아발 시카고 노선을 확장하고 베트남 내 항공화물 서비스를 강화한다.</t>
+        </is>
+      </c>
+      <c r="F102" s="4" t="inlineStr">
+        <is>
+          <t>특정 포워더의 신규 전세편 운항 소식으로, 우리 회사의 직접적인 물류 운영에 즉각적인 영향은 없으며 참고할 만한 정보이다.</t>
+        </is>
+      </c>
+      <c r="G102" s="4" t="n"/>
+      <c r="H102" s="4" t="inlineStr">
+        <is>
+          <t>cargonews</t>
+        </is>
+      </c>
+      <c r="I102" s="4" t="inlineStr">
+        <is>
+          <t>https://www.cargonews.co.kr/news/articleView.html?idxno=60401</t>
+        </is>
+      </c>
+      <c r="J102" s="4" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B103" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C103" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D103" s="4" t="inlineStr">
+        <is>
+          <t>WMES 2026 Speech - Stuart Fox, IATA's Director Flight and Operations</t>
+        </is>
+      </c>
+      <c r="E103" s="4" t="inlineStr">
+        <is>
+          <t>IATA 연설에서 항공기 인도 지연, 엔진 수명 단축, 예비 부품 확보 어려움, 수리 시간 증가 등 항공사들이 직면한 현실적인 공급망 문제들이 언급되었다.</t>
+        </is>
+      </c>
+      <c r="F103" s="4" t="inlineStr">
+        <is>
+          <t>항공기 공급망 전반의 어려움을 언급하는 내용으로, 우리 회사의 항공 운송 능력이나 비용에 직접적인 영향을 미친다고 보기는 어렵다.</t>
+        </is>
+      </c>
+      <c r="G103" s="4" t="n"/>
+      <c r="H103" s="4" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I103" s="4" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-speeches/06-24-wmes-2026-speech-stuart-fox-iata-director-flight-operations/</t>
+        </is>
+      </c>
+      <c r="J103" s="4" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B104" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C104" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D104" s="4" t="inlineStr">
+        <is>
+          <t>States and Supporting Partners Join IATA’s Alliance to Expand CORSIA Carbon Credit Supply</t>
+        </is>
+      </c>
+      <c r="E104" s="4" t="inlineStr">
+        <is>
+          <t>IATA는 CORSIA 탄소 배출권 공급 확대를 위한 연합에 더 많은 국가 및 파트너들이 참여했다고 발표했다.</t>
+        </is>
+      </c>
+      <c r="F104" s="4" t="inlineStr">
+        <is>
+          <t>항공 부문의 탄소 배출권 관련 소식으로, 우리 회사의 물류 운영에 즉각적인 영향은 없으며 장기적인 환경 규제 동향으로 참고할 만하다.</t>
+        </is>
+      </c>
+      <c r="G104" s="4" t="n"/>
+      <c r="H104" s="4" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I104" s="4" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-23-states-supporting-partners-join-iata-alliance-expand-corsia-carbon-credit-supply/</t>
+        </is>
+      </c>
+      <c r="J104" s="4" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B105" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C105" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D105" s="4" t="inlineStr">
+        <is>
+          <t>2026년 4월 글로벌 선박 스케줄 신뢰도, 올해 최고치 기록</t>
+        </is>
+      </c>
+      <c r="E105" s="4" t="inlineStr">
+        <is>
+          <t>2026년 4월 글로벌 선박 스케줄 신뢰도가 올해 들어 가장 높은 수준을 기록하여 해운 서비스의 정시성이 개선되었습니다.</t>
+        </is>
+      </c>
+      <c r="F105" s="4" t="inlineStr">
+        <is>
+          <t>선박 스케줄 신뢰도 개선은 긍정적인 소식이지만, 과거 데이터 분석 결과이며 당사의 즉각적인 물류 운영에 직접적인 영향을 미치기보다는 참고 수준입니다.</t>
+        </is>
+      </c>
+      <c r="G105" s="4" t="n"/>
+      <c r="H105" s="4" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I105" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/390-global-schedule-reliability-for-april-2026-the-highest-of-the-year</t>
+        </is>
+      </c>
+      <c r="J105" s="4" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B106" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C106" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D106" s="4" t="inlineStr">
+        <is>
+          <t>Transpacific: Ripe for new non-alliance services</t>
+        </is>
+      </c>
+      <c r="E106" s="4" t="inlineStr">
+        <is>
+          <t>아시아-북미 서안 항로에서 비동맹 선사들의 컨테이너 선박 용량 확대 가능성이 분석되었습니다.</t>
+        </is>
+      </c>
+      <c r="F106" s="4" t="inlineStr">
+        <is>
+          <t>특정 항로의 시장 역학 변화 가능성에 대한 분석으로, 당장 물류 운영에 직접적인 영향을 미치기보다는 장기적인 시장 동향 참고 수준입니다.</t>
+        </is>
+      </c>
+      <c r="G106" s="4" t="n"/>
+      <c r="H106" s="4" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I106" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/393-transpacific-ripe-for-new-non-alliance-services</t>
+        </is>
+      </c>
+      <c r="J106" s="4" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B107" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C107" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D107" s="4" t="inlineStr">
+        <is>
+          <t>2026년 1분기 북미 동부 해안 항만, 시장 점유율 유지</t>
+        </is>
+      </c>
+      <c r="E107" s="4" t="inlineStr">
+        <is>
+          <t>2026년 1분기 북미 동부 해안(NAEC) 항만 물동량이 전년 대비 감소했음에도 불구하고 시장 점유율을 유지했습니다.</t>
+        </is>
+      </c>
+      <c r="F107" s="4" t="inlineStr">
+        <is>
+          <t>과거 항만 물동량 분석 결과로, 당사의 즉각적인 물류 운영에 직접적인 영향을 미치기보다는 북미 동부 항만 이용 시 참고할 수 있는 수준입니다.</t>
+        </is>
+      </c>
+      <c r="G107" s="4" t="n"/>
+      <c r="H107" s="4" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I107" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/391-2026-q1-naec-ports-consolidate-market-share</t>
+        </is>
+      </c>
+      <c r="J107" s="4" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B108" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C108" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D108" s="4" t="inlineStr">
+        <is>
+          <t>Gemini Cooperation, 지중해 항로 선박 재배치 분석</t>
+        </is>
+      </c>
+      <c r="E108" s="4" t="inlineStr">
+        <is>
+          <t>Gemini Cooperation이 동서 컨테이너 선박 배치를 재조정하며 지중해 항로에서 시장 점유율을 확대하고 있는 것으로 분석되었습니다.</t>
+        </is>
+      </c>
+      <c r="F108" s="4" t="inlineStr">
+        <is>
+          <t>특정 선사의 전략적 선박 재배치에 대한 분석으로, 당사의 물류 운영에 직접적인 영향을 미치기보다는 해운 시장 동향 참고 수준입니다.</t>
+        </is>
+      </c>
+      <c r="G108" s="4" t="n"/>
+      <c r="H108" s="4" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I108" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/392-decoding-gemini-s-mediterranean-surge</t>
+        </is>
+      </c>
+      <c r="J108" s="4" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B109" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C109" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D109" s="4" t="inlineStr">
+        <is>
+          <t>The Future of Planning Isn't Another Chatbot: Board Introduces Supply Chain and Merchandiser Agents for Agentic Continuous Planning</t>
+        </is>
+      </c>
+      <c r="E109" s="4" t="inlineStr">
+        <is>
+          <t>Board사가 공급망 및 머천다이저 에이전트를 도입하여 계획 데이터, 운영 신호, 예측 정보 및 시나리오 분석을 결합함으로써 공급망 중단 영향을 예측하고 대응 옵션을 신속하게 평가할 수 있도록 돕는다.</t>
+        </is>
+      </c>
+      <c r="F109" s="4" t="inlineStr">
+        <is>
+          <t>새로운 공급망 계획 기술 도입에 대한 정보로, 당장 우리 회사의 물류 운영에 직접적인 영향을 미치지는 않지만 장기적인 관점에서 참고할 만하다.</t>
+        </is>
+      </c>
+      <c r="G109" s="4" t="n"/>
+      <c r="H109" s="4" t="inlineStr">
+        <is>
+          <t>prnewswire.com</t>
+        </is>
+      </c>
+      <c r="I109" s="4" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/the-future-of-planning-isnt-another-chatbot-board-introduces-supply-chain-and-merchandiser-agents-for-agentic-continuous-planning-302808321.html</t>
+        </is>
+      </c>
+      <c r="J109" s="4" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B110" s="4" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C110" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D110" s="4" t="inlineStr">
+        <is>
+          <t>“K-배터리, 반도체 버금가는 전략산업”…세제지원 실효성 촉구</t>
+        </is>
+      </c>
+      <c r="E110" s="4" t="inlineStr">
+        <is>
+          <t>K-배터리 산업이 반도체에 버금가는 전략산업으로 부상하며, 적자 기업도 혜택을 볼 수 있는 실효성 있는 세제지원 체계 마련이 촉구되고 있다.</t>
+        </is>
+      </c>
+      <c r="F110" s="4" t="inlineStr">
+        <is>
+          <t>세제지원 논의는 장기적으로 산업 경쟁력에 영향을 미칠 수 있으나, 당장의 물류 운영에 직접적인 영향은 미미하다.</t>
+        </is>
+      </c>
+      <c r="G110" s="4" t="n"/>
+      <c r="H110" s="4" t="inlineStr">
+        <is>
+          <t>전자신문</t>
+        </is>
+      </c>
+      <c r="I110" s="4" t="inlineStr">
+        <is>
+          <t>https://etnews.com/20260624000346</t>
+        </is>
+      </c>
+      <c r="J110" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4390,7 +5706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4537,6 +5853,49 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>3121.69</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>+136 (+4.6%)</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>+881 (+39.3%)</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>3747</v>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>+398 (+11.9%)</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>+940 (+33.5%)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4549,7 +5908,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5100,6 +6459,76 @@
       </c>
       <c r="I15" s="6" t="inlineStr"/>
     </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>RSK-015</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 폐쇄로 화물 192조원어치 고립</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr"/>
+      <c r="G16" s="6" t="inlineStr"/>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>중동 항로 이용 시 대체 경로 및 운송 수단 검토, 비상 계획 수립 및 관련 부서와 비상 상황 대응 시나리오 공유.</t>
+        </is>
+      </c>
+      <c r="I16" s="6" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>RSK-016</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>EU산 배터리 현지화 요구 강세&amp;hellip;韓 배터리 소재, 유럽 거점 효과 본다 [배터리레이다]</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr"/>
+      <c r="G17" s="6" t="inlineStr"/>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>EU 시장 공급을 위한 현지 생산 및 소재 조달 전략을 재검토하고, 유럽 내 물류 거점 및 공급망 최적화 방안을 수립.</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
📰 뉴스 데이터 2026-06-25_19:28
</commit_message>
<xml_diff>
--- a/data/SCM_물류_브리핑.xlsx
+++ b/data/SCM_물류_브리핑.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J110"/>
+  <dimension ref="A1:J139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5693,6 +5693,1358 @@
         </is>
       </c>
       <c r="J110" s="4" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>美 세관, 단속 대폭 강화…수입업자·중개인 '충격'</t>
+        </is>
+      </c>
+      <c r="E111" s="2" t="inlineStr">
+        <is>
+          <t>미국 정부가 수입업자 자격, 공시 의무, 전자상거래 통관 절차 등 세관 단속을 대폭 강화하여 수입업자와 세관 중개인의 규제 부담이 커질 것으로 예상된다.</t>
+        </is>
+      </c>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>미국으로의 배터리/전자부품 수출 시 통관 지연 및 추가 비용 발생 가능성이 높아 즉각적인 대응이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G111" s="2" t="inlineStr">
+        <is>
+          <t>미국 수출 통관 절차 및 필요 서류 재검토, 현지 파트너와 협력하여 강화된 규제 준수 방안 마련, 잠재적 지연에 대비한 재고 및 운송 계획 조정</t>
+        </is>
+      </c>
+      <c r="H111" s="2" t="inlineStr">
+        <is>
+          <t>kita</t>
+        </is>
+      </c>
+      <c r="I111" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kita.net/shippers/board/newsView.do?morgueCode=2&amp;dataCls=A&amp;dataSeq=2525</t>
+        </is>
+      </c>
+      <c r="J111" s="2" t="inlineStr">
+        <is>
+          <t>RSK-017</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>中, 핵심광물 대일 수출 0…日기업들, 외교적 해결 SOS | 한국경제</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="inlineStr">
+        <is>
+          <t>중국이 핵심광물(텅스텐, 이트륨 등)의 대일 수출을 중단하여 일본 기업들이 재고 소진 및 생산 차질 위기에 직면했으며, 외교적 해결을 모색하고 있다.</t>
+        </is>
+      </c>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>핵심광물은 배터리 및 전자부품 제조에 필수적인 원자재로, 중국의 수출 통제는 당사의 원자재 수급 및 생산 계획에 직접적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G112" s="2" t="inlineStr">
+        <is>
+          <t>중국산 핵심광물 의존도를 재평가하고, 대체 공급처 발굴 및 재고 확보 방안을 즉시 검토하며, 공급망 다변화 전략을 수립한다.</t>
+        </is>
+      </c>
+      <c r="H112" s="2" t="inlineStr">
+        <is>
+          <t>한국경제</t>
+        </is>
+      </c>
+      <c r="I112" s="2" t="inlineStr">
+        <is>
+          <t>https://hankyung.com/article/202606246260i</t>
+        </is>
+      </c>
+      <c r="J112" s="2" t="inlineStr">
+        <is>
+          <t>RSK-018</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B113" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C113" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D113" s="3" t="inlineStr">
+        <is>
+          <t>States and Supporting Partners Join IATA’s Alliance to Expand CORSIA Carbon Credit Supply</t>
+        </is>
+      </c>
+      <c r="E113" s="3" t="inlineStr">
+        <is>
+          <t>IATA가 CORSIA 탄소 크레딧 공급 확대를 위한 연합에 더 많은 국가 및 파트너들이 참여했다고 발표하며, 항공 산업의 탄소 배출량 감축 노력을 강화하고 있다.</t>
+        </is>
+      </c>
+      <c r="F113" s="3" t="inlineStr">
+        <is>
+          <t>항공 운송의 탄소 배출 규제 강화는 장기적으로 항공 운임 상승 요인이 될 수 있으므로 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G113" s="3" t="inlineStr">
+        <is>
+          <t>항공 운송 탄소 규제 동향 및 잠재적 운임 영향 분석</t>
+        </is>
+      </c>
+      <c r="H113" s="3" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I113" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-23-states-supporting-partners-join-iata-alliance-expand-corsia-carbon-credit-supply/</t>
+        </is>
+      </c>
+      <c r="J113" s="3" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B114" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C114" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D114" s="3" t="inlineStr">
+        <is>
+          <t>[2026.6.25.] 중동 전쟁 관련 유가 및 물류 동향</t>
+        </is>
+      </c>
+      <c r="E114" s="3" t="inlineStr">
+        <is>
+          <t>중동 전쟁 관련 유가 및 물류 동향에 대한 모니터링 보고서로, 지역 불안정이 유가 변동 및 해상 운송에 미치는 영향을 분석한다.</t>
+        </is>
+      </c>
+      <c r="F114" s="3" t="inlineStr">
+        <is>
+          <t>중동 지역의 지정학적 리스크는 유가 및 해상 운임에 지속적인 영향을 미치므로, 물류비 변동 가능성에 대비하여 추이를 면밀히 주시해야 한다.</t>
+        </is>
+      </c>
+      <c r="G114" s="3" t="inlineStr">
+        <is>
+          <t>유가 및 해상 운임 변동 추이 지속 모니터링, 비상 운송 경로 및 운송사 옵션 검토</t>
+        </is>
+      </c>
+      <c r="H114" s="3" t="inlineStr">
+        <is>
+          <t>kotra</t>
+        </is>
+      </c>
+      <c r="I114" s="3" t="inlineStr">
+        <is>
+          <t>https://dream.kotra.or.kr/kotranews/cms/news/actionKotraBoardDetail.do?SITE_NO=3&amp;MENU_ID=70&amp;CONTENTS_NO=1&amp;pNttSn=242420</t>
+        </is>
+      </c>
+      <c r="J114" s="3" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B115" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C115" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D115" s="3" t="inlineStr">
+        <is>
+          <t>Tracking True Vessel Delay</t>
+        </is>
+      </c>
+      <c r="E115" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence 분석에 따르면 선사들이 운송 시간을 늘리는 스케줄 버퍼링을 통해 선박 지연을 관리하고 있으며, 이는 실제 운항 지연과 조기 도착 간의 관계를 보여준다.</t>
+        </is>
+      </c>
+      <c r="F115" s="3" t="inlineStr">
+        <is>
+          <t>선사들의 스케줄 버퍼링 전략은 실제 운송 리드타임에 영향을 미칠 수 있으므로, 선박 스케줄 신뢰도 및 운송 계획 수립 시 참고해야 한다.</t>
+        </is>
+      </c>
+      <c r="G115" s="3" t="inlineStr">
+        <is>
+          <t>주요 항로의 선박 스케줄 신뢰도 및 실제 운송 리드타임 추이 지속 모니터링</t>
+        </is>
+      </c>
+      <c r="H115" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I115" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/394-tracking-true-vessel-delay</t>
+        </is>
+      </c>
+      <c r="J115" s="3" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B116" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C116" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D116" s="3" t="inlineStr">
+        <is>
+          <t>Transpacific: Ripe for new non-alliance services</t>
+        </is>
+      </c>
+      <c r="E116" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence 분석에 따르면 태평양 횡단 항로에서 비동맹 선사들의 컨테이너 선박 용량과 스팟 운임 간의 관계를 분석하며, 새로운 비동맹 서비스의 출현 가능성을 시사한다.</t>
+        </is>
+      </c>
+      <c r="F116" s="3" t="inlineStr">
+        <is>
+          <t>태평양 횡단 항로의 운임 및 서비스 옵션 변화 가능성을 시사하므로, 해당 항로를 이용하는 우리 회사의 운송 전략 및 비용에 영향을 미칠 수 있어 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G116" s="3" t="inlineStr">
+        <is>
+          <t>태평양 횡단 항로의 운임 및 서비스 공급 동향 지속 모니터링, 비동맹 선사 서비스 활용 가능성 검토</t>
+        </is>
+      </c>
+      <c r="H116" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I116" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/393-transpacific-ripe-for-new-non-alliance-services</t>
+        </is>
+      </c>
+      <c r="J116" s="3" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B117" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C117" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D117" s="3" t="inlineStr">
+        <is>
+          <t>2026-Q1: NAEC Ports Consolidate Market Share</t>
+        </is>
+      </c>
+      <c r="E117" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence 분석에 따르면 2026년 1분기 북미 동부 해안(NAEC) 항만의 컨테이너 물동량이 전년 대비 감소했음에도 불구하고 시장 점유율을 공고히 하고 있음을 보여준다.</t>
+        </is>
+      </c>
+      <c r="F117" s="3" t="inlineStr">
+        <is>
+          <t>북미 동부 해안 항만의 물동량 및 시장 점유율 변화는 해당 지역으로의 운송 계획 수립 시 고려해야 할 요소이므로 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G117" s="3" t="inlineStr">
+        <is>
+          <t>북미 동부 해안 항만의 물동량 및 운영 효율성 추이 지속 모니터링, 잠재적 병목 현상 발생 시 대체 항만 또는 운송 경로 검토</t>
+        </is>
+      </c>
+      <c r="H117" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I117" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/391-2026-q1-naec-ports-consolidate-market-share</t>
+        </is>
+      </c>
+      <c r="J117" s="3" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B118" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C118" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D118" s="3" t="inlineStr">
+        <is>
+          <t>Global Schedule Reliability for April 2026 the Highest of the Year</t>
+        </is>
+      </c>
+      <c r="E118" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence 보고서에 따르면 2026년 4월 전 세계 선박 스케줄 신뢰도가 올해 최고치를 기록하며 해상 운송의 정시성이 개선되고 있음을 나타낸다.</t>
+        </is>
+      </c>
+      <c r="F118" s="3" t="inlineStr">
+        <is>
+          <t>전반적인 선박 스케줄 신뢰도 개선은 운송 계획 수립에 긍정적인 영향을 미칠 수 있으나, 특정 항로 및 선사의 신뢰도를 지속적으로 확인해야 한다.</t>
+        </is>
+      </c>
+      <c r="G118" s="3" t="inlineStr">
+        <is>
+          <t>주요 운송 항로 및 계약 선사의 스케줄 신뢰도 지표 지속 모니터링 및 운송 계획에 반영</t>
+        </is>
+      </c>
+      <c r="H118" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I118" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/390-global-schedule-reliability-for-april-2026-the-highest-of-the-year</t>
+        </is>
+      </c>
+      <c r="J118" s="3" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B119" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C119" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D119" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 통항 재개를 환영하며, 선원 안전 보호조치는 지속되어야 한다</t>
+        </is>
+      </c>
+      <c r="E119" s="3" t="inlineStr">
+        <is>
+          <t>선원노련이 호르무즈 해협 통항 재개를 환영하면서도, 해당 지역의 긴장이 여전히 지속되고 있어 선원 안전 확보 및 통항 지원 조치가 계속되어야 한다고 강조했다.</t>
+        </is>
+      </c>
+      <c r="F119" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협은 주요 해상 운송 경로 중 하나로, 통항 재개는 긍정적이나 지역 긴장이 지속되어 언제든 운송 차질이 발생할 수 있으므로 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G119" s="3" t="inlineStr">
+        <is>
+          <t>중동 지역 지정학적 상황 및 해상 운송 경로 안전성 지속 모니터링, 비상 운송 경로 및 보험 적용 여부 검토</t>
+        </is>
+      </c>
+      <c r="H119" s="3" t="inlineStr">
+        <is>
+          <t>shippingnews</t>
+        </is>
+      </c>
+      <c r="I119" s="3" t="inlineStr">
+        <is>
+          <t>https://www.shippingnewsnet.com/news/articleView.html?idxno=70904</t>
+        </is>
+      </c>
+      <c r="J119" s="3" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B120" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C120" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D120" s="3" t="inlineStr">
+        <is>
+          <t>7월 1일부터 160Wh 초과 대용량 리튬배터리 지하철 반입 제한</t>
+        </is>
+      </c>
+      <c r="E120" s="3" t="inlineStr">
+        <is>
+          <t>서울교통공사가 7월 1일부터 160Wh 초과 대용량 리튬배터리 및 개인형 이동장치(PM)의 지하철 반입을 제한하여 화재 예방을 강화한다.</t>
+        </is>
+      </c>
+      <c r="F120" s="3" t="inlineStr">
+        <is>
+          <t>대용량 리튬배터리 운송에 대한 안전 규제 강화 추세를 보여주며, 향후 물류 전반의 규제 강화로 이어질 가능성이 있어 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G120" s="3" t="inlineStr">
+        <is>
+          <t>사내 임직원 대상 대용량 배터리 휴대 관련 안내 및 물류/CS 부서에 해당 규제 내용 공유.</t>
+        </is>
+      </c>
+      <c r="H120" s="3" t="inlineStr">
+        <is>
+          <t>The PR 더피알</t>
+        </is>
+      </c>
+      <c r="I120" s="3" t="inlineStr">
+        <is>
+          <t>https://the-pr.co.kr/news/articleView.html?idxno=61703</t>
+        </is>
+      </c>
+      <c r="J120" s="3" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B121" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C121" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D121" s="3" t="inlineStr">
+        <is>
+          <t>미중, 희토류 이어 구리 전쟁?…기술 패권경쟁 새 전선 부각</t>
+        </is>
+      </c>
+      <c r="E121" s="3" t="inlineStr">
+        <is>
+          <t>미중 기술 패권 경쟁이 희토류에 이어 구리로 확대될 조짐을 보이며, 핵심 광물 공급망의 지정학적 리스크가 부각되고 있다.</t>
+        </is>
+      </c>
+      <c r="F121" s="3" t="inlineStr">
+        <is>
+          <t>배터리 및 전자부품 제조에 필수적인 구리의 공급망이 미중 갈등으로 불안정해질 가능성이 있어 원자재 수급 및 가격 변동에 대한 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G121" s="3" t="inlineStr">
+        <is>
+          <t>구리 등 핵심 원자재의 공급망 다변화 전략 검토 및 재고 수준 점검, 관련 시장 동향 지속 모니터링.</t>
+        </is>
+      </c>
+      <c r="H121" s="3" t="inlineStr">
+        <is>
+          <t>연합뉴스</t>
+        </is>
+      </c>
+      <c r="I121" s="3" t="inlineStr">
+        <is>
+          <t>https://yna.co.kr/view/AKR20260624085400009</t>
+        </is>
+      </c>
+      <c r="J121" s="3" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B122" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C122" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D122" s="3" t="inlineStr">
+        <is>
+          <t>[2026 기후경쟁력포럼] 'AI데이터센터·반도체·배터리' 한국 지탱하는 산업에 불어오는 친환경 요구, 탈탄소 전력이 미래 경쟁력 가른다</t>
+        </is>
+      </c>
+      <c r="E122" s="3" t="inlineStr">
+        <is>
+          <t>AI 데이터센터, 반도체, 배터리 등 한국의 주요 산업에서 친환경 요구와 탈탄소 전력의 중요성이 커지며, 이는 미래 경쟁력을 좌우할 핵심 요소로 부각되고 있다.</t>
+        </is>
+      </c>
+      <c r="F122" s="3" t="inlineStr">
+        <is>
+          <t>배터리 산업의 친환경 및 탈탄소 요구 증가는 장기적인 생산 및 물류 전략에 영향을 미치므로, ESG 경영 및 녹색 물류 전환을 위한 준비 차원에서 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G122" s="3" t="inlineStr">
+        <is>
+          <t>ESG 경영 전략에 따른 친환경 물류 방안 검토, 재생에너지 사용 및 탄소 배출 저감 목표 설정.</t>
+        </is>
+      </c>
+      <c r="H122" s="3" t="inlineStr">
+        <is>
+          <t>허핑턴포스트</t>
+        </is>
+      </c>
+      <c r="I122" s="3" t="inlineStr">
+        <is>
+          <t>https://huffingtonpost.kr/article/258207</t>
+        </is>
+      </c>
+      <c r="J122" s="3" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B123" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C123" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D123" s="3" t="inlineStr">
+        <is>
+          <t>EU산 배터리 현지화 요구 강세…韓 배터리 소재, 유럽 거점 효과 본다 [배터리레이다]</t>
+        </is>
+      </c>
+      <c r="E123" s="3" t="inlineStr">
+        <is>
+          <t>유럽연합(EU)이 '메이드 인 유럽' 기조를 강화하면서 배터리 현지화 요구가 강해지고 있으며, 이는 한국 배터리 소재 기업들이 유럽 내 거점을 확보할 경우 수혜를 볼 수 있다는 전망이다.</t>
+        </is>
+      </c>
+      <c r="F123" s="3" t="inlineStr">
+        <is>
+          <t>EU의 현지화 요구는 장기적으로 유럽향 배터리 및 부품 수출 전략과 공급망 구축에 영향을 미칠 수 있으므로 추이를 주시해야 한다.</t>
+        </is>
+      </c>
+      <c r="G123" s="3" t="inlineStr">
+        <is>
+          <t>EU의 배터리 현지화 정책 구체화 동향을 지속적으로 모니터링하고, 유럽 내 생산 및 공급망 전략을 검토할 필요가 있다.</t>
+        </is>
+      </c>
+      <c r="H123" s="3" t="inlineStr">
+        <is>
+          <t>디지털데일리</t>
+        </is>
+      </c>
+      <c r="I123" s="3" t="inlineStr">
+        <is>
+          <t>https://ddaily.co.kr/page/view/2026062413521879081</t>
+        </is>
+      </c>
+      <c r="J123" s="3" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B124" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C124" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D124" s="3" t="inlineStr">
+        <is>
+          <t>미 재무 "동맹도 미국 시장접근엔 의무 수반" | 연합뉴스</t>
+        </is>
+      </c>
+      <c r="E124" s="3" t="inlineStr">
+        <is>
+          <t>미국 재무장관이 적대 세력의 공급망 차단에 대비한 경제 회복력 구축을 강조하며, 동맹국들도 미국 시장 접근에 상응하는 의무가 수반된다고 언급했다.</t>
+        </is>
+      </c>
+      <c r="F124" s="3" t="inlineStr">
+        <is>
+          <t>미국의 공급망 재편 및 자국 우선주의 기조가 강화될 수 있음을 시사하며, 이는 향후 글로벌 공급망 전략 및 무역 정책에 영향을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="G124" s="3" t="inlineStr">
+        <is>
+          <t>미국 정부의 공급망 관련 정책 및 무역 규제 동향을 지속적으로 모니터링하고, 공급망 다변화 및 리스크 분산 전략을 검토한다.</t>
+        </is>
+      </c>
+      <c r="H124" s="3" t="inlineStr">
+        <is>
+          <t>연합뉴스</t>
+        </is>
+      </c>
+      <c r="I124" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20260624091800009</t>
+        </is>
+      </c>
+      <c r="J124" s="3" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B125" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C125" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D125" s="3" t="inlineStr">
+        <is>
+          <t>이란-오만, 호르무즈 해협 통항 비용 협정 논의…국제 해운업계 우려</t>
+        </is>
+      </c>
+      <c r="E125" s="3" t="inlineStr">
+        <is>
+          <t>이란과 오만이 호르무즈 해협 관리 및 통항 비용 협정을 논의 중이며, 이란의 해협 관리 권한 강화 시도로 국제 해운업계는 통행료 도입 가능성에 대한 우려를 표하고 있다.</t>
+        </is>
+      </c>
+      <c r="F125" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협은 주요 해상 운송로로, 통행료가 도입될 경우 해상 운임 상승 및 물류비 증가로 이어질 수 있어 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G125" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 통항 비용 협정 진행 상황을 주시하고, 해상 운임 변동 가능성에 대비하여 운송 계약 조건 및 예산을 검토한다.</t>
+        </is>
+      </c>
+      <c r="H125" s="3" t="inlineStr">
+        <is>
+          <t>더구루(the guru)</t>
+        </is>
+      </c>
+      <c r="I125" s="3" t="inlineStr">
+        <is>
+          <t>https://theguru.co.kr/news/article.html?no=103495</t>
+        </is>
+      </c>
+      <c r="J125" s="3" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B126" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C126" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D126" s="3" t="inlineStr">
+        <is>
+          <t>드론에 뚫린 러 정유공장... 항공유 64% 폭등에 비행기 멈춘다</t>
+        </is>
+      </c>
+      <c r="E126" s="3" t="inlineStr">
+        <is>
+          <t>우크라이나의 드론 공격으로 러시아 정유공장 가동이 중단되면서 항공유 가격이 최대 64% 폭등하여 러시아 지역 항공사들이 운항 위기에 처했다.</t>
+        </is>
+      </c>
+      <c r="F126" s="3" t="inlineStr">
+        <is>
+          <t>러시아 지역의 항공유 가격 폭등은 해당 지역 항공 운송에 직접적인 영향을 미치며, 글로벌 항공유 시장에도 간접적인 영향을 주어 항공 운임 상승으로 이어질 수 있다.</t>
+        </is>
+      </c>
+      <c r="G126" s="3" t="inlineStr">
+        <is>
+          <t>글로벌 항공유 가격 및 항공 운임 변동 추이를 모니터링하고, 러시아 및 인접 지역으로의 항공 운송 계획에 대한 잠재적 리스크를 평가한다.</t>
+        </is>
+      </c>
+      <c r="H126" s="3" t="inlineStr">
+        <is>
+          <t>인사이트</t>
+        </is>
+      </c>
+      <c r="I126" s="3" t="inlineStr">
+        <is>
+          <t>https://insight.co.kr/news/560195</t>
+        </is>
+      </c>
+      <c r="J126" s="3" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B127" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C127" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D127" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 재개방에도 국제유가 70달러 유지 전망 : 한국 조선업 플랜트 사업에 기회 오나</t>
+        </is>
+      </c>
+      <c r="E127" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 재개방이 가시화되었음에도 불구하고 기뢰, 항만시설 훼손, 중동 석유시설 재가동 지연 등의 이유로 국제유가가 배럴당 70달러대를 유지할 것으로 전망된다.</t>
+        </is>
+      </c>
+      <c r="F127" s="3" t="inlineStr">
+        <is>
+          <t>국제유가가 높은 수준을 유지할 경우 항공 및 해상 운송의 유류할증료 상승으로 이어져 물류비 부담이 지속될 수 있다.</t>
+        </is>
+      </c>
+      <c r="G127" s="3" t="inlineStr">
+        <is>
+          <t>유가 변동 추이를 지속적으로 모니터링하고, 유류할증료 변화에 따른 물류비 예산 및 운송 계약 조건을 주기적으로 검토한다.</t>
+        </is>
+      </c>
+      <c r="H127" s="3" t="inlineStr">
+        <is>
+          <t>허핑턴포스트</t>
+        </is>
+      </c>
+      <c r="I127" s="3" t="inlineStr">
+        <is>
+          <t>https://www.huffingtonpost.kr/article/258200</t>
+        </is>
+      </c>
+      <c r="J127" s="3" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B128" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C128" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D128" s="4" t="inlineStr">
+        <is>
+          <t>IATA and IATP Collaborate to Support Airline Supply Chain Resilience</t>
+        </is>
+      </c>
+      <c r="E128" s="4" t="inlineStr">
+        <is>
+          <t>IATA와 IATP가 항공기 부품 가시성 및 접근성 개선을 위해 협력하여 항공사 공급망 복원력을 지원하기로 합의했다.</t>
+        </is>
+      </c>
+      <c r="F128" s="4" t="inlineStr">
+        <is>
+          <t>항공기 부품 공급망 개선에 대한 내용으로, 우리 회사의 배터리/전자부품 운송과는 직접적인 관련이 낮다.</t>
+        </is>
+      </c>
+      <c r="G128" s="4" t="n"/>
+      <c r="H128" s="4" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I128" s="4" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-25-iata-iatp-collaborate-support-airline-supply-chain-resilience/</t>
+        </is>
+      </c>
+      <c r="J128" s="4" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B129" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C129" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D129" s="4" t="inlineStr">
+        <is>
+          <t>Urgent Action Needed to Ease Engine MRO Bottlenecks</t>
+        </is>
+      </c>
+      <c r="E129" s="4" t="inlineStr">
+        <is>
+          <t>IATA가 최신 단일 통로 항공기 엔진의 유지보수, 수리, 정비(MRO) 병목 현상 완화를 위한 긴급 조치가 필요하다는 연구 결과를 발표했다.</t>
+        </is>
+      </c>
+      <c r="F129" s="4" t="inlineStr">
+        <is>
+          <t>항공기 엔진 MRO 병목 현상에 대한 내용으로, 우리 회사의 배터리/전자부품 운송과는 직접적인 관련이 낮다.</t>
+        </is>
+      </c>
+      <c r="G129" s="4" t="n"/>
+      <c r="H129" s="4" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I129" s="4" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-24-urgent-action-needed-to-ease-engine-mro-bottlenecks/</t>
+        </is>
+      </c>
+      <c r="J129" s="4" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B130" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C130" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D130" s="4" t="inlineStr">
+        <is>
+          <t>IATA Outlines Four Priorities to Strengthen the Aviation Supply Chain</t>
+        </is>
+      </c>
+      <c r="E130" s="4" t="inlineStr">
+        <is>
+          <t>IATA가 항공우주 공급망의 지속적인 문제 해결을 위해 공급망 가시성 강화, 부품 가용성 개선, MRO 효율성 증대, 인력 확보 등 네 가지 우선순위를 제시했다.</t>
+        </is>
+      </c>
+      <c r="F130" s="4" t="inlineStr">
+        <is>
+          <t>항공우주 산업의 내부 공급망 강화에 대한 내용으로, 우리 회사의 배터리/전자부품 운송과는 직접적인 관련이 낮다.</t>
+        </is>
+      </c>
+      <c r="G130" s="4" t="n"/>
+      <c r="H130" s="4" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I130" s="4" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-24-iata-outlines-four-priorities-to-strengthen-aviation-supply-chain/</t>
+        </is>
+      </c>
+      <c r="J130" s="4" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B131" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C131" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D131" s="4" t="inlineStr">
+        <is>
+          <t>WMES 2026 Speech - Stuart Fox, IATA's Director Flight and Operations</t>
+        </is>
+      </c>
+      <c r="E131" s="4" t="inlineStr">
+        <is>
+          <t>IATA 관계자가 항공기 납기 지연, 엔진 수명 단축, 예비 부품 확보 어려움, 수리 기간 장기화 등 항공사들이 직면한 현실적인 공급망 문제를 언급했다.</t>
+        </is>
+      </c>
+      <c r="F131" s="4" t="inlineStr">
+        <is>
+          <t>항공사 내부 운영 및 항공기 부품 공급망 문제에 대한 내용으로, 우리 회사의 배터리/전자부품 운송과는 직접적인 관련이 낮다.</t>
+        </is>
+      </c>
+      <c r="G131" s="4" t="n"/>
+      <c r="H131" s="4" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I131" s="4" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-speeches/06-24-wmes-2026-speech-stuart-fox-iata-director-flight-operations/</t>
+        </is>
+      </c>
+      <c r="J131" s="4" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B132" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C132" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D132" s="4" t="inlineStr">
+        <is>
+          <t>광양항 세풍항만배후단지 입주기업 모집</t>
+        </is>
+      </c>
+      <c r="E132" s="4" t="inlineStr">
+        <is>
+          <t>여수광양항만공사가 2차전지 기회발전특구로 지정된 광양항 세풍항만배후단지 입주기업을 모집하며, 인근에 2차전지 기업들이 위치하여 원료 조달 및 생산 연계에 유리하다.</t>
+        </is>
+      </c>
+      <c r="F132" s="4" t="inlineStr">
+        <is>
+          <t>국내 특정 항만 배후단지 입주기업 모집 소식으로, 현재 우리 회사의 물류 운영에 직접적인 영향은 없으나, 향후 국내 생산 및 물류 거점 확장 시 참고할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G132" s="4" t="n"/>
+      <c r="H132" s="4" t="inlineStr">
+        <is>
+          <t>ksg</t>
+        </is>
+      </c>
+      <c r="I132" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksg.co.kr/news/main_newsView.jsp?pNum=147484</t>
+        </is>
+      </c>
+      <c r="J132" s="4" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B133" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C133" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D133" s="4" t="inlineStr">
+        <is>
+          <t>HMM, 10억달러 뉴캐슬막스급 8척·VLGC 2척 발주</t>
+        </is>
+      </c>
+      <c r="E133" s="4" t="inlineStr">
+        <is>
+          <t>HMM이 총 10억 8,300만 달러 규모의 벌크선 8척과 가스운반선 2척을 발주하며 사업 포트폴리오 다각화 및 선단 경쟁력 강화를 추진한다.</t>
+        </is>
+      </c>
+      <c r="F133" s="4" t="inlineStr">
+        <is>
+          <t>HMM의 벌크선 및 가스운반선 발주 소식으로, 우리 회사의 주력 운송 수단인 컨테이너 운송과는 직접적인 관련이 낮다.</t>
+        </is>
+      </c>
+      <c r="G133" s="4" t="n"/>
+      <c r="H133" s="4" t="inlineStr">
+        <is>
+          <t>oceanpress</t>
+        </is>
+      </c>
+      <c r="I133" s="4" t="inlineStr">
+        <is>
+          <t>https://www.oceanpress.co.kr/news/article.html?no=30435</t>
+        </is>
+      </c>
+      <c r="J133" s="4" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B134" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C134" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D134" s="4" t="inlineStr">
+        <is>
+          <t>Decoding Gemini’s Mediterranean Surge</t>
+        </is>
+      </c>
+      <c r="E134" s="4" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence 분석에 따르면 제미니 협력(Gemini Cooperation)이 동서 컨테이너 선박 배치를 재조정하며 지중해 지역에서 시장 점유율을 확대하고 있음을 보여준다.</t>
+        </is>
+      </c>
+      <c r="F134" s="4" t="inlineStr">
+        <is>
+          <t>특정 선사 동맹의 선박 배치 전략 변화에 대한 내용으로, 우리 회사의 주력 운송 항로에 직접적인 영향이 크지 않다.</t>
+        </is>
+      </c>
+      <c r="G134" s="4" t="n"/>
+      <c r="H134" s="4" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I134" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/392-decoding-gemini-s-mediterranean-surge</t>
+        </is>
+      </c>
+      <c r="J134" s="4" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B135" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C135" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D135" s="4" t="inlineStr">
+        <is>
+          <t>"수도권에 땅·전력·용수 없다"…후공정 예상 깨고 생산라인 배치</t>
+        </is>
+      </c>
+      <c r="E135" s="4" t="inlineStr">
+        <is>
+          <t>삼성전자와 SK하이닉스가 수도권의 땅, 전력, 용수 부족 문제로 호남에 반도체 클러스터를 추진하며 생산라인 배치 전략에 변화를 주고 있다.</t>
+        </is>
+      </c>
+      <c r="F135" s="4" t="inlineStr">
+        <is>
+          <t>반도체 산업의 장기적인 생산기지 배치 전략 변화로, 당사 물류 운영에 직접적인 영향은 없으나 산업 전반의 인프라 동향으로 참고할 만하다.</t>
+        </is>
+      </c>
+      <c r="G135" s="4" t="n"/>
+      <c r="H135" s="4" t="inlineStr">
+        <is>
+          <t>이데일리</t>
+        </is>
+      </c>
+      <c r="I135" s="4" t="inlineStr">
+        <is>
+          <t>https://edaily.co.kr/News/Read?mediaCodeNo=257&amp;newsId=05205366645485000</t>
+        </is>
+      </c>
+      <c r="J135" s="4" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B136" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C136" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D136" s="4" t="inlineStr">
+        <is>
+          <t>한국세정신문</t>
+        </is>
+      </c>
+      <c r="E136" s="4" t="inlineStr">
+        <is>
+          <t>정부가 민생 물가 안정을 최우선 과제로 삼고 재정, 세제, 금융 등 가용한 수단을 총동원하여 물가 안정과 서민 부담 경감에 총력을 기울일 것이라고 밝혔다.</t>
+        </is>
+      </c>
+      <c r="F136" s="4" t="inlineStr">
+        <is>
+          <t>정부의 전반적인 물가 안정 정책 방향을 제시하는 것으로, 물류비에 간접적인 영향을 줄 수 있으나 당장 구체적인 변화는 없어 참고 수준이다.</t>
+        </is>
+      </c>
+      <c r="G136" s="4" t="n"/>
+      <c r="H136" s="4" t="inlineStr">
+        <is>
+          <t>한국세정신문</t>
+        </is>
+      </c>
+      <c r="I136" s="4" t="inlineStr">
+        <is>
+          <t>https://taxtimes.co.kr/news/article.html?no=275682</t>
+        </is>
+      </c>
+      <c r="J136" s="4" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B137" s="4" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C137" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D137" s="4" t="inlineStr">
+        <is>
+          <t>반도체도 ‘필수공익사업’ 지정 추진… 파업 시 국가경제 보호장치 마련되나</t>
+        </is>
+      </c>
+      <c r="E137" s="4" t="inlineStr">
+        <is>
+          <t>반도체 산업을 필수공익사업으로 지정하여 파업 시에도 최소한의 생산 및 설비 운영을 유지하도록 하는 법안이 추진 중이다. 이는 국가 경제 보호를 위한 조치로, 핵심 산업의 공급망 안정화에 기여할 수 있다.</t>
+        </is>
+      </c>
+      <c r="F137" s="4" t="inlineStr">
+        <is>
+          <t>현재 배터리/전자부품 산업에 직접적인 필수공익사업 지정 논의는 없으며, 반도체 산업에 대한 조치이므로 당사 물류 운영에 즉각적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G137" s="4" t="n"/>
+      <c r="H137" s="4" t="inlineStr">
+        <is>
+          <t>에너지데일리</t>
+        </is>
+      </c>
+      <c r="I137" s="4" t="inlineStr">
+        <is>
+          <t>https://energydaily.co.kr/news/articleView.html?idxno=200745</t>
+        </is>
+      </c>
+      <c r="J137" s="4" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B138" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C138" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D138" s="4" t="inlineStr">
+        <is>
+          <t>공급망 꽉 쥔 삼성물산, 친환경 ‘에너지 운영사’로 진화하는 게임체인저</t>
+        </is>
+      </c>
+      <c r="E138" s="4" t="inlineStr">
+        <is>
+          <t>삼성물산이 글로벌 통상 환경의 불확실성 속에서 단순 무역 중개를 넘어 공급망 자체를 최적화하고 친환경 에너지 운영사로 진화하며 역량을 강화하고 있다.</t>
+        </is>
+      </c>
+      <c r="F138" s="4" t="inlineStr">
+        <is>
+          <t>특정 기업의 공급망 전략 변화에 대한 기사로, 당사의 물류 운영이나 생산 계획에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G138" s="4" t="n"/>
+      <c r="H138" s="4" t="inlineStr">
+        <is>
+          <t>아시아투데이</t>
+        </is>
+      </c>
+      <c r="I138" s="4" t="inlineStr">
+        <is>
+          <t>https://www.asiatoday.co.kr/kn/view.php?key=20260624010008530</t>
+        </is>
+      </c>
+      <c r="J138" s="4" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B139" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C139" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D139" s="4" t="inlineStr">
+        <is>
+          <t>CJ대한통운, 세계은행그룹과 개발도상국 공급망 혁신 방안 논의</t>
+        </is>
+      </c>
+      <c r="E139" s="4" t="inlineStr">
+        <is>
+          <t>CJ대한통운이 세계은행그룹과 개발도상국의 공급망 경쟁력 강화 및 물류 연결성 향상을 위한 선진 물류 모델을 논의했다.</t>
+        </is>
+      </c>
+      <c r="F139" s="4" t="inlineStr">
+        <is>
+          <t>특정 물류 기업의 대외 협력 소식으로, 당사의 물류 운영이나 생산 계획에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G139" s="4" t="n"/>
+      <c r="H139" s="4" t="inlineStr">
+        <is>
+          <t>CJ 뉴스룸</t>
+        </is>
+      </c>
+      <c r="I139" s="4" t="inlineStr">
+        <is>
+          <t>https://cjnews.cj.net/cj%EB%8C%80%ED%95%9C%ED%86%B5%EC%9A%B4-%EC%84%B8%EA%B3%84%EC%9D%80%ED%96%89%EA%B7%B8%EB%A3%B9%EA%B3%BC-%EA%B0%9C%EB%B0%9C%EB%8F%84%EC%83%81%EA%B5%AD-%EA%B3%B5%EA%B8%89%EB%A7%9D-%ED%98%81%EC%8B%A0</t>
+        </is>
+      </c>
+      <c r="J139" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
@@ -5908,7 +7260,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6529,6 +7881,76 @@
       </c>
       <c r="I17" s="6" t="inlineStr"/>
     </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>RSK-017</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>美 세관, 단속 대폭 강화…수입업자·중개인 '충격'</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr"/>
+      <c r="G18" s="6" t="inlineStr"/>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>미국 수출 통관 절차 및 필요 서류 재검토, 현지 파트너와 협력하여 강화된 규제 준수 방안 마련, 잠재적 지연에 대비한 재고 및 운송 계획 조정</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>RSK-018</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>中, 핵심광물 대일 수출 0…日기업들, 외교적 해결 SOS | 한국경제</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr"/>
+      <c r="G19" s="6" t="inlineStr"/>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>중국산 핵심광물 의존도를 재평가하고, 대체 공급처 발굴 및 재고 확보 방안을 즉시 검토하며, 공급망 다변화 전략을 수립한다.</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
📰 뉴스 데이터 2026-06-26_09:13
</commit_message>
<xml_diff>
--- a/data/SCM_물류_브리핑.xlsx
+++ b/data/SCM_물류_브리핑.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J139"/>
+  <dimension ref="A1:J169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7046,6 +7046,1406 @@
       </c>
       <c r="J139" s="4" t="inlineStr"/>
     </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C140" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D140" s="2" t="inlineStr">
+        <is>
+          <t>美 세관, 단속 대폭 강화…수입업자·중개인 '충격'</t>
+        </is>
+      </c>
+      <c r="E140" s="2" t="inlineStr">
+        <is>
+          <t>미국 정부가 수입업자 자격, 공시 의무, 전자상거래 통관 절차 등 세관 단속을 대폭 강화하여 수입업자와 세관 중개인의 규제 부담이 커질 것으로 예상된다.</t>
+        </is>
+      </c>
+      <c r="F140" s="2" t="inlineStr">
+        <is>
+          <t>미국으로의 배터리/전자부품 수출 시 통관 절차의 복잡성 증가 및 리스크 상승으로 인해 즉각적인 대응이 필요할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G140" s="2" t="inlineStr">
+        <is>
+          <t>미국 수출 관련 통관 절차 및 규제 변화에 대한 상세 검토, 내부 프로세스 점검 및 필요 시 외부 전문가 자문.</t>
+        </is>
+      </c>
+      <c r="H140" s="2" t="inlineStr">
+        <is>
+          <t>kita</t>
+        </is>
+      </c>
+      <c r="I140" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kita.net/shippers/board/newsView.do?morgueCode=2&amp;dataCls=A&amp;dataSeq=2525</t>
+        </is>
+      </c>
+      <c r="J140" s="2" t="inlineStr">
+        <is>
+          <t>RSK-019</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B141" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C141" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D141" s="2" t="inlineStr">
+        <is>
+          <t>선박 호르무즈 탈출 시작됐지만…운임은 요지부동 "3분기 지나야 안정"</t>
+        </is>
+      </c>
+      <c r="E141" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 통항이 재개되고 있으나, 위험 해역 보험료, 선박 대기 비용, 운항 지연 등으로 인해 해상 운임은 여전히 높은 수준을 유지하며 3분기 이후에나 안정될 것으로 전망됩니다.</t>
+        </is>
+      </c>
+      <c r="F141" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 상황 개선에도 불구하고 운임이 안정되지 않고 3분기 이후에나 안정될 것이라는 전망은 우리 물류 비용 및 계획에 직접적인 영향을 미치며, 위험 해역 보험료, 선박 대기 비용, 운항 지연 등이 운임에 반영되고 있기 때문입니다.</t>
+        </is>
+      </c>
+      <c r="G141" s="2" t="inlineStr">
+        <is>
+          <t>해상 운송 비용 상승에 대비하여 예산 재검토 및 대체 운송 방안(항공 등) 검토, 선사와의 운임 협상 시 해당 요인 반영, 3분기 이후 시장 동향 면밀히 주시.</t>
+        </is>
+      </c>
+      <c r="H141" s="2" t="inlineStr">
+        <is>
+          <t>파이낸셜뉴스</t>
+        </is>
+      </c>
+      <c r="I141" s="2" t="inlineStr">
+        <is>
+          <t>https://fnnews.com/news/202606260531107942</t>
+        </is>
+      </c>
+      <c r="J141" s="2" t="inlineStr">
+        <is>
+          <t>RSK-020</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D142" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈서 화물선 피격 신고…IMO "철수작전 일시 중단"(종합)</t>
+        </is>
+      </c>
+      <c r="E142" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협에서 화물선 피격 신고가 접수되어 IMO가 철수 작전을 일시 중단했으며, 이는 해당 해협을 지나는 선박의 안전에 대한 우려를 높이고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F142" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협은 주요 해상 운송로이며, 화물선 피격 및 IMO의 작전 중단은 중동발 원자재 및 부품 수급에 직접적인 운송 지연 및 비용 상승을 초래할 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G142" s="2" t="inlineStr">
+        <is>
+          <t>중동 항로를 이용하는 선박의 운항 상황을 즉시 확인하고, 대체 항로 또는 운송 수단 검토, 재고 수준 점검 및 비상 계획을 수립해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H142" s="2" t="inlineStr">
+        <is>
+          <t>파이낸셜뉴스</t>
+        </is>
+      </c>
+      <c r="I142" s="2" t="inlineStr">
+        <is>
+          <t>https://fnnews.com/news/202606260426268388</t>
+        </is>
+      </c>
+      <c r="J142" s="2" t="inlineStr">
+        <is>
+          <t>RSK-021</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B143" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C143" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D143" s="3" t="inlineStr">
+        <is>
+          <t>CPSC Mandatory eFiling Takes Effect July 8; TPEB Rates Surge ~10% as Peak Season Demand Outpaces Capacity</t>
+        </is>
+      </c>
+      <c r="E143" s="3" t="inlineStr">
+        <is>
+          <t>미국 CPSC의 의무 전자신고가 7월 8일 발효되고, CBP는 강제 노동 관련 통합 지침을 발표했으며, 성수기 수요로 인해 TPEB 운임이 약 10% 급등했다.</t>
+        </is>
+      </c>
+      <c r="F143" s="3" t="inlineStr">
+        <is>
+          <t>CPSC 전자신고 의무화는 통관 절차에 영향을 줄 수 있고, CBP의 강제 노동 지침 강화는 공급망 실사에 대한 부담을 높이며, TPEB 운임 급등은 물류비 상승 압박을 가한다.</t>
+        </is>
+      </c>
+      <c r="G143" s="3" t="inlineStr">
+        <is>
+          <t>CPSC 전자신고 의무화에 대한 내부 절차 확인, 강제 노동 관련 공급망 실사 강화 방안 검토, TPEB 운임 추이 지속 모니터링.</t>
+        </is>
+      </c>
+      <c r="H143" s="3" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I143" s="3" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/june-18-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J143" s="3" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B144" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C144" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D144" s="3" t="inlineStr">
+        <is>
+          <t>DOJ Appeals CIT's IEEPA Refund Injunction as CAPE Phase 2 Targets June 29; TPEB Rates Surge 30% Into Peak</t>
+        </is>
+      </c>
+      <c r="E144" s="3" t="inlineStr">
+        <is>
+          <t>미국 법무부가 IEEPA 환급 금지 명령에 항소하고 CAPE 2단계가 6월 29일 시행될 예정이며, 성수기 진입으로 TPEB 운임이 30% 급등했다.</t>
+        </is>
+      </c>
+      <c r="F144" s="3" t="inlineStr">
+        <is>
+          <t>IEEPA 환급 관련 법적 분쟁과 CAPE 시스템 변화는 관세 및 통관 절차에 불확실성을 가중시키고, TPEB 운임의 급격한 상승은 물류비 부담을 크게 증가시킨다.</t>
+        </is>
+      </c>
+      <c r="G144" s="3" t="inlineStr">
+        <is>
+          <t>IEEPA 환급 관련 법적 진행 상황 주시, TPEB 운임 상승에 대한 운송 계획 및 예산 재검토.</t>
+        </is>
+      </c>
+      <c r="H144" s="3" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I144" s="3" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/june-11-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J144" s="3" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B145" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C145" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D145" s="3" t="inlineStr">
+        <is>
+          <t>Section 232 Duties Reduced to 15% for Taiwanese Goods, Retroactive to May 1; China Air Rates Spike on Supply Contraction and Month-End Demand</t>
+        </is>
+      </c>
+      <c r="E145" s="3" t="inlineStr">
+        <is>
+          <t>대만산 자동차 부품 및 목재 제품에 대한 Section 232 관세가 15%로 인하되었으며, 공급 감소와 월말 수요로 인해 중국발 항공 운임이 급등했다.</t>
+        </is>
+      </c>
+      <c r="F145" s="3" t="inlineStr">
+        <is>
+          <t>대만산 제품 관세 인하는 우리 회사에 직접적인 영향은 없으나, 중국발 항공 운임 급등은 항공 운송을 사용하는 경우 물류비에 직접적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G145" s="3" t="inlineStr">
+        <is>
+          <t>중국발 항공 운송 계획 및 예산에 미칠 영향 검토, 대체 운송 방안 고려.</t>
+        </is>
+      </c>
+      <c r="H145" s="3" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I145" s="3" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/may-28-2026-cit-rejects-governments-stay-request/</t>
+        </is>
+      </c>
+      <c r="J145" s="3" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B146" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C146" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D146" s="3" t="inlineStr">
+        <is>
+          <t>WMES 2026 Speech - Stuart Fox, IATA's Director Flight and Operations</t>
+        </is>
+      </c>
+      <c r="E146" s="3" t="inlineStr">
+        <is>
+          <t>IATA 연설에서 항공기 인도 지연, 엔진 문제, 예비 부품 확보 어려움, 수리 시간 지연 등 항공사들이 직면한 공급망 현실이 강조되었다.</t>
+        </is>
+      </c>
+      <c r="F146" s="3" t="inlineStr">
+        <is>
+          <t>항공기 및 부품 공급망의 지속적인 문제는 항공 화물 운송 능력에 부정적인 영향을 미칠 수 있으므로, 관련 동향을 지속적으로 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G146" s="3" t="inlineStr">
+        <is>
+          <t>항공 화물 운송 시장의 공급 능력 변화 추이 모니터링.</t>
+        </is>
+      </c>
+      <c r="H146" s="3" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I146" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-speeches/06-24-wmes-2026-speech-stuart-fox-iata-director-flight-operations/</t>
+        </is>
+      </c>
+      <c r="J146" s="3" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B147" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C147" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D147" s="3" t="inlineStr">
+        <is>
+          <t>[2026.6.25.] 중동 전쟁 관련 유가 및 물류 동향</t>
+        </is>
+      </c>
+      <c r="E147" s="3" t="inlineStr">
+        <is>
+          <t>중동 전쟁 관련 유가 및 물류 동향에 대한 정보로, 유가 변동이 해상 및 항공 운임에 직접적인 영향을 미쳐 물류비 상승으로 이어질 수 있다.</t>
+        </is>
+      </c>
+      <c r="F147" s="3" t="inlineStr">
+        <is>
+          <t>중동 전쟁으로 인한 유가 변동은 해상 및 항공 운임에 직접적인 영향을 미쳐 물류비 상승으로 이어질 수 있으므로 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G147" s="3" t="inlineStr">
+        <is>
+          <t>유가 및 해상/항공 운임 추이 지속 모니터링, 비상 계획 검토.</t>
+        </is>
+      </c>
+      <c r="H147" s="3" t="inlineStr">
+        <is>
+          <t>kotra</t>
+        </is>
+      </c>
+      <c r="I147" s="3" t="inlineStr">
+        <is>
+          <t>https://dream.kotra.or.kr/kotranews/cms/news/actionKotraBoardDetail.do?SITE_NO=3&amp;MENU_ID=70&amp;CONTENTS_NO=1&amp;pNttSn=242420</t>
+        </is>
+      </c>
+      <c r="J147" s="3" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B148" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C148" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D148" s="3" t="inlineStr">
+        <is>
+          <t>20260626 경제·물류 주요뉴스 (데일리스크랩)</t>
+        </is>
+      </c>
+      <c r="E148" s="3" t="inlineStr">
+        <is>
+          <t>미국과 이란의 합의 이후 호르무즈 해협 통항량이 급증하며 유조선 운항이 빠르게 회복되고 있으나, 급격히 유입될 물량이 글로벌 컨테이너 공급망에 새로운 지연을 만들 수 있어 비용과 운임이 쉽게 내려가지 않을 것이라는 분석이 나왔습니다.</t>
+        </is>
+      </c>
+      <c r="F148" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 재개방은 긍정적이나, 급격한 물량 유입으로 인한 새로운 운송 지연 및 유가/운임 상승 가능성이 언급되어 지속적인 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G148" s="3" t="n"/>
+      <c r="H148" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I148" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260626-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J148" s="3" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B149" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C149" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D149" s="3" t="inlineStr">
+        <is>
+          <t>Tracking True Vessel Delay (PRESS ROOM)</t>
+        </is>
+      </c>
+      <c r="E149" s="3" t="inlineStr">
+        <is>
+          <t>선사들이 선박 스케줄 지연을 관리하기 위해 운송 시간을 늘리는 '스케줄 버퍼링'에 점점 더 의존하고 있으며, 이는 실제 운송 리드타임에 영향을 미칠 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="F149" s="3" t="inlineStr">
+        <is>
+          <t>선사들이 운송 지연을 관리하기 위해 스케줄 버퍼를 늘리는 추세로, 이는 운송 리드타임에 영향을 줄 수 있어 지속적인 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G149" s="3" t="n"/>
+      <c r="H149" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I149" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/394-tracking-true-vessel-delay</t>
+        </is>
+      </c>
+      <c r="J149" s="3" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B150" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C150" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D150" s="3" t="inlineStr">
+        <is>
+          <t>20260622 경제·물류 주요뉴스 (데일리스크랩)</t>
+        </is>
+      </c>
+      <c r="E150" s="3" t="inlineStr">
+        <is>
+          <t>HMM은 운임 하락, 공급 증가, 관세 변수, 중동발 비용 부담 등 다양한 요인 속에서 2030 전략의 실행력을 시험받고 있으며, 이는 해운 시장 전반의 어려움을 반영합니다.</t>
+        </is>
+      </c>
+      <c r="F150" s="3" t="inlineStr">
+        <is>
+          <t>HMM의 운임 하락, 공급 증가, 관세 변수, 중동발 비용 부담 등은 해운 시장 전반의 어려움을 반영하며, 이는 우리 물류 비용에 영향을 줄 수 있어 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G150" s="3" t="n"/>
+      <c r="H150" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I150" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260622-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J150" s="3" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B151" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C151" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D151" s="3" t="inlineStr">
+        <is>
+          <t>Turning supply chain volatility into regional advantage</t>
+        </is>
+      </c>
+      <c r="E151" s="3" t="inlineStr">
+        <is>
+          <t>홍해 지역의 지속적인 운송 차질과 수에즈 운하 회피는 물류 네트워크, 항만, 세관 당국 간의 긴밀한 연관성을 강조하며, 공급망 탄력성을 위해 인프라, 정책 조정, 제도적 준비가 중요함을 보여준다.</t>
+        </is>
+      </c>
+      <c r="F151" s="3" t="inlineStr">
+        <is>
+          <t>홍해 지역의 운송 차질은 해상 운송 경로와 운임에 영향을 미칠 수 있으며, 이는 배터리/전자부품 운송에도 간접적인 영향을 줄 수 있으므로 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G151" s="3" t="inlineStr">
+        <is>
+          <t>해상 운송 경로 및 운임 변동 추이 지속 모니터링, 비상 운송 경로 및 대체 운송 수단 검토.</t>
+        </is>
+      </c>
+      <c r="H151" s="3" t="inlineStr">
+        <is>
+          <t>Arab News</t>
+        </is>
+      </c>
+      <c r="I151" s="3" t="inlineStr">
+        <is>
+          <t>https://arabnews.com/node/2648593</t>
+        </is>
+      </c>
+      <c r="J151" s="3" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B152" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C152" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D152" s="3" t="inlineStr">
+        <is>
+          <t>서울 지하철 대용량 리튬배터리 반입 금지</t>
+        </is>
+      </c>
+      <c r="E152" s="3" t="inlineStr">
+        <is>
+          <t>서울교통공사가 7월 1일부터 160Wh를 초과하는 대용량 리튬배터리와 전동킥보드 등 배터리 구동 개인형 이동장치의 지하철 역사 반입을 금지하며, 이는 지하철 내 화재 위험을 줄이기 위한 안전 강화 조치이다.</t>
+        </is>
+      </c>
+      <c r="F152" s="3" t="inlineStr">
+        <is>
+          <t>지하철 내 대용량 리튬배터리 반입 제한은 배터리 제품의 개인 운송 방식에 영향을 미치며, 향후 다른 운송 수단이나 물류 채널에도 유사한 규제가 확대될 가능성이 있어 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G152" s="3" t="inlineStr">
+        <is>
+          <t>배터리 제품의 운송 및 보관 관련 국내외 규제 동향 지속 모니터링, 고객 안내 및 관련 부서(영업, 마케팅)와 협의하여 소비자 대상 정보 제공 방안 검토.</t>
+        </is>
+      </c>
+      <c r="H152" s="3" t="inlineStr">
+        <is>
+          <t>서울Pn</t>
+        </is>
+      </c>
+      <c r="I152" s="3" t="inlineStr">
+        <is>
+          <t>https://go.seoul.co.kr/news/newsView.php?id=20260626019001</t>
+        </is>
+      </c>
+      <c r="J152" s="3" t="inlineStr"/>
+    </row>
+    <row r="153">
+      <c r="A153" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B153" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C153" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D153" s="3" t="inlineStr">
+        <is>
+          <t>버려진 것에서 가치를 찾다…‘순환 경제’가 돈이 되는 시대</t>
+        </is>
+      </c>
+      <c r="E153" s="3" t="inlineStr">
+        <is>
+          <t>순환 경제 모델이 ESG 경영 강화 추세와 맞물려 각광받고 있으며, 자원 절약 및 재활용을 통한 지속 가능성을 추구합니다. 이는 배터리/전자부품 산업의 자원 관리 및 폐기물 처리 방식에 영향을 미칠 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="F153" s="3" t="inlineStr">
+        <is>
+          <t>순환 경제는 장기적으로 배터리 및 전자부품의 생산, 재활용, 폐기물 관리에 대한 규제 및 비즈니스 모델 변화를 가져올 수 있으므로 추이를 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G153" s="3" t="inlineStr">
+        <is>
+          <t>순환 경제 관련 국내외 정책 및 규제 동향을 지속적으로 파악하고, 배터리 재활용 및 폐기물 관리 전략에 미칠 영향을 분석해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H153" s="3" t="inlineStr">
+        <is>
+          <t>매일일보</t>
+        </is>
+      </c>
+      <c r="I153" s="3" t="inlineStr">
+        <is>
+          <t>https://m-i.kr/news/articleView.html?idxno=1383806</t>
+        </is>
+      </c>
+      <c r="J153" s="3" t="inlineStr"/>
+    </row>
+    <row r="154">
+      <c r="A154" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B154" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C154" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D154" s="3" t="inlineStr">
+        <is>
+          <t>정부, 자원안보 전면 강화…공급망 위기 대응 로드맵 본격 추진</t>
+        </is>
+      </c>
+      <c r="E154" s="3" t="inlineStr">
+        <is>
+          <t>정부가 미국-이란 전쟁 이후 드러난 에너지·자원 수급 취약점을 보완하고 핵심광물 및 소재·부품 공급망을 강화하기 위한 로드맵을 추진합니다.</t>
+        </is>
+      </c>
+      <c r="F154" s="3" t="inlineStr">
+        <is>
+          <t>정부의 자원안보 및 공급망 강화 정책은 배터리/전자부품 제조에 필요한 핵심 원자재 수급에 장기적인 영향을 미칠 수 있으므로 관련 정책 변화를 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G154" s="3" t="inlineStr">
+        <is>
+          <t>정부의 공급망 로드맵 세부 내용을 주시하고, 핵심 원자재의 안정적 확보를 위한 공급망 다변화 및 국내외 협력 방안을 검토해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H154" s="3" t="inlineStr">
+        <is>
+          <t>경북일보</t>
+        </is>
+      </c>
+      <c r="I154" s="3" t="inlineStr">
+        <is>
+          <t>https://kyongbuk.co.kr/news/articleView.html?idxno=4076675</t>
+        </is>
+      </c>
+      <c r="J154" s="3" t="inlineStr"/>
+    </row>
+    <row r="155">
+      <c r="A155" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B155" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C155" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D155" s="3" t="inlineStr">
+        <is>
+          <t>미-이란 MOU 이후 호르무즈 해협 통해 원유 3500만배럴 빠져나와</t>
+        </is>
+      </c>
+      <c r="E155" s="3" t="inlineStr">
+        <is>
+          <t>미국과 이란의 합의로 호르무즈 해협의 해상 항로가 개방되어 페르시아만에 묶여 있던 유조선들이 통과하기 시작했으며, 이는 중동 지역의 긴장 완화를 시사합니다.</t>
+        </is>
+      </c>
+      <c r="F155" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협의 긴장 완화는 국제 유가 안정화 및 중동발 물류 리스크 감소에 긍정적인 영향을 줄 수 있으나, 상황의 지속적인 안정 여부를 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G155" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협의 안정화 추이를 지속적으로 관찰하고, 국제 유가 및 해상 운임 변동 가능성을 예측하여 물류 비용 계획에 반영해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H155" s="3" t="inlineStr">
+        <is>
+          <t>파이낸셜뉴스</t>
+        </is>
+      </c>
+      <c r="I155" s="3" t="inlineStr">
+        <is>
+          <t>https://fnnews.com/news/202606250748267610</t>
+        </is>
+      </c>
+      <c r="J155" s="3" t="inlineStr"/>
+    </row>
+    <row r="156">
+      <c r="A156" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B156" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C156" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D156" s="3" t="inlineStr">
+        <is>
+          <t>"급여 반납합니다" 파라타항공 비상경영</t>
+        </is>
+      </c>
+      <c r="E156" s="3" t="inlineStr">
+        <is>
+          <t>고유가 후폭풍으로 파라타항공이 비상경영에 돌입하며 급여 반납을 결정했는데, 이는 항공 운송 시장의 비용 압박을 시사합니다.</t>
+        </is>
+      </c>
+      <c r="F156" s="3" t="inlineStr">
+        <is>
+          <t>고유가로 인한 항공사의 비상경영은 항공 운송 비용 상승 압박 및 잠재적인 항공 화물 운송 서비스 불안정으로 이어질 수 있으므로 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G156" s="3" t="inlineStr">
+        <is>
+          <t>항공 운송 시장의 운임 및 서비스 변동 가능성을 주시하고, 필요시 대체 운송 수단 또는 항공사와의 계약 조건 재검토를 고려해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H156" s="3" t="inlineStr">
+        <is>
+          <t>매일경제</t>
+        </is>
+      </c>
+      <c r="I156" s="3" t="inlineStr">
+        <is>
+          <t>https://mk.co.kr/news/business/12083301</t>
+        </is>
+      </c>
+      <c r="J156" s="3" t="inlineStr"/>
+    </row>
+    <row r="157">
+      <c r="A157" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B157" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C157" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D157" s="3" t="inlineStr">
+        <is>
+          <t>국내 기름값 2000원선 아래로?…7차 석유 최고가격 하향 전망</t>
+        </is>
+      </c>
+      <c r="E157" s="3" t="inlineStr">
+        <is>
+          <t>미국과 이란 협상 진전으로 국제유가가 중동 전쟁 이전 수준으로 낮아지면서 정부가 국내 석유 최고가격을 하향 조정하는 방안을 검토 중입니다.</t>
+        </is>
+      </c>
+      <c r="F157" s="3" t="inlineStr">
+        <is>
+          <t>국제유가 하락 및 국내 기름값 인하 전망은 육상 운송 비용 감소에 긍정적인 영향을 미칠 수 있으나, 유가 변동성을 지속적으로 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G157" s="3" t="inlineStr">
+        <is>
+          <t>유가 하락 추세를 주시하고, 국내외 운송 계약 시 유가 연동 조항을 검토하거나 운송 비용 절감 방안을 모색해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H157" s="3" t="inlineStr">
+        <is>
+          <t>헤럴드경제</t>
+        </is>
+      </c>
+      <c r="I157" s="3" t="inlineStr">
+        <is>
+          <t>https://biz.heraldcorp.com/article/10788726</t>
+        </is>
+      </c>
+      <c r="J157" s="3" t="inlineStr"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B158" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C158" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D158" s="3" t="inlineStr">
+        <is>
+          <t>전쟁 이전으로 돌아간 국제유가…석유 최고가격 하향 전망</t>
+        </is>
+      </c>
+      <c r="E158" s="3" t="inlineStr">
+        <is>
+          <t>국제유가가 중동 전쟁 이전 수준으로 하락하여 정부가 서민 경제 부담 완화를 위해 석유 최고가격 하향 조정을 검토 중이다.</t>
+        </is>
+      </c>
+      <c r="F158" s="3" t="inlineStr">
+        <is>
+          <t>국제유가 하락은 해상/항공 운임의 유류할증료 인하로 이어져 물류비용 절감에 긍정적인 영향을 미칠 수 있으므로 추이를 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G158" s="3" t="inlineStr">
+        <is>
+          <t>유류할증료 변동 추이 및 운송 계약 조건 검토, 잠재적 비용 절감 기회 분석.</t>
+        </is>
+      </c>
+      <c r="H158" s="3" t="inlineStr">
+        <is>
+          <t>세계일보</t>
+        </is>
+      </c>
+      <c r="I158" s="3" t="inlineStr">
+        <is>
+          <t>https://segye.com/newsView/20260626502219</t>
+        </is>
+      </c>
+      <c r="J158" s="3" t="inlineStr"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B159" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C159" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D159" s="4" t="inlineStr">
+        <is>
+          <t>터키카고, 車전문 항공운송상품 출시</t>
+        </is>
+      </c>
+      <c r="E159" s="4" t="inlineStr">
+        <is>
+          <t>터키항공 화물부문이 자동차 산업을 위한 긴급 운송 상품인 'TK 오토'를 출시하여 자동차 부품 및 완성차 운송 서비스를 제공한다.</t>
+        </is>
+      </c>
+      <c r="F159" s="4" t="inlineStr">
+        <is>
+          <t>우리 회사의 배터리/전자부품 운송과는 직접적인 관련이 없는 자동차 산업 특화 서비스이다.</t>
+        </is>
+      </c>
+      <c r="G159" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H159" s="4" t="inlineStr">
+        <is>
+          <t>cargonews</t>
+        </is>
+      </c>
+      <c r="I159" s="4" t="inlineStr">
+        <is>
+          <t>https://www.cargonews.co.kr/news/articleView.html?idxno=60411</t>
+        </is>
+      </c>
+      <c r="J159" s="4" t="inlineStr"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B160" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C160" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D160" s="4" t="inlineStr">
+        <is>
+          <t>Transpacific: Ripe for new non-alliance services (PRESS ROOM)</t>
+        </is>
+      </c>
+      <c r="E160" s="4" t="inlineStr">
+        <is>
+          <t>아시아-북미 서안 항로의 컨테이너 스팟 운임과 비동맹 선사의 선박 용량 점유율 간의 관계를 분석하며, 새로운 비동맹 서비스의 출현 가능성을 시사합니다.</t>
+        </is>
+      </c>
+      <c r="F160" s="4" t="inlineStr">
+        <is>
+          <t>아시아-북미 서안 항로의 비동맹 선사 서비스 확대 가능성에 대한 분석으로, 당장 우리 물류 운영에 직접적인 영향을 미치지는 않습니다.</t>
+        </is>
+      </c>
+      <c r="G160" s="4" t="n"/>
+      <c r="H160" s="4" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I160" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/393-transpacific-ripe-for-new-non-alliance-services</t>
+        </is>
+      </c>
+      <c r="J160" s="4" t="inlineStr"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B161" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C161" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D161" s="4" t="inlineStr">
+        <is>
+          <t>Decoding Gemini’s Mediterranean Surge (PRESS ROOM)</t>
+        </is>
+      </c>
+      <c r="E161" s="4" t="inlineStr">
+        <is>
+          <t>Gemini Cooperation이 동서 컨테이너 선박 배치를 재조정하며 전반적인 시장 점유율 손실에도 불구하고 지중해 지역에 대한 배치를 크게 늘리고 있음을 분석합니다.</t>
+        </is>
+      </c>
+      <c r="F161" s="4" t="inlineStr">
+        <is>
+          <t>특정 선사 동맹의 선대 재배치 전략에 대한 분석으로, 우리 물류 운영에 직접적인 영향을 미치지 않습니다.</t>
+        </is>
+      </c>
+      <c r="G161" s="4" t="n"/>
+      <c r="H161" s="4" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I161" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/392-decoding-gemini-s-mediterranean-surge</t>
+        </is>
+      </c>
+      <c r="J161" s="4" t="inlineStr"/>
+    </row>
+    <row r="162">
+      <c r="A162" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B162" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C162" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D162" s="4" t="inlineStr">
+        <is>
+          <t>2026-Q1: NAEC Ports Consolidate Market Share (PRESS ROOM)</t>
+        </is>
+      </c>
+      <c r="E162" s="4" t="inlineStr">
+        <is>
+          <t>2026년 1분기 북미 동안(NAEC) 항만의 컨테이너 물동량이 전년 대비 감소했음에도 불구하고 시장 점유율을 공고히 했다는 분석입니다.</t>
+        </is>
+      </c>
+      <c r="F162" s="4" t="inlineStr">
+        <is>
+          <t>북미 동안 항만의 2026년 1분기 컨테이너 물동량 분석으로, 현재 우리 물류 운영에 직접적인 영향을 주지 않습니다.</t>
+        </is>
+      </c>
+      <c r="G162" s="4" t="n"/>
+      <c r="H162" s="4" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I162" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/391-2026-q1-naec-ports-consolidate-market-share</t>
+        </is>
+      </c>
+      <c r="J162" s="4" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B163" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C163" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D163" s="4" t="inlineStr">
+        <is>
+          <t>Global Schedule Reliability for April 2026 the Highest of the Year (PRESS ROOM)</t>
+        </is>
+      </c>
+      <c r="E163" s="4" t="inlineStr">
+        <is>
+          <t>2026년 4월 글로벌 선박 스케줄 정시성이 연중 최고치를 기록했다는 Sea-Intelligence의 보고서입니다.</t>
+        </is>
+      </c>
+      <c r="F163" s="4" t="inlineStr">
+        <is>
+          <t>2026년 4월 글로벌 선박 스케줄 정시성이 연중 최고치를 기록했다는 과거 데이터로, 현재 물류 운영에 직접적인 영향을 주지 않습니다.</t>
+        </is>
+      </c>
+      <c r="G163" s="4" t="n"/>
+      <c r="H163" s="4" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I163" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/390-global-schedule-reliability-for-april-2026-the-highest-of-the-year</t>
+        </is>
+      </c>
+      <c r="J163" s="4" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B164" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C164" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D164" s="4" t="inlineStr">
+        <is>
+          <t>일본 조선업계, LNG 운반선 건조 시장 재진입 계획... 건조 가능 시점은 2030년 이후 전망</t>
+        </is>
+      </c>
+      <c r="E164" s="4" t="inlineStr">
+        <is>
+          <t>일본 조선업계가 에너지 안보를 위해 LNG 운반선 건조 시장 재진입을 계획하고 있으나, 기존 수주 물량과 공급망 문제로 인해 2030년 이후에나 건조가 가능할 것으로 전망됩니다.</t>
+        </is>
+      </c>
+      <c r="F164" s="4" t="inlineStr">
+        <is>
+          <t>일본 조선업계의 LNG 운반선 시장 재진입 계획은 2030년 이후의 장기적인 이슈로, 우리 회사의 단기 물류 운영에 직접적인 영향은 없습니다.</t>
+        </is>
+      </c>
+      <c r="G164" s="4" t="n"/>
+      <c r="H164" s="4" t="inlineStr">
+        <is>
+          <t>shippingnewsnet</t>
+        </is>
+      </c>
+      <c r="I164" s="4" t="inlineStr">
+        <is>
+          <t>https://www.shippingnewsnet.com/news/articleView.html?idxno=70909</t>
+        </is>
+      </c>
+      <c r="J164" s="4" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B165" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C165" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D165" s="4" t="inlineStr">
+        <is>
+          <t>씨메스로보틱스 / ‘물류·제조 대형 수주 잇달아’ 피지컬 AI 기반 로봇 자동화 사업 가속</t>
+        </is>
+      </c>
+      <c r="E165" s="4" t="inlineStr">
+        <is>
+          <t>씨메스로보틱스가 물류 및 제조 현장에서 피지컬 AI 기반 로봇 자동화 대형 프로젝트를 연이어 수주하며 사업을 확대하고 있으며, 1분기 사상 최대 매출을 달성했습니다.</t>
+        </is>
+      </c>
+      <c r="F165" s="4" t="inlineStr">
+        <is>
+          <t>물류 자동화 및 로봇 기술 발전 동향에 대한 뉴스로, 우리 회사의 장기적인 물류 전략 수립 시 참고할 수 있으나 당장 직접적인 영향은 없습니다.</t>
+        </is>
+      </c>
+      <c r="G165" s="4" t="n"/>
+      <c r="H165" s="4" t="inlineStr">
+        <is>
+          <t>ulogistics</t>
+        </is>
+      </c>
+      <c r="I165" s="4" t="inlineStr">
+        <is>
+          <t>http://www.ulogistics.co.kr/test/board.php?board=all2&amp;command=body&amp;no=5202</t>
+        </is>
+      </c>
+      <c r="J165" s="4" t="inlineStr"/>
+    </row>
+    <row r="166">
+      <c r="A166" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B166" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C166" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D166" s="4" t="inlineStr">
+        <is>
+          <t>UK DBT creates Supply Chain Centre to battle logistics uncertainty</t>
+        </is>
+      </c>
+      <c r="E166" s="4" t="inlineStr">
+        <is>
+          <t>영국 정부가 물류 불확실성에 대응하기 위해 공급망 센터를 설립하고 행동 계획을 발표했으며, 이는 영국 물류를 지원하고 공급망 탄력성을 강화하기 위한 목적이다.</t>
+        </is>
+      </c>
+      <c r="F166" s="4" t="inlineStr">
+        <is>
+          <t>영국 정부의 공급망 강화 노력은 우리 기업의 직접적인 물류 운영에 당장 영향을 미치기보다는 전반적인 물류 환경 개선에 기여할 수 있는 참고 수준의 뉴스이다.</t>
+        </is>
+      </c>
+      <c r="G166" s="4" t="n"/>
+      <c r="H166" s="4" t="inlineStr">
+        <is>
+          <t>Logistics Manager</t>
+        </is>
+      </c>
+      <c r="I166" s="4" t="inlineStr">
+        <is>
+          <t>https://logisticsmanager.com/uk-dbt-creates-supply-chain-centre-to-battle-logistics-uncertainty</t>
+        </is>
+      </c>
+      <c r="J166" s="4" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B167" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C167" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D167" s="4" t="inlineStr">
+        <is>
+          <t>How autonomous systems are reshaping warehouse operations</t>
+        </is>
+      </c>
+      <c r="E167" s="4" t="inlineStr">
+        <is>
+          <t>자율 시스템이 창고 운영을 혁신하며, 자동화, AI, 실시간 운영 인텔리전스를 결합하여 공급망 혼란에 대응하고 지속 가능한 확장을 가능하게 한다.</t>
+        </is>
+      </c>
+      <c r="F167" s="4" t="inlineStr">
+        <is>
+          <t>창고 운영의 자율 시스템 도입은 장기적인 효율성 증대와 관련이 있으나, 우리 회사의 현재 물류 운영에 즉각적인 영향을 미치는 내용은 아니다.</t>
+        </is>
+      </c>
+      <c r="G167" s="4" t="n"/>
+      <c r="H167" s="4" t="inlineStr">
+        <is>
+          <t>TechRadar</t>
+        </is>
+      </c>
+      <c r="I167" s="4" t="inlineStr">
+        <is>
+          <t>https://techradar.com/pro/how-autonomous-systems-are-reshaping-warehouse-operations</t>
+        </is>
+      </c>
+      <c r="J167" s="4" t="inlineStr"/>
+    </row>
+    <row r="168">
+      <c r="A168" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B168" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C168" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D168" s="4" t="inlineStr">
+        <is>
+          <t>울산해경, 부산 대변 남동방 22해리 해상 상선과 어선 충돌 사고 발생 긴급 구조 중 (3보)</t>
+        </is>
+      </c>
+      <c r="E168" s="4" t="inlineStr">
+        <is>
+          <t>부산 대변 남동방 해상에서 상선과 어선 충돌 사고가 발생하여 해경이 긴급 구조 중이며, 이는 해당 해역의 해상 운송에 일시적인 영향을 줄 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="F168" s="4" t="inlineStr">
+        <is>
+          <t>국내 특정 해역에서의 소규모 해상 사고는 우리 회사의 글로벌 물류 운영에 직접적인 영향을 미치기보다는 국지적인 운송 지연 가능성만 있습니다.</t>
+        </is>
+      </c>
+      <c r="G168" s="4" t="n"/>
+      <c r="H168" s="4" t="inlineStr">
+        <is>
+          <t>정필</t>
+        </is>
+      </c>
+      <c r="I168" s="4" t="inlineStr">
+        <is>
+          <t>https://jeongpil.com/2575563</t>
+        </is>
+      </c>
+      <c r="J168" s="4" t="inlineStr"/>
+    </row>
+    <row r="169">
+      <c r="A169" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B169" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C169" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D169" s="4" t="inlineStr">
+        <is>
+          <t>CJ대한통운, 세계은행그룹과 개발도상국 공급망 혁신 방안 논의</t>
+        </is>
+      </c>
+      <c r="E169" s="4" t="inlineStr">
+        <is>
+          <t>CJ대한통운이 세계은행그룹과 개발도상국의 공급망 경쟁력 강화 및 물류 연결성 향상을 위한 선진 물류 모델을 논의했습니다.</t>
+        </is>
+      </c>
+      <c r="F169" s="4" t="inlineStr">
+        <is>
+          <t>개발도상국 공급망 혁신 논의는 장기적인 물류 트렌드에 대한 정보는 제공하지만, 우리 회사의 현재 물류 운영에 직접적인 영향을 미치지는 않습니다.</t>
+        </is>
+      </c>
+      <c r="G169" s="4" t="n"/>
+      <c r="H169" s="4" t="inlineStr">
+        <is>
+          <t>CJ 뉴스룸</t>
+        </is>
+      </c>
+      <c r="I169" s="4" t="inlineStr">
+        <is>
+          <t>https://cjnews.cj.net/cj%EB%8C%80%ED%95%9C%ED%86%B5%EC%9A%B4-%EC%84%B8%EA%B3%84%EC%9D%80%ED%96%89%EA%B7%B8%EB%A3%B9%EA%B3%BC-%EA%B0%9C%EB%B0%9C%EB%8F%84%EC%83%81%EA%B5%AD-%EA%B3%B5%EA%B8%89%EB%A7%9D-%ED%98%81%EC%8B%A0</t>
+        </is>
+      </c>
+      <c r="J169" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7058,7 +8458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7248,6 +8648,49 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>3121.69</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>+136 (+4.6%)</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>+881 (+39.3%)</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>3747</v>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>+398 (+11.9%)</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>+940 (+33.5%)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7260,7 +8703,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7951,6 +9394,111 @@
       </c>
       <c r="I19" s="6" t="inlineStr"/>
     </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>RSK-019</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>美 세관, 단속 대폭 강화…수입업자·중개인 '충격'</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr"/>
+      <c r="G20" s="6" t="inlineStr"/>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>미국 수출 관련 통관 절차 및 규제 변화에 대한 상세 검토, 내부 프로세스 점검 및 필요 시 외부 전문가 자문.</t>
+        </is>
+      </c>
+      <c r="I20" s="6" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>RSK-020</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>선박 호르무즈 탈출 시작됐지만…운임은 요지부동 "3분기 지나야 안정"</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr"/>
+      <c r="G21" s="6" t="inlineStr"/>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>해상 운송 비용 상승에 대비하여 예산 재검토 및 대체 운송 방안(항공 등) 검토, 선사와의 운임 협상 시 해당 요인 반영, 3분기 이후 시장 동향 면밀히 주시.</t>
+        </is>
+      </c>
+      <c r="I21" s="6" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>RSK-021</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈서 화물선 피격 신고…IMO "철수작전 일시 중단"(종합)</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr"/>
+      <c r="G22" s="6" t="inlineStr"/>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>중동 항로를 이용하는 선박의 운항 상황을 즉시 확인하고, 대체 항로 또는 운송 수단 검토, 재고 수준 점검 및 비상 계획을 수립해야 합니다.</t>
+        </is>
+      </c>
+      <c r="I22" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
📰 뉴스 데이터 2026-06-26_19:30
</commit_message>
<xml_diff>
--- a/data/SCM_물류_브리핑.xlsx
+++ b/data/SCM_물류_브리핑.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J169"/>
+  <dimension ref="A1:J195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8445,6 +8445,1230 @@
         </is>
       </c>
       <c r="J169" s="4" t="inlineStr"/>
+    </row>
+    <row r="170">
+      <c r="A170" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B170" s="2" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C170" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D170" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 통과 화물선 피격…이란 '지정 항로' 경고 현실화</t>
+        </is>
+      </c>
+      <c r="E170" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협에서 화물선이 피격되고 이란의 '지정 항로' 경고가 현실화됨에 따라 IMO가 선박 집단 이동 프로그램을 중단하는 등 해상 운송 안전에 대한 우려가 커지고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F170" s="2" t="inlineStr">
+        <is>
+          <t>주요 해상 운송로인 호르무즈 해협에서의 선박 피격은 즉각적인 운송 지연 및 안전 위험을 초래하며, 우리 기업의 중동발 원자재 수급 및 제품 운송에 직접적인 영향을 미칠 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G170" s="2" t="inlineStr">
+        <is>
+          <t>중동 항로를 이용하는 선박의 안전 운항 여부 및 대체 항로 가능성을 즉시 확인하고, 보험 및 비상 운송 계획을 점검해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H170" s="2" t="inlineStr">
+        <is>
+          <t>청년일보</t>
+        </is>
+      </c>
+      <c r="I170" s="2" t="inlineStr">
+        <is>
+          <t>https://youthdaily.co.kr/news/article.html?no=221697</t>
+        </is>
+      </c>
+      <c r="J170" s="2" t="inlineStr">
+        <is>
+          <t>RSK-022</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B171" s="2" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C171" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D171" s="2" t="inlineStr">
+        <is>
+          <t>🚢🚚 복합 운송 기반 근거리 아웃소싱 솔루션 🌍📜⚖️ 새로운 EU 법률이 모든 것을 바꿉니다 🔗❌🗓️ 2026년부터 선형 공급망이 쓸모없어지는 이유</t>
+        </is>
+      </c>
+      <c r="E171" s="2" t="inlineStr">
+        <is>
+          <t>새로운 EU 순환 경제법이 2026년부터 선형 공급망을 시대에 뒤떨어지게 만들고 순환 경제를 산업 규제로 전환하며, 복합 운송 기반 근거리 아웃소싱 솔루션과 역물류의 중요성을 강조한다.</t>
+        </is>
+      </c>
+      <c r="F171" s="2" t="inlineStr">
+        <is>
+          <t>2026년부터 시행될 EU 순환 경제법은 배터리 제조기업의 제품 설계, 생산, 물류(특히 역물류) 및 재활용 프로세스 전반에 걸쳐 근본적인 변화를 요구하며, 유럽 시장 진출 및 운영에 직접적인 영향을 미칠 것이다.</t>
+        </is>
+      </c>
+      <c r="G171" s="2" t="inlineStr">
+        <is>
+          <t>EU 순환 경제법 및 관련 배터리 규제(예: EU Battery Regulation) 상세 분석, 2026년까지 공급망 및 역물류 전략 재수립, 제품 설계 단계부터 순환 경제 원칙 반영 검토.</t>
+        </is>
+      </c>
+      <c r="H171" s="2" t="inlineStr">
+        <is>
+          <t>xpert.digital</t>
+        </is>
+      </c>
+      <c r="I171" s="2" t="inlineStr">
+        <is>
+          <t>https://xpert.digital/ko/%EB%B3%B5%ED%95%A9%EC%9A%B4%EC%86%A1-%EA%B7%BC%EA%B1%B0%EB%A6%AC%EC%A0%84-%EC%86%94%EB%A3%A8%EC%85%98</t>
+        </is>
+      </c>
+      <c r="J171" s="2" t="inlineStr">
+        <is>
+          <t>RSK-023</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B172" s="2" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C172" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D172" s="2" t="inlineStr">
+        <is>
+          <t>"이러다 중소기업 줄줄이 망한다"…한국 정부가 중국에 황급히 SOS 친 '진짜 이유'</t>
+        </is>
+      </c>
+      <c r="E172" s="2" t="inlineStr">
+        <is>
+          <t>중국이 휴대용 보조배터리와 리튬이온 배터리의 안전 규정을 갑자기 강화하여 한국 수출 기업들의 공급망에 비상이 걸렸습니다.</t>
+        </is>
+      </c>
+      <c r="F172" s="2" t="inlineStr">
+        <is>
+          <t>중국의 휴대용 보조배터리 및 리튬이온 배터리 안전 규정 강화는 우리 기업의 대중국 수출에 직접적인 물류 및 통관 지연을 초래할 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G172" s="2" t="inlineStr">
+        <is>
+          <t>대중국 수출 제품의 규정 준수 여부 즉시 확인 및 필요 시 인증 획득 절차 가속화, 대체 시장 또는 운송 경로 검토.</t>
+        </is>
+      </c>
+      <c r="H172" s="2" t="inlineStr">
+        <is>
+          <t>withnews.kr</t>
+        </is>
+      </c>
+      <c r="I172" s="2" t="inlineStr">
+        <is>
+          <t>https://car.withnews.kr/economy/china-battery-technical-barrier</t>
+        </is>
+      </c>
+      <c r="J172" s="2" t="inlineStr">
+        <is>
+          <t>RSK-024</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B173" s="2" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C173" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D173" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 화물선 피격에도 韓 선박 8척 추가 통과…5척만 남아 - 이투데이</t>
+        </is>
+      </c>
+      <c r="E173" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협에서 화물선 피격 사건이 발생했음에도 한국 선박 8척이 추가 통과했으며, 5척이 남아있는 상황입니다.</t>
+        </is>
+      </c>
+      <c r="F173" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협에서의 화물선 피격은 해당 지역을 통과하는 우리 제품 운송 선박의 안전을 위협하고, 보험료 상승 및 운송 지연을 유발할 수 있어 즉각적인 대응이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G173" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협을 통과하는 선박의 운항 상황 및 안전 정보 실시간 확인, 필요 시 대체 항로 또는 운송 수단 검토, 해상 보험 조건 재검토.</t>
+        </is>
+      </c>
+      <c r="H173" s="2" t="inlineStr">
+        <is>
+          <t>etoday.co.kr</t>
+        </is>
+      </c>
+      <c r="I173" s="2" t="inlineStr">
+        <is>
+          <t>https://etoday.co.kr/news/view/2597512</t>
+        </is>
+      </c>
+      <c r="J173" s="2" t="inlineStr">
+        <is>
+          <t>RSK-025</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B174" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C174" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D174" s="3" t="inlineStr">
+        <is>
+          <t>IATA Outlines Four Priorities to Strengthen the Aviation Supply Chain (PRESSROOM)</t>
+        </is>
+      </c>
+      <c r="E174" s="3" t="inlineStr">
+        <is>
+          <t>IATA는 항공기 인도 지연, 엔진 MRO 병목 현상, 예비 부품 확보 어려움 등 항공 공급망 강화를 위한 네 가지 우선순위를 제시했다.</t>
+        </is>
+      </c>
+      <c r="F174" s="3" t="inlineStr">
+        <is>
+          <t>항공사의 운영 효율성 저하는 장기적으로 항공 화물 운송의 가용성 및 신뢰성에 영향을 미칠 수 있으므로 추이를 지켜봐야 한다.</t>
+        </is>
+      </c>
+      <c r="G174" s="3" t="inlineStr">
+        <is>
+          <t>항공 화물 운송 파트너와 정기적인 커뮤니케이션을 통해 항공기 가용성 및 운송 스케줄 변화 가능성을 확인한다.</t>
+        </is>
+      </c>
+      <c r="H174" s="3" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I174" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-24-iata-outlines-four-priorities-to-strengthen-aviation-supply-chain/</t>
+        </is>
+      </c>
+      <c r="J174" s="3" t="inlineStr"/>
+    </row>
+    <row r="175">
+      <c r="A175" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B175" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C175" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D175" s="3" t="inlineStr">
+        <is>
+          <t>Tracking True Vessel Delay (PRESS ROOM)</t>
+        </is>
+      </c>
+      <c r="E175" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence 분석에 따르면 선사들이 운송 시간을 늘리는 스케줄 버퍼링을 통해 선박 지연을 관리하고 있으며, 이는 실제 지연과 조기 도착 간의 관계를 분석한 결과이다.</t>
+        </is>
+      </c>
+      <c r="F175" s="3" t="inlineStr">
+        <is>
+          <t>선사들의 스케줄 버퍼링은 겉으로 보이는 정시성을 높일 수 있으나, 실제 운송 시간 증가로 이어질 수 있어 운송 리드타임에 영향을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="G175" s="3" t="inlineStr">
+        <is>
+          <t>주요 항로의 선박 스케줄 및 실제 운송 리드타임 변화를 지속적으로 모니터링하고, 필요시 운송 계획에 반영한다.</t>
+        </is>
+      </c>
+      <c r="H175" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I175" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/394-tracking-true-vessel-delay</t>
+        </is>
+      </c>
+      <c r="J175" s="3" t="inlineStr"/>
+    </row>
+    <row r="176">
+      <c r="A176" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B176" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C176" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D176" s="3" t="inlineStr">
+        <is>
+          <t>Transpacific: Ripe for new non-alliance services (PRESS ROOM)</t>
+        </is>
+      </c>
+      <c r="E176" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence 분석 결과, 태평양 횡단 노선의 컨테이너 스팟 운임과 비동맹 선사의 운송 능력 점유율 간의 관계를 통해 새로운 비동맹 서비스의 출현 가능성이 높다고 전망했다.</t>
+        </is>
+      </c>
+      <c r="F176" s="3" t="inlineStr">
+        <is>
+          <t>태평양 횡단 노선에 새로운 비동맹 서비스가 등장할 경우, 운임 경쟁 심화 및 서비스 옵션 확대 가능성이 있어 운송 비용 및 전략에 영향을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="G176" s="3" t="inlineStr">
+        <is>
+          <t>태평양 횡단 노선의 신규 서비스 동향과 운임 변동 추이를 면밀히 모니터링하고, 잠재적 운송 파트너를 검토한다.</t>
+        </is>
+      </c>
+      <c r="H176" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I176" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/393-transpacific-ripe-for-new-non-alliance-services</t>
+        </is>
+      </c>
+      <c r="J176" s="3" t="inlineStr"/>
+    </row>
+    <row r="177">
+      <c r="A177" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B177" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C177" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D177" s="3" t="inlineStr">
+        <is>
+          <t>2026-Q1: NAEC Ports Consolidate Market Share (PRESS ROOM)</t>
+        </is>
+      </c>
+      <c r="E177" s="3" t="inlineStr">
+        <is>
+          <t>2026년 1분기 북미 동부 해안(NAEC) 항만의 컨테이너 물동량이 전년 대비 감소했음에도 불구하고, NAEC 항만들이 시장 점유율을 공고히 하고 있음을 Sea-Intelligence가 분석했다.</t>
+        </is>
+      </c>
+      <c r="F177" s="3" t="inlineStr">
+        <is>
+          <t>북미 동부 해안 항만의 물동량 변화 및 시장 점유율 공고화는 향후 해당 항로의 혼잡도, 서비스 품질 및 운임에 간접적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G177" s="3" t="inlineStr">
+        <is>
+          <t>북미 동부 해안 항만의 물동량 추이와 서비스 신뢰도를 지속적으로 모니터링하여 운송 경로 및 항만 선택 전략에 참고한다.</t>
+        </is>
+      </c>
+      <c r="H177" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I177" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/391-2026-q1-naec-ports-consolidate-market-share</t>
+        </is>
+      </c>
+      <c r="J177" s="3" t="inlineStr"/>
+    </row>
+    <row r="178">
+      <c r="A178" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B178" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C178" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D178" s="3" t="inlineStr">
+        <is>
+          <t>선박 호르무즈 탈출 시작됐지만…운임은 요지부동 "3분기 지나야 안정"</t>
+        </is>
+      </c>
+      <c r="E178" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 통항이 재개되며 선박들이 빠져나오고 있지만, 급격히 유입될 물량으로 인한 컨테이너 공급망 지연 우려로 해상 운임은 여전히 높은 수준을 유지하며 3분기 이후에나 안정될 것으로 전망됩니다.</t>
+        </is>
+      </c>
+      <c r="F178" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협의 통항 재개에도 불구하고 해상 운임이 단기간에 안정되기 어렵고, 급증하는 물량으로 인한 추가적인 운송 지연 가능성이 있어 물류 비용 및 납기 계획에 영향을 줄 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G178" s="3" t="inlineStr">
+        <is>
+          <t>해상 운임 추이를 면밀히 모니터링하고, 장기 운송 계약 조건 및 대체 운송 수단(항공 등)의 비용 효율성을 재검토하여 물류비 상승에 대비해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H178" s="3" t="inlineStr">
+        <is>
+          <t>파이낸셜뉴스</t>
+        </is>
+      </c>
+      <c r="I178" s="3" t="inlineStr">
+        <is>
+          <t>https://fnnews.com/news/202606260531107942</t>
+        </is>
+      </c>
+      <c r="J178" s="3" t="inlineStr"/>
+    </row>
+    <row r="179">
+      <c r="A179" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B179" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C179" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D179" s="3" t="inlineStr">
+        <is>
+          <t>머스크, 북미 배터리 물류 시장 진출…리튬이온 배터리 육상운송 서비스 개시</t>
+        </is>
+      </c>
+      <c r="E179" s="3" t="inlineStr">
+        <is>
+          <t>머스크가 북미 육상운송망에 리튬이온 배터리 전용 운송 솔루션을 도입하며 급성장하는 배터리 물류 시장 공략에 나섰습니다.</t>
+        </is>
+      </c>
+      <c r="F179" s="3" t="inlineStr">
+        <is>
+          <t>주요 선사가 리튬이온 배터리 전용 물류 서비스를 확장하는 것은 향후 북미 지역 배터리 운송의 효율성과 안전성을 높일 수 있는 기회가 될 수 있으므로, 서비스의 구체적인 내용과 비용 구조를 파악할 필요가 있습니다.</t>
+        </is>
+      </c>
+      <c r="G179" s="3" t="inlineStr">
+        <is>
+          <t>머스크의 배터리 운송 서비스 상세 내용을 파악하고, 북미 지역 배터리 물류 파트너십 및 비용 효율성 측면에서 검토를 진행해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H179" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I179" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/vol129-주간-선사별-동향-week-26-2026</t>
+        </is>
+      </c>
+      <c r="J179" s="3" t="inlineStr"/>
+    </row>
+    <row r="180">
+      <c r="A180" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B180" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C180" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D180" s="3" t="inlineStr">
+        <is>
+          <t>서울 지하철 대용량 리튬배터리 반입 금지</t>
+        </is>
+      </c>
+      <c r="E180" s="3" t="inlineStr">
+        <is>
+          <t>서울교통공사가 7월 1일부터 160Wh 초과 리튬배터리와 전동킥보드 등 전동식 개인 이동장치의 지하철 반입을 금지하여 리튬배터리 화재 위험을 예방한다.</t>
+        </is>
+      </c>
+      <c r="F180" s="3" t="inlineStr">
+        <is>
+          <t>지하철 내 대용량 리튬배터리 반입 금지는 일반 소비자 운송에 대한 규제이나, 리튬배터리 안전에 대한 사회적 경각심과 규제 강화 추세를 보여주므로 향후 물류 및 보관 규제에 영향을 줄 수 있어 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G180" s="3" t="inlineStr">
+        <is>
+          <t>리튬배터리 관련 국내외 운송 및 보관 규제 동향 지속 모니터링 및 내부 안전 지침 검토.</t>
+        </is>
+      </c>
+      <c r="H180" s="3" t="inlineStr">
+        <is>
+          <t>서울Pn</t>
+        </is>
+      </c>
+      <c r="I180" s="3" t="inlineStr">
+        <is>
+          <t>https://go.seoul.co.kr/news/newsView.php?id=20260626019010</t>
+        </is>
+      </c>
+      <c r="J180" s="3" t="inlineStr"/>
+    </row>
+    <row r="181">
+      <c r="A181" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B181" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C181" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D181" s="3" t="inlineStr">
+        <is>
+          <t>미국, 이란과 전쟁으로 '군수품 고갈' 심각하다 : NYT "서태평양에서 중국 견제에 공백 생길 우려"</t>
+        </is>
+      </c>
+      <c r="E181" s="3" t="inlineStr">
+        <is>
+          <t>미국이 이란과의 전쟁으로 군수품이 고갈되어 서태평양에서 중국 견제 역량에 공백이 생길 수 있다는 보도가 나왔으며, 이는 글로벌 지정학적 불안정성을 시사한다.</t>
+        </is>
+      </c>
+      <c r="F181" s="3" t="inlineStr">
+        <is>
+          <t>미국의 군수품 고갈 및 중국 견제 역량 공백 우려는 글로벌 지정학적 불안정성을 심화시키고, 이는 장기적으로 원자재 공급망, 해상 운송 경로, 특정 국가와의 무역 관계 등에 간접적인 영향을 미칠 수 있으므로 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G181" s="3" t="inlineStr">
+        <is>
+          <t>글로벌 지정학적 리스크 보고서 및 전문가 분석 지속 검토, 주요 원자재 및 부품 공급망의 다변화 전략 재점검.</t>
+        </is>
+      </c>
+      <c r="H181" s="3" t="inlineStr">
+        <is>
+          <t>허프포스트코리아</t>
+        </is>
+      </c>
+      <c r="I181" s="3" t="inlineStr">
+        <is>
+          <t>https://huffingtonpost.kr/article/258266</t>
+        </is>
+      </c>
+      <c r="J181" s="3" t="inlineStr"/>
+    </row>
+    <row r="182">
+      <c r="A182" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B182" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C182" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D182" s="3" t="inlineStr">
+        <is>
+          <t>미국이 중국 상대로 '구리 전쟁' 벌이고 있다 : 올해 6월 말 '구리 관세' 확대 결정</t>
+        </is>
+      </c>
+      <c r="E182" s="3" t="inlineStr">
+        <is>
+          <t>미국이 반제품 구리에 이어 올해 6월 말부터 구리 정련동에 대한 관세 부과를 확대하며 글로벌 구리 시장에 긴장감이 고조되고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F182" s="3" t="inlineStr">
+        <is>
+          <t>구리 관세 확대는 배터리 및 전자부품의 핵심 원자재 가격 상승을 유발하여 장기적으로 우리 제품의 원가 및 공급망 안정성에 영향을 줄 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G182" s="3" t="inlineStr">
+        <is>
+          <t>글로벌 구리 시장 동향 및 가격 변동 추이 모니터링, 주요 공급업체의 원자재 수급 및 가격 정책 변화 확인.</t>
+        </is>
+      </c>
+      <c r="H182" s="3" t="inlineStr">
+        <is>
+          <t>huffingtonpost.kr</t>
+        </is>
+      </c>
+      <c r="I182" s="3" t="inlineStr">
+        <is>
+          <t>https://huffingtonpost.kr/article/258270</t>
+        </is>
+      </c>
+      <c r="J182" s="3" t="inlineStr"/>
+    </row>
+    <row r="183">
+      <c r="A183" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B183" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C183" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D183" s="3" t="inlineStr">
+        <is>
+          <t>"급여 반납합니다" 파라타항공 비상경영 - 매일경제</t>
+        </is>
+      </c>
+      <c r="E183" s="3" t="inlineStr">
+        <is>
+          <t>고유가 후폭풍으로 파라타항공이 대표 및 직원 급여 반납 등 비상경영에 돌입했습니다.</t>
+        </is>
+      </c>
+      <c r="F183" s="3" t="inlineStr">
+        <is>
+          <t>고유가로 인한 특정 항공사의 비상경영은 향후 항공 화물 운임 상승 또는 운송 서비스의 불안정성을 초래할 가능성이 있어 추이를 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G183" s="3" t="inlineStr">
+        <is>
+          <t>항공 화물 운송 시장 동향 및 주요 항공사의 재무 상태 지속 모니터링, 필요 시 대체 항공사 또는 운송 수단 검토.</t>
+        </is>
+      </c>
+      <c r="H183" s="3" t="inlineStr">
+        <is>
+          <t>mk.co.kr</t>
+        </is>
+      </c>
+      <c r="I183" s="3" t="inlineStr">
+        <is>
+          <t>https://mk.co.kr/news/business/12083301</t>
+        </is>
+      </c>
+      <c r="J183" s="3" t="inlineStr"/>
+    </row>
+    <row r="184">
+      <c r="A184" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B184" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C184" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D184" s="3" t="inlineStr">
+        <is>
+          <t>국제유가, 전쟁 이전 수준으로 하락…석유 최고가격 인하 검토 | 한국경제</t>
+        </is>
+      </c>
+      <c r="E184" s="3" t="inlineStr">
+        <is>
+          <t>국제 유가가 전쟁 이전 수준으로 하락하여 정부가 석유 최고가격 인하를 검토하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F184" s="3" t="inlineStr">
+        <is>
+          <t>국제 유가 하락은 해상 및 항공 운송 비용 절감에 긍정적인 영향을 미칠 수 있으나, 유가는 변동성이 크므로 지속적인 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G184" s="3" t="inlineStr">
+        <is>
+          <t>유가 변동에 따른 운임 계약 조건 검토, 연료 할증료(BAF/FAF) 조정 가능성 확인.</t>
+        </is>
+      </c>
+      <c r="H184" s="3" t="inlineStr">
+        <is>
+          <t>hankyung.com</t>
+        </is>
+      </c>
+      <c r="I184" s="3" t="inlineStr">
+        <is>
+          <t>https://www.hankyung.com/article/2026062689377</t>
+        </is>
+      </c>
+      <c r="J184" s="3" t="inlineStr"/>
+    </row>
+    <row r="185">
+      <c r="A185" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B185" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C185" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D185" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 선박 피격에 국제유가 반등…WTI 2.3%↑ | 연합뉴스</t>
+        </is>
+      </c>
+      <c r="E185" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협에서 발생한 선박 피격 사건의 영향으로 국제유가가 2.3% 반등했습니다.</t>
+        </is>
+      </c>
+      <c r="F185" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 선박 피격으로 인한 국제 유가 반등은 해상 및 항공 운송 비용에 영향을 미칠 수 있으므로 추이를 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G185" s="3" t="inlineStr">
+        <is>
+          <t>유가 변동에 따른 운임 계약 조건 및 연료 할증료(BAF/FAF) 변동 가능성 확인.</t>
+        </is>
+      </c>
+      <c r="H185" s="3" t="inlineStr">
+        <is>
+          <t>연합뉴스</t>
+        </is>
+      </c>
+      <c r="I185" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20260626005500072</t>
+        </is>
+      </c>
+      <c r="J185" s="3" t="inlineStr"/>
+    </row>
+    <row r="186">
+      <c r="A186" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B186" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C186" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D186" s="4" t="inlineStr">
+        <is>
+          <t>고려해운, 日–韓–큐슈 노선 ‘JKW4’로 일원화 (해운)</t>
+        </is>
+      </c>
+      <c r="E186" s="4" t="inlineStr">
+        <is>
+          <t>고려해운이 일본-한국-큐슈 노선을 JKW4로 통합하고 야쓰시로항 기항을 주 1회로 확대하여 서비스 효율성을 높였다.</t>
+        </is>
+      </c>
+      <c r="F186" s="4" t="inlineStr">
+        <is>
+          <t>특정 노선의 서비스 개편으로, 우리 회사의 주요 운송 경로에 직접적인 영향은 없으며, 오히려 서비스 선택지가 늘어날 수 있다.</t>
+        </is>
+      </c>
+      <c r="G186" s="4" t="n"/>
+      <c r="H186" s="4" t="inlineStr">
+        <is>
+          <t>kita</t>
+        </is>
+      </c>
+      <c r="I186" s="4" t="inlineStr">
+        <is>
+          <t>https://www.kita.net/shippers/board/newsView.do?morgueCode=2&amp;dataCls=B&amp;dataSeq=8137</t>
+        </is>
+      </c>
+      <c r="J186" s="4" t="inlineStr"/>
+    </row>
+    <row r="187">
+      <c r="A187" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B187" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C187" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D187" s="4" t="inlineStr">
+        <is>
+          <t>해진공, '강화된' 중소선사 대상 특별지원 프로그램 발표 (해운/항만/물류)</t>
+        </is>
+      </c>
+      <c r="E187" s="4" t="inlineStr">
+        <is>
+          <t>한국해양진흥공사가 중소선사의 안정적인 자금 조달 및 경영 지원을 위한 특별지원 프로그램을 강화하여 발표했다.</t>
+        </is>
+      </c>
+      <c r="F187" s="4" t="inlineStr">
+        <is>
+          <t>국내 중소선사 지원 프로그램으로, 우리 회사의 해상 운송 비용이나 서비스에 직접적인 영향은 미미하다.</t>
+        </is>
+      </c>
+      <c r="G187" s="4" t="n"/>
+      <c r="H187" s="4" t="inlineStr">
+        <is>
+          <t>oceanpress</t>
+        </is>
+      </c>
+      <c r="I187" s="4" t="inlineStr">
+        <is>
+          <t>https://www.oceanpress.co.kr/news/article.html?no=30446</t>
+        </is>
+      </c>
+      <c r="J187" s="4" t="inlineStr"/>
+    </row>
+    <row r="188">
+      <c r="A188" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B188" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C188" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D188" s="4" t="inlineStr">
+        <is>
+          <t>Global Schedule Reliability for April 2026 the Highest of the Year (PRESS ROOM)</t>
+        </is>
+      </c>
+      <c r="E188" s="4" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence 보고서에 따르면 2026년 4월 전 세계 정기선 스케줄 신뢰도가 올해 최고치를 기록했다.</t>
+        </is>
+      </c>
+      <c r="F188" s="4" t="inlineStr">
+        <is>
+          <t>전반적인 스케줄 신뢰도 개선은 긍정적이나, 특정 항로 및 선사의 신뢰도는 다를 수 있어 당장 우리 물류 운영에 큰 변화를 요구하지는 않는다.</t>
+        </is>
+      </c>
+      <c r="G188" s="4" t="n"/>
+      <c r="H188" s="4" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I188" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/390-global-schedule-reliability-for-april-2026-the-highest-of-the-year</t>
+        </is>
+      </c>
+      <c r="J188" s="4" t="inlineStr"/>
+    </row>
+    <row r="189">
+      <c r="A189" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B189" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C189" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D189" s="4" t="inlineStr">
+        <is>
+          <t>황종우 해수부 장관, 연안해운 업계와 현안 논의 (홈 &gt; 뉴스 &gt; 해운)</t>
+        </is>
+      </c>
+      <c r="E189" s="4" t="inlineStr">
+        <is>
+          <t>황종우 해양수산부 장관이 연안해운 업계와 간담회를 통해 연안해운 경쟁력 강화 및 자생력 확보 방안을 논의하고, 연안 선박 현대화 및 친환경 해상 운송 전환을 강조했다.</t>
+        </is>
+      </c>
+      <c r="F189" s="4" t="inlineStr">
+        <is>
+          <t>국내 연안 해운 산업의 정책 논의로, 우리 회사의 주요 국제 물류 운영에 직접적인 영향은 미미하다.</t>
+        </is>
+      </c>
+      <c r="G189" s="4" t="n"/>
+      <c r="H189" s="4" t="inlineStr">
+        <is>
+          <t>shippingnews</t>
+        </is>
+      </c>
+      <c r="I189" s="4" t="inlineStr">
+        <is>
+          <t>https://www.shippingnewsnet.com/news/articleView.html?idxno=70920</t>
+        </is>
+      </c>
+      <c r="J189" s="4" t="inlineStr"/>
+    </row>
+    <row r="190">
+      <c r="A190" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B190" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C190" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D190" s="4" t="inlineStr">
+        <is>
+          <t>씨메스로보틱스 / ‘물류·제조 대형 수주 잇달아’ 피지컬 AI 기반 로봇 자동화 사업 가속</t>
+        </is>
+      </c>
+      <c r="E190" s="4" t="inlineStr">
+        <is>
+          <t>씨메스로보틱스가 물류 및 제조 현장에서 피지컬 AI 기반 로봇 자동화 프로젝트를 연이어 수주하며 사업을 확대하고 있으며, 이는 1분기 사상 최대 매출 달성으로 이어졌습니다.</t>
+        </is>
+      </c>
+      <c r="F190" s="4" t="inlineStr">
+        <is>
+          <t>물류 자동화 기술 발전 동향을 보여주는 뉴스이나, 당사의 즉각적인 물류 운영에 직접적인 영향을 미치기보다는 장기적인 관점에서 참고할 정보입니다.</t>
+        </is>
+      </c>
+      <c r="G190" s="4" t="inlineStr"/>
+      <c r="H190" s="4" t="inlineStr">
+        <is>
+          <t>ulogistics</t>
+        </is>
+      </c>
+      <c r="I190" s="4" t="inlineStr">
+        <is>
+          <t>http://www.ulogistics.co.kr/test/board.php?board=all2&amp;command=body&amp;no=5202</t>
+        </is>
+      </c>
+      <c r="J190" s="4" t="inlineStr"/>
+    </row>
+    <row r="191">
+      <c r="A191" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B191" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C191" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D191" s="4" t="inlineStr">
+        <is>
+          <t>How OTRM enables effective management of supply chain disruptions</t>
+        </is>
+      </c>
+      <c r="E191" s="4" t="inlineStr">
+        <is>
+          <t>OTRM(Operational Trade Risk Management) 시스템이 계약, 물리적 이동, 운영 조치를 지속적으로 동기화하여 공급망 중단을 효과적으로 관리하고 물류 위기를 예방하는 데 기여할 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="F191" s="4" t="inlineStr">
+        <is>
+          <t>공급망 관리 시스템의 중요성을 강조하는 내용으로, 당사의 현재 시스템 운영에 즉각적인 변화를 요구하기보다는 장기적인 시스템 개선 방향을 모색하는 데 참고할 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G191" s="4" t="inlineStr"/>
+      <c r="H191" s="4" t="inlineStr">
+        <is>
+          <t>CTRM Center</t>
+        </is>
+      </c>
+      <c r="I191" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ctrmcenter.com/blog/commodity-trading/how-otrm-enables-effective-management-of-supply-chain-disruptions/</t>
+        </is>
+      </c>
+      <c r="J191" s="4" t="inlineStr"/>
+    </row>
+    <row r="192">
+      <c r="A192" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B192" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C192" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D192" s="4" t="inlineStr">
+        <is>
+          <t>UK DBT creates Supply Chain Centre to battle logistics uncertainty</t>
+        </is>
+      </c>
+      <c r="E192" s="4" t="inlineStr">
+        <is>
+          <t>영국 기업무역부가 물류 불확실성에 대응하기 위해 공급망 센터를 설립하고 영국 물류 지원을 위한 임무 선언문과 실행 계획을 발표했습니다.</t>
+        </is>
+      </c>
+      <c r="F192" s="4" t="inlineStr">
+        <is>
+          <t>영국 정부의 공급망 안정화 노력에 대한 소식으로, 당사의 직접적인 물류 운영에 미치는 영향은 적지만 글로벌 공급망 정책 동향을 파악하는 데 참고할 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G192" s="4" t="inlineStr"/>
+      <c r="H192" s="4" t="inlineStr">
+        <is>
+          <t>Logistics Manager</t>
+        </is>
+      </c>
+      <c r="I192" s="4" t="inlineStr">
+        <is>
+          <t>https://logisticsmanager.com/uk-dbt-creates-supply-chain-centre-to-battle-logistics-uncertainty</t>
+        </is>
+      </c>
+      <c r="J192" s="4" t="inlineStr"/>
+    </row>
+    <row r="193">
+      <c r="A193" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B193" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C193" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D193" s="4" t="inlineStr">
+        <is>
+          <t>How autonomous systems are reshaping warehouse operations</t>
+        </is>
+      </c>
+      <c r="E193" s="4" t="inlineStr">
+        <is>
+          <t>자율 시스템이 물류 운영의 핵심 역량이 되고 있으며, 자동화, AI, 실시간 운영 인텔리전스를 결합하여 창고 운영을 혁신하고 공급망 중단에 효과적으로 대응할 수 있도록 합니다.</t>
+        </is>
+      </c>
+      <c r="F193" s="4" t="inlineStr">
+        <is>
+          <t>창고 운영 자동화 및 AI 기술 동향을 보여주는 뉴스이나, 당사의 즉각적인 창고 운영 계획에 직접적인 영향을 미치기보다는 장기적인 기술 도입 검토에 참고할 정보입니다.</t>
+        </is>
+      </c>
+      <c r="G193" s="4" t="inlineStr"/>
+      <c r="H193" s="4" t="inlineStr">
+        <is>
+          <t>TechRadar</t>
+        </is>
+      </c>
+      <c r="I193" s="4" t="inlineStr">
+        <is>
+          <t>https://techradar.com/pro/how-autonomous-systems-are-reshaping-warehouse-operations</t>
+        </is>
+      </c>
+      <c r="J193" s="4" t="inlineStr"/>
+    </row>
+    <row r="194">
+      <c r="A194" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B194" s="4" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C194" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D194" s="4" t="inlineStr">
+        <is>
+          <t>정부, 자원안보 전면 강화…공급망 위기 대응 로드맵 본격 추진</t>
+        </is>
+      </c>
+      <c r="E194" s="4" t="inlineStr">
+        <is>
+          <t>정부가 에너지·자원 수급 취약점 보완과 핵심광물 및 소재·부품 공급망 강화를 위한 대책 마련에 착수했습니다.</t>
+        </is>
+      </c>
+      <c r="F194" s="4" t="inlineStr">
+        <is>
+          <t>정부의 자원안보 강화 및 공급망 위기 대응 로드맵 추진은 장기적인 관점에서 우리 기업의 공급망 안정화에 기여할 수 있으나, 즉각적인 물류 운영 변화를 요구하지는 않습니다.</t>
+        </is>
+      </c>
+      <c r="G194" s="4" t="inlineStr"/>
+      <c r="H194" s="4" t="inlineStr">
+        <is>
+          <t>kyongbuk.co.kr</t>
+        </is>
+      </c>
+      <c r="I194" s="4" t="inlineStr">
+        <is>
+          <t>https://kyongbuk.co.kr/news/articleView.html?idxno=4076675</t>
+        </is>
+      </c>
+      <c r="J194" s="4" t="inlineStr"/>
+    </row>
+    <row r="195">
+      <c r="A195" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B195" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C195" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D195" s="4" t="inlineStr">
+        <is>
+          <t>울산해경, 부산 대변 남동방 22해리 해상 상선과 어선 충돌 사고 발생 긴급 구조 중 (3보):正筆</t>
+        </is>
+      </c>
+      <c r="E195" s="4" t="inlineStr">
+        <is>
+          <t>부산 대변 남동방 해상에서 상선과 어선이 충돌하는 사고가 발생하여 해경이 긴급 구조 작업을 진행 중입니다.</t>
+        </is>
+      </c>
+      <c r="F195" s="4" t="inlineStr">
+        <is>
+          <t>부산 인근 해상에서의 상선과 어선 충돌 사고는 국지적인 사건으로, 우리 회사의 글로벌 물류 운영에 직접적인 영향을 주지 않습니다.</t>
+        </is>
+      </c>
+      <c r="G195" s="4" t="inlineStr"/>
+      <c r="H195" s="4" t="inlineStr">
+        <is>
+          <t>jeongpil.com</t>
+        </is>
+      </c>
+      <c r="I195" s="4" t="inlineStr">
+        <is>
+          <t>https://jeongpil.com/2575563</t>
+        </is>
+      </c>
+      <c r="J195" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
@@ -8703,7 +9927,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9499,6 +10723,146 @@
       </c>
       <c r="I22" s="6" t="inlineStr"/>
     </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>RSK-022</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 통과 화물선 피격…이란 '지정 항로' 경고 현실화</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr"/>
+      <c r="G23" s="6" t="inlineStr"/>
+      <c r="H23" s="6" t="inlineStr">
+        <is>
+          <t>중동 항로를 이용하는 선박의 안전 운항 여부 및 대체 항로 가능성을 즉시 확인하고, 보험 및 비상 운송 계획을 점검해야 합니다.</t>
+        </is>
+      </c>
+      <c r="I23" s="6" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>RSK-023</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>🚢🚚 복합 운송 기반 근거리 아웃소싱 솔루션 🌍📜⚖️ 새로운 EU 법률이 모든 것을 바꿉니다 🔗❌🗓️ 2026년부터 선형 공급망이 쓸모없어지는 이유</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr"/>
+      <c r="G24" s="6" t="inlineStr"/>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>EU 순환 경제법 및 관련 배터리 규제(예: EU Battery Regulation) 상세 분석, 2026년까지 공급망 및 역물류 전략 재수립, 제품 설계 단계부터 순환 경제 원칙 반영 검토.</t>
+        </is>
+      </c>
+      <c r="I24" s="6" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>RSK-024</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>"이러다 중소기업 줄줄이 망한다"…한국 정부가 중국에 황급히 SOS 친 '진짜 이유'</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr"/>
+      <c r="G25" s="6" t="inlineStr"/>
+      <c r="H25" s="6" t="inlineStr">
+        <is>
+          <t>대중국 수출 제품의 규정 준수 여부 즉시 확인 및 필요 시 인증 획득 절차 가속화, 대체 시장 또는 운송 경로 검토.</t>
+        </is>
+      </c>
+      <c r="I25" s="6" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>RSK-025</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈 화물선 피격에도 韓 선박 8척 추가 통과…5척만 남아 - 이투데이</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr"/>
+      <c r="G26" s="6" t="inlineStr"/>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈 해협을 통과하는 선박의 운항 상황 및 안전 정보 실시간 확인, 필요 시 대체 항로 또는 운송 수단 검토, 해상 보험 조건 재검토.</t>
+        </is>
+      </c>
+      <c r="I26" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
📰 뉴스 데이터 2026-06-29_09:09
</commit_message>
<xml_diff>
--- a/data/SCM_물류_브리핑.xlsx
+++ b/data/SCM_물류_브리핑.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J195"/>
+  <dimension ref="A1:J222"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9670,6 +9670,1266 @@
       </c>
       <c r="J195" s="4" t="inlineStr"/>
     </row>
+    <row r="196">
+      <c r="A196" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B196" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C196" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D196" s="2" t="inlineStr">
+        <is>
+          <t>북미항로/ ‘관세대응 영향’ 물동량 9개월만에 플러스성장</t>
+        </is>
+      </c>
+      <c r="E196" s="2" t="inlineStr">
+        <is>
+          <t>트럼프 정부의 관세 유예 종료 전 수요가 몰리면서 북미항로 물동량이 9개월 만에 플러스 성장했으며, 선사들의 소석률이 100%를 기록하고 6월 말까지 선적 예약이 마감되었다.</t>
+        </is>
+      </c>
+      <c r="F196" s="2" t="inlineStr">
+        <is>
+          <t>트럼프 정부의 관세 부과 움직임에 따른 선적 수요 급증으로 북미항로의 운송 공간 부족 및 운임 상승이 심화되어 우리 회사의 북미향 물류 운영 및 비용에 직접적인 영향을 미친다.</t>
+        </is>
+      </c>
+      <c r="G196" s="2" t="inlineStr">
+        <is>
+          <t>북미향 선적 계획 긴급 점검 및 대체 운송 방안 모색, 운임 변동성 대비 예산 조정, 관세 부과 대상 품목 및 시기 확인.</t>
+        </is>
+      </c>
+      <c r="H196" s="2" t="inlineStr">
+        <is>
+          <t>ksg</t>
+        </is>
+      </c>
+      <c r="I196" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ksg.co.kr/news/main_newsView.jsp?pNum=147496</t>
+        </is>
+      </c>
+      <c r="J196" s="2" t="inlineStr">
+        <is>
+          <t>RSK-026</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B197" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C197" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D197" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 물류 불확실성 지속: 한국 선박 3척 잔류, 해상운임 9주 연속 상승</t>
+        </is>
+      </c>
+      <c r="E197" s="2" t="inlineStr">
+        <is>
+          <t>미국-이란 충돌 재개로 호르무즈 해협의 물류 불확실성이 다시 커졌으며, 한국 선박 3척이 여전히 남아있고 글로벌 해상운임은 9주 연속 상승하여 물류비 부담이 가중되고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F197" s="2" t="inlineStr">
+        <is>
+          <t>중동 지역의 지정학적 리스크가 주요 해상 운송로의 안전과 운임에 직접적인 영향을 미치고 있어 즉각적인 운송 계획 검토 및 비상 계획 수립이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G197" s="2" t="inlineStr">
+        <is>
+          <t>중동 경유 선박의 운항 스케줄 및 경로 재확인, 대체 운송 경로(예: 육상, 항공) 및 운송사 옵션 검토, 비상 재고 수준 점검 및 확보, 운임 변동성 모니터링 강화.</t>
+        </is>
+      </c>
+      <c r="H197" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I197" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260629-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J197" s="2" t="inlineStr">
+        <is>
+          <t>RSK-027</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B198" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C198" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D198" s="2" t="inlineStr">
+        <is>
+          <t>연합뉴스TV</t>
+        </is>
+      </c>
+      <c r="E198" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 안쪽에서 발이 묶였던 우리 선박들의 '탈출 물결'이 이어지고 있으며, 정부는 이들의 안전한 통항을 적극 지원할 방침이다. 이는 중동 지역의 지정학적 불안정성이 해상 운송에 직접적인 영향을 미치고 있음을 보여준다.</t>
+        </is>
+      </c>
+      <c r="F198" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협은 주요 원자재 및 제품 운송 경로로, 해당 지역의 불안정성으로 인한 선박 통항 문제는 우리 회사의 원자재 수급 및 완제품 출하에 심각한 지연을 초래할 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G198" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협을 경유하는 운송 계획을 즉시 점검하고, 대체 항로 및 운송 수단 확보 가능성을 타진하며, 비상 재고 수준을 검토해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H198" s="2" t="inlineStr">
+        <is>
+          <t>연합뉴스TV</t>
+        </is>
+      </c>
+      <c r="I198" s="2" t="inlineStr">
+        <is>
+          <t>https://yonhapnewstv.co.kr/news/MYH20260628091455mRG</t>
+        </is>
+      </c>
+      <c r="J198" s="2" t="inlineStr">
+        <is>
+          <t>RSK-028</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B199" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C199" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D199" s="2" t="inlineStr">
+        <is>
+          <t>'호르무즈 통제' 놓고 보복 난타전 … 美·이란 다시 전면전 위기</t>
+        </is>
+      </c>
+      <c r="E199" s="2" t="inlineStr">
+        <is>
+          <t>미국과 이란 간 호르무즈 해협 통제권을 둘러싼 군사적 긴장이 고조되며 전면전 위기가 다시 불거지고 있다. 이란이 해협 통행료를 요구하고 미국은 자유로운 통항을 주장하며 충돌하고 있다.</t>
+        </is>
+      </c>
+      <c r="F199" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협은 주요 해상 운송로이자 유류 수송의 핵심 길목으로, 긴장 고조는 해상 운송 지연 및 유가 급등으로 이어져 물류 비용과 운영에 즉각적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G199" s="2" t="inlineStr">
+        <is>
+          <t>해상 운송 경로 및 운임 변동성 모니터링 강화, 비상 운송 계획 검토, 유류 재고 및 구매 전략 점검.</t>
+        </is>
+      </c>
+      <c r="H199" s="2" t="inlineStr">
+        <is>
+          <t>매일경제</t>
+        </is>
+      </c>
+      <c r="I199" s="2" t="inlineStr">
+        <is>
+          <t>https://mk.co.kr/news/world/12085090</t>
+        </is>
+      </c>
+      <c r="J199" s="2" t="inlineStr">
+        <is>
+          <t>RSK-029</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B200" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C200" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D200" s="3" t="inlineStr">
+        <is>
+          <t>CAPE Phase 2 Launches June 29 for Reconciliation-Flagged Entries; TPEB Rates Rise 10% for Sixth Consecutive Week</t>
+        </is>
+      </c>
+      <c r="E200" s="3" t="inlineStr">
+        <is>
+          <t>미국 CBP의 CAPE 2단계가 6월 29일 발효되어 관세 환급 대상이 확대되며, 태평양 횡단 동향(TPEB) 운임이 6주 연속 10% 상승했다.</t>
+        </is>
+      </c>
+      <c r="F200" s="3" t="inlineStr">
+        <is>
+          <t>CAPE 2단계 발효는 관세 환급 절차에 영향을 줄 수 있으며, TPEB 운임의 지속적인 상승 추세는 북미향 해상 운송 비용 증가로 이어질 수 있다.</t>
+        </is>
+      </c>
+      <c r="G200" s="3" t="inlineStr">
+        <is>
+          <t>북미향 해상 운송 계획 및 예산 재검토, CAPE 2단계 적용 대상 여부 확인 및 관련 절차 숙지.</t>
+        </is>
+      </c>
+      <c r="H200" s="3" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I200" s="3" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/june-25-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J200" s="3" t="inlineStr"/>
+    </row>
+    <row r="201">
+      <c r="A201" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B201" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C201" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D201" s="3" t="inlineStr">
+        <is>
+          <t>CPSC Mandatory eFiling Takes Effect July 8; TPEB Rates Surge ~10% as Peak Season Demand Outpaces Capacity</t>
+        </is>
+      </c>
+      <c r="E201" s="3" t="inlineStr">
+        <is>
+          <t>미국 CPSC의 의무 전자 신고가 7월 8일 발효되고, CBP는 강제 노동 관련 통합 지침을 발표했으며, 성수기 수요로 인해 TPEB 운임이 약 10% 급등했다.</t>
+        </is>
+      </c>
+      <c r="F201" s="3" t="inlineStr">
+        <is>
+          <t>CPSC 전자 신고 의무화는 통관 절차에 영향을 주고, CBP의 강제 노동 지침은 공급망 실사 리스크를 높이며, TPEB 운임 급등은 북미향 물류비 부담을 가중시킨다.</t>
+        </is>
+      </c>
+      <c r="G201" s="3" t="inlineStr">
+        <is>
+          <t>CPSC 전자 신고 시스템 및 절차 확인, 공급망 내 강제 노동 리스크 점검, 북미향 해상 운송 비용 변동 추이 모니터링.</t>
+        </is>
+      </c>
+      <c r="H201" s="3" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I201" s="3" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/june-18-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J201" s="3" t="inlineStr"/>
+    </row>
+    <row r="202">
+      <c r="A202" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B202" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C202" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D202" s="3" t="inlineStr">
+        <is>
+          <t>DOJ Appeals CIT's IEEPA Refund Injunction as CAPE Phase 2 Targets June 29; TPEB Rates Surge 30% Into Peak</t>
+        </is>
+      </c>
+      <c r="E202" s="3" t="inlineStr">
+        <is>
+          <t>법무부가 CIT의 IEEPA 환급 명령에 항소하고 CAPE 2단계가 6월 29일 시행될 예정이며, 성수기 진입으로 TPEB 운임이 30% 급등했다.</t>
+        </is>
+      </c>
+      <c r="F202" s="3" t="inlineStr">
+        <is>
+          <t>TPEB 운임의 30% 급등은 북미향 해상 운송 비용에 상당한 부담을 줄 수 있으며, IEEPA 환급 관련 법적 분쟁은 관세 환급 절차의 불확실성을 높인다.</t>
+        </is>
+      </c>
+      <c r="G202" s="3" t="inlineStr">
+        <is>
+          <t>북미향 해상 운송 비용 상승에 대비한 운송 계획 및 예산 재검토, IEEPA 환급 관련 법적 진행 상황 주시.</t>
+        </is>
+      </c>
+      <c r="H202" s="3" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I202" s="3" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/june-11-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J202" s="3" t="inlineStr"/>
+    </row>
+    <row r="203">
+      <c r="A203" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B203" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C203" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D203" s="3" t="inlineStr">
+        <is>
+          <t>U.S. Appeals CIT's IEEPA Refund Order to Federal Circuit; TPEB Rates Rise as Peak Season Demand Tightens Capacity</t>
+        </is>
+      </c>
+      <c r="E203" s="3" t="inlineStr">
+        <is>
+          <t>미국이 CIT의 IEEPA 환급 명령에 항소하고 트럼프 대통령이 세관 집행 개혁 행정명령에 서명했으며, 성수기 수요로 TPEB 운임이 상승하고 있다.</t>
+        </is>
+      </c>
+      <c r="F203" s="3" t="inlineStr">
+        <is>
+          <t>IEEPA 환급 관련 항소는 관세 환급의 불확실성을 높이고, 세관 집행 개혁은 수입자 요건 및 정보 공개 의무를 강화하여 통관 절차에 영향을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="G203" s="3" t="inlineStr">
+        <is>
+          <t>IEEPA 환급 관련 법적 진행 상황 주시, 강화된 수입자 요건 및 정보 공개 의무에 대한 대비.</t>
+        </is>
+      </c>
+      <c r="H203" s="3" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I203" s="3" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/june-3-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J203" s="3" t="inlineStr"/>
+    </row>
+    <row r="204">
+      <c r="A204" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B204" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C204" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D204" s="3" t="inlineStr">
+        <is>
+          <t>Section 232 Duties Reduced to 15% for Taiwanese Goods, Retroactive to May 1; China Air Rates Spike on Supply Contraction and Month-End Demand</t>
+        </is>
+      </c>
+      <c r="E204" s="3" t="inlineStr">
+        <is>
+          <t>대만산 특정 품목에 대한 232조 관세가 5월 1일부로 15%로 인하되었으며, 공급 감소와 월말 수요로 인해 중국발 항공 운임이 급등했다.</t>
+        </is>
+      </c>
+      <c r="F204" s="3" t="inlineStr">
+        <is>
+          <t>중국발 항공 운임 급등은 항공 운송 비용에 직접적인 영향을 미치며, 대만산 부품/제품을 사용하는 경우 232조 관세 인하로 비용 절감 효과를 기대할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G204" s="3" t="inlineStr">
+        <is>
+          <t>중국발 항공 운송 계획 및 예산 재검토, 대만산 부품/제품 수입 시 관세 인하 적용 여부 확인.</t>
+        </is>
+      </c>
+      <c r="H204" s="3" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I204" s="3" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/may-28-2026-cit-rejects-governments-stay-request/</t>
+        </is>
+      </c>
+      <c r="J204" s="3" t="inlineStr"/>
+    </row>
+    <row r="205">
+      <c r="A205" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B205" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C205" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D205" s="3" t="inlineStr">
+        <is>
+          <t>Urgent Action Needed to Ease Engine MRO Bottlenecks</t>
+        </is>
+      </c>
+      <c r="E205" s="3" t="inlineStr">
+        <is>
+          <t>IATA는 항공기 엔진 유지보수(MRO) 병목 현상 완화를 위한 긴급 조치가 필요하다고 강조했다.</t>
+        </is>
+      </c>
+      <c r="F205" s="3" t="inlineStr">
+        <is>
+          <t>엔진 MRO 병목 현상은 항공기 가동률 저하로 이어져 항공 화물 운송 능력에 부정적인 영향을 미칠 수 있으므로, 항공 운송 계획에 잠재적 리스크로 작용할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G205" s="3" t="inlineStr">
+        <is>
+          <t>항공 화물 운송 시장의 공급 능력 변화 추이 모니터링.</t>
+        </is>
+      </c>
+      <c r="H205" s="3" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I205" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-24-urgent-action-needed-to-ease-engine-mro-bottlenecks/</t>
+        </is>
+      </c>
+      <c r="J205" s="3" t="inlineStr"/>
+    </row>
+    <row r="206">
+      <c r="A206" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B206" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C206" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D206" s="3" t="inlineStr">
+        <is>
+          <t>WMES 2026 Speech - Stuart Fox, IATA's Director Flight and Operations</t>
+        </is>
+      </c>
+      <c r="E206" s="3" t="inlineStr">
+        <is>
+          <t>IATA 관계자는 항공기 인도 지연, 엔진 문제, 부품 부족, 수리 기간 장기화 등 항공사들이 직면한 현실적인 공급망 문제를 언급했다.</t>
+        </is>
+      </c>
+      <c r="F206" s="3" t="inlineStr">
+        <is>
+          <t>항공기 인도 지연 및 부품 부족 등은 항공 화물 운송 능력에 지속적인 제약을 가할 수 있어, 항공 운송 계획 수립 시 잠재적 리스크로 고려해야 한다.</t>
+        </is>
+      </c>
+      <c r="G206" s="3" t="inlineStr">
+        <is>
+          <t>항공 화물 운송 시장의 공급 능력 및 안정성 변화 추이 모니터링.</t>
+        </is>
+      </c>
+      <c r="H206" s="3" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I206" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-speeches/06-24-wmes-2026-speech-stuart-fox-iata-director-flight-operations/</t>
+        </is>
+      </c>
+      <c r="J206" s="3" t="inlineStr"/>
+    </row>
+    <row r="207">
+      <c r="A207" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B207" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C207" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D207" s="3" t="inlineStr">
+        <is>
+          <t>Tracking True Vessel Delay</t>
+        </is>
+      </c>
+      <c r="E207" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence는 선박 스케줄 버퍼링과 조기 입항 간의 관계를 분석하며, 선사들이 운송 시간을 늘려 스케줄 안정성을 높이려 한다고 밝혔다.</t>
+        </is>
+      </c>
+      <c r="F207" s="3" t="inlineStr">
+        <is>
+          <t>선사들의 스케줄 버퍼링 증가는 명목상 운송 시간 증가로 이어질 수 있으나, 실제 지연 감소를 통해 스케줄 안정성에는 긍정적 영향을 줄 수 있으므로 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G207" s="3" t="n"/>
+      <c r="H207" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I207" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/394-tracking-true-vessel-delay</t>
+        </is>
+      </c>
+      <c r="J207" s="3" t="inlineStr"/>
+    </row>
+    <row r="208">
+      <c r="A208" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B208" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C208" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D208" s="3" t="inlineStr">
+        <is>
+          <t>[오션 뷰] 부산항의 미래는 친환경·탈탄소에 달려 있다</t>
+        </is>
+      </c>
+      <c r="E208" s="3" t="inlineStr">
+        <is>
+          <t>부산항의 미래가 국제해사기구(IMO)의 온실가스 감축 전략 채택과 같은 친환경·탈탄소 노력에 달려 있음을 강조하며, 관련 정책 변화에 대한 중요성을 시사합니다.</t>
+        </is>
+      </c>
+      <c r="F208" s="3" t="inlineStr">
+        <is>
+          <t>친환경 및 탈탄소 규제는 장기적으로 해상 운송 비용 및 선박 선택에 영향을 미칠 수 있으므로, 관련 규제 동향을 지속적으로 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G208" s="3" t="inlineStr">
+        <is>
+          <t>IMO 및 국내외 해운 환경 규제 동향 지속 모니터링, 친환경 운송 옵션 도입 가능성 검토.</t>
+        </is>
+      </c>
+      <c r="H208" s="3" t="inlineStr">
+        <is>
+          <t>부산일보</t>
+        </is>
+      </c>
+      <c r="I208" s="3" t="inlineStr">
+        <is>
+          <t>https://busan.com/view/busan/view.php?code=2026062818061632366</t>
+        </is>
+      </c>
+      <c r="J208" s="3" t="inlineStr"/>
+    </row>
+    <row r="209">
+      <c r="A209" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B209" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C209" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D209" s="3" t="inlineStr">
+        <is>
+          <t>금리 인상·하이닉스 美 상장…하반기 환율 향방 가를 핵심 변수</t>
+        </is>
+      </c>
+      <c r="E209" s="3" t="inlineStr">
+        <is>
+          <t>하반기 환율이 금리 인상, 하이닉스 미국 상장, 중동 전쟁 등 대외 리스크로 인해 1500원대 고환율이 장기화될 수 있다는 우려가 커지고 있다. 이는 달러 강세와 원화 약세 요인이 복합적으로 작용한 결과이다.</t>
+        </is>
+      </c>
+      <c r="F209" s="3" t="inlineStr">
+        <is>
+          <t>고환율 장기화는 수입 원자재 비용 및 해외 운송 비용 증가로 이어져 우리 회사의 물류비 및 생산 비용에 부정적인 영향을 미칠 수 있으므로 지속적인 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G209" s="3" t="inlineStr">
+        <is>
+          <t>환율 변동 추이를 면밀히 모니터링하고, 환헤지 전략 검토 및 원가 절감 방안을 모색해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H209" s="3" t="inlineStr">
+        <is>
+          <t>이데일리</t>
+        </is>
+      </c>
+      <c r="I209" s="3" t="inlineStr">
+        <is>
+          <t>https://edaily.co.kr/News/Read?mediaCodeNo=257&amp;newsId=01472726645486640</t>
+        </is>
+      </c>
+      <c r="J209" s="3" t="inlineStr"/>
+    </row>
+    <row r="210">
+      <c r="A210" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B210" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C210" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D210" s="3" t="inlineStr">
+        <is>
+          <t>국제유가 하락, 서울 휘발유 1800원대 주유소 [포토]</t>
+        </is>
+      </c>
+      <c r="E210" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 통항량 증가로 국제유가가 하락하면서 서울 시내 휘발유 가격이 1800원대로 내려왔다.</t>
+        </is>
+      </c>
+      <c r="F210" s="3" t="inlineStr">
+        <is>
+          <t>국제유가 하락은 물류비용 감소에 긍정적이나, 호르무즈 해협의 지정학적 긴장 고조 뉴스(49번)와 상반되는 동향이므로 유가 변동 추이를 면밀히 모니터링하며 상충되는 정보의 원인을 파악해야 한다.</t>
+        </is>
+      </c>
+      <c r="G210" s="3" t="inlineStr">
+        <is>
+          <t>유가 변동 추이 및 물류비에 미치는 영향 분석, 유류 구매 계약 조건 검토 및 지정학적 리스크와의 연관성 분석.</t>
+        </is>
+      </c>
+      <c r="H210" s="3" t="inlineStr">
+        <is>
+          <t>이투데이</t>
+        </is>
+      </c>
+      <c r="I210" s="3" t="inlineStr">
+        <is>
+          <t>https://www.etoday.co.kr/news/view/2597900</t>
+        </is>
+      </c>
+      <c r="J210" s="3" t="inlineStr"/>
+    </row>
+    <row r="211">
+      <c r="A211" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B211" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C211" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D211" s="4" t="inlineStr">
+        <is>
+          <t>CZ, ‘B777’ 7대 발주 ‘중국적 항공사 최초’</t>
+        </is>
+      </c>
+      <c r="E211" s="4" t="inlineStr">
+        <is>
+          <t>중국남방항공이 보잉 777F 및 777-8F 화물기 7대를 발주하고, YTO카고항공이 지아싱-부다페스트 신규 화물 노선을 개설했다.</t>
+        </is>
+      </c>
+      <c r="F211" s="4" t="inlineStr">
+        <is>
+          <t>항공사의 화물기 도입 및 신규 노선 개설은 장기적인 항공 화물 공급 능력 증대에 기여할 수 있으나, 당장 우리 회사의 물류 운영에 직접적인 영향을 미치지는 않는다.</t>
+        </is>
+      </c>
+      <c r="G211" s="4" t="n"/>
+      <c r="H211" s="4" t="inlineStr">
+        <is>
+          <t>cargonews</t>
+        </is>
+      </c>
+      <c r="I211" s="4" t="inlineStr">
+        <is>
+          <t>https://www.cargonews.co.kr/news/articleView.html?idxno=60421</t>
+        </is>
+      </c>
+      <c r="J211" s="4" t="inlineStr"/>
+    </row>
+    <row r="212">
+      <c r="A212" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B212" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C212" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D212" s="4" t="inlineStr">
+        <is>
+          <t>IATA and IATP Collaborate to Support Airline Supply Chain Resilience</t>
+        </is>
+      </c>
+      <c r="E212" s="4" t="inlineStr">
+        <is>
+          <t>IATA와 IATP가 항공기 부품 가시성 및 접근성 개선을 위해 협력하여 항공 공급망 복원력을 지원하기로 합의했다.</t>
+        </is>
+      </c>
+      <c r="F212" s="4" t="inlineStr">
+        <is>
+          <t>항공기 부품 공급망 개선 노력은 장기적으로 항공 화물 운송 안정성에 긍정적 영향을 줄 수 있으나, 당장 우리 회사의 물류 운영에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G212" s="4" t="n"/>
+      <c r="H212" s="4" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I212" s="4" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-25-iata-iatp-collaborate-support-airline-supply-chain-resilience/</t>
+        </is>
+      </c>
+      <c r="J212" s="4" t="inlineStr"/>
+    </row>
+    <row r="213">
+      <c r="A213" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B213" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C213" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D213" s="4" t="inlineStr">
+        <is>
+          <t>IATA Outlines Four Priorities to Strengthen the Aviation Supply Chain</t>
+        </is>
+      </c>
+      <c r="E213" s="4" t="inlineStr">
+        <is>
+          <t>IATA는 항공 공급망 강화를 위한 네 가지 우선순위를 제시했다.</t>
+        </is>
+      </c>
+      <c r="F213" s="4" t="inlineStr">
+        <is>
+          <t>항공 공급망 강화 노력은 장기적인 관점에서 항공 운송 안정성에 긍정적이나, 당장 우리 회사의 물류 운영에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G213" s="4" t="n"/>
+      <c r="H213" s="4" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I213" s="4" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-24-iata-outlines-four-priorities-to-strengthen-aviation-supply-chain/</t>
+        </is>
+      </c>
+      <c r="J213" s="4" t="inlineStr"/>
+    </row>
+    <row r="214">
+      <c r="A214" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B214" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C214" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D214" s="4" t="inlineStr">
+        <is>
+          <t>States and Supporting Partners Join IATA’s Alliance to Expand CORSIA Carbon Credit Supply</t>
+        </is>
+      </c>
+      <c r="E214" s="4" t="inlineStr">
+        <is>
+          <t>IATA는 CORSIA 탄소 배출권 공급 확대를 위한 연합에 더 많은 국가 및 파트너들이 참여했다고 발표했다.</t>
+        </is>
+      </c>
+      <c r="F214" s="4" t="inlineStr">
+        <is>
+          <t>CORSIA 탄소 배출권 관련 소식은 항공 산업의 환경 규제 준수와 관련되나, 당장 우리 회사의 물류 운영에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G214" s="4" t="n"/>
+      <c r="H214" s="4" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I214" s="4" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-23-states-supporting-partners-join-iata-alliance-expand-corsia-carbon-credit-supply/</t>
+        </is>
+      </c>
+      <c r="J214" s="4" t="inlineStr"/>
+    </row>
+    <row r="215">
+      <c r="A215" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B215" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C215" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D215" s="4" t="inlineStr">
+        <is>
+          <t>고려해운, 日–韓–큐슈 노선 ‘JKW4’로 일원화</t>
+        </is>
+      </c>
+      <c r="E215" s="4" t="inlineStr">
+        <is>
+          <t>고려해운이 기존 JKW3과 JKW4 노선을 JKW4로 통합하고 야쓰시로항 기항을 주 1회로 확대하여 일본-한국-큐슈 항로 서비스를 개편했다.</t>
+        </is>
+      </c>
+      <c r="F215" s="4" t="inlineStr">
+        <is>
+          <t>특정 선사의 노선 개편은 해당 노선을 이용하는 경우 서비스 개선 효과가 있을 수 있으나, 우리 회사의 주요 운송 경로에 직접적인 영향은 미미하다.</t>
+        </is>
+      </c>
+      <c r="G215" s="4" t="n"/>
+      <c r="H215" s="4" t="inlineStr">
+        <is>
+          <t>kita</t>
+        </is>
+      </c>
+      <c r="I215" s="4" t="inlineStr">
+        <is>
+          <t>https://www.kita.net/shippers/board/newsView.do?morgueCode=2&amp;dataCls=B&amp;dataSeq=8137</t>
+        </is>
+      </c>
+      <c r="J215" s="4" t="inlineStr"/>
+    </row>
+    <row r="216">
+      <c r="A216" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B216" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C216" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D216" s="4" t="inlineStr">
+        <is>
+          <t>인도네시아 산업분류체계(KBLI) 2025 개정</t>
+        </is>
+      </c>
+      <c r="E216" s="4" t="inlineStr">
+        <is>
+          <t>인도네시아 통계청이 사업자 등록, 허가, 외국인 투자 신청 등에 활용되는 산업분류체계(KBLI) 2020을 전면 개정한 KBLI 2025를 공표했다.</t>
+        </is>
+      </c>
+      <c r="F216" s="4" t="inlineStr">
+        <is>
+          <t>인도네시아 산업분류체계 개정은 현지 사업 활동 및 투자 절차에 영향을 미치지만, 우리 회사의 직접적인 물류 운영에는 당장 영향이 없다.</t>
+        </is>
+      </c>
+      <c r="G216" s="4" t="n"/>
+      <c r="H216" s="4" t="inlineStr">
+        <is>
+          <t>kotra</t>
+        </is>
+      </c>
+      <c r="I216" s="4" t="inlineStr">
+        <is>
+          <t>https://dream.kotra.or.kr/kotranews/cms/news/actionKotraBoardDetail.do?SITE_NO=3&amp;MENU_ID=70&amp;CONTENTS_NO=1&amp;pNttSn=242416</t>
+        </is>
+      </c>
+      <c r="J216" s="4" t="inlineStr"/>
+    </row>
+    <row r="217">
+      <c r="A217" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B217" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C217" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D217" s="4" t="inlineStr">
+        <is>
+          <t>Transpacific: Ripe for new non-alliance services</t>
+        </is>
+      </c>
+      <c r="E217" s="4" t="inlineStr">
+        <is>
+          <t>아시아-북미 서안 항로의 컨테이너 스팟 운임과 비동맹 선사의 선박 용량 점유율 분석 결과, 새로운 비동맹 서비스의 출현 가능성이 높다는 분석입니다.</t>
+        </is>
+      </c>
+      <c r="F217" s="4" t="inlineStr">
+        <is>
+          <t>시장 분석 보고서로, 즉각적인 물류 운영 영향보다는 장기적인 시장 동향 참고 수준입니다.</t>
+        </is>
+      </c>
+      <c r="G217" s="4" t="n"/>
+      <c r="H217" s="4" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I217" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/393-transpacific-ripe-for-new-non-alliance-services</t>
+        </is>
+      </c>
+      <c r="J217" s="4" t="inlineStr"/>
+    </row>
+    <row r="218">
+      <c r="A218" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B218" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C218" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D218" s="4" t="inlineStr">
+        <is>
+          <t>Decoding Gemini’s Mediterranean Surge</t>
+        </is>
+      </c>
+      <c r="E218" s="4" t="inlineStr">
+        <is>
+          <t>Gemini Cooperation이 동서 컨테이너 선박 배치를 재조정하며 전반적인 시장 점유율은 감소했지만, 지중해 지역에서는 선박 배치를 늘려 시장 점유율이 급증했습니다.</t>
+        </is>
+      </c>
+      <c r="F218" s="4" t="inlineStr">
+        <is>
+          <t>특정 해운 동맹의 전략 변화 분석으로, 우리 회사의 지중해 노선 의존도가 높지 않다면 직접적인 영향은 낮습니다.</t>
+        </is>
+      </c>
+      <c r="G218" s="4" t="n"/>
+      <c r="H218" s="4" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I218" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/392-decoding-gemini-s-mediterranean-surge</t>
+        </is>
+      </c>
+      <c r="J218" s="4" t="inlineStr"/>
+    </row>
+    <row r="219">
+      <c r="A219" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B219" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C219" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D219" s="4" t="inlineStr">
+        <is>
+          <t>2026-Q1: NAEC Ports Consolidate Market Share</t>
+        </is>
+      </c>
+      <c r="E219" s="4" t="inlineStr">
+        <is>
+          <t>2026년 1분기 북미 동부 해안(NAEC) 항만의 컨테이너 물동량은 전년 대비 감소했으나, NAEC 항만들이 시장 점유율을 통합하는 경향을 보였습니다.</t>
+        </is>
+      </c>
+      <c r="F219" s="4" t="inlineStr">
+        <is>
+          <t>과거 데이터 분석으로, 현재 항만 운영에 대한 즉각적인 영향보다는 장기적인 항만 전략 수립에 참고할 정보입니다.</t>
+        </is>
+      </c>
+      <c r="G219" s="4" t="n"/>
+      <c r="H219" s="4" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I219" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/391-2026-q1-naec-ports-consolidate-market-share</t>
+        </is>
+      </c>
+      <c r="J219" s="4" t="inlineStr"/>
+    </row>
+    <row r="220">
+      <c r="A220" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B220" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C220" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D220" s="4" t="inlineStr">
+        <is>
+          <t>Global Schedule Reliability for April 2026 the Highest of the Year</t>
+        </is>
+      </c>
+      <c r="E220" s="4" t="inlineStr">
+        <is>
+          <t>2026년 4월 글로벌 선박 스케줄 신뢰도가 올해 최고치를 기록하여 해상 운송의 정시성이 개선되고 있음을 보여줍니다.</t>
+        </is>
+      </c>
+      <c r="F220" s="4" t="inlineStr">
+        <is>
+          <t>과거 데이터 기반의 긍정적인 추세 보고로, 즉각적인 조치보다는 지속적인 모니터링을 통해 운송 계획에 반영할 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G220" s="4" t="n"/>
+      <c r="H220" s="4" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I220" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/390-global-schedule-reliability-for-april-2026-the-highest-of-the-year</t>
+        </is>
+      </c>
+      <c r="J220" s="4" t="inlineStr"/>
+    </row>
+    <row r="221">
+      <c r="A221" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B221" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C221" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D221" s="4" t="inlineStr">
+        <is>
+          <t>씨메스로보틱스 / ‘물류·제조 대형 수주 잇달아’ 피지컬 AI 기반 로봇 자동화 사업 가속</t>
+        </is>
+      </c>
+      <c r="E221" s="4" t="inlineStr">
+        <is>
+          <t>씨메스로보틱스가 물류 및 제조 현장에서 피지컬 AI 기반 로봇 자동화 대형 프로젝트를 연이어 수주하며 사업을 확대하고, 1분기 사상 최대 매출을 달성했습니다.</t>
+        </is>
+      </c>
+      <c r="F221" s="4" t="inlineStr">
+        <is>
+          <t>물류 자동화 기술 동향에 대한 정보로, 당사의 즉각적인 물류 운영에 영향을 미치기보다는 장기적인 관점에서 참고할 만한 내용입니다.</t>
+        </is>
+      </c>
+      <c r="G221" s="4" t="n"/>
+      <c r="H221" s="4" t="inlineStr">
+        <is>
+          <t>ulogistics</t>
+        </is>
+      </c>
+      <c r="I221" s="4" t="inlineStr">
+        <is>
+          <t>http://www.ulogistics.co.kr/test/board.php?board=all2&amp;command=body&amp;no=5202</t>
+        </is>
+      </c>
+      <c r="J221" s="4" t="inlineStr"/>
+    </row>
+    <row r="222">
+      <c r="A222" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B222" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C222" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D222" s="4" t="inlineStr">
+        <is>
+          <t>[르포] ‘시간당 400개 생산’ 차단기 라인에 사람은 단 한명…전력기기 업계 최초 물류 AI 도입 - 헤럴드경제</t>
+        </is>
+      </c>
+      <c r="E222" s="4" t="inlineStr">
+        <is>
+          <t>HD현대일렉트릭이 전력기기 업계 최초로 물류 AI를 도입하여 생산 라인의 자동화율을 높이고 효율성을 극대화하고 있다. 이는 생산성 향상과 물류 최적화에 기여할 것으로 보인다.</t>
+        </is>
+      </c>
+      <c r="F222" s="4" t="inlineStr">
+        <is>
+          <t>타사의 물류 AI 도입 사례는 우리 회사의 물류 운영에 직접적인 영향을 주지는 않지만, 장기적인 관점에서 물류 효율화 및 기술 도입을 위한 참고 자료가 될 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G222" s="4" t="inlineStr"/>
+      <c r="H222" s="4" t="inlineStr">
+        <is>
+          <t>헤럴드경제</t>
+        </is>
+      </c>
+      <c r="I222" s="4" t="inlineStr">
+        <is>
+          <t>https://biz.heraldcorp.com/article/10789729</t>
+        </is>
+      </c>
+      <c r="J222" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9682,7 +10942,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9915,6 +11175,49 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>3239.64</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>+118 (+3.8%)</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>+1,151 (+55.1%)</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>3747</v>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>+398 (+11.9%)</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>+940 (+33.5%)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9927,7 +11230,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10863,6 +12166,146 @@
       </c>
       <c r="I26" s="6" t="inlineStr"/>
     </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>RSK-026</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>북미항로/ ‘관세대응 영향’ 물동량 9개월만에 플러스성장</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr"/>
+      <c r="G27" s="6" t="inlineStr"/>
+      <c r="H27" s="6" t="inlineStr">
+        <is>
+          <t>북미향 선적 계획 긴급 점검 및 대체 운송 방안 모색, 운임 변동성 대비 예산 조정, 관세 부과 대상 품목 및 시기 확인.</t>
+        </is>
+      </c>
+      <c r="I27" s="6" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>RSK-027</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 물류 불확실성 지속: 한국 선박 3척 잔류, 해상운임 9주 연속 상승</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr"/>
+      <c r="G28" s="6" t="inlineStr"/>
+      <c r="H28" s="6" t="inlineStr">
+        <is>
+          <t>중동 경유 선박의 운항 스케줄 및 경로 재확인, 대체 운송 경로(예: 육상, 항공) 및 운송사 옵션 검토, 비상 재고 수준 점검 및 확보, 운임 변동성 모니터링 강화.</t>
+        </is>
+      </c>
+      <c r="I28" s="6" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>RSK-028</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>연합뉴스TV</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="inlineStr"/>
+      <c r="G29" s="6" t="inlineStr"/>
+      <c r="H29" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈 해협을 경유하는 운송 계획을 즉시 점검하고, 대체 항로 및 운송 수단 확보 가능성을 타진하며, 비상 재고 수준을 검토해야 합니다.</t>
+        </is>
+      </c>
+      <c r="I29" s="6" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>RSK-029</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
+        <is>
+          <t>'호르무즈 통제' 놓고 보복 난타전 … 美·이란 다시 전면전 위기</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr"/>
+      <c r="G30" s="6" t="inlineStr"/>
+      <c r="H30" s="6" t="inlineStr">
+        <is>
+          <t>해상 운송 경로 및 운임 변동성 모니터링 강화, 비상 운송 계획 검토, 유류 재고 및 구매 전략 점검.</t>
+        </is>
+      </c>
+      <c r="I30" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
📰 뉴스 데이터 2026-06-29_21:05
</commit_message>
<xml_diff>
--- a/data/SCM_물류_브리핑.xlsx
+++ b/data/SCM_물류_브리핑.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J222"/>
+  <dimension ref="A1:J249"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10929,6 +10929,1282 @@
         </is>
       </c>
       <c r="J222" s="4" t="inlineStr"/>
+    </row>
+    <row r="223">
+      <c r="A223" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B223" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C223" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D223" s="2" t="inlineStr">
+        <is>
+          <t>DOJ Appeals CIT's IEEPA Refund Injunction as CAPE Phase 2 Targets June 29; TPEB Rates Surge 30% Into Peak (GLOBAL LOGISTICS UPDATE)</t>
+        </is>
+      </c>
+      <c r="E223" s="2" t="inlineStr">
+        <is>
+          <t>법무부가 IEEPA 환급 금지 명령에 항소하고 CAPE Phase 2가 6월 29일 시행될 예정인 가운데, 성수기 진입으로 태평양 횡단 동향(TPEB) 운임이 30% 급등했습니다.</t>
+        </is>
+      </c>
+      <c r="F223" s="2" t="inlineStr">
+        <is>
+          <t>TPEB 운임 30% 급등은 즉각적인 물류 비용 상승을 야기하며, IEEPA 환급 관련 법적 분쟁은 향후 관세 환급 가능성에 불확실성을 더합니다.</t>
+        </is>
+      </c>
+      <c r="G223" s="2" t="inlineStr">
+        <is>
+          <t>급등하는 TPEB 운임에 대한 단기 및 중장기 대응 전략(예: 선사 계약 재검토, 운송 방식 다변화)을 수립하고, IEEPA 환급 관련 법적 진행 상황을 면밀히 주시해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H223" s="2" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I223" s="2" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/june-11-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J223" s="2" t="inlineStr">
+        <is>
+          <t>RSK-030</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B224" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C224" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D224" s="2" t="inlineStr">
+        <is>
+          <t>KOBC컨테이너운임종합지수(KCCI), 29일 3920달러로 전주대비 173달러(4.62%) 상승</t>
+        </is>
+      </c>
+      <c r="E224" s="2" t="inlineStr">
+        <is>
+          <t>한국해양진흥공사의 KOBC컨테이너운임종합지수(KCCI)가 전주 대비 4.62% 상승한 3920달러를 기록하며, 주요 원양 및 중장거리 항로 운임이 모두 올랐다.</t>
+        </is>
+      </c>
+      <c r="F224" s="2" t="inlineStr">
+        <is>
+          <t>주요 항로 운임이 지속적으로 상승하고 있어 우리 회사의 물류 비용에 직접적인 영향을 미치므로, 즉각적인 운송 계획 및 예산 검토가 필요하다.</t>
+        </is>
+      </c>
+      <c r="G224" s="2" t="inlineStr">
+        <is>
+          <t>운송 계약 조건 재검토, 대체 운송 방안 모색, 운임 상승분 반영한 예산 조정 검토.</t>
+        </is>
+      </c>
+      <c r="H224" s="2" t="inlineStr">
+        <is>
+          <t>Shippingnewsnet</t>
+        </is>
+      </c>
+      <c r="I224" s="2" t="inlineStr">
+        <is>
+          <t>https://www.shippingnewsnet.com/news/articleView.html?idxno=70948</t>
+        </is>
+      </c>
+      <c r="J224" s="2" t="inlineStr">
+        <is>
+          <t>RSK-031</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B225" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C225" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D225" s="2" t="inlineStr">
+        <is>
+          <t>미-이란, 호르무즈 무력 충돌 재개...종전 합의 9일 만</t>
+        </is>
+      </c>
+      <c r="E225" s="2" t="inlineStr">
+        <is>
+          <t>미국과 이란의 호르무즈 해협 무력 충돌이 종전 합의 9일 만에 재개되고 이스라엘의 추가 공격까지 겹치며 중동발 에너지 및 해상 운송 리스크가 다시 확대되고 있다.</t>
+        </is>
+      </c>
+      <c r="F225" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협의 지정학적 긴장 재고조는 주요 해상 운송로의 안전을 위협하고 운송 지연 및 비용 상승을 유발할 수 있어 즉각적인 대응이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G225" s="2" t="inlineStr">
+        <is>
+          <t>중동 항로 이용 시 대체 경로 및 운송 수단 검토, 운송 보험 확인, 실시간 운항 정보 모니터링 강화.</t>
+        </is>
+      </c>
+      <c r="H225" s="2" t="inlineStr">
+        <is>
+          <t>Surff</t>
+        </is>
+      </c>
+      <c r="I225" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260628-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J225" s="2" t="inlineStr">
+        <is>
+          <t>RSK-032</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B226" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C226" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D226" s="2" t="inlineStr">
+        <is>
+          <t>"트럼프 신규 관세 피하자"…기업들 선적 경쟁에 해상 운임 급등</t>
+        </is>
+      </c>
+      <c r="E226" s="2" t="inlineStr">
+        <is>
+          <t>트럼프의 신규 관세 부과를 피하기 위한 기업들의 선적 경쟁이 심화되면서 해상 운임이 급등하고 있다.</t>
+        </is>
+      </c>
+      <c r="F226" s="2" t="inlineStr">
+        <is>
+          <t>잠재적 관세 부과에 대한 선제적 대응으로 인한 선적 경쟁은 해상 운임 상승과 운송 지연을 유발하여 우리 회사의 물류 비용 및 계획에 직접적인 영향을 미친다.</t>
+        </is>
+      </c>
+      <c r="G226" s="2" t="inlineStr">
+        <is>
+          <t>관세 부과 가능성 있는 품목 및 지역 확인, 운송 계획 조정, 운임 변동성 대비 예산 검토.</t>
+        </is>
+      </c>
+      <c r="H226" s="2" t="inlineStr">
+        <is>
+          <t>Newspim</t>
+        </is>
+      </c>
+      <c r="I226" s="2" t="inlineStr">
+        <is>
+          <t>https://www.newspim.com/news/view/20260629001067</t>
+        </is>
+      </c>
+      <c r="J226" s="2" t="inlineStr">
+        <is>
+          <t>RSK-033</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B227" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C227" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D227" s="3" t="inlineStr">
+        <is>
+          <t>CAPE Phase 2 Launches June 29 for Reconciliation-Flagged Entries; TPEB Rates Rise 10% for Sixth Consecutive Week (GLOBAL LOGISTICS UPDATE)</t>
+        </is>
+      </c>
+      <c r="E227" s="3" t="inlineStr">
+        <is>
+          <t>미국 CBP가 IEEPA 관세 환급 시스템인 CAPE Phase 2를 6월 29일 확장 적용하며, 태평양 횡단 동향(TPEB) 운임이 6주 연속 10% 상승했습니다.</t>
+        </is>
+      </c>
+      <c r="F227" s="3" t="inlineStr">
+        <is>
+          <t>TPEB 해상 운임의 지속적인 상승은 물류 비용 증가로 이어질 수 있으며, CAPE Phase 2는 관세 환급 절차에 영향을 미치므로 지속적인 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G227" s="3" t="inlineStr">
+        <is>
+          <t>해상 운임 상승 추이를 면밀히 주시하고, CAPE Phase 2를 통한 관세 환급 가능성을 검토하여 비용 절감 방안을 모색해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H227" s="3" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I227" s="3" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/june-25-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J227" s="3" t="inlineStr"/>
+    </row>
+    <row r="228">
+      <c r="A228" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B228" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C228" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D228" s="3" t="inlineStr">
+        <is>
+          <t>CPSC Mandatory eFiling Takes Effect July 8; TPEB Rates Surge ~10% as Peak Season Demand Outpaces Capacity (GLOBAL LOGISTICS UPDATE)</t>
+        </is>
+      </c>
+      <c r="E228" s="3" t="inlineStr">
+        <is>
+          <t>미국 소비자제품안전위원회(CPSC)의 의무 전자신고가 7월 8일 발효되며, CBP는 강제 노동 관련 통합 지침을 발표했습니다. 또한, 성수기 수요가 공급을 초과하면서 태평양 횡단 동향(TPEB) 운임이 약 10% 급등했습니다.</t>
+        </is>
+      </c>
+      <c r="F228" s="3" t="inlineStr">
+        <is>
+          <t>TPEB 운임 급등은 물류 비용에 직접적인 영향을 미치고, CPSC 전자신고 의무화 및 강제 노동 지침은 통관 절차 및 공급망 실사에 대한 추가적인 주의를 요구합니다.</t>
+        </is>
+      </c>
+      <c r="G228" s="3" t="inlineStr">
+        <is>
+          <t>TPEB 운임 변동을 주시하고, CPSC 전자신고 시스템 준비 및 CBP의 강제 노동 지침에 따른 공급망 실사 강화 방안을 검토해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H228" s="3" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I228" s="3" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/june-18-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J228" s="3" t="inlineStr"/>
+    </row>
+    <row r="229">
+      <c r="A229" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B229" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C229" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D229" s="3" t="inlineStr">
+        <is>
+          <t>U.S. Appeals CIT's IEEPA Refund Order to Federal Circuit; TPEB Rates Rise as Peak Season Demand Tightens Capacity (GLOBAL LOGISTICS UPDATE)</t>
+        </is>
+      </c>
+      <c r="E229" s="3" t="inlineStr">
+        <is>
+          <t>미국 정부가 IEEPA 환급 명령에 항소하고 트럼프 대통령이 세관 집행 개혁 행정명령에 서명한 가운데, 성수기 수요로 인해 태평양 횡단 동향(TPEB) 운임이 상승하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F229" s="3" t="inlineStr">
+        <is>
+          <t>TPEB 운임 상승은 물류 비용에 영향을 미치고, 세관 집행 개혁 및 IEEPA 환급 관련 항소는 수입 절차 및 관세 환급 가능성에 변화를 가져올 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G229" s="3" t="inlineStr">
+        <is>
+          <t>TPEB 운임 추이를 지속적으로 모니터링하고, 세관 집행 강화 및 IOR(Importer of Record) 요건 변경 가능성에 대비하여 통관 절차를 검토해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H229" s="3" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I229" s="3" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/june-3-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J229" s="3" t="inlineStr"/>
+    </row>
+    <row r="230">
+      <c r="A230" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B230" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C230" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D230" s="3" t="inlineStr">
+        <is>
+          <t>Section 232 Duties Reduced to 15% for Taiwanese Goods, Retroactive to May 1; China Air Rates Spike on Supply Contraction and Month-End Demand (GLOBAL LOGISTICS UPDATE)</t>
+        </is>
+      </c>
+      <c r="E230" s="3" t="inlineStr">
+        <is>
+          <t>대만산 특정 품목에 대한 Section 232 관세가 15%로 인하되어 5월 1일부로 소급 적용되며, 공급 감소와 월말 수요로 인해 중국발 항공 운임이 급등했습니다.</t>
+        </is>
+      </c>
+      <c r="F230" s="3" t="inlineStr">
+        <is>
+          <t>중국발 항공 운임 급등은 항공 운송 비용에 직접적인 영향을 미치며, 대만산 품목 관세 인하는 해당 품목을 취급하는 경우 긍정적이지만 전반적인 지정학적 리스크는 여전히 존재합니다.</t>
+        </is>
+      </c>
+      <c r="G230" s="3" t="inlineStr">
+        <is>
+          <t>중국발 항공 운임 변동을 주시하고, 대만산 부품/제품 수입 시 관세 인하 혜택을 확인하여 비용 절감 기회를 모색해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H230" s="3" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I230" s="3" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/may-28-2026-cit-rejects-governments-stay-request/</t>
+        </is>
+      </c>
+      <c r="J230" s="3" t="inlineStr"/>
+    </row>
+    <row r="231">
+      <c r="A231" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B231" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C231" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D231" s="3" t="inlineStr">
+        <is>
+          <t>Air Cargo Demand up 6.0% in May (PRESSROOM)</t>
+        </is>
+      </c>
+      <c r="E231" s="3" t="inlineStr">
+        <is>
+          <t>국제항공운송협회(IATA)에 따르면 2026년 5월 전 세계 항공 화물 수요가 전년 대비 6.0% 증가했으며, 국제선 운영은 6.5% 증가했습니다.</t>
+        </is>
+      </c>
+      <c r="F231" s="3" t="inlineStr">
+        <is>
+          <t>항공 화물 수요 증가는 향후 항공 운임 상승 압력으로 작용할 수 있으며, 이는 배터리/전자부품의 항공 운송 비용에 영향을 미칠 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G231" s="3" t="inlineStr">
+        <is>
+          <t>항공 화물 운임 추이를 지속적으로 모니터링하고, 필요시 항공 운송 계약 조건을 검토하여 비용 변동에 대비해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H231" s="3" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I231" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-29-air-cargo-demand-up-may/</t>
+        </is>
+      </c>
+      <c r="J231" s="3" t="inlineStr"/>
+    </row>
+    <row r="232">
+      <c r="A232" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B232" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C232" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D232" s="3" t="inlineStr">
+        <is>
+          <t>Urgent Action Needed to Ease Engine MRO Bottlenecks (PRESSROOM)</t>
+        </is>
+      </c>
+      <c r="E232" s="3" t="inlineStr">
+        <is>
+          <t>IATA는 항공기 엔진 유지보수(MRO) 병목 현상을 완화하기 위한 긴급 조치가 필요하다고 강조했습니다.</t>
+        </is>
+      </c>
+      <c r="F232" s="3" t="inlineStr">
+        <is>
+          <t>엔진 MRO 병목 현상은 항공기 가용성을 감소시켜 항공 화물 운송 능력에 부정적인 영향을 미칠 수 있으며, 이는 운임 상승이나 운송 지연으로 이어질 가능성이 있습니다.</t>
+        </is>
+      </c>
+      <c r="G232" s="3" t="inlineStr">
+        <is>
+          <t>항공 화물 운송 시장의 공급 능력 변화를 주시하고, 잠재적인 운송 지연이나 운임 상승에 대비하여 운송 계획을 유연하게 수립해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H232" s="3" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I232" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-24-urgent-action-needed-to-ease-engine-mro-bottlenecks/</t>
+        </is>
+      </c>
+      <c r="J232" s="3" t="inlineStr"/>
+    </row>
+    <row r="233">
+      <c r="A233" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B233" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C233" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D233" s="3" t="inlineStr">
+        <is>
+          <t>IATA Outlines Four Priorities to Strengthen the Aviation Supply Chain (PRESSROOM)</t>
+        </is>
+      </c>
+      <c r="E233" s="3" t="inlineStr">
+        <is>
+          <t>IATA는 항공 공급망 강화를 위한 네 가지 우선순위를 제시했으며, 이는 항공기 부품 부족, 엔진 MRO 병목 현상, 지상 조업 인력 부족 등의 문제를 해결하는 데 중점을 둡니다.</t>
+        </is>
+      </c>
+      <c r="F233" s="3" t="inlineStr">
+        <is>
+          <t>항공 공급망 강화 노력은 장기적으로 항공 화물 운송의 안정성과 효율성을 높일 수 있으나, 단기적인 우리 물류 운영에 미치는 직접적인 영향은 제한적입니다.</t>
+        </is>
+      </c>
+      <c r="G233" s="3" t="inlineStr">
+        <is>
+          <t>항공 공급망 개선 동향을 참고하여 장기적인 운송 전략 수립에 활용할 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="H233" s="3" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I233" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-24-iata-outlines-four-priorities-to-strengthen-aviation-supply-chain/</t>
+        </is>
+      </c>
+      <c r="J233" s="3" t="inlineStr"/>
+    </row>
+    <row r="234">
+      <c r="A234" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B234" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C234" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D234" s="3" t="inlineStr">
+        <is>
+          <t>WMES 2026 Speech - Stuart Fox, IATA's Director Flight and Operations (PRESSROOM)</t>
+        </is>
+      </c>
+      <c r="E234" s="3" t="inlineStr">
+        <is>
+          <t>IATA 연설에서 항공기 납기 지연, 엔진 유지보수 문제, 예비 부품 확보 난항, 수리 기간 증가 등 항공사들이 직면한 현실적인 공급망 문제를 지적하며 항공 운송 능력에 대한 우려를 표명했습니다.</t>
+        </is>
+      </c>
+      <c r="F234" s="3" t="inlineStr">
+        <is>
+          <t>항공기 및 부품 공급망의 지속적인 문제는 항공 화물 운송 능력 감소와 운송 지연 가능성을 높여 우리 물류 운영에 간접적인 영향을 미칠 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G234" s="3" t="inlineStr">
+        <is>
+          <t>항공 화물 운송 시장의 공급 제약 요인을 지속적으로 주시하고, 잠재적인 운송 지연 및 운임 상승에 대비하여 운송 계획을 유연하게 조정할 필요가 있습니다.</t>
+        </is>
+      </c>
+      <c r="H234" s="3" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I234" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-speeches/06-24-wmes-2026-speech-stuart-fox-iata-director-flight-operations/</t>
+        </is>
+      </c>
+      <c r="J234" s="3" t="inlineStr"/>
+    </row>
+    <row r="235">
+      <c r="A235" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B235" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C235" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D235" s="3" t="inlineStr">
+        <is>
+          <t>Global Schedule Reliability for May 2026 the Highest of the Year (PRESS ROOM)</t>
+        </is>
+      </c>
+      <c r="E235" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence 보고서에 따르면 2026년 5월 전 세계 선박 스케줄 신뢰도가 올해 최고치를 기록하여 해상 운송의 정시성이 개선되었습니다.</t>
+        </is>
+      </c>
+      <c r="F235" s="3" t="inlineStr">
+        <is>
+          <t>선박 스케줄 신뢰도 개선은 해상 운송의 예측 가능성을 높여 물류 계획 수립에 긍정적이나, 여전히 변동성이 존재하므로 지속적인 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G235" s="3" t="inlineStr">
+        <is>
+          <t>해상 운송 스케줄 신뢰도 개선 추이를 참고하여 운송 계획의 정확도를 높이고, 잠재적인 지연 리스크를 지속적으로 관리해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H235" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I235" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/395-global-schedule-reliability-for-may-2026-the-highest-of-the-year</t>
+        </is>
+      </c>
+      <c r="J235" s="3" t="inlineStr"/>
+    </row>
+    <row r="236">
+      <c r="A236" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B236" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C236" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D236" s="3" t="inlineStr">
+        <is>
+          <t>Tracking True Vessel Delay</t>
+        </is>
+      </c>
+      <c r="E236" s="3" t="inlineStr">
+        <is>
+          <t>해운사들이 선박 스케줄 버퍼를 늘려 운송 시간을 연장하고 있으며, 이는 실제 선박 지연에 영향을 미치고 있다.</t>
+        </is>
+      </c>
+      <c r="F236" s="3" t="inlineStr">
+        <is>
+          <t>선박 지연의 구조적 요인 분석으로, 장기적인 운송 계획 및 재고 관리에 잠재적 영향을 미칠 수 있어 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G236" s="3" t="n"/>
+      <c r="H236" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I236" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/394-tracking-true-vessel-delay</t>
+        </is>
+      </c>
+      <c r="J236" s="3" t="inlineStr"/>
+    </row>
+    <row r="237">
+      <c r="A237" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B237" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C237" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D237" s="3" t="inlineStr">
+        <is>
+          <t>Transpacific: Ripe for new non-alliance services</t>
+        </is>
+      </c>
+      <c r="E237" s="3" t="inlineStr">
+        <is>
+          <t>아시아-북미 서안 항로에서 컨테이너 스팟 운임과 비동맹 선사의 선박 용량 간의 관계를 분석하며, 새로운 비동맹 서비스의 출현 가능성을 시사한다.</t>
+        </is>
+      </c>
+      <c r="F237" s="3" t="inlineStr">
+        <is>
+          <t>새로운 서비스 출현은 운임 경쟁 심화 및 서비스 선택지 확대로 이어질 수 있으므로, 향후 운송 전략 수립에 참고하기 위해 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G237" s="3" t="n"/>
+      <c r="H237" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I237" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/393-transpacific-ripe-for-new-non-alliance-services</t>
+        </is>
+      </c>
+      <c r="J237" s="3" t="inlineStr"/>
+    </row>
+    <row r="238">
+      <c r="A238" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B238" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C238" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D238" s="3" t="inlineStr">
+        <is>
+          <t>글로벌 선박 엔진 품귀…韓 조선업계 반사이익 기대</t>
+        </is>
+      </c>
+      <c r="E238" s="3" t="inlineStr">
+        <is>
+          <t>기록적인 신조선 건조 물량으로 인해 전 세계적으로 선박 엔진 품귀 현상이 발생하고 있으며, 이는 장기적으로 선박 공급에 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="F238" s="3" t="inlineStr">
+        <is>
+          <t>선박 엔진 품귀는 신조선 인도 지연으로 이어져 장기적인 해운 시장의 선박 공급 부족을 심화시키고 운임에 영향을 줄 수 있으므로 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G238" s="3" t="n"/>
+      <c r="H238" s="3" t="inlineStr">
+        <is>
+          <t>EBN</t>
+        </is>
+      </c>
+      <c r="I238" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebn.co.kr/news/articleView.html?idxno=1714238</t>
+        </is>
+      </c>
+      <c r="J238" s="3" t="inlineStr"/>
+    </row>
+    <row r="239">
+      <c r="A239" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B239" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C239" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D239" s="3" t="inlineStr">
+        <is>
+          <t>공급 폭탄 앞둔 컨테이너선…해상 저장 ‘특수’ 유조선</t>
+        </is>
+      </c>
+      <c r="E239" s="3" t="inlineStr">
+        <is>
+          <t>향후 컨테이너선 공급 과잉이 예상되는 반면, 유조선은 해상 저장 용도로 특별한 수요를 맞고 있어 선종별 시장 상황이 상이하다.</t>
+        </is>
+      </c>
+      <c r="F239" s="3" t="inlineStr">
+        <is>
+          <t>컨테이너선 공급 과잉은 장기적으로 해상 운임 하락 요인이 될 수 있으므로, 향후 운송 계약 및 전략 수립에 참고하기 위해 시장 동향을 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G239" s="3" t="n"/>
+      <c r="H239" s="3" t="inlineStr">
+        <is>
+          <t>Newstomato</t>
+        </is>
+      </c>
+      <c r="I239" s="3" t="inlineStr">
+        <is>
+          <t>https://newstomato.com/ReadNews.aspx?no=1305485</t>
+        </is>
+      </c>
+      <c r="J239" s="3" t="inlineStr"/>
+    </row>
+    <row r="240">
+      <c r="A240" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B240" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C240" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D240" s="3" t="inlineStr">
+        <is>
+          <t>West Asian crisis hit Keralam’s air cargo exports from CIAL, Calicut airports</t>
+        </is>
+      </c>
+      <c r="E240" s="3" t="inlineStr">
+        <is>
+          <t>서아시아 분쟁으로 인해 케랄람 지역의 항공 화물 수출이 타격을 입어 운임 상승, 보험료 증가, 운송 시간 지연 및 공급망 불확실성이 커지고 있다.</t>
+        </is>
+      </c>
+      <c r="F240" s="3" t="inlineStr">
+        <is>
+          <t>중동 지역의 지정학적 리스크가 항공 운송 비용 및 시간에 직접적인 영향을 미치고 있어 우리 회사의 항공 물류 계획에 잠재적 영향을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="G240" s="3" t="inlineStr">
+        <is>
+          <t>중동 경유 항공 노선 및 대체 노선 운임/스케줄 변동 추이 모니터링, 비상 운송 계획 검토.</t>
+        </is>
+      </c>
+      <c r="H240" s="3" t="inlineStr">
+        <is>
+          <t>The HinduBusinessLine</t>
+        </is>
+      </c>
+      <c r="I240" s="3" t="inlineStr">
+        <is>
+          <t>https://www.thehindubusinessline.com/economy/logistics/west-asian-crisis-hit-keralams-air-cargo-exports-from-cial-calicut-airports/article71160558.ece</t>
+        </is>
+      </c>
+      <c r="J240" s="3" t="inlineStr"/>
+    </row>
+    <row r="241">
+      <c r="A241" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B241" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C241" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D241" s="3" t="inlineStr">
+        <is>
+          <t>일본 신칸센, 보조배터리 화재 진압도구 비치</t>
+        </is>
+      </c>
+      <c r="E241" s="3" t="inlineStr">
+        <is>
+          <t>일본 신칸센이 보조배터리 화재에 대비해 객실 내 화재 진압 장비를 비치하는 방안을 도입했다. 이는 항공기의 반입 금지 조치와는 다른 접근 방식이다.</t>
+        </is>
+      </c>
+      <c r="F241" s="3" t="inlineStr">
+        <is>
+          <t>배터리 화재 안전에 대한 사회적 관심과 규제 논의가 확산될 수 있으며, 이는 향후 배터리 운송 및 보관 규제 강화로 이어질 가능성이 있다.</t>
+        </is>
+      </c>
+      <c r="G241" s="3" t="inlineStr">
+        <is>
+          <t>배터리 운송 및 보관 관련 국내외 안전 규제 동향 지속 모니터링, 제품 안전성 강화 방안 검토.</t>
+        </is>
+      </c>
+      <c r="H241" s="3" t="inlineStr">
+        <is>
+          <t>ZDNet korea</t>
+        </is>
+      </c>
+      <c r="I241" s="3" t="inlineStr">
+        <is>
+          <t>https://zdnet.co.kr/view/?no=20260629100736</t>
+        </is>
+      </c>
+      <c r="J241" s="3" t="inlineStr"/>
+    </row>
+    <row r="242">
+      <c r="A242" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B242" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C242" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D242" s="3" t="inlineStr">
+        <is>
+          <t>미국이 구리 관세 카드를 다시 꺼낼 가능성이 높아지면서, 글로벌 구리 공급망 재편이 한국 기업의 조달 전략에도 직접적 변수가 될 공산이 커지고 있다.</t>
+        </is>
+      </c>
+      <c r="E242" s="3" t="inlineStr">
+        <is>
+          <t>미국이 구리 관세 카드를 다시 꺼낼 가능성이 높아지면서, 글로벌 구리 공급망 재편이 한국 기업의 원자재 조달 전략에 직접적인 변수가 될 수 있다.</t>
+        </is>
+      </c>
+      <c r="F242" s="3" t="inlineStr">
+        <is>
+          <t>구리는 배터리 및 전자부품 제조의 핵심 원자재이므로, 미국의 구리 관세 부과는 원자재 조달 비용 및 공급망 안정성에 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G242" s="3" t="inlineStr">
+        <is>
+          <t>구리 등 주요 원자재의 글로벌 공급망 및 가격 변동 추이 모니터링, 대체 조달처 확보 가능성 검토.</t>
+        </is>
+      </c>
+      <c r="H242" s="3" t="inlineStr">
+        <is>
+          <t>허프포스트코리아</t>
+        </is>
+      </c>
+      <c r="I242" s="3" t="inlineStr">
+        <is>
+          <t>https://huffingtonpost.kr/article/258311</t>
+        </is>
+      </c>
+      <c r="J242" s="3" t="inlineStr"/>
+    </row>
+    <row r="243">
+      <c r="A243" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B243" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C243" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D243" s="3" t="inlineStr">
+        <is>
+          <t>"제2의 국자원 화재, 제도적으로 막는다"</t>
+        </is>
+      </c>
+      <c r="E243" s="3" t="inlineStr">
+        <is>
+          <t>조달당국이 국가정보자원관리원 화재 사고를 계기로 리튬배터리 설치 등 높은 안전성이 요구되는 공공 공사 입찰에 관련 실적 있는 전문 업체만 참여하도록 발주 방식을 개선한다.</t>
+        </is>
+      </c>
+      <c r="F243" s="3" t="inlineStr">
+        <is>
+          <t>리튬배터리 관련 공공 프로젝트의 안전 규제 강화는 향후 우리 회사의 제품 설치 및 관련 서비스 제공 방식에 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G243" s="3" t="inlineStr">
+        <is>
+          <t>리튬배터리 관련 공공 프로젝트 안전 규제 동향 모니터링, 제품 설치 및 서비스 관련 안전 표준 준수 여부 점검.</t>
+        </is>
+      </c>
+      <c r="H243" s="3" t="inlineStr">
+        <is>
+          <t>이데일리</t>
+        </is>
+      </c>
+      <c r="I243" s="3" t="inlineStr">
+        <is>
+          <t>https://edaily.co.kr/News/Read?mediaCodeNo=257&amp;newsId=04306646645486640</t>
+        </is>
+      </c>
+      <c r="J243" s="3" t="inlineStr"/>
+    </row>
+    <row r="244">
+      <c r="A244" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B244" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C244" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D244" s="4" t="inlineStr">
+        <is>
+          <t>동해신항 석탄부두 건설로 원자재 공급기반 확충 (해운)</t>
+        </is>
+      </c>
+      <c r="E244" s="4" t="inlineStr">
+        <is>
+          <t>해양수산부가 동해신항에 10만DWT급 석탄부두 1선석을 조성하여 석탄 등 원자재 하역 능력과 항만 운영 효율을 높일 계획입니다.</t>
+        </is>
+      </c>
+      <c r="F244" s="4" t="inlineStr">
+        <is>
+          <t>석탄 부두 건설은 주로 에너지/원자재 산업에 영향을 미치며, 배터리/전자부품 물류에는 직접적인 영향이 없습니다.</t>
+        </is>
+      </c>
+      <c r="G244" s="4" t="n"/>
+      <c r="H244" s="4" t="inlineStr">
+        <is>
+          <t>kita</t>
+        </is>
+      </c>
+      <c r="I244" s="4" t="inlineStr">
+        <is>
+          <t>https://www.kita.net/shippers/board/newsView.do?morgueCode=2&amp;dataCls=B&amp;dataSeq=8139</t>
+        </is>
+      </c>
+      <c r="J244" s="4" t="inlineStr"/>
+    </row>
+    <row r="245">
+      <c r="A245" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B245" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C245" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D245" s="4" t="inlineStr">
+        <is>
+          <t>북극항로 시험운항 선박 '확보'…"8월 말 출항 유력" (해운/항만/물류 홈 산업 해운/항만/물류)</t>
+        </is>
+      </c>
+      <c r="E245" s="4" t="inlineStr">
+        <is>
+          <t>해양수산부가 북극항로 시험 운항을 위한 내빙 컨테이너선 확보에 성공했으며, 8월 말 출항이 유력하여 새로운 해상 운송 경로 개발 가능성을 열었습니다.</t>
+        </is>
+      </c>
+      <c r="F245" s="4" t="inlineStr">
+        <is>
+          <t>북극항로 시험 운항은 장기적인 운송 경로 다변화 가능성을 제시하지만, 현재 배터리/전자부품의 주요 운송 경로가 아니므로 당장 우리 물류 운영에 직접적인 영향은 없습니다.</t>
+        </is>
+      </c>
+      <c r="G245" s="4" t="n"/>
+      <c r="H245" s="4" t="inlineStr">
+        <is>
+          <t>oceanpress</t>
+        </is>
+      </c>
+      <c r="I245" s="4" t="inlineStr">
+        <is>
+          <t>https://www.oceanpress.co.kr/news/article.html?no=30469</t>
+        </is>
+      </c>
+      <c r="J245" s="4" t="inlineStr"/>
+    </row>
+    <row r="246">
+      <c r="A246" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B246" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C246" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D246" s="4" t="inlineStr">
+        <is>
+          <t>Decoding Gemini’s Mediterranean Surge</t>
+        </is>
+      </c>
+      <c r="E246" s="4" t="inlineStr">
+        <is>
+          <t>Gemini Cooperation이 동서 컨테이너 선박 배치에서 지중해 지역으로 선대를 재배치하고 있으며, 이는 시장 점유율 변화를 가져올 수 있다.</t>
+        </is>
+      </c>
+      <c r="F246" s="4" t="inlineStr">
+        <is>
+          <t>특정 선사의 선대 재배치 전략으로, 우리 회사의 주요 운송 경로에 직접적인 영향은 당장 없으므로 참고 수준이다.</t>
+        </is>
+      </c>
+      <c r="G246" s="4" t="n"/>
+      <c r="H246" s="4" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I246" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/392-decoding-gemini-s-mediterranean-surge</t>
+        </is>
+      </c>
+      <c r="J246" s="4" t="inlineStr"/>
+    </row>
+    <row r="247">
+      <c r="A247" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B247" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C247" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D247" s="4" t="inlineStr">
+        <is>
+          <t>씨메스로보틱스 / ‘물류·제조 대형 수주 잇달아’ 피지컬 AI 기반 로봇 자동화 사업 가속</t>
+        </is>
+      </c>
+      <c r="E247" s="4" t="inlineStr">
+        <is>
+          <t>씨메스로보틱스가 물류 및 제조 현장에서 피지컬 AI 기반 로봇 자동화 대형 프로젝트를 연이어 수주하며 사업을 확대하고 있다.</t>
+        </is>
+      </c>
+      <c r="F247" s="4" t="inlineStr">
+        <is>
+          <t>물류 자동화 기술 동향에 대한 정보로, 우리 회사의 현재 물류 운영에 직접적인 영향은 없으나 장기적인 관점에서 참고할 만하다.</t>
+        </is>
+      </c>
+      <c r="G247" s="4" t="n"/>
+      <c r="H247" s="4" t="inlineStr">
+        <is>
+          <t>Ulogistics</t>
+        </is>
+      </c>
+      <c r="I247" s="4" t="inlineStr">
+        <is>
+          <t>http://www.ulogistics.co.kr/test/board.php?board=all2&amp;command=body&amp;no=5202</t>
+        </is>
+      </c>
+      <c r="J247" s="4" t="inlineStr"/>
+    </row>
+    <row r="248">
+      <c r="A248" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B248" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C248" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D248" s="4" t="inlineStr">
+        <is>
+          <t>전력기기 다음은 배전…HD현대일렉, 로봇이 만들고 납기로 뚫는다</t>
+        </is>
+      </c>
+      <c r="E248" s="4" t="inlineStr">
+        <is>
+          <t>HD현대일렉트릭이 청주 배전캠퍼스에서 생산능력을 70% 늘리고 공장 자동화율을 높여 납기 준수를 강화하고 있다. 이는 AI 데이터센터발 전력 수요 증가에 대응하기 위한 전략이다.</t>
+        </is>
+      </c>
+      <c r="F248" s="4" t="inlineStr">
+        <is>
+          <t>우리 회사의 직접적인 물류 운영에 영향을 미치기보다는 타사의 생산 및 납기 전략에 대한 정보이다.</t>
+        </is>
+      </c>
+      <c r="G248" s="4" t="n"/>
+      <c r="H248" s="4" t="inlineStr">
+        <is>
+          <t>이투데이</t>
+        </is>
+      </c>
+      <c r="I248" s="4" t="inlineStr">
+        <is>
+          <t>https://etoday.co.kr/news/view/2597821</t>
+        </is>
+      </c>
+      <c r="J248" s="4" t="inlineStr"/>
+    </row>
+    <row r="249">
+      <c r="A249" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B249" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C249" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D249" s="4" t="inlineStr">
+        <is>
+          <t>AI-Powered Logistics Revolution: C.H. Robinson Unveils World's First Continuous AI System to Optimize &amp; Manage Global Supply Chains in Real-Time</t>
+        </is>
+      </c>
+      <c r="E249" s="4" t="inlineStr">
+        <is>
+          <t>C.H. Robinson이 날씨, 항만 적체, 지정학적 변화 등 글로벌 공급망 혼란을 실시간으로 최적화하고 관리하는 AI 시스템을 공개했다. 이 시스템은 물류 산업의 판도를 바꿀 잠재력이 있다.</t>
+        </is>
+      </c>
+      <c r="F249" s="4" t="inlineStr">
+        <is>
+          <t>현재 우리 회사의 물류 운영에 직접적인 영향을 미치기보다는 미래 물류 기술 동향에 대한 정보이다.</t>
+        </is>
+      </c>
+      <c r="G249" s="4" t="inlineStr">
+        <is>
+          <t>AI 기반 물류 솔루션 도입 가능성 및 시장 동향 지속 모니터링.</t>
+        </is>
+      </c>
+      <c r="H249" s="4" t="inlineStr">
+        <is>
+          <t>World Today Journal</t>
+        </is>
+      </c>
+      <c r="I249" s="4" t="inlineStr">
+        <is>
+          <t>https://www.world-today-journal.com/ai-powered-logistics-revolution-c-h-robinson-unveils-worlds-first-continuous-ai-system-to-optimize-manage-global-supply-chains-in-real-time/</t>
+        </is>
+      </c>
+      <c r="J249" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
@@ -11230,7 +12506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12306,6 +13582,146 @@
       </c>
       <c r="I30" s="6" t="inlineStr"/>
     </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>RSK-030</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="inlineStr">
+        <is>
+          <t>DOJ Appeals CIT's IEEPA Refund Injunction as CAPE Phase 2 Targets June 29; TPEB Rates Surge 30% Into Peak (GLOBAL LOGISTICS UPDATE)</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="inlineStr"/>
+      <c r="G31" s="6" t="inlineStr"/>
+      <c r="H31" s="6" t="inlineStr">
+        <is>
+          <t>급등하는 TPEB 운임에 대한 단기 및 중장기 대응 전략(예: 선사 계약 재검토, 운송 방식 다변화)을 수립하고, IEEPA 환급 관련 법적 진행 상황을 면밀히 주시해야 합니다.</t>
+        </is>
+      </c>
+      <c r="I31" s="6" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>RSK-031</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr">
+        <is>
+          <t>KOBC컨테이너운임종합지수(KCCI), 29일 3920달러로 전주대비 173달러(4.62%) 상승</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="inlineStr"/>
+      <c r="G32" s="6" t="inlineStr"/>
+      <c r="H32" s="6" t="inlineStr">
+        <is>
+          <t>운송 계약 조건 재검토, 대체 운송 방안 모색, 운임 상승분 반영한 예산 조정 검토.</t>
+        </is>
+      </c>
+      <c r="I32" s="6" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>RSK-032</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="inlineStr">
+        <is>
+          <t>미-이란, 호르무즈 무력 충돌 재개...종전 합의 9일 만</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="inlineStr"/>
+      <c r="G33" s="6" t="inlineStr"/>
+      <c r="H33" s="6" t="inlineStr">
+        <is>
+          <t>중동 항로 이용 시 대체 경로 및 운송 수단 검토, 운송 보험 확인, 실시간 운항 정보 모니터링 강화.</t>
+        </is>
+      </c>
+      <c r="I33" s="6" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>RSK-033</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E34" s="6" t="inlineStr">
+        <is>
+          <t>"트럼프 신규 관세 피하자"…기업들 선적 경쟁에 해상 운임 급등</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="inlineStr"/>
+      <c r="G34" s="6" t="inlineStr"/>
+      <c r="H34" s="6" t="inlineStr">
+        <is>
+          <t>관세 부과 가능성 있는 품목 및 지역 확인, 운송 계획 조정, 운임 변동성 대비 예산 검토.</t>
+        </is>
+      </c>
+      <c r="I34" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
📰 뉴스 데이터 2026-06-30_09:05
</commit_message>
<xml_diff>
--- a/data/SCM_물류_브리핑.xlsx
+++ b/data/SCM_물류_브리핑.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J249"/>
+  <dimension ref="A1:J283"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12206,6 +12206,1630 @@
       </c>
       <c r="J249" s="4" t="inlineStr"/>
     </row>
+    <row r="250">
+      <c r="A250" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B250" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C250" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D250" s="2" t="inlineStr">
+        <is>
+          <t>머스크, 올해 실적 전망 대폭 상향 조정</t>
+        </is>
+      </c>
+      <c r="E250" s="2" t="inlineStr">
+        <is>
+          <t>머스크가 예상보다 견조한 글로벌 컨테이너 물동량과 스팟 운임 강세를 반영하여 올해 실적 전망을 대폭 상향 조정했다.</t>
+        </is>
+      </c>
+      <c r="F250" s="2" t="inlineStr">
+        <is>
+          <t>주요 선사의 실적 상향 조정은 컨테이너 물동량 증가와 스팟 운임 강세에 기반하므로, 해상 운임 상승 압력이 높아져 우리 회사의 물류비에 직접적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G250" s="2" t="inlineStr">
+        <is>
+          <t>해상 운임 변동 추이 면밀히 모니터링 및 운송 계약 조건 재검토, 대체 운송 방안 또는 선사 다변화 검토</t>
+        </is>
+      </c>
+      <c r="H250" s="2" t="inlineStr">
+        <is>
+          <t>oceanpress</t>
+        </is>
+      </c>
+      <c r="I250" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oceanpress.co.kr/news/article.html?no=30472</t>
+        </is>
+      </c>
+      <c r="J250" s="2" t="inlineStr">
+        <is>
+          <t>RSK-034</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B251" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C251" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D251" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 내 한국 선박 2척 추가 탈출...3척만 남아</t>
+        </is>
+      </c>
+      <c r="E251" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 내 한국 선박 2척이 추가 탈출했으나 3척이 남아있어 중동발 물류 불확실성이 지속되고 있다.</t>
+        </is>
+      </c>
+      <c r="F251" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협의 불안정은 주요 해상 운송로의 지연 및 비용 증가를 야기하며, 원자재 수급 및 완제품 운송에 직접적인 영향을 미친다.</t>
+        </is>
+      </c>
+      <c r="G251" s="2" t="inlineStr">
+        <is>
+          <t>중동 경유 선박의 운항 현황을 실시간으로 확인하고, 필요시 대체 항로 또는 운송 수단 검토, 재고 수준 점검 및 비상 계획을 수립한다.</t>
+        </is>
+      </c>
+      <c r="H251" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I251" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260629-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J251" s="2" t="inlineStr">
+        <is>
+          <t>RSK-035</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B252" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C252" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D252" s="2" t="inlineStr">
+        <is>
+          <t>중동전쟁 장기화에 중소기업 피해 '962건'</t>
+        </is>
+      </c>
+      <c r="E252" s="2" t="inlineStr">
+        <is>
+          <t>중동전쟁 장기화로 해상운임 증가와 우회 운송이 겹치며 중소기업의 물류 피해 사례가 누적되고 있다.</t>
+        </is>
+      </c>
+      <c r="F252" s="2" t="inlineStr">
+        <is>
+          <t>중동전쟁 장기화로 인한 해상운임 상승 및 우회 운송은 우리 물류 비용과 리드타임에 직접적인 영향을 미친다.</t>
+        </is>
+      </c>
+      <c r="G252" s="2" t="inlineStr">
+        <is>
+          <t>중동 지역을 경유하는 모든 운송 경로를 재검토하고, 운송 파트너와 긴밀히 협력하여 최적의 경로 및 비용 절감 방안을 모색하며, 비상 재고 확보를 고려한다.</t>
+        </is>
+      </c>
+      <c r="H252" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I252" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260629-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J252" s="2" t="inlineStr">
+        <is>
+          <t>RSK-036</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B253" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C253" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D253" s="2" t="inlineStr">
+        <is>
+          <t>글로벌 해운운임, 9주 연속 상승…3200대 돌파</t>
+        </is>
+      </c>
+      <c r="E253" s="2" t="inlineStr">
+        <is>
+          <t>상하이컨테이너운임지수(SCFI)가 9주 연속 상승하여 3200선을 돌파하며 글로벌 해상물류 비용 부담이 크게 증가하고 있다.</t>
+        </is>
+      </c>
+      <c r="F253" s="2" t="inlineStr">
+        <is>
+          <t>글로벌 해운 운임의 급등은 우리 제품의 수출입 물류 비용을 직접적으로 증가시켜 수익성에 영향을 미친다.</t>
+        </is>
+      </c>
+      <c r="G253" s="2" t="inlineStr">
+        <is>
+          <t>운송 계약 조건을 재검토하고, 장기 계약 협상 또는 복수 운송사 활용을 통해 운임 변동 리스크를 분산하며, 물류비용 상승분을 제품 가격에 반영할지 검토한다.</t>
+        </is>
+      </c>
+      <c r="H253" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I253" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260629-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J253" s="2" t="inlineStr">
+        <is>
+          <t>RSK-037</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B254" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C254" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D254" s="2" t="inlineStr">
+        <is>
+          <t>휴전 했다는데 기름값은 왜 그대로인가</t>
+        </is>
+      </c>
+      <c r="E254" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 휴전에도 불구하고 유가가 내려가지 않는 것은 급격히 유입될 물량이 글로벌 컨테이너 공급망에 새로운 지연을 만들 수 있기 때문이라는 분석이다.</t>
+        </is>
+      </c>
+      <c r="F254" s="2" t="inlineStr">
+        <is>
+          <t>유가 및 운임 하락 지연은 물류 비용 상승 압력의 장기화를 의미하며, 이는 우리 물류 예산 및 수익성에 직접적인 영향을 미친다.</t>
+        </is>
+      </c>
+      <c r="G254" s="2" t="inlineStr">
+        <is>
+          <t>장기적인 물류비용 상승에 대비하여 운송 계약 재협상, 운송 모드 최적화, 재고 관리 전략 재검토 등 다각적인 비용 절감 방안을 모색한다.</t>
+        </is>
+      </c>
+      <c r="H254" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I254" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260626-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J254" s="2" t="inlineStr">
+        <is>
+          <t>RSK-038</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B255" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C255" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D255" s="2" t="inlineStr">
+        <is>
+          <t>"트럼프 신규 관세 피하자"…기업들 선적 경쟁에 해상 운임 급등</t>
+        </is>
+      </c>
+      <c r="E255" s="2" t="inlineStr">
+        <is>
+          <t>트럼프의 신규 관세 부과를 피하려는 기업들의 선적 경쟁으로 해상 화물 운임이 2년 만에 최고치로 치솟아 물류 비용 부담이 가중되고 있다.</t>
+        </is>
+      </c>
+      <c r="F255" s="2" t="inlineStr">
+        <is>
+          <t>신규 관세 우려로 인한 선적 경쟁과 해상 운임 급등은 우리 물류 비용과 스케줄에 직접적인 영향을 미친다.</t>
+        </is>
+      </c>
+      <c r="G255" s="2" t="inlineStr">
+        <is>
+          <t>주요 수출입 노선의 운임 변동을 면밀히 모니터링하고, 운송 파트너와 협력하여 선적 공간 확보 및 비용 최적화 방안을 논의하며, 관세 부과 시나리오에 따른 대응 계획을 수립한다.</t>
+        </is>
+      </c>
+      <c r="H255" s="2" t="inlineStr">
+        <is>
+          <t>newspim</t>
+        </is>
+      </c>
+      <c r="I255" s="2" t="inlineStr">
+        <is>
+          <t>https://www.newspim.com/news/view/20260629001067</t>
+        </is>
+      </c>
+      <c r="J255" s="2" t="inlineStr">
+        <is>
+          <t>RSK-039</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B256" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C256" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D256" s="2" t="inlineStr">
+        <is>
+          <t>West Asia conflict hits real estate business, residential sales drop 6% in Q2: Report</t>
+        </is>
+      </c>
+      <c r="E256" s="2" t="inlineStr">
+        <is>
+          <t>서아시아 분쟁이 공급망을 교란하여 부동산 시장에 영향을 미치고 있으며, 이는 지정학적 리스크가 광범위한 경제 부문에 미치는 영향을 보여준다.</t>
+        </is>
+      </c>
+      <c r="F256" s="2" t="inlineStr">
+        <is>
+          <t>서아시아 분쟁으로 인한 공급망 교란은 우리 물류 운영의 안정성과 비용에 직접적인 영향을 미친다.</t>
+        </is>
+      </c>
+      <c r="G256" s="2" t="inlineStr">
+        <is>
+          <t>서아시아 지역 관련 공급망 리스크를 재평가하고, 대체 공급처 및 운송 경로 확보, 비상 재고 확충 등 비상 계획을 강화한다.</t>
+        </is>
+      </c>
+      <c r="H256" s="2" t="inlineStr">
+        <is>
+          <t>The HinduBusinessLine</t>
+        </is>
+      </c>
+      <c r="I256" s="2" t="inlineStr">
+        <is>
+          <t>https://www.thehindubusinessline.com/news/real-estate/west-asia-conflict-hits-real-estate-business-residential-sales-drop-6-in-q2-report/article71160696.ece</t>
+        </is>
+      </c>
+      <c r="J256" s="2" t="inlineStr">
+        <is>
+          <t>RSK-040</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B257" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C257" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D257" s="2" t="inlineStr">
+        <is>
+          <t>"트럼프 신규 관세 피하자"…기업들 선적 경쟁에 해상 운임 급등</t>
+        </is>
+      </c>
+      <c r="E257" s="2" t="inlineStr">
+        <is>
+          <t>트럼프의 신규 관세 부과를 피하기 위한 기업들의 선적 경쟁으로 해상 화물 운임이 2년 전 홍해 위기 이후 최고치로 치솟았다. 이는 기업들이 재고를 미리 확보하려는 움직임 때문이다.</t>
+        </is>
+      </c>
+      <c r="F257" s="2" t="inlineStr">
+        <is>
+          <t>미국의 관세 정책 변화가 기업들의 선적 수요를 급증시켜 해상 운임을 직접적으로 상승시키고 있으며, 이는 우리 회사의 물류 비용에 즉각적인 영향을 미친다.</t>
+        </is>
+      </c>
+      <c r="G257" s="2" t="inlineStr">
+        <is>
+          <t>주요 수출입 항로의 운임 변동 추이를 면밀히 모니터링하고, 선적 계획 및 예산에 반영하며, 가능한 경우 대체 운송 방안을 검토해야 한다.</t>
+        </is>
+      </c>
+      <c r="H257" s="2" t="inlineStr">
+        <is>
+          <t>뉴스핌</t>
+        </is>
+      </c>
+      <c r="I257" s="2" t="inlineStr">
+        <is>
+          <t>https://newspim.com/news/view/20260629001067</t>
+        </is>
+      </c>
+      <c r="J257" s="2" t="inlineStr">
+        <is>
+          <t>RSK-041</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B258" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C258" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D258" s="2" t="inlineStr">
+        <is>
+          <t>무협 "美 관세 리스크 장기화…수출기업, 계약부터 다시 봐야"</t>
+        </is>
+      </c>
+      <c r="E258" s="2" t="inlineStr">
+        <is>
+          <t>한국무역협회는 미국의 고관세 기조가 장기화될 것으로 예상하며, 수출기업들이 무역계약 단계부터 관세 리스크를 점검해야 한다고 제언했다. 이는 관세 부과로 인한 비용 증가 및 경쟁력 약화에 대비하기 위함이다.</t>
+        </is>
+      </c>
+      <c r="F258" s="2" t="inlineStr">
+        <is>
+          <t>미국의 관세 정책은 우리 회사의 수출 비용과 경쟁력에 직접적인 영향을 미치므로, 무역 계약 및 물류 전략 수립 시 관세 리스크를 반드시 고려해야 한다.</t>
+        </is>
+      </c>
+      <c r="G258" s="2" t="inlineStr">
+        <is>
+          <t>미국 수출 관련 제품의 관세 영향도를 재분석하고, 무역 계약 조건 및 인코텀즈(Incoterms) 검토를 통해 관세 부담을 최소화할 방안을 모색해야 한다.</t>
+        </is>
+      </c>
+      <c r="H258" s="2" t="inlineStr">
+        <is>
+          <t>뉴스핌</t>
+        </is>
+      </c>
+      <c r="I258" s="2" t="inlineStr">
+        <is>
+          <t>https://newspim.com/news/view/20260629001344</t>
+        </is>
+      </c>
+      <c r="J258" s="2" t="inlineStr">
+        <is>
+          <t>RSK-042</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B259" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C259" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D259" s="3" t="inlineStr">
+        <is>
+          <t>Air Cargo Demand up 6.0% in May</t>
+        </is>
+      </c>
+      <c r="E259" s="3" t="inlineStr">
+        <is>
+          <t>IATA에 따르면 2026년 5월 전 세계 항공 화물 수요가 전년 대비 6.0% 증가했다.</t>
+        </is>
+      </c>
+      <c r="F259" s="3" t="inlineStr">
+        <is>
+          <t>항공 화물 수요 증가는 향후 항공 운임 상승 압력으로 작용할 수 있으므로 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G259" s="3" t="inlineStr">
+        <is>
+          <t>항공 운임 변동 추이 및 항공 화물 공급 상황 지속 모니터링</t>
+        </is>
+      </c>
+      <c r="H259" s="3" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I259" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-29-air-cargo-demand-up-may/</t>
+        </is>
+      </c>
+      <c r="J259" s="3" t="inlineStr"/>
+    </row>
+    <row r="260">
+      <c r="A260" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B260" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C260" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D260" s="3" t="inlineStr">
+        <is>
+          <t>WMES 2026 Speech - Stuart Fox, IATA's Director Flight and Operations</t>
+        </is>
+      </c>
+      <c r="E260" s="3" t="inlineStr">
+        <is>
+          <t>IATA 관계자는 항공기 인도 지연, 엔진 수명 단축, 부품 확보 어려움, 수리 기간 증가 등 항공 산업의 현실적인 문제들을 언급하며 공급망 강화를 촉구했다.</t>
+        </is>
+      </c>
+      <c r="F260" s="3" t="inlineStr">
+        <is>
+          <t>항공기 가용성 및 부품 공급 문제는 항공 화물 운송 용량과 스케줄에 영향을 미칠 수 있으므로, 관련 동향을 지속적으로 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G260" s="3" t="inlineStr">
+        <is>
+          <t>항공 화물 운송사의 항공기 가동률 및 용량 변화 추이 모니터링, 대체 운송 방안 검토</t>
+        </is>
+      </c>
+      <c r="H260" s="3" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I260" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-speeches/06-24-wmes-2026-speech-stuart-fox-iata-director-flight-operations/</t>
+        </is>
+      </c>
+      <c r="J260" s="3" t="inlineStr"/>
+    </row>
+    <row r="261">
+      <c r="A261" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B261" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C261" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D261" s="3" t="inlineStr">
+        <is>
+          <t>Global Schedule Reliability for May 2026 the Highest of the Year</t>
+        </is>
+      </c>
+      <c r="E261" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence 보고서에 따르면 2026년 5월 글로벌 선박 스케줄 신뢰도가 올해 최고치를 기록했다.</t>
+        </is>
+      </c>
+      <c r="F261" s="3" t="inlineStr">
+        <is>
+          <t>선박 스케줄 신뢰도 개선은 해상 운송 지연 감소에 긍정적인 신호이나, 특정 항로 및 우리 회사의 주요 운송 구간에 미치는 영향을 지속적으로 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G261" s="3" t="inlineStr">
+        <is>
+          <t>주요 항로의 스케줄 신뢰도 및 정시성 데이터 지속 모니터링</t>
+        </is>
+      </c>
+      <c r="H261" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I261" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/395-global-schedule-reliability-for-may-2026-the-highest-of-the-year</t>
+        </is>
+      </c>
+      <c r="J261" s="3" t="inlineStr"/>
+    </row>
+    <row r="262">
+      <c r="A262" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B262" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C262" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D262" s="3" t="inlineStr">
+        <is>
+          <t>Tracking True Vessel Delay</t>
+        </is>
+      </c>
+      <c r="E262" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence는 선박 지연과 스케줄 버퍼링 간의 관계를 분석하며, 선사들이 운송 시간을 늘려 스케줄 신뢰도를 높이는 경향을 보인다고 밝혔다.</t>
+        </is>
+      </c>
+      <c r="F262" s="3" t="inlineStr">
+        <is>
+          <t>선사들의 스케줄 버퍼링 증가는 겉으로는 정시성을 높이지만 실제 운송 시간은 길어질 수 있으므로, 우리 회사의 리드타임 계획에 미치는 영향을 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G262" s="3" t="inlineStr">
+        <is>
+          <t>주요 항로의 실제 운송 리드타임 데이터 분석 및 선사별 스케줄 버퍼링 전략 파악</t>
+        </is>
+      </c>
+      <c r="H262" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I262" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/394-tracking-true-vessel-delay</t>
+        </is>
+      </c>
+      <c r="J262" s="3" t="inlineStr"/>
+    </row>
+    <row r="263">
+      <c r="A263" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B263" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C263" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D263" s="3" t="inlineStr">
+        <is>
+          <t>Transpacific: Ripe for new non-alliance services</t>
+        </is>
+      </c>
+      <c r="E263" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence는 태평양 항로에서 비동맹 컨테이너 선박 용량과 스팟 운임 간의 관계를 분석하며, 새로운 비동맹 서비스의 출현 가능성을 시사했다.</t>
+        </is>
+      </c>
+      <c r="F263" s="3" t="inlineStr">
+        <is>
+          <t>태평양 항로는 우리 회사의 주요 운송 항로 중 하나이므로, 새로운 서비스 출현은 운임 경쟁 및 용량 변화에 영향을 미칠 수 있어 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G263" s="3" t="inlineStr">
+        <is>
+          <t>태평양 항로의 운임 및 용량 변화 추이, 신규 서비스 동향 지속 모니터링</t>
+        </is>
+      </c>
+      <c r="H263" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I263" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/393-transpacific-ripe-for-new-non-alliance-services</t>
+        </is>
+      </c>
+      <c r="J263" s="3" t="inlineStr"/>
+    </row>
+    <row r="264">
+      <c r="A264" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B264" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C264" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D264" s="3" t="inlineStr">
+        <is>
+          <t>2026-Q1: NAEC Ports Consolidate Market Share</t>
+        </is>
+      </c>
+      <c r="E264" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence 보고서에 따르면 2026년 1분기 북미 동부 항만(NAEC)의 컨테이너 물동량은 전년 대비 감소했으나, 시장 점유율은 공고히 했다.</t>
+        </is>
+      </c>
+      <c r="F264" s="3" t="inlineStr">
+        <is>
+          <t>북미 동부 항만은 우리 회사의 주요 수출입 거점 중 하나일 수 있으므로, 물동량 변화 및 시장 점유율 동향은 항만 운영 효율성에 영향을 미칠 수 있어 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G264" s="3" t="inlineStr">
+        <is>
+          <t>북미 동부 항만의 물동량 및 운영 효율성 변화 추이 지속 모니터링</t>
+        </is>
+      </c>
+      <c r="H264" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I264" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/391-2026-q1-naec-ports-consolidate-market-share</t>
+        </is>
+      </c>
+      <c r="J264" s="3" t="inlineStr"/>
+    </row>
+    <row r="265">
+      <c r="A265" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B265" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C265" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D265" s="3" t="inlineStr">
+        <is>
+          <t>미국 트럭운송 능력 부족, 운임 상승에 철도 복합운송으로 전환 가속...화주들 경제적인 대체 운송수단</t>
+        </is>
+      </c>
+      <c r="E265" s="3" t="inlineStr">
+        <is>
+          <t>미국 트럭 운송 능력 부족과 운임 상승으로 화주들이 비용 효율적인 철도 복합운송으로 전환을 가속화하고 있으며, 이는 북미 물류시장의 구조적 변화를 시사한다.</t>
+        </is>
+      </c>
+      <c r="F265" s="3" t="inlineStr">
+        <is>
+          <t>북미 내륙 운송 비용 상승 및 모드 전환 추세는 우리 제품의 북미 시장 공급망 전략에 잠재적 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G265" s="3" t="inlineStr">
+        <is>
+          <t>북미 내륙 운송 파트너와 철도 복합운송 옵션 및 비용 효율성을 논의하고, 장기적인 운송 전략에 미칠 영향을 분석한다.</t>
+        </is>
+      </c>
+      <c r="H265" s="3" t="inlineStr">
+        <is>
+          <t>shippingnews</t>
+        </is>
+      </c>
+      <c r="I265" s="3" t="inlineStr">
+        <is>
+          <t>https://www.shippingnewsnet.com/news/articleView.html?idxno=70953</t>
+        </is>
+      </c>
+      <c r="J265" s="3" t="inlineStr"/>
+    </row>
+    <row r="266">
+      <c r="A266" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B266" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C266" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D266" s="3" t="inlineStr">
+        <is>
+          <t>우회덤핑 차단 공조…관세청·무역위 공동 대응</t>
+        </is>
+      </c>
+      <c r="E266" s="3" t="inlineStr">
+        <is>
+          <t>관세청과 무역위가 우회덤핑 감시 정보를 공유하고 무역구제 조치의 실효성 강화를 논의하며, 이는 무역분쟁 및 규제 강화 가능성을 시사한다.</t>
+        </is>
+      </c>
+      <c r="F266" s="3" t="inlineStr">
+        <is>
+          <t>무역 규제 강화는 우리 제품의 수출입 절차 및 비용에 잠재적 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G266" s="3" t="inlineStr">
+        <is>
+          <t>관련 규제 동향을 지속적으로 모니터링하고, 필요시 무역 전문가와 상담하여 잠재적 리스크를 평가한다.</t>
+        </is>
+      </c>
+      <c r="H266" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I266" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260630-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J266" s="3" t="inlineStr"/>
+    </row>
+    <row r="267">
+      <c r="A267" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B267" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C267" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D267" s="3" t="inlineStr">
+        <is>
+          <t>국제유가, 주말 호르무즈 무력공방에 상승…WTI 2%↑</t>
+        </is>
+      </c>
+      <c r="E267" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 인근 무력 공방 등 지정학적 긴장으로 국제유가가 2% 상승하여 물류비용 상승 압력이 커지고 있다.</t>
+        </is>
+      </c>
+      <c r="F267" s="3" t="inlineStr">
+        <is>
+          <t>국제유가 상승은 해상 및 항공 운임에 직접적인 영향을 미쳐 물류비용 증가로 이어질 수 있다.</t>
+        </is>
+      </c>
+      <c r="G267" s="3" t="inlineStr">
+        <is>
+          <t>유가 및 운임 변동 추이를 면밀히 모니터링하고, 운송 계약 시 유류할증료 조건 등을 재검토한다.</t>
+        </is>
+      </c>
+      <c r="H267" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I267" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260630-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J267" s="3" t="inlineStr"/>
+    </row>
+    <row r="268">
+      <c r="A268" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B268" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C268" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D268" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 통항량 하루 만에 105% 급증…유조선 운항 빠르게 회복</t>
+        </is>
+      </c>
+      <c r="E268" s="3" t="inlineStr">
+        <is>
+          <t>미국과 이란의 해협 재개방 합의 이후 호르무즈 해협의 유조선 통항량이 급증하며 해상 운송이 일시적으로 회복되는 조짐을 보였다.</t>
+        </is>
+      </c>
+      <c r="F268" s="3" t="inlineStr">
+        <is>
+          <t>일시적 회복 조짐에도 불구하고 호르무즈 해협의 지정학적 리스크는 여전히 높아, 운송 안정성 확보를 위한 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G268" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협의 운항 상황을 지속적으로 주시하고, 지정학적 리스크 변화에 따른 비상 계획을 업데이트한다.</t>
+        </is>
+      </c>
+      <c r="H268" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I268" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260626-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J268" s="3" t="inlineStr"/>
+    </row>
+    <row r="269">
+      <c r="A269" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B269" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C269" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D269" s="3" t="inlineStr">
+        <is>
+          <t>글로벌 선박 엔진 품귀…韓 조선업계 반사이익 기대</t>
+        </is>
+      </c>
+      <c r="E269" s="3" t="inlineStr">
+        <is>
+          <t>전 세계 조선업의 기록적인 신조선 건조 물량으로 선박 엔진 품귀 현상이 발생하고 있으며, 이는 장기적으로 신규 선박 공급 지연을 야기할 수 있다.</t>
+        </is>
+      </c>
+      <c r="F269" s="3" t="inlineStr">
+        <is>
+          <t>선박 엔진 품귀는 신규 선박 공급 지연을 초래하여 장기적으로 해상 운송 능력 및 운임에 영향을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="G269" s="3" t="inlineStr">
+        <is>
+          <t>해운 시장의 선박 공급 동향을 지속적으로 모니터링하고, 장기적인 운송 계약 시 선박 확보 가능성을 고려한다.</t>
+        </is>
+      </c>
+      <c r="H269" s="3" t="inlineStr">
+        <is>
+          <t>EBN뉴스센터</t>
+        </is>
+      </c>
+      <c r="I269" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebn.co.kr/news/articleView.html?idxno=1714238</t>
+        </is>
+      </c>
+      <c r="J269" s="3" t="inlineStr"/>
+    </row>
+    <row r="270">
+      <c r="A270" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B270" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C270" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D270" s="3" t="inlineStr">
+        <is>
+          <t>공급 폭탄 앞둔 컨테이너선…해상 저장 ‘특수’ 유조선</t>
+        </is>
+      </c>
+      <c r="E270" s="3" t="inlineStr">
+        <is>
+          <t>컨테이너선 시장은 공급 과잉을 앞두고 있으나, 유조선은 해상 저장 특수를 누리고 있어 해운 시장의 복합적인 상황을 보여준다.</t>
+        </is>
+      </c>
+      <c r="F270" s="3" t="inlineStr">
+        <is>
+          <t>컨테이너선 공급 과잉은 장기적으로 운임 하락 가능성을 시사하나, 현재 시장 상황과 상충되어 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G270" s="3" t="inlineStr">
+        <is>
+          <t>컨테이너선 시장의 공급 및 수요 변화를 지속적으로 모니터링하여 장기적인 운임 예측에 활용한다.</t>
+        </is>
+      </c>
+      <c r="H270" s="3" t="inlineStr">
+        <is>
+          <t>뉴스토마토</t>
+        </is>
+      </c>
+      <c r="I270" s="3" t="inlineStr">
+        <is>
+          <t>https://newstomato.com/ReadNews.aspx?no=1305485</t>
+        </is>
+      </c>
+      <c r="J270" s="3" t="inlineStr"/>
+    </row>
+    <row r="271">
+      <c r="A271" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B271" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C271" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D271" s="3" t="inlineStr">
+        <is>
+          <t>일본 신칸센, 보조배터리 화재 진압도구 비치 - ZDNet korea</t>
+        </is>
+      </c>
+      <c r="E271" s="3" t="inlineStr">
+        <is>
+          <t>일본 신칸센이 보조배터리 화재 진압 도구를 객실 내에 비치하여 화재 피해를 막는 방안을 도입했다. 이는 항공기의 반입 금지와 달리 화재 발생 시 즉각적인 대응을 가능하게 한다.</t>
+        </is>
+      </c>
+      <c r="F271" s="3" t="inlineStr">
+        <is>
+          <t>철도 운송에 대한 직접적인 규제는 아니지만, 배터리 화재 위험에 대한 운송수단의 안전 조치 강화 추세를 보여주므로 향후 다른 운송 방식에도 유사한 규제나 요구사항이 생길 수 있다.</t>
+        </is>
+      </c>
+      <c r="G271" s="3" t="inlineStr"/>
+      <c r="H271" s="3" t="inlineStr">
+        <is>
+          <t>ZDNet korea</t>
+        </is>
+      </c>
+      <c r="I271" s="3" t="inlineStr">
+        <is>
+          <t>https://zdnet.co.kr/view/?no=20260629100736</t>
+        </is>
+      </c>
+      <c r="J271" s="3" t="inlineStr"/>
+    </row>
+    <row r="272">
+      <c r="A272" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B272" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C272" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D272" s="3" t="inlineStr">
+        <is>
+          <t>미국, 구리 관세 카드 재검토...글로벌 공급망 재편 가능성</t>
+        </is>
+      </c>
+      <c r="E272" s="3" t="inlineStr">
+        <is>
+          <t>미국이 구리 관세 카드를 다시 꺼낼 가능성이 높아지면서, 글로벌 구리 공급망 재편이 한국 기업의 조달 전략에 직접적인 변수가 될 수 있다. 이는 구리 정련동까지 관세 부과 대상이 될 수 있음을 시사한다.</t>
+        </is>
+      </c>
+      <c r="F272" s="3" t="inlineStr">
+        <is>
+          <t>구리는 전자부품 제조에 필수적인 원자재이므로, 미국의 관세 부과는 원자재 조달 비용 및 공급망 전략에 잠재적 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G272" s="3" t="inlineStr">
+        <is>
+          <t>구리 관련 원자재 조달처 다변화 및 관세 영향 분석 필요.</t>
+        </is>
+      </c>
+      <c r="H272" s="3" t="inlineStr">
+        <is>
+          <t>허프포스트코리아</t>
+        </is>
+      </c>
+      <c r="I272" s="3" t="inlineStr">
+        <is>
+          <t>https://huffingtonpost.kr/article/258311</t>
+        </is>
+      </c>
+      <c r="J272" s="3" t="inlineStr"/>
+    </row>
+    <row r="273">
+      <c r="A273" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B273" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C273" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D273" s="3" t="inlineStr">
+        <is>
+          <t>휘발유·경유 가격 2000원 아래…정부 최고가격 첫 인하 효과</t>
+        </is>
+      </c>
+      <c r="E273" s="3" t="inlineStr">
+        <is>
+          <t>국내 주유소 휘발유와 경유 평균 판매 가격이 국제 유가 하락과 정부의 7차 석유 최고가격 인하 조치로 L당 2,000원 아래로 내려왔다.</t>
+        </is>
+      </c>
+      <c r="F273" s="3" t="inlineStr">
+        <is>
+          <t>국내 육상 운송비용에 직접적인 영향을 미치는 유가 하락 추세이므로, 물류비 절감 가능성을 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G273" s="3" t="inlineStr">
+        <is>
+          <t>국내 운송 계약 시 유류할증료 변동 추이 확인 및 비용 절감 가능성 검토.</t>
+        </is>
+      </c>
+      <c r="H273" s="3" t="inlineStr">
+        <is>
+          <t>더쎈뉴스(The CEN News)</t>
+        </is>
+      </c>
+      <c r="I273" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mhns.co.kr/news/articleView.html?idxno=751655</t>
+        </is>
+      </c>
+      <c r="J273" s="3" t="inlineStr"/>
+    </row>
+    <row r="274">
+      <c r="A274" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B274" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C274" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D274" s="4" t="inlineStr">
+        <is>
+          <t>롯데글로벌, 지속가능경영보고서 발간</t>
+        </is>
+      </c>
+      <c r="E274" s="4" t="inlineStr">
+        <is>
+          <t>롯데글로벌로지스가 2025년 ESG 경영 성과를 담은 지속가능경영보고서를 발간했으며, 친환경 경영 활동을 강조했다.</t>
+        </is>
+      </c>
+      <c r="F274" s="4" t="inlineStr">
+        <is>
+          <t>우리 회사의 물류 운영에 직접적인 영향은 없으며, 물류 업계의 ESG 트렌드를 참고하는 수준이다.</t>
+        </is>
+      </c>
+      <c r="G274" s="4" t="n"/>
+      <c r="H274" s="4" t="inlineStr">
+        <is>
+          <t>cargonews</t>
+        </is>
+      </c>
+      <c r="I274" s="4" t="inlineStr">
+        <is>
+          <t>https://www.cargonews.co.kr/news/articleView.html?idxno=60424</t>
+        </is>
+      </c>
+      <c r="J274" s="4" t="inlineStr"/>
+    </row>
+    <row r="275">
+      <c r="A275" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B275" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C275" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D275" s="4" t="inlineStr">
+        <is>
+          <t>IATA and IATP Collaborate to Support Airline Supply Chain Resilience</t>
+        </is>
+      </c>
+      <c r="E275" s="4" t="inlineStr">
+        <is>
+          <t>IATA와 IATP가 항공기 부품 가시성 및 접근성 개선을 위해 협력하여 항공사의 공급망 회복력을 지원하기로 했다.</t>
+        </is>
+      </c>
+      <c r="F275" s="4" t="inlineStr">
+        <is>
+          <t>항공기 부품 공급망 개선은 항공 화물 운송 서비스의 장기적인 안정성에 긍정적일 수 있으나, 당장 우리 물류에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G275" s="4" t="n"/>
+      <c r="H275" s="4" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I275" s="4" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-25-iata-iatp-collaborate-support-airline-supply-chain-resilience/</t>
+        </is>
+      </c>
+      <c r="J275" s="4" t="inlineStr"/>
+    </row>
+    <row r="276">
+      <c r="A276" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B276" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C276" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D276" s="4" t="inlineStr">
+        <is>
+          <t>동해신항 석탄부두 건설로 원자재 공급기반 확충</t>
+        </is>
+      </c>
+      <c r="E276" s="4" t="inlineStr">
+        <is>
+          <t>해수부가 동해신항에 10만DWT급 석탄부두를 건설하여 석탄 등 원자재 하역 능력과 항만 운영 효율을 높일 계획이다.</t>
+        </is>
+      </c>
+      <c r="F276" s="4" t="inlineStr">
+        <is>
+          <t>석탄 부두 건설은 우리 회사의 배터리/전자부품 물류와 직접적인 관련이 없으며, 일반 화물 운송에 미치는 영향도 미미하다.</t>
+        </is>
+      </c>
+      <c r="G276" s="4" t="n"/>
+      <c r="H276" s="4" t="inlineStr">
+        <is>
+          <t>kita</t>
+        </is>
+      </c>
+      <c r="I276" s="4" t="inlineStr">
+        <is>
+          <t>https://www.kita.net/shippers/board/newsView.do?morgueCode=2&amp;dataCls=B&amp;dataSeq=8139</t>
+        </is>
+      </c>
+      <c r="J276" s="4" t="inlineStr"/>
+    </row>
+    <row r="277">
+      <c r="A277" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B277" s="4" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C277" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D277" s="4" t="inlineStr">
+        <is>
+          <t>더 까다롭지만 더 빠르게, 호주 환경 인허가법 전면 개정</t>
+        </is>
+      </c>
+      <c r="E277" s="4" t="inlineStr">
+        <is>
+          <t>호주 정부가 25년 만에 환경 인허가 체계를 전면 개편하여 대규모 개발 프로젝트 승인 환경에 변화가 예상되며, 2026년부터 세부 규정이 시행될 예정이다.</t>
+        </is>
+      </c>
+      <c r="F277" s="4" t="inlineStr">
+        <is>
+          <t>호주의 환경 인허가법 개정은 당장 우리 회사의 배터리/전자부품 물류 운영에 직접적인 영향을 미치지 않으며, 향후 호주 내 투자 계획 시 참고할 사항이다.</t>
+        </is>
+      </c>
+      <c r="G277" s="4" t="n"/>
+      <c r="H277" s="4" t="inlineStr">
+        <is>
+          <t>kotra</t>
+        </is>
+      </c>
+      <c r="I277" s="4" t="inlineStr">
+        <is>
+          <t>https://dream.kotra.or.kr/kotranews/cms/news/actionKotraBoardDetail.do?SITE_NO=3&amp;MENU_ID=70&amp;CONTENTS_NO=1&amp;pNttSn=242479</t>
+        </is>
+      </c>
+      <c r="J277" s="4" t="inlineStr"/>
+    </row>
+    <row r="278">
+      <c r="A278" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B278" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C278" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D278" s="4" t="inlineStr">
+        <is>
+          <t>WinGD Achieves next Ammonia Milestone with First X72DF-A Engine Approval</t>
+        </is>
+      </c>
+      <c r="E278" s="4" t="inlineStr">
+        <is>
+          <t>스위스 해양 동력 회사 WinGD가 암모니아 연료 해양 엔진(X72DF-A)의 공장 인수 테스트를 성공적으로 완료하며 저탄소 해운을 위한 중요한 이정표를 달성했다.</t>
+        </is>
+      </c>
+      <c r="F278" s="4" t="inlineStr">
+        <is>
+          <t>암모니아 연료 엔진 개발은 해운 산업의 장기적인 친환경 전환에 기여할 것이나, 우리 회사의 현재 물류 운영에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G278" s="4" t="n"/>
+      <c r="H278" s="4" t="inlineStr">
+        <is>
+          <t>ksg</t>
+        </is>
+      </c>
+      <c r="I278" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksg.co.kr/news/main_newsView.jsp?pNum=147517</t>
+        </is>
+      </c>
+      <c r="J278" s="4" t="inlineStr"/>
+    </row>
+    <row r="279">
+      <c r="A279" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B279" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C279" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D279" s="4" t="inlineStr">
+        <is>
+          <t>Decoding Gemini’s Mediterranean Surge</t>
+        </is>
+      </c>
+      <c r="E279" s="4" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence는 Gemini Cooperation의 함대 재배치 전략을 분석하며, 지중해 지역에서 시장 점유율을 확대하고 있음을 밝혔다.</t>
+        </is>
+      </c>
+      <c r="F279" s="4" t="inlineStr">
+        <is>
+          <t>특정 선사 동맹의 지중해 지역 함대 재배치는 우리 회사의 주요 운송 항로 및 물류 운영에 직접적인 영향을 미치지 않는다.</t>
+        </is>
+      </c>
+      <c r="G279" s="4" t="n"/>
+      <c r="H279" s="4" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I279" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/392-decoding-gemini-s-mediterranean-surge</t>
+        </is>
+      </c>
+      <c r="J279" s="4" t="inlineStr"/>
+    </row>
+    <row r="280">
+      <c r="A280" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B280" s="4" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C280" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D280" s="4" t="inlineStr">
+        <is>
+          <t>CPTPP 회원국, 인도네시아·필리핀·UAE와 가입 예비협상 개시</t>
+        </is>
+      </c>
+      <c r="E280" s="4" t="inlineStr">
+        <is>
+          <t>CPTPP가 인도네시아, 필리핀, UAE와 가입 예비협상을 개시하며, 이는 향후 무역 환경 변화 및 관세 정책에 영향을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="F280" s="4" t="inlineStr">
+        <is>
+          <t>CPTPP 가입 협상은 장기적인 무역 환경 변화를 가져올 수 있으나, 당장 우리 물류 운영에 직접적인 영향은 미미하다.</t>
+        </is>
+      </c>
+      <c r="G280" s="4" t="n"/>
+      <c r="H280" s="4" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I280" s="4" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260628-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J280" s="4" t="inlineStr"/>
+    </row>
+    <row r="281">
+      <c r="A281" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B281" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C281" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D281" s="4" t="inlineStr">
+        <is>
+          <t>씨메스로보틱스 / ‘물류·제조 대형 수주 잇달아’ 피지컬 AI 기반 로봇 자동화 사업 가속</t>
+        </is>
+      </c>
+      <c r="E281" s="4" t="inlineStr">
+        <is>
+          <t>씨메스로보틱스가 물류 및 제조 현장에서 피지컬 AI 기반 로봇 자동화 솔루션 수주를 확대하며 사업을 가속화하고 있으며, 이는 물류 자동화 기술 도입의 중요성을 보여준다.</t>
+        </is>
+      </c>
+      <c r="F281" s="4" t="inlineStr">
+        <is>
+          <t>물류 자동화 기술 발전은 장기적인 효율성 개선에 기여할 수 있으나, 당장 우리 물류 운영에 직접적인 영향은 미미하다.</t>
+        </is>
+      </c>
+      <c r="G281" s="4" t="n"/>
+      <c r="H281" s="4" t="inlineStr">
+        <is>
+          <t>ulogistics</t>
+        </is>
+      </c>
+      <c r="I281" s="4" t="inlineStr">
+        <is>
+          <t>http://www.ulogistics.co.kr/test/board.php?board=all2&amp;command=body&amp;no=5202</t>
+        </is>
+      </c>
+      <c r="J281" s="4" t="inlineStr"/>
+    </row>
+    <row r="282">
+      <c r="A282" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B282" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C282" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D282" s="4" t="inlineStr">
+        <is>
+          <t>Council Post: How Workforce Strategy Is Shaping Supply Chain Reliability</t>
+        </is>
+      </c>
+      <c r="E282" s="4" t="inlineStr">
+        <is>
+          <t>인력 전략이 공급망 신뢰성을 형성하는 데 중요하며, 이는 변화하는 공급망 운영 현실에 맞춰 인력, 도구, 워크플로우를 조정해야 함을 강조한다.</t>
+        </is>
+      </c>
+      <c r="F282" s="4" t="inlineStr">
+        <is>
+          <t>인력 전략은 장기적인 공급망 신뢰성에 영향을 미치지만, 당장 우리 물류 운영에 직접적인 영향은 미미하다.</t>
+        </is>
+      </c>
+      <c r="G282" s="4" t="n"/>
+      <c r="H282" s="4" t="inlineStr">
+        <is>
+          <t>forbes.com</t>
+        </is>
+      </c>
+      <c r="I282" s="4" t="inlineStr">
+        <is>
+          <t>https://forbes.com/councils/forbesbusinesscouncil/2026/06/29/how-workforce-strategy-is-shaping-supply-chain-reliability</t>
+        </is>
+      </c>
+      <c r="J282" s="4" t="inlineStr"/>
+    </row>
+    <row r="283">
+      <c r="A283" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B283" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C283" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D283" s="4" t="inlineStr">
+        <is>
+          <t>GHX Announces New AI-Powered Orchestration Layer to Sense Supply Chain Disruption | HPN Online</t>
+        </is>
+      </c>
+      <c r="E283" s="4" t="inlineStr">
+        <is>
+          <t>GHX가 AI 기반 오케스트레이션 레이어를 발표하여 공급망 중단을 감지하고 회복탄력성을 구축하며 절차를 간소화하려 한다. 이는 워크플로우 부채를 제거하고 공급망 효율성을 높이는 데 목적이 있다.</t>
+        </is>
+      </c>
+      <c r="F283" s="4" t="inlineStr">
+        <is>
+          <t>우리 회사의 직접적인 물류 운영에 당장 영향을 미치기보다는, 공급망 기술 트렌드에 대한 참고 자료이다.</t>
+        </is>
+      </c>
+      <c r="G283" s="4" t="inlineStr"/>
+      <c r="H283" s="4" t="inlineStr">
+        <is>
+          <t>HPN Online</t>
+        </is>
+      </c>
+      <c r="I283" s="4" t="inlineStr">
+        <is>
+          <t>https://www.hpnonline.com/sourcing-logistics/news/55387397/ghx-announces-new-ai-powered-orchestration-layer-to-sense-supply-chain-disruption</t>
+        </is>
+      </c>
+      <c r="J283" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -12218,7 +13842,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12494,6 +14118,49 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>3239.64</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>+118 (+3.8%)</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>+1,151 (+55.1%)</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>3920</v>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>+173 (+4.6%)</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>+1,093 (+38.7%)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -12506,7 +14173,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13722,6 +15389,321 @@
       </c>
       <c r="I34" s="6" t="inlineStr"/>
     </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>RSK-034</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E35" s="6" t="inlineStr">
+        <is>
+          <t>머스크, 올해 실적 전망 대폭 상향 조정</t>
+        </is>
+      </c>
+      <c r="F35" s="6" t="inlineStr"/>
+      <c r="G35" s="6" t="inlineStr"/>
+      <c r="H35" s="6" t="inlineStr">
+        <is>
+          <t>해상 운임 변동 추이 면밀히 모니터링 및 운송 계약 조건 재검토, 대체 운송 방안 또는 선사 다변화 검토</t>
+        </is>
+      </c>
+      <c r="I35" s="6" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>RSK-035</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D36" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈 내 한국 선박 2척 추가 탈출...3척만 남아</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="inlineStr"/>
+      <c r="G36" s="6" t="inlineStr"/>
+      <c r="H36" s="6" t="inlineStr">
+        <is>
+          <t>중동 경유 선박의 운항 현황을 실시간으로 확인하고, 필요시 대체 항로 또는 운송 수단 검토, 재고 수준 점검 및 비상 계획을 수립한다.</t>
+        </is>
+      </c>
+      <c r="I36" s="6" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>RSK-036</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D37" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E37" s="6" t="inlineStr">
+        <is>
+          <t>중동전쟁 장기화에 중소기업 피해 '962건'</t>
+        </is>
+      </c>
+      <c r="F37" s="6" t="inlineStr"/>
+      <c r="G37" s="6" t="inlineStr"/>
+      <c r="H37" s="6" t="inlineStr">
+        <is>
+          <t>중동 지역을 경유하는 모든 운송 경로를 재검토하고, 운송 파트너와 긴밀히 협력하여 최적의 경로 및 비용 절감 방안을 모색하며, 비상 재고 확보를 고려한다.</t>
+        </is>
+      </c>
+      <c r="I37" s="6" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>RSK-037</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D38" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E38" s="6" t="inlineStr">
+        <is>
+          <t>글로벌 해운운임, 9주 연속 상승…3200대 돌파</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="inlineStr"/>
+      <c r="G38" s="6" t="inlineStr"/>
+      <c r="H38" s="6" t="inlineStr">
+        <is>
+          <t>운송 계약 조건을 재검토하고, 장기 계약 협상 또는 복수 운송사 활용을 통해 운임 변동 리스크를 분산하며, 물류비용 상승분을 제품 가격에 반영할지 검토한다.</t>
+        </is>
+      </c>
+      <c r="I38" s="6" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>RSK-038</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E39" s="6" t="inlineStr">
+        <is>
+          <t>휴전 했다는데 기름값은 왜 그대로인가</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="inlineStr"/>
+      <c r="G39" s="6" t="inlineStr"/>
+      <c r="H39" s="6" t="inlineStr">
+        <is>
+          <t>장기적인 물류비용 상승에 대비하여 운송 계약 재협상, 운송 모드 최적화, 재고 관리 전략 재검토 등 다각적인 비용 절감 방안을 모색한다.</t>
+        </is>
+      </c>
+      <c r="I39" s="6" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>RSK-039</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D40" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E40" s="6" t="inlineStr">
+        <is>
+          <t>"트럼프 신규 관세 피하자"…기업들 선적 경쟁에 해상 운임 급등</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="inlineStr"/>
+      <c r="G40" s="6" t="inlineStr"/>
+      <c r="H40" s="6" t="inlineStr">
+        <is>
+          <t>주요 수출입 노선의 운임 변동을 면밀히 모니터링하고, 운송 파트너와 협력하여 선적 공간 확보 및 비용 최적화 방안을 논의하며, 관세 부과 시나리오에 따른 대응 계획을 수립한다.</t>
+        </is>
+      </c>
+      <c r="I40" s="6" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>RSK-040</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E41" s="6" t="inlineStr">
+        <is>
+          <t>West Asia conflict hits real estate business, residential sales drop 6% in Q2: Report</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="inlineStr"/>
+      <c r="G41" s="6" t="inlineStr"/>
+      <c r="H41" s="6" t="inlineStr">
+        <is>
+          <t>서아시아 지역 관련 공급망 리스크를 재평가하고, 대체 공급처 및 운송 경로 확보, 비상 재고 확충 등 비상 계획을 강화한다.</t>
+        </is>
+      </c>
+      <c r="I41" s="6" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>RSK-041</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D42" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E42" s="6" t="inlineStr">
+        <is>
+          <t>"트럼프 신규 관세 피하자"…기업들 선적 경쟁에 해상 운임 급등</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="inlineStr"/>
+      <c r="G42" s="6" t="inlineStr"/>
+      <c r="H42" s="6" t="inlineStr">
+        <is>
+          <t>주요 수출입 항로의 운임 변동 추이를 면밀히 모니터링하고, 선적 계획 및 예산에 반영하며, 가능한 경우 대체 운송 방안을 검토해야 한다.</t>
+        </is>
+      </c>
+      <c r="I42" s="6" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>RSK-042</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D43" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E43" s="6" t="inlineStr">
+        <is>
+          <t>무협 "美 관세 리스크 장기화…수출기업, 계약부터 다시 봐야"</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="inlineStr"/>
+      <c r="G43" s="6" t="inlineStr"/>
+      <c r="H43" s="6" t="inlineStr">
+        <is>
+          <t>미국 수출 관련 제품의 관세 영향도를 재분석하고, 무역 계약 조건 및 인코텀즈(Incoterms) 검토를 통해 관세 부담을 최소화할 방안을 모색해야 한다.</t>
+        </is>
+      </c>
+      <c r="I43" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
📰 뉴스 데이터 2026-06-30_19:41
</commit_message>
<xml_diff>
--- a/data/SCM_물류_브리핑.xlsx
+++ b/data/SCM_물류_브리핑.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J283"/>
+  <dimension ref="A1:J307"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13829,6 +13829,1158 @@
         </is>
       </c>
       <c r="J283" s="4" t="inlineStr"/>
+    </row>
+    <row r="284">
+      <c r="A284" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B284" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C284" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D284" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 지정학적 리스크 재확대 및 해운운임 9주 연속 상승</t>
+        </is>
+      </c>
+      <c r="E284" s="2" t="inlineStr">
+        <is>
+          <t>중동전쟁 장기화로 호르무즈 해협의 지정학적 불확실성이 재확대되고 미-이란 간 무력 충돌이 재개되면서 해상운임 증가와 우회 운송 피해가 누적되고 있으며, 글로벌 해운운임(SCFI)은 9주 연속 상승해 3200선을 돌파했다.</t>
+        </is>
+      </c>
+      <c r="F284" s="2" t="inlineStr">
+        <is>
+          <t>주요 해상 운송 경로인 호르무즈 해협의 군사적 긴장 재고조는 운송 지연 및 안전 문제를 야기하고, 해운 운임의 지속적인 상승은 우리 회사의 물류 비용에 직접적인 부담을 준다.</t>
+        </is>
+      </c>
+      <c r="G284" s="2" t="inlineStr">
+        <is>
+          <t>중동 경유 항로의 선박 스케줄 및 운임 변동을 면밀히 주시하고, 필요시 대체 운송 경로 및 운송사 확보 방안을 즉시 검토해야 한다.</t>
+        </is>
+      </c>
+      <c r="H284" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I284" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260629-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J284" s="2" t="inlineStr">
+        <is>
+          <t>RSK-043</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B285" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C285" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D285" s="2" t="inlineStr">
+        <is>
+          <t>"트럼프 신규 관세 피하자"…기업들 선적 경쟁에 해상 운임 급등</t>
+        </is>
+      </c>
+      <c r="E285" s="2" t="inlineStr">
+        <is>
+          <t>미국의 새로운 관세 부과를 앞두고 기업들이 재고를 미리 확보하려는 선적 경쟁이 심화되면서 해상 화물 운임이 2년 만에 최고치로 치솟았다.</t>
+        </is>
+      </c>
+      <c r="F285" s="2" t="inlineStr">
+        <is>
+          <t>미국의 관세 부과 우려로 인한 선적 경쟁은 해상 운임 상승을 가속화하며, 이는 미국향 물량을 포함한 우리 회사의 물류 비용에 직접적인 부담을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="G285" s="2" t="inlineStr">
+        <is>
+          <t>미국향 물량의 운임 변동 추이를 면밀히 모니터링하고, 관세 부과 시나리오에 따른 재고 전략 및 운송 계획 조정 가능성을 검토해야 한다.</t>
+        </is>
+      </c>
+      <c r="H285" s="2" t="inlineStr">
+        <is>
+          <t>newspim</t>
+        </is>
+      </c>
+      <c r="I285" s="2" t="inlineStr">
+        <is>
+          <t>https://www.newspim.com/news/view/20260629001067</t>
+        </is>
+      </c>
+      <c r="J285" s="2" t="inlineStr">
+        <is>
+          <t>RSK-044</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B286" s="2" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C286" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D286" s="2" t="inlineStr">
+        <is>
+          <t>광주·전남 통합 맞춰 위험물 안전관리 기준 일원화…7월부터 과태료 강화</t>
+        </is>
+      </c>
+      <c r="E286" s="2" t="inlineStr">
+        <is>
+          <t>7월부터 광주·전남 지역의 위험물 안전관리 행정 기준이 통합되며, 1회 위반 시부터 과태료가 부과되는 등 규제가 강화된다.</t>
+        </is>
+      </c>
+      <c r="F286" s="2" t="inlineStr">
+        <is>
+          <t>특정 지역의 위험물 안전관리 기준이 통합되고 강화되는 것은 해당 지역을 경유하거나 해당 지역에 물류 거점이 있는 경우 즉각적인 운영 변경 및 준수 필요성을 야기한다.</t>
+        </is>
+      </c>
+      <c r="G286" s="2" t="inlineStr">
+        <is>
+          <t>광주/전남 지역 물류 운영 및 창고 관리 규정 즉시 검토 및 필요 시 절차 업데이트, 관련 직원 교육.</t>
+        </is>
+      </c>
+      <c r="H286" s="2" t="inlineStr">
+        <is>
+          <t>GETNEWS</t>
+        </is>
+      </c>
+      <c r="I286" s="2" t="inlineStr">
+        <is>
+          <t>https://www.getnews.co.kr/news/articleView.html?idxno=873627</t>
+        </is>
+      </c>
+      <c r="J286" s="2" t="inlineStr">
+        <is>
+          <t>RSK-045</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B287" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C287" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D287" s="2" t="inlineStr">
+        <is>
+          <t>"트럼프 신규 관세 피하자"…기업들 선적 경쟁에 해상 운임 급등</t>
+        </is>
+      </c>
+      <c r="E287" s="2" t="inlineStr">
+        <is>
+          <t>트럼프 전 대통령의 신규 관세 부과를 앞두고 기업들이 재고를 미리 확보하려는 선적 경쟁으로 해상 화물 운임이 2년 전 '홍해 위기' 이후 최고치로 치솟았다.</t>
+        </is>
+      </c>
+      <c r="F287" s="2" t="inlineStr">
+        <is>
+          <t>미국의 관세 부과 우려로 인한 선적 경쟁은 해상 운임을 즉각적으로 상승시켜 당사의 수출입 물류 비용에 직접적인 영향을 미친다.</t>
+        </is>
+      </c>
+      <c r="G287" s="2" t="inlineStr">
+        <is>
+          <t>단기 운송 계획 재검토, 장기 운송 계약 조건 확인, 대체 운송 수단(항공 등)의 비용 효율성 분석, 재고 전략 조정 검토.</t>
+        </is>
+      </c>
+      <c r="H287" s="2" t="inlineStr">
+        <is>
+          <t>뉴스핌</t>
+        </is>
+      </c>
+      <c r="I287" s="2" t="inlineStr">
+        <is>
+          <t>https://newspim.com/news/view/20260629001067</t>
+        </is>
+      </c>
+      <c r="J287" s="2" t="inlineStr">
+        <is>
+          <t>RSK-046</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B288" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C288" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D288" s="2" t="inlineStr">
+        <is>
+          <t>휴전은 왜 일주일도 버티지 못했나… 호르무즈가 다시 세계를 흔들고 있다</t>
+        </is>
+      </c>
+      <c r="E288" s="2" t="inlineStr">
+        <is>
+          <t>미국과 이란의 중동 정세 불안이 호르무즈 해협에서의 민간 선박 공격으로 다시 고조되고 있으며, 이는 국제 유가 및 해상 운송에 영향을 미칠 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="F288" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협은 주요 원유 수송로이자 해상 운송의 핵심 길목으로, 분쟁 심화 시 유가 급등 및 해상 운송 차질, 보험료 인상 등 물류 비용 및 안정성에 직접적인 영향을 미칠 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G288" s="2" t="inlineStr">
+        <is>
+          <t>중동발 원유 및 원자재 가격 변동성 모니터링 강화, 대체 운송 경로 및 재고 확보 방안 검토, 해상 보험 조건 변화 주시.</t>
+        </is>
+      </c>
+      <c r="H288" s="2" t="inlineStr">
+        <is>
+          <t>시사프리즘(GIPRISM)</t>
+        </is>
+      </c>
+      <c r="I288" s="2" t="inlineStr">
+        <is>
+          <t>https://giprism.com/news/articleView.html?idxno=12376</t>
+        </is>
+      </c>
+      <c r="J288" s="2" t="inlineStr">
+        <is>
+          <t>RSK-047</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B289" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C289" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D289" s="2" t="inlineStr">
+        <is>
+          <t>[국제유가] 미·이란 군사 충돌 여파에 반등…WTI 70달러선 회복</t>
+        </is>
+      </c>
+      <c r="E289" s="2" t="inlineStr">
+        <is>
+          <t>미국과 이란의 군사 충돌 여파로 국제 유가가 반등하여 WTI가 70달러선을 회복했으며, 중동 정세 불안으로 인한 원유 공급 차질 우려가 지속되고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F289" s="2" t="inlineStr">
+        <is>
+          <t>국제 유가 상승은 해상 및 항공 운임의 유류할증료 인상으로 이어져 물류비용에 직접적인 영향을 미치므로 즉각적인 대응이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G289" s="2" t="inlineStr">
+        <is>
+          <t>유가 및 유류할증료 변동 추이 실시간 모니터링, 운송 계약 시 유류할증료 조건 재검토, 운송비용 절감 방안 모색.</t>
+        </is>
+      </c>
+      <c r="H289" s="2" t="inlineStr">
+        <is>
+          <t>굿모닝경제</t>
+        </is>
+      </c>
+      <c r="I289" s="2" t="inlineStr">
+        <is>
+          <t>https://www.goodkyung.com/news/articleView.html?idxno=288676</t>
+        </is>
+      </c>
+      <c r="J289" s="2" t="inlineStr">
+        <is>
+          <t>RSK-048</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B290" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C290" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D290" s="3" t="inlineStr">
+        <is>
+          <t>Air Cargo Demand up 6.0% in May</t>
+        </is>
+      </c>
+      <c r="E290" s="3" t="inlineStr">
+        <is>
+          <t>IATA에 따르면 2026년 5월 전 세계 항공 화물 수요가 전년 동월 대비 6.0% 증가했다.</t>
+        </is>
+      </c>
+      <c r="F290" s="3" t="inlineStr">
+        <is>
+          <t>항공 화물 수요 증가는 운임 상승 압력 및 항공 화물 공간 확보의 어려움으로 이어질 수 있어 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G290" s="3" t="inlineStr">
+        <is>
+          <t>항공 운임 및 가용 공간 추이 모니터링, 포워더와 긴밀한 소통을 통해 잠재적 운송 지연 및 비용 상승에 대비.</t>
+        </is>
+      </c>
+      <c r="H290" s="3" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I290" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-29-air-cargo-demand-up-may/</t>
+        </is>
+      </c>
+      <c r="J290" s="3" t="inlineStr"/>
+    </row>
+    <row r="291">
+      <c r="A291" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B291" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C291" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D291" s="3" t="inlineStr">
+        <is>
+          <t>이 대통령 “우리 선박 호르무즈 해협서 2척 빼고 빠져나와”</t>
+        </is>
+      </c>
+      <c r="E291" s="3" t="inlineStr">
+        <is>
+          <t>대통령이 호르무즈 해협에서 우리 선박 대부분이 벗어났다고 밝혔으나, 공급망 및 경제 불확실성에 대비한 위기관리는 여전히 필요하다.</t>
+        </is>
+      </c>
+      <c r="F291" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협의 지정학적 리스크는 중동발 해상 운송에 직접적인 영향을 미치며, 유가 상승 및 해상 운임 변동 가능성이 있어 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G291" s="3" t="inlineStr">
+        <is>
+          <t>중동 지역 정세 변화 및 해상 운송 경로의 잠재적 위험을 지속적으로 모니터링하고, 비상 운송 계획 수립을 검토한다.</t>
+        </is>
+      </c>
+      <c r="H291" s="3" t="inlineStr">
+        <is>
+          <t>kita</t>
+        </is>
+      </c>
+      <c r="I291" s="3" t="inlineStr">
+        <is>
+          <t>https://www.kita.net/shippers/board/newsView.do?morgueCode=2&amp;dataCls=B&amp;dataSeq=8142</t>
+        </is>
+      </c>
+      <c r="J291" s="3" t="inlineStr"/>
+    </row>
+    <row r="292">
+      <c r="A292" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B292" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C292" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D292" s="3" t="inlineStr">
+        <is>
+          <t>(GIM)中, 日 기업 대상 이중용도 품목 수출통제 및 심사 강화6.29</t>
+        </is>
+      </c>
+      <c r="E292" s="3" t="inlineStr">
+        <is>
+          <t>중국이 일본 기업을 대상으로 이중용도 품목에 대한 수출 통제 및 심사를 강화하고 있어, 관련 기업들의 공급망에 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="F292" s="3" t="inlineStr">
+        <is>
+          <t>이중용도 품목에 대한 수출 통제 강화는 우리 회사가 일본에서 조달하는 부품이나 중국으로 수출하는 제품에 영향을 미칠 수 있으므로, 관련 규제 변화를 면밀히 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G292" s="3" t="inlineStr">
+        <is>
+          <t>중국의 이중용도 품목 수출 통제 대상 및 범위에 대한 상세 정보 파악, 일본 공급망 내 해당 품목 여부 확인, 잠재적 영향 분석 및 대체 조달처 검토.</t>
+        </is>
+      </c>
+      <c r="H292" s="3" t="inlineStr">
+        <is>
+          <t>kotra</t>
+        </is>
+      </c>
+      <c r="I292" s="3" t="inlineStr">
+        <is>
+          <t>https://dream.kotra.or.kr/kotranews/cms/news/actionKotraBoardDetail.do?SITE_NO=3&amp;MENU_ID=70&amp;CONTENTS_NO=1&amp;pNttSn=242516</t>
+        </is>
+      </c>
+      <c r="J292" s="3" t="inlineStr"/>
+    </row>
+    <row r="293">
+      <c r="A293" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B293" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C293" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D293" s="3" t="inlineStr">
+        <is>
+          <t>Transpacific: Ripe for new non-alliance services</t>
+        </is>
+      </c>
+      <c r="E293" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence는 태평양 횡단 노선에서 비동맹 선사 서비스의 새로운 기회가 있음을 분석하며, 이는 운임 및 가용성에 영향을 미칠 수 있다고 밝혔다.</t>
+        </is>
+      </c>
+      <c r="F293" s="3" t="inlineStr">
+        <is>
+          <t>태평양 횡단 노선의 서비스 변화 가능성은 해당 노선을 이용하는 우리 회사의 운송 옵션 및 운임에 영향을 줄 수 있으므로 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G293" s="3" t="inlineStr">
+        <is>
+          <t>태평양 횡단 노선의 신규 서비스 동향 및 운임 변화를 모니터링하고, 필요시 포워더와 협의하여 운송 전략을 조정한다.</t>
+        </is>
+      </c>
+      <c r="H293" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I293" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/393-transpacific-ripe-for-new-non-alliance-services</t>
+        </is>
+      </c>
+      <c r="J293" s="3" t="inlineStr"/>
+    </row>
+    <row r="294">
+      <c r="A294" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B294" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C294" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D294" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 무력 공방에 국제유가 상승 및 물류비 하락 어려움 전망</t>
+        </is>
+      </c>
+      <c r="E294" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 인근 무력 공방 등 지정학적 긴장으로 국제유가가 상승 압력을 받고 있으며, 해협 휴전 합의에도 불구하고 급격한 물량 유입으로 글로벌 컨테이너 공급망 지연이 예상되어 유가 및 운임이 쉽게 내려가지 않을 것이라는 분석이다.</t>
+        </is>
+      </c>
+      <c r="F294" s="3" t="inlineStr">
+        <is>
+          <t>유가 상승은 해상 및 항공 운임에 직접적인 영향을 미쳐 물류비 증가로 이어질 수 있으며, 하락 요인이 제한적이라는 분석은 지속적인 비용 부담을 시사한다.</t>
+        </is>
+      </c>
+      <c r="G294" s="3" t="inlineStr">
+        <is>
+          <t>유가 및 운임 변동 추이를 지속적으로 모니터링하고, 물류비용 증가에 대비한 예산 및 운송 전략을 검토해야 한다.</t>
+        </is>
+      </c>
+      <c r="H294" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I294" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260630-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J294" s="3" t="inlineStr"/>
+    </row>
+    <row r="295">
+      <c r="A295" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B295" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C295" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D295" s="3" t="inlineStr">
+        <is>
+          <t>U.S. Bank Freight Payment Index shows spot rates surging 31%</t>
+        </is>
+      </c>
+      <c r="E295" s="3" t="inlineStr">
+        <is>
+          <t>U.S. Bank Freight Payment Index에 따르면 2026년 5월 건식 밴 스팟 운임이 전년 대비 31% 급등했으며, 이는 공급 부족으로 인한 트럭 운임 재조정 때문이다.</t>
+        </is>
+      </c>
+      <c r="F295" s="3" t="inlineStr">
+        <is>
+          <t>내륙 운송 비용 상승 추세는 물류 예산 및 운송 전략에 영향을 미칠 수 있어 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G295" s="3" t="inlineStr">
+        <is>
+          <t>내륙 운송 계약 조건 검토 및 대체 운송 방안(철도 등) 가능성 사전 조사.</t>
+        </is>
+      </c>
+      <c r="H295" s="3" t="inlineStr">
+        <is>
+          <t>FreightWaves</t>
+        </is>
+      </c>
+      <c r="I295" s="3" t="inlineStr">
+        <is>
+          <t>https://www.freightwaves.com/news/us-bank-freight-payment-index-rates</t>
+        </is>
+      </c>
+      <c r="J295" s="3" t="inlineStr"/>
+    </row>
+    <row r="296">
+      <c r="A296" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B296" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C296" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D296" s="3" t="inlineStr">
+        <is>
+          <t>“리튬배터리 설치 공사, 실적 있는 업체만 입찰 참여”:FPN Daily</t>
+        </is>
+      </c>
+      <c r="E296" s="3" t="inlineStr">
+        <is>
+          <t>대전 국가정보자원관리원 화재 이후 리튬배터리 설치 공사에 실적 있는 업체만 입찰에 참여할 수 있도록 규제가 강화될 예정이다.</t>
+        </is>
+      </c>
+      <c r="F296" s="3" t="inlineStr">
+        <is>
+          <t>리튬 배터리 관련 공사 및 설치에 대한 안전 규제 강화는 당사 제품의 최종 설치 및 활용 단계에 간접적인 영향을 미칠 수 있으며, 향후 물류 창고 등 자체 시설에도 유사한 규제가 적용될 가능성이 있다.</t>
+        </is>
+      </c>
+      <c r="G296" s="3" t="inlineStr">
+        <is>
+          <t>관련 규제 동향 지속 모니터링 및 자체 시설 안전 관리 기준 검토.</t>
+        </is>
+      </c>
+      <c r="H296" s="3" t="inlineStr">
+        <is>
+          <t>FPN Daily</t>
+        </is>
+      </c>
+      <c r="I296" s="3" t="inlineStr">
+        <is>
+          <t>https://fpn119.co.kr/sub_read.html?uid=253143</t>
+        </is>
+      </c>
+      <c r="J296" s="3" t="inlineStr"/>
+    </row>
+    <row r="297">
+      <c r="A297" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B297" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C297" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D297" s="3" t="inlineStr">
+        <is>
+          <t>G.ECONOMY(지이코노미)</t>
+        </is>
+      </c>
+      <c r="E297" s="3" t="inlineStr">
+        <is>
+          <t>물류 현장의 안전사고가 잇따르면서 사회적 경각심이 높아지고 있으며, 작은 부주의가 대형 인명 사고로 이어질 수 있음을 강조한다.</t>
+        </is>
+      </c>
+      <c r="F297" s="3" t="inlineStr">
+        <is>
+          <t>물류 현장 전반의 안전사고 증가와 사회적 경각심 고조는 위험물 취급이 많은 당사 물류 운영에 대한 안전 규제 강화로 이어질 수 있다.</t>
+        </is>
+      </c>
+      <c r="G297" s="3" t="inlineStr">
+        <is>
+          <t>물류 창고 및 운송 과정의 안전 절차 재점검 및 직원 교육 강화.</t>
+        </is>
+      </c>
+      <c r="H297" s="3" t="inlineStr">
+        <is>
+          <t>G.ECONOMY(지이코노미)</t>
+        </is>
+      </c>
+      <c r="I297" s="3" t="inlineStr">
+        <is>
+          <t>https://geconomy.co.kr/news/article.html?no=321287</t>
+        </is>
+      </c>
+      <c r="J297" s="3" t="inlineStr"/>
+    </row>
+    <row r="298">
+      <c r="A298" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B298" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C298" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D298" s="3" t="inlineStr">
+        <is>
+          <t>허프포스트코리아</t>
+        </is>
+      </c>
+      <c r="E298" s="3" t="inlineStr">
+        <is>
+          <t>미국이 구리 관세 카드를 다시 꺼낼 가능성이 높아지면서, 글로벌 구리 공급망 재편이 한국 기업의 조달 전략에 직접적인 변수가 될 수 있다.</t>
+        </is>
+      </c>
+      <c r="F298" s="3" t="inlineStr">
+        <is>
+          <t>구리는 배터리 및 전자부품 제조의 핵심 원자재이므로, 미국의 구리 관세 부과는 원가 상승 및 공급망 불안정으로 이어질 수 있다.</t>
+        </is>
+      </c>
+      <c r="G298" s="3" t="inlineStr">
+        <is>
+          <t>구리 조달처 다변화 가능성 검토, 관세 부과 시나리오별 원가 영향 분석.</t>
+        </is>
+      </c>
+      <c r="H298" s="3" t="inlineStr">
+        <is>
+          <t>허프포스트코리아</t>
+        </is>
+      </c>
+      <c r="I298" s="3" t="inlineStr">
+        <is>
+          <t>https://huffingtonpost.kr/article/258311</t>
+        </is>
+      </c>
+      <c r="J298" s="3" t="inlineStr"/>
+    </row>
+    <row r="299">
+      <c r="A299" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B299" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C299" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D299" s="3" t="inlineStr">
+        <is>
+          <t>관세청·무역위원회, 불공정 덤핑행위 차단 공조 강화</t>
+        </is>
+      </c>
+      <c r="E299" s="3" t="inlineStr">
+        <is>
+          <t>관세청과 무역위원회가 우회 덤핑 가능성이 높은 수입 물품에 대한 분석 정보를 공유하며 불공정 덤핑 행위 차단 공조를 강화하여 국내 산업 피해를 예방합니다.</t>
+        </is>
+      </c>
+      <c r="F299" s="3" t="inlineStr">
+        <is>
+          <t>수입하는 전자부품이나 원자재에 대한 덤핑 규제 강화는 향후 수입 단가 및 공급처 다변화 전략에 영향을 줄 수 있으므로 지속적인 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G299" s="3" t="inlineStr">
+        <is>
+          <t>주요 수입 원자재 및 부품의 원산지 및 수입 가격 동향 모니터링, 덤핑 규제 대상 품목 확대 가능성 주시.</t>
+        </is>
+      </c>
+      <c r="H299" s="3" t="inlineStr">
+        <is>
+          <t>한국세정신문</t>
+        </is>
+      </c>
+      <c r="I299" s="3" t="inlineStr">
+        <is>
+          <t>https://taxtimes.co.kr/news/article.html?no=275751</t>
+        </is>
+      </c>
+      <c r="J299" s="3" t="inlineStr"/>
+    </row>
+    <row r="300">
+      <c r="A300" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B300" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C300" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D300" s="3" t="inlineStr">
+        <is>
+          <t>코레일 자회사 5곳→3곳으로 개편…서비스·물류·유지관리로 통합</t>
+        </is>
+      </c>
+      <c r="E300" s="3" t="inlineStr">
+        <is>
+          <t>한국철도공사(코레일) 자회사가 고객서비스, 유통·물류, 유지관리 3개사 체제로 재편되어 철도 이용 편의와 안전성을 높이고 물류 분야 전문성을 강화할 예정입니다.</t>
+        </is>
+      </c>
+      <c r="F300" s="3" t="inlineStr">
+        <is>
+          <t>코레일 자회사 개편으로 국내 철도 물류 서비스의 효율성 및 안정성 변화 가능성이 있으므로, 국내 운송 전략에 미칠 영향을 모니터링할 필요가 있습니다.</t>
+        </is>
+      </c>
+      <c r="G300" s="3" t="inlineStr">
+        <is>
+          <t>국내 철도 운송을 활용하는 경우, 코레일 자회사 개편에 따른 서비스 변화 및 운임 정책 변화 여부 확인.</t>
+        </is>
+      </c>
+      <c r="H300" s="3" t="inlineStr">
+        <is>
+          <t>뉴스핌</t>
+        </is>
+      </c>
+      <c r="I300" s="3" t="inlineStr">
+        <is>
+          <t>https://newspim.com/news/view/20260630001134</t>
+        </is>
+      </c>
+      <c r="J300" s="3" t="inlineStr"/>
+    </row>
+    <row r="301">
+      <c r="A301" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B301" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C301" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D301" s="3" t="inlineStr">
+        <is>
+          <t>서울 기름값, 2개월 만에 1900원대…휘발유·경유 동반 하락</t>
+        </is>
+      </c>
+      <c r="E301" s="3" t="inlineStr">
+        <is>
+          <t>국제유가 하락과 정부의 석유 최고가격 인하가 맞물리면서 서울 지역 휘발유와 경유 평균 판매가격이 약 2개월 만에 1900원대로 내려왔습니다.</t>
+        </is>
+      </c>
+      <c r="F301" s="3" t="inlineStr">
+        <is>
+          <t>국내 유가 하락은 국내 육상 운송 비용 절감에 긍정적인 영향을 줄 수 있으나, 국제 유가 변동성이 커 지속적인 추이 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G301" s="3" t="inlineStr">
+        <is>
+          <t>국내 운송 계약 시 유류할증료 조건 재검토, 국내 운송비용 절감 기회 모색.</t>
+        </is>
+      </c>
+      <c r="H301" s="3" t="inlineStr">
+        <is>
+          <t>시사저널</t>
+        </is>
+      </c>
+      <c r="I301" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sisajournal.com/news/articleView.html?idxno=378001</t>
+        </is>
+      </c>
+      <c r="J301" s="3" t="inlineStr"/>
+    </row>
+    <row r="302">
+      <c r="A302" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B302" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C302" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D302" s="4" t="inlineStr">
+        <is>
+          <t>Global Schedule Reliability for May 2026 the Highest of the Year</t>
+        </is>
+      </c>
+      <c r="E302" s="4" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence 보고서에 따르면 2026년 5월 전 세계 선박 스케줄 정시성이 올해 최고치를 기록하며 개선되었다.</t>
+        </is>
+      </c>
+      <c r="F302" s="4" t="inlineStr">
+        <is>
+          <t>선박 스케줄 정시성 개선은 해상 운송의 안정성 증가를 의미하나, 이는 일반적인 시장 동향으로 당장 우리 물류 운영에 즉각적인 변화를 요구하지는 않는다.</t>
+        </is>
+      </c>
+      <c r="G302" s="4" t="inlineStr"/>
+      <c r="H302" s="4" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I302" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/395-global-schedule-reliability-for-may-2026-the-highest-of-the-year</t>
+        </is>
+      </c>
+      <c r="J302" s="4" t="inlineStr"/>
+    </row>
+    <row r="303">
+      <c r="A303" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B303" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C303" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D303" s="4" t="inlineStr">
+        <is>
+          <t>씨메스로보틱스, 피지컬 AI 기반 로봇 자동화 사업 확대</t>
+        </is>
+      </c>
+      <c r="E303" s="4" t="inlineStr">
+        <is>
+          <t>씨메스로보틱스가 물류 및 제조 현장에서 피지컬 AI 기반 로봇 자동화 사업을 확대하며 대형 프로젝트를 연이어 수주, 사상 최대 분기 매출을 달성했다.</t>
+        </is>
+      </c>
+      <c r="F303" s="4" t="inlineStr">
+        <is>
+          <t>물류 자동화 기술 발전 동향을 파악하는 데 참고할 수 있으나, 우리 회사의 현재 물류 운영에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G303" s="4" t="n"/>
+      <c r="H303" s="4" t="inlineStr">
+        <is>
+          <t>ulogistics</t>
+        </is>
+      </c>
+      <c r="I303" s="4" t="inlineStr">
+        <is>
+          <t>http://www.ulogistics.co.kr/test/board.php?board=all2&amp;command=body&amp;no=5202</t>
+        </is>
+      </c>
+      <c r="J303" s="4" t="inlineStr"/>
+    </row>
+    <row r="304">
+      <c r="A304" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B304" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C304" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D304" s="4" t="inlineStr">
+        <is>
+          <t>(주)한진, 글로벌 물류 매출 성장 및 택배 시장 경쟁 심화</t>
+        </is>
+      </c>
+      <c r="E304" s="4" t="inlineStr">
+        <is>
+          <t>(주)한진의 글로벌 물류 부문 매출액이 2년 사이 2배 가까이 성장하며 국내 물류(택배 제외)를 빠르게 따라잡고 있으며, 택배 시장에서는 서비스 차별화 경쟁이 심화되고 있다.</t>
+        </is>
+      </c>
+      <c r="F304" s="4" t="inlineStr">
+        <is>
+          <t>물류 서비스 제공업체의 사업 동향을 파악하는 데 참고할 수 있으나, 우리 회사의 직접적인 운송 지연, 비용, 규제 등에는 영향이 없다.</t>
+        </is>
+      </c>
+      <c r="G304" s="4" t="n"/>
+      <c r="H304" s="4" t="inlineStr">
+        <is>
+          <t>shippingnews</t>
+        </is>
+      </c>
+      <c r="I304" s="4" t="inlineStr">
+        <is>
+          <t>https://www.shippingnewsnet.com/news/articleView.html?idxno=70973</t>
+        </is>
+      </c>
+      <c r="J304" s="4" t="inlineStr"/>
+    </row>
+    <row r="305">
+      <c r="A305" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B305" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C305" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D305" s="4" t="inlineStr">
+        <is>
+          <t>글로벌 선박 엔진 품귀 현상 재등장, 한국 조선업계 반사이익 기대</t>
+        </is>
+      </c>
+      <c r="E305" s="4" t="inlineStr">
+        <is>
+          <t>전 세계 조선업계에 선박 엔진 부족 현상이 다시 발생하여 기록적인 신조선 건조 물량 소화에 어려움이 예상되며, 이는 한국 조선업계에 반사이익을 가져올 수 있다.</t>
+        </is>
+      </c>
+      <c r="F305" s="4" t="inlineStr">
+        <is>
+          <t>선박 엔진 품귀는 장기적으로 선박 공급에 영향을 줄 수 있으나, 우리 회사의 단기적인 물류 운영에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G305" s="4" t="n"/>
+      <c r="H305" s="4" t="inlineStr">
+        <is>
+          <t>ebn</t>
+        </is>
+      </c>
+      <c r="I305" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ebn.co.kr/news/articleView.html?idxno=1714238</t>
+        </is>
+      </c>
+      <c r="J305" s="4" t="inlineStr"/>
+    </row>
+    <row r="306">
+      <c r="A306" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B306" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C306" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D306" s="4" t="inlineStr">
+        <is>
+          <t>GHX, AI 기반 공급망 혼란 감지 및 회복력 구축 솔루션 발표</t>
+        </is>
+      </c>
+      <c r="E306" s="4" t="inlineStr">
+        <is>
+          <t>GHX가 공급망 혼란을 감지하고 회복력을 구축하기 위한 새로운 AI 기반 오케스트레이션 레이어를 발표하며 공급망 절차 간소화를 목표로 한다.</t>
+        </is>
+      </c>
+      <c r="F306" s="4" t="inlineStr">
+        <is>
+          <t>공급망 기술 동향을 파악하는 데 참고할 수 있으나, 우리 회사의 현재 물류 운영에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G306" s="4" t="n"/>
+      <c r="H306" s="4" t="inlineStr">
+        <is>
+          <t>HPN Online</t>
+        </is>
+      </c>
+      <c r="I306" s="4" t="inlineStr">
+        <is>
+          <t>https://www.hpnonline.com/sourcing-logistics/news/55387397/ghx-announces-new-ai-powered-orchestration-layer-to-sense-supply-chain-disruption</t>
+        </is>
+      </c>
+      <c r="J306" s="4" t="inlineStr"/>
+    </row>
+    <row r="307">
+      <c r="A307" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B307" s="4" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C307" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D307" s="4" t="inlineStr">
+        <is>
+          <t>“화재 예방 위해” 서울 지하철, 대용량 리튬 배터리 반입 금지</t>
+        </is>
+      </c>
+      <c r="E307" s="4" t="inlineStr">
+        <is>
+          <t>서울교통공사가 내달 1일부터 서울 지하철에 대용량 리튬 배터리와 리튬 배터리 구동 개인형 이동장치(PM)의 반입을 제한하여 화재 위험을 차단한다.</t>
+        </is>
+      </c>
+      <c r="F307" s="4" t="inlineStr">
+        <is>
+          <t>당사 제품의 대량 운송에는 직접적인 영향이 없으나, 리튬 배터리에 대한 대중의 안전 우려와 규제 강화 추세를 보여준다.</t>
+        </is>
+      </c>
+      <c r="G307" s="4" t="n"/>
+      <c r="H307" s="4" t="inlineStr">
+        <is>
+          <t>헬스조선</t>
+        </is>
+      </c>
+      <c r="I307" s="4" t="inlineStr">
+        <is>
+          <t>https://health.chosun.com/site/data/html_dir/2026/06/29/2026062901814.html</t>
+        </is>
+      </c>
+      <c r="J307" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
@@ -14173,7 +15325,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I43"/>
+  <dimension ref="A1:I49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15704,6 +16856,216 @@
       </c>
       <c r="I43" s="6" t="inlineStr"/>
     </row>
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>RSK-043</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D44" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E44" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 지정학적 리스크 재확대 및 해운운임 9주 연속 상승</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="inlineStr"/>
+      <c r="G44" s="6" t="inlineStr"/>
+      <c r="H44" s="6" t="inlineStr">
+        <is>
+          <t>중동 경유 항로의 선박 스케줄 및 운임 변동을 면밀히 주시하고, 필요시 대체 운송 경로 및 운송사 확보 방안을 즉시 검토해야 한다.</t>
+        </is>
+      </c>
+      <c r="I44" s="6" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>RSK-044</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D45" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E45" s="6" t="inlineStr">
+        <is>
+          <t>"트럼프 신규 관세 피하자"…기업들 선적 경쟁에 해상 운임 급등</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="inlineStr"/>
+      <c r="G45" s="6" t="inlineStr"/>
+      <c r="H45" s="6" t="inlineStr">
+        <is>
+          <t>미국향 물량의 운임 변동 추이를 면밀히 모니터링하고, 관세 부과 시나리오에 따른 재고 전략 및 운송 계획 조정 가능성을 검토해야 한다.</t>
+        </is>
+      </c>
+      <c r="I45" s="6" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>RSK-045</t>
+        </is>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="D46" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E46" s="6" t="inlineStr">
+        <is>
+          <t>광주·전남 통합 맞춰 위험물 안전관리 기준 일원화…7월부터 과태료 강화</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="inlineStr"/>
+      <c r="G46" s="6" t="inlineStr"/>
+      <c r="H46" s="6" t="inlineStr">
+        <is>
+          <t>광주/전남 지역 물류 운영 및 창고 관리 규정 즉시 검토 및 필요 시 절차 업데이트, 관련 직원 교육.</t>
+        </is>
+      </c>
+      <c r="I46" s="6" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t>RSK-046</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D47" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E47" s="6" t="inlineStr">
+        <is>
+          <t>"트럼프 신규 관세 피하자"…기업들 선적 경쟁에 해상 운임 급등</t>
+        </is>
+      </c>
+      <c r="F47" s="6" t="inlineStr"/>
+      <c r="G47" s="6" t="inlineStr"/>
+      <c r="H47" s="6" t="inlineStr">
+        <is>
+          <t>단기 운송 계획 재검토, 장기 운송 계약 조건 확인, 대체 운송 수단(항공 등)의 비용 효율성 분석, 재고 전략 조정 검토.</t>
+        </is>
+      </c>
+      <c r="I47" s="6" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>RSK-047</t>
+        </is>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D48" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E48" s="6" t="inlineStr">
+        <is>
+          <t>휴전은 왜 일주일도 버티지 못했나… 호르무즈가 다시 세계를 흔들고 있다</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="inlineStr"/>
+      <c r="G48" s="6" t="inlineStr"/>
+      <c r="H48" s="6" t="inlineStr">
+        <is>
+          <t>중동발 원유 및 원자재 가격 변동성 모니터링 강화, 대체 운송 경로 및 재고 확보 방안 검토, 해상 보험 조건 변화 주시.</t>
+        </is>
+      </c>
+      <c r="I48" s="6" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t>RSK-048</t>
+        </is>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D49" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E49" s="6" t="inlineStr">
+        <is>
+          <t>[국제유가] 미·이란 군사 충돌 여파에 반등…WTI 70달러선 회복</t>
+        </is>
+      </c>
+      <c r="F49" s="6" t="inlineStr"/>
+      <c r="G49" s="6" t="inlineStr"/>
+      <c r="H49" s="6" t="inlineStr">
+        <is>
+          <t>유가 및 유류할증료 변동 추이 실시간 모니터링, 운송 계약 시 유류할증료 조건 재검토, 운송비용 절감 방안 모색.</t>
+        </is>
+      </c>
+      <c r="I49" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
📰 뉴스 데이터 2026-07-01_09:13
</commit_message>
<xml_diff>
--- a/data/SCM_물류_브리핑.xlsx
+++ b/data/SCM_물류_브리핑.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J307"/>
+  <dimension ref="A1:J331"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14982,6 +14982,1138 @@
       </c>
       <c r="J307" s="4" t="inlineStr"/>
     </row>
+    <row r="308">
+      <c r="A308" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B308" s="2" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C308" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D308" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 내 한국 선박 2척 추가 탈출...3척만 남아</t>
+        </is>
+      </c>
+      <c r="E308" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협에 3척의 한국 선박이 남아있어 해협 통항의 불확실성이 지속되며 물류 지연 및 운송 리스크가 상존한다.</t>
+        </is>
+      </c>
+      <c r="F308" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협은 주요 원자재 및 에너지 운송의 핵심 통로로, 통항 불확실성은 우리 회사의 원자재 수급 및 제품 운송에 직접적인 지연과 비용 상승을 초래할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G308" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 통항 상황을 실시간으로 모니터링하고, 해당 경로를 이용하는 선박의 안전 확보 및 대체 운송 경로(예: 육상 운송, 항공 운송) 또는 재고 확보 방안을 긴급 검토해야 함.</t>
+        </is>
+      </c>
+      <c r="H308" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I308" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260629-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J308" s="2" t="inlineStr">
+        <is>
+          <t>RSK-049</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B309" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C309" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D309" s="2" t="inlineStr">
+        <is>
+          <t>글로벌 해운운임, 9주 연속 상승…3200대 돌파</t>
+        </is>
+      </c>
+      <c r="E309" s="2" t="inlineStr">
+        <is>
+          <t>상하이컨테이너운임지수(SCFI)가 9주 연속 상승하여 3200선을 돌파하며 글로벌 해상물류 비용 부담이 크게 증가하고 있다.</t>
+        </is>
+      </c>
+      <c r="F309" s="2" t="inlineStr">
+        <is>
+          <t>해운 운임의 지속적인 급등은 우리 회사의 수출입 물류비용을 직접적으로 증가시켜 수익성에 악영향을 미치고, 제품 가격 경쟁력에도 부담을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="G309" s="2" t="inlineStr">
+        <is>
+          <t>현재 운송 계약 조건을 재검토하고, 장기 운송 계약 협상, 선사 다변화, 운송 모드 전환(예: 항공 운송 검토) 등 물류비 절감 및 안정화 방안을 즉시 강구해야 함.</t>
+        </is>
+      </c>
+      <c r="H309" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I309" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260629-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J309" s="2" t="inlineStr">
+        <is>
+          <t>RSK-050</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B310" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C310" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D310" s="2" t="inlineStr">
+        <is>
+          <t>미-이란, 호르무즈 무력 충돌 재개...중동발 에너지·해상운송 리스크 확대</t>
+        </is>
+      </c>
+      <c r="E310" s="2" t="inlineStr">
+        <is>
+          <t>미국과 이란의 호르무즈 해협 무력 충돌이 재개되고 이스라엘의 레바논 공격까지 겹치며 중동발 에너지 및 해상운송 리스크가 크게 확대되고 있다.</t>
+        </is>
+      </c>
+      <c r="F310" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협의 군사적 긴장 고조는 주요 해상 운송로의 봉쇄 또는 지연 가능성을 높여 원자재 수급 및 제품 운송에 심각한 차질과 물류비 급등을 야기할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G310" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협을 경유하는 모든 운송 계획을 즉시 재검토하고, 대체 운송 경로 및 수단 확보, 비상 재고 확충 등 비상 계획을 수립 및 실행해야 함.</t>
+        </is>
+      </c>
+      <c r="H310" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I310" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260628-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J310" s="2" t="inlineStr">
+        <is>
+          <t>RSK-051</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B311" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C311" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D311" s="2" t="inlineStr">
+        <is>
+          <t>[국제유가] 미·이란 군사 충돌 여파에 반등…WTI 70달러선 회복 &lt; 국제 &lt; 세계 &lt; 기사본문 - 굿모닝경제</t>
+        </is>
+      </c>
+      <c r="E311" s="2" t="inlineStr">
+        <is>
+          <t>미국과 이란의 군사 충돌 여파로 국제유가가 반등하여 서부 텍사스산 원유(WTI)가 70달러선을 회복했으며, 중동 정세 불안정으로 인한 원유 공급 차질 우려가 지속되고 있다.</t>
+        </is>
+      </c>
+      <c r="F311" s="2" t="inlineStr">
+        <is>
+          <t>국제유가 반등은 해상 및 항공 운임 상승으로 직결되어 우리 회사의 물류비용에 즉각적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G311" s="2" t="inlineStr">
+        <is>
+          <t>유가 변동에 따른 운임 인상 가능성 대비, 운송 계약 조건 재검토 및 대체 운송 방안 마련 검토.</t>
+        </is>
+      </c>
+      <c r="H311" s="2" t="inlineStr">
+        <is>
+          <t>굿모닝경제</t>
+        </is>
+      </c>
+      <c r="I311" s="2" t="inlineStr">
+        <is>
+          <t>https://www.goodkyung.com/news/articleView.html?idxno=288676</t>
+        </is>
+      </c>
+      <c r="J311" s="2" t="inlineStr">
+        <is>
+          <t>RSK-052</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B312" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C312" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D312" s="3" t="inlineStr">
+        <is>
+          <t>美, USMCA 연장 거부 방침… 북미 자유무역체제 ‘중대 분수령’</t>
+        </is>
+      </c>
+      <c r="E312" s="3" t="inlineStr">
+        <is>
+          <t>미국이 USMCA 연장 거부 방침을 밝히며 북미 자유무역체제에 중대 분수령을 맞게 되어, 북미 지역과의 무역 환경 변화가 예상된다.</t>
+        </is>
+      </c>
+      <c r="F312" s="3" t="inlineStr">
+        <is>
+          <t>북미 지역으로의 수출입 관세 및 무역 조건에 변화가 생길 수 있어 향후 우리 제품의 북미 시장 공급망 전략에 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G312" s="3" t="inlineStr">
+        <is>
+          <t>북미 지역 무역 정책 변화 동향을 지속적으로 모니터링하고, 잠재적 관세 및 규제 변화에 대비한 시나리오를 검토해야 함.</t>
+        </is>
+      </c>
+      <c r="H312" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I312" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260701-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J312" s="3" t="inlineStr"/>
+    </row>
+    <row r="313">
+      <c r="A313" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B313" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C313" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D313" s="3" t="inlineStr">
+        <is>
+          <t>우회덤핑 차단 공조…관세청·무역위 공동 대응</t>
+        </is>
+      </c>
+      <c r="E313" s="3" t="inlineStr">
+        <is>
+          <t>관세청과 무역위원회가 우회덤핑 감시 정보를 공유하고 무역구제 조치 실효성 강화를 논의하며, 불공정 무역 행위에 대한 단속이 강화될 예정이다.</t>
+        </is>
+      </c>
+      <c r="F313" s="3" t="inlineStr">
+        <is>
+          <t>우회덤핑 규제 강화는 특정 원자재나 부품 수입 시 예상치 못한 관세 부과나 통관 지연을 야기할 수 있어 공급망 안정성에 영향을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="G313" s="3" t="inlineStr">
+        <is>
+          <t>주요 원자재 및 부품의 수입 경로와 공급업체에 대한 실사를 강화하고, 무역 규제 변화에 대한 정보를 지속적으로 파악해야 함.</t>
+        </is>
+      </c>
+      <c r="H313" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I313" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260630-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J313" s="3" t="inlineStr"/>
+    </row>
+    <row r="314">
+      <c r="A314" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B314" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C314" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D314" s="3" t="inlineStr">
+        <is>
+          <t>국제유가, 주말 호르무즈 무력공방에 상승…WTI 2%↑</t>
+        </is>
+      </c>
+      <c r="E314" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 인근 무력 공방 등 지정학적 긴장으로 국제유가(WTI)가 2% 상승 압력을 받았다.</t>
+        </is>
+      </c>
+      <c r="F314" s="3" t="inlineStr">
+        <is>
+          <t>국제유가 상승은 해상 및 항공 운임 상승으로 이어져 물류비용 증가에 영향을 미칠 수 있으며, 호르무즈 리스크는 유가 변동성을 높인다.</t>
+        </is>
+      </c>
+      <c r="G314" s="3" t="inlineStr">
+        <is>
+          <t>유가 및 운임 변동 추이를 면밀히 모니터링하고, 장기적인 유가 상승에 대비하여 운송 계약 조건 재검토 및 대체 운송 방안을 고려해야 함.</t>
+        </is>
+      </c>
+      <c r="H314" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I314" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260630-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J314" s="3" t="inlineStr"/>
+    </row>
+    <row r="315">
+      <c r="A315" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B315" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C315" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D315" s="3" t="inlineStr">
+        <is>
+          <t>CPTPP 회원국, 인도네시아·필리핀·UAE와 가입 예비협상 개시</t>
+        </is>
+      </c>
+      <c r="E315" s="3" t="inlineStr">
+        <is>
+          <t>CPTPP가 인도네시아, 필리핀, UAE와 가입 예비협상을 개시하며 역내 포괄적 경제 동반자 협정의 확대 가능성이 커지고 있다.</t>
+        </is>
+      </c>
+      <c r="F315" s="3" t="inlineStr">
+        <is>
+          <t>CPTPP 확대는 해당 국가들과의 무역 환경 변화를 가져올 수 있으며, 장기적으로 우리 회사의 수출입 전략 및 공급망 재편에 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G315" s="3" t="inlineStr">
+        <is>
+          <t>CPTPP 가입 협상 진행 상황을 주시하고, 해당 국가들과의 무역 조건 변화에 따른 기회 및 위협 요인을 분석하여 선제적 대응 방안을 모색해야 함.</t>
+        </is>
+      </c>
+      <c r="H315" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I315" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260628-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J315" s="3" t="inlineStr"/>
+    </row>
+    <row r="316">
+      <c r="A316" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B316" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C316" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D316" s="3" t="inlineStr">
+        <is>
+          <t>Middle East air cargo weakest performance of all regions, IATA data suggests</t>
+        </is>
+      </c>
+      <c r="E316" s="3" t="inlineStr">
+        <is>
+          <t>IATA 데이터에 따르면 중동 지역 항공 화물 실적이 모든 지역 중 가장 저조한 것으로 나타나, 중동발 물류 불안정성이 항공 운송에도 영향을 미치고 있음을 시사한다.</t>
+        </is>
+      </c>
+      <c r="F316" s="3" t="inlineStr">
+        <is>
+          <t>중동 지역의 항공 화물 실적 저조는 해당 지역을 경유하거나 목적지로 하는 항공 운송에 지연 및 비용 상승을 야기할 수 있어 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G316" s="3" t="inlineStr">
+        <is>
+          <t>중동 지역을 경유하는 항공 운송 경로 및 스케줄에 대한 잠재적 영향을 평가하고, 필요시 대체 항공 운송 옵션을 검토해야 함.</t>
+        </is>
+      </c>
+      <c r="H316" s="3" t="inlineStr">
+        <is>
+          <t>Logistics Manager</t>
+        </is>
+      </c>
+      <c r="I316" s="3" t="inlineStr">
+        <is>
+          <t>https://logisticsmanager.com/middle-east-air-cargo-weakest-performance-of-all-regions-iata-data-suggests</t>
+        </is>
+      </c>
+      <c r="J316" s="3" t="inlineStr"/>
+    </row>
+    <row r="317">
+      <c r="A317" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B317" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C317" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D317" s="3" t="inlineStr">
+        <is>
+          <t>7월 1일부터 대용량 리튬배터리 지하철 휴대 불가 :: 공감언론 뉴시스 ::</t>
+        </is>
+      </c>
+      <c r="E317" s="3" t="inlineStr">
+        <is>
+          <t>서울교통공사가 7월 1일부터 대용량 리튬배터리 및 리튬배터리 장착 이동수단의 지하철 반입 및 휴대를 금지합니다. 이는 지하철 내 화재 위험 요인을 줄이기 위한 조치입니다.</t>
+        </is>
+      </c>
+      <c r="F317" s="3" t="inlineStr">
+        <is>
+          <t>대용량 리튬배터리의 대중교통 휴대 금지는 소비자 배송 방식이나 소량 샘플 운송 등 특정 상황에서 물류 방식에 간접적인 영향을 줄 수 있으므로 추이를 모니터링할 필요가 있습니다.</t>
+        </is>
+      </c>
+      <c r="G317" s="3" t="inlineStr">
+        <is>
+          <t>소량 샘플 운송 등 대중교통 이용 가능성이 있는 경우, 대체 운송 방안 검토 및 관련 부서에 정보 공유.</t>
+        </is>
+      </c>
+      <c r="H317" s="3" t="inlineStr">
+        <is>
+          <t>뉴시스</t>
+        </is>
+      </c>
+      <c r="I317" s="3" t="inlineStr">
+        <is>
+          <t>https://newsis.com/view/NISI20260630_0021343535</t>
+        </is>
+      </c>
+      <c r="J317" s="3" t="inlineStr"/>
+    </row>
+    <row r="318">
+      <c r="A318" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B318" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C318" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D318" s="3" t="inlineStr">
+        <is>
+          <t>광주·전남 통합 맞춰 위험물 안전관리 기준 일원화…7월부터 과태료 강화</t>
+        </is>
+      </c>
+      <c r="E318" s="3" t="inlineStr">
+        <is>
+          <t>7월부터 광주·전남 지역의 위험물 안전관리 관련 행정 기준이 통합되고 과태료가 강화됩니다. 이는 기존 광주시와 전남도로 나뉘어 운영되던 규정을 일원화하는 조치입니다.</t>
+        </is>
+      </c>
+      <c r="F318" s="3" t="inlineStr">
+        <is>
+          <t>특정 지역의 위험물 안전관리 기준 일원화 및 과태료 강화는 해당 지역 내 물류 운영 시 규정 준수 및 비용에 영향을 줄 수 있으므로 관련 규정 변화를 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G318" s="3" t="inlineStr">
+        <is>
+          <t>광주/전남 지역 내 위험물 취급 및 운송 시 변경된 안전관리 기준 및 과태료 규정 확인, 관련 부서에 정보 공유.</t>
+        </is>
+      </c>
+      <c r="H318" s="3" t="inlineStr">
+        <is>
+          <t>글로벌이코노믹</t>
+        </is>
+      </c>
+      <c r="I318" s="3" t="inlineStr">
+        <is>
+          <t>https://www.getnews.co.kr/news/articleView.html?idxno=873627</t>
+        </is>
+      </c>
+      <c r="J318" s="3" t="inlineStr"/>
+    </row>
+    <row r="319">
+      <c r="A319" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B319" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C319" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D319" s="3" t="inlineStr">
+        <is>
+          <t>EU, 내달 1일 새 ‘50% 철강 관세 폭탄’ 시행…원산지 규제도 강화 - 이투데이</t>
+        </is>
+      </c>
+      <c r="E319" s="3" t="inlineStr">
+        <is>
+          <t>EU가 7월 1일부터 철강 관세를 기존 25%에서 50%로 인상하고, '용해·주조 규정' 도입을 통해 원산지 검증을 강화합니다. 이는 유럽 철강 시장의 장벽을 높이는 조치입니다.</t>
+        </is>
+      </c>
+      <c r="F319" s="3" t="inlineStr">
+        <is>
+          <t>EU의 철강 관세 및 원산지 규제 강화는 우리 회사가 철강을 직접 사용하지 않더라도, 관련 부품이나 장비의 조달 비용에 간접적인 영향을 미칠 수 있으므로 추이를 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G319" s="3" t="inlineStr">
+        <is>
+          <t>EU로 수출되는 제품 또는 EU에서 조달하는 부품/장비에 철강이 포함될 경우, 원산지 규제 및 관세 인상에 따른 영향 분석 및 대응 방안 검토.</t>
+        </is>
+      </c>
+      <c r="H319" s="3" t="inlineStr">
+        <is>
+          <t>이투데이</t>
+        </is>
+      </c>
+      <c r="I319" s="3" t="inlineStr">
+        <is>
+          <t>https://etoday.co.kr/news/view/2598745</t>
+        </is>
+      </c>
+      <c r="J319" s="3" t="inlineStr"/>
+    </row>
+    <row r="320">
+      <c r="A320" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B320" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C320" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D320" s="3" t="inlineStr">
+        <is>
+          <t>유엔, 호르무즈 재개방에도 식량·연료비 고공행진 경고 By Investing.com</t>
+        </is>
+      </c>
+      <c r="E320" s="3" t="inlineStr">
+        <is>
+          <t>유엔은 호르무즈 해협 재개방에도 불구하고 중동 분쟁으로 인한 공급망 재정비에 시간이 걸려 식량 및 연료비 고공행진이 지속될 수 있다고 경고했다.</t>
+        </is>
+      </c>
+      <c r="F320" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협은 주요 원유 수송로이며, 연료비 상승은 해상/항공 운임에 직접적인 영향을 미쳐 물류비 증가로 이어질 수 있다.</t>
+        </is>
+      </c>
+      <c r="G320" s="3" t="inlineStr">
+        <is>
+          <t>국제 유가 및 해상/항공 운임 추이 지속 모니터링 및 비상 운송 계획 검토.</t>
+        </is>
+      </c>
+      <c r="H320" s="3" t="inlineStr">
+        <is>
+          <t>Investing.com</t>
+        </is>
+      </c>
+      <c r="I320" s="3" t="inlineStr">
+        <is>
+          <t>https://kr.investing.com/news/economy-news/article-93CH-2000462</t>
+        </is>
+      </c>
+      <c r="J320" s="3" t="inlineStr"/>
+    </row>
+    <row r="321">
+      <c r="A321" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B321" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C321" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D321" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 원유 수송 전쟁 전 수준 회복…밴스 "일부 날엔 더 많아" | 아주경제</t>
+        </is>
+      </c>
+      <c r="E321" s="3" t="inlineStr">
+        <is>
+          <t>미국 부통령은 호르무즈 해협을 통한 원유 수송이 중동 전쟁 이전 수준을 회복했다고 밝혀, 원유 공급 안정화에 긍정적인 신호를 보냈다.</t>
+        </is>
+      </c>
+      <c r="F321" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협의 원유 수송량 회복은 유가 안정화에 긍정적 요인이지만, 국제 정세 불안정성 및 공급망 재정비 시간 소요로 인한 유가 변동 가능성은 여전히 존재한다.</t>
+        </is>
+      </c>
+      <c r="G321" s="3" t="inlineStr">
+        <is>
+          <t>국제 유가 및 해상/항공 운임 추이 지속 모니터링.</t>
+        </is>
+      </c>
+      <c r="H321" s="3" t="inlineStr">
+        <is>
+          <t>아주경제</t>
+        </is>
+      </c>
+      <c r="I321" s="3" t="inlineStr">
+        <is>
+          <t>https://ajunews.com/view/20260701075502790</t>
+        </is>
+      </c>
+      <c r="J321" s="3" t="inlineStr"/>
+    </row>
+    <row r="322">
+      <c r="A322" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B322" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C322" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D322" s="3" t="inlineStr">
+        <is>
+          <t>인니·태국·필리핀 화폐 가치 급락…동남아, 환율 방어 안간힘 | 연합뉴스</t>
+        </is>
+      </c>
+      <c r="E322" s="3" t="inlineStr">
+        <is>
+          <t>중동 전쟁으로 인한 국제유가 급등과 미국 달러화 강세 여파로 인도네시아, 태국, 필리핀 등 동남아 국가들의 화폐 가치가 급락하고 있어 환율 방어에 비상이 걸렸다.</t>
+        </is>
+      </c>
+      <c r="F322" s="3" t="inlineStr">
+        <is>
+          <t>동남아시아는 주요 생산 및 소비 시장이 될 수 있으며, 해당 지역 화폐 가치 급락은 부품 조달 비용 및 수출 수익성에 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G322" s="3" t="inlineStr">
+        <is>
+          <t>동남아시아 주요 국가의 환율 변동 추이 모니터링 및 환 헤지 전략 검토.</t>
+        </is>
+      </c>
+      <c r="H322" s="3" t="inlineStr">
+        <is>
+          <t>연합뉴스</t>
+        </is>
+      </c>
+      <c r="I322" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20260630111100104</t>
+        </is>
+      </c>
+      <c r="J322" s="3" t="inlineStr"/>
+    </row>
+    <row r="323">
+      <c r="A323" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B323" s="4" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C323" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D323" s="4" t="inlineStr">
+        <is>
+          <t>7월 LPG 판매가격 '소폭 인상'... kg당 50원</t>
+        </is>
+      </c>
+      <c r="E323" s="4" t="inlineStr">
+        <is>
+          <t>E1이 국제 LPG 가격, 운임, 환율 상승 요인을 반영하여 7월 LPG 판매가격을 kg당 50원 소폭 인상했다.</t>
+        </is>
+      </c>
+      <c r="F323" s="4" t="inlineStr">
+        <is>
+          <t>LPG는 우리 회사의 주요 운송 연료가 아니며, 소폭 인상이라 전체 물류비에 미치는 직접적인 영향은 미미하다.</t>
+        </is>
+      </c>
+      <c r="G323" s="4" t="n"/>
+      <c r="H323" s="4" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I323" s="4" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260701-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J323" s="4" t="inlineStr"/>
+    </row>
+    <row r="324">
+      <c r="A324" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B324" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C324" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D324" s="4" t="inlineStr">
+        <is>
+          <t>씨메스로보틱스 / ‘물류·제조 대형 수주 잇달아’ 피지컬 AI 기반 로봇 자동화 사업 가속</t>
+        </is>
+      </c>
+      <c r="E324" s="4" t="inlineStr">
+        <is>
+          <t>씨메스로보틱스가 물류 및 제조 현장에서 피지컬 AI 기반 로봇 자동화 프로젝트를 연이어 수주하며 사업을 확대하고 있으며, 이는 물류 자동화 기술 발전의 흐름을 보여준다.</t>
+        </is>
+      </c>
+      <c r="F324" s="4" t="inlineStr">
+        <is>
+          <t>특정 기업의 물류 자동화 솔루션 수주 소식으로, 우리 회사의 당면한 물류 운영에 직접적인 영향은 없으나 장기적인 물류 기술 트렌드 파악에 참고할 만하다.</t>
+        </is>
+      </c>
+      <c r="G324" s="4" t="n"/>
+      <c r="H324" s="4" t="inlineStr">
+        <is>
+          <t>ulogistics</t>
+        </is>
+      </c>
+      <c r="I324" s="4" t="inlineStr">
+        <is>
+          <t>http://www.ulogistics.co.kr/test/board.php?board=all2&amp;command=body&amp;no=5202</t>
+        </is>
+      </c>
+      <c r="J324" s="4" t="inlineStr"/>
+    </row>
+    <row r="325">
+      <c r="A325" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B325" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C325" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D325" s="4" t="inlineStr">
+        <is>
+          <t>한·중 해운물류 전문가 상하이 집결…KMI, 미래 공급망 전략 논의</t>
+        </is>
+      </c>
+      <c r="E325" s="4" t="inlineStr">
+        <is>
+          <t>한국해양수산개발원(KMI)이 중국 상하이에서 한·중 해운·물류 전문가들과 글로벌 무역 환경 변화 및 미래 공급망 전략에 대해 논의하는 자리를 마련했다.</t>
+        </is>
+      </c>
+      <c r="F325" s="4" t="inlineStr">
+        <is>
+          <t>한중 물류 전문가들의 논의 소식으로, 당장 우리 회사의 물류 운영에 직접적인 영향은 없으나 장기적인 공급망 전략 수립에 참고할 수 있는 정보이다.</t>
+        </is>
+      </c>
+      <c r="G325" s="4" t="n"/>
+      <c r="H325" s="4" t="inlineStr">
+        <is>
+          <t>해사신문</t>
+        </is>
+      </c>
+      <c r="I325" s="4" t="inlineStr">
+        <is>
+          <t>http://www.haesanews.com/news/articleView.html?idxno=148975</t>
+        </is>
+      </c>
+      <c r="J325" s="4" t="inlineStr"/>
+    </row>
+    <row r="326">
+      <c r="A326" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B326" s="4" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C326" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D326" s="4" t="inlineStr">
+        <is>
+          <t>충주시, 폐배터리 전용 수거함 확대… 화재 예방·자원순환 강화</t>
+        </is>
+      </c>
+      <c r="E326" s="4" t="inlineStr">
+        <is>
+          <t>충주시가 폐배터리 전용 수거함 설치를 대폭 확대하여 충전식 배터리 사용 증가에 따른 화재 위험을 줄이고 자원 재활용을 활성화합니다. 이는 폐배터리 관리 및 재활용 인프라 강화의 일환입니다.</t>
+        </is>
+      </c>
+      <c r="F326" s="4" t="inlineStr">
+        <is>
+          <t>지역 단위의 폐배터리 수거함 확대는 우리 회사의 직접적인 물류 운영이나 생산 계획에 당장 큰 영향을 미치지 않습니다.</t>
+        </is>
+      </c>
+      <c r="G326" s="4" t="inlineStr"/>
+      <c r="H326" s="4" t="inlineStr">
+        <is>
+          <t>충청도민일보</t>
+        </is>
+      </c>
+      <c r="I326" s="4" t="inlineStr">
+        <is>
+          <t>https://dominilbo.com/news/articleView.html?idxno=271772</t>
+        </is>
+      </c>
+      <c r="J326" s="4" t="inlineStr"/>
+    </row>
+    <row r="327">
+      <c r="A327" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B327" s="4" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C327" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D327" s="4" t="inlineStr">
+        <is>
+          <t>연합뉴스TV</t>
+        </is>
+      </c>
+      <c r="E327" s="4" t="inlineStr">
+        <is>
+          <t>경기 부천시의 한 화학공장에서 암모니아 가스가 누출되는 사고가 발생했습니다. 이는 가스 탱크 밸브 조정 과정에서 발생한 것으로 보고되었습니다.</t>
+        </is>
+      </c>
+      <c r="F327" s="4" t="inlineStr">
+        <is>
+          <t>특정 지역의 화학공장 가스 누출 사고는 우리 회사의 배터리/전자부품 물류 운영에 직접적인 영향을 미치지 않습니다.</t>
+        </is>
+      </c>
+      <c r="G327" s="4" t="inlineStr"/>
+      <c r="H327" s="4" t="inlineStr">
+        <is>
+          <t>연합뉴스TV</t>
+        </is>
+      </c>
+      <c r="I327" s="4" t="inlineStr">
+        <is>
+          <t>https://yonhapnewstv.co.kr/news/AKR20260630132047yEt</t>
+        </is>
+      </c>
+      <c r="J327" s="4" t="inlineStr"/>
+    </row>
+    <row r="328">
+      <c r="A328" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B328" s="4" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C328" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D328" s="4" t="inlineStr">
+        <is>
+          <t>[해양통신] 美, SHIPS Act 대폭 축소…韓 조선 김칫국?</t>
+        </is>
+      </c>
+      <c r="E328" s="4" t="inlineStr">
+        <is>
+          <t>미국 의회의 SHIPS Act 수정안이 하원 표결을 앞두고 대폭 축소되어, 미국 국적 전략상선대 조성 및 조선·해운산업 세제 지원 등 핵심 조항들이 대부분 삭제되었습니다. 이는 미국 해운 산업 지원 정책의 변화를 의미합니다.</t>
+        </is>
+      </c>
+      <c r="F328" s="4" t="inlineStr">
+        <is>
+          <t>미국 해운 산업 지원 법안의 축소는 장기적으로 해운 시장에 영향을 줄 수 있으나, 우리 회사의 단기적인 물류 운영에 직접적인 영향은 미미합니다.</t>
+        </is>
+      </c>
+      <c r="G328" s="4" t="inlineStr"/>
+      <c r="H328" s="4" t="inlineStr">
+        <is>
+          <t>해양통신</t>
+        </is>
+      </c>
+      <c r="I328" s="4" t="inlineStr">
+        <is>
+          <t>https://oceanpress.co.kr/news/article.html?no=30478</t>
+        </is>
+      </c>
+      <c r="J328" s="4" t="inlineStr"/>
+    </row>
+    <row r="329">
+      <c r="A329" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B329" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C329" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D329" s="4" t="inlineStr">
+        <is>
+          <t>엘앤에프, 씨아이에스케미칼에 전략적 투자…배터리 재활용 공급망 강화 - 이투데이</t>
+        </is>
+      </c>
+      <c r="E329" s="4" t="inlineStr">
+        <is>
+          <t>엘앤에프가 씨아이에스케미칼에 전략적 투자를 단행하여 LFP 및 NCM 배터리 재활용 협력을 본격화하고, 2027년 LFP 재활용 물량을 우선 확보하여 재생원료 규제 대응 및 원가 절감을 추진합니다.</t>
+        </is>
+      </c>
+      <c r="F329" s="4" t="inlineStr">
+        <is>
+          <t>특정 기업의 배터리 재활용 공급망 강화 투자는 업계 전반의 재활용 동향을 보여주지만, 우리 회사의 직접적인 물류 운영에 당장 영향을 미치지는 않습니다.</t>
+        </is>
+      </c>
+      <c r="G329" s="4" t="inlineStr"/>
+      <c r="H329" s="4" t="inlineStr">
+        <is>
+          <t>이투데이</t>
+        </is>
+      </c>
+      <c r="I329" s="4" t="inlineStr">
+        <is>
+          <t>https://etoday.co.kr/news/view/2598546</t>
+        </is>
+      </c>
+      <c r="J329" s="4" t="inlineStr"/>
+    </row>
+    <row r="330">
+      <c r="A330" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B330" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C330" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D330" s="4" t="inlineStr">
+        <is>
+          <t>제주 스마트공동물류센터 준공…오는 9월 운영 준비 ‘착착’ &lt; 자치행정 &lt; 정치행정 &lt; 기사본문 - 제주도민일보</t>
+        </is>
+      </c>
+      <c r="E330" s="4" t="inlineStr">
+        <is>
+          <t>제주 지역 물류 체계를 혁신할 '제주 스마트공동물류센터'가 준공되어 9월 운영을 목표로 시스템 구축 및 시운전 등 준비에 들어갔습니다. 이는 제주 지역 물류 효율성 향상에 기여할 것으로 보입니다.</t>
+        </is>
+      </c>
+      <c r="F330" s="4" t="inlineStr">
+        <is>
+          <t>제주 지역의 스마트 공동물류센터 준공은 해당 지역의 물류 효율성을 높일 수 있으나, 우리 회사의 전국 또는 글로벌 물류 운영에 직접적인 영향은 미미합니다.</t>
+        </is>
+      </c>
+      <c r="G330" s="4" t="inlineStr"/>
+      <c r="H330" s="4" t="inlineStr">
+        <is>
+          <t>제주도민일보</t>
+        </is>
+      </c>
+      <c r="I330" s="4" t="inlineStr">
+        <is>
+          <t>https://jejudomin.co.kr/news/articleView.html?idxno=320293</t>
+        </is>
+      </c>
+      <c r="J330" s="4" t="inlineStr"/>
+    </row>
+    <row r="331">
+      <c r="A331" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B331" s="4" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C331" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D331" s="4" t="inlineStr">
+        <is>
+          <t>EU, 1일 ‘50% 철강관세 폭탄’ 시행…“쿼터 확보에도 여전히 충격 커” - 이투데이</t>
+        </is>
+      </c>
+      <c r="E331" s="4" t="inlineStr">
+        <is>
+          <t>EU가 7월 1일부터 철강 초과 물량에 대한 관세를 25%에서 50%로 상향 조정하며, 한국산 무관세 물량 축소 우려가 제기되고 있다.</t>
+        </is>
+      </c>
+      <c r="F331" s="4" t="inlineStr">
+        <is>
+          <t>우리 회사는 배터리/전자부품 제조기업으로, 철강 관세는 직접적인 물류 운영에 영향을 미치지 않는다.</t>
+        </is>
+      </c>
+      <c r="G331" s="4" t="n"/>
+      <c r="H331" s="4" t="inlineStr">
+        <is>
+          <t>이투데이</t>
+        </is>
+      </c>
+      <c r="I331" s="4" t="inlineStr">
+        <is>
+          <t>https://etoday.co.kr/news/view/2598706</t>
+        </is>
+      </c>
+      <c r="J331" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -14994,7 +16126,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15313,6 +16445,49 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>3239.64</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>+118 (+3.8%)</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>+1,151 (+55.1%)</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>3920</v>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>+173 (+4.6%)</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>+1,093 (+38.7%)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -15325,7 +16500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:I53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17066,6 +18241,146 @@
       </c>
       <c r="I49" s="6" t="inlineStr"/>
     </row>
+    <row r="50">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t>RSK-049</t>
+        </is>
+      </c>
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="D50" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E50" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈 내 한국 선박 2척 추가 탈출...3척만 남아</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="inlineStr"/>
+      <c r="G50" s="6" t="inlineStr"/>
+      <c r="H50" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 통항 상황을 실시간으로 모니터링하고, 해당 경로를 이용하는 선박의 안전 확보 및 대체 운송 경로(예: 육상 운송, 항공 운송) 또는 재고 확보 방안을 긴급 검토해야 함.</t>
+        </is>
+      </c>
+      <c r="I50" s="6" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>RSK-050</t>
+        </is>
+      </c>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D51" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E51" s="6" t="inlineStr">
+        <is>
+          <t>글로벌 해운운임, 9주 연속 상승…3200대 돌파</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="inlineStr"/>
+      <c r="G51" s="6" t="inlineStr"/>
+      <c r="H51" s="6" t="inlineStr">
+        <is>
+          <t>현재 운송 계약 조건을 재검토하고, 장기 운송 계약 협상, 선사 다변화, 운송 모드 전환(예: 항공 운송 검토) 등 물류비 절감 및 안정화 방안을 즉시 강구해야 함.</t>
+        </is>
+      </c>
+      <c r="I51" s="6" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>RSK-051</t>
+        </is>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D52" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E52" s="6" t="inlineStr">
+        <is>
+          <t>미-이란, 호르무즈 무력 충돌 재개...중동발 에너지·해상운송 리스크 확대</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="inlineStr"/>
+      <c r="G52" s="6" t="inlineStr"/>
+      <c r="H52" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈 해협을 경유하는 모든 운송 계획을 즉시 재검토하고, 대체 운송 경로 및 수단 확보, 비상 재고 확충 등 비상 계획을 수립 및 실행해야 함.</t>
+        </is>
+      </c>
+      <c r="I52" s="6" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="inlineStr">
+        <is>
+          <t>RSK-052</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D53" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E53" s="6" t="inlineStr">
+        <is>
+          <t>[국제유가] 미·이란 군사 충돌 여파에 반등…WTI 70달러선 회복 &lt; 국제 &lt; 세계 &lt; 기사본문 - 굿모닝경제</t>
+        </is>
+      </c>
+      <c r="F53" s="6" t="inlineStr"/>
+      <c r="G53" s="6" t="inlineStr"/>
+      <c r="H53" s="6" t="inlineStr">
+        <is>
+          <t>유가 변동에 따른 운임 인상 가능성 대비, 운송 계약 조건 재검토 및 대체 운송 방안 마련 검토.</t>
+        </is>
+      </c>
+      <c r="I53" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
📰 뉴스 데이터 2026-07-01_19:49
</commit_message>
<xml_diff>
--- a/data/SCM_물류_브리핑.xlsx
+++ b/data/SCM_물류_브리핑.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J331"/>
+  <dimension ref="A1:J364"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16113,6 +16113,1582 @@
         </is>
       </c>
       <c r="J331" s="4" t="inlineStr"/>
+    </row>
+    <row r="332">
+      <c r="A332" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B332" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C332" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D332" s="2" t="inlineStr">
+        <is>
+          <t>DOJ Appeals CIT's IEEPA Refund Injunction as CAPE Phase 2 Targets June 29; TPEB Rates Surge 30% Into Peak</t>
+        </is>
+      </c>
+      <c r="E332" s="2" t="inlineStr">
+        <is>
+          <t>미국 법무부가 IEEPA 환급 금지 명령에 항소하는 가운데, 태평양 동향(TPEB) 해상 운임이 성수기를 앞두고 30% 급등했다.</t>
+        </is>
+      </c>
+      <c r="F332" s="2" t="inlineStr">
+        <is>
+          <t>주요 태평양 동향(TPEB) 해상 운임이 30% 급등하여 우리 회사의 물류 비용에 즉각적인 직접적인 영향을 미치기 때문이다.</t>
+        </is>
+      </c>
+      <c r="G332" s="2" t="inlineStr">
+        <is>
+          <t>태평양 동향 운송 계획 및 예산을 즉시 재검토하고, 운임 상승에 대비한 운송사와의 협상 또는 대체 운송 방안을 모색해야 한다.</t>
+        </is>
+      </c>
+      <c r="H332" s="2" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I332" s="2" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/june-11-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J332" s="2" t="inlineStr">
+        <is>
+          <t>RSK-053</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B333" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C333" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D333" s="2" t="inlineStr">
+        <is>
+          <t>Section 232 Duties Reduced to 15% for Taiwanese Goods, Retroactive to May 1; China Air Rates Spike on Supply Contraction and Month-End Demand</t>
+        </is>
+      </c>
+      <c r="E333" s="2" t="inlineStr">
+        <is>
+          <t>대만산 제품에 대한 Section 232 관세가 15%로 인하되었으며, 중국발 항공 운임은 공급 감소와 월말 수요로 인해 급등했다.</t>
+        </is>
+      </c>
+      <c r="F333" s="2" t="inlineStr">
+        <is>
+          <t>대만산 부품 수입 시 관세 인하는 비용 절감 기회를 제공하며, 중국발 항공 운임 급등은 긴급 운송 비용에 직접적인 영향을 미친다.</t>
+        </is>
+      </c>
+      <c r="G333" s="2" t="inlineStr">
+        <is>
+          <t>대만산 부품 수입 시 관세 인하 혜택을 즉시 활용할 방안을 검토하고, 중국발 항공 운송 계획 및 예산을 재검토하여 비용 상승에 대비해야 한다.</t>
+        </is>
+      </c>
+      <c r="H333" s="2" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I333" s="2" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/may-28-2026-cit-rejects-governments-stay-request/</t>
+        </is>
+      </c>
+      <c r="J333" s="2" t="inlineStr">
+        <is>
+          <t>RSK-054</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B334" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C334" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D334" s="2" t="inlineStr">
+        <is>
+          <t>머스크, 연간 실적 전망 상향 수정...아시아발 호조로 운임 상승</t>
+        </is>
+      </c>
+      <c r="E334" s="2" t="inlineStr">
+        <is>
+          <t>머스크가 아시아발 컨테이너 화물 수요 호조와 스팟 운임 상승을 반영하여 연간 실적 전망을 상향 조정했으며, 전 세계 컨테이너 물동량 증가율 전망도 상향했다.</t>
+        </is>
+      </c>
+      <c r="F334" s="2" t="inlineStr">
+        <is>
+          <t>주요 선사의 운임 상승 및 물동량 증가 전망은 당사의 해상 운송 비용 증가로 직결되며, 이는 물류 예산 및 생산 계획에 즉각적인 영향을 미칩니다.</t>
+        </is>
+      </c>
+      <c r="G334" s="2" t="inlineStr">
+        <is>
+          <t>해상 운임 상승 추이를 면밀히 모니터링하고, 장기 계약 조건 재검토 및 대체 운송 방안(항공, 복합운송 등)을 검토하여 물류 비용 증가에 대비해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H334" s="2" t="inlineStr">
+        <is>
+          <t>shippingnewsnet.com</t>
+        </is>
+      </c>
+      <c r="I334" s="2" t="inlineStr">
+        <is>
+          <t>https://www.shippingnewsnet.com/news/articleView.html?idxno=70989</t>
+        </is>
+      </c>
+      <c r="J334" s="2" t="inlineStr">
+        <is>
+          <t>RSK-055</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B335" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C335" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D335" s="2" t="inlineStr">
+        <is>
+          <t>국제유가, 주말 호르무즈 무력공방에 상승…WTI 2%↑</t>
+        </is>
+      </c>
+      <c r="E335" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 인근 무력 공방 등 지정학적 긴장으로 국제유가가 상승 압력을 받고 있다.</t>
+        </is>
+      </c>
+      <c r="F335" s="2" t="inlineStr">
+        <is>
+          <t>국제유가 상승은 해상 및 항공 운임의 유류할증료 인상으로 이어져 당사의 물류비용에 직접적인 영향을 미치므로 즉시 대응이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G335" s="2" t="inlineStr">
+        <is>
+          <t>유가 변동 추이를 면밀히 모니터링하고, 운송 계약 시 유류할증료 조건 재검토 및 비용 절감 방안을 모색해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H335" s="2" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I335" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260630-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J335" s="2" t="inlineStr">
+        <is>
+          <t>RSK-056</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B336" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C336" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D336" s="2" t="inlineStr">
+        <is>
+          <t>미-이란, 호르무즈 무력 충돌 재개...종전 합의 9일 만</t>
+        </is>
+      </c>
+      <c r="E336" s="2" t="inlineStr">
+        <is>
+          <t>미국과 이란의 호르무즈 해협 무력 충돌이 재개되고 이스라엘의 추가 공격까지 겹치면서 중동발 에너지 및 해상 운송 리스크가 확대되고 있다.</t>
+        </is>
+      </c>
+      <c r="F336" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협의 군사적 긴장 고조는 주요 해상 무역 통로의 봉쇄 또는 운항 지연을 초래하여 당사의 원자재 및 제품 운송에 심각한 차질을 줄 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G336" s="2" t="inlineStr">
+        <is>
+          <t>중동 지역의 지정학적 상황을 실시간으로 모니터링하고, 해당 지역을 경유하는 선박의 안전 확보 및 대체 항로 또는 운송 수단 확보 방안을 즉시 검토해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H336" s="2" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I336" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260628-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J336" s="2" t="inlineStr">
+        <is>
+          <t>RSK-057</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B337" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C337" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D337" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 개방에도 운임은 고공행진…해운사 2분기 ‘순항’</t>
+        </is>
+      </c>
+      <c r="E337" s="2" t="inlineStr">
+        <is>
+          <t>미국과 이란의 종전 양해각서 체결 이후 호르무즈 해협에 묶였던 선박들이 빠져나왔음에도 불구하고 해상 운임 상승세가 계속되고 있다.</t>
+        </is>
+      </c>
+      <c r="F337" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협의 긴장 완화에도 불구하고 해상 운임이 지속적으로 상승하는 것은 당사의 물류 비용 부담이 장기화될 수 있음을 의미하며, 즉각적인 비용 관리 전략이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G337" s="2" t="inlineStr">
+        <is>
+          <t>해상 운임 상승 추이를 면밀히 모니터링하고, 장기 계약 조건 재검토 및 대체 운송 방안(항공, 복합운송 등)을 검토하여 물류 비용 증가에 대비해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H337" s="2" t="inlineStr">
+        <is>
+          <t>헤럴드경제</t>
+        </is>
+      </c>
+      <c r="I337" s="2" t="inlineStr">
+        <is>
+          <t>https://biz.heraldcorp.com/article/10794828</t>
+        </is>
+      </c>
+      <c r="J337" s="2" t="inlineStr">
+        <is>
+          <t>RSK-058</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B338" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C338" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D338" s="2" t="inlineStr">
+        <is>
+          <t>‘호르무즈 통행료’, 세계 경제 새 부담…물류비 쇼크 오나 - 이투데이</t>
+        </is>
+      </c>
+      <c r="E338" s="2" t="inlineStr">
+        <is>
+          <t>이란이 호르무즈 해협에 통행료 부과를 검토하며 세계 원유 및 LNG 운송에 새로운 물류비 부담을 초래하고 아시아 제조업에 직격탄이 우려됩니다.</t>
+        </is>
+      </c>
+      <c r="F338" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협은 주요 해상 운송 경로로, 통행료 부과는 즉각적인 물류비 상승을 유발하여 운송 계획 및 비용 예측에 중대한 영향을 미칩니다.</t>
+        </is>
+      </c>
+      <c r="G338" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 경유 운송 물량 및 비용 영향 분석, 대체 운송 경로 및 운송사 다변화 방안 검토, 재고 수준 조정 검토.</t>
+        </is>
+      </c>
+      <c r="H338" s="2" t="inlineStr">
+        <is>
+          <t>이투데이</t>
+        </is>
+      </c>
+      <c r="I338" s="2" t="inlineStr">
+        <is>
+          <t>https://etoday.co.kr/news/view/2599250</t>
+        </is>
+      </c>
+      <c r="J338" s="2" t="inlineStr">
+        <is>
+          <t>RSK-059</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B339" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C339" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D339" s="2" t="inlineStr">
+        <is>
+          <t>[국제유가] 미·이란 군사 충돌 여파에 반등…WTI 70달러선 회복 &lt; 국제 &lt; 세계 &lt; 기사본문 - 굿모닝경제</t>
+        </is>
+      </c>
+      <c r="E339" s="2" t="inlineStr">
+        <is>
+          <t>미국과 이란의 군사 충돌 여파로 국제유가가 반등하여 WTI가 70달러선을 회복했으며, 중동 정세 불안으로 인한 원유 공급 차질 우려가 지속되고 있다.</t>
+        </is>
+      </c>
+      <c r="F339" s="2" t="inlineStr">
+        <is>
+          <t>국제유가 상승은 해상 및 항공 운임의 유류할증료 인상으로 직결되어 전체 물류비용에 즉각적인 영향을 미치므로, 비용 상승 압박이 예상된다.</t>
+        </is>
+      </c>
+      <c r="G339" s="2" t="inlineStr">
+        <is>
+          <t>유류할증료 변동 추이를 면밀히 주시하고, 운송 계약 시 유류할증료 조건 재검토 및 비용 절감 방안을 모색한다.</t>
+        </is>
+      </c>
+      <c r="H339" s="2" t="inlineStr">
+        <is>
+          <t>굿모닝경제</t>
+        </is>
+      </c>
+      <c r="I339" s="2" t="inlineStr">
+        <is>
+          <t>https://www.goodkyung.com/news/articleView.html?idxno=288676</t>
+        </is>
+      </c>
+      <c r="J339" s="2" t="inlineStr">
+        <is>
+          <t>RSK-060</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B340" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C340" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D340" s="3" t="inlineStr">
+        <is>
+          <t>Air Cargo Demand up 6.0% in May</t>
+        </is>
+      </c>
+      <c r="E340" s="3" t="inlineStr">
+        <is>
+          <t>2026년 5월 전 세계 항공 화물 수요가 전년 대비 6.0% 증가하여 항공 화물 시장의 강세를 나타냈다.</t>
+        </is>
+      </c>
+      <c r="F340" s="3" t="inlineStr">
+        <is>
+          <t>항공 화물 수요 증가는 향후 항공 운임 상승 압력 및 공간 부족으로 이어질 수 있으므로 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G340" s="3" t="inlineStr">
+        <is>
+          <t>항공 운송 시장 동향을 면밀히 주시하고, 성수기 대비 항공 운송 공간 확보 전략을 검토해야 한다.</t>
+        </is>
+      </c>
+      <c r="H340" s="3" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I340" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-29-air-cargo-demand-up-may/</t>
+        </is>
+      </c>
+      <c r="J340" s="3" t="inlineStr"/>
+    </row>
+    <row r="341">
+      <c r="A341" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B341" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C341" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D341" s="3" t="inlineStr">
+        <is>
+          <t>Global Schedule Reliability for May 2026 the Highest of the Year</t>
+        </is>
+      </c>
+      <c r="E341" s="3" t="inlineStr">
+        <is>
+          <t>2026년 5월 전 세계 선박 스케줄 정시성이 올해 최고치를 기록하며 해상 운송의 안정성이 개선되었다.</t>
+        </is>
+      </c>
+      <c r="F341" s="3" t="inlineStr">
+        <is>
+          <t>스케줄 정시성 개선은 운송 지연 리스크 감소에 긍정적이나, 지속적인 추이 모니터링을 통해 안정성 유지 여부를 확인해야 한다.</t>
+        </is>
+      </c>
+      <c r="G341" s="3" t="inlineStr">
+        <is>
+          <t>해상 운송 스케줄 정시성 지표를 지속적으로 모니터링하고, 개선 추세가 유지될 경우 재고 수준 및 운송 계획 최적화 가능성을 검토한다.</t>
+        </is>
+      </c>
+      <c r="H341" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I341" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/395-global-schedule-reliability-for-may-2026-the-highest-of-the-year</t>
+        </is>
+      </c>
+      <c r="J341" s="3" t="inlineStr"/>
+    </row>
+    <row r="342">
+      <c r="A342" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B342" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C342" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D342" s="3" t="inlineStr">
+        <is>
+          <t>Tracking True Vessel Delay</t>
+        </is>
+      </c>
+      <c r="E342" s="3" t="inlineStr">
+        <is>
+          <t>선사들이 운송 시간을 늘리는 스케줄 버퍼링을 통해 정시성을 확보하려는 경향이 증가하고 있으며, 이는 실제 운송 리드타임 증가로 이어질 수 있다.</t>
+        </is>
+      </c>
+      <c r="F342" s="3" t="inlineStr">
+        <is>
+          <t>선사들의 스케줄 버퍼링 증가는 겉보기 정시성 개선에도 불구하고 실제 운송 리드타임 증가로 이어질 수 있어 면밀한 분석이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G342" s="3" t="inlineStr">
+        <is>
+          <t>선사별 실제 운송 리드타임을 면밀히 분석하고, 스케줄 버퍼링으로 인한 잠재적 리드타임 증가를 고려하여 재고 및 생산 계획을 수립해야 한다.</t>
+        </is>
+      </c>
+      <c r="H342" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I342" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/394-tracking-true-vessel-delay</t>
+        </is>
+      </c>
+      <c r="J342" s="3" t="inlineStr"/>
+    </row>
+    <row r="343">
+      <c r="A343" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B343" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C343" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D343" s="3" t="inlineStr">
+        <is>
+          <t>Transpacific: Ripe for new non-alliance services</t>
+        </is>
+      </c>
+      <c r="E343" s="3" t="inlineStr">
+        <is>
+          <t>아시아-북미 서안 항로에서 비동맹 선사들의 새로운 서비스 도입 가능성이 높아지고 있으며, 이는 컨테이너 스팟 운임과 관련이 있다.</t>
+        </is>
+      </c>
+      <c r="F343" s="3" t="inlineStr">
+        <is>
+          <t>새로운 비동맹 서비스 도입은 태평양 항로의 운송 선택지를 넓히고 운임 경쟁을 촉진할 수 있으므로, 시장 변화를 주시해야 한다.</t>
+        </is>
+      </c>
+      <c r="G343" s="3" t="inlineStr">
+        <is>
+          <t>태평양 항로의 신규 서비스 동향을 모니터링하고, 잠재적인 운송 옵션 확대 및 운임 협상 기회를 모색해야 한다.</t>
+        </is>
+      </c>
+      <c r="H343" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I343" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/393-transpacific-ripe-for-new-non-alliance-services</t>
+        </is>
+      </c>
+      <c r="J343" s="3" t="inlineStr"/>
+    </row>
+    <row r="344">
+      <c r="A344" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B344" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C344" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D344" s="3" t="inlineStr">
+        <is>
+          <t>Decoding Gemini’s Mediterranean Surge</t>
+        </is>
+      </c>
+      <c r="E344" s="3" t="inlineStr">
+        <is>
+          <t>주요 해운 동맹인 Gemini Cooperation이 지중해 지역에서 선대 재배치를 진행 중이며, 이는 동서 컨테이너 선박 배치에 변화를 가져오고 있다.</t>
+        </is>
+      </c>
+      <c r="F344" s="3" t="inlineStr">
+        <is>
+          <t>주요 해운 동맹의 선대 재편은 특정 항로의 서비스 수준이나 운항 스케줄에 영향을 미칠 수 있으므로 추이를 지켜봐야 합니다.</t>
+        </is>
+      </c>
+      <c r="G344" s="3" t="inlineStr">
+        <is>
+          <t>해당 동맹의 지중해 항로 서비스 변화를 주시하고, 우리 회사의 해당 지역 운송 스케줄에 미칠 영향을 평가해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H344" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I344" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/392-decoding-gemini-s-mediterranean-surge</t>
+        </is>
+      </c>
+      <c r="J344" s="3" t="inlineStr"/>
+    </row>
+    <row r="345">
+      <c r="A345" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B345" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C345" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D345" s="3" t="inlineStr">
+        <is>
+          <t>7월 LPG 판매가격 '소폭 인상'... kg당 50원</t>
+        </is>
+      </c>
+      <c r="E345" s="3" t="inlineStr">
+        <is>
+          <t>E1이 국제 LPG 가격, 운임, 환율 상승 요인을 반영해 7월 LPG 판매가격을 kg당 50원 수준으로 소폭 인상했다.</t>
+        </is>
+      </c>
+      <c r="F345" s="3" t="inlineStr">
+        <is>
+          <t>LPG 가격 인상은 직접적인 운송 비용(특히 육상 운송)에 영향을 줄 수 있으며, 전반적인 유가 상승 추세와 연관되어 물류비 증가 가능성을 시사합니다.</t>
+        </is>
+      </c>
+      <c r="G345" s="3" t="inlineStr">
+        <is>
+          <t>육상 운송 파트너의 유류할증료 변동을 주시하고, 전반적인 유가 추이를 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H345" s="3" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I345" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260701-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J345" s="3" t="inlineStr"/>
+    </row>
+    <row r="346">
+      <c r="A346" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B346" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C346" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D346" s="3" t="inlineStr">
+        <is>
+          <t>美, USMCA 연장 거부 방침… 북미 자유무역체제 ‘중대 분수령’</t>
+        </is>
+      </c>
+      <c r="E346" s="3" t="inlineStr">
+        <is>
+          <t>미국이 USMCA(미국-멕시코-캐나다 협정) 연장 거부 방침을 밝히면서 북미 자유무역체제에 중대한 변화가 예상된다.</t>
+        </is>
+      </c>
+      <c r="F346" s="3" t="inlineStr">
+        <is>
+          <t>북미 자유무역협정의 변화는 해당 지역으로의 수출입 관세 및 무역 조건에 영향을 미쳐, 장기적으로 북미 시장 공급망 전략 재검토가 필요할 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G346" s="3" t="inlineStr">
+        <is>
+          <t>북미 지역 무역 정책 변화를 주시하고, 관세 및 통관 절차에 대한 잠재적 영향을 평가해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H346" s="3" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I346" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260701-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J346" s="3" t="inlineStr"/>
+    </row>
+    <row r="347">
+      <c r="A347" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B347" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C347" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D347" s="3" t="inlineStr">
+        <is>
+          <t>우회덤핑 차단 공조…관세청·무역위 공동 대응</t>
+        </is>
+      </c>
+      <c r="E347" s="3" t="inlineStr">
+        <is>
+          <t>관세청과 무역위가 협의체를 통해 우회덤핑 감시 정보를 공유하고 무역구제 조치의 실효성 강화를 논의하며 무역 규제 강화 움직임을 보이고 있다.</t>
+        </is>
+      </c>
+      <c r="F347" s="3" t="inlineStr">
+        <is>
+          <t>우회덤핑 감시 강화는 특정 품목의 수출입 통관 절차를 복잡하게 하거나 추가적인 규제 리스크를 발생시킬 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G347" s="3" t="inlineStr">
+        <is>
+          <t>관련 무역 규제 동향을 주시하고, 잠재적 영향을 받을 수 있는 품목이 있는지 확인해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H347" s="3" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I347" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260630-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J347" s="3" t="inlineStr"/>
+    </row>
+    <row r="348">
+      <c r="A348" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B348" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C348" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D348" s="3" t="inlineStr">
+        <is>
+          <t>CPTPP 회원국, 인도네시아·필리핀·UAE와 가입 예비협상 개시</t>
+        </is>
+      </c>
+      <c r="E348" s="3" t="inlineStr">
+        <is>
+          <t>CPTPP(포괄적·점진적 환태평양경제동반자협정)가 인도네시아, 필리핀, UAE와 가입 예비협상을 개시하며 역내 무역 환경 변화 가능성을 시사하고 있다.</t>
+        </is>
+      </c>
+      <c r="F348" s="3" t="inlineStr">
+        <is>
+          <t>CPTPP 확장 논의는 해당 국가들과의 무역 조건 및 관세에 장기적인 영향을 미칠 수 있으므로, 향후 무역 환경 변화에 대비해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G348" s="3" t="inlineStr">
+        <is>
+          <t>CPTPP 협상 진행 상황을 주시하고, 해당 국가들과의 수출입 물량 및 관세 영향을 평가해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H348" s="3" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I348" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260628-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J348" s="3" t="inlineStr"/>
+    </row>
+    <row r="349">
+      <c r="A349" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B349" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C349" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D349" s="3" t="inlineStr">
+        <is>
+          <t>새 지형도…메가 허브 '하락', 지역 항만 '부상'</t>
+        </is>
+      </c>
+      <c r="E349" s="3" t="inlineStr">
+        <is>
+          <t>컨테이너 선사들이 서비스 네트워크를 재구성하면서 싱가포르 등 기존 메가 허브 항만의 연결성이 약화되고 중동, 동남아, 인도 아대륙의 지역 항만들이 부상하고 있다.</t>
+        </is>
+      </c>
+      <c r="F349" s="3" t="inlineStr">
+        <is>
+          <t>주요 항만의 역할 변화는 당사의 특정 지역 수출입 항로 선택 및 리드타임에 영향을 미칠 수 있으므로, 장기적인 관점에서 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G349" s="3" t="inlineStr">
+        <is>
+          <t>주요 항만 및 지역 항만의 서비스 변화를 주시하고, 당사의 주요 수출입 지역에 대한 항만 전략을 재검토해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H349" s="3" t="inlineStr">
+        <is>
+          <t>해양통신</t>
+        </is>
+      </c>
+      <c r="I349" s="3" t="inlineStr">
+        <is>
+          <t>https://oceanpress.co.kr/news/article.html?no=30483</t>
+        </is>
+      </c>
+      <c r="J349" s="3" t="inlineStr"/>
+    </row>
+    <row r="350">
+      <c r="A350" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B350" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C350" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D350" s="3" t="inlineStr">
+        <is>
+          <t>The supply chain is not recovering; it is restructuring</t>
+        </is>
+      </c>
+      <c r="E350" s="3" t="inlineStr">
+        <is>
+          <t>공급망은 회복되는 것이 아니라 재편되고 있으며, 유통업체는 고객을 통제할 수 없는 변동성으로부터 보호하기 위한 구조적 지원을 제공해야 한다고 강조한다.</t>
+        </is>
+      </c>
+      <c r="F350" s="3" t="inlineStr">
+        <is>
+          <t>공급망 재편은 당사의 글로벌 공급망 전략 및 리스크 관리에 대한 근본적인 접근 방식에 영향을 미칠 수 있으므로, 장기적인 관점에서 모니터링하고 대응 전략을 수립해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G350" s="3" t="inlineStr">
+        <is>
+          <t>글로벌 공급망 재편 동향을 지속적으로 분석하고, 당사의 공급망 탄력성 및 회복력 강화를 위한 전략을 검토해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H350" s="3" t="inlineStr">
+        <is>
+          <t>ITWeb</t>
+        </is>
+      </c>
+      <c r="I350" s="3" t="inlineStr">
+        <is>
+          <t>https://www.itweb.co.za/article/the-supply-chain-is-not-recovering-it-is-restructuring/kLgB1Mezp9mq59N4</t>
+        </is>
+      </c>
+      <c r="J350" s="3" t="inlineStr"/>
+    </row>
+    <row r="351">
+      <c r="A351" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B351" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C351" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D351" s="3" t="inlineStr">
+        <is>
+          <t>Hormuz de-escalation does not guarantee "business as usual" for steelmaking supply chain: Iron Ore Decoded 2026 - Fastmarkets</t>
+        </is>
+      </c>
+      <c r="E351" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협의 긴장 완화가 철강 공급망의 정상화를 보장하지 않으며, 지정학적 긴장이 해상 운송 경로에 계속 영향을 미칠 수 있음을 경고합니다.</t>
+        </is>
+      </c>
+      <c r="F351" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협의 지정학적 리스크가 해상 운송 경로에 지속적인 영향을 미칠 수 있어 운송 지연 및 비용 상승 가능성을 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G351" s="3" t="inlineStr">
+        <is>
+          <t>중동 경유 해상 운송 계획 재검토 및 대체 경로, 재고 확보 방안 검토.</t>
+        </is>
+      </c>
+      <c r="H351" s="3" t="inlineStr">
+        <is>
+          <t>Fastmarkets</t>
+        </is>
+      </c>
+      <c r="I351" s="3" t="inlineStr">
+        <is>
+          <t>https://fastmarkets.com/insights/hormuz-de-escalation-does-not-guarantee-business-as-usual-for-steelmaking-supply-chain-iron-ore-decoded-2026</t>
+        </is>
+      </c>
+      <c r="J351" s="3" t="inlineStr"/>
+    </row>
+    <row r="352">
+      <c r="A352" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B352" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C352" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D352" s="3" t="inlineStr">
+        <is>
+          <t>[G.ECONOMY(지이코노미)] 광주·전남 통합 맞춰 위험물 안전관리 기준 통일…1차 위반부터 과태료</t>
+        </is>
+      </c>
+      <c r="E352" s="3" t="inlineStr">
+        <is>
+          <t>광주·전남 통합에 맞춰 위험물 안전관리 기준이 통일되며, 1차 위반부터 과태료가 부과되는 등 안전관리 실효성이 강화됩니다.</t>
+        </is>
+      </c>
+      <c r="F352" s="3" t="inlineStr">
+        <is>
+          <t>위험물 안전관리 기준 통일 및 과태료 부과 강화는 지역 내 위험물 취급 및 운송 절차에 영향을 미칠 수 있어 관련 규정 준수 여부를 확인해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G352" s="3" t="inlineStr">
+        <is>
+          <t>광주/전남 지역 내 위험물 취급 및 운송 관련 규정 변경 사항 확인 및 내부 프로세스 점검.</t>
+        </is>
+      </c>
+      <c r="H352" s="3" t="inlineStr">
+        <is>
+          <t>G.ECONOMY(지이코노미)</t>
+        </is>
+      </c>
+      <c r="I352" s="3" t="inlineStr">
+        <is>
+          <t>https://geconomy.co.kr/news/article.html?no=321332</t>
+        </is>
+      </c>
+      <c r="J352" s="3" t="inlineStr"/>
+    </row>
+    <row r="353">
+      <c r="A353" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B353" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C353" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D353" s="3" t="inlineStr">
+        <is>
+          <t>[한국세정신문] 관세청·무역위원회, 불공정 덤핑행위 차단 공조 강화</t>
+        </is>
+      </c>
+      <c r="E353" s="3" t="inlineStr">
+        <is>
+          <t>관세청과 무역위원회가 불공정 덤핑 수입을 차단하기 위한 공조를 강화하며, 우회 덤핑 가능성이 높은 수입 물품 분석 및 무역구제 조치 실효성 제고에 나선다.</t>
+        </is>
+      </c>
+      <c r="F353" s="3" t="inlineStr">
+        <is>
+          <t>국내 산업 보호를 위한 덤핑 규제 강화는 원자재 수입 또는 완제품 수출 시 관세 및 통관 절차에 영향을 미칠 수 있어 잠재적 비용 상승 및 리스크를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G353" s="3" t="inlineStr">
+        <is>
+          <t>주요 원자재 및 부품 수입 품목에 대한 덤핑 조사 가능성을 주기적으로 확인하고, 관련 규제 변화에 대한 정보를 수집한다.</t>
+        </is>
+      </c>
+      <c r="H353" s="3" t="inlineStr">
+        <is>
+          <t>한국세정신문</t>
+        </is>
+      </c>
+      <c r="I353" s="3" t="inlineStr">
+        <is>
+          <t>https://taxtimes.co.kr/news/article.html?no=275751</t>
+        </is>
+      </c>
+      <c r="J353" s="3" t="inlineStr"/>
+    </row>
+    <row r="354">
+      <c r="A354" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B354" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C354" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D354" s="3" t="inlineStr">
+        <is>
+          <t>인니·태국·필리핀 화폐 가치 급락…동남아, 환율 방어 안간힘 | 연합뉴스</t>
+        </is>
+      </c>
+      <c r="E354" s="3" t="inlineStr">
+        <is>
+          <t>중동 전쟁과 미국 달러 강세의 영향으로 인도네시아, 태국, 필리핀 등 동남아시아 국가들의 화폐 가치가 급락하여 각국이 환율 방어에 나서고 있다.</t>
+        </is>
+      </c>
+      <c r="F354" s="3" t="inlineStr">
+        <is>
+          <t>동남아시아 지역의 환율 변동은 해당 지역에서 원자재를 조달하거나 완제품을 수출할 경우 물류비용 및 구매/판매 가격에 직접적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G354" s="3" t="inlineStr">
+        <is>
+          <t>동남아시아 주요 거래 국가의 환율 추이를 면밀히 모니터링하고, 환율 변동에 따른 구매 및 판매 전략 조정을 검토한다.</t>
+        </is>
+      </c>
+      <c r="H354" s="3" t="inlineStr">
+        <is>
+          <t>연합뉴스</t>
+        </is>
+      </c>
+      <c r="I354" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20260630111100104</t>
+        </is>
+      </c>
+      <c r="J354" s="3" t="inlineStr"/>
+    </row>
+    <row r="355">
+      <c r="A355" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B355" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C355" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D355" s="4" t="inlineStr">
+        <is>
+          <t>日 금융그룹 노무라, 해운업 본격 진출</t>
+        </is>
+      </c>
+      <c r="E355" s="4" t="inlineStr">
+        <is>
+          <t>일본 금융 대기업 노무라가 독일 해운투자플랫폼에 지분 투자를 단행하며 글로벌 해운금융시장에 본격 진출했다.</t>
+        </is>
+      </c>
+      <c r="F355" s="4" t="inlineStr">
+        <is>
+          <t>금융 그룹의 해운업 진출은 장기적으로 해운 시장 구조에 영향을 미칠 수 있으나, 당사의 물류 운영에 즉각적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G355" s="4" t="n"/>
+      <c r="H355" s="4" t="inlineStr">
+        <is>
+          <t>kita</t>
+        </is>
+      </c>
+      <c r="I355" s="4" t="inlineStr">
+        <is>
+          <t>https://www.kita.net/shippers/board/newsView.do?morgueCode=2&amp;dataCls=B&amp;dataSeq=8145</t>
+        </is>
+      </c>
+      <c r="J355" s="4" t="inlineStr"/>
+    </row>
+    <row r="356">
+      <c r="A356" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B356" s="4" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C356" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D356" s="4" t="inlineStr">
+        <is>
+          <t>벌크선 시장, 中 철광석 수요 감소에 케이프선 부진</t>
+        </is>
+      </c>
+      <c r="E356" s="4" t="inlineStr">
+        <is>
+          <t>6월 마지막 주 벌크선 시장은 중국 철광석 수요 감소로 케이프선 운임이 부진했으며, 해상운임 선물거래 시장도 약세를 유지했다.</t>
+        </is>
+      </c>
+      <c r="F356" s="4" t="inlineStr">
+        <is>
+          <t>벌크선 시장의 동향은 컨테이너 운송에 직접적인 영향을 미치지 않으며, 당사의 배터리/전자부품 운송과는 관련성이 낮다.</t>
+        </is>
+      </c>
+      <c r="G356" s="4" t="n"/>
+      <c r="H356" s="4" t="inlineStr">
+        <is>
+          <t>ksg</t>
+        </is>
+      </c>
+      <c r="I356" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksg.co.kr/news/main_newsView.jsp?pNum=147528</t>
+        </is>
+      </c>
+      <c r="J356" s="4" t="inlineStr"/>
+    </row>
+    <row r="357">
+      <c r="A357" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B357" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C357" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D357" s="4" t="inlineStr">
+        <is>
+          <t>中 산동성항구그룹 대표단, 인천항 방문</t>
+        </is>
+      </c>
+      <c r="E357" s="4" t="inlineStr">
+        <is>
+          <t>중국 산동성항구그룹 대표단이 인천항을 방문하여 양 항만 간 협력 강화를 논의했다.</t>
+        </is>
+      </c>
+      <c r="F357" s="4" t="inlineStr">
+        <is>
+          <t>양 항만 간 협력 강화는 장기적으로 물류 효율성 증대에 기여할 수 있으나, 당장의 물류 운영에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G357" s="4" t="n"/>
+      <c r="H357" s="4" t="inlineStr">
+        <is>
+          <t>oceanpress</t>
+        </is>
+      </c>
+      <c r="I357" s="4" t="inlineStr">
+        <is>
+          <t>https://www.oceanpress.co.kr/news/article.html?no=30496</t>
+        </is>
+      </c>
+      <c r="J357" s="4" t="inlineStr"/>
+    </row>
+    <row r="358">
+      <c r="A358" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B358" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C358" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D358" s="4" t="inlineStr">
+        <is>
+          <t>2026-Q1: NAEC Ports Consolidate Market Share</t>
+        </is>
+      </c>
+      <c r="E358" s="4" t="inlineStr">
+        <is>
+          <t>2026년 1분기 북미 동부 해안(NAEC) 항만의 컨테이너 물동량이 전년 대비 감소했음에도 불구하고, NAEC 항만들이 시장 점유율을 공고히 하고 있다.</t>
+        </is>
+      </c>
+      <c r="F358" s="4" t="inlineStr">
+        <is>
+          <t>북미 동부 해안 항만의 전반적인 물동량 감소는 당사 물류 운영에 직접적인 영향을 미치기보다는 전반적인 시장 동향을 파악하는 참고 자료입니다.</t>
+        </is>
+      </c>
+      <c r="G358" s="4" t="n"/>
+      <c r="H358" s="4" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I358" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/391-2026-q1-naec-ports-consolidate-market-share</t>
+        </is>
+      </c>
+      <c r="J358" s="4" t="inlineStr"/>
+    </row>
+    <row r="359">
+      <c r="A359" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B359" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C359" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D359" s="4" t="inlineStr">
+        <is>
+          <t>씨메스로보틱스 / ‘물류·제조 대형 수주 잇달아’ 피지컬 AI 기반 로봇 자동화 사업 가속</t>
+        </is>
+      </c>
+      <c r="E359" s="4" t="inlineStr">
+        <is>
+          <t>씨메스로보틱스가 쿠팡풀필먼트서비스 등 물류 및 제조 현장에서 피지컬 AI 기반 로봇 자동화 프로젝트를 연이어 수주하며 사업을 확대하고 있다.</t>
+        </is>
+      </c>
+      <c r="F359" s="4" t="inlineStr">
+        <is>
+          <t>물류 자동화 기술 발전은 장기적으로 물류 효율성 향상에 기여할 수 있으나, 당사의 현재 물류 운영에 직접적인 영향을 미치지는 않습니다.</t>
+        </is>
+      </c>
+      <c r="G359" s="4" t="n"/>
+      <c r="H359" s="4" t="inlineStr">
+        <is>
+          <t>ulogistics.co.kr</t>
+        </is>
+      </c>
+      <c r="I359" s="4" t="inlineStr">
+        <is>
+          <t>http://www.ulogistics.co.kr/test/board.php?board=all2&amp;command=body&amp;no=5202</t>
+        </is>
+      </c>
+      <c r="J359" s="4" t="inlineStr"/>
+    </row>
+    <row r="360">
+      <c r="A360" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B360" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C360" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D360" s="4" t="inlineStr">
+        <is>
+          <t>美 ’선박법’ 대폭 완화…글로벌 규제 리스크 해소</t>
+        </is>
+      </c>
+      <c r="E360" s="4" t="inlineStr">
+        <is>
+          <t>미국이 선박법 개정안을 통해 해운·조선업계 지원 취지와 달리 규제와 혜택을 모두 줄이면서 글로벌 해운 시장의 단기적 혼란을 피하게 되었다.</t>
+        </is>
+      </c>
+      <c r="F360" s="4" t="inlineStr">
+        <is>
+          <t>미국 선박법 완화는 글로벌 해운 시장의 단기적 혼란을 줄이는 데 기여할 수 있으나, 당사의 물류 운영에 직접적인 영향을 미치지는 않습니다.</t>
+        </is>
+      </c>
+      <c r="G360" s="4" t="n"/>
+      <c r="H360" s="4" t="inlineStr">
+        <is>
+          <t>EBN</t>
+        </is>
+      </c>
+      <c r="I360" s="4" t="inlineStr">
+        <is>
+          <t>https://kr.investing.com/news/stock-market-news/article-1999956</t>
+        </is>
+      </c>
+      <c r="J360" s="4" t="inlineStr"/>
+    </row>
+    <row r="361">
+      <c r="A361" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B361" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C361" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D361" s="4" t="inlineStr">
+        <is>
+          <t>HMM, 1조7000억원 승부수…'컨테이너 편중' 벗어나 벌크·에너지 운송 키운다</t>
+        </is>
+      </c>
+      <c r="E361" s="4" t="inlineStr">
+        <is>
+          <t>HMM이 1조 6천억 원 규모의 신조선 투자를 통해 컨테이너 편중에서 벗어나 벌크 및 에너지 운송 분야를 확대하며 종합 해운사로의 체질 개선을 가속화하고 있다.</t>
+        </is>
+      </c>
+      <c r="F361" s="4" t="inlineStr">
+        <is>
+          <t>HMM의 사업 다각화는 장기적인 해운 시장 구조에 영향을 줄 수 있으나, 당사의 컨테이너 기반 물류 운영에 즉각적인 영향은 없습니다.</t>
+        </is>
+      </c>
+      <c r="G361" s="4" t="n"/>
+      <c r="H361" s="4" t="inlineStr">
+        <is>
+          <t>해사신문</t>
+        </is>
+      </c>
+      <c r="I361" s="4" t="inlineStr">
+        <is>
+          <t>https://haesanews.com/news/articleView.html?idxno=148979</t>
+        </is>
+      </c>
+      <c r="J361" s="4" t="inlineStr"/>
+    </row>
+    <row r="362">
+      <c r="A362" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B362" s="4" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C362" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D362" s="4" t="inlineStr">
+        <is>
+          <t>다음달부터 서울지하철 대용량 리튬배터리 장착 교통수단 휴대 불가 :: 공감언론 뉴시스 ::</t>
+        </is>
+      </c>
+      <c r="E362" s="4" t="inlineStr">
+        <is>
+          <t>서울교통공사가 7월 1일부터 지하철 내 화재 위험을 줄이기 위해 대용량 리튬배터리 및 장착 이동수단의 휴대를 금지합니다.</t>
+        </is>
+      </c>
+      <c r="F362" s="4" t="inlineStr">
+        <is>
+          <t>지하철 내 개인 휴대 규제로, 우리 회사의 대규모 물류 운송에는 직접적인 영향이 없지만, 배터리 안전 규제 강화의 일환으로 참고할 만합니다.</t>
+        </is>
+      </c>
+      <c r="G362" s="4" t="n"/>
+      <c r="H362" s="4" t="inlineStr">
+        <is>
+          <t>뉴시스</t>
+        </is>
+      </c>
+      <c r="I362" s="4" t="inlineStr">
+        <is>
+          <t>https://newsis.com/view/NISI20260630_0021343554</t>
+        </is>
+      </c>
+      <c r="J362" s="4" t="inlineStr"/>
+    </row>
+    <row r="363">
+      <c r="A363" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B363" s="4" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C363" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D363" s="4" t="inlineStr">
+        <is>
+          <t>충주시, 폐배터리 전용 수거함 확대… 화재 예방·자원순환 강화 &lt; 충주 &lt; 충북 &lt; 지역 &lt; 기사본문 - 충청도민일보</t>
+        </is>
+      </c>
+      <c r="E363" s="4" t="inlineStr">
+        <is>
+          <t>충주시가 충전식 배터리 사용 증가에 따른 화재 위험을 줄이고 자원 재활용을 활성화하기 위해 폐배터리 전용 수거함 설치를 확대합니다.</t>
+        </is>
+      </c>
+      <c r="F363" s="4" t="inlineStr">
+        <is>
+          <t>폐배터리 수거 인프라 확충은 장기적인 자원 순환 및 환경 규제 대응에 긍정적이나, 현재 물류 운영에 즉각적인 영향은 없습니다.</t>
+        </is>
+      </c>
+      <c r="G363" s="4" t="n"/>
+      <c r="H363" s="4" t="inlineStr">
+        <is>
+          <t>충청도민일보</t>
+        </is>
+      </c>
+      <c r="I363" s="4" t="inlineStr">
+        <is>
+          <t>https://dominilbo.com/news/articleView.html?idxno=271772</t>
+        </is>
+      </c>
+      <c r="J363" s="4" t="inlineStr"/>
+    </row>
+    <row r="364">
+      <c r="A364" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B364" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C364" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D364" s="4" t="inlineStr">
+        <is>
+          <t>제주 스마트공동물류센터 준공…오는 9월 운영 준비 ‘착착’ &lt; 자치행정 &lt; 정치행정 &lt; 기사본문 - 제주도민일보</t>
+        </is>
+      </c>
+      <c r="E364" s="4" t="inlineStr">
+        <is>
+          <t>제주 지역 물류 체계를 혁신할 '제주 스마트공동물류센터'가 준공되어 오는 9월 본격적인 운영을 준비하며 시스템 구축 및 시운전이 진행 중입니다.</t>
+        </is>
+      </c>
+      <c r="F364" s="4" t="inlineStr">
+        <is>
+          <t>제주 지역에 특화된 물류센터 준공으로, 전국 단위 또는 해외 물류 운영에 즉각적인 영향은 없으며, 향후 제주 지역 비즈니스 확장 시 참고할 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G364" s="4" t="n"/>
+      <c r="H364" s="4" t="inlineStr">
+        <is>
+          <t>제주도민일보</t>
+        </is>
+      </c>
+      <c r="I364" s="4" t="inlineStr">
+        <is>
+          <t>https://jejudomin.co.kr/news/articleView.html?idxno=320293</t>
+        </is>
+      </c>
+      <c r="J364" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
@@ -16500,7 +18076,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I53"/>
+  <dimension ref="A1:I61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18381,6 +19957,286 @@
       </c>
       <c r="I53" s="6" t="inlineStr"/>
     </row>
+    <row r="54">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t>RSK-053</t>
+        </is>
+      </c>
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D54" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E54" s="6" t="inlineStr">
+        <is>
+          <t>DOJ Appeals CIT's IEEPA Refund Injunction as CAPE Phase 2 Targets June 29; TPEB Rates Surge 30% Into Peak</t>
+        </is>
+      </c>
+      <c r="F54" s="6" t="inlineStr"/>
+      <c r="G54" s="6" t="inlineStr"/>
+      <c r="H54" s="6" t="inlineStr">
+        <is>
+          <t>태평양 동향 운송 계획 및 예산을 즉시 재검토하고, 운임 상승에 대비한 운송사와의 협상 또는 대체 운송 방안을 모색해야 한다.</t>
+        </is>
+      </c>
+      <c r="I54" s="6" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t>RSK-054</t>
+        </is>
+      </c>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D55" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E55" s="6" t="inlineStr">
+        <is>
+          <t>Section 232 Duties Reduced to 15% for Taiwanese Goods, Retroactive to May 1; China Air Rates Spike on Supply Contraction and Month-End Demand</t>
+        </is>
+      </c>
+      <c r="F55" s="6" t="inlineStr"/>
+      <c r="G55" s="6" t="inlineStr"/>
+      <c r="H55" s="6" t="inlineStr">
+        <is>
+          <t>대만산 부품 수입 시 관세 인하 혜택을 즉시 활용할 방안을 검토하고, 중국발 항공 운송 계획 및 예산을 재검토하여 비용 상승에 대비해야 한다.</t>
+        </is>
+      </c>
+      <c r="I55" s="6" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t>RSK-055</t>
+        </is>
+      </c>
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D56" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E56" s="6" t="inlineStr">
+        <is>
+          <t>머스크, 연간 실적 전망 상향 수정...아시아발 호조로 운임 상승</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="inlineStr"/>
+      <c r="G56" s="6" t="inlineStr"/>
+      <c r="H56" s="6" t="inlineStr">
+        <is>
+          <t>해상 운임 상승 추이를 면밀히 모니터링하고, 장기 계약 조건 재검토 및 대체 운송 방안(항공, 복합운송 등)을 검토하여 물류 비용 증가에 대비해야 합니다.</t>
+        </is>
+      </c>
+      <c r="I56" s="6" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="inlineStr">
+        <is>
+          <t>RSK-056</t>
+        </is>
+      </c>
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D57" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E57" s="6" t="inlineStr">
+        <is>
+          <t>국제유가, 주말 호르무즈 무력공방에 상승…WTI 2%↑</t>
+        </is>
+      </c>
+      <c r="F57" s="6" t="inlineStr"/>
+      <c r="G57" s="6" t="inlineStr"/>
+      <c r="H57" s="6" t="inlineStr">
+        <is>
+          <t>유가 변동 추이를 면밀히 모니터링하고, 운송 계약 시 유류할증료 조건 재검토 및 비용 절감 방안을 모색해야 합니다.</t>
+        </is>
+      </c>
+      <c r="I57" s="6" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>RSK-057</t>
+        </is>
+      </c>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D58" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E58" s="6" t="inlineStr">
+        <is>
+          <t>미-이란, 호르무즈 무력 충돌 재개...종전 합의 9일 만</t>
+        </is>
+      </c>
+      <c r="F58" s="6" t="inlineStr"/>
+      <c r="G58" s="6" t="inlineStr"/>
+      <c r="H58" s="6" t="inlineStr">
+        <is>
+          <t>중동 지역의 지정학적 상황을 실시간으로 모니터링하고, 해당 지역을 경유하는 선박의 안전 확보 및 대체 항로 또는 운송 수단 확보 방안을 즉시 검토해야 합니다.</t>
+        </is>
+      </c>
+      <c r="I58" s="6" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t>RSK-058</t>
+        </is>
+      </c>
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D59" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E59" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 개방에도 운임은 고공행진…해운사 2분기 ‘순항’</t>
+        </is>
+      </c>
+      <c r="F59" s="6" t="inlineStr"/>
+      <c r="G59" s="6" t="inlineStr"/>
+      <c r="H59" s="6" t="inlineStr">
+        <is>
+          <t>해상 운임 상승 추이를 면밀히 모니터링하고, 장기 계약 조건 재검토 및 대체 운송 방안(항공, 복합운송 등)을 검토하여 물류 비용 증가에 대비해야 합니다.</t>
+        </is>
+      </c>
+      <c r="I59" s="6" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t>RSK-059</t>
+        </is>
+      </c>
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C60" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D60" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E60" s="6" t="inlineStr">
+        <is>
+          <t>‘호르무즈 통행료’, 세계 경제 새 부담…물류비 쇼크 오나 - 이투데이</t>
+        </is>
+      </c>
+      <c r="F60" s="6" t="inlineStr"/>
+      <c r="G60" s="6" t="inlineStr"/>
+      <c r="H60" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 경유 운송 물량 및 비용 영향 분석, 대체 운송 경로 및 운송사 다변화 방안 검토, 재고 수준 조정 검토.</t>
+        </is>
+      </c>
+      <c r="I60" s="6" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="inlineStr">
+        <is>
+          <t>RSK-060</t>
+        </is>
+      </c>
+      <c r="B61" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C61" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D61" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E61" s="6" t="inlineStr">
+        <is>
+          <t>[국제유가] 미·이란 군사 충돌 여파에 반등…WTI 70달러선 회복 &lt; 국제 &lt; 세계 &lt; 기사본문 - 굿모닝경제</t>
+        </is>
+      </c>
+      <c r="F61" s="6" t="inlineStr"/>
+      <c r="G61" s="6" t="inlineStr"/>
+      <c r="H61" s="6" t="inlineStr">
+        <is>
+          <t>유류할증료 변동 추이를 면밀히 주시하고, 운송 계약 시 유류할증료 조건 재검토 및 비용 절감 방안을 모색한다.</t>
+        </is>
+      </c>
+      <c r="I61" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
📰 뉴스 데이터 2026-07-02_09:13
</commit_message>
<xml_diff>
--- a/data/SCM_물류_브리핑.xlsx
+++ b/data/SCM_물류_브리핑.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J364"/>
+  <dimension ref="A1:J393"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17690,6 +17690,1390 @@
       </c>
       <c r="J364" s="4" t="inlineStr"/>
     </row>
+    <row r="365">
+      <c r="A365" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B365" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C365" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D365" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 군사 충돌 계속... 이스라엘은 레바논 또 공격</t>
+        </is>
+      </c>
+      <c r="E365" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 인근 군사 충돌과 이스라엘의 레바논 공격이 지속되며 중동발 에너지 및 해상운송 리스크가 심화되고 있다.</t>
+        </is>
+      </c>
+      <c r="F365" s="2" t="inlineStr">
+        <is>
+          <t>중동 지역의 전반적인 불안정 심화는 유가 상승 및 주요 해상 운송로의 차질로 이어져 당사의 물류 비용과 리드타임에 광범위하고 직접적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G365" s="2" t="inlineStr">
+        <is>
+          <t>중동 지역 정세 변화를 면밀히 주시하고, 비상 계획(B.C.P)을 재검토하며, 대체 공급망 및 운송 옵션 확보에 집중해야 한다.</t>
+        </is>
+      </c>
+      <c r="H365" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I365" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260628-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J365" s="2" t="inlineStr">
+        <is>
+          <t>RSK-061</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B366" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C366" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D366" s="2" t="inlineStr">
+        <is>
+          <t>글로벌 해운운임, 9주 연속 상승…3200대 돌파</t>
+        </is>
+      </c>
+      <c r="E366" s="2" t="inlineStr">
+        <is>
+          <t>상하이컨테이너운임지수(SCFI)가 9주 연속 상승하여 3200선을 돌파하며 해상물류 비용 부담이 가중되고 있다.</t>
+        </is>
+      </c>
+      <c r="F366" s="2" t="inlineStr">
+        <is>
+          <t>글로벌 해운운임의 지속적인 상승은 당사의 해상 물류비용에 직접적인 영향을 미치므로, 즉각적인 비용 관리 및 운송 계획 재검토가 필요하다.</t>
+        </is>
+      </c>
+      <c r="G366" s="2" t="inlineStr">
+        <is>
+          <t>주요 항로별 운임 계약 조건 재검토, 장기 계약 또는 스팟 시장 활용 전략 수립, 운송사와의 협상 강화를 통해 비용 절감 방안을 모색해야 한다.</t>
+        </is>
+      </c>
+      <c r="H366" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I366" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260629-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J366" s="2" t="inlineStr">
+        <is>
+          <t>RSK-062</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B367" s="2" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C367" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D367" s="2" t="inlineStr">
+        <is>
+          <t>중동전쟁 장기화에 중소기업 피해 '962건'</t>
+        </is>
+      </c>
+      <c r="E367" s="2" t="inlineStr">
+        <is>
+          <t>중동전쟁 장기화로 해상운임 증가와 우회 운송이 발생하여 중소기업의 물류 피해가 누적되고 있다.</t>
+        </is>
+      </c>
+      <c r="F367" s="2" t="inlineStr">
+        <is>
+          <t>중동전쟁으로 인한 해상운임 상승 및 우회 운송은 당사의 물류 비용 및 리드타임에 직접적인 영향을 미치고 있음을 시사한다.</t>
+        </is>
+      </c>
+      <c r="G367" s="2" t="inlineStr">
+        <is>
+          <t>중동 항로 이용 시 운임 및 리드타임 변화를 면밀히 분석하고, 대체 운송 경로 및 운송사 확보 방안을 검토해야 한다.</t>
+        </is>
+      </c>
+      <c r="H367" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I367" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260629-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J367" s="2" t="inlineStr">
+        <is>
+          <t>RSK-063</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B368" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C368" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D368" s="2" t="inlineStr">
+        <is>
+          <t>‘호르무즈 통행료’, 세계 경제 새 부담…물류비 쇼크 오나</t>
+        </is>
+      </c>
+      <c r="E368" s="2" t="inlineStr">
+        <is>
+          <t>이란이 호르무즈 해협 통행료 부과를 검토하며 세계 원유 및 LNG 물동량의 20%가 통과하는 이 해협의 물류비 상승과 아시아 제조업에 대한 직격탄이 우려된다.</t>
+        </is>
+      </c>
+      <c r="F368" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협은 주요 에너지 및 원자재 운송 경로로, 통행료 부과는 해상 운임 및 유가 상승을 유발하여 우리 물류비에 직접적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G368" s="2" t="inlineStr">
+        <is>
+          <t>중동발 원자재 및 부품 수급 경로의 운임 변동성 분석 및 대체 운송 경로/재고 확보 방안 검토.</t>
+        </is>
+      </c>
+      <c r="H368" s="2" t="inlineStr">
+        <is>
+          <t>이투데이</t>
+        </is>
+      </c>
+      <c r="I368" s="2" t="inlineStr">
+        <is>
+          <t>https://etoday.co.kr/news/view/2599250</t>
+        </is>
+      </c>
+      <c r="J368" s="2" t="inlineStr">
+        <is>
+          <t>RSK-064</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B369" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C369" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D369" s="3" t="inlineStr">
+        <is>
+          <t>Air Cargo Demand Up 6.0% in May</t>
+        </is>
+      </c>
+      <c r="E369" s="3" t="inlineStr">
+        <is>
+          <t>2026년 5월 전 세계 항공 화물 수요가 전년 대비 6.0% 증가했으며, 이는 항공 화물 시장의 지속적인 성장을 나타낸다.</t>
+        </is>
+      </c>
+      <c r="F369" s="3" t="inlineStr">
+        <is>
+          <t>항공 화물 수요 증가는 향후 항공 운임 상승 압력으로 작용할 수 있어 물류비에 잠재적 영향을 미친다.</t>
+        </is>
+      </c>
+      <c r="G369" s="3" t="inlineStr">
+        <is>
+          <t>항공 운임 추이 지속 모니터링 및 필요시 대체 운송 방안 검토.</t>
+        </is>
+      </c>
+      <c r="H369" s="3" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I369" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-29-air-cargo-demand-up-may/</t>
+        </is>
+      </c>
+      <c r="J369" s="3" t="inlineStr"/>
+    </row>
+    <row r="370">
+      <c r="A370" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B370" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C370" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D370" s="3" t="inlineStr">
+        <is>
+          <t>Tracking True Vessel Delay</t>
+        </is>
+      </c>
+      <c r="E370" s="3" t="inlineStr">
+        <is>
+          <t>선사들이 운송 시간을 늘려 스케줄 버퍼링을 통해 실제 지연을 관리하고 있으며, 이는 조기 도착과 관련이 있다.</t>
+        </is>
+      </c>
+      <c r="F370" s="3" t="inlineStr">
+        <is>
+          <t>선사들의 스케줄 버퍼링 전략은 공시된 운송 시간과 실제 도착 시간 간의 차이를 유발할 수 있어 리드타임 관리에 영향을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="G370" s="3" t="inlineStr">
+        <is>
+          <t>주요 항로의 실제 운송 리드타임과 선사 스케줄 버퍼링 동향을 지속적으로 분석하여 운송 계획에 반영.</t>
+        </is>
+      </c>
+      <c r="H370" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I370" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/394-tracking-true-vessel-delay</t>
+        </is>
+      </c>
+      <c r="J370" s="3" t="inlineStr"/>
+    </row>
+    <row r="371">
+      <c r="A371" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B371" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C371" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D371" s="3" t="inlineStr">
+        <is>
+          <t>Transpacific: Ripe for new non-alliance services</t>
+        </is>
+      </c>
+      <c r="E371" s="3" t="inlineStr">
+        <is>
+          <t>태평양 횡단 항로에서 비동맹 선사들의 신규 서비스 도입 가능성이 높아지고 있으며, 이는 운임과 시장 점유율에 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="F371" s="3" t="inlineStr">
+        <is>
+          <t>비동맹 선사의 신규 서비스는 태평양 횡단 항로의 운임 경쟁을 심화시키고 운송 옵션을 다양화할 가능성이 있다.</t>
+        </is>
+      </c>
+      <c r="G371" s="3" t="inlineStr">
+        <is>
+          <t>태평양 횡단 항로의 신규 서비스 동향 및 운임 변동 추이 모니터링.</t>
+        </is>
+      </c>
+      <c r="H371" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I371" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/393-transpacific-ripe-for-new-non-alliance-services</t>
+        </is>
+      </c>
+      <c r="J371" s="3" t="inlineStr"/>
+    </row>
+    <row r="372">
+      <c r="A372" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B372" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C372" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D372" s="3" t="inlineStr">
+        <is>
+          <t>2026-Q1: NAEC Ports Consolidate Market Share</t>
+        </is>
+      </c>
+      <c r="E372" s="3" t="inlineStr">
+        <is>
+          <t>2026년 1분기 북미 동부 해안(NAEC) 항만의 컨테이너 처리량이 전년 대비 감소했음에도 불구하고 시장 점유율을 공고히 했다.</t>
+        </is>
+      </c>
+      <c r="F372" s="3" t="inlineStr">
+        <is>
+          <t>북미 동부 해안 항만은 주요 수출입 거점 중 하나이므로 물동량 변화는 운송 계획 및 잠재적 병목 현상에 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G372" s="3" t="inlineStr">
+        <is>
+          <t>북미 동부 해안 항만의 물동량 및 혼잡도 추이를 지속적으로 모니터링하고, 필요시 대체 항만 또는 운송 경로를 검토.</t>
+        </is>
+      </c>
+      <c r="H372" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I372" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/391-2026-q1-naec-ports-consolidate-market-share</t>
+        </is>
+      </c>
+      <c r="J372" s="3" t="inlineStr"/>
+    </row>
+    <row r="373">
+      <c r="A373" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B373" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C373" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D373" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 내 한국 선박 2척 추가 탈출...3척만 남아</t>
+        </is>
+      </c>
+      <c r="E373" s="3" t="inlineStr">
+        <is>
+          <t>종전 합의 이후 호르무즈 해협에 갇혔던 한국 선박 2척이 추가 탈출했으나, 아직 3척이 남아 물류 불확실성이 지속된다.</t>
+        </is>
+      </c>
+      <c r="F373" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협의 지정학적 리스크가 완전히 해소되지 않아 중동 항로의 불확실성이 여전히 존재하며, 선박 운항에 영향을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="G373" s="3" t="inlineStr">
+        <is>
+          <t>중동 항로 이용 시 선박 스케줄 및 운항 상황을 지속적으로 모니터링하고, 필요 시 운송 계획을 조정해야 한다.</t>
+        </is>
+      </c>
+      <c r="H373" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I373" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260629-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J373" s="3" t="inlineStr"/>
+    </row>
+    <row r="374">
+      <c r="A374" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B374" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C374" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D374" s="3" t="inlineStr">
+        <is>
+          <t>국제유가, 주말 호르무즈 무력공방에 상승…WTI 2%↑</t>
+        </is>
+      </c>
+      <c r="E374" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 인근 무력 공방 등 지정학적 긴장으로 국제유가(WTI)가 2% 상승 압력을 받았다.</t>
+        </is>
+      </c>
+      <c r="F374" s="3" t="inlineStr">
+        <is>
+          <t>국제유가 상승은 해상 및 항공 운임 상승으로 이어져 물류비용에 영향을 미치므로 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G374" s="3" t="inlineStr">
+        <is>
+          <t>유가 및 운임 변동 추이를 지속 모니터링하고, 물류비 예산에 반영하는 것을 검토해야 한다.</t>
+        </is>
+      </c>
+      <c r="H374" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I374" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260630-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J374" s="3" t="inlineStr"/>
+    </row>
+    <row r="375">
+      <c r="A375" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B375" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C375" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D375" s="3" t="inlineStr">
+        <is>
+          <t>7월 LPG 판매가격 '소폭 인상'... kg당 50원</t>
+        </is>
+      </c>
+      <c r="E375" s="3" t="inlineStr">
+        <is>
+          <t>국제 LPG 가격, 운임, 환율 상승 요인을 반영하여 7월 LPG 판매가격이 kg당 50원 수준으로 소폭 인상되었다.</t>
+        </is>
+      </c>
+      <c r="F375" s="3" t="inlineStr">
+        <is>
+          <t>유가 및 운임 상승 추세의 일부로, 물류비 전반에 영향을 미칠 수 있어 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G375" s="3" t="inlineStr">
+        <is>
+          <t>유가 및 운임 변동 추이를 지속 모니터링하고, 물류비 예산에 반영하는 것을 검토해야 한다.</t>
+        </is>
+      </c>
+      <c r="H375" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I375" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260701-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J375" s="3" t="inlineStr"/>
+    </row>
+    <row r="376">
+      <c r="A376" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B376" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C376" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D376" s="3" t="inlineStr">
+        <is>
+          <t>인천항 1만6000TEU급 시대 열었다</t>
+        </is>
+      </c>
+      <c r="E376" s="3" t="inlineStr">
+        <is>
+          <t>인천항 미주 정기항로에 1만6000TEU급 초대형 컨테이너선이 처음 투입되며 인천항의 대형선 시대가 본격화되었다.</t>
+        </is>
+      </c>
+      <c r="F376" s="3" t="inlineStr">
+        <is>
+          <t>인천항의 처리 능력 및 미주 노선 효율성 개선 가능성을 시사하며, 향후 물류 계획 수립 시 고려할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G376" s="3" t="inlineStr">
+        <is>
+          <t>인천항 이용 시 대형선 투입에 따른 운송 효율성 변화 추이를 모니터링하고, 필요 시 운송 경로 최적화에 반영을 검토해야 한다.</t>
+        </is>
+      </c>
+      <c r="H376" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I376" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260702-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J376" s="3" t="inlineStr"/>
+    </row>
+    <row r="377">
+      <c r="A377" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B377" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C377" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D377" s="3" t="inlineStr">
+        <is>
+          <t>美, USMCA 연장 거부 방침… 북미 자유무역체제 ‘중대 분수령’</t>
+        </is>
+      </c>
+      <c r="E377" s="3" t="inlineStr">
+        <is>
+          <t>미국이 USMCA 연장 거부 방침을 밝히며 북미 자유무역체제에 중대한 변화가 예상된다.</t>
+        </is>
+      </c>
+      <c r="F377" s="3" t="inlineStr">
+        <is>
+          <t>북미 지역 무역 정책 변화는 해당 지역으로의 수출입 관세 및 절차에 영향을 미칠 수 있어 추이를 지켜봐야 한다.</t>
+        </is>
+      </c>
+      <c r="G377" s="3" t="inlineStr">
+        <is>
+          <t>북미 지역 무역 정책 변화 동향을 지속적으로 모니터링하고, 필요 시 통상팀과 협의하여 대응 방안을 마련해야 한다.</t>
+        </is>
+      </c>
+      <c r="H377" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I377" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260701-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J377" s="3" t="inlineStr"/>
+    </row>
+    <row r="378">
+      <c r="A378" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B378" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C378" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D378" s="3" t="inlineStr">
+        <is>
+          <t>Maersk Europe Market Update | July 2026 | Maersk</t>
+        </is>
+      </c>
+      <c r="E378" s="3" t="inlineStr">
+        <is>
+          <t>Maersk가 2026년 7월 유럽 시장에 대한 해상, 주요 항만, 항공 운송, 내륙 운송 및 통관 관련 최신 업데이트를 발표했다.</t>
+        </is>
+      </c>
+      <c r="F378" s="3" t="inlineStr">
+        <is>
+          <t>주요 운송사의 시장 업데이트는 유럽 지역의 물류 상황 변화를 파악하는 데 중요하며, 향후 운송 계획에 참고할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G378" s="3" t="inlineStr">
+        <is>
+          <t>Maersk 보고서 상세 검토를 통해 유럽 지역 물류 상황 변화를 파악하고, 필요 시 대응 방안을 모색해야 한다.</t>
+        </is>
+      </c>
+      <c r="H378" s="3" t="inlineStr">
+        <is>
+          <t>Maersk</t>
+        </is>
+      </c>
+      <c r="I378" s="3" t="inlineStr">
+        <is>
+          <t>https://maersk.com/news/articles/2026/07/01/europe-market-update-july</t>
+        </is>
+      </c>
+      <c r="J378" s="3" t="inlineStr"/>
+    </row>
+    <row r="379">
+      <c r="A379" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B379" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C379" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D379" s="3" t="inlineStr">
+        <is>
+          <t>The supply chain is not recovering; it is restructuring</t>
+        </is>
+      </c>
+      <c r="E379" s="3" t="inlineStr">
+        <is>
+          <t>공급망이 회복되는 것이 아니라 재편되고 있으며, 유통업체는 고객을 변동성으로부터 보호하기 위한 구조적 지원이 필요하다.</t>
+        </is>
+      </c>
+      <c r="F379" s="3" t="inlineStr">
+        <is>
+          <t>글로벌 공급망의 구조적 변화는 장기적으로 당사의 공급망 전략 및 물류 운영 방식에 영향을 미칠 수 있으므로 추이를 지켜봐야 한다.</t>
+        </is>
+      </c>
+      <c r="G379" s="3" t="inlineStr">
+        <is>
+          <t>글로벌 공급망 재편 동향을 지속적으로 모니터링하고, 공급망 탄력성 강화를 위한 전략적 검토를 시작해야 한다.</t>
+        </is>
+      </c>
+      <c r="H379" s="3" t="inlineStr">
+        <is>
+          <t>ITWeb</t>
+        </is>
+      </c>
+      <c r="I379" s="3" t="inlineStr">
+        <is>
+          <t>https://itweb.co.za/article/the-supply-chain-is-not-recovering-it-is-restructuring/kLgB1Mezp9mq59N4</t>
+        </is>
+      </c>
+      <c r="J379" s="3" t="inlineStr"/>
+    </row>
+    <row r="380">
+      <c r="A380" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B380" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C380" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D380" s="3" t="inlineStr">
+        <is>
+          <t>장마는 이제 계절의 변화를 알리는 비가 아니라 재난의 신호가 됐다. 기후변화로 세계 곳곳에서 기록적인 폭우와 대형 홍수가 반복되면서 수많은 인명 피해와 막대한 경제적 손실이 이어지고 있다.</t>
+        </is>
+      </c>
+      <c r="E380" s="3" t="inlineStr">
+        <is>
+          <t>기후변화로 인한 기록적인 폭우와 대형 홍수가 전 세계적으로 반복되며 인명 및 경제적 손실이 커지고 있어, 이는 물류 운영에도 잠재적인 위험 요인이 될 수 있다.</t>
+        </is>
+      </c>
+      <c r="F380" s="3" t="inlineStr">
+        <is>
+          <t>기후변화로 인한 극단적인 기상 현상은 운송 지연, 창고 피해 등 물류 운영에 간접적인 영향을 미칠 수 있으므로 추이를 주시해야 한다.</t>
+        </is>
+      </c>
+      <c r="G380" s="3" t="inlineStr">
+        <is>
+          <t>기상 이변에 따른 운송 경로 및 창고 운영 리스크 점검, 비상 계획 수립 필요성 검토.</t>
+        </is>
+      </c>
+      <c r="H380" s="3" t="inlineStr">
+        <is>
+          <t>허프포스트코리아</t>
+        </is>
+      </c>
+      <c r="I380" s="3" t="inlineStr">
+        <is>
+          <t>https://huffingtonpost.kr/article/258378</t>
+        </is>
+      </c>
+      <c r="J380" s="3" t="inlineStr"/>
+    </row>
+    <row r="381">
+      <c r="A381" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B381" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C381" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D381" s="3" t="inlineStr">
+        <is>
+          <t>美, USMCA 연장 거부…'매년 재검토'로 10년 시한부 유지</t>
+        </is>
+      </c>
+      <c r="E381" s="3" t="inlineStr">
+        <is>
+          <t>미국 트럼프 행정부가 USMCA의 장기 연장을 거부하고 매년 재검토 및 재협상을 거치는 '상시 협상' 체제로 전환되어 10년간 효력을 유지하게 되었다.</t>
+        </is>
+      </c>
+      <c r="F381" s="3" t="inlineStr">
+        <is>
+          <t>USMCA의 상시 협상 체제 전환은 북미 지역의 무역 정책 불확실성을 높여 향후 관세 변동이나 무역 장벽 발생 가능성을 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G381" s="3" t="inlineStr">
+        <is>
+          <t>북미 지역 공급망 및 고객사와의 거래에 대한 잠재적 영향 분석 및 대응 전략 수립 준비.</t>
+        </is>
+      </c>
+      <c r="H381" s="3" t="inlineStr">
+        <is>
+          <t>이데일리</t>
+        </is>
+      </c>
+      <c r="I381" s="3" t="inlineStr">
+        <is>
+          <t>https://edaily.co.kr/News/Read?mediaCodeNo=257&amp;newsId=02414086645510584</t>
+        </is>
+      </c>
+      <c r="J381" s="3" t="inlineStr"/>
+    </row>
+    <row r="382">
+      <c r="A382" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B382" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C382" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D382" s="3" t="inlineStr">
+        <is>
+          <t>중국 車업계, 배터리 이어 차량용 반도체 자급자족 박차</t>
+        </is>
+      </c>
+      <c r="E382" s="3" t="inlineStr">
+        <is>
+          <t>중국 자동차 업계가 전기차 배터리에 이어 차량용 반도체 자급자족에 박차를 가하고 있으며, 이는 글로벌 경쟁 우위 확보를 목표로 한다.</t>
+        </is>
+      </c>
+      <c r="F382" s="3" t="inlineStr">
+        <is>
+          <t>중국의 배터리 및 차량용 반도체 자급률 증가는 글로벌 공급망 재편 및 경쟁 심화로 이어질 수 있어 장기적인 시장 동향과 공급망 전략에 영향을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="G382" s="3" t="inlineStr">
+        <is>
+          <t>중국 시장 동향 및 경쟁사 전략 분석, 핵심 부품의 공급망 다변화 및 기술 경쟁력 강화 방안 검토.</t>
+        </is>
+      </c>
+      <c r="H382" s="3" t="inlineStr">
+        <is>
+          <t>뉴스핌</t>
+        </is>
+      </c>
+      <c r="I382" s="3" t="inlineStr">
+        <is>
+          <t>https://newspim.com/news/view/20260701000921</t>
+        </is>
+      </c>
+      <c r="J382" s="3" t="inlineStr"/>
+    </row>
+    <row r="383">
+      <c r="A383" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B383" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C383" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D383" s="3" t="inlineStr">
+        <is>
+          <t>요소수 등 300개 품목 '3중 체계' 관리 - 매일경제</t>
+        </is>
+      </c>
+      <c r="E383" s="3" t="inlineStr">
+        <is>
+          <t>정부가 요소수 등 300개 핵심 품목에 대해 국내 생산, 비축, 해외 기지 확보의 '3중 체계'로 공급망을 관리하는 대책을 다음 달 발표할 예정이다.</t>
+        </is>
+      </c>
+      <c r="F383" s="3" t="inlineStr">
+        <is>
+          <t>정부의 핵심 품목 공급망 안정화 대책은 우리 회사의 원자재 조달 및 생산 계획에 간접적인 영향을 미칠 수 있으며, 향후 정책 발표 내용을 주시해야 한다.</t>
+        </is>
+      </c>
+      <c r="G383" s="3" t="inlineStr">
+        <is>
+          <t>정부의 공급망 안정화 대책 발표 내용 확인 및 우리 회사 제품/원자재와의 연관성 분석.</t>
+        </is>
+      </c>
+      <c r="H383" s="3" t="inlineStr">
+        <is>
+          <t>매일경제</t>
+        </is>
+      </c>
+      <c r="I383" s="3" t="inlineStr">
+        <is>
+          <t>https://mk.co.kr/news/economy/12088014</t>
+        </is>
+      </c>
+      <c r="J383" s="3" t="inlineStr"/>
+    </row>
+    <row r="384">
+      <c r="A384" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B384" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C384" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D384" s="3" t="inlineStr">
+        <is>
+          <t>6월 물가 3.2% ‘2년 6개월 만에 최고’…기름값이 끌어올렸다 - 헤럴드경제</t>
+        </is>
+      </c>
+      <c r="E384" s="3" t="inlineStr">
+        <is>
+          <t>6월 소비자물가가 3.2% 상승하며 2년 6개월 만에 최고치를 기록했는데, 이는 국제유가 상승으로 인한 석유류 가격 인상이 주원인이며, 정부는 하반기 물가 안정을 위해 석유 최고가격제 등 대책을 추진할 예정이다.</t>
+        </is>
+      </c>
+      <c r="F384" s="3" t="inlineStr">
+        <is>
+          <t>국제유가 상승은 해상/항공 운임 및 육상 운송비용에 직접적인 영향을 미쳐 물류비 증가로 이어질 수 있으므로 유가 및 정부 정책 변화를 지속적으로 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G384" s="3" t="inlineStr">
+        <is>
+          <t>유가 변동에 따른 물류비용 변화 추이 분석, 운송 계약 시 유가 연동 조항 검토, 에너지 효율 개선 방안 모색.</t>
+        </is>
+      </c>
+      <c r="H384" s="3" t="inlineStr">
+        <is>
+          <t>헤럴드경제</t>
+        </is>
+      </c>
+      <c r="I384" s="3" t="inlineStr">
+        <is>
+          <t>https://biz.heraldcorp.com/article/10795291</t>
+        </is>
+      </c>
+      <c r="J384" s="3" t="inlineStr"/>
+    </row>
+    <row r="385">
+      <c r="A385" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B385" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C385" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D385" s="4" t="inlineStr">
+        <is>
+          <t>북극항로 시험운항 선박 '확보'…"8월 말 출항 유력"</t>
+        </is>
+      </c>
+      <c r="E385" s="4" t="inlineStr">
+        <is>
+          <t>해양수산부와 해운업계가 북극항로 시험 운항을 위한 내빙 컨테이너선 확보에 성공했으며, 8월 말 출항이 유력하다.</t>
+        </is>
+      </c>
+      <c r="F385" s="4" t="inlineStr">
+        <is>
+          <t>북극항로 시험 운항은 장기적인 운송 효율성 개선 가능성을 제시하지만, 당사의 현재 물류 운영에 즉각적인 변화를 요구하지 않는다.</t>
+        </is>
+      </c>
+      <c r="G385" s="4" t="inlineStr">
+        <is>
+          <t>해당 없음</t>
+        </is>
+      </c>
+      <c r="H385" s="4" t="inlineStr">
+        <is>
+          <t>oceanpress</t>
+        </is>
+      </c>
+      <c r="I385" s="4" t="inlineStr">
+        <is>
+          <t>https://www.oceanpress.co.kr/news/article.html?no=30469</t>
+        </is>
+      </c>
+      <c r="J385" s="4" t="inlineStr"/>
+    </row>
+    <row r="386">
+      <c r="A386" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B386" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C386" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D386" s="4" t="inlineStr">
+        <is>
+          <t>Global Schedule Reliability for May 2026 the Highest of the Year</t>
+        </is>
+      </c>
+      <c r="E386" s="4" t="inlineStr">
+        <is>
+          <t>2026년 5월 글로벌 선박 스케줄 정시성이 올해 최고치를 기록하며 해상 운송의 안정성이 개선되었다.</t>
+        </is>
+      </c>
+      <c r="F386" s="4" t="inlineStr">
+        <is>
+          <t>해상 운송의 정시성 개선은 긍정적인 신호이지만, 현재 물류 계획에 즉각적인 조정이 필요한 수준은 아니다.</t>
+        </is>
+      </c>
+      <c r="G386" s="4" t="inlineStr">
+        <is>
+          <t>해당 없음</t>
+        </is>
+      </c>
+      <c r="H386" s="4" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I386" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/395-global-schedule-reliability-for-may-2026-the-highest-of-the-year</t>
+        </is>
+      </c>
+      <c r="J386" s="4" t="inlineStr"/>
+    </row>
+    <row r="387">
+      <c r="A387" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B387" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C387" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D387" s="4" t="inlineStr">
+        <is>
+          <t>Decoding Gemini’s Mediterranean Surge</t>
+        </is>
+      </c>
+      <c r="E387" s="4" t="inlineStr">
+        <is>
+          <t>Gemini 협력이 지중해 지역에서 선대 재배치를 진행 중이며, 이는 해당 지역의 시장 점유율 및 서비스에 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="F387" s="4" t="inlineStr">
+        <is>
+          <t>지중해 지역은 당사의 주요 운송 경로가 아니며, 특정 얼라이언스의 선대 재배치가 즉각적인 물류 운영에 미치는 영향은 미미하다.</t>
+        </is>
+      </c>
+      <c r="G387" s="4" t="inlineStr">
+        <is>
+          <t>해당 없음</t>
+        </is>
+      </c>
+      <c r="H387" s="4" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I387" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/392-decoding-gemini-s-mediterranean-surge</t>
+        </is>
+      </c>
+      <c r="J387" s="4" t="inlineStr"/>
+    </row>
+    <row r="388">
+      <c r="A388" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B388" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C388" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D388" s="4" t="inlineStr">
+        <is>
+          <t>[현장] '미국서 인증된 자율주행' 마스오토, 물류 혁신 승부수</t>
+        </is>
+      </c>
+      <c r="E388" s="4" t="inlineStr">
+        <is>
+          <t>마스오토가 미국에서 인증받은 자율주행 기술로 부산항을 거점으로 물류 혁신을 추진하겠다는 구상을 밝혔다.</t>
+        </is>
+      </c>
+      <c r="F388" s="4" t="inlineStr">
+        <is>
+          <t>장기적인 물류 효율성 개선 가능성을 시사하지만, 당사 물류 운영에 즉각적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G388" s="4" t="n"/>
+      <c r="H388" s="4" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I388" s="4" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260702-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J388" s="4" t="inlineStr"/>
+    </row>
+    <row r="389">
+      <c r="A389" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B389" s="4" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C389" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D389" s="4" t="inlineStr">
+        <is>
+          <t>우회덤핑 차단 공조…관세청·무역위 공동 대응</t>
+        </is>
+      </c>
+      <c r="E389" s="4" t="inlineStr">
+        <is>
+          <t>관세청과 무역위원회가 우회덤핑 차단을 위해 공조하며 무역구제 조치의 실효성 강화를 논의했다.</t>
+        </is>
+      </c>
+      <c r="F389" s="4" t="inlineStr">
+        <is>
+          <t>불법적인 무역 행위에 대한 감시 강화로, 정상적인 물류 운영에는 직접적인 영향이 없다.</t>
+        </is>
+      </c>
+      <c r="G389" s="4" t="n"/>
+      <c r="H389" s="4" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I389" s="4" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260630-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J389" s="4" t="inlineStr"/>
+    </row>
+    <row r="390">
+      <c r="A390" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B390" s="4" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C390" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D390" s="4" t="inlineStr">
+        <is>
+          <t>CPTPP 회원국, 인도네시아·필리핀·UAE와 가입 예비협상 개시</t>
+        </is>
+      </c>
+      <c r="E390" s="4" t="inlineStr">
+        <is>
+          <t>CPTPP 회원국들이 인도네시아, 필리핀, UAE와 가입 예비협상을 개시했다.</t>
+        </is>
+      </c>
+      <c r="F390" s="4" t="inlineStr">
+        <is>
+          <t>무역 협정 확대는 장기적으로 관세 등에 영향을 줄 수 있으나, 당장 물류 운영에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G390" s="4" t="n"/>
+      <c r="H390" s="4" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I390" s="4" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260628-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J390" s="4" t="inlineStr"/>
+    </row>
+    <row r="391">
+      <c r="A391" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B391" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C391" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D391" s="4" t="inlineStr">
+        <is>
+          <t>씨메스로보틱스 / ‘물류·제조 대형 수주 잇달아’ 피지컬 AI 기반 로봇 자동화 사업 가속 (기기)</t>
+        </is>
+      </c>
+      <c r="E391" s="4" t="inlineStr">
+        <is>
+          <t>씨메스로보틱스가 물류 및 제조 현장에서 피지컬 AI 기반 로봇 자동화 사업을 확대하며 대형 수주를 잇달아 확보했다.</t>
+        </is>
+      </c>
+      <c r="F391" s="4" t="inlineStr">
+        <is>
+          <t>물류 자동화 기술 발전 소식으로, 당사 물류 운영에 즉각적인 영향은 없으나 장기적인 관점에서 참고할 만하다.</t>
+        </is>
+      </c>
+      <c r="G391" s="4" t="n"/>
+      <c r="H391" s="4" t="inlineStr">
+        <is>
+          <t>ulogistics</t>
+        </is>
+      </c>
+      <c r="I391" s="4" t="inlineStr">
+        <is>
+          <t>http://www.ulogistics.co.kr/test/board.php?board=all2&amp;command=body&amp;no=5202</t>
+        </is>
+      </c>
+      <c r="J391" s="4" t="inlineStr"/>
+    </row>
+    <row r="392">
+      <c r="A392" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B392" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C392" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D392" s="4" t="inlineStr">
+        <is>
+          <t>SK해운, 알짜 '가스선' 구조조정 통했다</t>
+        </is>
+      </c>
+      <c r="E392" s="4" t="inlineStr">
+        <is>
+          <t>SK해운이 수익성이 높은 가스운반선 중심으로 선대를 재편하며 이익 창출력을 강화하고 있어, 이는 장기적으로 특정 선종의 운송 서비스 가용성 및 운임에 영향을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="F392" s="4" t="inlineStr">
+        <is>
+          <t>특정 해운사의 선대 재편은 장기적인 시장 변화의 일부이나, 당장 우리 물류 운영에 직접적인 영향을 미치지는 않는다.</t>
+        </is>
+      </c>
+      <c r="G392" s="4" t="n"/>
+      <c r="H392" s="4" t="inlineStr">
+        <is>
+          <t>파이낸셜뉴스</t>
+        </is>
+      </c>
+      <c r="I392" s="4" t="inlineStr">
+        <is>
+          <t>https://fnnews.com/news/202607010804409585</t>
+        </is>
+      </c>
+      <c r="J392" s="4" t="inlineStr"/>
+    </row>
+    <row r="393">
+      <c r="A393" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B393" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C393" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D393" s="4" t="inlineStr">
+        <is>
+          <t>6월 수출 1000억弗 돌파…獨·中·美 이어 네 번째 천억불 클럽(종합)</t>
+        </is>
+      </c>
+      <c r="E393" s="4" t="inlineStr">
+        <is>
+          <t>지난 6월 우리나라 수출액이 반도체 슈퍼사이클에 힘입어 사상 처음으로 1000억 달러를 돌파하며 세계 4번째로 '월 수출 1000억 달러 클럽'에 가입했다.</t>
+        </is>
+      </c>
+      <c r="F393" s="4" t="inlineStr">
+        <is>
+          <t>수출 호조는 긍정적인 경제 지표이나, 당장 우리 기업의 물류 운영에 직접적인 영향을 미치기보다는 전반적인 시장 활성화에 기여한다.</t>
+        </is>
+      </c>
+      <c r="G393" s="4" t="n"/>
+      <c r="H393" s="4" t="inlineStr">
+        <is>
+          <t>파이낸셜뉴스</t>
+        </is>
+      </c>
+      <c r="I393" s="4" t="inlineStr">
+        <is>
+          <t>https://fnnews.com/news/202607011054242419</t>
+        </is>
+      </c>
+      <c r="J393" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -17702,7 +19086,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18064,6 +19448,49 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>3239.64</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>+118 (+3.8%)</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>+1,151 (+55.1%)</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>3920</v>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>+173 (+4.6%)</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>+1,093 (+38.7%)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -18076,7 +19503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I61"/>
+  <dimension ref="A1:I65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -20237,6 +21664,146 @@
       </c>
       <c r="I61" s="6" t="inlineStr"/>
     </row>
+    <row r="62">
+      <c r="A62" s="6" t="inlineStr">
+        <is>
+          <t>RSK-061</t>
+        </is>
+      </c>
+      <c r="B62" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C62" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D62" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E62" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈 군사 충돌 계속... 이스라엘은 레바논 또 공격</t>
+        </is>
+      </c>
+      <c r="F62" s="6" t="inlineStr"/>
+      <c r="G62" s="6" t="inlineStr"/>
+      <c r="H62" s="6" t="inlineStr">
+        <is>
+          <t>중동 지역 정세 변화를 면밀히 주시하고, 비상 계획(B.C.P)을 재검토하며, 대체 공급망 및 운송 옵션 확보에 집중해야 한다.</t>
+        </is>
+      </c>
+      <c r="I62" s="6" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="inlineStr">
+        <is>
+          <t>RSK-062</t>
+        </is>
+      </c>
+      <c r="B63" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C63" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D63" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E63" s="6" t="inlineStr">
+        <is>
+          <t>글로벌 해운운임, 9주 연속 상승…3200대 돌파</t>
+        </is>
+      </c>
+      <c r="F63" s="6" t="inlineStr"/>
+      <c r="G63" s="6" t="inlineStr"/>
+      <c r="H63" s="6" t="inlineStr">
+        <is>
+          <t>주요 항로별 운임 계약 조건 재검토, 장기 계약 또는 스팟 시장 활용 전략 수립, 운송사와의 협상 강화를 통해 비용 절감 방안을 모색해야 한다.</t>
+        </is>
+      </c>
+      <c r="I63" s="6" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="6" t="inlineStr">
+        <is>
+          <t>RSK-063</t>
+        </is>
+      </c>
+      <c r="B64" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C64" s="6" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="D64" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E64" s="6" t="inlineStr">
+        <is>
+          <t>중동전쟁 장기화에 중소기업 피해 '962건'</t>
+        </is>
+      </c>
+      <c r="F64" s="6" t="inlineStr"/>
+      <c r="G64" s="6" t="inlineStr"/>
+      <c r="H64" s="6" t="inlineStr">
+        <is>
+          <t>중동 항로 이용 시 운임 및 리드타임 변화를 면밀히 분석하고, 대체 운송 경로 및 운송사 확보 방안을 검토해야 한다.</t>
+        </is>
+      </c>
+      <c r="I64" s="6" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="6" t="inlineStr">
+        <is>
+          <t>RSK-064</t>
+        </is>
+      </c>
+      <c r="B65" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C65" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D65" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E65" s="6" t="inlineStr">
+        <is>
+          <t>‘호르무즈 통행료’, 세계 경제 새 부담…물류비 쇼크 오나</t>
+        </is>
+      </c>
+      <c r="F65" s="6" t="inlineStr"/>
+      <c r="G65" s="6" t="inlineStr"/>
+      <c r="H65" s="6" t="inlineStr">
+        <is>
+          <t>중동발 원자재 및 부품 수급 경로의 운임 변동성 분석 및 대체 운송 경로/재고 확보 방안 검토.</t>
+        </is>
+      </c>
+      <c r="I65" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
📰 뉴스 데이터 2026-07-02_19:08
</commit_message>
<xml_diff>
--- a/data/SCM_물류_브리핑.xlsx
+++ b/data/SCM_물류_브리핑.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J393"/>
+  <dimension ref="A1:J425"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19073,6 +19073,1518 @@
         </is>
       </c>
       <c r="J393" s="4" t="inlineStr"/>
+    </row>
+    <row r="394">
+      <c r="A394" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B394" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C394" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D394" s="2" t="inlineStr">
+        <is>
+          <t>U.S. Appeals CIT's IEEPA Refund Order to Federal Circuit; TPEB Rates Rise as Peak Season Demand Tightens Capacity</t>
+        </is>
+      </c>
+      <c r="E394" s="2" t="inlineStr">
+        <is>
+          <t>성수기 수요로 인한 선복량 부족으로 태평양 횡단 동향(TPEB) 운임이 6주 연속 10% 상승하고 있으며, 미국은 CIT의 IEEPA 환불 명령에 항소했다.</t>
+        </is>
+      </c>
+      <c r="F394" s="2" t="inlineStr">
+        <is>
+          <t>성수기 수요로 인한 선복량 부족과 TPEB 운임의 6주 연속 10% 상승은 물류 비용 및 운송 계획에 즉각적이고 직접적인 영향을 미치므로 즉시 대응이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G394" s="2" t="inlineStr">
+        <is>
+          <t>TPEB 노선 운임 변동성 주시 및 운송 계약 조건 재검토, 대체 운송 방안 또는 선사 협상 준비, 성수기 물량 예측 및 선복 확보 계획 수립.</t>
+        </is>
+      </c>
+      <c r="H394" s="2" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I394" s="2" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/june-3-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J394" s="2" t="inlineStr">
+        <is>
+          <t>RSK-065</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B395" s="2" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C395" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D395" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈에서 컨선 '좌초'…이란, "항로 이탈이 원인"</t>
+        </is>
+      </c>
+      <c r="E395" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 인근에서 컨테이너선이 항로 이탈로 좌초되어 운항 지연 및 변수가 발생했다.</t>
+        </is>
+      </c>
+      <c r="F395" s="2" t="inlineStr">
+        <is>
+          <t>주요 해상 운송 경로인 호르무즈 해협에서의 컨테이너선 좌초는 해당 지역을 통과하는 선박의 운항 지연을 유발하여 우리 물류 운영에 직접적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G395" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 통과 예정 선박의 운항 스케줄 확인 및 지연 가능성 평가, 대체 항로 또는 운송 수단 검토.</t>
+        </is>
+      </c>
+      <c r="H395" s="2" t="inlineStr">
+        <is>
+          <t>kita</t>
+        </is>
+      </c>
+      <c r="I395" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kita.net/shippers/board/newsView.do?morgueCode=2&amp;dataCls=B&amp;dataSeq=8147</t>
+        </is>
+      </c>
+      <c r="J395" s="2" t="inlineStr">
+        <is>
+          <t>RSK-066</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B396" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C396" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D396" s="2" t="inlineStr">
+        <is>
+          <t>글로벌 해운운임, 9주 연속 상승…3200대 돌파</t>
+        </is>
+      </c>
+      <c r="E396" s="2" t="inlineStr">
+        <is>
+          <t>글로벌 해운운임 지수인 상하이컨테이너운임지수(SCFI)가 9주 연속 상승하여 3200선을 돌파하며 해상물류 비용 부담이 커지고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F396" s="2" t="inlineStr">
+        <is>
+          <t>SCFI의 지속적인 상승은 해상 운송 비용의 직접적인 증가로 이어져 우리 회사의 물류 예산 및 제품 원가에 즉각적인 영향을 미칩니다.</t>
+        </is>
+      </c>
+      <c r="G396" s="2" t="inlineStr">
+        <is>
+          <t>긴급 물량에 대한 항공 운송 전환 검토, 선사와의 운임 협상 재검토, 장기 계약 조건 확인, 운임 상승에 따른 물류비 예산 재조정.</t>
+        </is>
+      </c>
+      <c r="H396" s="2" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I396" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260629-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J396" s="2" t="inlineStr">
+        <is>
+          <t>RSK-067</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B397" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C397" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D397" s="2" t="inlineStr">
+        <is>
+          <t>미-이란, 호르무즈 무력 충돌 재개...종전 합의 9일 만</t>
+        </is>
+      </c>
+      <c r="E397" s="2" t="inlineStr">
+        <is>
+          <t>미-이란 간 호르무즈 해협 무력 충돌이 재개되면서 해당 해협을 둘러싼 해상 물류 불확실성이 다시 커지고 중동발 에너지 및 해상운송 리스크가 확대되고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F397" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협은 주요 원유 및 가스 운송로이며, 충돌 재개는 유가 상승 및 중동발 해상 운송 지연/차질을 유발하여 우리 물류 운영에 직접적인 위험을 초래할 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G397" s="2" t="inlineStr">
+        <is>
+          <t>중동 경유 노선 선박 스케줄 및 운항 정보 실시간 모니터링, 대체 항로 및 운송 수단(항공) 검토, 비상 재고 확보 여부 점검.</t>
+        </is>
+      </c>
+      <c r="H397" s="2" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I397" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260628-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J397" s="2" t="inlineStr">
+        <is>
+          <t>RSK-068</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B398" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C398" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D398" s="2" t="inlineStr">
+        <is>
+          <t>6월 소비자물가 3.2%↑…석유류 급등에 30개월 만에 최대폭 상승 [종합]</t>
+        </is>
+      </c>
+      <c r="E398" s="2" t="inlineStr">
+        <is>
+          <t>6월 소비자물가가 중동 사태 영향으로 석유류 가격이 급등하며 3.2% 상승, 30개월 만에 최대 폭을 기록했으며, 이는 물가 상승을 주도했습니다.</t>
+        </is>
+      </c>
+      <c r="F398" s="2" t="inlineStr">
+        <is>
+          <t>석유류 가격 급등은 해상/항공/육상 운송비 등 물류비용 전반에 직접적인 상승 압력으로 작용하여 즉각적인 대응이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G398" s="2" t="inlineStr">
+        <is>
+          <t>유가 변동에 따른 운송비 상승분을 분석하고, 운송 계약 재검토, 운송 모드 최적화, 연료 효율 개선 방안 등을 검토하여 물류비 절감 대책을 수립해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H398" s="2" t="inlineStr">
+        <is>
+          <t>이투데이</t>
+        </is>
+      </c>
+      <c r="I398" s="2" t="inlineStr">
+        <is>
+          <t>https://etoday.co.kr/news/view/2599487</t>
+        </is>
+      </c>
+      <c r="J398" s="2" t="inlineStr">
+        <is>
+          <t>RSK-069</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B399" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C399" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D399" s="2" t="inlineStr">
+        <is>
+          <t>6월 물가 3.2% ‘2년 6개월 만에 최고’…기름값이 끌어올렸다</t>
+        </is>
+      </c>
+      <c r="E399" s="2" t="inlineStr">
+        <is>
+          <t>지난 6월 소비자물가가 3.2% 상승하며 2년 6개월 만에 최고치를 기록했으며, 이는 중동 분쟁으로 인한 국제유가 상승과 석유류 가격 인상이 주된 원인입니다.</t>
+        </is>
+      </c>
+      <c r="F399" s="2" t="inlineStr">
+        <is>
+          <t>국제유가 상승은 해상/항공/육상 운임 상승으로 직결되어 우리 회사의 물류비용 증가 및 SCM 운영에 직접적인 영향을 미칠 것입니다.</t>
+        </is>
+      </c>
+      <c r="G399" s="2" t="inlineStr">
+        <is>
+          <t>물류비용 상승에 대비하여 운송 계약 재검토 및 운임 협상 전략을 수립하고, 연료 효율적인 운송수단 또는 경로를 검토해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H399" s="2" t="inlineStr">
+        <is>
+          <t>헤럴드경제</t>
+        </is>
+      </c>
+      <c r="I399" s="2" t="inlineStr">
+        <is>
+          <t>https://biz.heraldcorp.com/article/10795291</t>
+        </is>
+      </c>
+      <c r="J399" s="2" t="inlineStr">
+        <is>
+          <t>RSK-070</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B400" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C400" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D400" s="3" t="inlineStr">
+        <is>
+          <t>Air Cargo Demand Up 6.0% in May</t>
+        </is>
+      </c>
+      <c r="E400" s="3" t="inlineStr">
+        <is>
+          <t>2026년 5월 전 세계 항공 화물 수요가 전년 동월 대비 6.0% 증가했다.</t>
+        </is>
+      </c>
+      <c r="F400" s="3" t="inlineStr">
+        <is>
+          <t>항공 화물 수요 증가는 항공 운임 상승 압력으로 작용할 수 있으며, 이는 배터리/전자부품 운송 비용에 영향을 줄 수 있으므로 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G400" s="3" t="inlineStr">
+        <is>
+          <t>항공 화물 운임 및 선복 동향 지속 모니터링, 필요 시 항공 운송 계획 조정 검토.</t>
+        </is>
+      </c>
+      <c r="H400" s="3" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I400" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-29-air-cargo-demand-up-may/</t>
+        </is>
+      </c>
+      <c r="J400" s="3" t="inlineStr"/>
+    </row>
+    <row r="401">
+      <c r="A401" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B401" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C401" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D401" s="3" t="inlineStr">
+        <is>
+          <t>Urgent Action Needed to Ease Engine MRO Bottlenecks</t>
+        </is>
+      </c>
+      <c r="E401" s="3" t="inlineStr">
+        <is>
+          <t>IATA는 항공기 엔진 유지보수(MRO) 병목 현상 완화를 위한 긴급 조치를 촉구했다.</t>
+        </is>
+      </c>
+      <c r="F401" s="3" t="inlineStr">
+        <is>
+          <t>항공기 엔진 MRO 병목 현상은 항공 운항 지연 및 항공 화물 운송 능력에 영향을 미칠 수 있으므로, 잠재적 영향을 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G401" s="3" t="inlineStr">
+        <is>
+          <t>항공 운송 지연 가능성 및 항공 화물 선복량 변화 추이 모니터링.</t>
+        </is>
+      </c>
+      <c r="H401" s="3" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I401" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-24-urgent-action-needed-to-ease-engine-mro-bottlenecks/</t>
+        </is>
+      </c>
+      <c r="J401" s="3" t="inlineStr"/>
+    </row>
+    <row r="402">
+      <c r="A402" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B402" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C402" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D402" s="3" t="inlineStr">
+        <is>
+          <t>Tracking True Vessel Delay</t>
+        </is>
+      </c>
+      <c r="E402" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence는 선사들이 운송 시간을 늘려 스케줄 버퍼링을 활용하는 경향이 증가하고 있음을 분석하며, 실제 선박 지연 추적의 중요성을 강조했다.</t>
+        </is>
+      </c>
+      <c r="F402" s="3" t="inlineStr">
+        <is>
+          <t>선사들의 스케줄 버퍼링 증가는 겉으로는 정시성을 높이나 실제 운송 시간은 길어질 수 있어, 우리 회사의 리드타임 예측 및 재고 계획에 잠재적 영향을 미칠 수 있으므로 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G402" s="3" t="inlineStr">
+        <is>
+          <t>주요 항로의 실제 운송 리드타임 데이터 분석 및 선사별 스케줄 버퍼링 전략 확인, 리드타임 예측 모델 업데이트 검토.</t>
+        </is>
+      </c>
+      <c r="H402" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I402" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/394-tracking-true-vessel-delay</t>
+        </is>
+      </c>
+      <c r="J402" s="3" t="inlineStr"/>
+    </row>
+    <row r="403">
+      <c r="A403" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B403" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C403" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D403" s="3" t="inlineStr">
+        <is>
+          <t>Transpacific: Ripe for new non-alliance services</t>
+        </is>
+      </c>
+      <c r="E403" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence는 태평양 횡단 노선에서 비동맹 선사들의 새로운 서비스가 증가할 가능성이 높다고 분석했다.</t>
+        </is>
+      </c>
+      <c r="F403" s="3" t="inlineStr">
+        <is>
+          <t>태평양 횡단 노선에 비동맹 선사 서비스 증가는 운임 경쟁 심화 및 선복량 증가로 이어질 수 있어, 향후 운송 옵션 및 비용에 영향을 미칠 수 있으므로 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G403" s="3" t="inlineStr">
+        <is>
+          <t>태평양 횡단 노선 신규 서비스 동향 및 운임 경쟁 상황 지속 모니터링, 잠재적 신규 선사와의 협력 가능성 검토.</t>
+        </is>
+      </c>
+      <c r="H403" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I403" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/393-transpacific-ripe-for-new-non-alliance-services</t>
+        </is>
+      </c>
+      <c r="J403" s="3" t="inlineStr"/>
+    </row>
+    <row r="404">
+      <c r="A404" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B404" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C404" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D404" s="3" t="inlineStr">
+        <is>
+          <t>Decoding Gemini’s Mediterranean Surge</t>
+        </is>
+      </c>
+      <c r="E404" s="3" t="inlineStr">
+        <is>
+          <t>Gemini Cooperation이 동서 컨테이너 선박 배치 및 지중해 노선에 대한 선대 재배치를 진행 중이며, 이는 시장 점유율 변화를 야기할 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="F404" s="3" t="inlineStr">
+        <is>
+          <t>주요 해운 얼라이언스의 선대 재배치는 특정 항로의 선복량 및 서비스 안정성에 영향을 줄 수 있으므로, 지중해 노선을 이용하는 경우 서비스 변화를 주시해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G404" s="3" t="inlineStr">
+        <is>
+          <t>해당 노선 이용 시 선사 서비스 변경 사항 확인 및 대체 운송 방안 검토.</t>
+        </is>
+      </c>
+      <c r="H404" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence Press Room</t>
+        </is>
+      </c>
+      <c r="I404" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/392-decoding-gemini-s-mediterranean-surge</t>
+        </is>
+      </c>
+      <c r="J404" s="3" t="inlineStr"/>
+    </row>
+    <row r="405">
+      <c r="A405" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B405" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C405" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D405" s="3" t="inlineStr">
+        <is>
+          <t>컨테이너선 정시 준수율, 5월 65%로 연초 이후 최고...전년 동월 대비로는 1.2 포인트 하락</t>
+        </is>
+      </c>
+      <c r="E405" s="3" t="inlineStr">
+        <is>
+          <t>5월 전 세계 컨테이너선 정시 준수율은 64.7%로 올해 최고치를 기록했으나, 전년 동월 대비 하락했으며 지연 선박의 평균 도착 지연일은 증가했습니다.</t>
+        </is>
+      </c>
+      <c r="F405" s="3" t="inlineStr">
+        <is>
+          <t>정시 준수율이 개선되는 추세이나 여전히 낮은 수준이며, 평균 지연일이 증가하고 있어 해상 운송의 예측 불확실성이 지속될 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G405" s="3" t="inlineStr">
+        <is>
+          <t>해상 운송 리드타임 변동성 고려, 재고 수준 및 안전 재고 정책 재검토, 주요 선사별 정시성 데이터 모니터링.</t>
+        </is>
+      </c>
+      <c r="H405" s="3" t="inlineStr">
+        <is>
+          <t>shippingnewsnet.com</t>
+        </is>
+      </c>
+      <c r="I405" s="3" t="inlineStr">
+        <is>
+          <t>https://www.shippingnewsnet.com/news/articleView.html?idxno=71009</t>
+        </is>
+      </c>
+      <c r="J405" s="3" t="inlineStr"/>
+    </row>
+    <row r="406">
+      <c r="A406" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B406" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C406" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D406" s="3" t="inlineStr">
+        <is>
+          <t>인천항 1만6000TEU급 시대 열었다</t>
+        </is>
+      </c>
+      <c r="E406" s="3" t="inlineStr">
+        <is>
+          <t>인천항 미주 정기항로에 1만6000TEU급 초대형 컨테이너선이 처음 투입되며 대형선 시대가 본격화되었습니다.</t>
+        </is>
+      </c>
+      <c r="F406" s="3" t="inlineStr">
+        <is>
+          <t>인천항의 미주 노선 대형선 투입은 해당 노선의 선복량 증가 및 운송 효율성 개선으로 이어질 수 있어, 미주향 물류 운영에 긍정적인 영향을 줄 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G406" s="3" t="inlineStr">
+        <is>
+          <t>인천항 이용 시 미주 노선 서비스 변화 및 운임 동향 주시.</t>
+        </is>
+      </c>
+      <c r="H406" s="3" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I406" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260702-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J406" s="3" t="inlineStr"/>
+    </row>
+    <row r="407">
+      <c r="A407" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B407" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C407" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D407" s="3" t="inlineStr">
+        <is>
+          <t>美, USMCA 연장 거부 방침… 북미 자유무역체제 ‘중대 분수령’</t>
+        </is>
+      </c>
+      <c r="E407" s="3" t="inlineStr">
+        <is>
+          <t>미국이 북미자유무역협정(USMCA) 연장 거부 방침을 밝히면서 북미 자유무역 체제에 중대한 변화가 예상됩니다.</t>
+        </is>
+      </c>
+      <c r="F407" s="3" t="inlineStr">
+        <is>
+          <t>USMCA 연장 거부는 북미 지역 내 무역 조건 및 관세에 변화를 가져와, 해당 지역으로의 수출입 물류 비용 및 절차에 영향을 미칠 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G407" s="3" t="inlineStr">
+        <is>
+          <t>북미 지역 수출입 물량 및 관련 규제 변화 동향 지속 모니터링, 잠재적 관세 및 무역 장벽 변화에 대비.</t>
+        </is>
+      </c>
+      <c r="H407" s="3" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I407" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260701-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J407" s="3" t="inlineStr"/>
+    </row>
+    <row r="408">
+      <c r="A408" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B408" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C408" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D408" s="3" t="inlineStr">
+        <is>
+          <t>국제유가, 주말 호르무즈 무력공방에 상승…WTI 2%↑</t>
+        </is>
+      </c>
+      <c r="E408" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 인근 무력 공방 등 지정학적 긴장으로 국제유가(WTI)가 2% 상승했습니다.</t>
+        </is>
+      </c>
+      <c r="F408" s="3" t="inlineStr">
+        <is>
+          <t>국제유가 상승은 해상 및 항공 운임의 유류할증료 인상으로 이어져 전체 물류비용 증가에 직접적인 영향을 미칠 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G408" s="3" t="inlineStr">
+        <is>
+          <t>유가 및 유류할증료 변동 추이 모니터링, 운송 계약 시 유류할증료 조건 검토.</t>
+        </is>
+      </c>
+      <c r="H408" s="3" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I408" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260630-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J408" s="3" t="inlineStr"/>
+    </row>
+    <row r="409">
+      <c r="A409" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B409" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C409" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D409" s="3" t="inlineStr">
+        <is>
+          <t>CPTPP 회원국, 인도네시아·필리핀·UAE와 가입 예비협상 개시</t>
+        </is>
+      </c>
+      <c r="E409" s="3" t="inlineStr">
+        <is>
+          <t>CPTPP 회원국들이 인도네시아, 필리핀, UAE와 가입 예비협상을 개시하여 아시아-태평양 지역 무역 환경 변화가 예상됩니다.</t>
+        </is>
+      </c>
+      <c r="F409" s="3" t="inlineStr">
+        <is>
+          <t>CPTPP 확대는 해당 국가들과의 무역 조건 및 관세에 영향을 미쳐, 향후 우리 회사의 수출입 전략 및 물류 네트워크 최적화에 고려될 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G409" s="3" t="inlineStr">
+        <is>
+          <t>CPTPP 가입 협상 진행 상황 및 회원국 확대에 따른 무역 규제 변화 동향 지속 모니터링.</t>
+        </is>
+      </c>
+      <c r="H409" s="3" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I409" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260628-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J409" s="3" t="inlineStr"/>
+    </row>
+    <row r="410">
+      <c r="A410" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B410" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C410" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D410" s="3" t="inlineStr">
+        <is>
+          <t>Chinese Companies Prioritise Supply Chain Resilience, AI and New Markets for Growth | The Manila Times</t>
+        </is>
+      </c>
+      <c r="E410" s="3" t="inlineStr">
+        <is>
+          <t>DP World 조사에 따르면 중국 기업들은 최근 글로벌 무역의 혼란과 불확실성에 대응하여 공급망 탄력성, AI 도입, 신시장 접근을 장기 성장 전략으로 우선시하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F410" s="3" t="inlineStr">
+        <is>
+          <t>주요 경쟁국 기업들의 공급망 전략 변화는 장기적으로 글로벌 물류 환경 및 경쟁 구도에 영향을 미칠 수 있으므로 추이를 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G410" s="3" t="inlineStr">
+        <is>
+          <t>글로벌 공급망 트렌드 및 경쟁사 동향 분석, AI 기반 물류 시스템 도입 가능성 검토.</t>
+        </is>
+      </c>
+      <c r="H410" s="3" t="inlineStr">
+        <is>
+          <t>The Manila Times</t>
+        </is>
+      </c>
+      <c r="I410" s="3" t="inlineStr">
+        <is>
+          <t>https://www.manilatimes.net/2026/07/02/tmt-newswire/media-outreach-newswire/chinese-companies-prioritise-supply-chain-resilience-ai-and-new-markets-for-growth/2377234</t>
+        </is>
+      </c>
+      <c r="J410" s="3" t="inlineStr"/>
+    </row>
+    <row r="411">
+      <c r="A411" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B411" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C411" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D411" s="3" t="inlineStr">
+        <is>
+          <t>The supply chain is not recovering; it is restructuring | ITWeb</t>
+        </is>
+      </c>
+      <c r="E411" s="3" t="inlineStr">
+        <is>
+          <t>DCC Technologies 관계자는 공급망이 회복되는 것이 아니라 재편되고 있으며, 고객을 변동성으로부터 보호할 구조적 지원이 필요하다고 강조했습니다.</t>
+        </is>
+      </c>
+      <c r="F411" s="3" t="inlineStr">
+        <is>
+          <t>공급망의 구조적 재편은 우리 회사의 물류 전략 및 파트너십에 장기적인 영향을 미칠 수 있으므로 지속적인 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G411" s="3" t="inlineStr">
+        <is>
+          <t>현재 공급망 구조의 취약점 분석 및 재편 가능성 검토, 유통 파트너와의 협력 강화 방안 모색.</t>
+        </is>
+      </c>
+      <c r="H411" s="3" t="inlineStr">
+        <is>
+          <t>ITWeb</t>
+        </is>
+      </c>
+      <c r="I411" s="3" t="inlineStr">
+        <is>
+          <t>https://www.itweb.co.za/article/the-supply-chain-is-not-recovering-it-is-restructuring/kLgB1Mezp9mq59N4</t>
+        </is>
+      </c>
+      <c r="J411" s="3" t="inlineStr"/>
+    </row>
+    <row r="412">
+      <c r="A412" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B412" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C412" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D412" s="3" t="inlineStr">
+        <is>
+          <t>오늘(2일) 오전 9시 괌 동쪽 약 1690㎞ 부근에서 9호 태풍 ’바비’가 발생했습니다.</t>
+        </is>
+      </c>
+      <c r="E412" s="3" t="inlineStr">
+        <is>
+          <t>9호 태풍 '바비'가 괌 동쪽에서 발생하여 사이판 부근을 통과할 것으로 예상되며, 고수온 해역을 지나며 발달할 가능성이 있습니다.</t>
+        </is>
+      </c>
+      <c r="F412" s="3" t="inlineStr">
+        <is>
+          <t>태풍의 진로와 강도에 따라 주요 해상 운송 경로 및 항만 운영에 지연이 발생할 수 있으므로 지속적인 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G412" s="3" t="inlineStr">
+        <is>
+          <t>태풍 진로 및 예상 영향 지역을 지속적으로 모니터링하고, 선박 스케줄 변경 가능성에 대비하여 운송 계획을 점검해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H412" s="3" t="inlineStr">
+        <is>
+          <t>연합뉴스TV</t>
+        </is>
+      </c>
+      <c r="I412" s="3" t="inlineStr">
+        <is>
+          <t>https://yonhapnewstv.co.kr/news/AKR20260702112529WFk</t>
+        </is>
+      </c>
+      <c r="J412" s="3" t="inlineStr"/>
+    </row>
+    <row r="413">
+      <c r="A413" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B413" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C413" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D413" s="3" t="inlineStr">
+        <is>
+          <t>미국, 멕시코·캐나다와 북미무역협정 연장 거부...매년 재검토 방침 [종합]</t>
+        </is>
+      </c>
+      <c r="E413" s="3" t="inlineStr">
+        <is>
+          <t>미국이 멕시코, 캐나다와의 북미무역협정(USMCA) 연장을 거부하고 매년 재검토 방침을 밝히면서, 2036년 협정 종료 가능성과 함께 역내 교역의 불확실성이 커졌습니다.</t>
+        </is>
+      </c>
+      <c r="F413" s="3" t="inlineStr">
+        <is>
+          <t>북미 지역의 무역 정책 불확실성 증가는 글로벌 공급망 재편 및 주요 원자재/부품 조달 비용에 간접적인 영향을 미칠 수 있어 추이를 지켜봐야 합니다.</t>
+        </is>
+      </c>
+      <c r="G413" s="3" t="inlineStr">
+        <is>
+          <t>북미 지역의 무역 정책 변화가 글로벌 공급망 및 원자재 시장에 미칠 잠재적 영향을 분석하고, 장기적인 공급망 전략에 대한 시사점을 검토해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H413" s="3" t="inlineStr">
+        <is>
+          <t>이투데이</t>
+        </is>
+      </c>
+      <c r="I413" s="3" t="inlineStr">
+        <is>
+          <t>https://etoday.co.kr/news/view/2599620</t>
+        </is>
+      </c>
+      <c r="J413" s="3" t="inlineStr"/>
+    </row>
+    <row r="414">
+      <c r="A414" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B414" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C414" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D414" s="4" t="inlineStr">
+        <is>
+          <t>캐세이카고, GBA 저온 복합운송 강화</t>
+        </is>
+      </c>
+      <c r="E414" s="4" t="inlineStr">
+        <is>
+          <t>캐세이카고가 홍콩공항을 중심으로 광동·홍콩·마카오 대만구(GBA) 내 신선물류 네트워크를 강화하며 냉장 바지수송을 신설하고 마카오까지 복합운송 서비스를 확대한다.</t>
+        </is>
+      </c>
+      <c r="F414" s="4" t="inlineStr">
+        <is>
+          <t>특정 지역(GBA)의 신선물류 네트워크 강화 소식으로, 배터리/전자부품 제조사의 일반적인 물류 운영에 직접적인 영향은 미미하다.</t>
+        </is>
+      </c>
+      <c r="G414" s="4" t="n"/>
+      <c r="H414" s="4" t="inlineStr">
+        <is>
+          <t>cargonews</t>
+        </is>
+      </c>
+      <c r="I414" s="4" t="inlineStr">
+        <is>
+          <t>https://www.cargonews.co.kr/news/articleView.html?idxno=60435</t>
+        </is>
+      </c>
+      <c r="J414" s="4" t="inlineStr"/>
+    </row>
+    <row r="415">
+      <c r="A415" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B415" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C415" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D415" s="4" t="inlineStr">
+        <is>
+          <t>Air Passenger Demand Falls 2.2% in May</t>
+        </is>
+      </c>
+      <c r="E415" s="4" t="inlineStr">
+        <is>
+          <t>2026년 5월 전 세계 항공 여객 수요가 전년 동월 대비 2.2% 감소했다.</t>
+        </is>
+      </c>
+      <c r="F415" s="4" t="inlineStr">
+        <is>
+          <t>항공 여객 수요 감소는 항공 화물 운송에 간접적인 영향을 미칠 수 있으나, 배터리/전자부품 제조사의 물류 운영에 직접적인 영향은 미미하다.</t>
+        </is>
+      </c>
+      <c r="G415" s="4" t="n"/>
+      <c r="H415" s="4" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I415" s="4" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-30-air-passenger-demand-falls-may/</t>
+        </is>
+      </c>
+      <c r="J415" s="4" t="inlineStr"/>
+    </row>
+    <row r="416">
+      <c r="A416" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B416" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C416" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D416" s="4" t="inlineStr">
+        <is>
+          <t>IATA and IATP Collaborate to Support Airline Supply Chain Resilience</t>
+        </is>
+      </c>
+      <c r="E416" s="4" t="inlineStr">
+        <is>
+          <t>IATA와 IATP가 항공기 부품 가시성 및 접근성 개선을 통해 항공사 공급망 탄력성을 지원하기 위해 협력하기로 합의했다.</t>
+        </is>
+      </c>
+      <c r="F416" s="4" t="inlineStr">
+        <is>
+          <t>항공기 부품 공급망 개선은 항공 운항 안정성에 긍정적이나, 배터리/전자부품 제조사의 물류 운영에 직접적인 영향은 미미하다.</t>
+        </is>
+      </c>
+      <c r="G416" s="4" t="n"/>
+      <c r="H416" s="4" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I416" s="4" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-25-iata-iatp-collaborate-support-airline-supply-chain-resilience/</t>
+        </is>
+      </c>
+      <c r="J416" s="4" t="inlineStr"/>
+    </row>
+    <row r="417">
+      <c r="A417" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B417" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C417" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D417" s="4" t="inlineStr">
+        <is>
+          <t>IATA Outlines Four Priorities to Strengthen the Aviation Supply Chain</t>
+        </is>
+      </c>
+      <c r="E417" s="4" t="inlineStr">
+        <is>
+          <t>IATA는 항공 공급망 강화를 위한 네 가지 우선순위를 제시했다.</t>
+        </is>
+      </c>
+      <c r="F417" s="4" t="inlineStr">
+        <is>
+          <t>항공 공급망 강화 노력은 장기적으로 긍정적이나, 배터리/전자부품 제조사의 현재 물류 운영에 직접적인 영향은 미미하다.</t>
+        </is>
+      </c>
+      <c r="G417" s="4" t="n"/>
+      <c r="H417" s="4" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I417" s="4" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-24-iata-outlines-four-priorities-to-strengthen-aviation-supply-chain/</t>
+        </is>
+      </c>
+      <c r="J417" s="4" t="inlineStr"/>
+    </row>
+    <row r="418">
+      <c r="A418" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B418" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C418" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D418" s="4" t="inlineStr">
+        <is>
+          <t>영국 5월 선거 이후 달라진 지방정치 지형과 우리 기업 대응 방향</t>
+        </is>
+      </c>
+      <c r="E418" s="4" t="inlineStr">
+        <is>
+          <t>2026년 5월 영국 선거 결과, 기존 양당 구도가 약화되고 영국개혁당과 녹색당의 영향력이 확대되는 등 지방정치 지형이 다변화되었다.</t>
+        </is>
+      </c>
+      <c r="F418" s="4" t="inlineStr">
+        <is>
+          <t>영국 지방정치 지형 변화는 거시적인 경제 및 무역 환경에 영향을 줄 수 있으나, 배터리/전자부품 제조사의 물류 운영에 당장 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G418" s="4" t="n"/>
+      <c r="H418" s="4" t="inlineStr">
+        <is>
+          <t>kotra</t>
+        </is>
+      </c>
+      <c r="I418" s="4" t="inlineStr">
+        <is>
+          <t>https://dream.kotra.or.kr/kotranews/cms/news/actionKotraBoardDetail.do?SITE_NO=3&amp;MENU_ID=70&amp;CONTENTS_NO=1&amp;pNttSn=242454</t>
+        </is>
+      </c>
+      <c r="J418" s="4" t="inlineStr"/>
+    </row>
+    <row r="419">
+      <c r="A419" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B419" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C419" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D419" s="4" t="inlineStr">
+        <is>
+          <t>삼성중공업, 싱가포르 쿠옥그룹과 조선·해양사업 협력 강화</t>
+        </is>
+      </c>
+      <c r="E419" s="4" t="inlineStr">
+        <is>
+          <t>삼성중공업이 싱가포르 쿠옥그룹과 조선·해양사업 및 해상 물류, 디지털 인프라 등 미래 사업 협력을 위한 전략적 합의서를 체결했다.</t>
+        </is>
+      </c>
+      <c r="F419" s="4" t="inlineStr">
+        <is>
+          <t>특정 기업 간의 조선·해양 및 물류 사업 협력 강화 소식으로, 우리 회사의 물류 운영에 직접적인 영향은 미미하다.</t>
+        </is>
+      </c>
+      <c r="G419" s="4" t="n"/>
+      <c r="H419" s="4" t="inlineStr">
+        <is>
+          <t>ksg</t>
+        </is>
+      </c>
+      <c r="I419" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksg.co.kr/news/main_newsView.jsp?pNum=147544</t>
+        </is>
+      </c>
+      <c r="J419" s="4" t="inlineStr"/>
+    </row>
+    <row r="420">
+      <c r="A420" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B420" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C420" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D420" s="4" t="inlineStr">
+        <is>
+          <t>'내항 선원 400만원 비과세' 사실상 포기?…정부의 면세 폐지 정책에 '불똥'</t>
+        </is>
+      </c>
+      <c r="E420" s="4" t="inlineStr">
+        <is>
+          <t>정부의 면세 폐지 및 보조금 전환 정책으로 내항 선원 비과세 확대 추진이 사실상 좌초 위기에 처해 해운업계의 우려가 커지고 있다.</t>
+        </is>
+      </c>
+      <c r="F420" s="4" t="inlineStr">
+        <is>
+          <t>내항 선원 비과세 정책 변화는 국내 해운업계에 영향을 미치지만, 배터리/전자부품 제조사의 글로벌 물류 운영에 직접적인 영향은 미미하다.</t>
+        </is>
+      </c>
+      <c r="G420" s="4" t="n"/>
+      <c r="H420" s="4" t="inlineStr">
+        <is>
+          <t>oceanpress</t>
+        </is>
+      </c>
+      <c r="I420" s="4" t="inlineStr">
+        <is>
+          <t>https://www.oceanpress.co.kr/news/article.html?no=30507</t>
+        </is>
+      </c>
+      <c r="J420" s="4" t="inlineStr"/>
+    </row>
+    <row r="421">
+      <c r="A421" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B421" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C421" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D421" s="4" t="inlineStr">
+        <is>
+          <t>Global Schedule Reliability for May 2026 the Highest of the Year</t>
+        </is>
+      </c>
+      <c r="E421" s="4" t="inlineStr">
+        <is>
+          <t>2026년 5월 전 세계 선박 스케줄 정시성이 올해 최고치를 기록했다.</t>
+        </is>
+      </c>
+      <c r="F421" s="4" t="inlineStr">
+        <is>
+          <t>전반적인 스케줄 정시성 개선은 긍정적이나, 이미 높은 수준을 유지하고 있었을 가능성이 크며, 특정 항로의 지연 이슈가 여전히 존재할 수 있어 당장 큰 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G421" s="4" t="n"/>
+      <c r="H421" s="4" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I421" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/395-global-schedule-reliability-for-may-2026-the-highest-of-the-year</t>
+        </is>
+      </c>
+      <c r="J421" s="4" t="inlineStr"/>
+    </row>
+    <row r="422">
+      <c r="A422" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B422" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C422" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D422" s="4" t="inlineStr">
+        <is>
+          <t>2026-Q1: NAEC Ports Consolidate Market Share</t>
+        </is>
+      </c>
+      <c r="E422" s="4" t="inlineStr">
+        <is>
+          <t>2026년 1분기 북미 동부 해안(NAEC) 항만의 컨테이너 물동량은 전년 대비 감소했으나, 해당 항만들이 시장 점유율을 공고히 했습니다.</t>
+        </is>
+      </c>
+      <c r="F422" s="4" t="inlineStr">
+        <is>
+          <t>북미 동부 항만의 물동량 감소는 당장 항만 적체를 심화시키지 않으며, 시장 점유율 공고화는 장기적인 안정성 측면에서 긍정적일 수 있어 즉각적인 영향은 낮습니다.</t>
+        </is>
+      </c>
+      <c r="G422" s="4" t="n"/>
+      <c r="H422" s="4" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence Press Room</t>
+        </is>
+      </c>
+      <c r="I422" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/391-2026-q1-naec-ports-consolidate-market-share</t>
+        </is>
+      </c>
+      <c r="J422" s="4" t="inlineStr"/>
+    </row>
+    <row r="423">
+      <c r="A423" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B423" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C423" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D423" s="4" t="inlineStr">
+        <is>
+          <t>씨메스로보틱스 / ‘물류·제조 대형 수주 잇달아’ 피지컬 AI 기반 로봇 자동화 사업 가속</t>
+        </is>
+      </c>
+      <c r="E423" s="4" t="inlineStr">
+        <is>
+          <t>씨메스로보틱스가 쿠팡풀필먼트서비스 등 물류 및 제조 현장에서 대형 로봇 자동화 프로젝트를 연이어 수주하며 사업 확장에 속도를 내고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F423" s="4" t="inlineStr">
+        <is>
+          <t>물류 자동화 기술 발전 동향을 보여주지만, 당사 물류 운영에 즉각적인 영향을 미치는 뉴스는 아니며 참고 수준입니다.</t>
+        </is>
+      </c>
+      <c r="G423" s="4" t="n"/>
+      <c r="H423" s="4" t="inlineStr">
+        <is>
+          <t>ulogistics.co.kr</t>
+        </is>
+      </c>
+      <c r="I423" s="4" t="inlineStr">
+        <is>
+          <t>http://www.ulogistics.co.kr/test/board.php?board=all2&amp;command=body&amp;no=5202</t>
+        </is>
+      </c>
+      <c r="J423" s="4" t="inlineStr"/>
+    </row>
+    <row r="424">
+      <c r="A424" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B424" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C424" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D424" s="4" t="inlineStr">
+        <is>
+          <t>Kharon Named "Risk Management Company of the Year” By SupplyTech Breakthrough | The Manila Times</t>
+        </is>
+      </c>
+      <c r="E424" s="4" t="inlineStr">
+        <is>
+          <t>Kharon이 공급망 및 물류 기술 혁신을 기리는 SupplyTech Breakthrough Awards에서 "올해의 리스크 관리 회사"로 선정되었습니다.</t>
+        </is>
+      </c>
+      <c r="F424" s="4" t="inlineStr">
+        <is>
+          <t>특정 기업의 수상 소식으로, 우리 회사의 물류 운영에 직접적인 영향은 없으며 참고 수준의 정보입니다.</t>
+        </is>
+      </c>
+      <c r="G424" s="4" t="n"/>
+      <c r="H424" s="4" t="inlineStr">
+        <is>
+          <t>The Manila Times</t>
+        </is>
+      </c>
+      <c r="I424" s="4" t="inlineStr">
+        <is>
+          <t>https://manilatimes.net/2026/07/02/tmt-newswire/globenewswire/kharon-named-risk-management-company-of-the-year-by-supplytech-breakthrough/2377008</t>
+        </is>
+      </c>
+      <c r="J424" s="4" t="inlineStr"/>
+    </row>
+    <row r="425">
+      <c r="A425" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B425" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C425" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D425" s="4" t="inlineStr">
+        <is>
+          <t>중국 산둥성항구그룹, 인천항 방문…신규항로 개설 협력</t>
+        </is>
+      </c>
+      <c r="E425" s="4" t="inlineStr">
+        <is>
+          <t>중국 산둥성항구그룹이 인천항을 방문하여 신규 항로 개설 등 협력 방안을 논의했으며, 이는 인천항의 물동량 증대와 물류 서비스 확대로 이어질 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="F425" s="4" t="inlineStr">
+        <is>
+          <t>신규 항로 개설 논의는 장기적으로 물류 효율성 증대에 긍정적이지만, 당장 우리 회사의 물류 운영에 직접적인 영향을 미치지는 않습니다.</t>
+        </is>
+      </c>
+      <c r="G425" s="4" t="n"/>
+      <c r="H425" s="4" t="inlineStr">
+        <is>
+          <t>디지털타임스</t>
+        </is>
+      </c>
+      <c r="I425" s="4" t="inlineStr">
+        <is>
+          <t>https://dt.co.kr/article/12070522</t>
+        </is>
+      </c>
+      <c r="J425" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
@@ -19503,7 +21015,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I65"/>
+  <dimension ref="A1:I71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -21804,6 +23316,216 @@
       </c>
       <c r="I65" s="6" t="inlineStr"/>
     </row>
+    <row r="66">
+      <c r="A66" s="6" t="inlineStr">
+        <is>
+          <t>RSK-065</t>
+        </is>
+      </c>
+      <c r="B66" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C66" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D66" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E66" s="6" t="inlineStr">
+        <is>
+          <t>U.S. Appeals CIT's IEEPA Refund Order to Federal Circuit; TPEB Rates Rise as Peak Season Demand Tightens Capacity</t>
+        </is>
+      </c>
+      <c r="F66" s="6" t="inlineStr"/>
+      <c r="G66" s="6" t="inlineStr"/>
+      <c r="H66" s="6" t="inlineStr">
+        <is>
+          <t>TPEB 노선 운임 변동성 주시 및 운송 계약 조건 재검토, 대체 운송 방안 또는 선사 협상 준비, 성수기 물량 예측 및 선복 확보 계획 수립.</t>
+        </is>
+      </c>
+      <c r="I66" s="6" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="6" t="inlineStr">
+        <is>
+          <t>RSK-066</t>
+        </is>
+      </c>
+      <c r="B67" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C67" s="6" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="D67" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E67" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈에서 컨선 '좌초'…이란, "항로 이탈이 원인"</t>
+        </is>
+      </c>
+      <c r="F67" s="6" t="inlineStr"/>
+      <c r="G67" s="6" t="inlineStr"/>
+      <c r="H67" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 통과 예정 선박의 운항 스케줄 확인 및 지연 가능성 평가, 대체 항로 또는 운송 수단 검토.</t>
+        </is>
+      </c>
+      <c r="I67" s="6" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="6" t="inlineStr">
+        <is>
+          <t>RSK-067</t>
+        </is>
+      </c>
+      <c r="B68" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C68" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D68" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E68" s="6" t="inlineStr">
+        <is>
+          <t>글로벌 해운운임, 9주 연속 상승…3200대 돌파</t>
+        </is>
+      </c>
+      <c r="F68" s="6" t="inlineStr"/>
+      <c r="G68" s="6" t="inlineStr"/>
+      <c r="H68" s="6" t="inlineStr">
+        <is>
+          <t>긴급 물량에 대한 항공 운송 전환 검토, 선사와의 운임 협상 재검토, 장기 계약 조건 확인, 운임 상승에 따른 물류비 예산 재조정.</t>
+        </is>
+      </c>
+      <c r="I68" s="6" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="6" t="inlineStr">
+        <is>
+          <t>RSK-068</t>
+        </is>
+      </c>
+      <c r="B69" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C69" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D69" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E69" s="6" t="inlineStr">
+        <is>
+          <t>미-이란, 호르무즈 무력 충돌 재개...종전 합의 9일 만</t>
+        </is>
+      </c>
+      <c r="F69" s="6" t="inlineStr"/>
+      <c r="G69" s="6" t="inlineStr"/>
+      <c r="H69" s="6" t="inlineStr">
+        <is>
+          <t>중동 경유 노선 선박 스케줄 및 운항 정보 실시간 모니터링, 대체 항로 및 운송 수단(항공) 검토, 비상 재고 확보 여부 점검.</t>
+        </is>
+      </c>
+      <c r="I69" s="6" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="6" t="inlineStr">
+        <is>
+          <t>RSK-069</t>
+        </is>
+      </c>
+      <c r="B70" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C70" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D70" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E70" s="6" t="inlineStr">
+        <is>
+          <t>6월 소비자물가 3.2%↑…석유류 급등에 30개월 만에 최대폭 상승 [종합]</t>
+        </is>
+      </c>
+      <c r="F70" s="6" t="inlineStr"/>
+      <c r="G70" s="6" t="inlineStr"/>
+      <c r="H70" s="6" t="inlineStr">
+        <is>
+          <t>유가 변동에 따른 운송비 상승분을 분석하고, 운송 계약 재검토, 운송 모드 최적화, 연료 효율 개선 방안 등을 검토하여 물류비 절감 대책을 수립해야 합니다.</t>
+        </is>
+      </c>
+      <c r="I70" s="6" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="6" t="inlineStr">
+        <is>
+          <t>RSK-070</t>
+        </is>
+      </c>
+      <c r="B71" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C71" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D71" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E71" s="6" t="inlineStr">
+        <is>
+          <t>6월 물가 3.2% ‘2년 6개월 만에 최고’…기름값이 끌어올렸다</t>
+        </is>
+      </c>
+      <c r="F71" s="6" t="inlineStr"/>
+      <c r="G71" s="6" t="inlineStr"/>
+      <c r="H71" s="6" t="inlineStr">
+        <is>
+          <t>물류비용 상승에 대비하여 운송 계약 재검토 및 운임 협상 전략을 수립하고, 연료 효율적인 운송수단 또는 경로를 검토해야 합니다.</t>
+        </is>
+      </c>
+      <c r="I71" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
📰 뉴스 데이터 2026-07-03_09:07
</commit_message>
<xml_diff>
--- a/data/SCM_물류_브리핑.xlsx
+++ b/data/SCM_물류_브리핑.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J425"/>
+  <dimension ref="A1:J463"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -20586,6 +20586,1802 @@
       </c>
       <c r="J425" s="4" t="inlineStr"/>
     </row>
+    <row r="426">
+      <c r="A426" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B426" s="2" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C426" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D426" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈에서 컨선 '좌초'…이란, "항로 이탈이 원인"</t>
+        </is>
+      </c>
+      <c r="E426" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 라락섬 인근 수역에서 컨테이너선이 항로를 이탈하여 좌초되었으며, 이는 해당 해역의 운항 지연 및 변수로 작용할 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="F426" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협은 주요 해상 운송로이며, 컨테이너선 좌초는 해당 항로의 운항 지연을 유발하여 우리 물류 운영에 직접적인 영향을 미칠 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G426" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협을 통과하는 선박의 운항 상황을 즉시 확인하고, 해당 노선을 이용하는 물품의 운송 지연 가능성에 대비하여 비상 계획을 수립.</t>
+        </is>
+      </c>
+      <c r="H426" s="2" t="inlineStr">
+        <is>
+          <t>kita</t>
+        </is>
+      </c>
+      <c r="I426" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kita.net/shippers/board/newsView.do?morgueCode=2&amp;dataCls=B&amp;dataSeq=8147</t>
+        </is>
+      </c>
+      <c r="J426" s="2" t="inlineStr">
+        <is>
+          <t>RSK-071</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B427" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C427" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D427" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 통행 수수료…오만, 이란과 공동징수 추진</t>
+        </is>
+      </c>
+      <c r="E427" s="2" t="inlineStr">
+        <is>
+          <t>오만과 이란이 호르무즈 해협 통행 수수료 공동 징수를 추진하며 해운 운임 상승과 물류비 부담 가중이 우려된다.</t>
+        </is>
+      </c>
+      <c r="F427" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 통행 수수료 부과는 중동발 원자재 및 제품 운송 비용을 즉각적으로 상승시켜 우리 회사의 물류비에 직접적인 영향을 미친다.</t>
+        </is>
+      </c>
+      <c r="G427" s="2" t="inlineStr">
+        <is>
+          <t>중동발 원자재 및 제품 운송 경로 및 비용 영향 분석, 대체 운송 경로 및 공급처 검토, 장기 운송 계약 조건 재검토.</t>
+        </is>
+      </c>
+      <c r="H427" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I427" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260703-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J427" s="2" t="inlineStr">
+        <is>
+          <t>RSK-072</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B428" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C428" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D428" s="2" t="inlineStr">
+        <is>
+          <t>국제유가, 주말 호르무즈 무력공방에 상승…WTI 2%↑</t>
+        </is>
+      </c>
+      <c r="E428" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 인근 무력 공방 등 지정학적 긴장으로 국제유가가 2% 상승 압력을 받았다.</t>
+        </is>
+      </c>
+      <c r="F428" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협의 지정학적 긴장으로 인한 국제유가 상승은 해상 및 항공 운임 상승으로 이어져 우리 회사의 물류비에 직접적인 영향을 미친다.</t>
+        </is>
+      </c>
+      <c r="G428" s="2" t="inlineStr">
+        <is>
+          <t>유가 및 운임 변동 추이 면밀히 모니터링, 운송 계약 조건 재검토, 연료 효율 개선 방안 모색.</t>
+        </is>
+      </c>
+      <c r="H428" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I428" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260630-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J428" s="2" t="inlineStr">
+        <is>
+          <t>RSK-073</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B429" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C429" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D429" s="2" t="inlineStr">
+        <is>
+          <t>중동전쟁 장기화에 중소기업 피해 '962건'</t>
+        </is>
+      </c>
+      <c r="E429" s="2" t="inlineStr">
+        <is>
+          <t>중동전쟁 장기화로 해상운임 증가 및 우회 운송이 발생하며 중소기업의 물류 피해 사례가 누적되고 있다.</t>
+        </is>
+      </c>
+      <c r="F429" s="2" t="inlineStr">
+        <is>
+          <t>중동전쟁 장기화는 해상운임 상승과 우회 운송을 유발하여 우리 회사의 물류 비용과 납기 준수에 직접적인 영향을 미친다.</t>
+        </is>
+      </c>
+      <c r="G429" s="2" t="inlineStr">
+        <is>
+          <t>중동발 공급망 리스크 재평가, 대체 운송 경로 및 운송사 확보, 재고 수준 조정 검토.</t>
+        </is>
+      </c>
+      <c r="H429" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I429" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260629-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J429" s="2" t="inlineStr">
+        <is>
+          <t>RSK-074</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B430" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C430" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D430" s="2" t="inlineStr">
+        <is>
+          <t>글로벌 해운운임, 9주 연속 상승…3200대 돌파</t>
+        </is>
+      </c>
+      <c r="E430" s="2" t="inlineStr">
+        <is>
+          <t>상하이컨테이너운임지수(SCFI)가 9주 연속 상승하여 3200선을 돌파하며 해상물류 비용 부담이 가중되고 있다.</t>
+        </is>
+      </c>
+      <c r="F430" s="2" t="inlineStr">
+        <is>
+          <t>글로벌 해운 운임의 9주 연속 상승은 우리 회사의 해상 물류비용을 직접적으로 증가시켜 생산 계획 및 제품 가격 경쟁력에 영향을 미친다.</t>
+        </is>
+      </c>
+      <c r="G430" s="2" t="inlineStr">
+        <is>
+          <t>운송 계약 조건 재검토, 장기 운송 계약 협상, 운송 모드 전환 검토 (해당 시), 재고 최적화.</t>
+        </is>
+      </c>
+      <c r="H430" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I430" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260629-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J430" s="2" t="inlineStr">
+        <is>
+          <t>RSK-075</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B431" s="2" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C431" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D431" s="2" t="inlineStr">
+        <is>
+          <t>EU, 2026~2028년 에너지 저장 45GW 로드맵 확정…한국 배터리·ESS 산업 수혜 기대 - 아이티인사이트</t>
+        </is>
+      </c>
+      <c r="E431" s="2" t="inlineStr">
+        <is>
+          <t>유럽연합(EU)이 2026년부터 2028년까지 45GW 규모의 에너지 저장 용량을 추가하는 로드맵을 확정했으며, 이는 한국 배터리 및 ESS 산업에 큰 수혜가 될 것으로 기대됩니다.</t>
+        </is>
+      </c>
+      <c r="F431" s="2" t="inlineStr">
+        <is>
+          <t>EU의 대규모 에너지 저장 로드맵은 우리 회사의 배터리 및 ESS 부품 수요를 크게 증가시킬 것으로 예상되어, 생산 및 물류 계획에 즉각적인 반영이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G431" s="2" t="inlineStr">
+        <is>
+          <t>EU 시장의 예상 수요 증가에 맞춰 생산 계획을 조정하고, 유럽향 물류 네트워크 및 운송 역량을 선제적으로 확보하는 방안을 검토합니다.</t>
+        </is>
+      </c>
+      <c r="H431" s="2" t="inlineStr">
+        <is>
+          <t>아이티인사이트</t>
+        </is>
+      </c>
+      <c r="I431" s="2" t="inlineStr">
+        <is>
+          <t>https://www.itinsight.kr/news/477698</t>
+        </is>
+      </c>
+      <c r="J431" s="2" t="inlineStr">
+        <is>
+          <t>RSK-076</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B432" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C432" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D432" s="3" t="inlineStr">
+        <is>
+          <t>주요 항공사들, 中東항공노선 점차 재개</t>
+        </is>
+      </c>
+      <c r="E432" s="3" t="inlineStr">
+        <is>
+          <t>중동 사태가 진정 기미를 보이면서 캐세이퍼시픽항공(CX) 등 주요 항공사들이 중동 노선 운항을 점차 재개하고 있으며, 8월 1일부터 리야드 화물 노선이 재개될 예정입니다.</t>
+        </is>
+      </c>
+      <c r="F432" s="3" t="inlineStr">
+        <is>
+          <t>중동 노선 재개는 항공 화물 운송 옵션 증가 및 안정화에 긍정적이나, 아직 완전 정상화가 아니므로 추이를 지켜볼 필요가 있습니다.</t>
+        </is>
+      </c>
+      <c r="G432" s="3" t="inlineStr">
+        <is>
+          <t>중동 지역으로의 항공 화물 운송 계획 시 해당 항공사의 스케줄 변동 사항을 지속적으로 확인.</t>
+        </is>
+      </c>
+      <c r="H432" s="3" t="inlineStr">
+        <is>
+          <t>cargonews</t>
+        </is>
+      </c>
+      <c r="I432" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cargonews.co.kr/news/articleView.html?idxno=60438</t>
+        </is>
+      </c>
+      <c r="J432" s="3" t="inlineStr"/>
+    </row>
+    <row r="433">
+      <c r="A433" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B433" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C433" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D433" s="3" t="inlineStr">
+        <is>
+          <t>Air Cargo Demand Up 6.0% in May</t>
+        </is>
+      </c>
+      <c r="E433" s="3" t="inlineStr">
+        <is>
+          <t>IATA에 따르면 2026년 5월 전 세계 항공 화물 수요(CTK 기준)가 전년 동월 대비 6.0% 증가하여 항공 화물 시장의 강세를 보였습니다.</t>
+        </is>
+      </c>
+      <c r="F433" s="3" t="inlineStr">
+        <is>
+          <t>항공 화물 수요 증가는 운임 상승 압력으로 작용할 수 있으며, 이는 배터리/전자부품 운송 비용에 영향을 줄 수 있으므로 추이를 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G433" s="3" t="inlineStr">
+        <is>
+          <t>항공 화물 운임 동향을 주시하고, 필요시 장기 계약 조건 검토 또는 대체 운송 방안을 고려.</t>
+        </is>
+      </c>
+      <c r="H433" s="3" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I433" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-29-air-cargo-demand-up-may/</t>
+        </is>
+      </c>
+      <c r="J433" s="3" t="inlineStr"/>
+    </row>
+    <row r="434">
+      <c r="A434" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B434" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C434" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D434" s="3" t="inlineStr">
+        <is>
+          <t>PLSCI Data Indicates Mega-Hub Retrenchment</t>
+        </is>
+      </c>
+      <c r="E434" s="3" t="inlineStr">
+        <is>
+          <t>UNCTAD의 PLSCI 데이터 분석 결과, 최근 해운 네트워크 재조정이 메가 허브 항만의 후퇴를 시사하며, 이는 항만 연결성 및 효율성에 영향을 줄 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="F434" s="3" t="inlineStr">
+        <is>
+          <t>메가 허브 항만의 역할 변화는 장기적으로 항만 적체 및 운송 스케줄에 영향을 미칠 수 있으므로, 주요 항만의 연결성 변화 추이를 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G434" s="3" t="inlineStr">
+        <is>
+          <t>주요 물류 거점 항만의 연결성 및 서비스 변화를 지속적으로 모니터링하고, 필요시 대체 항만 또는 운송 경로를 검토.</t>
+        </is>
+      </c>
+      <c r="H434" s="3" t="inlineStr">
+        <is>
+          <t>sea-intelligence</t>
+        </is>
+      </c>
+      <c r="I434" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/396-plsci-data-indicates-mega-hub-retrenchment</t>
+        </is>
+      </c>
+      <c r="J434" s="3" t="inlineStr"/>
+    </row>
+    <row r="435">
+      <c r="A435" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B435" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C435" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D435" s="3" t="inlineStr">
+        <is>
+          <t>Transpacific: Ripe for new non-alliance services</t>
+        </is>
+      </c>
+      <c r="E435" s="3" t="inlineStr">
+        <is>
+          <t>아시아-북미 서안(NAWC) 항로에서 비동맹 선사의 컨테이너 선박 용량 점유율과 스팟 운임 간의 관계를 분석한 결과, 새로운 비동맹 서비스의 출현 가능성이 높습니다.</t>
+        </is>
+      </c>
+      <c r="F435" s="3" t="inlineStr">
+        <is>
+          <t>태평양 횡단 노선에 새로운 비동맹 서비스가 등장할 경우 운임 경쟁 심화 및 서비스 옵션 확대 가능성이 있어, 우리 물류 비용 및 스케줄에 영향을 줄 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G435" s="3" t="inlineStr">
+        <is>
+          <t>태평양 횡단 노선의 신규 서비스 동향 및 운임 변화를 모니터링하고, 필요시 운송 계약 전략을 재검토.</t>
+        </is>
+      </c>
+      <c r="H435" s="3" t="inlineStr">
+        <is>
+          <t>sea-intelligence</t>
+        </is>
+      </c>
+      <c r="I435" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/393-transpacific-ripe-for-new-non-alliance-services</t>
+        </is>
+      </c>
+      <c r="J435" s="3" t="inlineStr"/>
+    </row>
+    <row r="436">
+      <c r="A436" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B436" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C436" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D436" s="3" t="inlineStr">
+        <is>
+          <t>Decoding Gemini’s Mediterranean Surge</t>
+        </is>
+      </c>
+      <c r="E436" s="3" t="inlineStr">
+        <is>
+          <t>Gemini Cooperation이 동서 컨테이너 선박 배치를 재조정하여 지중해 지역에 선박을 집중하고 있으며, 이는 해당 지역의 운송 서비스에 변화를 가져올 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="F436" s="3" t="inlineStr">
+        <is>
+          <t>주요 선사 얼라이언스의 선박 재배치는 특정 지역(지중해)의 운송 서비스 가용성 및 스케줄에 영향을 미칠 수 있으므로, 해당 지역으로의 운송이 있다면 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G436" s="3" t="inlineStr">
+        <is>
+          <t>지중해 지역으로의 운송이 있는 경우, Gemini Cooperation의 서비스 변화를 주시하고 운송 계획에 미칠 영향을 평가.</t>
+        </is>
+      </c>
+      <c r="H436" s="3" t="inlineStr">
+        <is>
+          <t>sea-intelligence</t>
+        </is>
+      </c>
+      <c r="I436" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/392-decoding-gemini-s-mediterranean-surge</t>
+        </is>
+      </c>
+      <c r="J436" s="3" t="inlineStr"/>
+    </row>
+    <row r="437">
+      <c r="A437" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B437" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C437" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D437" s="3" t="inlineStr">
+        <is>
+          <t>미·이란, 카타르 중재 간접 종전 협상…호르무즈 해협 통제권 쟁점</t>
+        </is>
+      </c>
+      <c r="E437" s="3" t="inlineStr">
+        <is>
+          <t>미-이란 간 호르무즈 해협 통제권 협상이 진행 중인 가운데, 중동전쟁으로 갇혔던 한국 선박 중 HMM 원유운반선이 처음으로 해협을 빠져나왔다.</t>
+        </is>
+      </c>
+      <c r="F437" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협의 긴장 완화는 긍정적이나, 통제권 쟁점이 남아있어 중동발 원자재 및 제품 운송의 안정성 확보를 위해 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G437" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 관련 지정학적 상황 및 선박 통행 현황 지속 모니터링.</t>
+        </is>
+      </c>
+      <c r="H437" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I437" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260702-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J437" s="3" t="inlineStr"/>
+    </row>
+    <row r="438">
+      <c r="A438" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B438" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C438" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D438" s="3" t="inlineStr">
+        <is>
+          <t>7월 LPG 판매가격 '소폭 인상'... kg당 50원</t>
+        </is>
+      </c>
+      <c r="E438" s="3" t="inlineStr">
+        <is>
+          <t>국제 LPG 가격, 운임, 환율 상승 요인으로 인해 7월 LPG 판매가격이 kg당 50원 소폭 인상되었다.</t>
+        </is>
+      </c>
+      <c r="F438" s="3" t="inlineStr">
+        <is>
+          <t>LPG 가격 인상은 운송비에 간접적인 영향을 줄 수 있으므로, 우리 회사의 운송 수단별 연료 사용 현황을 고려하여 추이를 모니터링할 필요가 있다.</t>
+        </is>
+      </c>
+      <c r="G438" s="3" t="inlineStr">
+        <is>
+          <t>운송 협력사들의 연료비 변동 추이 및 운임 인상 압력 모니터링.</t>
+        </is>
+      </c>
+      <c r="H438" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I438" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260701-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J438" s="3" t="inlineStr"/>
+    </row>
+    <row r="439">
+      <c r="A439" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B439" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C439" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D439" s="3" t="inlineStr">
+        <is>
+          <t>美, USMCA 연장 거부 방침… 북미 자유무역체제 ‘중대 분수령’</t>
+        </is>
+      </c>
+      <c r="E439" s="3" t="inlineStr">
+        <is>
+          <t>미국이 USMCA 연장 거부 방침을 밝히며 북미 자유무역체제에 중대한 변화가 예상된다.</t>
+        </is>
+      </c>
+      <c r="F439" s="3" t="inlineStr">
+        <is>
+          <t>북미 자유무역체제 변화는 북미 시장으로의 수출 및 부품 조달에 영향을 미칠 수 있으므로, 관련 정책 변화와 관세 변동 가능성을 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G439" s="3" t="inlineStr">
+        <is>
+          <t>북미 시장 수출 및 조달 관련 정책 변화 모니터링, 잠재적 관세 영향 분석.</t>
+        </is>
+      </c>
+      <c r="H439" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I439" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260701-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J439" s="3" t="inlineStr"/>
+    </row>
+    <row r="440">
+      <c r="A440" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B440" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C440" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D440" s="3" t="inlineStr">
+        <is>
+          <t>우회덤핑 차단 공조…관세청·무역위 공동 대응</t>
+        </is>
+      </c>
+      <c r="E440" s="3" t="inlineStr">
+        <is>
+          <t>관세청과 무역위원회가 우회덤핑 차단을 위해 공조하며 무역구제 조치의 실효성 강화를 논의한다.</t>
+        </is>
+      </c>
+      <c r="F440" s="3" t="inlineStr">
+        <is>
+          <t>우회덤핑 규제 강화는 특정 국가를 통한 수출입 전략에 영향을 미칠 수 있으므로, 관련 규제 동향을 모니터링하여 잠재적 리스크를 파악해야 한다.</t>
+        </is>
+      </c>
+      <c r="G440" s="3" t="inlineStr">
+        <is>
+          <t>무역 규제 동향 모니터링, 공급망 내 우회 경로 활용 여부 점검.</t>
+        </is>
+      </c>
+      <c r="H440" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I440" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260630-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J440" s="3" t="inlineStr"/>
+    </row>
+    <row r="441">
+      <c r="A441" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B441" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C441" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D441" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 내 한국 선박 2척 추가 탈출...3척만 남아</t>
+        </is>
+      </c>
+      <c r="E441" s="3" t="inlineStr">
+        <is>
+          <t>종전 합의 이후 호르무즈 해협을 빠져나온 한국 선박이 늘었으나 아직 3척이 남아있어 물류 불확실성이 지속된다.</t>
+        </is>
+      </c>
+      <c r="F441" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협의 선박 통행 불확실성은 중동발 원자재 및 제품 운송의 안정성에 영향을 미치므로, 상황 안정화 추이를 지속 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G441" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 관련 지정학적 상황 및 선박 통행 현황 지속 모니터링.</t>
+        </is>
+      </c>
+      <c r="H441" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I441" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260629-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J441" s="3" t="inlineStr"/>
+    </row>
+    <row r="442">
+      <c r="A442" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B442" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C442" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D442" s="3" t="inlineStr">
+        <is>
+          <t>Forced Labor Is Becoming a Geopolitical Risk for Global Supply Chains</t>
+        </is>
+      </c>
+      <c r="E442" s="3" t="inlineStr">
+        <is>
+          <t>강제 노동이 글로벌 공급망의 지정학적 리스크로 부상하고 있으며, 기업들이 이를 우선순위로 다루지 못하고 있다는 보고서가 나왔다.</t>
+        </is>
+      </c>
+      <c r="F442" s="3" t="inlineStr">
+        <is>
+          <t>강제 노동 관련 규제 강화는 우리 회사의 공급망 실사 및 협력사 관리에 영향을 미칠 수 있으며, 특히 원자재 조달 시 윤리적 공급망 이슈가 중요하므로 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G442" s="3" t="inlineStr">
+        <is>
+          <t>공급망 내 강제 노동 리스크 평가, 협력사 ESG 실사 강화, 관련 국제 규제 동향 모니터링.</t>
+        </is>
+      </c>
+      <c r="H442" s="3" t="inlineStr">
+        <is>
+          <t>wwd.com</t>
+        </is>
+      </c>
+      <c r="I442" s="3" t="inlineStr">
+        <is>
+          <t>https://wwd.com/sourcing-journal/sustainability/forced-labor-supply-chains-verisk-maplecroft-1239050394</t>
+        </is>
+      </c>
+      <c r="J442" s="3" t="inlineStr"/>
+    </row>
+    <row r="443">
+      <c r="A443" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B443" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C443" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D443" s="3" t="inlineStr">
+        <is>
+          <t>Chinese Companies Prioritise Supply Chain Resilience, AI and New Markets for Growth | The Manila Times</t>
+        </is>
+      </c>
+      <c r="E443" s="3" t="inlineStr">
+        <is>
+          <t>중국 기업들이 최근 글로벌 무역 혼란에 대응하여 공급망 탄력성 강화, AI 도입, 신시장 개척을 장기 성장 전략으로 삼고 있다는 조사 결과가 나왔습니다. 이는 전 세계 기업들의 공급망 전략 변화를 보여줍니다.</t>
+        </is>
+      </c>
+      <c r="F443" s="3" t="inlineStr">
+        <is>
+          <t>주요 경쟁사이자 협력사인 중국 기업들의 공급망 전략 변화는 장기적으로 우리 회사의 공급망 운영 및 파트너십 전략에 영향을 미칠 수 있으므로 추이를 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G443" s="3" t="inlineStr">
+        <is>
+          <t>글로벌 공급망 트렌드 변화를 지속적으로 분석하고, 우리 회사의 공급망 탄력성 강화 및 AI 도입 전략을 검토합니다.</t>
+        </is>
+      </c>
+      <c r="H443" s="3" t="inlineStr">
+        <is>
+          <t>The Manila Times</t>
+        </is>
+      </c>
+      <c r="I443" s="3" t="inlineStr">
+        <is>
+          <t>https://www.manilatimes.net/2026/07/02/tmt-newswire/media-outreach-newswire/chinese-companies-prioritise-supply-chain-resilience-ai-and-new-markets-for-growth/2377234</t>
+        </is>
+      </c>
+      <c r="J443" s="3" t="inlineStr"/>
+    </row>
+    <row r="444">
+      <c r="A444" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B444" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C444" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D444" s="3" t="inlineStr">
+        <is>
+          <t>연합뉴스TV</t>
+        </is>
+      </c>
+      <c r="E444" s="3" t="inlineStr">
+        <is>
+          <t>9호 태풍 '바비'가 괌 동쪽 해상에서 발생하여 사이판 부근을 통과할 것으로 예상되며, 고수온 해역을 지나며 세력이 강해질 가능성이 있습니다.</t>
+        </is>
+      </c>
+      <c r="F444" s="3" t="inlineStr">
+        <is>
+          <t>태풍 '바비'의 이동 경로와 강도에 따라 괌 및 사이판 인근 해상 운송 경로와 항만 운영에 지연이 발생할 수 있으므로 지속적인 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G444" s="3" t="inlineStr">
+        <is>
+          <t>태풍 이동 경로를 실시간으로 확인하고, 해당 지역을 경유하는 선박 스케줄 및 항공 운송 가능성에 대한 잠재적 영향을 평가합니다.</t>
+        </is>
+      </c>
+      <c r="H444" s="3" t="inlineStr">
+        <is>
+          <t>연합뉴스TV</t>
+        </is>
+      </c>
+      <c r="I444" s="3" t="inlineStr">
+        <is>
+          <t>https://yonhapnewstv.co.kr/news/AKR20260702112529WFk</t>
+        </is>
+      </c>
+      <c r="J444" s="3" t="inlineStr"/>
+    </row>
+    <row r="445">
+      <c r="A445" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B445" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C445" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D445" s="3" t="inlineStr">
+        <is>
+          <t>미국, 멕시코·캐나다와 북미무역협정 연장 거부...매년 재검토 방침 [종합] - 이투데이</t>
+        </is>
+      </c>
+      <c r="E445" s="3" t="inlineStr">
+        <is>
+          <t>미국이 멕시코, 캐나다와의 북미무역협정(USMCA) 연장을 거부하고 매년 재검토 방침을 밝히면서, 2036년 협정 종료 가능성이 제기되어 북미 지역 무역 불확실성이 커지고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F445" s="3" t="inlineStr">
+        <is>
+          <t>북미무역협정의 불확실성은 향후 관세 변동, 통관 절차 복잡화 등 북미 지역으로의 수출입 물류 비용 및 리드타임에 영향을 미칠 수 있으므로 추이를 면밀히 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G445" s="3" t="inlineStr">
+        <is>
+          <t>북미무역협정 관련 논의 진행 상황을 지속적으로 주시하고, 잠재적인 관세 및 무역 장벽 변화에 대비한 시나리오별 대응 방안을 마련합니다.</t>
+        </is>
+      </c>
+      <c r="H445" s="3" t="inlineStr">
+        <is>
+          <t>이투데이</t>
+        </is>
+      </c>
+      <c r="I445" s="3" t="inlineStr">
+        <is>
+          <t>https://etoday.co.kr/news/view/2599620</t>
+        </is>
+      </c>
+      <c r="J445" s="3" t="inlineStr"/>
+    </row>
+    <row r="446">
+      <c r="A446" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B446" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C446" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D446" s="3" t="inlineStr">
+        <is>
+          <t>6월 소비자물가 3.2%↑…석유류 급등에 30개월 만에 최대폭 상승 [종합]</t>
+        </is>
+      </c>
+      <c r="E446" s="3" t="inlineStr">
+        <is>
+          <t>6월 소비자물가가 중동 사태 영향으로 석유류 가격이 급등하며 30개월 만에 최대 폭인 3.2% 상승하여 물류비 상승 압력이 커지고 있다.</t>
+        </is>
+      </c>
+      <c r="F446" s="3" t="inlineStr">
+        <is>
+          <t>석유류 가격 급등은 유가 상승으로 이어져 해상/항공 운임 및 내륙 운송비에 직접적인 영향을 미치므로 지속적인 추이 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G446" s="3" t="inlineStr">
+        <is>
+          <t>유가 변동에 따른 운송비 상승 가능성을 고려하여 운송 계약 조건 및 예산 계획을 검토.</t>
+        </is>
+      </c>
+      <c r="H446" s="3" t="inlineStr">
+        <is>
+          <t>이투데이</t>
+        </is>
+      </c>
+      <c r="I446" s="3" t="inlineStr">
+        <is>
+          <t>https://etoday.co.kr/news/view/2599487</t>
+        </is>
+      </c>
+      <c r="J446" s="3" t="inlineStr"/>
+    </row>
+    <row r="447">
+      <c r="A447" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B447" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C447" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D447" s="3" t="inlineStr">
+        <is>
+          <t>“애플, 메모리 부족 사태에 중국산 구매 협상 중”</t>
+        </is>
+      </c>
+      <c r="E447" s="3" t="inlineStr">
+        <is>
+          <t>애플이 메모리 부족 해결을 위해 중국 CXMT, YMTC와 구매 협상을 진행하며 미국 정부에 로비 중으로, 반도체 공급망의 지정학적 리스크가 부각되고 있다.</t>
+        </is>
+      </c>
+      <c r="F447" s="3" t="inlineStr">
+        <is>
+          <t>반도체/전자부품 공급망의 지정학적 리스크(미중 갈등) 심화는 우리 기업의 부품 조달 및 수출입에 영향을 미칠 수 있으므로 공급망 다변화 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G447" s="3" t="inlineStr">
+        <is>
+          <t>주요 부품의 공급망 다변화 전략 및 잠재적 규제 변화에 대한 대응 방안을 검토.</t>
+        </is>
+      </c>
+      <c r="H447" s="3" t="inlineStr">
+        <is>
+          <t>이투데이</t>
+        </is>
+      </c>
+      <c r="I447" s="3" t="inlineStr">
+        <is>
+          <t>https://etoday.co.kr/news/view/2599675</t>
+        </is>
+      </c>
+      <c r="J447" s="3" t="inlineStr"/>
+    </row>
+    <row r="448">
+      <c r="A448" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B448" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C448" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D448" s="3" t="inlineStr">
+        <is>
+          <t>홍해 통해 원유 실어 나른 우리 선박 11척으로 늘어</t>
+        </is>
+      </c>
+      <c r="E448" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 봉쇄 이후 우회로인 홍해를 통해 원유를 운송한 우리 선박이 11척으로 늘었으며, 이는 중동 정세 불안정의 영향을 보여준다.</t>
+        </is>
+      </c>
+      <c r="F448" s="3" t="inlineStr">
+        <is>
+          <t>중동 정세 불안정으로 인한 주요 해협의 운항 변화는 유가 및 해상 운임에 영향을 미칠 수 있으므로, 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G448" s="3" t="inlineStr">
+        <is>
+          <t>중동 지역 해상 운송 경로 및 유가 변동 추이를 지속적으로 모니터링하고, 비상 운송 계획을 검토.</t>
+        </is>
+      </c>
+      <c r="H448" s="3" t="inlineStr">
+        <is>
+          <t>연합뉴스TV</t>
+        </is>
+      </c>
+      <c r="I448" s="3" t="inlineStr">
+        <is>
+          <t>https://yonhapnewstv.co.kr/news/AKR202607021040527f7</t>
+        </is>
+      </c>
+      <c r="J448" s="3" t="inlineStr"/>
+    </row>
+    <row r="449">
+      <c r="A449" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B449" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C449" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D449" s="3" t="inlineStr">
+        <is>
+          <t>유류할증료 인하… 여름철 해외여행 수요 살아날까</t>
+        </is>
+      </c>
+      <c r="E449" s="3" t="inlineStr">
+        <is>
+          <t>중동전쟁 영향으로 급등했던 유류할증료가 점차 내림세를 보이면서 항공 및 해상 운임 하락 가능성이 제기되고 있다.</t>
+        </is>
+      </c>
+      <c r="F449" s="3" t="inlineStr">
+        <is>
+          <t>유류할증료 인하는 항공 및 해상 운임 하락으로 이어져 물류비 절감 가능성을 제공하므로, 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G449" s="3" t="inlineStr">
+        <is>
+          <t>유류할증료 변동 추이를 지속적으로 모니터링하고, 운송 계약 갱신 시 운임 협상에 반영할 가능성을 검토.</t>
+        </is>
+      </c>
+      <c r="H449" s="3" t="inlineStr">
+        <is>
+          <t>경인일보</t>
+        </is>
+      </c>
+      <c r="I449" s="3" t="inlineStr">
+        <is>
+          <t>https://kyeongin.com/article/1766688</t>
+        </is>
+      </c>
+      <c r="J449" s="3" t="inlineStr"/>
+    </row>
+    <row r="450">
+      <c r="A450" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B450" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C450" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D450" s="3" t="inlineStr">
+        <is>
+          <t>환율·물가·경기 얽힌 통화정책 '고차방정식' … 한은, 해법은 있나</t>
+        </is>
+      </c>
+      <c r="E450" s="3" t="inlineStr">
+        <is>
+          <t>6월 소비자물가가 30개월 만에 최고치를 기록했으나 유가는 내리고 환율은 오르는 등 복잡한 경제 상황 속에서 한국은행의 통화정책 셈법이 복잡해지고 있다.</t>
+        </is>
+      </c>
+      <c r="F450" s="3" t="inlineStr">
+        <is>
+          <t>유가, 환율, 물가 등 거시경제 지표는 물류비(운임, 유류할증료, 환차손 등)에 직접적인 영향을 미치므로, 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G450" s="3" t="inlineStr">
+        <is>
+          <t>환율 및 유가 변동에 따른 물류비 예산 및 운송 계약 조건을 주기적으로 검토.</t>
+        </is>
+      </c>
+      <c r="H450" s="3" t="inlineStr">
+        <is>
+          <t>뉴데일리</t>
+        </is>
+      </c>
+      <c r="I450" s="3" t="inlineStr">
+        <is>
+          <t>https://biz.newdaily.co.kr/site/data/html/2026/07/02/2026070200227.html</t>
+        </is>
+      </c>
+      <c r="J450" s="3" t="inlineStr"/>
+    </row>
+    <row r="451">
+      <c r="A451" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B451" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C451" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D451" s="4" t="inlineStr">
+        <is>
+          <t>日 이스턴카라이너, 신조선 앞세워 美 중량물운송 경쟁력 강화</t>
+        </is>
+      </c>
+      <c r="E451" s="4" t="inlineStr">
+        <is>
+          <t>일본 선사 이스턴카라이너(ECL)가 최대 500톤의 중량물 운송이 가능한 신조 다목적선을 미주 노선에 투입하여 중량물 운송 경쟁력을 강화했습니다.</t>
+        </is>
+      </c>
+      <c r="F451" s="4" t="inlineStr">
+        <is>
+          <t>특정 선사의 중량물 운송 역량 강화는 일반적인 배터리/전자부품 운송에 직접적인 영향은 없으며, 특수 화물 운송 시 참고할 수 있는 정보입니다.</t>
+        </is>
+      </c>
+      <c r="G451" s="4" t="n"/>
+      <c r="H451" s="4" t="inlineStr">
+        <is>
+          <t>ksg</t>
+        </is>
+      </c>
+      <c r="I451" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksg.co.kr/news/main_newsView.jsp?pNum=147508</t>
+        </is>
+      </c>
+      <c r="J451" s="4" t="inlineStr"/>
+    </row>
+    <row r="452">
+      <c r="A452" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B452" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C452" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D452" s="4" t="inlineStr">
+        <is>
+          <t>Global Schedule Reliability for May 2026 the Highest of the Year</t>
+        </is>
+      </c>
+      <c r="E452" s="4" t="inlineStr">
+        <is>
+          <t>2026년 5월 전 세계 선박 스케줄 신뢰도가 올해 최고치를 기록하여 해상 운송의 정시성이 개선되고 있음을 나타냅니다.</t>
+        </is>
+      </c>
+      <c r="F452" s="4" t="inlineStr">
+        <is>
+          <t>전반적인 스케줄 신뢰도 개선은 긍정적인 신호이나, 특정 노선이나 항만의 개별적인 상황은 다를 수 있으므로 당장 직접적인 영향은 낮습니다.</t>
+        </is>
+      </c>
+      <c r="G452" s="4" t="n"/>
+      <c r="H452" s="4" t="inlineStr">
+        <is>
+          <t>sea-intelligence</t>
+        </is>
+      </c>
+      <c r="I452" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/395-global-schedule-reliability-for-may-2026-the-highest-of-the-year</t>
+        </is>
+      </c>
+      <c r="J452" s="4" t="inlineStr"/>
+    </row>
+    <row r="453">
+      <c r="A453" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B453" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C453" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D453" s="4" t="inlineStr">
+        <is>
+          <t>Tracking True Vessel Delay</t>
+        </is>
+      </c>
+      <c r="E453" s="4" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence는 선박 스케줄 버퍼링과 조기 입항 간의 관계를 분석하여 실제 선박 지연을 추적하는 중요성을 강조했습니다.</t>
+        </is>
+      </c>
+      <c r="F453" s="4" t="inlineStr">
+        <is>
+          <t>선박 지연 분석 방법론에 대한 연구는 물류 운영 효율성 개선에 간접적으로 기여할 수 있으나, 당장 우리 물류 운영에 직접적인 영향은 없습니다.</t>
+        </is>
+      </c>
+      <c r="G453" s="4" t="n"/>
+      <c r="H453" s="4" t="inlineStr">
+        <is>
+          <t>sea-intelligence</t>
+        </is>
+      </c>
+      <c r="I453" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/394-tracking-true-vessel-delay</t>
+        </is>
+      </c>
+      <c r="J453" s="4" t="inlineStr"/>
+    </row>
+    <row r="454">
+      <c r="A454" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B454" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C454" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D454" s="4" t="inlineStr">
+        <is>
+          <t>마스오토 "부산항까지 트레일러 자율주행…2028년 화물 완전 무인화"</t>
+        </is>
+      </c>
+      <c r="E454" s="4" t="inlineStr">
+        <is>
+          <t>마스오토가 부산항 물동량을 기반으로 트레일러 자율주행 상용화를 추진하며 2028년 화물 운송의 완전 무인화를 목표로 한다.</t>
+        </is>
+      </c>
+      <c r="F454" s="4" t="inlineStr">
+        <is>
+          <t>자율주행 트레일러 상용화는 장기적인 물류 효율성 개선에 기여할 수 있으나, 현재 우리 회사의 물류 운영에 즉각적인 영향은 미미하다.</t>
+        </is>
+      </c>
+      <c r="G454" s="4" t="n"/>
+      <c r="H454" s="4" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I454" s="4" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260703-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J454" s="4" t="inlineStr"/>
+    </row>
+    <row r="455">
+      <c r="A455" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B455" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C455" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D455" s="4" t="inlineStr">
+        <is>
+          <t>인천항 1만6000TEU급 시대 열었다</t>
+        </is>
+      </c>
+      <c r="E455" s="4" t="inlineStr">
+        <is>
+          <t>인천항 미주 정기항로에 1만6000TEU급 초대형 컨테이너선이 처음 투입되며 대형선 시대가 본격화되었다.</t>
+        </is>
+      </c>
+      <c r="F455" s="4" t="inlineStr">
+        <is>
+          <t>인천항의 대형선 수용 능력 증가는 장기적인 물류 효율성 개선에 기여할 수 있으나, 현재 우리 회사의 운송 계획에 즉각적인 영향은 미미하다.</t>
+        </is>
+      </c>
+      <c r="G455" s="4" t="n"/>
+      <c r="H455" s="4" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I455" s="4" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260702-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J455" s="4" t="inlineStr"/>
+    </row>
+    <row r="456">
+      <c r="A456" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B456" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C456" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D456" s="4" t="inlineStr">
+        <is>
+          <t>씨메스로보틱스 / ‘물류·제조 대형 수주 잇달아’ 피지컬 AI 기반 로봇 자동화 사업 가속</t>
+        </is>
+      </c>
+      <c r="E456" s="4" t="inlineStr">
+        <is>
+          <t>씨메스로보틱스가 쿠팡풀필먼트서비스 등 물류 및 제조 현장에서 피지컬 AI 기반 로봇 자동화 솔루션 대형 수주를 잇달아 확보하며 사업을 확대하고 있다.</t>
+        </is>
+      </c>
+      <c r="F456" s="4" t="inlineStr">
+        <is>
+          <t>물류 자동화 기술 발전 동향을 보여주지만, 현재 우리 회사의 물류 운영에 즉각적인 영향은 미미하다.</t>
+        </is>
+      </c>
+      <c r="G456" s="4" t="n"/>
+      <c r="H456" s="4" t="inlineStr">
+        <is>
+          <t>ulogistics</t>
+        </is>
+      </c>
+      <c r="I456" s="4" t="inlineStr">
+        <is>
+          <t>http://www.ulogistics.co.kr/test/board.php?board=all2&amp;command=body&amp;no=5202</t>
+        </is>
+      </c>
+      <c r="J456" s="4" t="inlineStr"/>
+    </row>
+    <row r="457">
+      <c r="A457" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B457" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C457" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D457" s="4" t="inlineStr">
+        <is>
+          <t>Ivalua: New Research Reveals the Rise of Skimpflation | Supply Chain Outlook</t>
+        </is>
+      </c>
+      <c r="E457" s="4" t="inlineStr">
+        <is>
+          <t>새로운 연구에 따르면 기업들이 비용 관리를 위해 품질을 은밀히 낮추는 '스킴플레이션'이 증가하고 있으며, AI가 탄력적이고 투명한 공급망 구축의 핵심으로 부상하고 있다.</t>
+        </is>
+      </c>
+      <c r="F457" s="4" t="inlineStr">
+        <is>
+          <t>스킴플레이션은 기업의 전략적 선택에 관한 내용이며, AI 활용은 장기적인 공급망 개선에 도움이 될 수 있으나 당장 우리 물류 운영에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G457" s="4" t="n"/>
+      <c r="H457" s="4" t="inlineStr">
+        <is>
+          <t>supplychain-outlook.com</t>
+        </is>
+      </c>
+      <c r="I457" s="4" t="inlineStr">
+        <is>
+          <t>https://www.supplychain-outlook.com/supply-chain-technology/ivalua-the-rise-of-skimpflation</t>
+        </is>
+      </c>
+      <c r="J457" s="4" t="inlineStr"/>
+    </row>
+    <row r="458">
+      <c r="A458" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B458" s="4" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C458" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D458" s="4" t="inlineStr">
+        <is>
+          <t>수도권대기환경청, 진로발효 현장점검… "오존 원인물질 질소산화물 관리 강화" &lt; 신재생.환경 &lt; 기사본문 - 에너지데일리</t>
+        </is>
+      </c>
+      <c r="E458" s="4" t="inlineStr">
+        <is>
+          <t>수도권대기환경청이 특정 사업장을 현장 점검하며 오존 원인물질인 질소산화물(NOx) 관리를 강화할 것을 주문했습니다.</t>
+        </is>
+      </c>
+      <c r="F458" s="4" t="inlineStr">
+        <is>
+          <t>특정 기업에 대한 환경 규제 점검 소식으로, 우리 회사의 직접적인 물류 운영이나 위험물 운송 규제와는 거리가 멀어 당장 영향은 낮습니다.</t>
+        </is>
+      </c>
+      <c r="G458" s="4" t="n"/>
+      <c r="H458" s="4" t="inlineStr">
+        <is>
+          <t>에너지데일리</t>
+        </is>
+      </c>
+      <c r="I458" s="4" t="inlineStr">
+        <is>
+          <t>https://energydaily.co.kr/news/articleView.html?idxno=201068</t>
+        </is>
+      </c>
+      <c r="J458" s="4" t="inlineStr"/>
+    </row>
+    <row r="459">
+      <c r="A459" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B459" s="4" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C459" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D459" s="4" t="inlineStr">
+        <is>
+          <t>[AI로 읽는 경제] 미·이란 종전 국면…한국 산업 대응 방향은?</t>
+        </is>
+      </c>
+      <c r="E459" s="4" t="inlineStr">
+        <is>
+          <t>AI가 미-이란 종전 국면이 한국 산업에 미칠 영향과 대응 방향을 분석한 기사로, 중동 정세 변화가 경제 전반에 영향을 줄 수 있음을 시사한다.</t>
+        </is>
+      </c>
+      <c r="F459" s="4" t="inlineStr">
+        <is>
+          <t>중동 정세 변화는 유가에 간접적인 영향을 줄 수 있으나, 아직 구체적인 물류 관련 영향이 명시되지 않아 직접적인 물류 운영 영향은 미미하다.</t>
+        </is>
+      </c>
+      <c r="G459" s="4" t="inlineStr"/>
+      <c r="H459" s="4" t="inlineStr">
+        <is>
+          <t>뉴스핌</t>
+        </is>
+      </c>
+      <c r="I459" s="4" t="inlineStr">
+        <is>
+          <t>https://newspim.com/news/view/20260702000418</t>
+        </is>
+      </c>
+      <c r="J459" s="4" t="inlineStr"/>
+    </row>
+    <row r="460">
+      <c r="A460" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B460" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C460" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D460" s="4" t="inlineStr">
+        <is>
+          <t>이 대통령 "기업 압박해 투자 유치 못해…최적 환경 만드는 게 정부 역할"</t>
+        </is>
+      </c>
+      <c r="E460" s="4" t="inlineStr">
+        <is>
+          <t>이재명 대통령이 기업 투자 유치를 위해 정부가 최적의 환경을 조성해야 한다고 강조하며, 충청권 첨단산업 발전 비전을 제시했다.</t>
+        </is>
+      </c>
+      <c r="F460" s="4" t="inlineStr">
+        <is>
+          <t>정부의 산업 정책 방향을 제시하는 내용으로, 물류 운영에 직접적인 영향은 없으며 참고 수준이다.</t>
+        </is>
+      </c>
+      <c r="G460" s="4" t="inlineStr"/>
+      <c r="H460" s="4" t="inlineStr">
+        <is>
+          <t>이투데이</t>
+        </is>
+      </c>
+      <c r="I460" s="4" t="inlineStr">
+        <is>
+          <t>https://etoday.co.kr/news/view/2599576</t>
+        </is>
+      </c>
+      <c r="J460" s="4" t="inlineStr"/>
+    </row>
+    <row r="461">
+      <c r="A461" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B461" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C461" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D461" s="4" t="inlineStr">
+        <is>
+          <t>대한상의 “하반기 산업기상도 ‘ABCD’ 맑음”…반도체 ‘최고’, 석화는 ‘비’</t>
+        </is>
+      </c>
+      <c r="E461" s="4" t="inlineStr">
+        <is>
+          <t>대한상의가 하반기 산업기상도를 발표하며 AI, 친환경차, OLED 수요에 힘입어 반도체, 배터리, 디스플레이 산업은 맑을 것으로 전망했다.</t>
+        </is>
+      </c>
+      <c r="F461" s="4" t="inlineStr">
+        <is>
+          <t>배터리 산업의 긍정적 전망은 우리 기업에 좋은 소식이지만, 물류 운영에 직접적인 영향을 미치는 내용은 아니다.</t>
+        </is>
+      </c>
+      <c r="G461" s="4" t="inlineStr"/>
+      <c r="H461" s="4" t="inlineStr">
+        <is>
+          <t>이투데이</t>
+        </is>
+      </c>
+      <c r="I461" s="4" t="inlineStr">
+        <is>
+          <t>https://etoday.co.kr/news/view/2599383</t>
+        </is>
+      </c>
+      <c r="J461" s="4" t="inlineStr"/>
+    </row>
+    <row r="462">
+      <c r="A462" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B462" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C462" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D462" s="4" t="inlineStr">
+        <is>
+          <t>[더구루] 카본식스, 600억 투자 유치…제조업용 AI 로봇 고도화</t>
+        </is>
+      </c>
+      <c r="E462" s="4" t="inlineStr">
+        <is>
+          <t>제조업용 피지컬 AI 기업 카본식스가 600억원 규모의 투자금을 유치하여 로봇 AI 제품 고도화 및 글로벌 시장 진출에 나설 계획이다.</t>
+        </is>
+      </c>
+      <c r="F462" s="4" t="inlineStr">
+        <is>
+          <t>제조업 AI 기술 발전은 장기적으로 물류 자동화 및 효율화에 기여할 수 있으나, 당장 우리 물류 운영에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G462" s="4" t="inlineStr"/>
+      <c r="H462" s="4" t="inlineStr">
+        <is>
+          <t>더구루</t>
+        </is>
+      </c>
+      <c r="I462" s="4" t="inlineStr">
+        <is>
+          <t>https://theguru.co.kr/news/article.html?no=103870</t>
+        </is>
+      </c>
+      <c r="J462" s="4" t="inlineStr"/>
+    </row>
+    <row r="463">
+      <c r="A463" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B463" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C463" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D463" s="4" t="inlineStr">
+        <is>
+          <t>[해양통신] 북극항로 시험운항 선박 '확보'…"8월 말 출항 유력"</t>
+        </is>
+      </c>
+      <c r="E463" s="4" t="inlineStr">
+        <is>
+          <t>북극항로 시험 운항을 위한 내빙 컨테이너선 확보가 완료되어 8월 말 출항이 유력하며, 이는 장기적인 운송 경로 다변화 가능성을 제시한다.</t>
+        </is>
+      </c>
+      <c r="F463" s="4" t="inlineStr">
+        <is>
+          <t>북극항로 시험 운항은 장기적인 관점에서 새로운 운송 경로 개발 가능성을 보여주지만, 당장 우리 기업의 물류 운영에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G463" s="4" t="inlineStr"/>
+      <c r="H463" s="4" t="inlineStr">
+        <is>
+          <t>해양통신</t>
+        </is>
+      </c>
+      <c r="I463" s="4" t="inlineStr">
+        <is>
+          <t>https://oceanpress.co.kr/news/article.html?no=30501</t>
+        </is>
+      </c>
+      <c r="J463" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -20598,7 +22394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -21003,6 +22799,49 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>3239.64</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>+118 (+3.8%)</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>+1,151 (+55.1%)</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>3920</v>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>+173 (+4.6%)</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>+1,093 (+38.7%)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -21015,7 +22854,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I71"/>
+  <dimension ref="A1:I77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -23526,6 +25365,216 @@
       </c>
       <c r="I71" s="6" t="inlineStr"/>
     </row>
+    <row r="72">
+      <c r="A72" s="6" t="inlineStr">
+        <is>
+          <t>RSK-071</t>
+        </is>
+      </c>
+      <c r="B72" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C72" s="6" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="D72" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E72" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈에서 컨선 '좌초'…이란, "항로 이탈이 원인"</t>
+        </is>
+      </c>
+      <c r="F72" s="6" t="inlineStr"/>
+      <c r="G72" s="6" t="inlineStr"/>
+      <c r="H72" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈 해협을 통과하는 선박의 운항 상황을 즉시 확인하고, 해당 노선을 이용하는 물품의 운송 지연 가능성에 대비하여 비상 계획을 수립.</t>
+        </is>
+      </c>
+      <c r="I72" s="6" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="6" t="inlineStr">
+        <is>
+          <t>RSK-072</t>
+        </is>
+      </c>
+      <c r="B73" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C73" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D73" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E73" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 통행 수수료…오만, 이란과 공동징수 추진</t>
+        </is>
+      </c>
+      <c r="F73" s="6" t="inlineStr"/>
+      <c r="G73" s="6" t="inlineStr"/>
+      <c r="H73" s="6" t="inlineStr">
+        <is>
+          <t>중동발 원자재 및 제품 운송 경로 및 비용 영향 분석, 대체 운송 경로 및 공급처 검토, 장기 운송 계약 조건 재검토.</t>
+        </is>
+      </c>
+      <c r="I73" s="6" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="6" t="inlineStr">
+        <is>
+          <t>RSK-073</t>
+        </is>
+      </c>
+      <c r="B74" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C74" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D74" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E74" s="6" t="inlineStr">
+        <is>
+          <t>국제유가, 주말 호르무즈 무력공방에 상승…WTI 2%↑</t>
+        </is>
+      </c>
+      <c r="F74" s="6" t="inlineStr"/>
+      <c r="G74" s="6" t="inlineStr"/>
+      <c r="H74" s="6" t="inlineStr">
+        <is>
+          <t>유가 및 운임 변동 추이 면밀히 모니터링, 운송 계약 조건 재검토, 연료 효율 개선 방안 모색.</t>
+        </is>
+      </c>
+      <c r="I74" s="6" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="6" t="inlineStr">
+        <is>
+          <t>RSK-074</t>
+        </is>
+      </c>
+      <c r="B75" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C75" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D75" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E75" s="6" t="inlineStr">
+        <is>
+          <t>중동전쟁 장기화에 중소기업 피해 '962건'</t>
+        </is>
+      </c>
+      <c r="F75" s="6" t="inlineStr"/>
+      <c r="G75" s="6" t="inlineStr"/>
+      <c r="H75" s="6" t="inlineStr">
+        <is>
+          <t>중동발 공급망 리스크 재평가, 대체 운송 경로 및 운송사 확보, 재고 수준 조정 검토.</t>
+        </is>
+      </c>
+      <c r="I75" s="6" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="6" t="inlineStr">
+        <is>
+          <t>RSK-075</t>
+        </is>
+      </c>
+      <c r="B76" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C76" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D76" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E76" s="6" t="inlineStr">
+        <is>
+          <t>글로벌 해운운임, 9주 연속 상승…3200대 돌파</t>
+        </is>
+      </c>
+      <c r="F76" s="6" t="inlineStr"/>
+      <c r="G76" s="6" t="inlineStr"/>
+      <c r="H76" s="6" t="inlineStr">
+        <is>
+          <t>운송 계약 조건 재검토, 장기 운송 계약 협상, 운송 모드 전환 검토 (해당 시), 재고 최적화.</t>
+        </is>
+      </c>
+      <c r="I76" s="6" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="6" t="inlineStr">
+        <is>
+          <t>RSK-076</t>
+        </is>
+      </c>
+      <c r="B77" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C77" s="6" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="D77" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E77" s="6" t="inlineStr">
+        <is>
+          <t>EU, 2026~2028년 에너지 저장 45GW 로드맵 확정…한국 배터리·ESS 산업 수혜 기대 - 아이티인사이트</t>
+        </is>
+      </c>
+      <c r="F77" s="6" t="inlineStr"/>
+      <c r="G77" s="6" t="inlineStr"/>
+      <c r="H77" s="6" t="inlineStr">
+        <is>
+          <t>EU 시장의 예상 수요 증가에 맞춰 생산 계획을 조정하고, 유럽향 물류 네트워크 및 운송 역량을 선제적으로 확보하는 방안을 검토합니다.</t>
+        </is>
+      </c>
+      <c r="I77" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
📰 뉴스 데이터 2026-07-03_19:03
</commit_message>
<xml_diff>
--- a/data/SCM_물류_브리핑.xlsx
+++ b/data/SCM_물류_브리핑.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J463"/>
+  <dimension ref="A1:J519"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -22381,6 +22381,2606 @@
         </is>
       </c>
       <c r="J463" s="4" t="inlineStr"/>
+    </row>
+    <row r="464">
+      <c r="A464" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B464" s="2" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C464" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D464" s="2" t="inlineStr">
+        <is>
+          <t>CPSC Mandatory eFiling Takes Effect July 8; TPEB Rates Surge ~10% as Peak Season Demand Outpaces Capacity</t>
+        </is>
+      </c>
+      <c r="E464" s="2" t="inlineStr">
+        <is>
+          <t>7월 8일부터 CPSC 의무 전자 신고가 발효되고, CBP는 강제 노동 관련 통합 지침을 발표했으며, 성수기 수요가 공급을 초과하며 태평양 횡단 동향(TPEB) 운임이 약 10% 급등했다.</t>
+        </is>
+      </c>
+      <c r="F464" s="2" t="inlineStr">
+        <is>
+          <t>CPSC 의무 전자 신고는 미국 수출 제품의 규제 준수 절차에 직접적인 영향을 미치며, 강제 노동 지침은 공급망 실사에 중요하고, TPEB 운임 급등은 물류비 증가를 야기하므로 즉각적인 대응과 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G464" s="2" t="inlineStr">
+        <is>
+          <t>미국 수출 제품의 CPSC 전자 신고 의무 준수 여부 확인 및 준비, 공급망 내 강제 노동 리스크 점검, TPEB 운임 상승에 대한 운송 계획 재검토.</t>
+        </is>
+      </c>
+      <c r="H464" s="2" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I464" s="2" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/june-18-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J464" s="2" t="inlineStr">
+        <is>
+          <t>RSK-077</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B465" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C465" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D465" s="2" t="inlineStr">
+        <is>
+          <t>DOJ Appeals CIT's IEEPA Refund Injunction as CAPE Phase 2 Targets June 29; TPEB Rates Surge 30% Into Peak</t>
+        </is>
+      </c>
+      <c r="E465" s="2" t="inlineStr">
+        <is>
+          <t>법무부가 IEEPA 관세 환급 명령에 항소했으며 CAPE 2단계가 6월 29일 예정된 가운데, 성수기 진입으로 태평양 횡단 동향(TPEB) 운임이 30% 급등했다.</t>
+        </is>
+      </c>
+      <c r="F465" s="2" t="inlineStr">
+        <is>
+          <t>TPEB 운임의 30% 급등은 물류비에 상당한 부담을 줄 수 있어 즉각적인 대응이 필요하며, IEEPA 관세 환급 관련 법적 분쟁은 향후 관세 환급 가능성에 불확실성을 준다.</t>
+        </is>
+      </c>
+      <c r="G465" s="2" t="inlineStr">
+        <is>
+          <t>IEEPA 관세 환급 관련 진행 상황 주시, TPEB 노선 이용 시 운임 급등에 대비한 운송 계획 및 예산 재검토.</t>
+        </is>
+      </c>
+      <c r="H465" s="2" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I465" s="2" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/june-11-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J465" s="2" t="inlineStr">
+        <is>
+          <t>RSK-078</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B466" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C466" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D466" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 통행 수수료…오만, 이란과 공동징수 추진 및 중동 지정학 리스크 고조</t>
+        </is>
+      </c>
+      <c r="E466" s="2" t="inlineStr">
+        <is>
+          <t>오만과 이란이 호르무즈 해협 통행 수수료 공동 징수를 추진하고 미-이란 간 호르무즈 해협 통제권 쟁점 및 무력 공방으로 국제유가가 상승하는 등 중동 지역의 지정학적 리스크가 고조되고 있다.</t>
+        </is>
+      </c>
+      <c r="F466" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협은 주요 원유 및 가스 운송로이자 핵심 해상 운송로로, 통행 수수료 부과, 통제권 쟁점, 무력 공방 등 지정학적 불안정성은 해상 운임 및 유가에 직접적인 영향을 미쳐 우리 회사의 물류비용을 즉시 상승시키고 운송 지연을 야기할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G466" s="2" t="inlineStr">
+        <is>
+          <t>중동/유럽 항로 이용 시 지정학적 리스크 모니터링 강화, 운임 변동성 및 추가 비용 발생 가능성을 고려하여 운송 계획 및 예산 재검토, 비상 운송 계획 수립, 대체 운송 경로 또는 재고 전략 검토.</t>
+        </is>
+      </c>
+      <c r="H466" s="2" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I466" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260703-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J466" s="2" t="inlineStr">
+        <is>
+          <t>RSK-079</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B467" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C467" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D467" s="2" t="inlineStr">
+        <is>
+          <t>머스크, 운임·물동량 급등에 2026년 실적 가이던스 대폭 상향</t>
+        </is>
+      </c>
+      <c r="E467" s="2" t="inlineStr">
+        <is>
+          <t>머스크가 극동발 수요 강세와 스팟 운임 급등을 반영하여 2026년 연간 실적 가이던스를 대폭 상향 조정했으며, 이는 해상 운임의 지속적인 상승 추세를 시사한다.</t>
+        </is>
+      </c>
+      <c r="F467" s="2" t="inlineStr">
+        <is>
+          <t>주요 선사의 실적 가이던스 상향은 해상 운임의 지속적인 상승 추세를 반영하며, 이는 우리 회사의 물류비용에 직접적인 부담으로 작용할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G467" s="2" t="inlineStr">
+        <is>
+          <t>해상 운임 변동성 모니터링 강화, 장기 운송 계약 조건 재검토, 운송비 절감 방안 및 예산 재조정 검토.</t>
+        </is>
+      </c>
+      <c r="H467" s="2" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I467" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/vol130-주간-선사별-동향-week-27-2026</t>
+        </is>
+      </c>
+      <c r="J467" s="2" t="inlineStr">
+        <is>
+          <t>RSK-080</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B468" s="2" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C468" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D468" s="2" t="inlineStr">
+        <is>
+          <t>머스크, 중동 운항 신중 기조 유지…유럽 항만 지연 대응</t>
+        </is>
+      </c>
+      <c r="E468" s="2" t="inlineStr">
+        <is>
+          <t>머스크가 중동 운항에 신중한 기조를 유지하며 유럽 항만 지연에 대응하고 있어, 중동 및 유럽 항로의 서비스 안정성에 영향을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="F468" s="2" t="inlineStr">
+        <is>
+          <t>주요 선사의 중동 운항 신중 기조와 유럽 항만 지연 대응은 해당 항로의 선복량 감소, 운송 지연 및 운임 상승을 야기하여 우리 회사의 물류 운영에 직접적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G468" s="2" t="inlineStr">
+        <is>
+          <t>중동/유럽 항로 이용 시 선사별 서비스 안정성 및 운송 리드타임 변화 모니터링, 대체 운송 방안 및 재고 확보 전략 검토.</t>
+        </is>
+      </c>
+      <c r="H468" s="2" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I468" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/vol130-주간-선사별-동향-week-27-2026</t>
+        </is>
+      </c>
+      <c r="J468" s="2" t="inlineStr">
+        <is>
+          <t>RSK-081</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B469" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C469" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D469" s="2" t="inlineStr">
+        <is>
+          <t>종전 합의에도 안 꺾이는 '운임 폭탄'… 수출 중소기업 숨 막힌다</t>
+        </is>
+      </c>
+      <c r="E469" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 봉쇄가 해제되고 미-이란 종전 합의가 진행됨에도 불구하고 해상 운임은 여전히 높은 수준을 유지하고 있어 수출 중소기업들이 어려움을 겪고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F469" s="2" t="inlineStr">
+        <is>
+          <t>중동 사태 완화에도 불구하고 해상 운임이 높은 수준을 유지하는 것은 우리 회사의 해상 운송 비용 부담을 지속시키며, 이는 물류 예산 및 제품 원가에 직접적인 영향을 미칩니다.</t>
+        </is>
+      </c>
+      <c r="G469" s="2" t="inlineStr">
+        <is>
+          <t>장기 운송 계약 재협상, 선사 다변화, 운송 모드 전환 검토 등 해상 운임 상승에 대한 적극적인 비용 절감 및 리스크 관리 방안을 수립하고 실행해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H469" s="2" t="inlineStr">
+        <is>
+          <t>베타뉴스</t>
+        </is>
+      </c>
+      <c r="I469" s="2" t="inlineStr">
+        <is>
+          <t>https://betanews.net/article/view/beta202607020069</t>
+        </is>
+      </c>
+      <c r="J469" s="2" t="inlineStr">
+        <is>
+          <t>RSK-082</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B470" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C470" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D470" s="2" t="inlineStr">
+        <is>
+          <t>소비자물가 2년 6개월 만에 최대폭 상승···중동 전쟁 여파로 석유류 물가 상승 원인</t>
+        </is>
+      </c>
+      <c r="E470" s="2" t="inlineStr">
+        <is>
+          <t>중동 전쟁 여파로 국제 유가가 오르면서 석유류 물가가 4년 만에 최대 폭으로 상승했고, 이로 인해 소비자물가도 2년 6개월 만에 최대폭으로 올랐습니다.</t>
+        </is>
+      </c>
+      <c r="F470" s="2" t="inlineStr">
+        <is>
+          <t>중동 전쟁으로 인한 국제 유가 급등은 해상 및 항공 운임 상승으로 직결되어 우리 회사의 물류비용에 직접적인 부담을 주며, 생산 원가에도 영향을 미칩니다.</t>
+        </is>
+      </c>
+      <c r="G470" s="2" t="inlineStr">
+        <is>
+          <t>유가 변동에 따른 물류비 상승 리스크를 최소화하기 위해 유류할증료 변동 추이를 면밀히 분석하고, 운송 계약 재검토 및 대체 운송 수단 확보 등 비용 절감 방안을 적극적으로 모색해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H470" s="2" t="inlineStr">
+        <is>
+          <t>한국NGO신문</t>
+        </is>
+      </c>
+      <c r="I470" s="2" t="inlineStr">
+        <is>
+          <t>https://ngonews.kr/news/articleView.html?idxno=232095</t>
+        </is>
+      </c>
+      <c r="J470" s="2" t="inlineStr">
+        <is>
+          <t>RSK-083</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B471" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C471" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D471" s="3" t="inlineStr">
+        <is>
+          <t>주요 항공사들, 中東항공노선 점차 재개</t>
+        </is>
+      </c>
+      <c r="E471" s="3" t="inlineStr">
+        <is>
+          <t>중동 사태 진정 기미에 따라 캐세이퍼시픽 등 주요 항공사들이 중동 노선(리야드 화물, 두바이/리야드 여객) 운항을 8월 1일부터 점차 재개할 예정이다.</t>
+        </is>
+      </c>
+      <c r="F471" s="3" t="inlineStr">
+        <is>
+          <t>중동 노선 재개는 해당 지역으로의 항공 화물 운송 옵션이 확대되어 잠재적인 운송 지연 위험을 줄일 수 있으나, 우리 회사의 중동 지역 물류 비중과 실제 운임 영향은 추가 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G471" s="3" t="inlineStr">
+        <is>
+          <t>중동 지역으로의 항공 운송 계획이 있다면 항공사 스케줄 및 운임 변동 추이 확인.</t>
+        </is>
+      </c>
+      <c r="H471" s="3" t="inlineStr">
+        <is>
+          <t>cargonews</t>
+        </is>
+      </c>
+      <c r="I471" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cargonews.co.kr/news/articleView.html?idxno=60438</t>
+        </is>
+      </c>
+      <c r="J471" s="3" t="inlineStr"/>
+    </row>
+    <row r="472">
+      <c r="A472" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B472" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C472" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D472" s="3" t="inlineStr">
+        <is>
+          <t>U.S.-EU Trade Agreement Eliminates Duties on Most U.S. Goods Starting July 1; TPEB Rates Rise as July Capacity Hits Three-Year High</t>
+        </is>
+      </c>
+      <c r="E472" s="3" t="inlineStr">
+        <is>
+          <t>7월 1일부터 미국-EU 무역 협정이 발효되어 대부분의 미국산 공산품에 대한 관세가 철폐되며, 동시에 태평양 횡단 동향(TPEB) 운임이 상승하고 7월 선복량이 3년 내 최고치를 기록했다.</t>
+        </is>
+      </c>
+      <c r="F472" s="3" t="inlineStr">
+        <is>
+          <t>미국-EU 간 관세 철폐는 해당 지역으로의 수출입 비용에 긍정적 영향을 줄 수 있으나, 우리 회사의 주요 수출입 품목 및 지역에 대한 직접적인 영향은 확인이 필요하며, TPEB 운임 상승은 전체 물류비에 영향을 미칠 수 있어 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G472" s="3" t="inlineStr">
+        <is>
+          <t>미국-EU 간 수출입 품목 및 관세 혜택 여부 확인, TPEB 노선 이용 시 운임 변동 추이 주시.</t>
+        </is>
+      </c>
+      <c r="H472" s="3" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I472" s="3" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/july-02-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J472" s="3" t="inlineStr"/>
+    </row>
+    <row r="473">
+      <c r="A473" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B473" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C473" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D473" s="3" t="inlineStr">
+        <is>
+          <t>U.S. Appeals CIT's IEEPA Refund Order to Federal Circuit; TPEB Rates Rise as Peak Season Demand Tightens Capacity</t>
+        </is>
+      </c>
+      <c r="E473" s="3" t="inlineStr">
+        <is>
+          <t>미국 정부가 IEEPA 관세 환급 명령에 항소했으며, 트럼프 대통령이 세관 집행 강화를 위한 행정 명령에 서명했고, 성수기 수요로 태평양 횡단 동향(TPEB) 운임이 상승하고 있다.</t>
+        </is>
+      </c>
+      <c r="F473" s="3" t="inlineStr">
+        <is>
+          <t>IEEPA 관세 환급 관련 법적 분쟁은 불확실성을 높이고, 세관 집행 강화 행정 명령은 수입 절차 및 IOR 요건에 영향을 미칠 수 있어 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G473" s="3" t="inlineStr">
+        <is>
+          <t>IEEPA 관세 환급 진행 상황 및 세관 집행 강화에 따른 수입 요건 변화 주시, TPEB 운임 변동에 대한 대비.</t>
+        </is>
+      </c>
+      <c r="H473" s="3" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I473" s="3" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/june-3-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J473" s="3" t="inlineStr"/>
+    </row>
+    <row r="474">
+      <c r="A474" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B474" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C474" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D474" s="3" t="inlineStr">
+        <is>
+          <t>Air Cargo Demand Up 6.0% in May</t>
+        </is>
+      </c>
+      <c r="E474" s="3" t="inlineStr">
+        <is>
+          <t>2026년 5월 전 세계 항공 화물 수요가 전년 동월 대비 6.0% 증가했다.</t>
+        </is>
+      </c>
+      <c r="F474" s="3" t="inlineStr">
+        <is>
+          <t>항공 화물 수요 증가는 항공 운임 상승 압력 및 선복량 부족으로 이어질 수 있어, 우리 회사의 항공 운송 계획 및 비용에 잠재적 영향을 미칠 수 있으므로 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G474" s="3" t="inlineStr">
+        <is>
+          <t>항공 화물 운송 계획 시 선복 확보 및 운임 변동 추이 주시.</t>
+        </is>
+      </c>
+      <c r="H474" s="3" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I474" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-29-air-cargo-demand-up-may/</t>
+        </is>
+      </c>
+      <c r="J474" s="3" t="inlineStr"/>
+    </row>
+    <row r="475">
+      <c r="A475" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B475" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C475" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D475" s="3" t="inlineStr">
+        <is>
+          <t>[2026.7.3.] 중동 주간 정세 및 유가·물류 동향</t>
+        </is>
+      </c>
+      <c r="E475" s="3" t="inlineStr">
+        <is>
+          <t>코트라에서 중동 지역의 주간 정세와 유가 및 물류 동향에 대한 정보를 제공한다.</t>
+        </is>
+      </c>
+      <c r="F475" s="3" t="inlineStr">
+        <is>
+          <t>중동 정세는 유가 변동에 직접적인 영향을 미치고, 유가는 해상/항공 운임에 영향을 주므로, 우리 회사의 물류비에 잠재적 영향을 미칠 수 있어 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G475" s="3" t="inlineStr">
+        <is>
+          <t>중동 지역 정세 및 유가 변동 추이 주시, 물류비 영향 분석.</t>
+        </is>
+      </c>
+      <c r="H475" s="3" t="inlineStr">
+        <is>
+          <t>kotra</t>
+        </is>
+      </c>
+      <c r="I475" s="3" t="inlineStr">
+        <is>
+          <t>https://dream.kotra.or.kr/kotranews/cms/news/actionKotraBoardDetail.do?SITE_NO=3&amp;MENU_ID=70&amp;CONTENTS_NO=1&amp;pNttSn=242596</t>
+        </is>
+      </c>
+      <c r="J475" s="3" t="inlineStr"/>
+    </row>
+    <row r="476">
+      <c r="A476" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B476" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C476" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D476" s="3" t="inlineStr">
+        <is>
+          <t>PLSCI Data Indicates Mega-Hub Retrenchment</t>
+        </is>
+      </c>
+      <c r="E476" s="3" t="inlineStr">
+        <is>
+          <t>UNCTAD의 2026년 2분기 PLSCI 데이터 분석 결과, 메가 허브 항만 연결성 지수가 재조정되고 있어 해운 네트워크의 변화가 감지된다.</t>
+        </is>
+      </c>
+      <c r="F476" s="3" t="inlineStr">
+        <is>
+          <t>항만 연결성 변화는 장기적으로 특정 항만의 적체 또는 효율성에 영향을 줄 수 있으므로 추이를 모니터링하여 최적의 항로 및 항만 선택에 참고해야 한다.</t>
+        </is>
+      </c>
+      <c r="G476" s="3" t="n"/>
+      <c r="H476" s="3" t="inlineStr">
+        <is>
+          <t>sea-intelligence.com</t>
+        </is>
+      </c>
+      <c r="I476" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/396-plsci-data-indicates-mega-hub-retrenchment</t>
+        </is>
+      </c>
+      <c r="J476" s="3" t="inlineStr"/>
+    </row>
+    <row r="477">
+      <c r="A477" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B477" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C477" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D477" s="3" t="inlineStr">
+        <is>
+          <t>Tracking True Vessel Delay</t>
+        </is>
+      </c>
+      <c r="E477" s="3" t="inlineStr">
+        <is>
+          <t>선사들이 운송 시간을 늘리는 스케줄 버퍼링을 통해 선박의 조기 도착을 유도하고 있으며, 이는 실제 선박 지연과 관련하여 분석되었다.</t>
+        </is>
+      </c>
+      <c r="F477" s="3" t="inlineStr">
+        <is>
+          <t>선사들의 스케줄 버퍼링 전략은 겉으로 보이는 정시성 개선에도 불구하고 실제 운송 리드타임에 영향을 줄 수 있으므로, 운송 계획 수립 시 고려해야 한다.</t>
+        </is>
+      </c>
+      <c r="G477" s="3" t="n"/>
+      <c r="H477" s="3" t="inlineStr">
+        <is>
+          <t>sea-intelligence.com</t>
+        </is>
+      </c>
+      <c r="I477" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/394-tracking-true-vessel-delay</t>
+        </is>
+      </c>
+      <c r="J477" s="3" t="inlineStr"/>
+    </row>
+    <row r="478">
+      <c r="A478" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B478" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C478" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D478" s="3" t="inlineStr">
+        <is>
+          <t>Transpacific: Ripe for new non-alliance services</t>
+        </is>
+      </c>
+      <c r="E478" s="3" t="inlineStr">
+        <is>
+          <t>태평양 횡단 항로에서 컨테이너 스팟 운임과 비동맹 선사의 아시아-북미 서안 운송 비중 간의 관계를 분석한 결과, 새로운 비동맹 서비스의 출현 가능성이 높다.</t>
+        </is>
+      </c>
+      <c r="F478" s="3" t="inlineStr">
+        <is>
+          <t>새로운 비동맹 서비스의 출현은 태평양 횡단 항로의 운임 경쟁 심화 및 서비스 옵션 확대로 이어질 수 있어, 향후 운송 계약 전략에 영향을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="G478" s="3" t="n"/>
+      <c r="H478" s="3" t="inlineStr">
+        <is>
+          <t>sea-intelligence.com</t>
+        </is>
+      </c>
+      <c r="I478" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/393-transpacific-ripe-for-new-non-alliance-services</t>
+        </is>
+      </c>
+      <c r="J478" s="3" t="inlineStr"/>
+    </row>
+    <row r="479">
+      <c r="A479" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B479" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C479" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D479" s="3" t="inlineStr">
+        <is>
+          <t>Decoding Gemini’s Mediterranean Surge</t>
+        </is>
+      </c>
+      <c r="E479" s="3" t="inlineStr">
+        <is>
+          <t>Gemini Cooperation이 함대를 재배치하여 지중해 지역에 컨테이너 선박 배치를 늘리고 있으며, 이는 동서 컨테이너 선박 배치에 영향을 미친다.</t>
+        </is>
+      </c>
+      <c r="F479" s="3" t="inlineStr">
+        <is>
+          <t>주요 선사 얼라이언스의 함대 재배치는 특정 지역의 선복량 변화를 야기하여 해당 지역의 운임 및 서비스 가용성에 영향을 줄 수 있으므로, 지중해 관련 운송이 있다면 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G479" s="3" t="n"/>
+      <c r="H479" s="3" t="inlineStr">
+        <is>
+          <t>sea-intelligence.com</t>
+        </is>
+      </c>
+      <c r="I479" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/392-decoding-gemini-s-mediterranean-surge</t>
+        </is>
+      </c>
+      <c r="J479" s="3" t="inlineStr"/>
+    </row>
+    <row r="480">
+      <c r="A480" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B480" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C480" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D480" s="3" t="inlineStr">
+        <is>
+          <t>인천항 1만6000TEU급 시대 열었다</t>
+        </is>
+      </c>
+      <c r="E480" s="3" t="inlineStr">
+        <is>
+          <t>인천항에 1만6000TEU급 초대형 컨테이너선이 처음 투입되며 대형선 시대가 본격화되어 항만 처리 능력 및 효율성이 증대될 것으로 기대된다.</t>
+        </is>
+      </c>
+      <c r="F480" s="3" t="inlineStr">
+        <is>
+          <t>인천항의 대형선 시대 개막은 해당 항만을 이용하는 물류의 효율성 증대 및 운임 하락 가능성을 시사하므로, 인천항 이용 여부에 따라 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G480" s="3" t="inlineStr">
+        <is>
+          <t>인천항 이용 시 서비스 개선 여부 및 운임 변화 추이 모니터링.</t>
+        </is>
+      </c>
+      <c r="H480" s="3" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I480" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260702-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J480" s="3" t="inlineStr"/>
+    </row>
+    <row r="481">
+      <c r="A481" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B481" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C481" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D481" s="3" t="inlineStr">
+        <is>
+          <t>7월 LPG 판매가격 '소폭 인상'... kg당 50원</t>
+        </is>
+      </c>
+      <c r="E481" s="3" t="inlineStr">
+        <is>
+          <t>E1이 국제 LPG 가격, 운임, 환율 상승 요인을 반영하여 7월 LPG 판매가격을 kg당 50원 소폭 인상했다.</t>
+        </is>
+      </c>
+      <c r="F481" s="3" t="inlineStr">
+        <is>
+          <t>LPG 가격 인상은 운송 차량의 유류비에 영향을 주어 육상 운송비 상승으로 이어질 수 있으므로, 물류비용 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G481" s="3" t="n"/>
+      <c r="H481" s="3" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I481" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260701-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J481" s="3" t="inlineStr"/>
+    </row>
+    <row r="482">
+      <c r="A482" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B482" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C482" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D482" s="3" t="inlineStr">
+        <is>
+          <t>美, USMCA 연장 거부 방침… 북미 자유무역체제 ‘중대 분수령’</t>
+        </is>
+      </c>
+      <c r="E482" s="3" t="inlineStr">
+        <is>
+          <t>미국이 USMCA 연장 거부 방침을 밝히며 북미 자유무역체제가 중대 분수령을 맞이하여, 북미 지역 무역 환경의 불확실성이 증대되고 있다.</t>
+        </is>
+      </c>
+      <c r="F482" s="3" t="inlineStr">
+        <is>
+          <t>USMCA 연장 거부 방침은 북미 지역의 관세 및 무역 규제 변화를 야기하여 해당 지역으로의 수출입 물류 비용 및 절차에 영향을 줄 수 있으므로, 북미 시장 비중이 있다면 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G482" s="3" t="inlineStr">
+        <is>
+          <t>북미 시장으로의 수출입 비중이 높을 경우, 관세 및 무역 규제 변화 가능성 모니터링.</t>
+        </is>
+      </c>
+      <c r="H482" s="3" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I482" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260701-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J482" s="3" t="inlineStr"/>
+    </row>
+    <row r="483">
+      <c r="A483" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B483" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C483" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D483" s="3" t="inlineStr">
+        <is>
+          <t>우회덤핑 차단 공조…관세청·무역위 공동 대응</t>
+        </is>
+      </c>
+      <c r="E483" s="3" t="inlineStr">
+        <is>
+          <t>관세청과 무역위원회가 협의체를 통해 우회덤핑 감시 정보를 공유하고 무역구제 조치의 실효성 강화를 논의했다.</t>
+        </is>
+      </c>
+      <c r="F483" s="3" t="inlineStr">
+        <is>
+          <t>우회덤핑 차단 공조는 무역 규제 강화로 이어질 수 있으며, 이는 특정 품목의 수출입 절차 및 비용에 영향을 줄 수 있으므로 관련 품목이 있다면 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G483" s="3" t="inlineStr">
+        <is>
+          <t>수출입 품목 중 덤핑 규제 대상이 될 수 있는 품목이 있는지 확인하고 관련 규제 변화 모니터링.</t>
+        </is>
+      </c>
+      <c r="H483" s="3" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I483" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260630-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J483" s="3" t="inlineStr"/>
+    </row>
+    <row r="484">
+      <c r="A484" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B484" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C484" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D484" s="3" t="inlineStr">
+        <is>
+          <t>북극항로 시험운항 선박 '확보'…"8월 말 출항 유력"</t>
+        </is>
+      </c>
+      <c r="E484" s="3" t="inlineStr">
+        <is>
+          <t>해양수산부가 북극항로 시험 운항을 위한 내빙 컨테이너선 확보에 성공하여 8월 말 출항이 유력해졌다. 이는 새로운 해상 운송 경로 개발의 진전을 의미한다.</t>
+        </is>
+      </c>
+      <c r="F484" s="3" t="inlineStr">
+        <is>
+          <t>북극항로는 장기적으로 운송 시간 단축 및 비용 절감 가능성을 제공하지만, 현재는 시험 운항 단계로 즉각적인 영향은 없으므로 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G484" s="3" t="inlineStr">
+        <is>
+          <t>북극항로 개발 진행 상황 및 상업 운항 가능성을 지속적으로 모니터링하고, 우리 제품 운송에 적용 가능성을 검토.</t>
+        </is>
+      </c>
+      <c r="H484" s="3" t="inlineStr">
+        <is>
+          <t>해양통신</t>
+        </is>
+      </c>
+      <c r="I484" s="3" t="inlineStr">
+        <is>
+          <t>https://oceanpress.co.kr/news/article.html?no=30501</t>
+        </is>
+      </c>
+      <c r="J484" s="3" t="inlineStr"/>
+    </row>
+    <row r="485">
+      <c r="A485" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B485" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C485" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D485" s="3" t="inlineStr">
+        <is>
+          <t>Korea Zinc Moves to Cut Ore Dependence and Build an Independent Critical Materials Supply Chain</t>
+        </is>
+      </c>
+      <c r="E485" s="3" t="inlineStr">
+        <is>
+          <t>고려아연이 폐기물에서 핵심 소재를 추출하여 광석 의존도를 줄이고 독립적인 핵심 소재 공급망을 구축하려는 움직임을 보이고 있다. 이는 공급망 안정성 확보를 위한 전략적 변화이다.</t>
+        </is>
+      </c>
+      <c r="F485" s="3" t="inlineStr">
+        <is>
+          <t>핵심 소재 공급망 독립성 강화는 장기적인 공급 안정성에 긍정적 영향을 줄 수 있으나, 당사에는 직접적인 영향이 없으므로 관련 동향을 모니터링할 필요가 있다.</t>
+        </is>
+      </c>
+      <c r="G485" s="3" t="inlineStr">
+        <is>
+          <t>핵심 소재 공급망 다변화 및 재활용 소재 활용 가능성 등 공급망 안정화 전략을 검토.</t>
+        </is>
+      </c>
+      <c r="H485" s="3" t="inlineStr">
+        <is>
+          <t>인사이트코리아</t>
+        </is>
+      </c>
+      <c r="I485" s="3" t="inlineStr">
+        <is>
+          <t>https://www.insightkorea.co.kr/news/articleView.html?idxno=249515</t>
+        </is>
+      </c>
+      <c r="J485" s="3" t="inlineStr"/>
+    </row>
+    <row r="486">
+      <c r="A486" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B486" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C486" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D486" s="3" t="inlineStr">
+        <is>
+          <t>Asia Pacific Logistics Markets Diverge Despite 47% Tenant-Favourable Conditions as Supply Constraints Begin to Shift Balance</t>
+        </is>
+      </c>
+      <c r="E486" s="3" t="inlineStr">
+        <is>
+          <t>아시아 태평양 지역 물류 시장은 공급망 다변화와 생산 거점 이동으로 인해 베트남, 인도네시아, 태국 등 동남아시아가 주요 성장 허브로 부상하고 있다. 이는 현대적 물류 시설의 중요성을 강화하고 있다.</t>
+        </is>
+      </c>
+      <c r="F486" s="3" t="inlineStr">
+        <is>
+          <t>동남아시아로의 생산 거점 이동 및 공급망 다변화 추세는 당사의 생산 및 물류 네트워크 전략에 장기적인 영향을 미칠 수 있으므로 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G486" s="3" t="inlineStr">
+        <is>
+          <t>동남아시아 지역의 물류 인프라 및 잠재적 생산 거점으로서의 매력을 지속적으로 분석하고, 공급망 다변화 전략에 반영할 가능성을 검토.</t>
+        </is>
+      </c>
+      <c r="H486" s="3" t="inlineStr">
+        <is>
+          <t>The Manila Times</t>
+        </is>
+      </c>
+      <c r="I486" s="3" t="inlineStr">
+        <is>
+          <t>https://manilatimes.net/2026/07/03/tmt-newswire/media-outreach-newswire/asia-pacific-logistics-markets-diverge-despite-47-tenant-favourable-conditions-as-supply-constraints-begin-to-shift-balance/2377953</t>
+        </is>
+      </c>
+      <c r="J486" s="3" t="inlineStr"/>
+    </row>
+    <row r="487">
+      <c r="A487" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B487" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C487" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D487" s="3" t="inlineStr">
+        <is>
+          <t>EU, 2026~2028년 에너지 저장 45GW 로드맵 확정…한국 배터리·ESS 산업 수혜 기대</t>
+        </is>
+      </c>
+      <c r="E487" s="3" t="inlineStr">
+        <is>
+          <t>EU가 2026년부터 2028년까지 45GW의 에너지 저장 용량을 추가하는 로드맵을 확정하여 한국 배터리 및 ESS 산업에 긍정적인 영향을 미칠 것으로 기대된다. 이는 에너지 저장 시스템 시장의 성장을 의미한다.</t>
+        </is>
+      </c>
+      <c r="F487" s="3" t="inlineStr">
+        <is>
+          <t>EU의 에너지 저장 로드맵은 배터리 및 ESS 수요 증가로 이어져 당사의 생산 및 수출 전략에 긍정적인 영향을 줄 수 있으므로, 관련 시장 동향을 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G487" s="3" t="inlineStr">
+        <is>
+          <t>EU 시장의 배터리 및 ESS 수요 변화를 예측하고, 생산 및 수출 계획에 반영할 준비.</t>
+        </is>
+      </c>
+      <c r="H487" s="3" t="inlineStr">
+        <is>
+          <t>아이티인사이트</t>
+        </is>
+      </c>
+      <c r="I487" s="3" t="inlineStr">
+        <is>
+          <t>https://www.itinsight.kr/news/477698</t>
+        </is>
+      </c>
+      <c r="J487" s="3" t="inlineStr"/>
+    </row>
+    <row r="488">
+      <c r="A488" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B488" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C488" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D488" s="3" t="inlineStr">
+        <is>
+          <t>산업안전 위협하는 불법 반입·유통물품 대거 적발</t>
+        </is>
+      </c>
+      <c r="E488" s="3" t="inlineStr">
+        <is>
+          <t>관세청이 산업안전 물품의 불법 반입 및 원산지 둔갑 행위에 대한 집중 단속을 통해 1천220억원 상당의 위해물품을 적발했다. 이는 수입 물품에 대한 규제 강화 추세를 보여준다.</t>
+        </is>
+      </c>
+      <c r="F488" s="3" t="inlineStr">
+        <is>
+          <t>관세청의 불법 반입 및 원산지 위반 단속 강화는 당사의 수입/수출 절차 및 공급망 관리의 준수 사항에 대한 주의를 요구하므로 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G488" s="3" t="inlineStr">
+        <is>
+          <t>수입/수출 품목의 원산지 규정 준수 여부 및 안전 관련 인증 서류를 재점검하고, 통관 절차의 투명성을 강화.</t>
+        </is>
+      </c>
+      <c r="H488" s="3" t="inlineStr">
+        <is>
+          <t>한국세정신문</t>
+        </is>
+      </c>
+      <c r="I488" s="3" t="inlineStr">
+        <is>
+          <t>https://taxtimes.co.kr/news/article.html?no=275827</t>
+        </is>
+      </c>
+      <c r="J488" s="3" t="inlineStr"/>
+    </row>
+    <row r="489">
+      <c r="A489" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B489" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C489" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D489" s="3" t="inlineStr">
+        <is>
+          <t>118억 피해 키운 인천 공장 화재…“해법은 불연 단열재”[중기+]</t>
+        </is>
+      </c>
+      <c r="E489" s="3" t="inlineStr">
+        <is>
+          <t>인천 및 김포 물류창고 화재 발생으로 샌드위치 패널 내부 단열재를 불연재로 사용해야 한다는 목소리가 높아지고 있으며, 이는 창고 안전 규제 강화로 이어질 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="F489" s="3" t="inlineStr">
+        <is>
+          <t>물류창고 화재는 배터리/전자부품 보관에 대한 안전 규제 강화 논의로 이어질 수 있으며, 이는 향후 창고 운영 및 투자 계획에 영향을 줄 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G489" s="3" t="inlineStr">
+        <is>
+          <t>국내 물류창고의 화재 안전 규제 동향을 지속적으로 모니터링하고, 필요시 창고 시설 개선 및 안전 관리 강화 방안을 검토해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H489" s="3" t="inlineStr">
+        <is>
+          <t>헤럴드경제</t>
+        </is>
+      </c>
+      <c r="I489" s="3" t="inlineStr">
+        <is>
+          <t>https://biz.heraldcorp.com/article/10795421</t>
+        </is>
+      </c>
+      <c r="J489" s="3" t="inlineStr"/>
+    </row>
+    <row r="490">
+      <c r="A490" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B490" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C490" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D490" s="3" t="inlineStr">
+        <is>
+          <t>[AI로 읽는 경제] 미·이란 종전 국면…한국 산업 대응 방향은?</t>
+        </is>
+      </c>
+      <c r="E490" s="3" t="inlineStr">
+        <is>
+          <t>미-이란 종전 국면이 형성되면서 국제 유가 및 중동 지역 공급망 안정화에 대한 기대감이 커지고 있으며, 이는 한국 산업 전반에 긍정적인 영향을 미칠 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="F490" s="3" t="inlineStr">
+        <is>
+          <t>미-이란 종전은 국제 유가 하락 및 중동 지역 해상 운송 안정화로 이어져 물류비 절감 및 공급망 리스크 완화에 긍정적인 영향을 줄 수 있으므로 추이를 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G490" s="3" t="inlineStr">
+        <is>
+          <t>국제 유가 및 해상 운임 변동 추이를 면밀히 주시하고, 중동 지역 공급망 안정화에 따른 운송 계획 조정 가능성을 검토합니다.</t>
+        </is>
+      </c>
+      <c r="H490" s="3" t="inlineStr">
+        <is>
+          <t>뉴스핌</t>
+        </is>
+      </c>
+      <c r="I490" s="3" t="inlineStr">
+        <is>
+          <t>https://newspim.com/news/view/20260702000418</t>
+        </is>
+      </c>
+      <c r="J490" s="3" t="inlineStr"/>
+    </row>
+    <row r="491">
+      <c r="A491" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B491" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C491" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D491" s="3" t="inlineStr">
+        <is>
+          <t>“애플, 메모리 부족 사태에 중국산 구매 협상 중”</t>
+        </is>
+      </c>
+      <c r="E491" s="3" t="inlineStr">
+        <is>
+          <t>애플이 메모리 부족 사태 해결을 위해 중국 CXMT, YMTC와 구매 협상을 진행 중이며, 이는 미국 정부에 대한 로비와 함께 진행되고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F491" s="3" t="inlineStr">
+        <is>
+          <t>주요 전자제품 제조사의 공급망 다변화 노력은 글로벌 부품 공급망의 변화를 시사하며, 이는 향후 우리 회사의 고객사 및 경쟁 환경에 간접적인 영향을 줄 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G491" s="3" t="inlineStr">
+        <is>
+          <t>글로벌 전자부품 공급망의 변화 동향을 주시하고, 주요 고객사의 공급망 전략 변화가 우리 회사에 미칠 잠재적 영향을 분석합니다.</t>
+        </is>
+      </c>
+      <c r="H491" s="3" t="inlineStr">
+        <is>
+          <t>이투데이</t>
+        </is>
+      </c>
+      <c r="I491" s="3" t="inlineStr">
+        <is>
+          <t>https://etoday.co.kr/news/view/2599675</t>
+        </is>
+      </c>
+      <c r="J491" s="3" t="inlineStr"/>
+    </row>
+    <row r="492">
+      <c r="A492" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B492" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C492" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D492" s="3" t="inlineStr">
+        <is>
+          <t>연합뉴스TV</t>
+        </is>
+      </c>
+      <c r="E492" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 봉쇄 이후 홍해를 통해 원유를 운송하는 우리 선박이 증가했으며, 현재 1척이 사우디 얀부항에서 원유를 싣고 홍해를 거쳐 국내로 운항 중입니다.</t>
+        </is>
+      </c>
+      <c r="F492" s="3" t="inlineStr">
+        <is>
+          <t>중동 지역의 해상 운송 경로 변화는 유가 및 해상 운임에 영향을 미칠 수 있으며, 이는 우리 회사의 원자재 수급 및 제품 운송 비용에 간접적인 영향을 줄 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G492" s="3" t="inlineStr">
+        <is>
+          <t>중동 지역의 해상 운송 동향 및 국제 유가 변동을 지속적으로 모니터링하고, 필요시 운송 경로 및 비용 변화에 대한 대응 방안을 검토합니다.</t>
+        </is>
+      </c>
+      <c r="H492" s="3" t="inlineStr">
+        <is>
+          <t>연합뉴스TV</t>
+        </is>
+      </c>
+      <c r="I492" s="3" t="inlineStr">
+        <is>
+          <t>https://yonhapnewstv.co.kr/news/AKR202607021040527f7</t>
+        </is>
+      </c>
+      <c r="J492" s="3" t="inlineStr"/>
+    </row>
+    <row r="493">
+      <c r="A493" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B493" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C493" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D493" s="3" t="inlineStr">
+        <is>
+          <t>유류할증료 인하… 여름철 해외여행 수요 살아날까</t>
+        </is>
+      </c>
+      <c r="E493" s="3" t="inlineStr">
+        <is>
+          <t>중동 전쟁 영향으로 급등했던 유류할증료가 차츰 내림세를 보이면서 여름철 해외여행 수요가 살아날 것으로 기대되고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F493" s="3" t="inlineStr">
+        <is>
+          <t>유류할증료 인하는 항공 운송 비용 감소로 이어질 수 있으며, 이는 우리 회사의 항공 운송 물류비 절감에 긍정적인 영향을 줄 수 있으므로 추이를 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G493" s="3" t="inlineStr">
+        <is>
+          <t>항공 운송 유류할증료 변동 추이를 주시하고, 운임 하락 시 항공 운송 비중 조정 등 물류비 절감 방안을 검토합니다.</t>
+        </is>
+      </c>
+      <c r="H493" s="3" t="inlineStr">
+        <is>
+          <t>경인일보</t>
+        </is>
+      </c>
+      <c r="I493" s="3" t="inlineStr">
+        <is>
+          <t>https://kyeongin.com/article/1766688</t>
+        </is>
+      </c>
+      <c r="J493" s="3" t="inlineStr"/>
+    </row>
+    <row r="494">
+      <c r="A494" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B494" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C494" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D494" s="3" t="inlineStr">
+        <is>
+          <t>[단독] 장금마리타임-MSC 합병 두고… 공정위, 정유·해운사 의견조회</t>
+        </is>
+      </c>
+      <c r="E494" s="3" t="inlineStr">
+        <is>
+          <t>장금마리타임과 MSC의 합병 추진에 대해 공정거래위원회가 정유 및 해운사 의견을 조회하며 유조선 시장 독과점 여부를 조사하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F494" s="3" t="inlineStr">
+        <is>
+          <t>주요 해운사의 합병은 해상 운임 시장의 경쟁 구도에 영향을 미쳐 향후 운임 변동성 증가 또는 독과점 심화로 이어질 수 있으므로 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G494" s="3" t="inlineStr">
+        <is>
+          <t>해운 시장의 경쟁 환경 변화를 주시하고, 합병 승인 여부 및 그에 따른 운임 시장 영향을 분석하여 운송 전략에 반영할 준비를 합니다.</t>
+        </is>
+      </c>
+      <c r="H494" s="3" t="inlineStr">
+        <is>
+          <t>매일경제</t>
+        </is>
+      </c>
+      <c r="I494" s="3" t="inlineStr">
+        <is>
+          <t>https://mk.co.kr/news/business/12089119</t>
+        </is>
+      </c>
+      <c r="J494" s="3" t="inlineStr"/>
+    </row>
+    <row r="495">
+      <c r="A495" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B495" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C495" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D495" s="3" t="inlineStr">
+        <is>
+          <t>국제유가, 미·이란 종전협상 답보 속 강보합</t>
+        </is>
+      </c>
+      <c r="E495" s="3" t="inlineStr">
+        <is>
+          <t>미-이란 종전 협상이 답보 상태에 머물면서 국제 유가가 강보합세를 보이고 있으며, 이는 유가 하락에 대한 기대감을 낮추고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F495" s="3" t="inlineStr">
+        <is>
+          <t>국제 유가의 강보합세는 해상 및 항공 운송 비용에 지속적인 영향을 미치므로, 물류비 관리 측면에서 유가 동향을 면밀히 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G495" s="3" t="inlineStr">
+        <is>
+          <t>국제 유가 변동 추이를 지속적으로 주시하고, 유가 상승에 대비한 물류비 예산 관리 및 운송 계약 조건을 검토합니다.</t>
+        </is>
+      </c>
+      <c r="H495" s="3" t="inlineStr">
+        <is>
+          <t>한국경제</t>
+        </is>
+      </c>
+      <c r="I495" s="3" t="inlineStr">
+        <is>
+          <t>https://www.hankyung.com/article/2026070331437</t>
+        </is>
+      </c>
+      <c r="J495" s="3" t="inlineStr"/>
+    </row>
+    <row r="496">
+      <c r="A496" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B496" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C496" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D496" s="4" t="inlineStr">
+        <is>
+          <t>Air Passenger Demand Falls 2.2% in May</t>
+        </is>
+      </c>
+      <c r="E496" s="4" t="inlineStr">
+        <is>
+          <t>2026년 5월 전 세계 항공 여객 수요가 전년 동월 대비 2.2% 감소했다.</t>
+        </is>
+      </c>
+      <c r="F496" s="4" t="inlineStr">
+        <is>
+          <t>여객 수요 감소는 항공 화물 운송에 간접적인 영향을 줄 수 있으나, 다음 뉴스에서 화물 수요는 증가했다고 언급되어 상쇄되며 우리 회사의 항공 화물 운송에 직접적인 영향은 미미하다.</t>
+        </is>
+      </c>
+      <c r="G496" s="4" t="n"/>
+      <c r="H496" s="4" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I496" s="4" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-30-air-passenger-demand-falls-may/</t>
+        </is>
+      </c>
+      <c r="J496" s="4" t="inlineStr"/>
+    </row>
+    <row r="497">
+      <c r="A497" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B497" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C497" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D497" s="4" t="inlineStr">
+        <is>
+          <t>IATA and IATP Collaborate to Support Airline Supply Chain Resilience</t>
+        </is>
+      </c>
+      <c r="E497" s="4" t="inlineStr">
+        <is>
+          <t>IATA와 IATP가 항공기 부품 가시성 및 접근성 개선을 위해 협력하여 항공사 공급망 복원력을 지원하기로 합의했다.</t>
+        </is>
+      </c>
+      <c r="F497" s="4" t="inlineStr">
+        <is>
+          <t>항공사 자체의 부품 공급망 개선에 관한 내용으로, 우리 회사의 배터리/전자부품 물류 운영에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G497" s="4" t="n"/>
+      <c r="H497" s="4" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I497" s="4" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-25-iata-iatp-collaborate-support-airline-supply-chain-resilience/</t>
+        </is>
+      </c>
+      <c r="J497" s="4" t="inlineStr"/>
+    </row>
+    <row r="498">
+      <c r="A498" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B498" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C498" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D498" s="4" t="inlineStr">
+        <is>
+          <t>Urgent Action Needed to Ease Engine MRO Bottlenecks</t>
+        </is>
+      </c>
+      <c r="E498" s="4" t="inlineStr">
+        <is>
+          <t>IATA는 항공기 엔진 유지보수(MRO) 병목 현상 완화를 위한 긴급 조치가 필요하다고 강조했다.</t>
+        </is>
+      </c>
+      <c r="F498" s="4" t="inlineStr">
+        <is>
+          <t>항공기 엔진 MRO 병목 현상은 항공기 가동률에 영향을 미쳐 간접적으로 항공 화물 선복량에 영향을 줄 수 있으나, 현재로서는 우리 회사의 물류 운영에 직접적인 영향은 낮다.</t>
+        </is>
+      </c>
+      <c r="G498" s="4" t="n"/>
+      <c r="H498" s="4" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I498" s="4" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-24-urgent-action-needed-to-ease-engine-mro-bottlenecks/</t>
+        </is>
+      </c>
+      <c r="J498" s="4" t="inlineStr"/>
+    </row>
+    <row r="499">
+      <c r="A499" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B499" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C499" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D499" s="4" t="inlineStr">
+        <is>
+          <t>IATA Outlines Four Priorities to Strengthen the Aviation Supply Chain</t>
+        </is>
+      </c>
+      <c r="E499" s="4" t="inlineStr">
+        <is>
+          <t>IATA는 항공 공급망 강화를 위한 네 가지 우선순위(예측 개선, 인력 확보, 디지털화, 지속가능성)를 제시했다.</t>
+        </is>
+      </c>
+      <c r="F499" s="4" t="inlineStr">
+        <is>
+          <t>항공 산업 전반의 공급망 개선 노력에 대한 내용으로, 장기적으로 항공 화물 서비스 품질에 긍정적 영향을 줄 수 있으나, 우리 회사의 물류 운영에 당장 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G499" s="4" t="n"/>
+      <c r="H499" s="4" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I499" s="4" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-24-iata-outlines-four-priorities-to-strengthen-aviation-supply-chain/</t>
+        </is>
+      </c>
+      <c r="J499" s="4" t="inlineStr"/>
+    </row>
+    <row r="500">
+      <c r="A500" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B500" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C500" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D500" s="4" t="inlineStr">
+        <is>
+          <t>"올 상반기 韓 선주들이 중고 유조선 매입 1위"</t>
+        </is>
+      </c>
+      <c r="E500" s="4" t="inlineStr">
+        <is>
+          <t>올해 상반기 한국 선주들이 중고 유조선 매입에서 세계 1위를 기록했으며, 유조선 및 벌크선 신조 및 중고 거래가 크게 증가했다.</t>
+        </is>
+      </c>
+      <c r="F500" s="4" t="inlineStr">
+        <is>
+          <t>유조선 및 벌크선 시장 동향은 주로 원유, 곡물 등 벌크 화물 운송에 영향을 미치며, 우리 회사의 배터리/전자부품 컨테이너 운송에는 직접적인 영향이 낮다.</t>
+        </is>
+      </c>
+      <c r="G500" s="4" t="n"/>
+      <c r="H500" s="4" t="inlineStr">
+        <is>
+          <t>kita</t>
+        </is>
+      </c>
+      <c r="I500" s="4" t="inlineStr">
+        <is>
+          <t>https://www.kita.net/shippers/board/newsView.do?morgueCode=2&amp;dataCls=B&amp;dataSeq=8149</t>
+        </is>
+      </c>
+      <c r="J500" s="4" t="inlineStr"/>
+    </row>
+    <row r="501">
+      <c r="A501" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B501" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C501" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D501" s="4" t="inlineStr">
+        <is>
+          <t>한국선급, 신임 유럽委 의장에 빔코 아론 쇠렌센 선임</t>
+        </is>
+      </c>
+      <c r="E501" s="4" t="inlineStr">
+        <is>
+          <t>한국선급(KR)이 제21차 유럽위원회를 개최하고 빔코 아론 쇠렌센을 신임 유럽위원회 의장으로 선임했으며, AI 기반 탈탄소화 및 디지털 전환 연구 성과 등을 공유했다.</t>
+        </is>
+      </c>
+      <c r="F501" s="4" t="inlineStr">
+        <is>
+          <t>선급의 인사이동 및 기술 동향 공유는 장기적으로 해운 산업의 안전 및 효율성에 영향을 줄 수 있으나, 우리 회사의 물류 운영에 당장 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G501" s="4" t="n"/>
+      <c r="H501" s="4" t="inlineStr">
+        <is>
+          <t>ksg</t>
+        </is>
+      </c>
+      <c r="I501" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksg.co.kr/news/main_newsView.jsp?pNum=147552</t>
+        </is>
+      </c>
+      <c r="J501" s="4" t="inlineStr"/>
+    </row>
+    <row r="502">
+      <c r="A502" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B502" s="4" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C502" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D502" s="4" t="inlineStr">
+        <is>
+          <t>BPA, 항만 내 불법드론 원천봉쇄를 위한 안티드론 시스템 본격 가동</t>
+        </is>
+      </c>
+      <c r="E502" s="4" t="inlineStr">
+        <is>
+          <t>부산항만공사(BPA)가 7월 1일부터 부산항의 불법 드론 위협을 방지하고 항만 운영의 안전성을 확보하기 위한 '무역항 안티드론 시스템'을 본격 가동한다.</t>
+        </is>
+      </c>
+      <c r="F502" s="4" t="inlineStr">
+        <is>
+          <t>부산항의 보안 강화는 항만 운영의 안정성을 높여 장기적으로 긍정적이나, 우리 회사의 물류 운영에 당장 직접적인 영향은 낮다.</t>
+        </is>
+      </c>
+      <c r="G502" s="4" t="n"/>
+      <c r="H502" s="4" t="inlineStr">
+        <is>
+          <t>oceanpress</t>
+        </is>
+      </c>
+      <c r="I502" s="4" t="inlineStr">
+        <is>
+          <t>https://www.oceanpress.co.kr/news/article.html?no=30516</t>
+        </is>
+      </c>
+      <c r="J502" s="4" t="inlineStr"/>
+    </row>
+    <row r="503">
+      <c r="A503" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B503" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C503" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D503" s="4" t="inlineStr">
+        <is>
+          <t>Global Schedule Reliability for May 2026 the Highest of the Year</t>
+        </is>
+      </c>
+      <c r="E503" s="4" t="inlineStr">
+        <is>
+          <t>2026년 5월 글로벌 선박 스케줄 신뢰도가 올해 최고치를 기록하여 해상 운송의 정시성이 개선되고 있음을 나타낸다.</t>
+        </is>
+      </c>
+      <c r="F503" s="4" t="inlineStr">
+        <is>
+          <t>스케줄 신뢰도 개선은 긍정적인 신호이나, 일시적인 개선일 수 있으며 우리 회사의 특정 항로에 대한 직접적인 영향은 아직 미미하다.</t>
+        </is>
+      </c>
+      <c r="G503" s="4" t="n"/>
+      <c r="H503" s="4" t="inlineStr">
+        <is>
+          <t>sea-intelligence.com</t>
+        </is>
+      </c>
+      <c r="I503" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/395-global-schedule-reliability-for-may-2026-the-highest-of-the-year</t>
+        </is>
+      </c>
+      <c r="J503" s="4" t="inlineStr"/>
+    </row>
+    <row r="504">
+      <c r="A504" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B504" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C504" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D504" s="4" t="inlineStr">
+        <is>
+          <t>KR, 제 21차 유럽위원회 성료</t>
+        </is>
+      </c>
+      <c r="E504" s="4" t="inlineStr">
+        <is>
+          <t>한국선급(KR)이 유럽 해사업계 인사들과 기술 교류 및 네트워크 강화를 위한 제21차 유럽위원회를 성공적으로 개최했다.</t>
+        </is>
+      </c>
+      <c r="F504" s="4" t="inlineStr">
+        <is>
+          <t>해사업계의 기술 교류 및 네트워크 강화는 장기적으로 산업 발전에 기여하나, 우리 회사의 단기적인 물류 운영에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G504" s="4" t="n"/>
+      <c r="H504" s="4" t="inlineStr">
+        <is>
+          <t>shippingnewsnet.com</t>
+        </is>
+      </c>
+      <c r="I504" s="4" t="inlineStr">
+        <is>
+          <t>https://www.shippingnewsnet.com/news/articleView.html?idxno=71021</t>
+        </is>
+      </c>
+      <c r="J504" s="4" t="inlineStr"/>
+    </row>
+    <row r="505">
+      <c r="A505" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B505" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C505" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D505" s="4" t="inlineStr">
+        <is>
+          <t>마스오토 "부산항까지 트레일러 자율주행…2028년 화물 완전 무인화"</t>
+        </is>
+      </c>
+      <c r="E505" s="4" t="inlineStr">
+        <is>
+          <t>마스오토가 부산항을 거점으로 트레일러 자율주행 상용화를 추진하며 2028년 화물 운송의 완전 무인화를 목표로 제시했다.</t>
+        </is>
+      </c>
+      <c r="F505" s="4" t="inlineStr">
+        <is>
+          <t>자율주행 트레일러는 미래 물류 혁신 기술이나, 2028년 상용화 목표로 당장 우리 회사의 물류 운영에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G505" s="4" t="n"/>
+      <c r="H505" s="4" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I505" s="4" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260703-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J505" s="4" t="inlineStr"/>
+    </row>
+    <row r="506">
+      <c r="A506" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B506" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C506" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D506" s="4" t="inlineStr">
+        <is>
+          <t>머스크, 브라질 북동부 수아페항 투자 확대…남미 물류 거점 육성</t>
+        </is>
+      </c>
+      <c r="E506" s="4" t="inlineStr">
+        <is>
+          <t>머스크가 브라질 북동부 수아페항 투자를 확대하여 남미 공급망의 전략 거점을 확보하고 복합물류망을 확충할 계획이다.</t>
+        </is>
+      </c>
+      <c r="F506" s="4" t="inlineStr">
+        <is>
+          <t>머스크의 남미 물류 거점 투자는 해당 지역의 물류 효율성 개선에 기여할 수 있으나, 우리 회사의 현재 물류 운영에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G506" s="4" t="n"/>
+      <c r="H506" s="4" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I506" s="4" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/vol130-주간-선사별-동향-week-27-2026</t>
+        </is>
+      </c>
+      <c r="J506" s="4" t="inlineStr"/>
+    </row>
+    <row r="507">
+      <c r="A507" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B507" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C507" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D507" s="4" t="inlineStr">
+        <is>
+          <t>55GW 규모 해상풍력 건설 로드맵 나왔다</t>
+        </is>
+      </c>
+      <c r="E507" s="4" t="inlineStr">
+        <is>
+          <t>향후 10년간 55GW 규모의 해상풍력 건설 로드맵이 제시되며 하부구조물, 케이블, 항만, 설치 선박 등 공급망 투자 필요성이 부각되었다.</t>
+        </is>
+      </c>
+      <c r="F507" s="4" t="inlineStr">
+        <is>
+          <t>해상풍력 공급망 투자는 특정 산업 분야의 물류 인프라 발전에 기여하나, 우리 회사의 배터리/전자부품 물류 운영에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G507" s="4" t="n"/>
+      <c r="H507" s="4" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I507" s="4" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260701-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J507" s="4" t="inlineStr"/>
+    </row>
+    <row r="508">
+      <c r="A508" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B508" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C508" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D508" s="4" t="inlineStr">
+        <is>
+          <t>미래산업, 아산 신공장 145억에 인수…생산능력 2.8배 ↑</t>
+        </is>
+      </c>
+      <c r="E508" s="4" t="inlineStr">
+        <is>
+          <t>미래산업이 아산 신공장을 인수하여 기존 생산체계와의 통합을 통해 생산능력을 2.8배 확대할 계획이다.</t>
+        </is>
+      </c>
+      <c r="F508" s="4" t="inlineStr">
+        <is>
+          <t>특정 기업의 생산능력 확대는 해당 기업의 공급망에 영향을 주지만, 우리 회사의 물류 운영에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G508" s="4" t="n"/>
+      <c r="H508" s="4" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I508" s="4" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260630-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J508" s="4" t="inlineStr"/>
+    </row>
+    <row r="509">
+      <c r="A509" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B509" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C509" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D509" s="4" t="inlineStr">
+        <is>
+          <t>씨메스로보틱스 / ‘물류·제조 대형 수주 잇달아’ 피지컬 AI 기반 로봇 자동화 사업 가속</t>
+        </is>
+      </c>
+      <c r="E509" s="4" t="inlineStr">
+        <is>
+          <t>씨메스로보틱스가 쿠팡풀필먼트서비스 등 물류 및 제조 현장에서 대형 로봇 자동화 프로젝트를 연이어 수주하며 피지컬 AI 기반 로봇 자동화 사업을 확대하고 있다.</t>
+        </is>
+      </c>
+      <c r="F509" s="4" t="inlineStr">
+        <is>
+          <t>물류 로봇 자동화 기술 발전은 장기적으로 물류 효율성 향상에 기여하나, 우리 회사의 현재 물류 운영에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G509" s="4" t="n"/>
+      <c r="H509" s="4" t="inlineStr">
+        <is>
+          <t>ulogistics.co.kr</t>
+        </is>
+      </c>
+      <c r="I509" s="4" t="inlineStr">
+        <is>
+          <t>http://www.ulogistics.co.kr/test/board.php?board=all2&amp;command=body&amp;no=5202</t>
+        </is>
+      </c>
+      <c r="J509" s="4" t="inlineStr"/>
+    </row>
+    <row r="510">
+      <c r="A510" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B510" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C510" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D510" s="4" t="inlineStr">
+        <is>
+          <t>삼성중공업, 쿠옥그룹과 조선·해양·디지털 인프라 협력</t>
+        </is>
+      </c>
+      <c r="E510" s="4" t="inlineStr">
+        <is>
+          <t>삼성중공업이 싱가포르 쿠옥그룹과 조선, 해양, 디지털 인프라 등 사업 협력을 확대하여 유연한 생산 체계와 미래 사업을 강화한다.</t>
+        </is>
+      </c>
+      <c r="F510" s="4" t="inlineStr">
+        <is>
+          <t>조선 및 해양 산업의 협력 확대는 장기적인 산업 발전에 기여하나, 우리 회사의 단기적인 물류 운영에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G510" s="4" t="n"/>
+      <c r="H510" s="4" t="inlineStr">
+        <is>
+          <t>newspim.com</t>
+        </is>
+      </c>
+      <c r="I510" s="4" t="inlineStr">
+        <is>
+          <t>https://www.newspim.com/news/view/20260702001026</t>
+        </is>
+      </c>
+      <c r="J510" s="4" t="inlineStr"/>
+    </row>
+    <row r="511">
+      <c r="A511" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B511" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C511" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D511" s="4" t="inlineStr">
+        <is>
+          <t>[현장] 폴스타코리아, ‘폴스타 3’ 글로벌 대비 2년 지연 출시에 숨은 ‘소비자 신뢰’의 가치</t>
+        </is>
+      </c>
+      <c r="E511" s="4" t="inlineStr">
+        <is>
+          <t>폴스타코리아가 플래그십 SUV '폴스타 3'를 글로벌 시장보다 2년 늦게 국내 출시했으며, 이는 단기 실적보다 소비자 신뢰를 중시한 결정이다.</t>
+        </is>
+      </c>
+      <c r="F511" s="4" t="inlineStr">
+        <is>
+          <t>특정 기업의 제품 출시 지연은 해당 기업의 마케팅 및 판매 전략과 관련되며, 우리 회사의 물류 운영에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G511" s="4" t="n"/>
+      <c r="H511" s="4" t="inlineStr">
+        <is>
+          <t>consumerwide.com</t>
+        </is>
+      </c>
+      <c r="I511" s="4" t="inlineStr">
+        <is>
+          <t>https://www.consumerwide.com/news/articleView.html?idxno=66441</t>
+        </is>
+      </c>
+      <c r="J511" s="4" t="inlineStr"/>
+    </row>
+    <row r="512">
+      <c r="A512" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B512" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C512" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D512" s="4" t="inlineStr">
+        <is>
+          <t>America at 250: How US Logistics Reinvented the Supply Chain</t>
+        </is>
+      </c>
+      <c r="E512" s="4" t="inlineStr">
+        <is>
+          <t>미국 물류 기업들이 재고 위치, 이동 방식, 그리고 공급망 중단에 대한 대응 속도를 재설계하며 공급망을 혁신하고 있다. 이는 단일 기술 돌파구보다는 전반적인 시스템 개선에 초점을 맞추고 있다.</t>
+        </is>
+      </c>
+      <c r="F512" s="4" t="inlineStr">
+        <is>
+          <t>미국 물류 시장의 전반적인 공급망 재설계 동향은 참고할 만하지만, 당사의 즉각적인 물류 운영에 직접적인 영향을 미치지는 않는다.</t>
+        </is>
+      </c>
+      <c r="G512" s="4" t="n"/>
+      <c r="H512" s="4" t="inlineStr">
+        <is>
+          <t>WWD</t>
+        </is>
+      </c>
+      <c r="I512" s="4" t="inlineStr">
+        <is>
+          <t>https://wwd.com/sourcing-journal/logistics/america-at-250-us-logistics-3pl-fulfillment-last-mile-delivery-returns-1239051063/</t>
+        </is>
+      </c>
+      <c r="J512" s="4" t="inlineStr"/>
+    </row>
+    <row r="513">
+      <c r="A513" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B513" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C513" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D513" s="4" t="inlineStr">
+        <is>
+          <t>작고 힘센 韓 배터리, 전기차선 中에 밀렸지만 로봇은 압도</t>
+        </is>
+      </c>
+      <c r="E513" s="4" t="inlineStr">
+        <is>
+          <t>한국 배터리 기업들이 전기차 시장에서는 중국에 밀리지만, 로봇 분야에서는 초경량·고출력 배터리 기술로 압도적인 경쟁력을 보이고 있다. LG에너지솔루션이 주요 로봇 기업에 납품 승인을 받았다.</t>
+        </is>
+      </c>
+      <c r="F513" s="4" t="inlineStr">
+        <is>
+          <t>한국 배터리 기술의 로봇 시장 경쟁력 강화는 당사의 제품 개발 및 시장 전략에 긍정적인 참고 자료가 될 수 있으나, 물류 운영에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G513" s="4" t="n"/>
+      <c r="H513" s="4" t="inlineStr">
+        <is>
+          <t>한국경제</t>
+        </is>
+      </c>
+      <c r="I513" s="4" t="inlineStr">
+        <is>
+          <t>https://hankyung.com/article/2026070227441</t>
+        </is>
+      </c>
+      <c r="J513" s="4" t="inlineStr"/>
+    </row>
+    <row r="514">
+      <c r="A514" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B514" s="4" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C514" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D514" s="4" t="inlineStr">
+        <is>
+          <t>진안소방서, '제3회 위험물 안전관리 우수사례 경진대회’ 홍보</t>
+        </is>
+      </c>
+      <c r="E514" s="4" t="inlineStr">
+        <is>
+          <t>진안소방서가 소방청 주관 '제3회 위험물 안전관리 우수사례 경진대회' 참여를 독려하고 있으며, 이는 위험물 현장 안전관리의 중요성을 강조한다.</t>
+        </is>
+      </c>
+      <c r="F514" s="4" t="inlineStr">
+        <is>
+          <t>위험물 안전관리 우수사례 경진대회 홍보는 일반적인 안전 관리의 중요성을 상기시키지만, 당사의 물류 운영에 즉각적인 규제 변경이나 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G514" s="4" t="n"/>
+      <c r="H514" s="4" t="inlineStr">
+        <is>
+          <t>무진장인터넷뉴스</t>
+        </is>
+      </c>
+      <c r="I514" s="4" t="inlineStr">
+        <is>
+          <t>https://www.mjjnews.net/news/article.html?no=57632</t>
+        </is>
+      </c>
+      <c r="J514" s="4" t="inlineStr"/>
+    </row>
+    <row r="515">
+      <c r="A515" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B515" s="4" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C515" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D515" s="4" t="inlineStr">
+        <is>
+          <t>우체국물류지원단, 전국 작업장 대상 집중안전점검 실시...위험요인 개선</t>
+        </is>
+      </c>
+      <c r="E515" s="4" t="inlineStr">
+        <is>
+          <t>우체국물류지원단이 산업재해 예방 및 안전한 작업환경 조성을 위해 전국 주요 사업장을 대상으로 집중 안전점검을 실시하고 위험요인을 개선하고 있다. 이는 물류 작업장의 안전 관리 강화 추세를 보여준다.</t>
+        </is>
+      </c>
+      <c r="F515" s="4" t="inlineStr">
+        <is>
+          <t>우체국물류지원단의 안전점검은 물류 산업 전반의 안전 관리 중요성을 보여주지만, 당사의 물류 운영에 직접적인 규제 변경이나 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G515" s="4" t="n"/>
+      <c r="H515" s="4" t="inlineStr">
+        <is>
+          <t>IDSN</t>
+        </is>
+      </c>
+      <c r="I515" s="4" t="inlineStr">
+        <is>
+          <t>https://idsn.co.kr/news/view/1065572839637120</t>
+        </is>
+      </c>
+      <c r="J515" s="4" t="inlineStr"/>
+    </row>
+    <row r="516">
+      <c r="A516" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B516" s="4" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C516" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D516" s="4" t="inlineStr">
+        <is>
+          <t>미국, 멕시코·캐나다와 북미무역협정 연장 거부...매년 재검토 방침 [종합]</t>
+        </is>
+      </c>
+      <c r="E516" s="4" t="inlineStr">
+        <is>
+          <t>미국이 멕시코, 캐나다와의 북미무역협정(USMCA) 16년 연장 제안을 거부하고 매년 재검토 방침을 밝히면서, 향후 북미 지역 무역 환경의 불확실성이 커지고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F516" s="4" t="inlineStr">
+        <is>
+          <t>북미무역협정 재검토는 북미 지역 내 무역 환경에 영향을 미치지만, 우리 회사의 주요 생산 및 판매 거점과는 직접적인 관련이 적어 당장 큰 영향은 없습니다.</t>
+        </is>
+      </c>
+      <c r="G516" s="4" t="n"/>
+      <c r="H516" s="4" t="inlineStr">
+        <is>
+          <t>이투데이</t>
+        </is>
+      </c>
+      <c r="I516" s="4" t="inlineStr">
+        <is>
+          <t>https://etoday.co.kr/news/view/2599620</t>
+        </is>
+      </c>
+      <c r="J516" s="4" t="inlineStr"/>
+    </row>
+    <row r="517">
+      <c r="A517" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B517" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C517" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D517" s="4" t="inlineStr">
+        <is>
+          <t>삼성·SK하닉, 충청권에 240조 투자…HBM·첨단소재 거점 키운다</t>
+        </is>
+      </c>
+      <c r="E517" s="4" t="inlineStr">
+        <is>
+          <t>삼성과 SK하이닉스가 충청권에 240조원을 투자하여 반도체, 디스플레이, 배터리 등 미래 산업 생산기지를 확대할 계획이며, 정부도 이를 지원할 예정입니다.</t>
+        </is>
+      </c>
+      <c r="F517" s="4" t="inlineStr">
+        <is>
+          <t>국내 주요 고객사의 생산 거점 확대는 장기적으로 국내 물류 수요 증가 및 공급망 안정화에 기여할 수 있으나, 당장 우리 회사의 물류 운영에 직접적인 영향은 없습니다.</t>
+        </is>
+      </c>
+      <c r="G517" s="4" t="n"/>
+      <c r="H517" s="4" t="inlineStr">
+        <is>
+          <t>겟뉴스</t>
+        </is>
+      </c>
+      <c r="I517" s="4" t="inlineStr">
+        <is>
+          <t>https://www.getnews.co.kr/news/articleView.html?idxno=873948</t>
+        </is>
+      </c>
+      <c r="J517" s="4" t="inlineStr"/>
+    </row>
+    <row r="518">
+      <c r="A518" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B518" s="4" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C518" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D518" s="4" t="inlineStr">
+        <is>
+          <t>반도체 수출 사상 최대에도…삼성전자·SK하이닉스 덮친 해외발 경고</t>
+        </is>
+      </c>
+      <c r="E518" s="4" t="inlineStr">
+        <is>
+          <t>지난달 반도체 수출이 사상 최고치를 경신했음에도 불구하고, 삼성전자와 SK하이닉스 주가가 해외발 부정적인 평가로 흔들리고 있어 국내 반도체 산업의 불확실성이 커지고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F518" s="4" t="inlineStr">
+        <is>
+          <t>주요 고객사의 주가 변동은 간접적인 시장 지표이지만, 당장 우리 회사의 배터리/전자부품 물류 운영에 직접적인 영향을 미치지는 않습니다.</t>
+        </is>
+      </c>
+      <c r="G518" s="4" t="n"/>
+      <c r="H518" s="4" t="inlineStr">
+        <is>
+          <t>더퍼블릭</t>
+        </is>
+      </c>
+      <c r="I518" s="4" t="inlineStr">
+        <is>
+          <t>https://thepublic.kr/news/articleView.html?idxno=309848</t>
+        </is>
+      </c>
+      <c r="J518" s="4" t="inlineStr"/>
+    </row>
+    <row r="519">
+      <c r="A519" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B519" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C519" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D519" s="4" t="inlineStr">
+        <is>
+          <t>글로벌 공급망 파고드는 ‘K-방산’</t>
+        </is>
+      </c>
+      <c r="E519" s="4" t="inlineStr">
+        <is>
+          <t>K-방산이 대기업 중심의 완제품 수출을 넘어 글로벌 밸류체인 중심으로 재편되고 있으며, 해외 무기체계 도입 시 국산 부품 수출이나 기술 이전을 요구하는 추세입니다.</t>
+        </is>
+      </c>
+      <c r="F519" s="4" t="inlineStr">
+        <is>
+          <t>방산 산업의 공급망 변화는 우리 회사의 배터리/전자부품 물류 운영과는 직접적인 관련이 없어 당장 영향은 없습니다.</t>
+        </is>
+      </c>
+      <c r="G519" s="4" t="n"/>
+      <c r="H519" s="4" t="inlineStr">
+        <is>
+          <t>아시아투데이</t>
+        </is>
+      </c>
+      <c r="I519" s="4" t="inlineStr">
+        <is>
+          <t>https://asiatoday.co.kr/kn/view.php?key=20260702010000915</t>
+        </is>
+      </c>
+      <c r="J519" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
@@ -22854,7 +25454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I77"/>
+  <dimension ref="A1:I84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -25575,6 +28175,251 @@
       </c>
       <c r="I77" s="6" t="inlineStr"/>
     </row>
+    <row r="78">
+      <c r="A78" s="6" t="inlineStr">
+        <is>
+          <t>RSK-077</t>
+        </is>
+      </c>
+      <c r="B78" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C78" s="6" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="D78" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E78" s="6" t="inlineStr">
+        <is>
+          <t>CPSC Mandatory eFiling Takes Effect July 8; TPEB Rates Surge ~10% as Peak Season Demand Outpaces Capacity</t>
+        </is>
+      </c>
+      <c r="F78" s="6" t="inlineStr"/>
+      <c r="G78" s="6" t="inlineStr"/>
+      <c r="H78" s="6" t="inlineStr">
+        <is>
+          <t>미국 수출 제품의 CPSC 전자 신고 의무 준수 여부 확인 및 준비, 공급망 내 강제 노동 리스크 점검, TPEB 운임 상승에 대한 운송 계획 재검토.</t>
+        </is>
+      </c>
+      <c r="I78" s="6" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="6" t="inlineStr">
+        <is>
+          <t>RSK-078</t>
+        </is>
+      </c>
+      <c r="B79" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C79" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D79" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E79" s="6" t="inlineStr">
+        <is>
+          <t>DOJ Appeals CIT's IEEPA Refund Injunction as CAPE Phase 2 Targets June 29; TPEB Rates Surge 30% Into Peak</t>
+        </is>
+      </c>
+      <c r="F79" s="6" t="inlineStr"/>
+      <c r="G79" s="6" t="inlineStr"/>
+      <c r="H79" s="6" t="inlineStr">
+        <is>
+          <t>IEEPA 관세 환급 관련 진행 상황 주시, TPEB 노선 이용 시 운임 급등에 대비한 운송 계획 및 예산 재검토.</t>
+        </is>
+      </c>
+      <c r="I79" s="6" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="6" t="inlineStr">
+        <is>
+          <t>RSK-079</t>
+        </is>
+      </c>
+      <c r="B80" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C80" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D80" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E80" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 통행 수수료…오만, 이란과 공동징수 추진 및 중동 지정학 리스크 고조</t>
+        </is>
+      </c>
+      <c r="F80" s="6" t="inlineStr"/>
+      <c r="G80" s="6" t="inlineStr"/>
+      <c r="H80" s="6" t="inlineStr">
+        <is>
+          <t>중동/유럽 항로 이용 시 지정학적 리스크 모니터링 강화, 운임 변동성 및 추가 비용 발생 가능성을 고려하여 운송 계획 및 예산 재검토, 비상 운송 계획 수립, 대체 운송 경로 또는 재고 전략 검토.</t>
+        </is>
+      </c>
+      <c r="I80" s="6" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="6" t="inlineStr">
+        <is>
+          <t>RSK-080</t>
+        </is>
+      </c>
+      <c r="B81" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C81" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D81" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E81" s="6" t="inlineStr">
+        <is>
+          <t>머스크, 운임·물동량 급등에 2026년 실적 가이던스 대폭 상향</t>
+        </is>
+      </c>
+      <c r="F81" s="6" t="inlineStr"/>
+      <c r="G81" s="6" t="inlineStr"/>
+      <c r="H81" s="6" t="inlineStr">
+        <is>
+          <t>해상 운임 변동성 모니터링 강화, 장기 운송 계약 조건 재검토, 운송비 절감 방안 및 예산 재조정 검토.</t>
+        </is>
+      </c>
+      <c r="I81" s="6" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="6" t="inlineStr">
+        <is>
+          <t>RSK-081</t>
+        </is>
+      </c>
+      <c r="B82" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C82" s="6" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="D82" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E82" s="6" t="inlineStr">
+        <is>
+          <t>머스크, 중동 운항 신중 기조 유지…유럽 항만 지연 대응</t>
+        </is>
+      </c>
+      <c r="F82" s="6" t="inlineStr"/>
+      <c r="G82" s="6" t="inlineStr"/>
+      <c r="H82" s="6" t="inlineStr">
+        <is>
+          <t>중동/유럽 항로 이용 시 선사별 서비스 안정성 및 운송 리드타임 변화 모니터링, 대체 운송 방안 및 재고 확보 전략 검토.</t>
+        </is>
+      </c>
+      <c r="I82" s="6" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="6" t="inlineStr">
+        <is>
+          <t>RSK-082</t>
+        </is>
+      </c>
+      <c r="B83" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C83" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D83" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E83" s="6" t="inlineStr">
+        <is>
+          <t>종전 합의에도 안 꺾이는 '운임 폭탄'… 수출 중소기업 숨 막힌다</t>
+        </is>
+      </c>
+      <c r="F83" s="6" t="inlineStr"/>
+      <c r="G83" s="6" t="inlineStr"/>
+      <c r="H83" s="6" t="inlineStr">
+        <is>
+          <t>장기 운송 계약 재협상, 선사 다변화, 운송 모드 전환 검토 등 해상 운임 상승에 대한 적극적인 비용 절감 및 리스크 관리 방안을 수립하고 실행해야 합니다.</t>
+        </is>
+      </c>
+      <c r="I83" s="6" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="6" t="inlineStr">
+        <is>
+          <t>RSK-083</t>
+        </is>
+      </c>
+      <c r="B84" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C84" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D84" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E84" s="6" t="inlineStr">
+        <is>
+          <t>소비자물가 2년 6개월 만에 최대폭 상승···중동 전쟁 여파로 석유류 물가 상승 원인</t>
+        </is>
+      </c>
+      <c r="F84" s="6" t="inlineStr"/>
+      <c r="G84" s="6" t="inlineStr"/>
+      <c r="H84" s="6" t="inlineStr">
+        <is>
+          <t>유가 변동에 따른 물류비 상승 리스크를 최소화하기 위해 유류할증료 변동 추이를 면밀히 분석하고, 운송 계약 재검토 및 대체 운송 수단 확보 등 비용 절감 방안을 적극적으로 모색해야 합니다.</t>
+        </is>
+      </c>
+      <c r="I84" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
📰 뉴스 데이터 2026-07-06_09:05
</commit_message>
<xml_diff>
--- a/data/SCM_물류_브리핑.xlsx
+++ b/data/SCM_물류_브리핑.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J519"/>
+  <dimension ref="A1:J552"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -24982,6 +24982,1586 @@
       </c>
       <c r="J519" s="4" t="inlineStr"/>
     </row>
+    <row r="520">
+      <c r="A520" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B520" s="2" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C520" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D520" s="2" t="inlineStr">
+        <is>
+          <t>CPSC Mandatory eFiling Takes Effect July 8; TPEB Rates Surge ~10% as Peak Season Demand Outpaces Capacity (GLOBAL LOGISTICS UPDATE)</t>
+        </is>
+      </c>
+      <c r="E520" s="2" t="inlineStr">
+        <is>
+          <t>CPSC의 의무 전자신고(eFiling)가 7월 8일 발효되며, 성수기 수요가 선복량을 초과하면서 태평양 횡단 동향(TPEB) 운임이 약 10% 급등했다. 또한 CBP는 강제 노동 관련 수입업체 지침을 통합 발표했다.</t>
+        </is>
+      </c>
+      <c r="F520" s="2" t="inlineStr">
+        <is>
+          <t>CPSC 의무 전자신고는 7월 8일부터 즉시 준수해야 하는 규제이며, TPEB 운임의 급등은 물류 비용에 직접적인 영향을 미친다.</t>
+        </is>
+      </c>
+      <c r="G520" s="2" t="inlineStr">
+        <is>
+          <t>CPSC 전자신고 요건 확인 및 시스템 준비, TPEB 운임 상승에 따른 운송 계약 및 예산 재검토, 강제 노동 관련 CBP 지침 준수 여부 확인.</t>
+        </is>
+      </c>
+      <c r="H520" s="2" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I520" s="2" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/june-18-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J520" s="2" t="inlineStr">
+        <is>
+          <t>RSK-084</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B521" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C521" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D521" s="2" t="inlineStr">
+        <is>
+          <t>DOJ Appeals CIT's IEEPA Refund Injunction as CAPE Phase 2 Targets June 29; TPEB Rates Surge 30% Into Peak (GLOBAL LOGISTICS UPDATE)</t>
+        </is>
+      </c>
+      <c r="E521" s="2" t="inlineStr">
+        <is>
+          <t>법무부가 CIT의 IEEPA 환급 명령에 항소했으며, CAPE 2단계가 6월 29일 목표로 진행되는 가운데 태평양 횡단 동향(TPEB) 운임이 성수기를 맞아 30% 급등했다.</t>
+        </is>
+      </c>
+      <c r="F521" s="2" t="inlineStr">
+        <is>
+          <t>TPEB 운임이 30% 급등한 것은 물류 비용에 즉각적이고 심각한 영향을 미치며, 관세 환급 관련 법적 분쟁은 향후 비용 회수에 불확실성을 더한다.</t>
+        </is>
+      </c>
+      <c r="G521" s="2" t="inlineStr">
+        <is>
+          <t>TPEB 운임 급등에 대한 즉각적인 운송 계획 및 예산 조정, 관세 환급 관련 법적 진행 상황 모니터링 및 잠재적 영향 분석.</t>
+        </is>
+      </c>
+      <c r="H521" s="2" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I521" s="2" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/june-11-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J521" s="2" t="inlineStr">
+        <is>
+          <t>RSK-085</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B522" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C522" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D522" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 봉쇄/통행료 추진 및 중동발 물류비 부담</t>
+        </is>
+      </c>
+      <c r="E522" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 봉쇄 가능성 및 통행료 부과 추진으로 항로 우회, 운임 상승, 보험료 할증 등 물류비 부담이 가중되어 한국 제조업 생산비가 최대 4.7% 상승할 수 있으며, 중동 전쟁 이후 해협 통제권이 주요 쟁점이다.</t>
+        </is>
+      </c>
+      <c r="F522" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협은 주요 원유 및 물류 동맥으로, 봉쇄 또는 통행료 부과는 유가 및 해상 운임에 직접적인 영향을 미쳐 우리 회사의 물류비용과 공급망 안정성에 심각한 위협이 될 수 있다.</t>
+        </is>
+      </c>
+      <c r="G522" s="2" t="inlineStr">
+        <is>
+          <t>중동발 원자재 및 부품 수급 현황 점검, 대체 항로 및 운송 수단 가능성 검토, 운송 계약 시 위험 할증료 및 유가 변동 조항 재검토, 비상 재고 확보 방안 논의.</t>
+        </is>
+      </c>
+      <c r="H522" s="2" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I522" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260706-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J522" s="2" t="inlineStr">
+        <is>
+          <t>RSK-086</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B523" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C523" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D523" s="2" t="inlineStr">
+        <is>
+          <t>머스크, 운임·물동량 급등에 2026년 실적 가이던스 대폭 상향</t>
+        </is>
+      </c>
+      <c r="E523" s="2" t="inlineStr">
+        <is>
+          <t>머스크가 극동발 수요 강세와 스팟 운임 급등을 반영하여 2026년 연간 실적 가이던스를 큰 폭으로 상향 조정했다.</t>
+        </is>
+      </c>
+      <c r="F523" s="2" t="inlineStr">
+        <is>
+          <t>주요 선사의 실적 상향은 극동발 운임 급등이 지속되고 있음을 시사하며, 이는 우리 회사의 해상 운송 비용에 직접적인 부담으로 작용한다.</t>
+        </is>
+      </c>
+      <c r="G523" s="2" t="inlineStr">
+        <is>
+          <t>극동발 주요 항로의 운임 변동 추이를 면밀히 모니터링하고, 운송 계약 조건 재검토 및 대체 운송 방안(예: 장기 계약, 복수 운송사 활용)을 적극적으로 모색.</t>
+        </is>
+      </c>
+      <c r="H523" s="2" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I523" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/vol130-주간-선사별-동향-week-27-2026</t>
+        </is>
+      </c>
+      <c r="J523" s="2" t="inlineStr">
+        <is>
+          <t>RSK-087</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B524" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C524" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D524" s="2" t="inlineStr">
+        <is>
+          <t>머스크, 중동 운항 신중 기조 유지…유럽 항만 지연 대응</t>
+        </is>
+      </c>
+      <c r="E524" s="2" t="inlineStr">
+        <is>
+          <t>머스크가 중동 운항에 신중한 기조를 유지하며 유럽 항만 지연에 대응하고 있어, 중동 및 유럽 항로의 서비스 안정성에 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="F524" s="2" t="inlineStr">
+        <is>
+          <t>주요 선사의 중동 운항 신중 기조는 중동발/경유 물류의 불안정성을 높이고, 유럽 항만 지연은 유럽향 물류의 리드타임 증가 및 비용 상승을 야기하여 우리 회사의 공급망에 직접적인 영향을 미친다.</t>
+        </is>
+      </c>
+      <c r="G524" s="2" t="inlineStr">
+        <is>
+          <t>중동 및 유럽 항로의 운송 계획을 재검토하고, 대체 항로 또는 운송사 옵션을 사전에 확보하며, 예상되는 지연에 대비한 재고 및 생산 계획 조정 방안을 수립.</t>
+        </is>
+      </c>
+      <c r="H524" s="2" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I524" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/vol130-주간-선사별-동향-week-27-2026</t>
+        </is>
+      </c>
+      <c r="J524" s="2" t="inlineStr">
+        <is>
+          <t>RSK-088</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B525" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C525" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D525" s="2" t="inlineStr">
+        <is>
+          <t>中 거리두는 韓반도체, 소부장 공급망 재편</t>
+        </is>
+      </c>
+      <c r="E525" s="2" t="inlineStr">
+        <is>
+          <t>삼성전자와 SK하이닉스가 미국의 대중국 규제 강화 가능성에 선제 대응하기 위해 중국 의존도가 높은 반도체 소부장 공급망을 재편하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F525" s="2" t="inlineStr">
+        <is>
+          <t>주요 고객사의 공급망 재편은 우리 회사의 부품 공급 전략 및 생산 계획에 직접적인 영향을 미칠 수 있으며, 지정학적 리스크 관리가 시급합니다.</t>
+        </is>
+      </c>
+      <c r="G525" s="2" t="inlineStr">
+        <is>
+          <t>중국 의존도가 높은 원자재 및 부품에 대한 대체 공급처 발굴, 공급망 다변화 전략 수립, 주요 고객사의 공급망 재편 동향 면밀히 주시.</t>
+        </is>
+      </c>
+      <c r="H525" s="2" t="inlineStr">
+        <is>
+          <t>전자신문</t>
+        </is>
+      </c>
+      <c r="I525" s="2" t="inlineStr">
+        <is>
+          <t>https://etnews.com/20260703000213</t>
+        </is>
+      </c>
+      <c r="J525" s="2" t="inlineStr">
+        <is>
+          <t>RSK-089</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B526" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C526" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D526" s="3" t="inlineStr">
+        <is>
+          <t>U.S.-EU Trade Agreement Eliminates Duties on Most U.S. Goods Starting July 1; TPEB Rates Rise as July Capacity Hits Three-Year High (GLOBAL LOGISTICS UPDATE)</t>
+        </is>
+      </c>
+      <c r="E526" s="3" t="inlineStr">
+        <is>
+          <t>미국-EU 무역 협정이 7월 1일부터 발효되어 대부분의 미국산 산업재에 대한 관세가 철폐되었으며, 동시에 태평양 횡단 동향(TPEB) 운임이 상승하고 7월 선복량이 3년 내 최고치를 기록했다.</t>
+        </is>
+      </c>
+      <c r="F526" s="3" t="inlineStr">
+        <is>
+          <t>미국-EU 관세 철폐는 긍정적이나, 태평양 횡단 동향 운임 상승은 물류비 증가로 이어질 수 있어 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G526" s="3" t="inlineStr">
+        <is>
+          <t>미국-EU 간 수출입 품목에 대한 관세 혜택 여부 확인 및 TPEB 운임 추이 지속 모니터링.</t>
+        </is>
+      </c>
+      <c r="H526" s="3" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I526" s="3" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/july-02-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J526" s="3" t="inlineStr"/>
+    </row>
+    <row r="527">
+      <c r="A527" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B527" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C527" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D527" s="3" t="inlineStr">
+        <is>
+          <t>U.S. Appeals CIT's IEEPA Refund Order to Federal Circuit; TPEB Rates Rise as Peak Season Demand Tightens Capacity (GLOBAL LOGISTICS UPDATE)</t>
+        </is>
+      </c>
+      <c r="E527" s="3" t="inlineStr">
+        <is>
+          <t>미국 정부가 CIT의 IEEPA 환급 명령에 연방 항소법원에 항소했으며, 트럼프 대통령은 수입자 기록(IOR) 요건 강화 등 세관 집행 개혁 행정명령에 서명했고, 성수기 수요로 선복량이 타이트해지면서 TPEB 운임이 상승했다.</t>
+        </is>
+      </c>
+      <c r="F527" s="3" t="inlineStr">
+        <is>
+          <t>관세 환급 관련 법적 분쟁과 IOR 요건 강화는 향후 수입 절차 및 비용에 영향을 미칠 수 있으며, TPEB 운임 상승 추세는 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G527" s="3" t="inlineStr">
+        <is>
+          <t>IOR 요건 강화에 따른 내부 프로세스 점검 및 준수 준비, 관세 환급 관련 법적 진행 상황 모니터링.</t>
+        </is>
+      </c>
+      <c r="H527" s="3" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I527" s="3" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/june-3-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J527" s="3" t="inlineStr"/>
+    </row>
+    <row r="528">
+      <c r="A528" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B528" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C528" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D528" s="3" t="inlineStr">
+        <is>
+          <t>Air Cargo Demand Up 6.0% in May (PRESSROOM)</t>
+        </is>
+      </c>
+      <c r="E528" s="3" t="inlineStr">
+        <is>
+          <t>5월 글로벌 항공 화물 수요가 전년 동기 대비 6.0% 증가하여 항공 화물 시장의 강세를 나타냈다.</t>
+        </is>
+      </c>
+      <c r="F528" s="3" t="inlineStr">
+        <is>
+          <t>항공 화물 수요 증가는 향후 항공 운임 상승 압력으로 작용할 수 있어, 항공 운송을 활용하는 우리 회사에 잠재적 비용 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G528" s="3" t="inlineStr">
+        <is>
+          <t>항공 운임 추이 지속 모니터링 및 필요시 대체 운송 방안 검토.</t>
+        </is>
+      </c>
+      <c r="H528" s="3" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I528" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-29-air-cargo-demand-up-may/</t>
+        </is>
+      </c>
+      <c r="J528" s="3" t="inlineStr"/>
+    </row>
+    <row r="529">
+      <c r="A529" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B529" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C529" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D529" s="3" t="inlineStr">
+        <is>
+          <t>6월 글로벌 석탄 해상운송 14% 급증 (해운/항만/물류 홈 산업 해운/항만/물류)</t>
+        </is>
+      </c>
+      <c r="E529" s="3" t="inlineStr">
+        <is>
+          <t>6월 글로벌 석탄 해상운송량이 전년 동기 대비 14% 급증했으며, 이는 중국 내 탄광 사고와 LNG 공급 차질로 인한 석탄 수입 증가에 기인한다.</t>
+        </is>
+      </c>
+      <c r="F529" s="3" t="inlineStr">
+        <is>
+          <t>특정 벌크 화물 운송량의 급증은 항만 혼잡을 야기하고 선박 가용성에 영향을 미쳐 간접적으로 컨테이너 운송에도 영향을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="G529" s="3" t="inlineStr">
+        <is>
+          <t>주요 항만의 혼잡도 및 선박 스케줄 변동 여부 지속 모니터링.</t>
+        </is>
+      </c>
+      <c r="H529" s="3" t="inlineStr">
+        <is>
+          <t>oceanpress</t>
+        </is>
+      </c>
+      <c r="I529" s="3" t="inlineStr">
+        <is>
+          <t>https://www.oceanpress.co.kr/news/article.html?no=30528</t>
+        </is>
+      </c>
+      <c r="J529" s="3" t="inlineStr"/>
+    </row>
+    <row r="530">
+      <c r="A530" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B530" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C530" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D530" s="3" t="inlineStr">
+        <is>
+          <t>PLSCI Data Indicates Mega-Hub Retrenchment (PRESS ROOM)</t>
+        </is>
+      </c>
+      <c r="E530" s="3" t="inlineStr">
+        <is>
+          <t>UNCTAD의 2026년 2분기 항만 정기선 연결성 지수(PLSCI) 분석 결과, 최근 네트워크 재조정이 메가 허브 항만들의 후퇴를 시사하며, 이는 반응적 대응에서 전략적 재편으로 전환되고 있음을 나타낸다.</t>
+        </is>
+      </c>
+      <c r="F530" s="3" t="inlineStr">
+        <is>
+          <t>주요 허브 항만의 네트워크 재편은 우리 회사의 주요 운송 경로 및 환적 효율성에 장기적인 영향을 미칠 수 있으므로 추이를 지켜봐야 한다.</t>
+        </is>
+      </c>
+      <c r="G530" s="3" t="inlineStr">
+        <is>
+          <t>주요 허브 항만의 서비스 변경 및 연결성 지표 변화 모니터링, 잠재적 운송 경로 최적화 기회 또는 리스크 분석.</t>
+        </is>
+      </c>
+      <c r="H530" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I530" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/396-plsci-data-indicates-mega-hub-retrenchment</t>
+        </is>
+      </c>
+      <c r="J530" s="3" t="inlineStr"/>
+    </row>
+    <row r="531">
+      <c r="A531" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B531" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C531" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D531" s="3" t="inlineStr">
+        <is>
+          <t>Transpacific: Ripe for new non-alliance services</t>
+        </is>
+      </c>
+      <c r="E531" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence 보고서에 따르면 아시아-북미 서안 항로에서 비동맹 선사의 컨테이너 선박 용량 점유율과 스팟 운임 간의 관계를 분석하며 새로운 비동맹 서비스의 가능성을 시사했다.</t>
+        </is>
+      </c>
+      <c r="F531" s="3" t="inlineStr">
+        <is>
+          <t>비동맹 서비스 증가는 운송 옵션 확대 및 운임 경쟁 심화로 이어질 수 있어 장기적인 관점에서 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G531" s="3" t="inlineStr">
+        <is>
+          <t>북미 항로 운송 계약 시 비동맹 선사 서비스 옵션 검토 및 시장 동향 지속 모니터링.</t>
+        </is>
+      </c>
+      <c r="H531" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I531" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/393-transpacific-ripe-for-new-non-alliance-services</t>
+        </is>
+      </c>
+      <c r="J531" s="3" t="inlineStr"/>
+    </row>
+    <row r="532">
+      <c r="A532" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B532" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C532" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D532" s="3" t="inlineStr">
+        <is>
+          <t>Decoding Gemini’s Mediterranean Surge</t>
+        </is>
+      </c>
+      <c r="E532" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence 보고서에 따르면 Gemini Cooperation이 동서 컨테이너 선박 배치를 재조정하며 지중해 지역에 선대를 집중하고 있어 시장 점유율 변화가 예상된다.</t>
+        </is>
+      </c>
+      <c r="F532" s="3" t="inlineStr">
+        <is>
+          <t>주요 선사 동맹의 선대 재배치는 특정 항로의 서비스 가용성 및 운임에 영향을 줄 수 있으므로 지중해 항로 이용 시 주의 깊은 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G532" s="3" t="inlineStr">
+        <is>
+          <t>지중해 항로 이용 시 Gemini Cooperation의 서비스 변화 및 경쟁사 동향을 주시하고, 필요시 운송 계획 조정 검토.</t>
+        </is>
+      </c>
+      <c r="H532" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I532" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/392-decoding-gemini-s-mediterranean-surge</t>
+        </is>
+      </c>
+      <c r="J532" s="3" t="inlineStr"/>
+    </row>
+    <row r="533">
+      <c r="A533" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B533" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C533" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D533" s="3" t="inlineStr">
+        <is>
+          <t>OPEC+ 5개월 연속 증산 합의…내년 공급과잉 우려</t>
+        </is>
+      </c>
+      <c r="E533" s="3" t="inlineStr">
+        <is>
+          <t>OPEC+가 5개월 연속 증산에 합의하면서 내년 공급과잉 우려가 커지고 있으며, 해상 운송 여건 정상화 시 공급 회복이 빨라질 수 있다는 전망이다.</t>
+        </is>
+      </c>
+      <c r="F533" s="3" t="inlineStr">
+        <is>
+          <t>OPEC+의 증산은 유가 하락 압력으로 작용하여 장기적으로 물류비 안정화에 긍정적일 수 있으나, 단기적인 유가 변동성은 지속될 수 있어 추이 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G533" s="3" t="inlineStr">
+        <is>
+          <t>유가 및 해상 운임 동향을 지속적으로 모니터링하고, 운송 계약 시 유가 연동 조항의 적정성 검토.</t>
+        </is>
+      </c>
+      <c r="H533" s="3" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I533" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260706-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J533" s="3" t="inlineStr"/>
+    </row>
+    <row r="534">
+      <c r="A534" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B534" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C534" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D534" s="3" t="inlineStr">
+        <is>
+          <t>삼성·LG, 중동발 물류비 부담에 하반기 가전 수익성 시험대</t>
+        </is>
+      </c>
+      <c r="E534" s="3" t="inlineStr">
+        <is>
+          <t>중동발 불확실성으로 물류비 부담이 커지면서 삼성·LG 등 가전업체들이 하반기 수익성 방어에 어려움을 겪을 수 있다는 전망이다.</t>
+        </is>
+      </c>
+      <c r="F534" s="3" t="inlineStr">
+        <is>
+          <t>중동발 물류비 부담 증가는 배터리/전자부품 산업에도 유사하게 적용될 수 있으며, 운임 정상화 및 선복 재배치까지 우리 회사의 물류비용에도 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G534" s="3" t="inlineStr">
+        <is>
+          <t>중동발 항로 이용 현황 점검, 운임 변동 추이 모니터링 및 운송사와의 협상 전략 재검토.</t>
+        </is>
+      </c>
+      <c r="H534" s="3" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I534" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260704-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J534" s="3" t="inlineStr"/>
+    </row>
+    <row r="535">
+      <c r="A535" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B535" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C535" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D535" s="3" t="inlineStr">
+        <is>
+          <t>인천항 1만6000TEU급 시대 열었다</t>
+        </is>
+      </c>
+      <c r="E535" s="3" t="inlineStr">
+        <is>
+          <t>인천항 미주 정기항로에 1만6000TEU급 초대형 컨테이너선이 처음 투입되며 대형선 시대가 본격적으로 열렸다.</t>
+        </is>
+      </c>
+      <c r="F535" s="3" t="inlineStr">
+        <is>
+          <t>인천항의 대형선 투입은 미주 항로의 운송 효율성 및 선복 공급에 긍정적인 영향을 줄 수 있으며, 인천항 이용 시 운송 계획에 고려할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G535" s="3" t="inlineStr">
+        <is>
+          <t>인천항을 통한 미주 항로 이용 시 운송 효율성 및 비용 절감 가능성을 검토하고, 선사 서비스 변화를 모니터링.</t>
+        </is>
+      </c>
+      <c r="H535" s="3" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I535" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260702-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J535" s="3" t="inlineStr"/>
+    </row>
+    <row r="536">
+      <c r="A536" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B536" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C536" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D536" s="3" t="inlineStr">
+        <is>
+          <t>How Manufacturing Leaders Can Close the Information Gap</t>
+        </is>
+      </c>
+      <c r="E536" s="3" t="inlineStr">
+        <is>
+          <t>제조 리더들이 시장 변화에 대한 정보를 더 일찍, 명확하게 파악하여 견적, 자재, 생산 능력, 자본 지출 결정에 연결하는 방법을 모색해야 한다는 내용입니다.</t>
+        </is>
+      </c>
+      <c r="F536" s="3" t="inlineStr">
+        <is>
+          <t>정보 격차 해소는 물류 및 생산 계획의 효율성을 높이는 데 중요하며, 장기적으로 SCM 경쟁력에 영향을 미칠 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G536" s="3" t="inlineStr">
+        <is>
+          <t>물류 및 SCM 데이터 분석 시스템 고도화 방안 검토 및 시장 변화 예측 역량 강화.</t>
+        </is>
+      </c>
+      <c r="H536" s="3" t="inlineStr">
+        <is>
+          <t>Modern Machine Shop</t>
+        </is>
+      </c>
+      <c r="I536" s="3" t="inlineStr">
+        <is>
+          <t>https://mmsonline.com/articles/how-manufacturing-leaders-can-close-the-information-gap-</t>
+        </is>
+      </c>
+      <c r="J536" s="3" t="inlineStr"/>
+    </row>
+    <row r="537">
+      <c r="A537" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B537" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C537" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D537" s="3" t="inlineStr">
+        <is>
+          <t>원유 '공급 부족→공급 과잉' 새 국면···한국경제 셈법 복잡</t>
+        </is>
+      </c>
+      <c r="E537" s="3" t="inlineStr">
+        <is>
+          <t>미국과 이란 평화협정 이후 호르무즈 해협 원유 공급 증가와 경기 둔화로 국제유가가 급락하며 공급 과잉 국면에 진입했습니다.</t>
+        </is>
+      </c>
+      <c r="F537" s="3" t="inlineStr">
+        <is>
+          <t>유가 하락은 해상 및 항공 운임에 긍정적인 영향을 미쳐 물류비 절감 가능성이 있으나, 장기적인 추이를 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G537" s="3" t="inlineStr">
+        <is>
+          <t>유가 변동 추이를 지속적으로 모니터링하고, 운임 계약 시 유가 연동 조항 검토 및 장기 운임 협상 전략 수립에 반영.</t>
+        </is>
+      </c>
+      <c r="H537" s="3" t="inlineStr">
+        <is>
+          <t>뉴스웨이</t>
+        </is>
+      </c>
+      <c r="I537" s="3" t="inlineStr">
+        <is>
+          <t>https://newsway.co.kr/news/view?ud=2026070510180681959</t>
+        </is>
+      </c>
+      <c r="J537" s="3" t="inlineStr"/>
+    </row>
+    <row r="538">
+      <c r="A538" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B538" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C538" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D538" s="3" t="inlineStr">
+        <is>
+          <t>[기획] 유통 성장 공식…대형 점포보다 ‘AI·물류망·플랫폼’ 경쟁력</t>
+        </is>
+      </c>
+      <c r="E538" s="3" t="inlineStr">
+        <is>
+          <t>국내 유통업계의 성장 공식이 대형 점포에서 인공지능(AI), 물류망, 플랫폼 경쟁력으로 변화하고 있으며, 이는 물류 효율성의 중요성을 강조합니다.</t>
+        </is>
+      </c>
+      <c r="F538" s="3" t="inlineStr">
+        <is>
+          <t>물류망 및 AI 기반 물류 시스템의 중요성 증가는 우리 회사의 SCM 전략 수립 및 물류 기술 투자 방향에 시사하는 바가 큽니다.</t>
+        </is>
+      </c>
+      <c r="G538" s="3" t="inlineStr">
+        <is>
+          <t>AI 및 자동화 기술을 활용한 물류 효율화 방안 검토, 물류 네트워크 최적화 전략 수립.</t>
+        </is>
+      </c>
+      <c r="H538" s="3" t="inlineStr">
+        <is>
+          <t>매일일보</t>
+        </is>
+      </c>
+      <c r="I538" s="3" t="inlineStr">
+        <is>
+          <t>https://m-i.kr/news/articleView.html?idxno=1388023</t>
+        </is>
+      </c>
+      <c r="J538" s="3" t="inlineStr"/>
+    </row>
+    <row r="539">
+      <c r="A539" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B539" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C539" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D539" s="3" t="inlineStr">
+        <is>
+          <t>고물가가 바꾼 유통 단계...정부는 온라인도매 키우고, 이커머스 ‘산지직송’ 구슬땀</t>
+        </is>
+      </c>
+      <c r="E539" s="3" t="inlineStr">
+        <is>
+          <t>고물가로 인해 유통 단계가 변화하며 정부는 온라인 도매시장을, 이커머스는 독자 물류망을 통한 산지직송을 강화하여 유통 비용 절감을 추진하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F539" s="3" t="inlineStr">
+        <is>
+          <t>유통 구조 변화와 물류망을 통한 비용 절감 노력은 우리 회사의 유통 및 물류 전략 수립에 참고할 만한 트렌드를 제시합니다.</t>
+        </is>
+      </c>
+      <c r="G539" s="3" t="inlineStr">
+        <is>
+          <t>물류 비용 절감을 위한 유통 채널 다변화 및 직거래 가능성 검토, 물류 네트워크 효율화 방안 모색.</t>
+        </is>
+      </c>
+      <c r="H539" s="3" t="inlineStr">
+        <is>
+          <t>이투데이</t>
+        </is>
+      </c>
+      <c r="I539" s="3" t="inlineStr">
+        <is>
+          <t>https://etoday.co.kr/news/view/2595689</t>
+        </is>
+      </c>
+      <c r="J539" s="3" t="inlineStr"/>
+    </row>
+    <row r="540">
+      <c r="A540" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B540" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C540" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D540" s="3" t="inlineStr">
+        <is>
+          <t>"택배차 싹 다 바꾼다"... 최대 할인 480만 원 할인에, 실구매가 2천만 원대 진입?</t>
+        </is>
+      </c>
+      <c r="E540" s="3" t="inlineStr">
+        <is>
+          <t>현대차 전기밴 ST1 등 전기 상용차에 대한 할인 혜택이 확대되어 택배 업계에서 전기차 도입을 가속화할 수 있는 기회가 생겼습니다.</t>
+        </is>
+      </c>
+      <c r="F540" s="3" t="inlineStr">
+        <is>
+          <t>전기 상용차 도입은 물류 운송 비용 절감 및 친환경 물류 전환에 기여할 수 있으며, 장기적으로 물류 운영 효율성에 영향을 미칠 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G540" s="3" t="inlineStr">
+        <is>
+          <t>물류 운송 차량의 전기차 전환 가능성 및 경제성 검토, 관련 정부 지원 및 할인 혜택 정보 지속적으로 파악.</t>
+        </is>
+      </c>
+      <c r="H540" s="3" t="inlineStr">
+        <is>
+          <t>오토트리뷴</t>
+        </is>
+      </c>
+      <c r="I540" s="3" t="inlineStr">
+        <is>
+          <t>https://autotribune.co.kr/news/articleView.html?idxno=44068</t>
+        </is>
+      </c>
+      <c r="J540" s="3" t="inlineStr"/>
+    </row>
+    <row r="541">
+      <c r="A541" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B541" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C541" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D541" s="3" t="inlineStr">
+        <is>
+          <t>인니 원자재 수출 규제 파장... 韓 전력·식품 가격 오르나 - 파이낸셜뉴스</t>
+        </is>
+      </c>
+      <c r="E541" s="3" t="inlineStr">
+        <is>
+          <t>인도네시아가 석탄, 팜유, 페로니켈 등 핵심 원자재의 수출을 국영기업이 관리하는 체제로 전환하여 글로벌 원자재 공급망에 변화가 예상된다.</t>
+        </is>
+      </c>
+      <c r="F541" s="3" t="inlineStr">
+        <is>
+          <t>주요 원자재 공급망의 변화는 원자재 가격 변동 및 수급 불안정을 야기하여 우리 생산 비용에 간접적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G541" s="3" t="inlineStr">
+        <is>
+          <t>해당 원자재(특히 페로니켈 등 금속류)의 글로벌 수급 동향 및 가격 변화를 지속적으로 모니터링하고, 필요시 대체 공급처 확보 가능성을 검토한다.</t>
+        </is>
+      </c>
+      <c r="H541" s="3" t="inlineStr">
+        <is>
+          <t>파이낸셜뉴스</t>
+        </is>
+      </c>
+      <c r="I541" s="3" t="inlineStr">
+        <is>
+          <t>https://www.fnnews.com/news/202607050742562659</t>
+        </is>
+      </c>
+      <c r="J541" s="3" t="inlineStr"/>
+    </row>
+    <row r="542">
+      <c r="A542" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B542" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C542" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D542" s="3" t="inlineStr">
+        <is>
+          <t>[사설] '반도체 소부장 주권' 더 높여가야 - 전자신문</t>
+        </is>
+      </c>
+      <c r="E542" s="3" t="inlineStr">
+        <is>
+          <t>삼성전자와 SK하이닉스가 중국 의존도가 높았던 반도체 소부장 공급망에 변화를 주기 시작하며 '반도체 소부장 주권' 강화 움직임이 포착되었다.</t>
+        </is>
+      </c>
+      <c r="F542" s="3" t="inlineStr">
+        <is>
+          <t>주요 전자부품 제조사들의 공급망 재편 움직임은 장기적으로 원자재 및 부품 수급 환경에 변화를 가져올 수 있으며, 우리 회사의 공급망 전략에도 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G542" s="3" t="inlineStr">
+        <is>
+          <t>주요 원자재 및 부품의 공급망 다변화 추세를 주시하고, 잠재적 공급 리스크를 평가하여 선제적인 공급처 다변화 전략을 검토한다.</t>
+        </is>
+      </c>
+      <c r="H542" s="3" t="inlineStr">
+        <is>
+          <t>전자신문</t>
+        </is>
+      </c>
+      <c r="I542" s="3" t="inlineStr">
+        <is>
+          <t>https://etnews.com/20260705000050</t>
+        </is>
+      </c>
+      <c r="J542" s="3" t="inlineStr"/>
+    </row>
+    <row r="543">
+      <c r="A543" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B543" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C543" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D543" s="3" t="inlineStr">
+        <is>
+          <t>美·EU·英 이어 日까지 … 높아지는 철강 보호무역 - 매일경제</t>
+        </is>
+      </c>
+      <c r="E543" s="3" t="inlineStr">
+        <is>
+          <t>미국, EU, 영국에 이어 일본까지 철강 보호무역 조치를 강화하며 한국산 철강에 대한 반덤핑 조사가 진행되는 등 글로벌 무역 환경의 불확실성이 커지고 있다.</t>
+        </is>
+      </c>
+      <c r="F543" s="3" t="inlineStr">
+        <is>
+          <t>철강 산업의 보호무역 강화는 전반적인 글로벌 무역 환경의 경색을 시사하며, 향후 전자부품 관련 원자재 및 제품에도 유사한 무역 장벽이 발생할 가능성을 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G543" s="3" t="inlineStr">
+        <is>
+          <t>주요 수출입 국가의 무역 정책 변화를 지속적으로 모니터링하고, 잠재적인 관세 및 비관세 장벽 발생 가능성에 대비한다.</t>
+        </is>
+      </c>
+      <c r="H543" s="3" t="inlineStr">
+        <is>
+          <t>매일경제</t>
+        </is>
+      </c>
+      <c r="I543" s="3" t="inlineStr">
+        <is>
+          <t>https://mk.co.kr/news/business/12090643</t>
+        </is>
+      </c>
+      <c r="J543" s="3" t="inlineStr"/>
+    </row>
+    <row r="544">
+      <c r="A544" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B544" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C544" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D544" s="3" t="inlineStr">
+        <is>
+          <t>[2026 재계 인물 탐구 ㉔] 이상윤 티웨이항공 대표, 중·장거리 노선·화물 사업·소노그룹 지원에 ‘훨훨’ &lt; 기획 &lt; 기사본문 - 이코노미트리뷴</t>
+        </is>
+      </c>
+      <c r="E544" s="3" t="inlineStr">
+        <is>
+          <t>티웨이항공이 중장거리 노선 및 화물 사업을 확대하고 있어 항공 운송 시장의 공급 능력 증가와 운임 변동 가능성이 예상된다.</t>
+        </is>
+      </c>
+      <c r="F544" s="3" t="inlineStr">
+        <is>
+          <t>항공사의 화물 사업 확대는 항공 운송 시장의 공급 능력 증가로 이어져, 향후 우리 회사의 항공 운임 및 운송 옵션에 긍정적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G544" s="3" t="inlineStr">
+        <is>
+          <t>항공 화물 시장의 공급 및 운임 동향을 지속적으로 모니터링하고, 필요시 신규 노선 활용 가능성을 검토한다.</t>
+        </is>
+      </c>
+      <c r="H544" s="3" t="inlineStr">
+        <is>
+          <t>이코노미트리뷴</t>
+        </is>
+      </c>
+      <c r="I544" s="3" t="inlineStr">
+        <is>
+          <t>https://economytribune.co.kr/news/articleView.html?idxno=3903249</t>
+        </is>
+      </c>
+      <c r="J544" s="3" t="inlineStr"/>
+    </row>
+    <row r="545">
+      <c r="A545" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B545" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C545" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D545" s="3" t="inlineStr">
+        <is>
+          <t>주유소 기름값 7주째 하락 - 매일경제</t>
+        </is>
+      </c>
+      <c r="E545" s="3" t="inlineStr">
+        <is>
+          <t>국제유가 하락의 영향으로 국내 주유소 휘발유·경유 가격이 7주째 하락하여 1900원대 중반을 기록했다.</t>
+        </is>
+      </c>
+      <c r="F545" s="3" t="inlineStr">
+        <is>
+          <t>유가 하락은 육상 운송 및 해상/항공 운송의 유류 할증료 감소로 이어져 우리 회사의 전반적인 물류비 절감에 긍정적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G545" s="3" t="inlineStr">
+        <is>
+          <t>유가 및 유류 할증료 추이를 지속적으로 모니터링하고, 물류비 절감 효과를 분석하여 운송 계약 협상 시 반영 가능성을 검토한다.</t>
+        </is>
+      </c>
+      <c r="H545" s="3" t="inlineStr">
+        <is>
+          <t>매일경제</t>
+        </is>
+      </c>
+      <c r="I545" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mk.co.kr/news/business/12090729</t>
+        </is>
+      </c>
+      <c r="J545" s="3" t="inlineStr"/>
+    </row>
+    <row r="546">
+      <c r="A546" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B546" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C546" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D546" s="4" t="inlineStr">
+        <is>
+          <t>Global Schedule Reliability for May 2026 the Highest of the Year</t>
+        </is>
+      </c>
+      <c r="E546" s="4" t="inlineStr">
+        <is>
+          <t>2026년 5월 글로벌 선박 스케줄 정시성이 연중 최고치를 기록했다는 Sea-Intelligence 보고서가 발표되었다.</t>
+        </is>
+      </c>
+      <c r="F546" s="4" t="inlineStr">
+        <is>
+          <t>스케줄 정시성 개선은 긍정적인 신호이나, 특정 월의 통계이며 우리 회사의 물류 운영에 직접적인 즉각적 영향은 낮다.</t>
+        </is>
+      </c>
+      <c r="G546" s="4" t="n"/>
+      <c r="H546" s="4" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I546" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/395-global-schedule-reliability-for-may-2026-the-highest-of-the-year</t>
+        </is>
+      </c>
+      <c r="J546" s="4" t="inlineStr"/>
+    </row>
+    <row r="547">
+      <c r="A547" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B547" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C547" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D547" s="4" t="inlineStr">
+        <is>
+          <t>Tracking True Vessel Delay</t>
+        </is>
+      </c>
+      <c r="E547" s="4" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence 보고서에 따르면 선사들이 운송 시간을 늘리는 스케줄 버퍼링에 의존하여 실제 선박 지연과 조기 도착 간의 관계를 분석했다.</t>
+        </is>
+      </c>
+      <c r="F547" s="4" t="inlineStr">
+        <is>
+          <t>선박 지연 분석에 대한 보고서로, 현재 우리 회사의 물류 운영에 직접적인 영향을 미치기보다는 업계 동향 파악에 가깝다.</t>
+        </is>
+      </c>
+      <c r="G547" s="4" t="n"/>
+      <c r="H547" s="4" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I547" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/394-tracking-true-vessel-delay</t>
+        </is>
+      </c>
+      <c r="J547" s="4" t="inlineStr"/>
+    </row>
+    <row r="548">
+      <c r="A548" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B548" s="4" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C548" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D548" s="4" t="inlineStr">
+        <is>
+          <t>현대글로비스, 단기 주가는 그룹사 로보틱스 투자 전략이 좌우...2분기, 유류비 상승분 시차 전가로 일시적 부진</t>
+        </is>
+      </c>
+      <c r="E548" s="4" t="inlineStr">
+        <is>
+          <t>현대글로비스의 2분기 실적이 유류비 상승분 전가 시차로 인해 일시적으로 부진할 것으로 전망되며, 단기 주가는 그룹사 로보틱스 투자 전략에 더 큰 영향을 받을 것으로 분석되었다.</t>
+        </is>
+      </c>
+      <c r="F548" s="4" t="inlineStr">
+        <is>
+          <t>특정 선사의 실적 전망이며, 유류비 상승으로 인한 운임 전가는 이미 시장에 반영되고 있는 추세이므로 당사 물류 운영에 직접적인 새로운 영향은 낮다.</t>
+        </is>
+      </c>
+      <c r="G548" s="4" t="n"/>
+      <c r="H548" s="4" t="inlineStr">
+        <is>
+          <t>shippingnewsnet</t>
+        </is>
+      </c>
+      <c r="I548" s="4" t="inlineStr">
+        <is>
+          <t>https://www.shippingnewsnet.com/news/articleView.html?idxno=71038</t>
+        </is>
+      </c>
+      <c r="J548" s="4" t="inlineStr"/>
+    </row>
+    <row r="549">
+      <c r="A549" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B549" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C549" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D549" s="4" t="inlineStr">
+        <is>
+          <t>마스오토, 부산항까지 트레일러 자율주행…2028년 화물 완전 무인화 목표</t>
+        </is>
+      </c>
+      <c r="E549" s="4" t="inlineStr">
+        <is>
+          <t>마스오토가 부산항을 거점으로 트레일러 자율주행 상용화를 추진하며 2028년 화물 운송의 완전 무인화를 목표로 물류 혁신을 시도하고 있다.</t>
+        </is>
+      </c>
+      <c r="F549" s="4" t="inlineStr">
+        <is>
+          <t>장기적인 물류 혁신 동향으로, 당장 우리 회사의 물류 운영에 직접적인 영향을 미치기보다는 미래 기술 도입 가능성을 참고하는 수준이다.</t>
+        </is>
+      </c>
+      <c r="G549" s="4" t="n"/>
+      <c r="H549" s="4" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I549" s="4" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260703-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J549" s="4" t="inlineStr"/>
+    </row>
+    <row r="550">
+      <c r="A550" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B550" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C550" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D550" s="4" t="inlineStr">
+        <is>
+          <t>머스크, 브라질 북동부 수아페항 투자 확대…남미 물류 거점 육성</t>
+        </is>
+      </c>
+      <c r="E550" s="4" t="inlineStr">
+        <is>
+          <t>머스크가 브라질 북동부 수아페항 투자를 확대하여 남미 공급망의 전략 거점을 확보하고 복합물류망을 확충하고 있다.</t>
+        </is>
+      </c>
+      <c r="F550" s="4" t="inlineStr">
+        <is>
+          <t>특정 선사의 남미 지역 투자 소식으로, 우리 회사의 남미 물류 운영에 직접적인 영향보다는 장기적인 시장 동향 참고 수준이다.</t>
+        </is>
+      </c>
+      <c r="G550" s="4" t="n"/>
+      <c r="H550" s="4" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I550" s="4" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/vol130-주간-선사별-동향-week-27-2026</t>
+        </is>
+      </c>
+      <c r="J550" s="4" t="inlineStr"/>
+    </row>
+    <row r="551">
+      <c r="A551" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B551" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C551" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D551" s="4" t="inlineStr">
+        <is>
+          <t>상반기 대체연료추진선 발주 137척, 2년 연속 감소</t>
+        </is>
+      </c>
+      <c r="E551" s="4" t="inlineStr">
+        <is>
+          <t>2026년 상반기 대체연료추진선 발주가 2년 연속 감소했으며, LPG·에탄 추진선 발주는 급증하는 등 선종 및 연료별 차별화가 나타났다.</t>
+        </is>
+      </c>
+      <c r="F551" s="4" t="inlineStr">
+        <is>
+          <t>장기적인 해운 산업의 선박 연료 전환 동향으로, 당장 우리 회사의 물류 운영에 직접적인 영향을 미치기보다는 장기적인 친환경 운송 옵션 변화를 참고하는 수준이다.</t>
+        </is>
+      </c>
+      <c r="G551" s="4" t="n"/>
+      <c r="H551" s="4" t="inlineStr">
+        <is>
+          <t>oceanpress.co.kr</t>
+        </is>
+      </c>
+      <c r="I551" s="4" t="inlineStr">
+        <is>
+          <t>https://oceanpress.co.kr/news/article.html?no=30525</t>
+        </is>
+      </c>
+      <c r="J551" s="4" t="inlineStr"/>
+    </row>
+    <row r="552">
+      <c r="A552" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B552" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C552" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D552" s="4" t="inlineStr">
+        <is>
+          <t>당정청 “반도체 생산 거점 조기 완성·전국 확산…전력부지 인허가 지원”</t>
+        </is>
+      </c>
+      <c r="E552" s="4" t="inlineStr">
+        <is>
+          <t>정부가 반도체 생산 거점 조기 완성 및 전국 확산을 위해 전력 부지 인허가 등을 지원하며, 서남권을 제2 반도체 거점으로 육성할 계획입니다.</t>
+        </is>
+      </c>
+      <c r="F552" s="4" t="inlineStr">
+        <is>
+          <t>장기적인 산업 인프라 구축 계획으로 당장 물류 운영에 직접적인 영향은 없으나, 향후 물류 거점 및 운송 경로 계획에 참고할 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G552" s="4" t="n"/>
+      <c r="H552" s="4" t="inlineStr">
+        <is>
+          <t>이투데이</t>
+        </is>
+      </c>
+      <c r="I552" s="4" t="inlineStr">
+        <is>
+          <t>https://www.etoday.co.kr/news/view/2600379</t>
+        </is>
+      </c>
+      <c r="J552" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -24994,7 +26574,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -25442,6 +27022,49 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>3326.87</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>+87 (+2.7%)</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>+1,457 (+77.9%)</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>3920</v>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>+173 (+4.6%)</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>+1,093 (+38.7%)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -25454,7 +27077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I84"/>
+  <dimension ref="A1:I90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -28420,6 +30043,216 @@
       </c>
       <c r="I84" s="6" t="inlineStr"/>
     </row>
+    <row r="85">
+      <c r="A85" s="6" t="inlineStr">
+        <is>
+          <t>RSK-084</t>
+        </is>
+      </c>
+      <c r="B85" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C85" s="6" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="D85" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E85" s="6" t="inlineStr">
+        <is>
+          <t>CPSC Mandatory eFiling Takes Effect July 8; TPEB Rates Surge ~10% as Peak Season Demand Outpaces Capacity (GLOBAL LOGISTICS UPDATE)</t>
+        </is>
+      </c>
+      <c r="F85" s="6" t="inlineStr"/>
+      <c r="G85" s="6" t="inlineStr"/>
+      <c r="H85" s="6" t="inlineStr">
+        <is>
+          <t>CPSC 전자신고 요건 확인 및 시스템 준비, TPEB 운임 상승에 따른 운송 계약 및 예산 재검토, 강제 노동 관련 CBP 지침 준수 여부 확인.</t>
+        </is>
+      </c>
+      <c r="I85" s="6" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="6" t="inlineStr">
+        <is>
+          <t>RSK-085</t>
+        </is>
+      </c>
+      <c r="B86" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C86" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D86" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E86" s="6" t="inlineStr">
+        <is>
+          <t>DOJ Appeals CIT's IEEPA Refund Injunction as CAPE Phase 2 Targets June 29; TPEB Rates Surge 30% Into Peak (GLOBAL LOGISTICS UPDATE)</t>
+        </is>
+      </c>
+      <c r="F86" s="6" t="inlineStr"/>
+      <c r="G86" s="6" t="inlineStr"/>
+      <c r="H86" s="6" t="inlineStr">
+        <is>
+          <t>TPEB 운임 급등에 대한 즉각적인 운송 계획 및 예산 조정, 관세 환급 관련 법적 진행 상황 모니터링 및 잠재적 영향 분석.</t>
+        </is>
+      </c>
+      <c r="I86" s="6" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="6" t="inlineStr">
+        <is>
+          <t>RSK-086</t>
+        </is>
+      </c>
+      <c r="B87" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C87" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D87" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E87" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 봉쇄/통행료 추진 및 중동발 물류비 부담</t>
+        </is>
+      </c>
+      <c r="F87" s="6" t="inlineStr"/>
+      <c r="G87" s="6" t="inlineStr"/>
+      <c r="H87" s="6" t="inlineStr">
+        <is>
+          <t>중동발 원자재 및 부품 수급 현황 점검, 대체 항로 및 운송 수단 가능성 검토, 운송 계약 시 위험 할증료 및 유가 변동 조항 재검토, 비상 재고 확보 방안 논의.</t>
+        </is>
+      </c>
+      <c r="I87" s="6" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="6" t="inlineStr">
+        <is>
+          <t>RSK-087</t>
+        </is>
+      </c>
+      <c r="B88" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C88" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D88" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E88" s="6" t="inlineStr">
+        <is>
+          <t>머스크, 운임·물동량 급등에 2026년 실적 가이던스 대폭 상향</t>
+        </is>
+      </c>
+      <c r="F88" s="6" t="inlineStr"/>
+      <c r="G88" s="6" t="inlineStr"/>
+      <c r="H88" s="6" t="inlineStr">
+        <is>
+          <t>극동발 주요 항로의 운임 변동 추이를 면밀히 모니터링하고, 운송 계약 조건 재검토 및 대체 운송 방안(예: 장기 계약, 복수 운송사 활용)을 적극적으로 모색.</t>
+        </is>
+      </c>
+      <c r="I88" s="6" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="6" t="inlineStr">
+        <is>
+          <t>RSK-088</t>
+        </is>
+      </c>
+      <c r="B89" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C89" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D89" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E89" s="6" t="inlineStr">
+        <is>
+          <t>머스크, 중동 운항 신중 기조 유지…유럽 항만 지연 대응</t>
+        </is>
+      </c>
+      <c r="F89" s="6" t="inlineStr"/>
+      <c r="G89" s="6" t="inlineStr"/>
+      <c r="H89" s="6" t="inlineStr">
+        <is>
+          <t>중동 및 유럽 항로의 운송 계획을 재검토하고, 대체 항로 또는 운송사 옵션을 사전에 확보하며, 예상되는 지연에 대비한 재고 및 생산 계획 조정 방안을 수립.</t>
+        </is>
+      </c>
+      <c r="I89" s="6" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="6" t="inlineStr">
+        <is>
+          <t>RSK-089</t>
+        </is>
+      </c>
+      <c r="B90" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C90" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D90" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E90" s="6" t="inlineStr">
+        <is>
+          <t>中 거리두는 韓반도체, 소부장 공급망 재편</t>
+        </is>
+      </c>
+      <c r="F90" s="6" t="inlineStr"/>
+      <c r="G90" s="6" t="inlineStr"/>
+      <c r="H90" s="6" t="inlineStr">
+        <is>
+          <t>중국 의존도가 높은 원자재 및 부품에 대한 대체 공급처 발굴, 공급망 다변화 전략 수립, 주요 고객사의 공급망 재편 동향 면밀히 주시.</t>
+        </is>
+      </c>
+      <c r="I90" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
📰 뉴스 데이터 2026-07-07_09:09
</commit_message>
<xml_diff>
--- a/data/SCM_물류_브리핑.xlsx
+++ b/data/SCM_물류_브리핑.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J552"/>
+  <dimension ref="A1:J585"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -26562,6 +26562,1526 @@
       </c>
       <c r="J552" s="4" t="inlineStr"/>
     </row>
+    <row r="553">
+      <c r="A553" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B553" s="2" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C553" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D553" s="2" t="inlineStr">
+        <is>
+          <t>제다항 혼잡, 육상 물류망 마비…선사들 예약 중단</t>
+        </is>
+      </c>
+      <c r="E553" s="2" t="inlineStr">
+        <is>
+          <t>사우디아라비아 제다항의 운송망 마비로 글로벌 선사들이 제다 경유 서비스를 중단하고 오만 살랄라항이나 UAE 코르파칸항 등 대체 우회 운송 체계를 가동하고 있다.</t>
+        </is>
+      </c>
+      <c r="F553" s="2" t="inlineStr">
+        <is>
+          <t>중동 지역으로의 해상 운송에 직접적인 지연 및 비용 증가를 초래하며, 해당 지역으로의 부품/제품 운송 계획에 즉각적인 변경이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G553" s="2" t="inlineStr">
+        <is>
+          <t>중동 지역 운송 예정 물량의 대체 항만 및 운송 경로 확인, 선사와의 긴밀한 소통을 통한 스케줄 조정 및 비용 영향 분석.</t>
+        </is>
+      </c>
+      <c r="H553" s="2" t="inlineStr">
+        <is>
+          <t>kita</t>
+        </is>
+      </c>
+      <c r="I553" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kita.net/shippers/board/newsView.do?morgueCode=2&amp;dataCls=B&amp;dataSeq=8151</t>
+        </is>
+      </c>
+      <c r="J553" s="2" t="inlineStr">
+        <is>
+          <t>RSK-090</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B554" s="2" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C554" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D554" s="2" t="inlineStr">
+        <is>
+          <t>20260706 경제·물류 주요뉴스 (데일리스크랩)</t>
+        </is>
+      </c>
+      <c r="E554" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 봉쇄 시 항로 우회, 선복 부족, 보험료 및 위험 할증료 증가로 한국 제조업 생산비가 4.7% 상승할 수 있으며, OPEC+의 증산 합의에도 불구하고 중동 리스크는 여전하다.</t>
+        </is>
+      </c>
+      <c r="F554" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 봉쇄는 주요 항로 중단 및 물류비 급증으로 이어져 우리 물류 운영 및 생산 계획에 직접적인 고위험 요소이다.</t>
+        </is>
+      </c>
+      <c r="G554" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 관련 중동 정세 및 해운 동향을 면밀히 모니터링하고, 비상시 대체 운송 경로 및 재고 확보 방안을 검토해야 한다.</t>
+        </is>
+      </c>
+      <c r="H554" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I554" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260706-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J554" s="2" t="inlineStr">
+        <is>
+          <t>RSK-091</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B555" s="2" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C555" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D555" s="2" t="inlineStr">
+        <is>
+          <t>20260703 경제·물류 주요뉴스 (데일리스크랩)</t>
+        </is>
+      </c>
+      <c r="E555" s="2" t="inlineStr">
+        <is>
+          <t>오만이 이란과 호르무즈 해협 통행 수수료 공동 징수를 추진하며 해운 운임 상승 국면에서 물류비 부담이 추가로 커질 수 있다는 우려가 제기되었다.</t>
+        </is>
+      </c>
+      <c r="F555" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 통행 수수료 부과는 즉각적인 물류비 상승으로 이어져 우리 회사의 운송 비용에 직접적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G555" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 통행료 부과 논의 진행 상황을 면밀히 모니터링하고, 예상되는 추가 물류비용을 분석하여 예산 및 운송 계획에 반영해야 한다.</t>
+        </is>
+      </c>
+      <c r="H555" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I555" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260703-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J555" s="2" t="inlineStr">
+        <is>
+          <t>RSK-092</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B556" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C556" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D556" s="3" t="inlineStr">
+        <is>
+          <t>Air Cargo Demand Up 6.0% in May</t>
+        </is>
+      </c>
+      <c r="E556" s="3" t="inlineStr">
+        <is>
+          <t>국제항공운송협회(IATA)에 따르면 2026년 5월 전 세계 항공 화물 수요가 전년 동기 대비 6.0% 증가했다.</t>
+        </is>
+      </c>
+      <c r="F556" s="3" t="inlineStr">
+        <is>
+          <t>항공 화물 수요 증가는 향후 항공 운임 상승 압력으로 작용할 수 있어 운송 비용에 영향을 줄 가능성이 있다.</t>
+        </is>
+      </c>
+      <c r="G556" s="3" t="inlineStr">
+        <is>
+          <t>항공 운임 추이 지속 모니터링 및 필요시 대체 운송 방안 검토.</t>
+        </is>
+      </c>
+      <c r="H556" s="3" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I556" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-29-air-cargo-demand-up-may/</t>
+        </is>
+      </c>
+      <c r="J556" s="3" t="inlineStr"/>
+    </row>
+    <row r="557">
+      <c r="A557" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B557" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C557" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D557" s="3" t="inlineStr">
+        <is>
+          <t>“중동전쟁 끝나면 컨선·탱크선 시황 하락세 탈 것”</t>
+        </is>
+      </c>
+      <c r="E557" s="3" t="inlineStr">
+        <is>
+          <t>중동 정세 불안으로 수에즈운하 정상화 여부가 컨테이너선 시황을 좌우할 것이며, 중동 사태 진정 시 컨테이너선 및 탱크선 시황은 하락세를 보이고 벌크선은 재건 수요로 호조를 띨 것으로 전망된다.</t>
+        </is>
+      </c>
+      <c r="F557" s="3" t="inlineStr">
+        <is>
+          <t>중동 정세 불안은 수에즈운하 통항에 지속적인 불확실성을 야기하여 해상 운송 경로 및 운임에 잠재적 영향을 미칠 수 있으므로 추이를 주시해야 한다.</t>
+        </is>
+      </c>
+      <c r="G557" s="3" t="inlineStr">
+        <is>
+          <t>중동 정세 및 수에즈운하 통항 상황 지속 모니터링, 장기적인 해상 운송 전략 수립 시 잠재적 운임 변동성 고려.</t>
+        </is>
+      </c>
+      <c r="H557" s="3" t="inlineStr">
+        <is>
+          <t>ksg</t>
+        </is>
+      </c>
+      <c r="I557" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ksg.co.kr/news/main_newsView.jsp?pNum=147553</t>
+        </is>
+      </c>
+      <c r="J557" s="3" t="inlineStr"/>
+    </row>
+    <row r="558">
+      <c r="A558" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B558" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C558" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D558" s="3" t="inlineStr">
+        <is>
+          <t>PLSCI Data Indicates Mega-Hub Retrenchment</t>
+        </is>
+      </c>
+      <c r="E558" s="3" t="inlineStr">
+        <is>
+          <t>UNCTAD의 2026년 2분기 PLSCI 데이터 분석 결과, 최근 선사들의 네트워크 재조정이 메가 허브 항만의 연결성 감소로 이어지고 있음을 시사한다.</t>
+        </is>
+      </c>
+      <c r="F558" s="3" t="inlineStr">
+        <is>
+          <t>주요 항만의 연결성 변화는 향후 해상 운송 경로 및 리드타임에 영향을 줄 수 있으므로, 우리 회사의 주요 운송 항로에 미칠 영향을 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G558" s="3" t="inlineStr">
+        <is>
+          <t>주요 운송 항로의 허브 항만 연결성 변화 추이 모니터링, 필요시 대체 항만 및 운송 경로 검토.</t>
+        </is>
+      </c>
+      <c r="H558" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I558" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/396-plsci-data-indicates-mega-hub-retrenchment</t>
+        </is>
+      </c>
+      <c r="J558" s="3" t="inlineStr"/>
+    </row>
+    <row r="559">
+      <c r="A559" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B559" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C559" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D559" s="3" t="inlineStr">
+        <is>
+          <t>Tracking True Vessel Delay</t>
+        </is>
+      </c>
+      <c r="E559" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence 분석에 따르면 선사들이 운송 시간을 늘리는 스케줄 버퍼링을 통해 선박의 조기 도착을 유도하고 있으며, 이는 실제 지연을 추적하는 데 영향을 미친다.</t>
+        </is>
+      </c>
+      <c r="F559" s="3" t="inlineStr">
+        <is>
+          <t>선사들의 스케줄 버퍼링 전략은 겉으로 보이는 정시성을 높일 수 있으나, 실제 운송 리드타임에 영향을 미치므로 정확한 도착 예측 및 재고 관리를 위해 지속적인 분석이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G559" s="3" t="inlineStr">
+        <is>
+          <t>선사별 실제 운송 리드타임 데이터 분석 강화, 운송 계획 수립 시 스케줄 버퍼링으로 인한 잠재적 리드타임 변화 고려.</t>
+        </is>
+      </c>
+      <c r="H559" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I559" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/394-tracking-true-vessel-delay</t>
+        </is>
+      </c>
+      <c r="J559" s="3" t="inlineStr"/>
+    </row>
+    <row r="560">
+      <c r="A560" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B560" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C560" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D560" s="3" t="inlineStr">
+        <is>
+          <t>Transpacific: Ripe for new non-alliance services</t>
+        </is>
+      </c>
+      <c r="E560" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence 분석에 따르면 태평양 횡단 항로에서 비동맹 선사들의 신규 서비스가 증가할 가능성이 있으며, 이는 컨테이너 스팟 운임과 관련이 있다.</t>
+        </is>
+      </c>
+      <c r="F560" s="3" t="inlineStr">
+        <is>
+          <t>태평양 횡단 항로의 비동맹 선사 서비스 증가는 경쟁 심화로 이어져 운임 변동성을 높일 수 있으므로, 주요 운송 비용에 미칠 영향을 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G560" s="3" t="inlineStr">
+        <is>
+          <t>태평양 횡단 항로의 신규 서비스 및 운임 동향 지속 모니터링, 다양한 선사 옵션 검토.</t>
+        </is>
+      </c>
+      <c r="H560" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I560" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/393-transpacific-ripe-for-new-non-alliance-services</t>
+        </is>
+      </c>
+      <c r="J560" s="3" t="inlineStr"/>
+    </row>
+    <row r="561">
+      <c r="A561" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B561" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C561" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D561" s="3" t="inlineStr">
+        <is>
+          <t>20260707 경제·물류 주요뉴스 (데일리스크랩)</t>
+        </is>
+      </c>
+      <c r="E561" s="3" t="inlineStr">
+        <is>
+          <t>OPEC+ 증산 전망 등 공급 증가 요인으로 국제유가가 소폭 하락했으나, 중동 불확실성은 여전하여 유가 변동 추이를 지속적으로 모니터링할 필요가 있다.</t>
+        </is>
+      </c>
+      <c r="F561" s="3" t="inlineStr">
+        <is>
+          <t>유가 하락은 물류비 부담 완화 가능성을 시사하지만, 중동 불확실성이 상존하여 추이를 지켜봐야 한다.</t>
+        </is>
+      </c>
+      <c r="G561" s="3" t="inlineStr">
+        <is>
+          <t>유가 및 해상/항공 운임 변동 추이 지속 모니터링.</t>
+        </is>
+      </c>
+      <c r="H561" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I561" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260707-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J561" s="3" t="inlineStr"/>
+    </row>
+    <row r="562">
+      <c r="A562" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B562" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C562" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D562" s="3" t="inlineStr">
+        <is>
+          <t>25만 원 이하 직구도 이제 관세? EU 소액면세 폐지가 바꾸는 것들 (Week 27, 2026)</t>
+        </is>
+      </c>
+      <c r="E562" s="3" t="inlineStr">
+        <is>
+          <t>2026년 7월 1일부터 EU의 150유로 이하 소액면세 제도가 폐지되어, 유럽으로 수출하는 모든 소포에 관세가 부과될 예정이며 이는 초저가 직구 모델에 큰 변화를 가져올 것이다.</t>
+        </is>
+      </c>
+      <c r="F562" s="3" t="inlineStr">
+        <is>
+          <t>EU로의 수출 시 관세 부담이 증가하여 가격 경쟁력에 영향을 미칠 수 있으므로, 관련 규정 변화를 주시하고 대응 방안을 마련해야 한다.</t>
+        </is>
+      </c>
+      <c r="G562" s="3" t="inlineStr">
+        <is>
+          <t>EU 수출 물량에 대한 관세 영향 분석 및 가격 정책, 통관 절차 변화에 대한 대응 방안 검토.</t>
+        </is>
+      </c>
+      <c r="H562" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I562" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/25만-원-이하-직구도-이제-관세-eu-소액면세-폐지가-바꾸는-것들-week-27-2026-</t>
+        </is>
+      </c>
+      <c r="J562" s="3" t="inlineStr"/>
+    </row>
+    <row r="563">
+      <c r="A563" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B563" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C563" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D563" s="3" t="inlineStr">
+        <is>
+          <t>20260704 경제·물류 주요뉴스 (데일리스크랩)</t>
+        </is>
+      </c>
+      <c r="E563" s="3" t="inlineStr">
+        <is>
+          <t>중동발 불확실성으로 인한 물류비 부담이 커지면서 가전업체들이 하반기 수익성 방어에 어려움을 겪을 수 있으며, 이는 운임 정상화와 선복 재배치가 이뤄질 때까지 지속될 전망이다.</t>
+        </is>
+      </c>
+      <c r="F563" s="3" t="inlineStr">
+        <is>
+          <t>중동 리스크로 인한 물류비 상승은 우리 회사의 운송 비용에도 영향을 미칠 수 있으므로, 추이를 지속적으로 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G563" s="3" t="inlineStr">
+        <is>
+          <t>중동 정세 및 해상 운임 변동 추이 모니터링, 물류비 상승 시나리오에 대한 대응 계획 검토.</t>
+        </is>
+      </c>
+      <c r="H563" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I563" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260704-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J563" s="3" t="inlineStr"/>
+    </row>
+    <row r="564">
+      <c r="A564" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B564" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C564" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D564" s="3" t="inlineStr">
+        <is>
+          <t>The Engine Room Problem And Why Machinery Failure Remains Shipping's Dominant Risk</t>
+        </is>
+      </c>
+      <c r="E564" s="3" t="inlineStr">
+        <is>
+          <t>Allianz Commercial 보고서에 따르면 선박의 기계 고장이 해운 산업에서 여전히 가장 큰 위험 요소로, 전체 손실 감소 추세에도 불구하고 사고의 주요 원인으로 지목됩니다.</t>
+        </is>
+      </c>
+      <c r="F564" s="3" t="inlineStr">
+        <is>
+          <t>선박 기계 고장은 해상 운송 지연 및 화물 손상으로 이어질 수 있어 우리 회사의 물류 스케줄과 비용에 잠재적 영향을 미칠 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G564" s="3" t="inlineStr">
+        <is>
+          <t>주요 선사들의 선박 유지보수 현황 및 사고 발생률 추이를 지속적으로 모니터링하고, 운송 계약 시 보험 조건 및 비상 계획을 검토합니다.</t>
+        </is>
+      </c>
+      <c r="H564" s="3" t="inlineStr">
+        <is>
+          <t>gCaptain</t>
+        </is>
+      </c>
+      <c r="I564" s="3" t="inlineStr">
+        <is>
+          <t>https://gcaptain.com/the-engine-room-problem-and-why-machinery-failure-remains-shippings-dominant-risk</t>
+        </is>
+      </c>
+      <c r="J564" s="3" t="inlineStr"/>
+    </row>
+    <row r="565">
+      <c r="A565" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B565" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C565" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D565" s="3" t="inlineStr">
+        <is>
+          <t>'배터리구독형' 전기차보조금 나온다…"전기차주·리스사 지원방식 검토"</t>
+        </is>
+      </c>
+      <c r="E565" s="3" t="inlineStr">
+        <is>
+          <t>기후부가 '배터리 구독형' 전기차 보조금 개편을 검토 중이며, 이는 전기차 구매 시 배터리 리스제를 도입하여 전기차 소유주와 리스사를 지원하는 방식을 포함합니다.</t>
+        </is>
+      </c>
+      <c r="F565" s="3" t="inlineStr">
+        <is>
+          <t>배터리 구독형 보조금 정책은 전기차 배터리 수요 및 유통 방식에 변화를 가져와 우리 회사의 생산 계획 및 물류 전략에 간접적인 영향을 미칠 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G565" s="3" t="inlineStr">
+        <is>
+          <t>관련 정책의 구체적인 내용과 시행 시기를 지속적으로 모니터링하고, 배터리 리스 모델 확산에 따른 물류 수요 변화 가능성을 분석합니다.</t>
+        </is>
+      </c>
+      <c r="H565" s="3" t="inlineStr">
+        <is>
+          <t>이투데이</t>
+        </is>
+      </c>
+      <c r="I565" s="3" t="inlineStr">
+        <is>
+          <t>https://etoday.co.kr/news/view/2600733</t>
+        </is>
+      </c>
+      <c r="J565" s="3" t="inlineStr"/>
+    </row>
+    <row r="566">
+      <c r="A566" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B566" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C566" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D566" s="3" t="inlineStr">
+        <is>
+          <t>6월 美서비스업 경기 확장세 둔화...물가 압력 줄고 고용 반등</t>
+        </is>
+      </c>
+      <c r="E566" s="3" t="inlineStr">
+        <is>
+          <t>6월 미국 서비스업 경기가 확장세를 유지했으나 둔화되었고, 이란과의 종전 협상으로 물가 압력이 줄고 고용이 반등하는 등 전반적인 경제 상황이 개선되는 조짐을 보입니다.</t>
+        </is>
+      </c>
+      <c r="F566" s="3" t="inlineStr">
+        <is>
+          <t>미국 경제의 둔화 및 물가 압력 변화는 글로벌 수요와 무역량에 영향을 미쳐 우리 회사의 수출입 물동량 및 운임 변동성에 간접적인 영향을 줄 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G566" s="3" t="inlineStr">
+        <is>
+          <t>미국 경제 지표 및 글로벌 무역 동향을 지속적으로 모니터링하여 향후 물동량 및 운임 변동 가능성에 대비합니다.</t>
+        </is>
+      </c>
+      <c r="H566" s="3" t="inlineStr">
+        <is>
+          <t>서울경제</t>
+        </is>
+      </c>
+      <c r="I566" s="3" t="inlineStr">
+        <is>
+          <t>https://sedaily.com/article/20064487</t>
+        </is>
+      </c>
+      <c r="J566" s="3" t="inlineStr"/>
+    </row>
+    <row r="567">
+      <c r="A567" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B567" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C567" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D567" s="3" t="inlineStr">
+        <is>
+          <t>관세청, 7703억 규모 무역안보 침해 범죄 적발...5개월 만에 최대</t>
+        </is>
+      </c>
+      <c r="E567" s="3" t="inlineStr">
+        <is>
+          <t>관세청이 올해 5월까지 7703억원 규모의 무역안보 침해 범죄를 적발했으며, 이는 지난해 연간 실적을 5개월 만에 넘어선 역대 최대 규모이다. 국산 둔갑 등 다양한 유형의 범죄가 포함되었다.</t>
+        </is>
+      </c>
+      <c r="F567" s="3" t="inlineStr">
+        <is>
+          <t>무역안보 침해 범죄 증가는 수출입 통관 절차 강화 및 잠재적 공급망 리스크를 야기할 수 있으므로 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G567" s="3" t="n"/>
+      <c r="H567" s="3" t="inlineStr">
+        <is>
+          <t>Newspim</t>
+        </is>
+      </c>
+      <c r="I567" s="3" t="inlineStr">
+        <is>
+          <t>https://newspim.com/news/view/20260706000195</t>
+        </is>
+      </c>
+      <c r="J567" s="3" t="inlineStr"/>
+    </row>
+    <row r="568">
+      <c r="A568" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B568" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C568" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D568" s="3" t="inlineStr">
+        <is>
+          <t>"안 팔면 우리가 만든다"…美 제재, 오히려 中 키웠다 [중국 반도체 굴기 2026 中]</t>
+        </is>
+      </c>
+      <c r="E568" s="3" t="inlineStr">
+        <is>
+          <t>미국의 제재에도 불구하고 중국은 화웨이 등을 중심으로 AI칩부터 메모리까지 반도체 국산화를 가속화하며 자체 생태계를 구축하고 있다. 이는 미국의 제재가 오히려 중국의 자립을 촉진하는 역효과를 낳고 있음을 시사한다.</t>
+        </is>
+      </c>
+      <c r="F568" s="3" t="inlineStr">
+        <is>
+          <t>미중 기술 패권 경쟁 심화는 배터리/전자부품 공급망에 지속적인 불확실성을 제공하며, 특정 부품의 조달처 다변화 및 기술 자립화 전략을 고려해야 할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G568" s="3" t="n"/>
+      <c r="H568" s="3" t="inlineStr">
+        <is>
+          <t>이투데이</t>
+        </is>
+      </c>
+      <c r="I568" s="3" t="inlineStr">
+        <is>
+          <t>https://etoday.co.kr/news/view/2600598</t>
+        </is>
+      </c>
+      <c r="J568" s="3" t="inlineStr"/>
+    </row>
+    <row r="569">
+      <c r="A569" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B569" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C569" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D569" s="3" t="inlineStr">
+        <is>
+          <t>[매일시론] 핵심광물, 공급망 위기에 미리 대비해야</t>
+        </is>
+      </c>
+      <c r="E569" s="3" t="inlineStr">
+        <is>
+          <t>중동 전쟁과 같은 지정학적 리스크는 에너지 및 핵심광물 공급망의 취약성을 드러내며, 2019년 일본의 반도체 소재 수출 규제 사례처럼 핵심광물 공급망 위기에 대한 사전 대비가 중요함을 강조한다.</t>
+        </is>
+      </c>
+      <c r="F569" s="3" t="inlineStr">
+        <is>
+          <t>배터리/전자부품 제조에 필수적인 핵심광물 공급망의 불안정성은 생산 계획 및 원가에 직접적인 영향을 미칠 수 있으므로, 공급망 다변화 및 재고 확보 전략을 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G569" s="3" t="n"/>
+      <c r="H569" s="3" t="inlineStr">
+        <is>
+          <t>울산매일</t>
+        </is>
+      </c>
+      <c r="I569" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iusm.co.kr/news/articleView.html?idxno=1065015</t>
+        </is>
+      </c>
+      <c r="J569" s="3" t="inlineStr"/>
+    </row>
+    <row r="570">
+      <c r="A570" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B570" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C570" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D570" s="3" t="inlineStr">
+        <is>
+          <t>[수출기업 생존기] ③ 팔도 "K-푸드 글로벌 인기 체감…정부 적극 지원 필요"(인터뷰)</t>
+        </is>
+      </c>
+      <c r="E570" s="3" t="inlineStr">
+        <is>
+          <t>반도체 수출 호조에도 불구하고 1500원대 고환율은 원자재와 부품을 수입하는 중소기업에 부담으로 작용하며, 수출 증가가 반드시 이익 증가로 이어지지 않는 상황이다.</t>
+        </is>
+      </c>
+      <c r="F570" s="3" t="inlineStr">
+        <is>
+          <t>고환율은 원자재 및 부품 수입 비용을 증가시켜 생산 원가에 영향을 미치므로, 환율 변동 추이를 지속적으로 모니터링하고 환 헤지 전략을 검토할 필요가 있다.</t>
+        </is>
+      </c>
+      <c r="G570" s="3" t="n"/>
+      <c r="H570" s="3" t="inlineStr">
+        <is>
+          <t>Newspim</t>
+        </is>
+      </c>
+      <c r="I570" s="3" t="inlineStr">
+        <is>
+          <t>https://www.newspim.com/news/view/20260704000044</t>
+        </is>
+      </c>
+      <c r="J570" s="3" t="inlineStr"/>
+    </row>
+    <row r="571">
+      <c r="A571" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B571" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C571" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D571" s="3" t="inlineStr">
+        <is>
+          <t>중동전쟁에 중기 절반 이상 "매출·이익 감소"</t>
+        </is>
+      </c>
+      <c r="E571" s="3" t="inlineStr">
+        <is>
+          <t>중소기업 절반 이상이 중동전쟁 등 국제 정세 변화로 인해 매출 및 이익 감소 등 심각한 경영 부담을 겪고 있다고 응답했다.</t>
+        </is>
+      </c>
+      <c r="F571" s="3" t="inlineStr">
+        <is>
+          <t>중동 전쟁은 유가 상승, 해상 운송 불안정 등 간접적인 물류 비용 증가 및 공급망 리스크를 유발할 수 있으므로, 관련 동향을 지속적으로 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G571" s="3" t="n"/>
+      <c r="H571" s="3" t="inlineStr">
+        <is>
+          <t>파이낸셜뉴스</t>
+        </is>
+      </c>
+      <c r="I571" s="3" t="inlineStr">
+        <is>
+          <t>https://fnnews.com/news/202607061451026856</t>
+        </is>
+      </c>
+      <c r="J571" s="3" t="inlineStr"/>
+    </row>
+    <row r="572">
+      <c r="A572" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B572" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C572" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D572" s="3" t="inlineStr">
+        <is>
+          <t>OPEC+ 5달 연속 증산에도 국제유가 하락 않고 그대로</t>
+        </is>
+      </c>
+      <c r="E572" s="3" t="inlineStr">
+        <is>
+          <t>OPEC+가 5달 연속 증산에 합의했음에도 불구하고 국제유가는 하락하지 않고 그대로 유지되고 있으며, 호르무즈 해협의 불확실성이 여전히 영향을 미치고 있다.</t>
+        </is>
+      </c>
+      <c r="F572" s="3" t="inlineStr">
+        <is>
+          <t>국제유가 안정화가 지연되고 호르무즈 해협의 지정학적 불확실성이 지속되면 해상/항공 운임 및 물류비용 상승 압박이 유지될 수 있으므로 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G572" s="3" t="n"/>
+      <c r="H572" s="3" t="inlineStr">
+        <is>
+          <t>매일경제</t>
+        </is>
+      </c>
+      <c r="I572" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mk.co.kr/news/world/12091614</t>
+        </is>
+      </c>
+      <c r="J572" s="3" t="inlineStr"/>
+    </row>
+    <row r="573">
+      <c r="A573" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B573" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C573" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D573" s="4" t="inlineStr">
+        <is>
+          <t>KMI, 북극 협력 네트워크 본격 출범</t>
+        </is>
+      </c>
+      <c r="E573" s="4" t="inlineStr">
+        <is>
+          <t>한국해양수산개발원(KMI)이 북극권과 비북극권 미래세대가 북극 정책, 환경, 해운 등을 학습하고 교류하는 '2026 북극아카데미'를 개최하며 북극 협력 네트워크를 본격 출범했다.</t>
+        </is>
+      </c>
+      <c r="F573" s="4" t="inlineStr">
+        <is>
+          <t>북극 항로 개발 및 협력은 장기적인 관점의 물류 전략으로, 당사의 현재 물류 운영에 즉각적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G573" s="4" t="n"/>
+      <c r="H573" s="4" t="inlineStr">
+        <is>
+          <t>cargonews</t>
+        </is>
+      </c>
+      <c r="I573" s="4" t="inlineStr">
+        <is>
+          <t>https://www.cargonews.co.kr/news/articleView.html?idxno=60456</t>
+        </is>
+      </c>
+      <c r="J573" s="4" t="inlineStr"/>
+    </row>
+    <row r="574">
+      <c r="A574" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B574" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C574" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D574" s="4" t="inlineStr">
+        <is>
+          <t>Global Schedule Reliability for May 2026 the Highest of the Year</t>
+        </is>
+      </c>
+      <c r="E574" s="4" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence 보고서에 따르면 2026년 5월 글로벌 선박 스케줄 신뢰도가 올해 최고치를 기록했다.</t>
+        </is>
+      </c>
+      <c r="F574" s="4" t="inlineStr">
+        <is>
+          <t>선박 스케줄 신뢰도 개선은 긍정적인 소식이지만, 이는 전반적인 추세이며 개별 항로의 지연 가능성은 여전히 존재하므로 당장 큰 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G574" s="4" t="n"/>
+      <c r="H574" s="4" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I574" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/395-global-schedule-reliability-for-may-2026-the-highest-of-the-year</t>
+        </is>
+      </c>
+      <c r="J574" s="4" t="inlineStr"/>
+    </row>
+    <row r="575">
+      <c r="A575" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B575" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C575" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D575" s="4" t="inlineStr">
+        <is>
+          <t>Decoding Gemini’s Mediterranean Surge</t>
+        </is>
+      </c>
+      <c r="E575" s="4" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence 분석에 따르면 Gemini Cooperation이 동서 컨테이너 선박 배치를 재조정하며 지중해 시장 점유율을 확대하고 있다.</t>
+        </is>
+      </c>
+      <c r="F575" s="4" t="inlineStr">
+        <is>
+          <t>특정 선사 얼라이언스의 선대 재배치 전략은 전반적인 시장에 미치는 영향이 제한적이며, 당사의 물류 운영에 직접적인 영향을 주지는 않는다.</t>
+        </is>
+      </c>
+      <c r="G575" s="4" t="n"/>
+      <c r="H575" s="4" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I575" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/392-decoding-gemini-s-mediterranean-surge</t>
+        </is>
+      </c>
+      <c r="J575" s="4" t="inlineStr"/>
+    </row>
+    <row r="576">
+      <c r="A576" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B576" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C576" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D576" s="4" t="inlineStr">
+        <is>
+          <t>인물 포커스/ SM그룹 대한해운, 민상기 전 건국대 총장 신임 대표이사 취임</t>
+        </is>
+      </c>
+      <c r="E576" s="4" t="inlineStr">
+        <is>
+          <t>SM그룹 대한해운에 민상기 전 건국대 총장이 신임 대표이사로 취임했으며, 조직 운영 및 인재 양성 전문가로서 기업 가치 제고와 지속 가능한 성장이 기대된다.</t>
+        </is>
+      </c>
+      <c r="F576" s="4" t="inlineStr">
+        <is>
+          <t>해운사의 경영진 교체 소식으로, 우리 회사의 물류 운영에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G576" s="4" t="n"/>
+      <c r="H576" s="4" t="inlineStr">
+        <is>
+          <t>shippingnews</t>
+        </is>
+      </c>
+      <c r="I576" s="4" t="inlineStr">
+        <is>
+          <t>https://www.shippingnewsnet.com/news/articleView.html?idxno=71057</t>
+        </is>
+      </c>
+      <c r="J576" s="4" t="inlineStr"/>
+    </row>
+    <row r="577">
+      <c r="A577" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B577" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C577" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D577" s="4" t="inlineStr">
+        <is>
+          <t>20260703 경제·물류 주요뉴스 (데일리스크랩)</t>
+        </is>
+      </c>
+      <c r="E577" s="4" t="inlineStr">
+        <is>
+          <t>마스오토가 부산항 물동량을 기반으로 트레일러 자율주행 상용화를 추진하며 2028년 화물 운송의 완전 무인화를 목표로 제시했다.</t>
+        </is>
+      </c>
+      <c r="F577" s="4" t="inlineStr">
+        <is>
+          <t>장기적인 물류 기술 혁신 소식으로, 당장 우리 회사의 물류 운영에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G577" s="4" t="n"/>
+      <c r="H577" s="4" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I577" s="4" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260703-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J577" s="4" t="inlineStr"/>
+    </row>
+    <row r="578">
+      <c r="A578" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B578" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C578" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D578" s="4" t="inlineStr">
+        <is>
+          <t>씨메스로보틱스 / ‘물류·제조 대형 수주 잇달아’ 피지컬 AI 기반 로봇 자동화 사업 가속</t>
+        </is>
+      </c>
+      <c r="E578" s="4" t="inlineStr">
+        <is>
+          <t>씨메스로보틱스가 쿠팡풀필먼트서비스 등 물류 및 제조 현장에서 피지컬 AI 기반 로봇 자동화 프로젝트를 연이어 수주하며 사업을 확대하고 있다.</t>
+        </is>
+      </c>
+      <c r="F578" s="4" t="inlineStr">
+        <is>
+          <t>물류 자동화 기술 도입 사례로, 우리 회사의 물류 운영에 당장 직접적인 영향은 없으나 장기적인 관점에서 참고할 만하다.</t>
+        </is>
+      </c>
+      <c r="G578" s="4" t="n"/>
+      <c r="H578" s="4" t="inlineStr">
+        <is>
+          <t>ulogistics</t>
+        </is>
+      </c>
+      <c r="I578" s="4" t="inlineStr">
+        <is>
+          <t>http://www.ulogistics.co.kr/test/board.php?board=all2&amp;command=body&amp;no=5202</t>
+        </is>
+      </c>
+      <c r="J578" s="4" t="inlineStr"/>
+    </row>
+    <row r="579">
+      <c r="A579" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B579" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C579" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D579" s="4" t="inlineStr">
+        <is>
+          <t>중국의 해상 장악에 맞서는 베트남의 40억 달러 '혼코아이' 사업</t>
+        </is>
+      </c>
+      <c r="E579" s="4" t="inlineStr">
+        <is>
+          <t>베트남이 중국의 해상 패권에 맞서 까마우성 혼코아이 섬에 40억 달러 규모의 해상 물류 거점을 개발하여 해상 물류 역량을 강화할 계획이다.</t>
+        </is>
+      </c>
+      <c r="F579" s="4" t="inlineStr">
+        <is>
+          <t>베트남의 장기적인 항만 인프라 개발 계획으로, 당장 우리 회사의 물류 운영에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G579" s="4" t="n"/>
+      <c r="H579" s="4" t="inlineStr">
+        <is>
+          <t>newspim</t>
+        </is>
+      </c>
+      <c r="I579" s="4" t="inlineStr">
+        <is>
+          <t>https://www.newspim.com/news/view/20260706000663</t>
+        </is>
+      </c>
+      <c r="J579" s="4" t="inlineStr"/>
+    </row>
+    <row r="580">
+      <c r="A580" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B580" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C580" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D580" s="4" t="inlineStr">
+        <is>
+          <t>[물류/항구] 호치민시, 연간 1,600만 톤 처리 규모 QTM 국제항 건설 시작</t>
+        </is>
+      </c>
+      <c r="E580" s="4" t="inlineStr">
+        <is>
+          <t>호치민시가 연간 1,600만 톤 처리 능력을 갖춘 QTM 국제항 건설을 시작했으며, 이는 까이멥-티바이 항만 클러스터 내에 위치한다.</t>
+        </is>
+      </c>
+      <c r="F580" s="4" t="inlineStr">
+        <is>
+          <t>베트남의 장기적인 항만 인프라 개발 계획으로, 당장 우리 회사의 물류 운영에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G580" s="4" t="n"/>
+      <c r="H580" s="4" t="inlineStr">
+        <is>
+          <t>goodmorningvietnam</t>
+        </is>
+      </c>
+      <c r="I580" s="4" t="inlineStr">
+        <is>
+          <t>https://goodmorningvietnam.co.kr/news/article.html?no=82498</t>
+        </is>
+      </c>
+      <c r="J580" s="4" t="inlineStr"/>
+    </row>
+    <row r="581">
+      <c r="A581" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B581" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C581" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D581" s="4" t="inlineStr">
+        <is>
+          <t>Asda’s supply chain woes bring lessons for IT project planning | Computer Weekly</t>
+        </is>
+      </c>
+      <c r="E581" s="4" t="inlineStr">
+        <is>
+          <t>Asda가 클라우드 기반 ERP 시스템 배포 준비에도 불구하고 수개월간 공급망 혼란을 겪었으며, 이는 IT 프로젝트 계획에 대한 교훈을 시사한다.</t>
+        </is>
+      </c>
+      <c r="F581" s="4" t="inlineStr">
+        <is>
+          <t>특정 기업의 내부 IT 시스템 도입으로 인한 공급망 혼란 사례로, 우리 회사의 물류 운영에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G581" s="4" t="n"/>
+      <c r="H581" s="4" t="inlineStr">
+        <is>
+          <t>Computer Weekly</t>
+        </is>
+      </c>
+      <c r="I581" s="4" t="inlineStr">
+        <is>
+          <t>https://www.computerweekly.com/news/366645382/Asdas-supply-chain-woes-bring-lessons-for-IT-project-planning</t>
+        </is>
+      </c>
+      <c r="J581" s="4" t="inlineStr"/>
+    </row>
+    <row r="582">
+      <c r="A582" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B582" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C582" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D582" s="4" t="inlineStr">
+        <is>
+          <t>Time for meaningful integration of AI at scale, not incremental experimentation: Mahindra Group CEO &amp; MD Anish Shah - The Economic Times</t>
+        </is>
+      </c>
+      <c r="E582" s="4" t="inlineStr">
+        <is>
+          <t>Mahindra Group CEO는 공급망 문제와 비용 변동성 등 글로벌 불확실성 속에서 AI의 점진적 실험이 아닌 대규모 통합의 필요성을 강조했다.</t>
+        </is>
+      </c>
+      <c r="F582" s="4" t="inlineStr">
+        <is>
+          <t>AI 기술의 대규모 통합 필요성에 대한 경영진의 의견으로, 우리 회사의 물류 운영에 당장 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G582" s="4" t="n"/>
+      <c r="H582" s="4" t="inlineStr">
+        <is>
+          <t>The Economic Times</t>
+        </is>
+      </c>
+      <c r="I582" s="4" t="inlineStr">
+        <is>
+          <t>https://economictimes.indiatimes.com/news/company/corporate-trends/time-for-meaningful-integration-of-ai-at-scale-not-incremental-experimentation-mahinda-group-ceo-md-anish-shah/articleshow/132219812.cms</t>
+        </is>
+      </c>
+      <c r="J582" s="4" t="inlineStr"/>
+    </row>
+    <row r="583">
+      <c r="A583" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B583" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C583" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D583" s="4" t="inlineStr">
+        <is>
+          <t>[르포] 광주 군공항이 반도체 클러스터로..."40년 만의 천지개벽" 주민 환호</t>
+        </is>
+      </c>
+      <c r="E583" s="4" t="inlineStr">
+        <is>
+          <t>광주 군공항 이전 부지에 반도체 클러스터 조성이 추진되면서 지역 주민들의 기대가 높으며, 이는 40년 만의 대규모 개발로 평가됩니다.</t>
+        </is>
+      </c>
+      <c r="F583" s="4" t="inlineStr">
+        <is>
+          <t>반도체 클러스터 조성은 장기적인 관점에서 물류 인프라 및 수요 변화를 가져올 수 있으나, 당장 우리 회사의 물류 운영에 직접적인 영향은 없습니다.</t>
+        </is>
+      </c>
+      <c r="G583" s="4" t="n"/>
+      <c r="H583" s="4" t="inlineStr">
+        <is>
+          <t>뉴스핌</t>
+        </is>
+      </c>
+      <c r="I583" s="4" t="inlineStr">
+        <is>
+          <t>https://www.newspim.com/news/view/20260706001183</t>
+        </is>
+      </c>
+      <c r="J583" s="4" t="inlineStr"/>
+    </row>
+    <row r="584">
+      <c r="A584" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B584" s="4" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C584" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D584" s="4" t="inlineStr">
+        <is>
+          <t>[손바닥 경제] 전쟁발 가격 변동 방어 전략… 항공사마다 천차만별</t>
+        </is>
+      </c>
+      <c r="E584" s="4" t="inlineStr">
+        <is>
+          <t>항공사들이 유가 변동에 대비하기 위해 다양한 헤지 전략을 사용하고 있으며, 이는 국가별, 회사별로 천차만별이다.</t>
+        </is>
+      </c>
+      <c r="F584" s="4" t="inlineStr">
+        <is>
+          <t>항공사의 유가 헤지 전략은 항공 운임 안정화에 기여할 수 있으나, 우리 회사의 직접적인 물류 비용에 미치는 영향은 간접적이고 제한적이다.</t>
+        </is>
+      </c>
+      <c r="G584" s="4" t="n"/>
+      <c r="H584" s="4" t="inlineStr">
+        <is>
+          <t>부산일보</t>
+        </is>
+      </c>
+      <c r="I584" s="4" t="inlineStr">
+        <is>
+          <t>https://busan.com/view/busan/view.php?code=2026070617274859854</t>
+        </is>
+      </c>
+      <c r="J584" s="4" t="inlineStr"/>
+    </row>
+    <row r="585">
+      <c r="A585" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B585" s="4" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C585" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D585" s="4" t="inlineStr">
+        <is>
+          <t>檢 "싸게 산 원유 놔두고 인상"…업계 "국제유가 반영"</t>
+        </is>
+      </c>
+      <c r="E585" s="4" t="inlineStr">
+        <is>
+          <t>검찰이 정유 4사의 담합 및 갑질 혐의로 기소했으나, 정유업계는 국제유가 반영 및 산업 특성을 고려해야 한다고 반박하며 비축분 판매 시 운영자금 부족 등을 주장하고 있다.</t>
+        </is>
+      </c>
+      <c r="F585" s="4" t="inlineStr">
+        <is>
+          <t>국내 정유사 간의 가격 담합 논란은 국내 유가에 영향을 줄 수 있으나, 국제 유가 및 해상/항공 운임에 미치는 직접적인 영향은 제한적이다.</t>
+        </is>
+      </c>
+      <c r="G585" s="4" t="n"/>
+      <c r="H585" s="4" t="inlineStr">
+        <is>
+          <t>매일경제</t>
+        </is>
+      </c>
+      <c r="I585" s="4" t="inlineStr">
+        <is>
+          <t>https://www.mk.co.kr/news/society/12091572</t>
+        </is>
+      </c>
+      <c r="J585" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -26574,7 +28094,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -27065,6 +28585,49 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>3326.87</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>+87 (+2.7%)</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>+1,457 (+77.9%)</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>4330</v>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>+410 (+10.5%)</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>+1,619 (+59.7%)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -27077,7 +28640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I90"/>
+  <dimension ref="A1:I93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -30253,6 +31816,111 @@
       </c>
       <c r="I90" s="6" t="inlineStr"/>
     </row>
+    <row r="91">
+      <c r="A91" s="6" t="inlineStr">
+        <is>
+          <t>RSK-090</t>
+        </is>
+      </c>
+      <c r="B91" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="C91" s="6" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="D91" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E91" s="6" t="inlineStr">
+        <is>
+          <t>제다항 혼잡, 육상 물류망 마비…선사들 예약 중단</t>
+        </is>
+      </c>
+      <c r="F91" s="6" t="inlineStr"/>
+      <c r="G91" s="6" t="inlineStr"/>
+      <c r="H91" s="6" t="inlineStr">
+        <is>
+          <t>중동 지역 운송 예정 물량의 대체 항만 및 운송 경로 확인, 선사와의 긴밀한 소통을 통한 스케줄 조정 및 비용 영향 분석.</t>
+        </is>
+      </c>
+      <c r="I91" s="6" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="6" t="inlineStr">
+        <is>
+          <t>RSK-091</t>
+        </is>
+      </c>
+      <c r="B92" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="C92" s="6" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="D92" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E92" s="6" t="inlineStr">
+        <is>
+          <t>20260706 경제·물류 주요뉴스 (데일리스크랩)</t>
+        </is>
+      </c>
+      <c r="F92" s="6" t="inlineStr"/>
+      <c r="G92" s="6" t="inlineStr"/>
+      <c r="H92" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 관련 중동 정세 및 해운 동향을 면밀히 모니터링하고, 비상시 대체 운송 경로 및 재고 확보 방안을 검토해야 한다.</t>
+        </is>
+      </c>
+      <c r="I92" s="6" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="6" t="inlineStr">
+        <is>
+          <t>RSK-092</t>
+        </is>
+      </c>
+      <c r="B93" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="C93" s="6" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="D93" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E93" s="6" t="inlineStr">
+        <is>
+          <t>20260703 경제·물류 주요뉴스 (데일리스크랩)</t>
+        </is>
+      </c>
+      <c r="F93" s="6" t="inlineStr"/>
+      <c r="G93" s="6" t="inlineStr"/>
+      <c r="H93" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 통행료 부과 논의 진행 상황을 면밀히 모니터링하고, 예상되는 추가 물류비용을 분석하여 예산 및 운송 계획에 반영해야 한다.</t>
+        </is>
+      </c>
+      <c r="I93" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
📰 뉴스 데이터 2026-07-08_08:58
</commit_message>
<xml_diff>
--- a/data/SCM_물류_브리핑.xlsx
+++ b/data/SCM_물류_브리핑.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J585"/>
+  <dimension ref="A1:J617"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -28082,6 +28082,1538 @@
       </c>
       <c r="J585" s="4" t="inlineStr"/>
     </row>
+    <row r="586">
+      <c r="A586" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B586" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C586" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D586" s="2" t="inlineStr">
+        <is>
+          <t>[surff] 20260708 경제·물류 주요뉴스 (데일리스크랩)</t>
+        </is>
+      </c>
+      <c r="E586" s="2" t="inlineStr">
+        <is>
+          <t>미군이 호르무즈 해협 선박 피격에 대한 보복으로 이란 공습을 시작하고 미국이 이란 원유 제재 면제를 철회하며 중동 긴장이 고조되고, 국제유가가 급등했다.</t>
+        </is>
+      </c>
+      <c r="F586" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협의 군사적 긴장 고조는 주요 해상 운송로의 안전을 위협하고 유가 및 해상 운임 상승을 유발하여 물류 운영에 즉각적인 차질과 비용 증가를 초래할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G586" s="2" t="inlineStr">
+        <is>
+          <t>중동 항로 이용 선박의 스케줄 및 운임 변동성 실시간 모니터링 강화, 대체 운송 경로 및 재고 확보 방안 검토, 유가 변동에 따른 물류비 예산 재검토.</t>
+        </is>
+      </c>
+      <c r="H586" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I586" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260708-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J586" s="2" t="inlineStr">
+        <is>
+          <t>RSK-093</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B587" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C587" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D587" s="2" t="inlineStr">
+        <is>
+          <t>[surff] 20260706 경제·물류 주요뉴스 (데일리스크랩)</t>
+        </is>
+      </c>
+      <c r="E587" s="2" t="inlineStr">
+        <is>
+          <t>산업연구원은 호르무즈 해협 봉쇄 시 항로 우회, 선복 부족, 보험료 할증 등으로 한국 제조업 생산비가 4.7% 상승할 수 있다고 분석했으며, OPEC+는 증산을 이어가 내년 공급과잉 우려가 제기되고 있다.</t>
+        </is>
+      </c>
+      <c r="F587" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 봉쇄 시나리오는 물류비용 급증과 운송 지연을 야기하여 생산 계획 및 공급망 안정성에 심각한 영향을 미칠 수 있으며, 이는 배터리/전자부품 산업에도 동일하게 적용된다.</t>
+        </is>
+      </c>
+      <c r="G587" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 상황 변화에 대한 실시간 모니터링 강화, 비상 운송 계획 수립 (대체 항로, 항공 운송 옵션 등), 물류비 상승 시나리오별 재무 영향 분석.</t>
+        </is>
+      </c>
+      <c r="H587" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I587" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260706-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J587" s="2" t="inlineStr">
+        <is>
+          <t>RSK-094</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B588" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C588" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D588" s="2" t="inlineStr">
+        <is>
+          <t>[surff] 20260704 경제·물류 주요뉴스 (데일리스크랩)</t>
+        </is>
+      </c>
+      <c r="E588" s="2" t="inlineStr">
+        <is>
+          <t>중동발 불확실성으로 인한 물류비 부담이 삼성, LG 등 가전업계의 하반기 수익성에 부정적인 영향을 미칠 수 있다는 전망이 나왔다.</t>
+        </is>
+      </c>
+      <c r="F588" s="2" t="inlineStr">
+        <is>
+          <t>중동발 물류비 상승은 배터리/전자부품 제조기업에도 동일하게 적용되어, 운임 정상화 전까지 수익성 방어에 어려움을 겪을 수 있으므로 즉각적인 대응이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G588" s="2" t="inlineStr">
+        <is>
+          <t>중동발 물류비 상승 추이 및 운임 정상화 시점 모니터링, 물류비 절감 방안 및 비용 전가 가능성 검토, 재고 관리 최적화.</t>
+        </is>
+      </c>
+      <c r="H588" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I588" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260704-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J588" s="2" t="inlineStr">
+        <is>
+          <t>RSK-095</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B589" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C589" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D589" s="2" t="inlineStr">
+        <is>
+          <t>[search_운송지연_항만적체] 미주·유럽 항로 강세에 컨테이너 운임 상승 - 매일일보</t>
+        </is>
+      </c>
+      <c r="E589" s="2" t="inlineStr">
+        <is>
+          <t>미주 및 유럽 항로를 중심으로 컨테이너 운임이 상승하고 있으며, 성수기 전 물량을 앞당기려는 움직임으로 선복 확보 경쟁이 심화되고 있다.</t>
+        </is>
+      </c>
+      <c r="F589" s="2" t="inlineStr">
+        <is>
+          <t>주요 항로의 운임 상승 및 선복 확보 경쟁 심화는 우리 회사의 수출입 물류 비용 증가와 운송 지연 가능성을 높여 생산 및 출하 계획에 직접적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G589" s="2" t="inlineStr">
+        <is>
+          <t>주요 항로 운임 및 선복 상황 실시간 모니터링, 포워더와 긴밀히 협력하여 선복 확보 노력, 필요 시 장기 계약 또는 대체 운송 방안 검토.</t>
+        </is>
+      </c>
+      <c r="H589" s="2" t="inlineStr">
+        <is>
+          <t>매일일보</t>
+        </is>
+      </c>
+      <c r="I589" s="2" t="inlineStr">
+        <is>
+          <t>https://m-i.kr/news/articleView.html?idxno=1388959</t>
+        </is>
+      </c>
+      <c r="J589" s="2" t="inlineStr">
+        <is>
+          <t>RSK-096</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B590" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C590" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D590" s="2" t="inlineStr">
+        <is>
+          <t>"호르무즈서 유조선 3척 또 피격"…국제유가 '들썩’</t>
+        </is>
+      </c>
+      <c r="E590" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협에서 유조선 3척이 잇따라 피격당하며 중동 정세가 악화되고 국제유가가 상승할 조짐을 보이고 있다. 이는 주요 해상 운송로의 불안정성을 높인다.</t>
+        </is>
+      </c>
+      <c r="F590" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협은 주요 해상 운송로이자 유가 변동에 직접적인 영향을 미치므로, 물류비 상승 및 운송 지연 가능성에 즉시 대응해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G590" s="2" t="inlineStr">
+        <is>
+          <t>유가 및 해상 운임 변동 추이 실시간 모니터링, 비상 운송 계획 및 대체 경로 검토, 운송 계약 조건 재검토.</t>
+        </is>
+      </c>
+      <c r="H590" s="2" t="inlineStr">
+        <is>
+          <t>데일리안</t>
+        </is>
+      </c>
+      <c r="I590" s="2" t="inlineStr">
+        <is>
+          <t>https://dailian.co.kr/news/view/1664542/%ED%98%B8%EB%A5%B4%EB%AC%B4%EC%A6%88-%EB%98%90-%EB%9A%AB%EB%A0%B8%EB%8B%A4%EC%9C%A0%EC%A1%B0%EC%84%A0-3%EC%B2%99-%EB%8F%99%EC%8B%9C-2026</t>
+        </is>
+      </c>
+      <c r="J590" s="2" t="inlineStr">
+        <is>
+          <t>RSK-097</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B591" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C591" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D591" s="2" t="inlineStr">
+        <is>
+          <t>"美 관세는 '소나기' 아닌 '기후변화'…수출기업 전략 재편해야"</t>
+        </is>
+      </c>
+      <c r="E591" s="2" t="inlineStr">
+        <is>
+          <t>미국의 보호무역 강화가 일시적 현상이 아닌 구조적 변화로 자리 잡으면서, 한국 수출기업들은 공급망과 투자 전략 전반을 재편해야 한다는 전문가 진단이 나왔다.</t>
+        </is>
+      </c>
+      <c r="F591" s="2" t="inlineStr">
+        <is>
+          <t>미국 관세 정책 변화는 우리 회사의 수출 전략, 공급망 재편, 생산 거점 다변화 등 전반적인 사업 운영에 직접적인 영향을 미치므로 즉시 대응이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G591" s="2" t="inlineStr">
+        <is>
+          <t>미국 관세 및 통상 정책 변화 동향 면밀히 분석, 공급망 다변화 및 생산 거점 재배치 전략 검토, 무역 규제 준수 여부 점검.</t>
+        </is>
+      </c>
+      <c r="H591" s="2" t="inlineStr">
+        <is>
+          <t>이데일리</t>
+        </is>
+      </c>
+      <c r="I591" s="2" t="inlineStr">
+        <is>
+          <t>https://edaily.co.kr/News/Read?mediaCodeNo=257&amp;newsId=04093446645512224</t>
+        </is>
+      </c>
+      <c r="J591" s="2" t="inlineStr">
+        <is>
+          <t>RSK-098</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B592" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C592" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D592" s="2" t="inlineStr">
+        <is>
+          <t>[매일시론] 핵심광물, 공급망 위기에 미리 대비해야</t>
+        </is>
+      </c>
+      <c r="E592" s="2" t="inlineStr">
+        <is>
+          <t>중동 전쟁과 같은 지정학적 사건들이 에너지 및 핵심광물 공급망의 취약성을 드러내고 있으며, 과거 일본의 반도체 핵심소재 수출 규제 사례를 언급하며 공급망 위기에 대한 사전 대비의 중요성을 강조한다.</t>
+        </is>
+      </c>
+      <c r="F592" s="2" t="inlineStr">
+        <is>
+          <t>핵심광물 공급망 위기는 배터리 및 전자부품 제조에 필수적인 원자재 조달에 직접적인 영향을 미치므로, 즉각적인 공급망 리스크 분석 및 대응 전략 수립이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G592" s="2" t="inlineStr">
+        <is>
+          <t>핵심광물 조달처 다변화 및 재고 확보 전략 강화, 공급망 리스크 평가 및 비상 계획 수립, 관련 정부 정책 및 국제 동향 면밀히 주시.</t>
+        </is>
+      </c>
+      <c r="H592" s="2" t="inlineStr">
+        <is>
+          <t>울산매일</t>
+        </is>
+      </c>
+      <c r="I592" s="2" t="inlineStr">
+        <is>
+          <t>https://www.iusm.co.kr/news/articleView.html?idxno=1065015</t>
+        </is>
+      </c>
+      <c r="J592" s="2" t="inlineStr">
+        <is>
+          <t>RSK-099</t>
+        </is>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B593" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C593" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D593" s="2" t="inlineStr">
+        <is>
+          <t>저가 외국산 배터리 국산 가장 수출·핵심설비 유출 등 적발</t>
+        </is>
+      </c>
+      <c r="E593" s="2" t="inlineStr">
+        <is>
+          <t>관세청이 저가 외국산 배터리를 국산으로 둔갑시켜 우회 수출하거나 핵심 설비를 불법 유출하는 등 7천703억원 규모의 무역안보 침해 범죄를 적발했다. 이는 전략물자 불법 수출 및 원산지 위반 사례를 포함한다.</t>
+        </is>
+      </c>
+      <c r="F593" s="2" t="inlineStr">
+        <is>
+          <t>배터리 제조기업으로서 원산지 위반 및 전략물자 불법 수출 적발 사례는 우리 기업의 수출 프로세스 및 컴플라이언스에 직접적인 위험을 초래할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G593" s="2" t="inlineStr">
+        <is>
+          <t>수출 품목의 원산지 관리 강화 및 전략물자 수출 규제 준수 여부 재점검, 내부 컴플라이언스 교육 강화.</t>
+        </is>
+      </c>
+      <c r="H593" s="2" t="inlineStr">
+        <is>
+          <t>한국세정신문</t>
+        </is>
+      </c>
+      <c r="I593" s="2" t="inlineStr">
+        <is>
+          <t>https://taxtimes.co.kr/news/article.html?no=275862</t>
+        </is>
+      </c>
+      <c r="J593" s="2" t="inlineStr">
+        <is>
+          <t>RSK-100</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B594" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C594" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D594" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 선박 잇단 피격에 국제유가 급등…브렌트유 3%↑</t>
+        </is>
+      </c>
+      <c r="E594" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 인근에서 LNG 운반선과 유조선이 잇달아 피격당하고 미국 정부의 이란산 원유 제재 가능성이 제기되면서 국제유가가 급등했다.</t>
+        </is>
+      </c>
+      <c r="F594" s="2" t="inlineStr">
+        <is>
+          <t>주요 해상 운송로인 호르무즈 해협의 불안정으로 인한 국제유가 급등은 해상 및 항공 운임 상승으로 이어져 물류비용에 즉각적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G594" s="2" t="inlineStr">
+        <is>
+          <t>유가 변동에 따른 운임 인상 가능성을 대비하여 운송 계약 조건 재검토, 대체 운송 경로 및 모드 검토, 재고 수준 조정 검토.</t>
+        </is>
+      </c>
+      <c r="H594" s="2" t="inlineStr">
+        <is>
+          <t>헤럴드경제</t>
+        </is>
+      </c>
+      <c r="I594" s="2" t="inlineStr">
+        <is>
+          <t>https://biz.heraldcorp.com/article/10801448</t>
+        </is>
+      </c>
+      <c r="J594" s="2" t="inlineStr">
+        <is>
+          <t>RSK-101</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B595" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C595" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D595" s="3" t="inlineStr">
+        <is>
+          <t>Air Cargo Demand Up 6.0% in May (PRESSROOM)</t>
+        </is>
+      </c>
+      <c r="E595" s="3" t="inlineStr">
+        <is>
+          <t>2026년 5월 전 세계 항공 화물 수요가 전년 대비 6.0% 증가하여 항공 화물 시장의 견조한 성장을 보였다.</t>
+        </is>
+      </c>
+      <c r="F595" s="3" t="inlineStr">
+        <is>
+          <t>항공 화물 수요 증가는 향후 항공 운임 상승 압력으로 작용할 수 있으므로 지속적인 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G595" s="3" t="inlineStr">
+        <is>
+          <t>항공 운임 추이 및 가용성 지속 모니터링, 필요시 운송 계획 조정 검토.</t>
+        </is>
+      </c>
+      <c r="H595" s="3" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I595" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-29-air-cargo-demand-up-may/</t>
+        </is>
+      </c>
+      <c r="J595" s="3" t="inlineStr"/>
+    </row>
+    <row r="596">
+      <c r="A596" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B596" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C596" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D596" s="3" t="inlineStr">
+        <is>
+          <t>PLSCI Data Indicates Mega-Hub Retrenchment (PRESS ROOM)</t>
+        </is>
+      </c>
+      <c r="E596" s="3" t="inlineStr">
+        <is>
+          <t>UNCTAD의 2026년 2분기 항만 정기선 연결성 지수(PLSCI) 분석 결과, 최근 해운 네트워크 재조정이 메가 허브 항만의 후퇴를 시사하며, 이는 항만 연결성 및 효율성에 영향을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="F596" s="3" t="inlineStr">
+        <is>
+          <t>주요 항만 네트워크의 변화는 당사의 운송 경로 및 리드타임에 영향을 미칠 수 있으므로, 주요 항만의 연결성 변화를 지속적으로 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G596" s="3" t="inlineStr">
+        <is>
+          <t>주요 항만 연결성 지표 및 선사 서비스 변경 동향 모니터링.</t>
+        </is>
+      </c>
+      <c r="H596" s="3" t="inlineStr">
+        <is>
+          <t>sea-intelligence</t>
+        </is>
+      </c>
+      <c r="I596" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/396-plsci-data-indicates-mega-hub-retrenchment</t>
+        </is>
+      </c>
+      <c r="J596" s="3" t="inlineStr"/>
+    </row>
+    <row r="597">
+      <c r="A597" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B597" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C597" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D597" s="3" t="inlineStr">
+        <is>
+          <t>Tracking True Vessel Delay (PRESS ROOM)</t>
+        </is>
+      </c>
+      <c r="E597" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence 분석에 따르면 선사들이 운송 시간을 늘리는 스케줄 버퍼링을 통해 정시 도착률을 높이고 있으며, 이는 실제 운송 지연과 스케줄 상의 지연 간의 관계를 분석하는 데 중요함을 시사한다.</t>
+        </is>
+      </c>
+      <c r="F597" s="3" t="inlineStr">
+        <is>
+          <t>선사들의 스케줄 버퍼링 전략은 실제 운송 리드타임에 영향을 미칠 수 있으므로, 운송 계획 수립 시 이를 고려하고 선사별 실제 운송 시간을 지속적으로 확인해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G597" s="3" t="inlineStr">
+        <is>
+          <t>선사별 실제 운송 리드타임 데이터 분석 및 운송 계획에 반영, 잠재적 리드타임 증가 가능성 고려.</t>
+        </is>
+      </c>
+      <c r="H597" s="3" t="inlineStr">
+        <is>
+          <t>sea-intelligence</t>
+        </is>
+      </c>
+      <c r="I597" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/394-tracking-true-vessel-delay</t>
+        </is>
+      </c>
+      <c r="J597" s="3" t="inlineStr"/>
+    </row>
+    <row r="598">
+      <c r="A598" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B598" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C598" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D598" s="3" t="inlineStr">
+        <is>
+          <t>Transpacific: Ripe for new non-alliance services (PRESS ROOM)</t>
+        </is>
+      </c>
+      <c r="E598" s="3" t="inlineStr">
+        <is>
+          <t>태평양 횡단 항로에서 비동맹 선사들의 신규 서비스 도입 가능성이 높아지고 있으며, 이는 운임 경쟁 심화 및 서비스 옵션 확대로 이어질 수 있다.</t>
+        </is>
+      </c>
+      <c r="F598" s="3" t="inlineStr">
+        <is>
+          <t>태평양 횡단 항로의 신규 서비스 증가는 운임 경쟁을 유발하고 운송 옵션을 다양화할 수 있으므로, 운임 및 서비스 동향을 모니터링하여 최적의 운송 방안을 모색해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G598" s="3" t="inlineStr">
+        <is>
+          <t>태평양 횡단 항로의 신규 선사 서비스 및 운임 동향 모니터링, 잠재적 운송 파트너십 검토.</t>
+        </is>
+      </c>
+      <c r="H598" s="3" t="inlineStr">
+        <is>
+          <t>sea-intelligence</t>
+        </is>
+      </c>
+      <c r="I598" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/393-transpacific-ripe-for-new-non-alliance-services</t>
+        </is>
+      </c>
+      <c r="J598" s="3" t="inlineStr"/>
+    </row>
+    <row r="599">
+      <c r="A599" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B599" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C599" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D599" s="3" t="inlineStr">
+        <is>
+          <t>[surff] 20260707 경제·물류 주요뉴스 (데일리스크랩)</t>
+        </is>
+      </c>
+      <c r="E599" s="3" t="inlineStr">
+        <is>
+          <t>OPEC+ 증산 전망으로 국제유가가 소폭 하락했으나, 우크라이나 드론이 러시아 정유시설을 공격하며 유가 변동성이 지속되고 있다.</t>
+        </is>
+      </c>
+      <c r="F599" s="3" t="inlineStr">
+        <is>
+          <t>유가 변동성은 물류비에 직접적인 영향을 미치므로, 공급 증가 요인과 지정학적 불안 요인이 상존하는 상황에서 유가 추이를 지속적으로 관찰해야 한다.</t>
+        </is>
+      </c>
+      <c r="G599" s="3" t="inlineStr">
+        <is>
+          <t>국제유가 및 유류할증료 추이 지속 모니터링.</t>
+        </is>
+      </c>
+      <c r="H599" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I599" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260707-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J599" s="3" t="inlineStr"/>
+    </row>
+    <row r="600">
+      <c r="A600" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B600" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C600" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D600" s="3" t="inlineStr">
+        <is>
+          <t>[surff] 25만 원 이하 직구도 이제 관세? EU 소액면세 폐지가 바꾸는 것들 (Week 27, 2026) (물류101)</t>
+        </is>
+      </c>
+      <c r="E600" s="3" t="inlineStr">
+        <is>
+          <t>EU가 150유로 이하 소포에 대한 소액면세 제도를 폐지하여, 유럽으로 수출되는 소량 샘플 및 부품 수출 시 관세 부담이 발생할 수 있다.</t>
+        </is>
+      </c>
+      <c r="F600" s="3" t="inlineStr">
+        <is>
+          <t>대량 B2B 수출에는 영향이 적지만, 소량 샘플, R&amp;D용 부품, 또는 특정 고객향 소액 주문의 경우 관세 부담이 발생하여 물류 프로세스 및 비용에 영향을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="G600" s="3" t="inlineStr">
+        <is>
+          <t>EU향 소량/소액 수출 건에 대한 관세 영향 분석 및 통관 절차 변화 숙지, 필요 시 고객 또는 포워더와 협의.</t>
+        </is>
+      </c>
+      <c r="H600" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I600" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/25만-원-이하-직구도-이제-관세-eu-소액면세-폐지가-바꾸는-것들-week-27-2026-</t>
+        </is>
+      </c>
+      <c r="J600" s="3" t="inlineStr"/>
+    </row>
+    <row r="601">
+      <c r="A601" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B601" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C601" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D601" s="3" t="inlineStr">
+        <is>
+          <t>[search_운송지연_항만적체] Fuel Price Volatility Is Creating A New Cross-border Challenge For SMEs | africa.com</t>
+        </is>
+      </c>
+      <c r="E601" s="3" t="inlineStr">
+        <is>
+          <t>유가 변동성이 중소기업의 국경 간 물류 비용에 새로운 도전 과제를 안겨주고 있으며, 이는 운송 및 물류 비용을 넘어 공급망 전반에 영향을 미치고 있다.</t>
+        </is>
+      </c>
+      <c r="F601" s="3" t="inlineStr">
+        <is>
+          <t>유가 변동성은 모든 기업의 물류비에 영향을 미치므로, 지속적인 모니터링이 필요하며, 특히 배터리/전자부품은 정밀 운송이 많아 유가 변동에 민감할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G601" s="3" t="inlineStr">
+        <is>
+          <t>국제유가 및 유류할증료 추이 지속 모니터링, 물류비 예산에 유가 변동성 반영 검토.</t>
+        </is>
+      </c>
+      <c r="H601" s="3" t="inlineStr">
+        <is>
+          <t>africa.com</t>
+        </is>
+      </c>
+      <c r="I601" s="3" t="inlineStr">
+        <is>
+          <t>https://www.africa.com/business/fuel-price-volatility-is-creating-a-new-cross-border-challenge-for-smes</t>
+        </is>
+      </c>
+      <c r="J601" s="3" t="inlineStr"/>
+    </row>
+    <row r="602">
+      <c r="A602" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B602" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C602" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D602" s="3" t="inlineStr">
+        <is>
+          <t>리튬배터리 PM 도시철도 반입 금지… 심야 갓길에 대리기사들 ‘위험한 질주’ 늘어나</t>
+        </is>
+      </c>
+      <c r="E602" s="3" t="inlineStr">
+        <is>
+          <t>전국 도시철도 운영기관들이 대용량(160Wh 초과) 리튬배터리 장착 개인형 이동장치(PM)의 역사 및 열차 내 반입을 전면 금지했다. 이는 지하철 밀폐 공간에서의 화재 위험을 막기 위한 조치이다.</t>
+        </is>
+      </c>
+      <c r="F602" s="3" t="inlineStr">
+        <is>
+          <t>리튬배터리 운송 및 보관에 대한 규제가 강화되는 추세로, 향후 물류 운송 방식 및 창고 보관 기준에 영향을 줄 수 있어 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G602" s="3" t="inlineStr">
+        <is>
+          <t>리튬배터리 운송 관련 국내외 규제 동향 지속 모니터링 및 내부 운송/보관 절차 점검.</t>
+        </is>
+      </c>
+      <c r="H602" s="3" t="inlineStr">
+        <is>
+          <t>대구일보</t>
+        </is>
+      </c>
+      <c r="I602" s="3" t="inlineStr">
+        <is>
+          <t>https://idaegu.com/news/articleView.html?idxno=664159</t>
+        </is>
+      </c>
+      <c r="J602" s="3" t="inlineStr"/>
+    </row>
+    <row r="603">
+      <c r="A603" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B603" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C603" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D603" s="3" t="inlineStr">
+        <is>
+          <t>[충북일보] 영동소방서 "위험물 안전관리 노하우 찾습니다"</t>
+        </is>
+      </c>
+      <c r="E603" s="3" t="inlineStr">
+        <is>
+          <t>영동소방서가 소방청 주최의 위험물 안전관리 노하우 공모전을 홍보하며, 위험물 사고 예방을 위한 현장 경험 공유의 중요성을 강조했다. 위험물 사고는 대형 화재나 인명피해로 이어질 가능성이 크다.</t>
+        </is>
+      </c>
+      <c r="F603" s="3" t="inlineStr">
+        <is>
+          <t>위험물 안전관리에 대한 사회적 관심과 규제 강화 움직임을 보여주며, 우리 회사의 위험물 취급 및 보관 절차에 대한 지속적인 점검과 개선이 필요함을 시사합니다.</t>
+        </is>
+      </c>
+      <c r="G603" s="3" t="inlineStr">
+        <is>
+          <t>내부 위험물 안전관리 절차 및 교육 프로그램 점검, 최신 안전관리 노하우 및 기술 도입 검토.</t>
+        </is>
+      </c>
+      <c r="H603" s="3" t="inlineStr">
+        <is>
+          <t>충북일보</t>
+        </is>
+      </c>
+      <c r="I603" s="3" t="inlineStr">
+        <is>
+          <t>https://www.inews365.com/news/article.html?no=926338</t>
+        </is>
+      </c>
+      <c r="J603" s="3" t="inlineStr"/>
+    </row>
+    <row r="604">
+      <c r="A604" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B604" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C604" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D604" s="3" t="inlineStr">
+        <is>
+          <t>[Moonshot-thinking] 공급 절벽 앞에서…물류센터 시장이 나뉜다</t>
+        </is>
+      </c>
+      <c r="E604" s="3" t="inlineStr">
+        <is>
+          <t>10년 전 대형으로 평가받던 물류센터가 현재는 일반적인 수준이 될 정도로 물류센터 시장의 규모와 기준이 변화하고 있으며, 공급 절벽과 함께 시장이 재편되고 있다.</t>
+        </is>
+      </c>
+      <c r="F604" s="3" t="inlineStr">
+        <is>
+          <t>물류센터 시장의 변화는 향후 우리 회사의 창고 확보 전략 및 물류 네트워크 구축에 영향을 미칠 수 있으므로 추이를 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G604" s="3" t="inlineStr">
+        <is>
+          <t>물류센터 시장 동향 및 공급망 변화를 지속적으로 모니터링하고, 중장기 물류 거점 전략 재검토.</t>
+        </is>
+      </c>
+      <c r="H604" s="3" t="inlineStr">
+        <is>
+          <t>뉴스페이스</t>
+        </is>
+      </c>
+      <c r="I604" s="3" t="inlineStr">
+        <is>
+          <t>https://newsspace.kr/news/article.html?no=14420</t>
+        </is>
+      </c>
+      <c r="J604" s="3" t="inlineStr"/>
+    </row>
+    <row r="605">
+      <c r="A605" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B605" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C605" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D605" s="3" t="inlineStr">
+        <is>
+          <t>딥시크도 '자체 AI 반도체' 개발 추진…중국 '탈 엔비디아' 속도전</t>
+        </is>
+      </c>
+      <c r="E605" s="3" t="inlineStr">
+        <is>
+          <t>중국 AI 스타트업 딥시크가 자체 AI 반도체 개발을 추진하며 엔비디아 등 특정 반도체 의존도를 줄이려는 움직임을 보이고 있다. 이는 중국의 '탈 엔비디아' 전략의 일환이다.</t>
+        </is>
+      </c>
+      <c r="F605" s="3" t="inlineStr">
+        <is>
+          <t>특정 국가의 핵심 부품 자립화 및 공급망 재편 노력은 장기적으로 전자부품 시장의 공급 안정성 및 가격에 영향을 줄 수 있으므로 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G605" s="3" t="inlineStr">
+        <is>
+          <t>글로벌 반도체 및 전자부품 공급망 동향 지속 모니터링, 잠재적 공급 리스크에 대비한 부품 조달 전략 검토.</t>
+        </is>
+      </c>
+      <c r="H605" s="3" t="inlineStr">
+        <is>
+          <t>뉴스핌</t>
+        </is>
+      </c>
+      <c r="I605" s="3" t="inlineStr">
+        <is>
+          <t>https://www.newspim.com/news/view/20260707001248</t>
+        </is>
+      </c>
+      <c r="J605" s="3" t="inlineStr"/>
+    </row>
+    <row r="606">
+      <c r="A606" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B606" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C606" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D606" s="3" t="inlineStr">
+        <is>
+          <t>중동전쟁에 중기 절반 이상 "매출·이익 감소"</t>
+        </is>
+      </c>
+      <c r="E606" s="3" t="inlineStr">
+        <is>
+          <t>중소기업 절반 이상이 중동전쟁 등 국제 정세 변화로 인해 매출 및 이익 감소 등 심각한 경영 부담을 겪고 있다고 응답했다.</t>
+        </is>
+      </c>
+      <c r="F606" s="3" t="inlineStr">
+        <is>
+          <t>중동 분쟁으로 인한 전반적인 경제적 부담 증가는 우리 회사의 물류비 상승 및 공급망 불안정성 심화로 이어질 수 있으므로 지속적인 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G606" s="3" t="inlineStr">
+        <is>
+          <t>중동 정세 변화에 따른 물류 비용 및 공급망 리스크 변화를 지속적으로 모니터링하고, 비상 계획을 점검.</t>
+        </is>
+      </c>
+      <c r="H606" s="3" t="inlineStr">
+        <is>
+          <t>파이낸셜뉴스</t>
+        </is>
+      </c>
+      <c r="I606" s="3" t="inlineStr">
+        <is>
+          <t>https://fnnews.com/news/202607061451026856</t>
+        </is>
+      </c>
+      <c r="J606" s="3" t="inlineStr"/>
+    </row>
+    <row r="607">
+      <c r="A607" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B607" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C607" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D607" s="3" t="inlineStr">
+        <is>
+          <t>[손바닥 경제] 전쟁발 가격 변동 방어 전략… 항공사마다 천차만별</t>
+        </is>
+      </c>
+      <c r="E607" s="3" t="inlineStr">
+        <is>
+          <t>항공사들이 전쟁 등으로 인한 유가 변동성에 대응하기 위해 다양한 유가 헤지 전략을 사용하고 있으며, 이는 항공사별로 천차만별이다.</t>
+        </is>
+      </c>
+      <c r="F607" s="3" t="inlineStr">
+        <is>
+          <t>항공사의 유가 헤지 전략은 항공 운임 안정성에 영향을 미치므로, 향후 항공 운송 비용 변동 추이를 예측하는 데 참고할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G607" s="3" t="inlineStr">
+        <is>
+          <t>항공 운송 계약 시 유류할증료 변동 조건 및 항공사별 헤지 전략 동향을 지속적으로 모니터링.</t>
+        </is>
+      </c>
+      <c r="H607" s="3" t="inlineStr">
+        <is>
+          <t>부산일보</t>
+        </is>
+      </c>
+      <c r="I607" s="3" t="inlineStr">
+        <is>
+          <t>https://busan.com/view/busan/view.php?code=2026070617274859854</t>
+        </is>
+      </c>
+      <c r="J607" s="3" t="inlineStr"/>
+    </row>
+    <row r="608">
+      <c r="A608" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B608" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C608" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D608" s="4" t="inlineStr">
+        <is>
+          <t>25년 만에 직배송 '결단'…쿠팡에 맞선 네이버 '초강수' (공통)</t>
+        </is>
+      </c>
+      <c r="E608" s="4" t="inlineStr">
+        <is>
+          <t>네이버가 쿠팡의 로켓배송에 대응하기 위해 자체 물류센터 구축 및 직배송 사업을 추진하며 국내 이커머스 물류 시장의 경쟁이 심화될 전망이다.</t>
+        </is>
+      </c>
+      <c r="F608" s="4" t="inlineStr">
+        <is>
+          <t>국내 이커머스 물류 시장의 변화는 당사 배터리/전자부품 제조 및 SCM 운영에 직접적인 영향은 없으며, 장기적인 시장 동향 참고 수준입니다.</t>
+        </is>
+      </c>
+      <c r="G608" s="4" t="n"/>
+      <c r="H608" s="4" t="inlineStr">
+        <is>
+          <t>kita</t>
+        </is>
+      </c>
+      <c r="I608" s="4" t="inlineStr">
+        <is>
+          <t>https://www.kita.net/shippers/board/newsView.do?morgueCode=2&amp;dataCls=A&amp;dataSeq=2530</t>
+        </is>
+      </c>
+      <c r="J608" s="4" t="inlineStr"/>
+    </row>
+    <row r="609">
+      <c r="A609" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B609" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C609" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D609" s="4" t="inlineStr">
+        <is>
+          <t>美 뉴욕∙뉴저지 항만청 450억 달러 투자, 교통 인프라 지형 바꾼다 (투자진출)</t>
+        </is>
+      </c>
+      <c r="E609" s="4" t="inlineStr">
+        <is>
+          <t>미국 뉴욕·뉴저지 항만청이 향후 10년간 450억 달러를 투자하여 교통 인프라를 재편할 계획이며, 이는 글로벌 물류 허브의 장기적인 효율성 개선에 기여할 것으로 예상된다.</t>
+        </is>
+      </c>
+      <c r="F609" s="4" t="inlineStr">
+        <is>
+          <t>장기적인 항만 인프라 개선 계획으로, 당장 물류 운영에 미치는 직접적인 영향은 없으나 향후 북미 지역 물류 효율성 증대에 긍정적 영향을 줄 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G609" s="4" t="n"/>
+      <c r="H609" s="4" t="inlineStr">
+        <is>
+          <t>kotra</t>
+        </is>
+      </c>
+      <c r="I609" s="4" t="inlineStr">
+        <is>
+          <t>https://dream.kotra.or.kr/kotranews/cms/news/actionKotraBoardDetail.do?SITE_NO=3&amp;MENU_ID=70&amp;CONTENTS_NO=1&amp;pNttSn=242672</t>
+        </is>
+      </c>
+      <c r="J609" s="4" t="inlineStr"/>
+    </row>
+    <row r="610">
+      <c r="A610" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B610" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C610" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D610" s="4" t="inlineStr">
+        <is>
+          <t>HMM, 비컨선사업 강화…2.4조규모 무더기 발주 (해운조선)</t>
+        </is>
+      </c>
+      <c r="E610" s="4" t="inlineStr">
+        <is>
+          <t>HMM이 2조 4천억 원 규모의 대형 벌크선, VLCC, VLGC 등 비컨테이너선 14척을 대량 발주하며 비컨테이너선 사업을 강화하고 있다.</t>
+        </is>
+      </c>
+      <c r="F610" s="4" t="inlineStr">
+        <is>
+          <t>HMM의 비컨테이너선 사업 강화는 당사의 컨테이너 운송에 직접적인 영향은 없으며, 해운 시장의 장기적인 동향을 파악하는 참고 자료입니다.</t>
+        </is>
+      </c>
+      <c r="G610" s="4" t="n"/>
+      <c r="H610" s="4" t="inlineStr">
+        <is>
+          <t>ksg</t>
+        </is>
+      </c>
+      <c r="I610" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksg.co.kr/news/main_newsView.jsp?pNum=147535</t>
+        </is>
+      </c>
+      <c r="J610" s="4" t="inlineStr"/>
+    </row>
+    <row r="611">
+      <c r="A611" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B611" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C611" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D611" s="4" t="inlineStr">
+        <is>
+          <t>Global Schedule Reliability for May 2026 the Highest of the Year (PRESS ROOM)</t>
+        </is>
+      </c>
+      <c r="E611" s="4" t="inlineStr">
+        <is>
+          <t>2026년 5월 전 세계 선박 스케줄 신뢰도가 올해 최고치를 기록하여 해상 운송의 정시성이 개선되고 있음을 나타낸다.</t>
+        </is>
+      </c>
+      <c r="F611" s="4" t="inlineStr">
+        <is>
+          <t>선박 스케줄 신뢰도 개선은 긍정적인 신호이나, 당사의 물류 운영에 즉각적인 변화를 요구하지는 않으며, 전반적인 해상 운송 환경 개선 추이를 참고합니다.</t>
+        </is>
+      </c>
+      <c r="G611" s="4" t="n"/>
+      <c r="H611" s="4" t="inlineStr">
+        <is>
+          <t>sea-intelligence</t>
+        </is>
+      </c>
+      <c r="I611" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/395-global-schedule-reliability-for-may-2026-the-highest-of-the-year</t>
+        </is>
+      </c>
+      <c r="J611" s="4" t="inlineStr"/>
+    </row>
+    <row r="612">
+      <c r="A612" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B612" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C612" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D612" s="4" t="inlineStr">
+        <is>
+          <t>[search_운송지연_항만적체] 중국의 해상 장악에 맞서는 베트남의 40억 달러 '혼코아이' 사업</t>
+        </is>
+      </c>
+      <c r="E612" s="4" t="inlineStr">
+        <is>
+          <t>베트남이 중국의 해상 패권에 맞서기 위해 40억 달러 규모의 해상 물류 거점 '혼코아이' 사업을 추진하며 동남아시아 지역의 물류 인프라를 강화하고 있다.</t>
+        </is>
+      </c>
+      <c r="F612" s="4" t="inlineStr">
+        <is>
+          <t>장기적인 동남아시아 물류 인프라 개선 소식이지만, 우리 회사의 즉각적인 물류 운영이나 생산 계획에는 직접적인 영향이 없다.</t>
+        </is>
+      </c>
+      <c r="G612" s="4" t="n"/>
+      <c r="H612" s="4" t="inlineStr">
+        <is>
+          <t>newspim</t>
+        </is>
+      </c>
+      <c r="I612" s="4" t="inlineStr">
+        <is>
+          <t>https://www.newspim.com/news/view/20260706000663</t>
+        </is>
+      </c>
+      <c r="J612" s="4" t="inlineStr"/>
+    </row>
+    <row r="613">
+      <c r="A613" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B613" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C613" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D613" s="4" t="inlineStr">
+        <is>
+          <t>[search_운송지연_항만적체] 전통적인 항구에 'AI 두뇌'를 탑재하면 생기는 일 - 오마이뉴스</t>
+        </is>
+      </c>
+      <c r="E613" s="4" t="inlineStr">
+        <is>
+          <t>중국 칭다오항이 AI 기술을 도입하여 항만 운영 효율성을 높이고 있으며, 이는 미래 항만 물류의 변화 방향을 보여준다.</t>
+        </is>
+      </c>
+      <c r="F613" s="4" t="inlineStr">
+        <is>
+          <t>AI 기반 항만 자동화는 장기적인 물류 효율성 향상에 기여할 수 있으나, 우리 회사의 현재 물류 운영에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G613" s="4" t="n"/>
+      <c r="H613" s="4" t="inlineStr">
+        <is>
+          <t>오마이뉴스</t>
+        </is>
+      </c>
+      <c r="I613" s="4" t="inlineStr">
+        <is>
+          <t>https://ohmynews.com/NWS_Web/View/at_pg.aspx?CMPT_CD=M0112&amp;CNTN_CD=A0003248545&amp;PAGE_CD=N0002</t>
+        </is>
+      </c>
+      <c r="J613" s="4" t="inlineStr"/>
+    </row>
+    <row r="614">
+      <c r="A614" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B614" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C614" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D614" s="4" t="inlineStr">
+        <is>
+          <t>[search_운송지연_항만적체] HMM, 유럽~서아프리카 노선 첫 출항 | 서울경제</t>
+        </is>
+      </c>
+      <c r="E614" s="4" t="inlineStr">
+        <is>
+          <t>HMM이 스페인과 서아프리카를 연결하는 신규 컨테이너 서비스 'MA2'를 첫 출항하며 노선 확장에 나섰다.</t>
+        </is>
+      </c>
+      <c r="F614" s="4" t="inlineStr">
+        <is>
+          <t>특정 해운사의 신규 노선 개설 소식으로, 우리 회사의 주력 운송 경로와 직접적인 관련이 없어 당장 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G614" s="4" t="n"/>
+      <c r="H614" s="4" t="inlineStr">
+        <is>
+          <t>서울경제</t>
+        </is>
+      </c>
+      <c r="I614" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sedaily.com/article/20064641</t>
+        </is>
+      </c>
+      <c r="J614" s="4" t="inlineStr"/>
+    </row>
+    <row r="615">
+      <c r="A615" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B615" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C615" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D615" s="4" t="inlineStr">
+        <is>
+          <t>[search_운송지연_항만적체] Why Smarter Supply Chains Are Also Lower-Emission Supply</t>
+        </is>
+      </c>
+      <c r="E615" s="4" t="inlineStr">
+        <is>
+          <t>지정학적 혼란, 무역 패턴 변화, 고객 기대치 및 기후 보고 요구사항 증가로 인해 공급망의 회복탄력성과 지속가능성 구축의 중요성이 커지고 있다.</t>
+        </is>
+      </c>
+      <c r="F615" s="4" t="inlineStr">
+        <is>
+          <t>장기적인 공급망 전략 방향에 대한 내용으로, 우리 회사의 즉각적인 물류 운영에 직접적인 영향은 없으나, 향후 전략 수립 시 참고할 만하다.</t>
+        </is>
+      </c>
+      <c r="G615" s="4" t="n"/>
+      <c r="H615" s="4" t="inlineStr">
+        <is>
+          <t>3blmedia.com</t>
+        </is>
+      </c>
+      <c r="I615" s="4" t="inlineStr">
+        <is>
+          <t>https://www.3blmedia.com/news/why-smarter-supply-chains-are-also-lower-emission-supply-chains</t>
+        </is>
+      </c>
+      <c r="J615" s="4" t="inlineStr"/>
+    </row>
+    <row r="616">
+      <c r="A616" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B616" s="4" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C616" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D616" s="4" t="inlineStr">
+        <is>
+          <t>[산업 View] 현장 점검에서 스마트 예방으로… 산업안전 패러다임 바뀐다</t>
+        </is>
+      </c>
+      <c r="E616" s="4" t="inlineStr">
+        <is>
+          <t>산업현장의 안전 관리가 사후 대응에서 설비 제어, 건강 모니터링, AI 기반 예방 기술을 결합하는 스마트 예방 방식으로 진화하고 있다. 이는 사고 발생 전 위험을 예측하고 방지하는 데 중점을 둔다.</t>
+        </is>
+      </c>
+      <c r="F616" s="4" t="inlineStr">
+        <is>
+          <t>당장 직접적인 물류 운영에 영향을 주지는 않지만, 장기적으로 물류센터 및 생산 현장의 안전 관리 시스템 고도화에 참고할 만한 동향입니다.</t>
+        </is>
+      </c>
+      <c r="G616" s="4" t="n"/>
+      <c r="H616" s="4" t="inlineStr">
+        <is>
+          <t>산업종합저널 FA</t>
+        </is>
+      </c>
+      <c r="I616" s="4" t="inlineStr">
+        <is>
+          <t>https://industryjournal.co.kr/news/246620</t>
+        </is>
+      </c>
+      <c r="J616" s="4" t="inlineStr"/>
+    </row>
+    <row r="617">
+      <c r="A617" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B617" s="4" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C617" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D617" s="4" t="inlineStr">
+        <is>
+          <t>EU, 中산 타이어 관세 5.5%p↓…K-타이어 ‘최악은 피했다’</t>
+        </is>
+      </c>
+      <c r="E617" s="4" t="inlineStr">
+        <is>
+          <t>EU가 중국산 타이어에 대한 반덤핑 관세를 부과하기로 결정했으나, 당초 예상보다 낮은 수준으로 결정되어 한국 타이어 업계는 최악의 상황을 피했다.</t>
+        </is>
+      </c>
+      <c r="F617" s="4" t="inlineStr">
+        <is>
+          <t>해당 뉴스는 타이어 산업에 대한 관세 부과 사례로, 배터리/전자부품 산업에 직접적인 관세 변동 영향을 주지는 않는다.</t>
+        </is>
+      </c>
+      <c r="G617" s="4" t="inlineStr"/>
+      <c r="H617" s="4" t="inlineStr">
+        <is>
+          <t>헤럴드경제</t>
+        </is>
+      </c>
+      <c r="I617" s="4" t="inlineStr">
+        <is>
+          <t>https://biz.heraldcorp.com/article/10800997</t>
+        </is>
+      </c>
+      <c r="J617" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -28094,7 +29626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -28628,6 +30160,49 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>3326.87</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>+87 (+2.7%)</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>+1,457 (+77.9%)</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>4330</v>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>+410 (+10.5%)</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>+1,619 (+59.7%)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -28640,7 +30215,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I93"/>
+  <dimension ref="A1:I102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -31921,6 +33496,321 @@
       </c>
       <c r="I93" s="6" t="inlineStr"/>
     </row>
+    <row r="94">
+      <c r="A94" s="6" t="inlineStr">
+        <is>
+          <t>RSK-093</t>
+        </is>
+      </c>
+      <c r="B94" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C94" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D94" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E94" s="6" t="inlineStr">
+        <is>
+          <t>[surff] 20260708 경제·물류 주요뉴스 (데일리스크랩)</t>
+        </is>
+      </c>
+      <c r="F94" s="6" t="inlineStr"/>
+      <c r="G94" s="6" t="inlineStr"/>
+      <c r="H94" s="6" t="inlineStr">
+        <is>
+          <t>중동 항로 이용 선박의 스케줄 및 운임 변동성 실시간 모니터링 강화, 대체 운송 경로 및 재고 확보 방안 검토, 유가 변동에 따른 물류비 예산 재검토.</t>
+        </is>
+      </c>
+      <c r="I94" s="6" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="6" t="inlineStr">
+        <is>
+          <t>RSK-094</t>
+        </is>
+      </c>
+      <c r="B95" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C95" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D95" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E95" s="6" t="inlineStr">
+        <is>
+          <t>[surff] 20260706 경제·물류 주요뉴스 (데일리스크랩)</t>
+        </is>
+      </c>
+      <c r="F95" s="6" t="inlineStr"/>
+      <c r="G95" s="6" t="inlineStr"/>
+      <c r="H95" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 상황 변화에 대한 실시간 모니터링 강화, 비상 운송 계획 수립 (대체 항로, 항공 운송 옵션 등), 물류비 상승 시나리오별 재무 영향 분석.</t>
+        </is>
+      </c>
+      <c r="I95" s="6" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="6" t="inlineStr">
+        <is>
+          <t>RSK-095</t>
+        </is>
+      </c>
+      <c r="B96" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C96" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D96" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E96" s="6" t="inlineStr">
+        <is>
+          <t>[surff] 20260704 경제·물류 주요뉴스 (데일리스크랩)</t>
+        </is>
+      </c>
+      <c r="F96" s="6" t="inlineStr"/>
+      <c r="G96" s="6" t="inlineStr"/>
+      <c r="H96" s="6" t="inlineStr">
+        <is>
+          <t>중동발 물류비 상승 추이 및 운임 정상화 시점 모니터링, 물류비 절감 방안 및 비용 전가 가능성 검토, 재고 관리 최적화.</t>
+        </is>
+      </c>
+      <c r="I96" s="6" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="6" t="inlineStr">
+        <is>
+          <t>RSK-096</t>
+        </is>
+      </c>
+      <c r="B97" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C97" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D97" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E97" s="6" t="inlineStr">
+        <is>
+          <t>[search_운송지연_항만적체] 미주·유럽 항로 강세에 컨테이너 운임 상승 - 매일일보</t>
+        </is>
+      </c>
+      <c r="F97" s="6" t="inlineStr"/>
+      <c r="G97" s="6" t="inlineStr"/>
+      <c r="H97" s="6" t="inlineStr">
+        <is>
+          <t>주요 항로 운임 및 선복 상황 실시간 모니터링, 포워더와 긴밀히 협력하여 선복 확보 노력, 필요 시 장기 계약 또는 대체 운송 방안 검토.</t>
+        </is>
+      </c>
+      <c r="I97" s="6" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="6" t="inlineStr">
+        <is>
+          <t>RSK-097</t>
+        </is>
+      </c>
+      <c r="B98" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C98" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D98" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E98" s="6" t="inlineStr">
+        <is>
+          <t>"호르무즈서 유조선 3척 또 피격"…국제유가 '들썩’</t>
+        </is>
+      </c>
+      <c r="F98" s="6" t="inlineStr"/>
+      <c r="G98" s="6" t="inlineStr"/>
+      <c r="H98" s="6" t="inlineStr">
+        <is>
+          <t>유가 및 해상 운임 변동 추이 실시간 모니터링, 비상 운송 계획 및 대체 경로 검토, 운송 계약 조건 재검토.</t>
+        </is>
+      </c>
+      <c r="I98" s="6" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="6" t="inlineStr">
+        <is>
+          <t>RSK-098</t>
+        </is>
+      </c>
+      <c r="B99" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C99" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D99" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E99" s="6" t="inlineStr">
+        <is>
+          <t>"美 관세는 '소나기' 아닌 '기후변화'…수출기업 전략 재편해야"</t>
+        </is>
+      </c>
+      <c r="F99" s="6" t="inlineStr"/>
+      <c r="G99" s="6" t="inlineStr"/>
+      <c r="H99" s="6" t="inlineStr">
+        <is>
+          <t>미국 관세 및 통상 정책 변화 동향 면밀히 분석, 공급망 다변화 및 생산 거점 재배치 전략 검토, 무역 규제 준수 여부 점검.</t>
+        </is>
+      </c>
+      <c r="I99" s="6" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="6" t="inlineStr">
+        <is>
+          <t>RSK-099</t>
+        </is>
+      </c>
+      <c r="B100" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C100" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D100" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E100" s="6" t="inlineStr">
+        <is>
+          <t>[매일시론] 핵심광물, 공급망 위기에 미리 대비해야</t>
+        </is>
+      </c>
+      <c r="F100" s="6" t="inlineStr"/>
+      <c r="G100" s="6" t="inlineStr"/>
+      <c r="H100" s="6" t="inlineStr">
+        <is>
+          <t>핵심광물 조달처 다변화 및 재고 확보 전략 강화, 공급망 리스크 평가 및 비상 계획 수립, 관련 정부 정책 및 국제 동향 면밀히 주시.</t>
+        </is>
+      </c>
+      <c r="I100" s="6" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="6" t="inlineStr">
+        <is>
+          <t>RSK-100</t>
+        </is>
+      </c>
+      <c r="B101" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C101" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D101" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E101" s="6" t="inlineStr">
+        <is>
+          <t>저가 외국산 배터리 국산 가장 수출·핵심설비 유출 등 적발</t>
+        </is>
+      </c>
+      <c r="F101" s="6" t="inlineStr"/>
+      <c r="G101" s="6" t="inlineStr"/>
+      <c r="H101" s="6" t="inlineStr">
+        <is>
+          <t>수출 품목의 원산지 관리 강화 및 전략물자 수출 규제 준수 여부 재점검, 내부 컴플라이언스 교육 강화.</t>
+        </is>
+      </c>
+      <c r="I101" s="6" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="6" t="inlineStr">
+        <is>
+          <t>RSK-101</t>
+        </is>
+      </c>
+      <c r="B102" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C102" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D102" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E102" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈 선박 잇단 피격에 국제유가 급등…브렌트유 3%↑</t>
+        </is>
+      </c>
+      <c r="F102" s="6" t="inlineStr"/>
+      <c r="G102" s="6" t="inlineStr"/>
+      <c r="H102" s="6" t="inlineStr">
+        <is>
+          <t>유가 변동에 따른 운임 인상 가능성을 대비하여 운송 계약 조건 재검토, 대체 운송 경로 및 모드 검토, 재고 수준 조정 검토.</t>
+        </is>
+      </c>
+      <c r="I102" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
📰 뉴스 데이터 2026-07-09_09:11
</commit_message>
<xml_diff>
--- a/data/SCM_물류_브리핑.xlsx
+++ b/data/SCM_물류_브리핑.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J617"/>
+  <dimension ref="A1:J652"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29614,6 +29614,1678 @@
       </c>
       <c r="J617" s="4" t="inlineStr"/>
     </row>
+    <row r="618">
+      <c r="A618" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B618" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C618" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D618" s="2" t="inlineStr">
+        <is>
+          <t>CPSC Mandatory eFiling Takes Effect July 8; TPEB Rates Surge ~10% as Peak Season Demand Outpaces Capacity</t>
+        </is>
+      </c>
+      <c r="E618" s="2" t="inlineStr">
+        <is>
+          <t>미국 CPSC의 전자 신고 의무화가 7월 8일 발효되며, 성수기 수요 초과로 태평양 동향(TPEB) 운임이 약 10% 급등했다.</t>
+        </is>
+      </c>
+      <c r="F618" s="2" t="inlineStr">
+        <is>
+          <t>주요 운송 노선(TPEB)의 운임 급등은 물류비에 즉각적인 영향을 미치며, CPSC 전자 신고 의무화는 미국 수출 시 새로운 절차 준수를 요구한다.</t>
+        </is>
+      </c>
+      <c r="G618" s="2" t="inlineStr">
+        <is>
+          <t>TPEB 운임 상승에 대비하여 운송 계약 검토 및 대체 운송 방안 모색. CPSC 전자 신고 시스템 및 절차 준수 여부 확인.</t>
+        </is>
+      </c>
+      <c r="H618" s="2" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I618" s="2" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/june-18-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J618" s="2" t="inlineStr">
+        <is>
+          <t>RSK-102</t>
+        </is>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B619" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C619" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D619" s="2" t="inlineStr">
+        <is>
+          <t>이란, 美공습에 맞불…“미사일·드론으로 미군시설 85곳 공격”</t>
+        </is>
+      </c>
+      <c r="E619" s="2" t="inlineStr">
+        <is>
+          <t>이란이 미국 공습에 대한 보복으로 미군 시설을 공격하며 호르무즈 해협의 군사적 긴장이 고조되고 있다.</t>
+        </is>
+      </c>
+      <c r="F619" s="2" t="inlineStr">
+        <is>
+          <t>주요 해상 운송 경로인 호르무즈 해협의 군사적 긴장은 선박 운항 안전 및 운송 비용에 즉각적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G619" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협을 통과하는 선박의 운항 상황 및 보험료 변동 주시, 필요시 대체 운송 경로 또는 운송 방식 검토.</t>
+        </is>
+      </c>
+      <c r="H619" s="2" t="inlineStr">
+        <is>
+          <t>kita</t>
+        </is>
+      </c>
+      <c r="I619" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kita.net/shippers/board/newsView.do?morgueCode=2&amp;dataCls=B&amp;dataSeq=8156</t>
+        </is>
+      </c>
+      <c r="J619" s="2" t="inlineStr">
+        <is>
+          <t>RSK-103</t>
+        </is>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B620" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C620" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D620" s="2" t="inlineStr">
+        <is>
+          <t>"어느새 해상운임 급등했다"...SCFI 3300p, CCFI 1800p 돌파, 2분기 평균 BDI는 지난 4년래 최고치</t>
+        </is>
+      </c>
+      <c r="E620" s="2" t="inlineStr">
+        <is>
+          <t>해상 컨테이너 운임지수(SCFI, CCFI)가 급등하여 선사들이 운임 협상에서 우위를 점하고 있으며, 7월 현재 운임 하락 요인이 없어 물류비 상승 압박이 지속될 것으로 보입니다.</t>
+        </is>
+      </c>
+      <c r="F620" s="2" t="inlineStr">
+        <is>
+          <t>해상 운임의 급등은 배터리/전자부품 운송 비용에 직접적인 영향을 미쳐 물류 예산 및 제품 원가에 즉각적인 부담을 줄 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G620" s="2" t="inlineStr">
+        <is>
+          <t>긴급 운임 협상 상황 점검, 대체 운송 방안 검토, 선적 계획 조정 및 비용 상승분 반영 검토.</t>
+        </is>
+      </c>
+      <c r="H620" s="2" t="inlineStr">
+        <is>
+          <t>shippingnewsnet.com</t>
+        </is>
+      </c>
+      <c r="I620" s="2" t="inlineStr">
+        <is>
+          <t>https://www.shippingnewsnet.com/news/articleView.html?idxno=71094</t>
+        </is>
+      </c>
+      <c r="J620" s="2" t="inlineStr">
+        <is>
+          <t>RSK-104</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B621" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C621" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D621" s="2" t="inlineStr">
+        <is>
+          <t>미군 이란 공습 시작 및 원유 제재 면제 철회, 호르무즈 선박 피격에 국제유가 급등</t>
+        </is>
+      </c>
+      <c r="E621" s="2" t="inlineStr">
+        <is>
+          <t>미군이 호르무즈 해협 선박 피격에 대한 보복으로 이란 공습을 시작하고 원유 제재 면제를 철회하면서, 중동 지정학적 리스크가 고조되고 국제유가가 급등했습니다.</t>
+        </is>
+      </c>
+      <c r="F621" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협의 지정학적 긴장 고조는 유가 상승을 넘어 해상 운송 차질 및 보험료 할증으로 이어져 물류 비용에 직접적인 영향을 미치고 공급망 안정성을 위협할 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G621" s="2" t="inlineStr">
+        <is>
+          <t>유가 및 해상 운임 변동성 모니터링 강화, 중동 항로 이용 시 대체 경로 및 운송 수단 검토, 비상 재고 확보 및 공급망 다변화 전략 재검토.</t>
+        </is>
+      </c>
+      <c r="H621" s="2" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I621" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260708-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J621" s="2" t="inlineStr">
+        <is>
+          <t>RSK-105</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B622" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C622" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D622" s="2" t="inlineStr">
+        <is>
+          <t>산업연구원 "호르무즈 해협 봉쇄 시 한국 제조업 생산비 4.7% 상승"</t>
+        </is>
+      </c>
+      <c r="E622" s="2" t="inlineStr">
+        <is>
+          <t>산업연구원은 호르무즈 해협 봉쇄 시 항로 우회, 선복 부족, 보험료 할증 등으로 운임이 상승하여 한국 제조업 생산비가 4.7% 증가할 수 있다고 분석하며, 이는 물류 비용과 공급망 안정성에 심각한 위협이 됩니다.</t>
+        </is>
+      </c>
+      <c r="F622" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 봉쇄 시나리오에 대한 구체적인 비용 상승 분석은 우리 회사의 물류 비용 및 생산 계획에 직접적인 잠재적 영향을 미치므로 즉각적인 대비책 마련이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G622" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 봉쇄 시나리오에 대한 비상 계획 수립, 대체 운송 경로 및 운송 수단 확보 방안 구체화, 보험료 및 할증료 변동성 분석, 주요 원자재 및 부품의 재고 수준 재검토.</t>
+        </is>
+      </c>
+      <c r="H622" s="2" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I622" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260706-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J622" s="2" t="inlineStr">
+        <is>
+          <t>RSK-106</t>
+        </is>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B623" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C623" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D623" s="2" t="inlineStr">
+        <is>
+          <t>25만 원 이하 직구도 이제 관세? EU 소액면세 폐지가 바꾸는 것들</t>
+        </is>
+      </c>
+      <c r="E623" s="2" t="inlineStr">
+        <is>
+          <t>2026년 7월 1일부터 EU 소액면세 제도가 폐지되어 150유로 이하 소포에도 관세가 부과되며, 이는 유럽으로 수출하는 기업들의 물류 비용 증가와 통관 절차 복잡성을 야기할 것입니다.</t>
+        </is>
+      </c>
+      <c r="F623" s="2" t="inlineStr">
+        <is>
+          <t>EU로의 소액 수출 물량에 대한 관세 및 부가세 부과와 통관 절차 복잡성 증가는 우리 회사의 유럽향 물류 비용과 운영 효율성에 직접적인 영향을 미치므로 즉시 대응해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G623" s="2" t="inlineStr">
+        <is>
+          <t>EU 수출 물량에 대한 관세 및 부가세 영향 분석, 통관 절차 변경에 따른 시스템 및 프로세스 업데이트, 고객 및 파트너사와의 정보 공유 및 협력 강화, DDP(Delivered Duty Paid) 조건 검토.</t>
+        </is>
+      </c>
+      <c r="H623" s="2" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I623" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/25만-원-이하-직구도-이제-관세-eu-소액면세-폐지가-바꾸는-것들-week-27-2026-</t>
+        </is>
+      </c>
+      <c r="J623" s="2" t="inlineStr">
+        <is>
+          <t>RSK-107</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B624" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C624" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D624" s="2" t="inlineStr">
+        <is>
+          <t>돈줄 막힌 이란, 미군 시설 타격…휴전 20일 만에 파국 위기 | 중앙일보</t>
+        </is>
+      </c>
+      <c r="E624" s="2" t="inlineStr">
+        <is>
+          <t>이란이 미군 시설을 타격하고 미국이 경제 제재와 군사 공격을 재개하면서 미국-이란 간 휴전 체제가 20일 만에 파국 위기에 처했으며, 이는 중동 정세 불안정을 심화시키고 호르무즈 해협의 해상 운송 안전에 심각한 위협을 가하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F624" s="2" t="inlineStr">
+        <is>
+          <t>미국과 이란 간의 직접적인 충돌 및 휴전 파기는 호르무즈 해협의 해상 운송 안전에 심각한 위협을 가하며, 유가 및 해상 운임에 즉각적이고 큰 영향을 미칠 것입니다.</t>
+        </is>
+      </c>
+      <c r="G624" s="2" t="inlineStr">
+        <is>
+          <t>중동발 원자재 및 부품 수급 현황을 즉시 점검하고, 대체 운송 경로 및 보험 적용 여부를 확인하며, 유가 및 해상 운임 변동성 대비 비상 운송 계획을 가동할 준비를 해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H624" s="2" t="inlineStr">
+        <is>
+          <t>중앙일보</t>
+        </is>
+      </c>
+      <c r="I624" s="2" t="inlineStr">
+        <is>
+          <t>https://joongang.co.kr/article/25443386</t>
+        </is>
+      </c>
+      <c r="J624" s="2" t="inlineStr">
+        <is>
+          <t>RSK-108</t>
+        </is>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B625" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C625" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D625" s="2" t="inlineStr">
+        <is>
+          <t>트럼프 "이란과 협상은 시간낭비"… 휴전 파기 카드로 압박</t>
+        </is>
+      </c>
+      <c r="E625" s="2" t="inlineStr">
+        <is>
+          <t>트럼프 전 대통령이 이란과의 협상을 시간 낭비로 규정하며 휴전 파기 카드로 압박하고 있습니다. 이는 미국과 이란 간의 긴장 고조를 시사하며, 중동 지역의 불안정성을 심화시킬 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="F625" s="2" t="inlineStr">
+        <is>
+          <t>이란과의 긴장 고조는 국제 유가 급등 및 중동 해상 운송로 불안정으로 이어져 물류 비용 및 운송 지연에 직접적인 영향을 미칠 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G625" s="2" t="inlineStr">
+        <is>
+          <t>중동 지역 정세 변화 및 호르무즈 해협 운송 상황 실시간 모니터링, 비상 운송 계획(대체 항로, 항공 운송 등) 검토 및 유가 변동에 따른 물류비 예산 재점검.</t>
+        </is>
+      </c>
+      <c r="H625" s="2" t="inlineStr">
+        <is>
+          <t>매일경제</t>
+        </is>
+      </c>
+      <c r="I625" s="2" t="inlineStr">
+        <is>
+          <t>https://mk.co.kr/news/world/12093703</t>
+        </is>
+      </c>
+      <c r="J625" s="2" t="inlineStr">
+        <is>
+          <t>RSK-109</t>
+        </is>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B626" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C626" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D626" s="2" t="inlineStr">
+        <is>
+          <t>트럼프 "오늘 밤 다시 공격"...국제유가 6% 급등</t>
+        </is>
+      </c>
+      <c r="E626" s="2" t="inlineStr">
+        <is>
+          <t>트럼프 전 대통령이 이란과의 휴전 종료를 선언하며 추가 공격 가능성을 시사하자 국제유가가 6% 가까이 급등했습니다. 이는 중동 정세 불안정으로 인한 유가 변동성을 보여줍니다.</t>
+        </is>
+      </c>
+      <c r="F626" s="2" t="inlineStr">
+        <is>
+          <t>국제유가 급등은 해상 및 항공 운송 비용에 직접적인 영향을 미쳐 물류비 증가로 이어지며, 이는 즉각적인 물류 예산 및 운송 계획 조정이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G626" s="2" t="inlineStr">
+        <is>
+          <t>유가 변동에 따른 물류비 예산 재점검, 운송 계약 조건(유류할증료 등) 확인, 운송사와의 협의를 통한 비용 절감 방안 모색.</t>
+        </is>
+      </c>
+      <c r="H626" s="2" t="inlineStr">
+        <is>
+          <t>파이낸셜뉴스</t>
+        </is>
+      </c>
+      <c r="I626" s="2" t="inlineStr">
+        <is>
+          <t>https://www.fnnews.com/news/202607082225531146</t>
+        </is>
+      </c>
+      <c r="J626" s="2" t="inlineStr">
+        <is>
+          <t>RSK-110</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B627" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C627" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D627" s="3" t="inlineStr">
+        <is>
+          <t>Air Cargo Demand Up 6.0% in May</t>
+        </is>
+      </c>
+      <c r="E627" s="3" t="inlineStr">
+        <is>
+          <t>IATA에 따르면 5월 글로벌 항공 화물 수요가 전년 대비 6.0% 증가했다.</t>
+        </is>
+      </c>
+      <c r="F627" s="3" t="inlineStr">
+        <is>
+          <t>항공 화물 수요 증가는 향후 운임 상승 및 성수기 항공 운송 공간 확보에 영향을 미칠 수 있으므로 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G627" s="3" t="inlineStr">
+        <is>
+          <t>항공 운송 계약 조건 및 대체 운송 옵션 검토.</t>
+        </is>
+      </c>
+      <c r="H627" s="3" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I627" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-29-air-cargo-demand-up-may/</t>
+        </is>
+      </c>
+      <c r="J627" s="3" t="inlineStr"/>
+    </row>
+    <row r="628">
+      <c r="A628" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B628" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C628" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D628" s="3" t="inlineStr">
+        <is>
+          <t>해운조합, 저탄소 선박연료 공급망 인증 획득</t>
+        </is>
+      </c>
+      <c r="E628" s="3" t="inlineStr">
+        <is>
+          <t>한국해운조합이 저탄소 선박연료 공급망에 대한 ISCC EU 인증을 획득하고 국내 선사에 친환경 바이오선박유 공급을 시작했다.</t>
+        </is>
+      </c>
+      <c r="F628" s="3" t="inlineStr">
+        <is>
+          <t>해운업계의 친환경 연료 전환은 장기적으로 운송 비용 및 규제 준수 요구사항에 영향을 미칠 수 있으므로 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G628" s="3" t="inlineStr">
+        <is>
+          <t>친환경 운송 옵션 및 관련 비용 변화 추이 모니터링, 지속가능성 목표에 부합하는 운송 파트너십 고려.</t>
+        </is>
+      </c>
+      <c r="H628" s="3" t="inlineStr">
+        <is>
+          <t>ksg</t>
+        </is>
+      </c>
+      <c r="I628" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ksg.co.kr/news/main_newsView.jsp?pNum=147578</t>
+        </is>
+      </c>
+      <c r="J628" s="3" t="inlineStr"/>
+    </row>
+    <row r="629">
+      <c r="A629" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B629" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C629" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D629" s="3" t="inlineStr">
+        <is>
+          <t>美 항소법원, “부당한 컨 보관료는 무효”…에버그린 패소</t>
+        </is>
+      </c>
+      <c r="E629" s="3" t="inlineStr">
+        <is>
+          <t>미국 연방항소법원이 연방해사위원회(FMC)의 컨테이너 지체료 규제 권한을 인정하며 부당한 지체료 부과 관행에 중요한 선례를 마련했다.</t>
+        </is>
+      </c>
+      <c r="F629" s="3" t="inlineStr">
+        <is>
+          <t>컨테이너 지체료 관련 규제 강화는 향후 물류 비용 절감에 긍정적 영향을 줄 수 있으나, 실제 적용 사례 및 업계 반응을 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G629" s="3" t="inlineStr">
+        <is>
+          <t>컨테이너 지체료 관련 계약 조건 및 실제 청구 내역 검토, FMC 가이드라인 준수 여부 확인.</t>
+        </is>
+      </c>
+      <c r="H629" s="3" t="inlineStr">
+        <is>
+          <t>oceanpress</t>
+        </is>
+      </c>
+      <c r="I629" s="3" t="inlineStr">
+        <is>
+          <t>https://www.oceanpress.co.kr/news/article.html?no=30558</t>
+        </is>
+      </c>
+      <c r="J629" s="3" t="inlineStr"/>
+    </row>
+    <row r="630">
+      <c r="A630" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B630" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C630" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D630" s="3" t="inlineStr">
+        <is>
+          <t>Tracking True Vessel Delay</t>
+        </is>
+      </c>
+      <c r="E630" s="3" t="inlineStr">
+        <is>
+          <t>해운사들이 스케줄 정시성을 높이기 위해 운송 시간을 늘리는(스케줄 버퍼링) 방식을 사용하고 있어, 실제 운송 지연 추적에 대한 분석이 필요하다.</t>
+        </is>
+      </c>
+      <c r="F630" s="3" t="inlineStr">
+        <is>
+          <t>해운사들의 스케줄 버퍼링 전략은 겉보기 정시성 개선에도 불구하고 실제 리드타임 증가를 야기할 수 있어 운송 계획에 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G630" s="3" t="inlineStr">
+        <is>
+          <t>실제 운송 리드타임 데이터 분석 및 운송 파트너와의 스케줄 버퍼링 전략 논의를 통해 정확한 도착 예측 및 재고 계획 수립.</t>
+        </is>
+      </c>
+      <c r="H630" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I630" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/394-tracking-true-vessel-delay</t>
+        </is>
+      </c>
+      <c r="J630" s="3" t="inlineStr"/>
+    </row>
+    <row r="631">
+      <c r="A631" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B631" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C631" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D631" s="3" t="inlineStr">
+        <is>
+          <t>Transpacific: Ripe for new non-alliance services</t>
+        </is>
+      </c>
+      <c r="E631" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence 분석에 따르면 태평양 횡단 노선에서 새로운 비동맹 선사 서비스가 증가할 가능성이 있으며, 이는 현물 운임과 연관성이 있다.</t>
+        </is>
+      </c>
+      <c r="F631" s="3" t="inlineStr">
+        <is>
+          <t>태평양 횡단 노선의 운송 시장 경쟁 심화는 향후 운임 및 서비스 선택에 긍정적인 영향을 미칠 수 있으므로 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G631" s="3" t="inlineStr">
+        <is>
+          <t>태평양 횡단 노선의 신규 서비스 및 운임 동향 지속적으로 파악.</t>
+        </is>
+      </c>
+      <c r="H631" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I631" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/393-transpacific-ripe-for-new-non-alliance-services</t>
+        </is>
+      </c>
+      <c r="J631" s="3" t="inlineStr"/>
+    </row>
+    <row r="632">
+      <c r="A632" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B632" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C632" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D632" s="3" t="inlineStr">
+        <is>
+          <t>Decoding Gemini’s Mediterranean Surge</t>
+        </is>
+      </c>
+      <c r="E632" s="3" t="inlineStr">
+        <is>
+          <t>Gemini Cooperation이 동서 컨테이너 선박 배치를 재조정하며 지중해 지역에서 시장 점유율을 늘리고 있어, 향후 해운 서비스 및 스케줄에 변화가 예상됩니다.</t>
+        </is>
+      </c>
+      <c r="F632" s="3" t="inlineStr">
+        <is>
+          <t>주요 선사 얼라이언스의 선박 배치 변화는 특정 항로의 서비스 수준, 운송 시간, 가용 선복량에 영향을 미칠 수 있으므로 지속적인 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G632" s="3" t="n"/>
+      <c r="H632" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I632" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/392-decoding-gemini-s-mediterranean-surge</t>
+        </is>
+      </c>
+      <c r="J632" s="3" t="inlineStr"/>
+    </row>
+    <row r="633">
+      <c r="A633" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B633" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C633" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D633" s="3" t="inlineStr">
+        <is>
+          <t>Toyota's Texas investment reflects a broader shift in North American truck manufacturing</t>
+        </is>
+      </c>
+      <c r="E633" s="3" t="inlineStr">
+        <is>
+          <t>토요타의 텍사스 공장 확장은 물류 비용 상승, 무역 정책 변화, 공급망 중단에 대응하여 북미 지역 제조 역량을 강화하는 추세를 보여주며, 이는 공급망 지역화의 중요성을 시사합니다.</t>
+        </is>
+      </c>
+      <c r="F633" s="3" t="inlineStr">
+        <is>
+          <t>주요 제조업체의 공급망 지역화 전략은 장기적으로 글로벌 물류 흐름 및 운송 방식에 변화를 가져올 수 있으므로, 우리 회사의 공급망 전략 수립에 참고할 필요가 있습니다.</t>
+        </is>
+      </c>
+      <c r="G633" s="3" t="inlineStr">
+        <is>
+          <t>글로벌 공급망 전략 재검토 시 지역화 추세 반영 고려.</t>
+        </is>
+      </c>
+      <c r="H633" s="3" t="inlineStr">
+        <is>
+          <t>manufacturing-today.com</t>
+        </is>
+      </c>
+      <c r="I633" s="3" t="inlineStr">
+        <is>
+          <t>https://manufacturing-today.com/news/toyota-announces-3-6-billion-expansion-of-texas-manufacturing-plant/</t>
+        </is>
+      </c>
+      <c r="J633" s="3" t="inlineStr"/>
+    </row>
+    <row r="634">
+      <c r="A634" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B634" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C634" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D634" s="3" t="inlineStr">
+        <is>
+          <t>Major supply chain shock would leave half of global businesses exposed within three weeks – new report</t>
+        </is>
+      </c>
+      <c r="E634" s="3" t="inlineStr">
+        <is>
+          <t>새로운 보고서에 따르면 전 세계 기업의 절반 이상이 주요 공급망 충격 발생 시 3주 이내에 운영에 차질을 겪을 것이라고 응답하여, 공급망 복원력 강화의 시급성을 강조합니다.</t>
+        </is>
+      </c>
+      <c r="F634" s="3" t="inlineStr">
+        <is>
+          <t>이 보고서는 공급망 충격에 대한 전반적인 취약성을 경고하며, 우리 회사의 공급망 복원력 및 비상 계획을 점검하고 강화할 필요성을 시사합니다.</t>
+        </is>
+      </c>
+      <c r="G634" s="3" t="inlineStr">
+        <is>
+          <t>공급망 리스크 평가 및 비상 계획 점검, 재고 관리 전략 재검토, 공급망 가시성 확보 방안 모색.</t>
+        </is>
+      </c>
+      <c r="H634" s="3" t="inlineStr">
+        <is>
+          <t>retailtimes.co.uk</t>
+        </is>
+      </c>
+      <c r="I634" s="3" t="inlineStr">
+        <is>
+          <t>https://retailtimes.co.uk/major-supply-chain-shock-would-leave-half-of-global-businesses-exposed-within-three-weeks-new-report/</t>
+        </is>
+      </c>
+      <c r="J634" s="3" t="inlineStr"/>
+    </row>
+    <row r="635">
+      <c r="A635" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B635" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C635" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D635" s="3" t="inlineStr">
+        <is>
+          <t>Supply chain shock could disrupt half of global businesses within three weeks - Retail Gazette</t>
+        </is>
+      </c>
+      <c r="E635" s="3" t="inlineStr">
+        <is>
+          <t>새로운 연구에 따르면 글로벌 기업의 절반이 주요 공급망 충격 발생 시 3주 이내에 운영 중단을 겪을 수 있으며, 이는 기업들의 공급망 취약성을 강조합니다.</t>
+        </is>
+      </c>
+      <c r="F635" s="3" t="inlineStr">
+        <is>
+          <t>이 연구 결과는 잠재적인 공급망 충격에 대한 우리 회사의 취약성을 평가하고 대비책을 마련할 필요성을 시사합니다.</t>
+        </is>
+      </c>
+      <c r="G635" s="3" t="inlineStr">
+        <is>
+          <t>잠재적 공급망 충격 시나리오별 비상 계획 검토 및 재고 수준, 대체 운송 경로, 공급처 다변화 등 대응 전략 점검.</t>
+        </is>
+      </c>
+      <c r="H635" s="3" t="inlineStr">
+        <is>
+          <t>Retail Gazette</t>
+        </is>
+      </c>
+      <c r="I635" s="3" t="inlineStr">
+        <is>
+          <t>https://www.retailgazette.co.uk/blog/2026/07/supply-chain-shock-could-disrupt-half-of-global-businesses-within-three-weeks/</t>
+        </is>
+      </c>
+      <c r="J635" s="3" t="inlineStr"/>
+    </row>
+    <row r="636">
+      <c r="A636" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B636" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C636" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D636" s="3" t="inlineStr">
+        <is>
+          <t>영종소방서, 배터리 화재 예방 안전수칙 홍보:FPN Daily</t>
+        </is>
+      </c>
+      <c r="E636" s="3" t="inlineStr">
+        <is>
+          <t>영종소방서가 리튬이온배터리 사용 증가에 따른 화재 예방 안전수칙을 홍보하며, 배터리 관련 화재 위험성에 대한 경각심을 높이고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F636" s="3" t="inlineStr">
+        <is>
+          <t>배터리 화재 예방은 우리 제품의 안전 규제 및 보관/운송에 대한 지속적인 관심이 필요하며, 향후 규제 강화로 이어질 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G636" s="3" t="inlineStr">
+        <is>
+          <t>배터리 보관 및 운송 관련 내부 안전 수칙 재점검, 관련 법규 및 규제 변화 동향 지속 모니터링.</t>
+        </is>
+      </c>
+      <c r="H636" s="3" t="inlineStr">
+        <is>
+          <t>FPN Daily</t>
+        </is>
+      </c>
+      <c r="I636" s="3" t="inlineStr">
+        <is>
+          <t>https://fpn119.co.kr/sub_read.html?uid=253557</t>
+        </is>
+      </c>
+      <c r="J636" s="3" t="inlineStr"/>
+    </row>
+    <row r="637">
+      <c r="A637" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B637" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C637" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D637" s="3" t="inlineStr">
+        <is>
+          <t>‘산업단지 화재 막아라’···대구소방, 전국 최초로 전담조직 꾸려 - 경향신문</t>
+        </is>
+      </c>
+      <c r="E637" s="3" t="inlineStr">
+        <is>
+          <t>대구소방안전본부가 전국 최초로 산업단지 화재 예방 전담조직을 꾸려 대형 화재 방지에 나섰으며, 이는 산업 시설 안전 강화의 일환입니다.</t>
+        </is>
+      </c>
+      <c r="F637" s="3" t="inlineStr">
+        <is>
+          <t>산업단지 화재 예방 강화 추세는 우리 공장 및 협력사들의 안전 관리 기준 강화로 이어질 수 있어 지속적인 관심이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G637" s="3" t="inlineStr">
+        <is>
+          <t>우리 공장 및 주요 협력사들의 화재 안전 관리 현황 점검, 산업단지 안전 규제 강화 동향 모니터링.</t>
+        </is>
+      </c>
+      <c r="H637" s="3" t="inlineStr">
+        <is>
+          <t>경향신문</t>
+        </is>
+      </c>
+      <c r="I637" s="3" t="inlineStr">
+        <is>
+          <t>https://khan.co.kr/article/202607081621001</t>
+        </is>
+      </c>
+      <c r="J637" s="3" t="inlineStr"/>
+    </row>
+    <row r="638">
+      <c r="A638" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B638" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C638" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D638" s="3" t="inlineStr">
+        <is>
+          <t>미국 국방부, 최대 3억달러 리튬 계약 추진...핵심광물 확보 가속 - 이투데이</t>
+        </is>
+      </c>
+      <c r="E638" s="3" t="inlineStr">
+        <is>
+          <t>미국 국방부가 5년간 최대 3억 달러 규모의 탄산리튬 입찰을 추진하며 핵심 광물 확보를 가속화하고 있으며, 이는 리튬 공급망에 영향을 줄 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="F638" s="3" t="inlineStr">
+        <is>
+          <t>미국 국방부의 대규모 리튬 확보 노력은 글로벌 리튬 시장의 수급과 가격에 영향을 미쳐 우리 원자재 조달에 잠재적 영향을 줄 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G638" s="3" t="inlineStr">
+        <is>
+          <t>리튬 등 핵심 원자재 시장 동향 및 가격 변동 추이 모니터링, 장기 공급 계약 및 다변화 전략 검토.</t>
+        </is>
+      </c>
+      <c r="H638" s="3" t="inlineStr">
+        <is>
+          <t>이투데이</t>
+        </is>
+      </c>
+      <c r="I638" s="3" t="inlineStr">
+        <is>
+          <t>https://etoday.co.kr/news/view/2601627</t>
+        </is>
+      </c>
+      <c r="J638" s="3" t="inlineStr"/>
+    </row>
+    <row r="639">
+      <c r="A639" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B639" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C639" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D639" s="3" t="inlineStr">
+        <is>
+          <t>폭염시 ‘배송 중지권’… 기사님 건강 챙기는 택배사들 | 문화일보</t>
+        </is>
+      </c>
+      <c r="E639" s="3" t="inlineStr">
+        <is>
+          <t>역대급 폭염이 예상됨에 따라 물류·택배업계가 혹서기 안전 대책으로 '배송 중지권' 등을 시행하며 근무자 건강 보호에 나서고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F639" s="3" t="inlineStr">
+        <is>
+          <t>택배사의 폭염 대책은 국내 운송 서비스의 지연 가능성을 시사하며, 특히 국내 배송 및 부품 조달에 영향을 줄 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G639" s="3" t="inlineStr">
+        <is>
+          <t>국내 운송 파트너사의 혹서기 운영 정책 확인 및 잠재적 배송 지연에 대한 비상 계획 수립, 국내 물류 리드타임 변동성 고려.</t>
+        </is>
+      </c>
+      <c r="H639" s="3" t="inlineStr">
+        <is>
+          <t>문화일보</t>
+        </is>
+      </c>
+      <c r="I639" s="3" t="inlineStr">
+        <is>
+          <t>https://munhwa.com/article/11601066</t>
+        </is>
+      </c>
+      <c r="J639" s="3" t="inlineStr"/>
+    </row>
+    <row r="640">
+      <c r="A640" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B640" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C640" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D640" s="3" t="inlineStr">
+        <is>
+          <t>반도체 못지않은 전략 자산…중국 이 기술 유출 막는다</t>
+        </is>
+      </c>
+      <c r="E640" s="3" t="inlineStr">
+        <is>
+          <t>중국이 AI 모델을 반도체에 버금가는 전략 자산으로 간주하고 해외 유출을 막기 위해 수출 통제를 검토하고 있습니다. 이는 첨단 기술에 대한 접근을 제한하려는 움직임으로 해석됩니다.</t>
+        </is>
+      </c>
+      <c r="F640" s="3" t="inlineStr">
+        <is>
+          <t>중국의 AI 모델 수출 통제는 장기적으로 전자부품의 기술 개발 및 공급망에 영향을 미칠 수 있으므로 추이를 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G640" s="3" t="inlineStr">
+        <is>
+          <t>중국의 AI 관련 기술 수출 통제 세부 내용 및 우리 제품/부품에 미칠 잠재적 영향 분석.</t>
+        </is>
+      </c>
+      <c r="H640" s="3" t="inlineStr">
+        <is>
+          <t>한국경제</t>
+        </is>
+      </c>
+      <c r="I640" s="3" t="inlineStr">
+        <is>
+          <t>https://hankyung.com/amp/202607082686i</t>
+        </is>
+      </c>
+      <c r="J640" s="3" t="inlineStr"/>
+    </row>
+    <row r="641">
+      <c r="A641" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B641" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C641" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D641" s="3" t="inlineStr">
+        <is>
+          <t>IMF, 이란 전쟁 여파에 세계 성장률 3.0%로 0.1%p 또 하향 조정</t>
+        </is>
+      </c>
+      <c r="E641" s="3" t="inlineStr">
+        <is>
+          <t>IMF가 이란 전쟁의 여파로 세계 경제 성장률을 3.0%로 0.1%p 하향 조정했습니다. 이는 분쟁 지역 노출 정도와 기술 가치 공급망 내 위치에 따라 각국에 미치는 영향이 다를 것으로 분석됩니다.</t>
+        </is>
+      </c>
+      <c r="F641" s="3" t="inlineStr">
+        <is>
+          <t>이란 전쟁으로 인한 세계 경제 성장률 하향 조정은 장기적으로 배터리/전자부품 수요 감소 및 물류 비용 변동으로 이어질 수 있어 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G641" s="3" t="inlineStr">
+        <is>
+          <t>글로벌 경제 지표 및 주요 시장 수요 변화 추이 지속 모니터링.</t>
+        </is>
+      </c>
+      <c r="H641" s="3" t="inlineStr">
+        <is>
+          <t>SBS 뉴스</t>
+        </is>
+      </c>
+      <c r="I641" s="3" t="inlineStr">
+        <is>
+          <t>https://news.sbs.co.kr/news/endPage.do?news_id=N1008648432</t>
+        </is>
+      </c>
+      <c r="J641" s="3" t="inlineStr"/>
+    </row>
+    <row r="642">
+      <c r="A642" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B642" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C642" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D642" s="3" t="inlineStr">
+        <is>
+          <t>임단협 난항 현대차 노조 3일 연속 2시간 부분파업</t>
+        </is>
+      </c>
+      <c r="E642" s="3" t="inlineStr">
+        <is>
+          <t>현대차 노조가 임단협 난항으로 3일 연속 2시간 부분파업을 진행하고 있습니다. 이는 현대차의 생산 차질로 이어질 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="F642" s="3" t="inlineStr">
+        <is>
+          <t>주요 고객사인 현대차의 부분파업은 당사 제품의 납품 일정 및 수요량에 영향을 미칠 수 있으므로 생산 및 재고 계획에 대한 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G642" s="3" t="inlineStr">
+        <is>
+          <t>현대차 생산 상황 및 파업 장기화 여부 모니터링, 고객사와의 납품 일정 조율 준비.</t>
+        </is>
+      </c>
+      <c r="H642" s="3" t="inlineStr">
+        <is>
+          <t>매일경제</t>
+        </is>
+      </c>
+      <c r="I642" s="3" t="inlineStr">
+        <is>
+          <t>https://mk.co.kr/news/society/12093640</t>
+        </is>
+      </c>
+      <c r="J642" s="3" t="inlineStr"/>
+    </row>
+    <row r="643">
+      <c r="A643" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B643" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C643" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D643" s="4" t="inlineStr">
+        <is>
+          <t>PLSCI Data Indicates Mega-Hub Retrenchment</t>
+        </is>
+      </c>
+      <c r="E643" s="4" t="inlineStr">
+        <is>
+          <t>UNCTAD의 PLSCI 데이터 분석 결과, 해운 네트워크가 메가 허브 중심에서 벗어나 재편되고 있음을 시사한다.</t>
+        </is>
+      </c>
+      <c r="F643" s="4" t="inlineStr">
+        <is>
+          <t>해운 네트워크의 장기적인 구조 변화를 나타내며, 즉각적인 물류 운영 영향은 낮지만 참고할 만한 정보이다.</t>
+        </is>
+      </c>
+      <c r="G643" s="4" t="n"/>
+      <c r="H643" s="4" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I643" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/396-plsci-data-indicates-mega-hub-retrenchment</t>
+        </is>
+      </c>
+      <c r="J643" s="4" t="inlineStr"/>
+    </row>
+    <row r="644">
+      <c r="A644" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B644" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C644" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D644" s="4" t="inlineStr">
+        <is>
+          <t>Global Schedule Reliability for May 2026 the Highest of the Year</t>
+        </is>
+      </c>
+      <c r="E644" s="4" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence 보고서에 따르면 2026년 5월 글로벌 선박 스케줄 정시성이 올해 최고치를 기록했다.</t>
+        </is>
+      </c>
+      <c r="F644" s="4" t="inlineStr">
+        <is>
+          <t>전반적인 해상 운송 스케줄 정시성 개선은 긍정적 신호이나, 특정 노선에 대한 직접적인 영향은 낮다.</t>
+        </is>
+      </c>
+      <c r="G644" s="4" t="n"/>
+      <c r="H644" s="4" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I644" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/395-global-schedule-reliability-for-may-2026-the-highest-of-the-year</t>
+        </is>
+      </c>
+      <c r="J644" s="4" t="inlineStr"/>
+    </row>
+    <row r="645">
+      <c r="A645" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B645" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C645" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D645" s="4" t="inlineStr">
+        <is>
+          <t>"원유 국적선사 운송 늘리자"… 정유·해운업계 '맞손'</t>
+        </is>
+      </c>
+      <c r="E645" s="4" t="inlineStr">
+        <is>
+          <t>에너지 수송 안정성 강화를 위해 정유 및 해운업계가 국적선사 운송 확대를 추진하고 있으며, 정부는 이에 대한 세제 및 운송비 지원을 검토 중입니다.</t>
+        </is>
+      </c>
+      <c r="F645" s="4" t="inlineStr">
+        <is>
+          <t>원유 운송에 대한 국적선사 활용 증가는 우리 회사의 배터리/전자부품 운송과는 직접적인 관련이 적으며, 전반적인 해운 시장 안정화에 간접적인 영향을 미칠 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G645" s="4" t="n"/>
+      <c r="H645" s="4" t="inlineStr">
+        <is>
+          <t>매일경제</t>
+        </is>
+      </c>
+      <c r="I645" s="4" t="inlineStr">
+        <is>
+          <t>https://mk.co.kr/news/economy/12093710</t>
+        </is>
+      </c>
+      <c r="J645" s="4" t="inlineStr"/>
+    </row>
+    <row r="646">
+      <c r="A646" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B646" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C646" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D646" s="4" t="inlineStr">
+        <is>
+          <t>벌크船도 초장기 계약…HMM 체질개선 속도</t>
+        </is>
+      </c>
+      <c r="E646" s="4" t="inlineStr">
+        <is>
+          <t>HMM이 글로벌 광산업체와 25년 초장기 벌크선 계약을 체결하며 사업 포트폴리오를 다변화하고 체질 개선에 속도를 내고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F646" s="4" t="inlineStr">
+        <is>
+          <t>HMM의 벌크선 장기 계약은 컨테이너 운송을 주로 이용하는 우리 회사의 물류 운영에 직접적인 영향은 없으며, 해운 시장 전반의 안정화에 간접적인 영향을 미칠 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G646" s="4" t="n"/>
+      <c r="H646" s="4" t="inlineStr">
+        <is>
+          <t>매일경제</t>
+        </is>
+      </c>
+      <c r="I646" s="4" t="inlineStr">
+        <is>
+          <t>https://mk.co.kr/news/business/12093625</t>
+        </is>
+      </c>
+      <c r="J646" s="4" t="inlineStr"/>
+    </row>
+    <row r="647">
+      <c r="A647" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B647" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C647" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D647" s="4" t="inlineStr">
+        <is>
+          <t>팬데믹과 분쟁 뚫은 ‘K-건설’ 저력... 대우건설이 이라크 초대형 인프라 ‘성공적 마침표’</t>
+        </is>
+      </c>
+      <c r="E647" s="4" t="inlineStr">
+        <is>
+          <t>대우건설이 이라크 알포 신항과 움카스르를 연결하는 고속도로 공사를 성공적으로 완공하여 중동 지역 물류 인프라 개선에 기여했습니다.</t>
+        </is>
+      </c>
+      <c r="F647" s="4" t="inlineStr">
+        <is>
+          <t>이라크 내륙 물류 인프라 개선은 우리 회사의 주요 운송 경로와 직접적인 관련이 적어 당장 물류 운영에 미치는 영향은 낮습니다.</t>
+        </is>
+      </c>
+      <c r="G647" s="4" t="n"/>
+      <c r="H647" s="4" t="inlineStr">
+        <is>
+          <t>insight.co.kr</t>
+        </is>
+      </c>
+      <c r="I647" s="4" t="inlineStr">
+        <is>
+          <t>https://www.insight.co.kr/news/562134</t>
+        </is>
+      </c>
+      <c r="J647" s="4" t="inlineStr"/>
+    </row>
+    <row r="648">
+      <c r="A648" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B648" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C648" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D648" s="4" t="inlineStr">
+        <is>
+          <t>프랑스 됭케르크항, 제2 컨테이너터미널 착공…2030년대 200만TEU 시대 연다</t>
+        </is>
+      </c>
+      <c r="E648" s="4" t="inlineStr">
+        <is>
+          <t>프랑스 됭케르크항이 제2 컨테이너터미널 건설을 시작하여 2030년대까지 처리 능력을 두 배 이상 확대할 예정이며, 이는 장기적으로 유럽 항만 적체 완화에 기여할 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="F648" s="4" t="inlineStr">
+        <is>
+          <t>됭케르크항의 터미널 확장은 장기적인 계획으로, 우리 회사의 현재 유럽향 물류 운영에 즉각적인 영향은 없으며, 2030년대 이후에나 긍정적인 영향을 기대할 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G648" s="4" t="n"/>
+      <c r="H648" s="4" t="inlineStr">
+        <is>
+          <t>해사신문</t>
+        </is>
+      </c>
+      <c r="I648" s="4" t="inlineStr">
+        <is>
+          <t>https://haesanews.com/news/articleView.html?idxno=149155</t>
+        </is>
+      </c>
+      <c r="J648" s="4" t="inlineStr"/>
+    </row>
+    <row r="649">
+      <c r="A649" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B649" s="4" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C649" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D649" s="4" t="inlineStr">
+        <is>
+          <t>전기차·ESS 판매 호조...K-배터리, 하반기 보릿고개 넘나</t>
+        </is>
+      </c>
+      <c r="E649" s="4" t="inlineStr">
+        <is>
+          <t>K-배터리 업계가 유럽 전기차 시장 회복과 AI 시대 ESS 수요 증가로 하반기 실적 개선을 기대하고 있습니다. 이는 전기차 캐즘을 극복하고 성장세를 이어갈 수 있는 긍정적인 신호로 해석됩니다.</t>
+        </is>
+      </c>
+      <c r="F649" s="4" t="inlineStr">
+        <is>
+          <t>배터리 시장의 긍정적 전망은 장기적인 생산 및 물류 계획에 영향을 줄 수 있으나, 당장 물류 운영에 직접적인 변화를 요구하지는 않습니다.</t>
+        </is>
+      </c>
+      <c r="G649" s="4" t="n"/>
+      <c r="H649" s="4" t="inlineStr">
+        <is>
+          <t>뉴스핌</t>
+        </is>
+      </c>
+      <c r="I649" s="4" t="inlineStr">
+        <is>
+          <t>https://newspim.com/news/view/20260708000861</t>
+        </is>
+      </c>
+      <c r="J649" s="4" t="inlineStr"/>
+    </row>
+    <row r="650">
+      <c r="A650" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B650" s="4" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C650" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D650" s="4" t="inlineStr">
+        <is>
+          <t>글로벌 비메모리 반도체 기업 NXP·ADI, 거액 과징금 부과 위기 ···공정위, 제재 절차 착수</t>
+        </is>
+      </c>
+      <c r="E650" s="4" t="inlineStr">
+        <is>
+          <t>공정거래위원회가 글로벌 비메모리 반도체 기업 NXP와 ADI에 대해 국내 유통업체에 판매 마진율을 강제한 혐의로 제재 절차에 착수했습니다. 이는 이들 기업에 거액의 과징금이 부과될 수 있음을 시사합니다.</t>
+        </is>
+      </c>
+      <c r="F650" s="4" t="inlineStr">
+        <is>
+          <t>비메모리 반도체 기업의 공정위 제재는 해당 기업의 사업 운영에 영향을 줄 수 있으나, 당사 물류 운영에 직접적인 영향을 미치지는 않습니다.</t>
+        </is>
+      </c>
+      <c r="G650" s="4" t="n"/>
+      <c r="H650" s="4" t="inlineStr">
+        <is>
+          <t>한국NGO신문</t>
+        </is>
+      </c>
+      <c r="I650" s="4" t="inlineStr">
+        <is>
+          <t>https://ngonews.kr/news/articleView.html?idxno=232419</t>
+        </is>
+      </c>
+      <c r="J650" s="4" t="inlineStr"/>
+    </row>
+    <row r="651">
+      <c r="A651" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B651" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C651" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D651" s="4" t="inlineStr">
+        <is>
+          <t>흥아해운도 부산행 합류... 4번째 이전 기업</t>
+        </is>
+      </c>
+      <c r="E651" s="4" t="inlineStr">
+        <is>
+          <t>흥아해운이 부산으로 본사를 이전하며, 현 정부 들어 네 번째 해운기업의 부산 이전 사례가 되었습니다. 이는 부산을 해운 중심지로 육성하려는 정책의 일환으로 보입니다.</t>
+        </is>
+      </c>
+      <c r="F651" s="4" t="inlineStr">
+        <is>
+          <t>해운사의 본사 이전은 지역 경제 및 해운 산업 구조에 영향을 줄 수 있으나, 당사 물류 운영의 운임이나 유가에 직접적인 영향을 미치지 않습니다.</t>
+        </is>
+      </c>
+      <c r="G651" s="4" t="n"/>
+      <c r="H651" s="4" t="inlineStr">
+        <is>
+          <t>오마이뉴스</t>
+        </is>
+      </c>
+      <c r="I651" s="4" t="inlineStr">
+        <is>
+          <t>https://ohmynews.com/NWS_Web/View/at_pg.aspx?CNTN_CD=A0003249656</t>
+        </is>
+      </c>
+      <c r="J651" s="4" t="inlineStr"/>
+    </row>
+    <row r="652">
+      <c r="A652" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B652" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C652" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D652" s="4" t="inlineStr">
+        <is>
+          <t>항만운송사업 등록?변경을 온라인으로 편리하게 신청하세요</t>
+        </is>
+      </c>
+      <c r="E652" s="4" t="inlineStr">
+        <is>
+          <t>해양수산부가 항만운송사업의 등록 및 변경 신청을 온라인으로 처리할 수 있는 서비스를 도입하여 사업자들의 행정 편의를 높일 예정입니다.</t>
+        </is>
+      </c>
+      <c r="F652" s="4" t="inlineStr">
+        <is>
+          <t>항만운송사업자들의 행정 편의 증진은 간접적인 긍정 효과를 줄 수 있으나, 당사 물류 운영에 직접적인 영향은 없습니다.</t>
+        </is>
+      </c>
+      <c r="G652" s="4" t="n"/>
+      <c r="H652" s="4" t="inlineStr">
+        <is>
+          <t>is보험</t>
+        </is>
+      </c>
+      <c r="I652" s="4" t="inlineStr">
+        <is>
+          <t>https://dazabi.com/insurance_magazine/article.php?id=7005</t>
+        </is>
+      </c>
+      <c r="J652" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -29626,7 +31298,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -30203,6 +31875,35 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n"/>
+      <c r="C14" s="5" t="inlineStr"/>
+      <c r="D14" s="5" t="inlineStr"/>
+      <c r="E14" s="5" t="inlineStr"/>
+      <c r="F14" s="5" t="n">
+        <v>4330</v>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>+410 (+10.5%)</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>+1,619 (+59.7%)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -30215,7 +31916,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I102"/>
+  <dimension ref="A1:I111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -33811,6 +35512,321 @@
       </c>
       <c r="I102" s="6" t="inlineStr"/>
     </row>
+    <row r="103">
+      <c r="A103" s="6" t="inlineStr">
+        <is>
+          <t>RSK-102</t>
+        </is>
+      </c>
+      <c r="B103" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="C103" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D103" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E103" s="6" t="inlineStr">
+        <is>
+          <t>CPSC Mandatory eFiling Takes Effect July 8; TPEB Rates Surge ~10% as Peak Season Demand Outpaces Capacity</t>
+        </is>
+      </c>
+      <c r="F103" s="6" t="inlineStr"/>
+      <c r="G103" s="6" t="inlineStr"/>
+      <c r="H103" s="6" t="inlineStr">
+        <is>
+          <t>TPEB 운임 상승에 대비하여 운송 계약 검토 및 대체 운송 방안 모색. CPSC 전자 신고 시스템 및 절차 준수 여부 확인.</t>
+        </is>
+      </c>
+      <c r="I103" s="6" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="6" t="inlineStr">
+        <is>
+          <t>RSK-103</t>
+        </is>
+      </c>
+      <c r="B104" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="C104" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D104" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E104" s="6" t="inlineStr">
+        <is>
+          <t>이란, 美공습에 맞불…“미사일·드론으로 미군시설 85곳 공격”</t>
+        </is>
+      </c>
+      <c r="F104" s="6" t="inlineStr"/>
+      <c r="G104" s="6" t="inlineStr"/>
+      <c r="H104" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈 해협을 통과하는 선박의 운항 상황 및 보험료 변동 주시, 필요시 대체 운송 경로 또는 운송 방식 검토.</t>
+        </is>
+      </c>
+      <c r="I104" s="6" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="6" t="inlineStr">
+        <is>
+          <t>RSK-104</t>
+        </is>
+      </c>
+      <c r="B105" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="C105" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D105" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E105" s="6" t="inlineStr">
+        <is>
+          <t>"어느새 해상운임 급등했다"...SCFI 3300p, CCFI 1800p 돌파, 2분기 평균 BDI는 지난 4년래 최고치</t>
+        </is>
+      </c>
+      <c r="F105" s="6" t="inlineStr"/>
+      <c r="G105" s="6" t="inlineStr"/>
+      <c r="H105" s="6" t="inlineStr">
+        <is>
+          <t>긴급 운임 협상 상황 점검, 대체 운송 방안 검토, 선적 계획 조정 및 비용 상승분 반영 검토.</t>
+        </is>
+      </c>
+      <c r="I105" s="6" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="6" t="inlineStr">
+        <is>
+          <t>RSK-105</t>
+        </is>
+      </c>
+      <c r="B106" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="C106" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D106" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E106" s="6" t="inlineStr">
+        <is>
+          <t>미군 이란 공습 시작 및 원유 제재 면제 철회, 호르무즈 선박 피격에 국제유가 급등</t>
+        </is>
+      </c>
+      <c r="F106" s="6" t="inlineStr"/>
+      <c r="G106" s="6" t="inlineStr"/>
+      <c r="H106" s="6" t="inlineStr">
+        <is>
+          <t>유가 및 해상 운임 변동성 모니터링 강화, 중동 항로 이용 시 대체 경로 및 운송 수단 검토, 비상 재고 확보 및 공급망 다변화 전략 재검토.</t>
+        </is>
+      </c>
+      <c r="I106" s="6" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="6" t="inlineStr">
+        <is>
+          <t>RSK-106</t>
+        </is>
+      </c>
+      <c r="B107" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="C107" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D107" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E107" s="6" t="inlineStr">
+        <is>
+          <t>산업연구원 "호르무즈 해협 봉쇄 시 한국 제조업 생산비 4.7% 상승"</t>
+        </is>
+      </c>
+      <c r="F107" s="6" t="inlineStr"/>
+      <c r="G107" s="6" t="inlineStr"/>
+      <c r="H107" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 봉쇄 시나리오에 대한 비상 계획 수립, 대체 운송 경로 및 운송 수단 확보 방안 구체화, 보험료 및 할증료 변동성 분석, 주요 원자재 및 부품의 재고 수준 재검토.</t>
+        </is>
+      </c>
+      <c r="I107" s="6" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="6" t="inlineStr">
+        <is>
+          <t>RSK-107</t>
+        </is>
+      </c>
+      <c r="B108" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="C108" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D108" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E108" s="6" t="inlineStr">
+        <is>
+          <t>25만 원 이하 직구도 이제 관세? EU 소액면세 폐지가 바꾸는 것들</t>
+        </is>
+      </c>
+      <c r="F108" s="6" t="inlineStr"/>
+      <c r="G108" s="6" t="inlineStr"/>
+      <c r="H108" s="6" t="inlineStr">
+        <is>
+          <t>EU 수출 물량에 대한 관세 및 부가세 영향 분석, 통관 절차 변경에 따른 시스템 및 프로세스 업데이트, 고객 및 파트너사와의 정보 공유 및 협력 강화, DDP(Delivered Duty Paid) 조건 검토.</t>
+        </is>
+      </c>
+      <c r="I108" s="6" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="6" t="inlineStr">
+        <is>
+          <t>RSK-108</t>
+        </is>
+      </c>
+      <c r="B109" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="C109" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D109" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E109" s="6" t="inlineStr">
+        <is>
+          <t>돈줄 막힌 이란, 미군 시설 타격…휴전 20일 만에 파국 위기 | 중앙일보</t>
+        </is>
+      </c>
+      <c r="F109" s="6" t="inlineStr"/>
+      <c r="G109" s="6" t="inlineStr"/>
+      <c r="H109" s="6" t="inlineStr">
+        <is>
+          <t>중동발 원자재 및 부품 수급 현황을 즉시 점검하고, 대체 운송 경로 및 보험 적용 여부를 확인하며, 유가 및 해상 운임 변동성 대비 비상 운송 계획을 가동할 준비를 해야 합니다.</t>
+        </is>
+      </c>
+      <c r="I109" s="6" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="6" t="inlineStr">
+        <is>
+          <t>RSK-109</t>
+        </is>
+      </c>
+      <c r="B110" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="C110" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D110" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E110" s="6" t="inlineStr">
+        <is>
+          <t>트럼프 "이란과 협상은 시간낭비"… 휴전 파기 카드로 압박</t>
+        </is>
+      </c>
+      <c r="F110" s="6" t="inlineStr"/>
+      <c r="G110" s="6" t="inlineStr"/>
+      <c r="H110" s="6" t="inlineStr">
+        <is>
+          <t>중동 지역 정세 변화 및 호르무즈 해협 운송 상황 실시간 모니터링, 비상 운송 계획(대체 항로, 항공 운송 등) 검토 및 유가 변동에 따른 물류비 예산 재점검.</t>
+        </is>
+      </c>
+      <c r="I110" s="6" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="6" t="inlineStr">
+        <is>
+          <t>RSK-110</t>
+        </is>
+      </c>
+      <c r="B111" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="C111" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D111" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E111" s="6" t="inlineStr">
+        <is>
+          <t>트럼프 "오늘 밤 다시 공격"...국제유가 6% 급등</t>
+        </is>
+      </c>
+      <c r="F111" s="6" t="inlineStr"/>
+      <c r="G111" s="6" t="inlineStr"/>
+      <c r="H111" s="6" t="inlineStr">
+        <is>
+          <t>유가 변동에 따른 물류비 예산 재점검, 운송 계약 조건(유류할증료 등) 확인, 운송사와의 협의를 통한 비용 절감 방안 모색.</t>
+        </is>
+      </c>
+      <c r="I111" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
📰 뉴스 데이터 2026-07-10_09:10
</commit_message>
<xml_diff>
--- a/data/SCM_물류_브리핑.xlsx
+++ b/data/SCM_물류_브리핑.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J652"/>
+  <dimension ref="A1:J687"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -31286,6 +31286,1694 @@
       </c>
       <c r="J652" s="4" t="inlineStr"/>
     </row>
+    <row r="653">
+      <c r="A653" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B653" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C653" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D653" s="2" t="inlineStr">
+        <is>
+          <t>"다시 강력 공격" 트럼프 예고대로…미군, 연이틀 이란 공습</t>
+        </is>
+      </c>
+      <c r="E653" s="2" t="inlineStr">
+        <is>
+          <t>미국이 이란을 이틀 연속 공습하며 호르무즈 해협을 둘러싼 미-이란 군사적 긴장이 고조되고 있다.</t>
+        </is>
+      </c>
+      <c r="F653" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협은 주요 원유 및 가스 운송로이며, 긴장 고조는 유가 상승 및 해상 운송 차질로 이어져 물류비와 운송 계획에 직접적인 영향을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="G653" s="2" t="inlineStr">
+        <is>
+          <t>유가 및 해상 운임 변동 추이를 면밀히 모니터링하고, 중동 경유 항로의 잠재적 지연 또는 중단 가능성에 대비하여 대체 운송 경로 및 비상 계획을 수립한다.</t>
+        </is>
+      </c>
+      <c r="H653" s="2" t="inlineStr">
+        <is>
+          <t>kita</t>
+        </is>
+      </c>
+      <c r="I653" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kita.net/shippers/board/newsView.do?morgueCode=2&amp;dataCls=A&amp;dataSeq=2532</t>
+        </is>
+      </c>
+      <c r="J653" s="2" t="inlineStr">
+        <is>
+          <t>RSK-111</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B654" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C654" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D654" s="2" t="inlineStr">
+        <is>
+          <t>현대글로비스, 일시적 충격에도 본질은 견조</t>
+        </is>
+      </c>
+      <c r="E654" s="2" t="inlineStr">
+        <is>
+          <t>현대글로비스의 2분기 실적이 미-이란 전쟁으로 인한 벙커유 가격 상승으로 시장 컨센서스를 하회할 전망이며, 유류비 부담이 가중되고 있다.</t>
+        </is>
+      </c>
+      <c r="F654" s="2" t="inlineStr">
+        <is>
+          <t>미-이란 전쟁으로 인한 벙커유 가격 상승은 해상 운임에 직접적인 영향을 미치며, BAF(유류할증료) 전가 시차로 인해 단기적인 물류비 증가가 예상된다.</t>
+        </is>
+      </c>
+      <c r="G654" s="2" t="inlineStr">
+        <is>
+          <t>유가 및 벙커유 가격 변동을 면밀히 모니터링하고, BAF 적용 시차에 따른 물류비 상승에 대비하여 운송 계약 조건을 재검토하거나 대체 운송 방안을 고려한다.</t>
+        </is>
+      </c>
+      <c r="H654" s="2" t="inlineStr">
+        <is>
+          <t>shippingnews</t>
+        </is>
+      </c>
+      <c r="I654" s="2" t="inlineStr">
+        <is>
+          <t>https://www.shippingnewsnet.com/news/articleView.html?idxno=71113</t>
+        </is>
+      </c>
+      <c r="J654" s="2" t="inlineStr">
+        <is>
+          <t>RSK-112</t>
+        </is>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B655" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C655" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D655" s="2" t="inlineStr">
+        <is>
+          <t>미군, 이란 공습 시작 및 원유 제재 면제 철회로 호르무즈 해협 긴장 최고조</t>
+        </is>
+      </c>
+      <c r="E655" s="2" t="inlineStr">
+        <is>
+          <t>미군이 호르무즈 해협 인근 선박 피격에 대한 보복으로 이란을 공습하고 이란 원유 제재 면제를 철회하며 중동 지역의 지정학적 긴장이 최고조에 달했다.</t>
+        </is>
+      </c>
+      <c r="F655" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협의 군사적 충돌 및 봉쇄 가능성은 유가 급등, 해상 운송 지연/중단으로 이어져 우리 물류 운영 및 생산 계획에 즉각적이고 직접적인 영향을 미친다.</t>
+        </is>
+      </c>
+      <c r="G655" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 상황을 실시간으로 모니터링하고, 비상시 대체 운송 경로(육상/항공) 및 재고 확보, 선사와의 긴밀한 소통을 통한 운송 계획 조정을 준비한다.</t>
+        </is>
+      </c>
+      <c r="H655" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I655" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260708-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J655" s="2" t="inlineStr">
+        <is>
+          <t>RSK-113</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B656" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C656" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D656" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 선박 피격에 국제유가 급등…브렌트유 3%↑</t>
+        </is>
+      </c>
+      <c r="E656" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 인근 선박 공격 소식으로 공급 불안 우려가 커지며 국제유가가 3% 급등했다.</t>
+        </is>
+      </c>
+      <c r="F656" s="2" t="inlineStr">
+        <is>
+          <t>국제유가 급등은 해상/항공 운임 상승으로 직결되어 우리 회사의 물류비용에 즉각적인 직접적 영향을 미친다.</t>
+        </is>
+      </c>
+      <c r="G656" s="2" t="inlineStr">
+        <is>
+          <t>유가 변동에 따른 물류비용 상승을 예측하고, 운송 계약 조건(유류할증료 등)을 검토하며, 필요시 재고 수준 조정 및 운송 방식 다변화를 고려한다.</t>
+        </is>
+      </c>
+      <c r="H656" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I656" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260708-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J656" s="2" t="inlineStr">
+        <is>
+          <t>RSK-114</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B657" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C657" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D657" s="2" t="inlineStr">
+        <is>
+          <t>산업硏 "호르무즈 봉쇄로 한국 제조업 생산비 4.7% 뛰어"</t>
+        </is>
+      </c>
+      <c r="E657" s="2" t="inlineStr">
+        <is>
+          <t>산업연구원은 호르무즈 해협 봉쇄 시 항로 우회, 선복 부족, 보험/위험 할증료 등으로 운임이 올라 한국 제조업 생산비가 4.7% 상승할 수 있다고 분석했다.</t>
+        </is>
+      </c>
+      <c r="F657" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 봉쇄 시 운임 급등 및 운송 지연으로 인한 생산비 증가는 우리 회사의 물류비용 및 생산 계획에 직접적이고 심각한 영향을 미친다.</t>
+        </is>
+      </c>
+      <c r="G657" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 봉쇄 시나리오에 대비하여 대체 운송 경로 및 운송 수단 확보 방안을 구체화하고, 비상 재고 수준을 검토하며, 물류비용 상승에 대한 재무적 영향을 분석한다.</t>
+        </is>
+      </c>
+      <c r="H657" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I657" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260706-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J657" s="2" t="inlineStr">
+        <is>
+          <t>RSK-115</t>
+        </is>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B658" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C658" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D658" s="2" t="inlineStr">
+        <is>
+          <t>전쟁 리스크에 출렁이는 해운시장…중동 항로 운임 변동성 80% 급증</t>
+        </is>
+      </c>
+      <c r="E658" s="2" t="inlineStr">
+        <is>
+          <t>중동 지역의 전쟁 리스크로 해운 시장의 운임 변동성이 80% 급증했으며, 항로 다변화 및 대체 허브 활용 노력이 필요하다.</t>
+        </is>
+      </c>
+      <c r="F658" s="2" t="inlineStr">
+        <is>
+          <t>중동 항로의 운임 변동성 급증은 우리 회사의 물류비용에 직접적인 영향을 미치며, 운송 계획 수립에 어려움을 가중시킨다.</t>
+        </is>
+      </c>
+      <c r="G658" s="2" t="inlineStr">
+        <is>
+          <t>중동 항로 운임 변동성 추이를 면밀히 주시하고, 대체 항로 및 운송 수단 확보 방안을 검토하며, 운송 계약 시 위험 분산 조항을 강화한다.</t>
+        </is>
+      </c>
+      <c r="H658" s="2" t="inlineStr">
+        <is>
+          <t>이투데이</t>
+        </is>
+      </c>
+      <c r="I658" s="2" t="inlineStr">
+        <is>
+          <t>https://etoday.co.kr/news/view/2602072</t>
+        </is>
+      </c>
+      <c r="J658" s="2" t="inlineStr">
+        <is>
+          <t>RSK-116</t>
+        </is>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B659" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C659" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D659" s="2" t="inlineStr">
+        <is>
+          <t>이란發 인플레 악몽 되살아나나…세계 공급망 다시 긴장</t>
+        </is>
+      </c>
+      <c r="E659" s="2" t="inlineStr">
+        <is>
+          <t>이란발 지정학적 긴장 고조로 유가가 급등하고 유조선 운임이 치솟으면서 세계 공급망에 인플레이션 압력이 다시 가해질 수 있다는 우려가 제기되었다.</t>
+        </is>
+      </c>
+      <c r="F659" s="2" t="inlineStr">
+        <is>
+          <t>이란발 지정학적 리스크는 유가 및 해상 운임 상승으로 직결되어 배터리/전자부품의 원자재 수입 및 완제품 수출 물류비용에 즉각적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G659" s="2" t="inlineStr">
+        <is>
+          <t>유가 및 해상 운임 변동성 모니터링 강화, 운송 계약 조건 재검토, 잠재적 비용 상승에 대비한 예산 조정 및 재고 전략 검토.</t>
+        </is>
+      </c>
+      <c r="H659" s="2" t="inlineStr">
+        <is>
+          <t>이투데이</t>
+        </is>
+      </c>
+      <c r="I659" s="2" t="inlineStr">
+        <is>
+          <t>https://etoday.co.kr/news/view/2602128</t>
+        </is>
+      </c>
+      <c r="J659" s="2" t="inlineStr">
+        <is>
+          <t>RSK-117</t>
+        </is>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B660" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C660" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D660" s="2" t="inlineStr">
+        <is>
+          <t>IMF, 美 경제 진단... “이란 전쟁 여파로 인플레 충격, 2027년까지 지속”</t>
+        </is>
+      </c>
+      <c r="E660" s="2" t="inlineStr">
+        <is>
+          <t>IMF는 이란 전쟁 여파와 트럼프 관세 정책, 국제유가 급등으로 인해 미국 물가 상승 압력이 2027년까지 지속될 것으로 전망하며 글로벌 인플레이션 우려를 표명했다.</t>
+        </is>
+      </c>
+      <c r="F660" s="2" t="inlineStr">
+        <is>
+          <t>이란발 지정학적 리스크와 유가 상승, 트럼프 관세 정책은 장기적인 물류비용 상승 압력으로 작용하며, 특히 미국 시장으로의 수출에 직접적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G660" s="2" t="inlineStr">
+        <is>
+          <t>장기적인 물류비용 상승 시나리오 분석, 미국 시장 수출 시 관세 및 운임 변동성 고려한 가격 및 공급망 전략 수립.</t>
+        </is>
+      </c>
+      <c r="H660" s="2" t="inlineStr">
+        <is>
+          <t>인사이트</t>
+        </is>
+      </c>
+      <c r="I660" s="2" t="inlineStr">
+        <is>
+          <t>https://insight.co.kr/news/562218</t>
+        </is>
+      </c>
+      <c r="J660" s="2" t="inlineStr">
+        <is>
+          <t>RSK-118</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B661" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C661" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D661" s="2" t="inlineStr">
+        <is>
+          <t>“중국산 막히면 서방 제조업 올스톱”…G2 전장, 칩에서 광물로 [텅스텐 War ②]</t>
+        </is>
+      </c>
+      <c r="E661" s="2" t="inlineStr">
+        <is>
+          <t>미국과 중국의 기술 패권 경쟁이 반도체를 넘어 텅스텐 등 핵심 광물로 확대되면서, 중국이 글로벌 생산량의 85%를 차지하는 광물 공급망에 차질이 생길 경우 서방 제조업에 큰 영향을 미칠 수 있다는 우려가 제기되었다.</t>
+        </is>
+      </c>
+      <c r="F661" s="2" t="inlineStr">
+        <is>
+          <t>배터리/전자부품 제조에 필수적인 핵심 광물 공급망이 미중 갈등으로 인해 불안정해질 경우, 원자재 수급에 직접적인 차질이 발생하여 생산 계획에 심각한 영향을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="G661" s="2" t="inlineStr">
+        <is>
+          <t>핵심 광물 재고 수준 점검, 중국 외 대체 공급처 발굴 및 다변화 전략 수립, 공급망 리스크 시나리오별 대응 계획 마련.</t>
+        </is>
+      </c>
+      <c r="H661" s="2" t="inlineStr">
+        <is>
+          <t>이투데이</t>
+        </is>
+      </c>
+      <c r="I661" s="2" t="inlineStr">
+        <is>
+          <t>https://etoday.co.kr/news/view/2602205</t>
+        </is>
+      </c>
+      <c r="J661" s="2" t="inlineStr">
+        <is>
+          <t>RSK-119</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B662" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C662" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D662" s="2" t="inlineStr">
+        <is>
+          <t>정부, WTO서 해외 기술규제 8건 제기…수출 애로 해소 나선다</t>
+        </is>
+      </c>
+      <c r="E662" s="2" t="inlineStr">
+        <is>
+          <t>정부가 WTO에 해외 기술규제 8건을 제기하며 수출 애로 해소에 나섰으며, 이는 배터리 등 주요 산업의 시험·인증 비용 증가, 통관 지연, 제품 설계 변경 등 물류 및 생산 부담으로 이어질 수 있다.</t>
+        </is>
+      </c>
+      <c r="F662" s="2" t="inlineStr">
+        <is>
+          <t>해외 기술규제는 배터리 제품의 수출 통관 지연 및 추가 비용 발생, 심지어 제품 설계 변경까지 요구할 수 있어 즉각적인 물류 및 생산 계획에 직접적인 영향을 미친다.</t>
+        </is>
+      </c>
+      <c r="G662" s="2" t="inlineStr">
+        <is>
+          <t>현재 수출 중인 제품에 대한 각국의 기술규제 현황을 파악하고, 잠재적 영향을 분석하여 필요시 제품 설계 변경 또는 인증 획득 계획을 수립해야 한다.</t>
+        </is>
+      </c>
+      <c r="H662" s="2" t="inlineStr">
+        <is>
+          <t>아주경제</t>
+        </is>
+      </c>
+      <c r="I662" s="2" t="inlineStr">
+        <is>
+          <t>https://ajunews.com/view/20260709100606240</t>
+        </is>
+      </c>
+      <c r="J662" s="2" t="inlineStr">
+        <is>
+          <t>RSK-120</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B663" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C663" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D663" s="3" t="inlineStr">
+        <is>
+          <t>Air Cargo Demand Up 6.0% in May</t>
+        </is>
+      </c>
+      <c r="E663" s="3" t="inlineStr">
+        <is>
+          <t>2026년 5월 전 세계 항공 화물 수요가 전년 대비 6.0% 증가했으며, 이는 국제선 수요 증가와 아시아 태평양 지역의 강력한 성장에 기인한다.</t>
+        </is>
+      </c>
+      <c r="F663" s="3" t="inlineStr">
+        <is>
+          <t>항공 화물 수요 증가는 향후 항공 운임 상승 압력으로 작용할 수 있어 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G663" s="3" t="inlineStr">
+        <is>
+          <t>항공 운임 추이 및 주요 항공사 스케줄 변동을 주시하고, 필요시 대체 운송 방안을 검토한다.</t>
+        </is>
+      </c>
+      <c r="H663" s="3" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I663" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-29-air-cargo-demand-up-may/</t>
+        </is>
+      </c>
+      <c r="J663" s="3" t="inlineStr"/>
+    </row>
+    <row r="664">
+      <c r="A664" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B664" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C664" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D664" s="3" t="inlineStr">
+        <is>
+          <t>맥스피드 “LCL 수출입 업무 디지털 전환”</t>
+        </is>
+      </c>
+      <c r="E664" s="3" t="inlineStr">
+        <is>
+          <t>소량화물 혼재(LCL) 전문기업 맥스피드가 온라인 플랫폼 'e-MAXPEED'를 출시하여 운송 스케줄 조회, 운임 확인, 선적 예약, 정산 등 LCL 수출입 업무의 디지털 전환을 지원한다.</t>
+        </is>
+      </c>
+      <c r="F664" s="3" t="inlineStr">
+        <is>
+          <t>LCL 디지털 플랫폼은 소량 화물 운송의 가시성과 효율성을 높일 수 있어, 당사의 LCL 운송 프로세스 개선에 참고할 만하다.</t>
+        </is>
+      </c>
+      <c r="G664" s="3" t="inlineStr">
+        <is>
+          <t>LCL 운송 시 해당 플랫폼의 활용 가능성을 검토하고, 유사 서비스 동향을 주시하여 물류 효율화 방안을 모색한다.</t>
+        </is>
+      </c>
+      <c r="H664" s="3" t="inlineStr">
+        <is>
+          <t>ksg</t>
+        </is>
+      </c>
+      <c r="I664" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ksg.co.kr/news/main_newsView.jsp?pNum=147554</t>
+        </is>
+      </c>
+      <c r="J664" s="3" t="inlineStr"/>
+    </row>
+    <row r="665">
+      <c r="A665" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B665" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C665" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D665" s="3" t="inlineStr">
+        <is>
+          <t>Structural Contraction of Global Liner Networks</t>
+        </is>
+      </c>
+      <c r="E665" s="3" t="inlineStr">
+        <is>
+          <t>2012년 이후 글로벌 정기선 네트워크 데이터 분석 결과, 선사들이 지리적 범위는 유지하면서도 서비스 빈도를 줄이는 등 네트워크 구조적 축소가 나타나고 있다.</t>
+        </is>
+      </c>
+      <c r="F665" s="3" t="inlineStr">
+        <is>
+          <t>선사들의 서비스 빈도 축소는 특정 항로의 운송 리드타임 증가 및 스케줄 선택의 폭 감소로 이어질 수 있어 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G665" s="3" t="inlineStr">
+        <is>
+          <t>주요 항로의 선사 서비스 빈도 및 스케줄 변화를 주시하고, 필요시 복수 선사와의 계약을 통해 유연성을 확보한다.</t>
+        </is>
+      </c>
+      <c r="H665" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I665" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/397-structural-contraction-of-global-liner-networks</t>
+        </is>
+      </c>
+      <c r="J665" s="3" t="inlineStr"/>
+    </row>
+    <row r="666">
+      <c r="A666" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B666" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C666" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D666" s="3" t="inlineStr">
+        <is>
+          <t>PLSCI Data Indicates Mega-Hub Retrenchment</t>
+        </is>
+      </c>
+      <c r="E666" s="3" t="inlineStr">
+        <is>
+          <t>2026년 2분기 항만 정기선 연결성 지수(PLSCI) 분석 결과, 최근 네트워크 재조정이 메가 허브 항만의 후퇴를 시사한다.</t>
+        </is>
+      </c>
+      <c r="F666" s="3" t="inlineStr">
+        <is>
+          <t>메가 허브 항만의 연결성 변화는 주요 항만 이용 전략 및 운송 경로 선택에 영향을 미칠 수 있으므로 추이를 지켜봐야 한다.</t>
+        </is>
+      </c>
+      <c r="G666" s="3" t="inlineStr">
+        <is>
+          <t>주요 수출입 항만의 PLSCI 변화를 모니터링하고, 필요시 대체 항만 및 운송 경로를 검토한다.</t>
+        </is>
+      </c>
+      <c r="H666" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I666" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/396-plsci-data-indicates-mega-hub-retrenchment</t>
+        </is>
+      </c>
+      <c r="J666" s="3" t="inlineStr"/>
+    </row>
+    <row r="667">
+      <c r="A667" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B667" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C667" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D667" s="3" t="inlineStr">
+        <is>
+          <t>Tracking True Vessel Delay</t>
+        </is>
+      </c>
+      <c r="E667" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence는 선사들이 운송 시간을 늘려 스케줄 버퍼링을 활용하고 있으며, 이는 실제 선박 지연과 조기 도착 간의 관계를 분석하는 데 중요하다고 밝혔다.</t>
+        </is>
+      </c>
+      <c r="F667" s="3" t="inlineStr">
+        <is>
+          <t>선사들의 스케줄 버퍼링 전략은 공시된 운송 시간과 실제 운송 시간 간의 차이를 발생시켜 물류 계획 수립 시 고려해야 할 요소이다.</t>
+        </is>
+      </c>
+      <c r="G667" s="3" t="inlineStr">
+        <is>
+          <t>선사별 공시 운송 시간과 실제 도착 시간 데이터를 비교 분석하여, 물류 리드타임 예측의 정확도를 높이는 데 활용한다.</t>
+        </is>
+      </c>
+      <c r="H667" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I667" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/394-tracking-true-vessel-delay</t>
+        </is>
+      </c>
+      <c r="J667" s="3" t="inlineStr"/>
+    </row>
+    <row r="668">
+      <c r="A668" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B668" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C668" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D668" s="3" t="inlineStr">
+        <is>
+          <t>Transpacific: Ripe for new non-alliance services</t>
+        </is>
+      </c>
+      <c r="E668" s="3" t="inlineStr">
+        <is>
+          <t>태평양 횡단 항로에서 비동맹 선사들의 신규 서비스 도입 가능성이 높아지고 있으며, 이는 컨테이너 현물 운임과 비동맹 선사 점유율 간의 관계 분석을 통해 확인되었다.</t>
+        </is>
+      </c>
+      <c r="F668" s="3" t="inlineStr">
+        <is>
+          <t>태평양 횡단 항로의 신규 서비스 증가는 운임 경쟁을 심화시키고 운송 옵션을 다양화하여 당사 물류 전략에 영향을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="G668" s="3" t="inlineStr">
+        <is>
+          <t>태평양 횡단 항로의 신규 서비스 출시 동향과 운임 변동을 주시하고, 잠재적 운송 파트너 확대를 고려한다.</t>
+        </is>
+      </c>
+      <c r="H668" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I668" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/393-transpacific-ripe-for-new-non-alliance-services</t>
+        </is>
+      </c>
+      <c r="J668" s="3" t="inlineStr"/>
+    </row>
+    <row r="669">
+      <c r="A669" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B669" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C669" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D669" s="3" t="inlineStr">
+        <is>
+          <t>해진공 "해운시장 예측보다 외부 충격 신속 대응이 중요해질 것"</t>
+        </is>
+      </c>
+      <c r="E669" s="3" t="inlineStr">
+        <is>
+          <t>해진공은 수에즈 운하 정상화와 우회 선복 복귀 속도가 향후 글로벌 컨테이너 시장의 핵심 변수이며, 외부 충격에 대한 신속 대응이 중요하다고 진단했다.</t>
+        </is>
+      </c>
+      <c r="F669" s="3" t="inlineStr">
+        <is>
+          <t>글로벌 해운 시장의 주요 변동성 요인(수에즈 운하, 우회 선복)에 대한 경고로, 운송 지연 및 운임에 영향을 미칠 수 있어 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G669" s="3" t="inlineStr">
+        <is>
+          <t>글로벌 해운 시장 동향 및 수에즈 운하 상황을 지속적으로 모니터링하고, 비상시 대체 운송 경로 및 선사 확보 방안을 검토한다.</t>
+        </is>
+      </c>
+      <c r="H669" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I669" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260710-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J669" s="3" t="inlineStr"/>
+    </row>
+    <row r="670">
+      <c r="A670" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B670" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C670" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D670" s="3" t="inlineStr">
+        <is>
+          <t>국제유가, 공급증가 전망에 약보합세…0.2% 하락</t>
+        </is>
+      </c>
+      <c r="E670" s="3" t="inlineStr">
+        <is>
+          <t>중동 불확실성에도 불구하고 OPEC+ 증산 전망 등 공급 증가 요인으로 국제유가가 소폭 하락했다.</t>
+        </is>
+      </c>
+      <c r="F670" s="3" t="inlineStr">
+        <is>
+          <t>유가 변동은 물류비에 직접적인 영향을 미치므로, 하락세가 지속될지 여부를 모니터링하여 물류비 절감 기회를 파악해야 한다.</t>
+        </is>
+      </c>
+      <c r="G670" s="3" t="inlineStr">
+        <is>
+          <t>국제유가 추이를 지속적으로 모니터링하고, 유가 변동에 따른 운임 계약 조건(유류할증료 등)의 영향을 분석한다.</t>
+        </is>
+      </c>
+      <c r="H670" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I670" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260707-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J670" s="3" t="inlineStr"/>
+    </row>
+    <row r="671">
+      <c r="A671" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B671" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C671" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D671" s="3" t="inlineStr">
+        <is>
+          <t>우크라 드론, 러 후방 정유공장 타격…최장거리 공격</t>
+        </is>
+      </c>
+      <c r="E671" s="3" t="inlineStr">
+        <is>
+          <t>우크라이나 드론이 러시아 후방의 정유시설과 선박을 공격하여 지정학적 긴장을 고조시키고 유가 변동성에 영향을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="F671" s="3" t="inlineStr">
+        <is>
+          <t>러시아 정유시설 공격은 글로벌 유가 공급에 영향을 미쳐 유가 변동성을 키울 수 있으므로 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G671" s="3" t="inlineStr">
+        <is>
+          <t>국제유가 및 러시아-우크라이나 전쟁 상황을 지속적으로 모니터링하여 유가 변동에 따른 물류비 영향을 예측한다.</t>
+        </is>
+      </c>
+      <c r="H671" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I671" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260707-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J671" s="3" t="inlineStr"/>
+    </row>
+    <row r="672">
+      <c r="A672" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B672" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C672" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D672" s="3" t="inlineStr">
+        <is>
+          <t>OPEC+ 5개월 연속 증산 합의…"내년 공급과잉 우려"</t>
+        </is>
+      </c>
+      <c r="E672" s="3" t="inlineStr">
+        <is>
+          <t>OPEC+가 5개월 연속 증산에 합의하면서 내년 공급과잉 우려가 커지는 가운데, 해상 운송 여건 정상화 시 공급 회복도 빨라질 수 있다는 전망이다.</t>
+        </is>
+      </c>
+      <c r="F672" s="3" t="inlineStr">
+        <is>
+          <t>OPEC+의 증산 합의는 장기적으로 유가 안정화에 기여할 수 있으나, 단기적인 시장 변동성을 모니터링하여 물류비 영향을 예측해야 한다.</t>
+        </is>
+      </c>
+      <c r="G672" s="3" t="inlineStr">
+        <is>
+          <t>OPEC+의 증산 정책 및 글로벌 원유 시장 동향을 지속적으로 모니터링하여 유가 변동에 따른 물류비 영향을 예측한다.</t>
+        </is>
+      </c>
+      <c r="H672" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I672" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260706-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J672" s="3" t="inlineStr"/>
+    </row>
+    <row r="673">
+      <c r="A673" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B673" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C673" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D673" s="3" t="inlineStr">
+        <is>
+          <t>미국 연방항소법원, 연방해사위원회(FMC)의 컨테이너 지체료 규제 권한 인정</t>
+        </is>
+      </c>
+      <c r="E673" s="3" t="inlineStr">
+        <is>
+          <t>미국 연방항소법원이 연방해사위원회(FMC)의 컨테이너 지체료 규제 권한을 인정하여 해운업계의 컨테이너 보관료 부과 관행에 중요한 선례를 마련했다.</t>
+        </is>
+      </c>
+      <c r="F673" s="3" t="inlineStr">
+        <is>
+          <t>미국 항만에서의 컨테이너 지체료 규제 강화는 향후 우리 회사의 미국향 수출입 물류 비용 및 운영에 영향을 미칠 수 있으므로 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G673" s="3" t="inlineStr">
+        <is>
+          <t>미국 항만 지체료 규제 동향을 지속적으로 모니터링하고, 미국향 수출입 시 컨테이너 반출입 지연을 최소화하기 위한 방안을 검토한다.</t>
+        </is>
+      </c>
+      <c r="H673" s="3" t="inlineStr">
+        <is>
+          <t>해양통신</t>
+        </is>
+      </c>
+      <c r="I673" s="3" t="inlineStr">
+        <is>
+          <t>https://oceanpress.co.kr/news/article.html?no=30558</t>
+        </is>
+      </c>
+      <c r="J673" s="3" t="inlineStr"/>
+    </row>
+    <row r="674">
+      <c r="A674" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B674" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C674" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D674" s="3" t="inlineStr">
+        <is>
+          <t>당국 화재로 석포제련소 내 유해 물질서 가스 발생 위험</t>
+        </is>
+      </c>
+      <c r="E674" s="3" t="inlineStr">
+        <is>
+          <t>석포제련소에서 발생한 화재로 인해 유해 물질에서 가스가 발생할 위험이 있다는 당국의 발표가 있었다.</t>
+        </is>
+      </c>
+      <c r="F674" s="3" t="inlineStr">
+        <is>
+          <t>제련소 화재 및 유해물질 발생은 원자재 공급망에 간접적인 영향을 미치거나 산업 전반의 안전 규제 강화 논의로 이어질 수 있어 추이를 모니터링할 필요가 있다.</t>
+        </is>
+      </c>
+      <c r="G674" s="3" t="inlineStr">
+        <is>
+          <t>해당 제련소의 생산 재개 여부 및 관련 산업 안전 규제 동향 주시.</t>
+        </is>
+      </c>
+      <c r="H674" s="3" t="inlineStr">
+        <is>
+          <t>한국경제</t>
+        </is>
+      </c>
+      <c r="I674" s="3" t="inlineStr">
+        <is>
+          <t>https://hankyung.com/article/2026070953077</t>
+        </is>
+      </c>
+      <c r="J674" s="3" t="inlineStr"/>
+    </row>
+    <row r="675">
+      <c r="A675" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B675" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C675" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D675" s="3" t="inlineStr">
+        <is>
+          <t>K-뷰티산업을 선도하는 전문 미디어,코스모닝</t>
+        </is>
+      </c>
+      <c r="E675" s="3" t="inlineStr">
+        <is>
+          <t>EU의 포장 및 포장 폐기물 규제(PPWR)가 다음 달부터 시행될 예정이며, 화장품 산업은 유해물질 관리, 재활용성 확보, 포장 최소화 등에서 구조적 충돌을 겪고 있어 우리 기업의 EU 수출 포장 전략에 영향을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="F675" s="3" t="inlineStr">
+        <is>
+          <t>EU PPWR은 화장품 산업에 대한 내용이지만, 포장재 및 유해물질 규제는 배터리/전자부품 수출에도 적용될 수 있으므로 우리 제품의 포장 및 재활용성 규제 준수 여부를 검토해야 한다.</t>
+        </is>
+      </c>
+      <c r="G675" s="3" t="inlineStr">
+        <is>
+          <t>EU 수출 제품의 포장재 및 유해물질 관련 규제(PPWR 포함) 준수 여부 점검 및 필요 시 포장 전략 재검토.</t>
+        </is>
+      </c>
+      <c r="H675" s="3" t="inlineStr">
+        <is>
+          <t>코스모닝</t>
+        </is>
+      </c>
+      <c r="I675" s="3" t="inlineStr">
+        <is>
+          <t>https://cosmorning.com/news/article.html?no=53123</t>
+        </is>
+      </c>
+      <c r="J675" s="3" t="inlineStr"/>
+    </row>
+    <row r="676">
+      <c r="A676" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B676" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C676" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D676" s="3" t="inlineStr">
+        <is>
+          <t>열차 멈추고 도로 잠기고…물폭탄 피해 속출</t>
+        </is>
+      </c>
+      <c r="E676" s="3" t="inlineStr">
+        <is>
+          <t>대전·세종 지역에 200mm 넘는 물폭탄이 쏟아져 KTX 등 열차 58대가 지연 운행되고 도로가 침수되는 등 국내 물류 운송에 차질이 발생했다.</t>
+        </is>
+      </c>
+      <c r="F676" s="3" t="inlineStr">
+        <is>
+          <t>집중호우로 인한 국내 철도 및 도로 운송 지연은 국내 공급망 및 생산 계획에 영향을 미칠 수 있으므로, 해당 지역의 운송 상황을 주시해야 한다.</t>
+        </is>
+      </c>
+      <c r="G676" s="3" t="inlineStr">
+        <is>
+          <t>국내 운송 경로 및 일정에 대한 잠재적 영향 평가, 대체 운송 수단 또는 경로 확보 가능성 검토.</t>
+        </is>
+      </c>
+      <c r="H676" s="3" t="inlineStr">
+        <is>
+          <t>매일경제</t>
+        </is>
+      </c>
+      <c r="I676" s="3" t="inlineStr">
+        <is>
+          <t>https://mk.co.kr/news/society/12094758</t>
+        </is>
+      </c>
+      <c r="J676" s="3" t="inlineStr"/>
+    </row>
+    <row r="677">
+      <c r="A677" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B677" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C677" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D677" s="3" t="inlineStr">
+        <is>
+          <t>[EBN 데이터센터] 중동 긴장 재부각에 국제유가 강세</t>
+        </is>
+      </c>
+      <c r="E677" s="3" t="inlineStr">
+        <is>
+          <t>중동 지역의 긴장 재부각과 미국-이란 간 군사적 대치로 국제유가가 강세를 보이며 상승 흐름을 나타내고 있다.</t>
+        </is>
+      </c>
+      <c r="F677" s="3" t="inlineStr">
+        <is>
+          <t>국제유가 강세는 해상 및 항공 운송 비용의 유류할증료 인상으로 이어져 물류비용 증가에 영향을 미칠 수 있으므로 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G677" s="3" t="inlineStr">
+        <is>
+          <t>유가 변동 추이를 면밀히 주시하고, 운송 계약 시 유류할증료 조건 등을 재검토하여 물류비용 증가에 대비해야 한다.</t>
+        </is>
+      </c>
+      <c r="H677" s="3" t="inlineStr">
+        <is>
+          <t>이비엔(EBN)뉴스센터</t>
+        </is>
+      </c>
+      <c r="I677" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebn.co.kr/news/articleView.html?idxno=1715662</t>
+        </is>
+      </c>
+      <c r="J677" s="3" t="inlineStr"/>
+    </row>
+    <row r="678">
+      <c r="A678" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B678" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C678" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D678" s="3" t="inlineStr">
+        <is>
+          <t>고유가·고환율 장기화...'밥상 물가 비상' [포토]</t>
+        </is>
+      </c>
+      <c r="E678" s="3" t="inlineStr">
+        <is>
+          <t>중동 정세 불안에 따른 국제유가 상승과 고환율 장기화로 수입 원자재 및 물류비가 동시에 상승하여 전반적인 물가 상승 압력이 커지고 있다.</t>
+        </is>
+      </c>
+      <c r="F678" s="3" t="inlineStr">
+        <is>
+          <t>고유가와 고환율 장기화는 수입 원자재 비용과 물류비용을 직접적으로 상승시켜 당사 SCM 비용에 부정적인 영향을 미칠 수 있으므로 면밀한 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G678" s="3" t="inlineStr">
+        <is>
+          <t>유가 및 환율 변동 추이를 지속적으로 모니터링하고, 물류비용 절감 방안 및 원자재 재고 관리 전략을 검토해야 한다.</t>
+        </is>
+      </c>
+      <c r="H678" s="3" t="inlineStr">
+        <is>
+          <t>이투데이</t>
+        </is>
+      </c>
+      <c r="I678" s="3" t="inlineStr">
+        <is>
+          <t>https://etoday.co.kr/news/view/2602036</t>
+        </is>
+      </c>
+      <c r="J678" s="3" t="inlineStr"/>
+    </row>
+    <row r="679">
+      <c r="A679" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B679" s="4" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C679" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D679" s="4" t="inlineStr">
+        <is>
+          <t>남아공 철강제품 수입관세 인상 동향과 우리 기업 대응 시사점</t>
+        </is>
+      </c>
+      <c r="E679" s="4" t="inlineStr">
+        <is>
+          <t>남아공 정부가 2026년 5월부터 철강 및 철강제품 전반에 대한 수입관세를 인상했으며, 이는 자국 산업 보호를 위한 조치이다.</t>
+        </is>
+      </c>
+      <c r="F679" s="4" t="inlineStr">
+        <is>
+          <t>당사는 배터리/전자부품 제조기업으로, 철강제품 관세 인상은 당사 수출입에 직접적인 영향이 없다.</t>
+        </is>
+      </c>
+      <c r="G679" s="4" t="inlineStr"/>
+      <c r="H679" s="4" t="inlineStr">
+        <is>
+          <t>kotra</t>
+        </is>
+      </c>
+      <c r="I679" s="4" t="inlineStr">
+        <is>
+          <t>https://dream.kotra.or.kr/kotranews/cms/news/actionKotraBoardDetail.do?SITE_NO=3&amp;MENU_ID=70&amp;CONTENTS_NO=1&amp;pNttSn=242572</t>
+        </is>
+      </c>
+      <c r="J679" s="4" t="inlineStr"/>
+    </row>
+    <row r="680">
+      <c r="A680" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B680" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C680" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D680" s="4" t="inlineStr">
+        <is>
+          <t>Global Schedule Reliability for May 2026 the Highest of the Year</t>
+        </is>
+      </c>
+      <c r="E680" s="4" t="inlineStr">
+        <is>
+          <t>2026년 5월 글로벌 선박 스케줄 신뢰도가 연중 최고치를 기록하며, 이는 운송 지연 감소에 긍정적인 신호이다.</t>
+        </is>
+      </c>
+      <c r="F680" s="4" t="inlineStr">
+        <is>
+          <t>스케줄 신뢰도 개선은 운송 지연 위험 감소에 긍정적이나, 지속적인 추이 확인이 필요하며 당장 높은 수준의 대응은 불필요하다.</t>
+        </is>
+      </c>
+      <c r="G680" s="4" t="inlineStr"/>
+      <c r="H680" s="4" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I680" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/395-global-schedule-reliability-for-may-2026-the-highest-of-the-year</t>
+        </is>
+      </c>
+      <c r="J680" s="4" t="inlineStr"/>
+    </row>
+    <row r="681">
+      <c r="A681" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B681" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C681" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D681" s="4" t="inlineStr">
+        <is>
+          <t>BPA, '제3회 친환경 북극항로 포럼' 성황리에 개최</t>
+        </is>
+      </c>
+      <c r="E681" s="4" t="inlineStr">
+        <is>
+          <t>부산항만공사가 친환경 북극항로 포럼을 개최하며 북극항로 활용 및 친환경 물류에 대한 논의를 본격화했다.</t>
+        </is>
+      </c>
+      <c r="F681" s="4" t="inlineStr">
+        <is>
+          <t>북극항로는 장기적인 관점의 대체 항로 논의로, 당장 우리 회사의 물류 운영에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G681" s="4" t="n"/>
+      <c r="H681" s="4" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I681" s="4" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260710-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J681" s="4" t="inlineStr"/>
+    </row>
+    <row r="682">
+      <c r="A682" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B682" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C682" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D682" s="4" t="inlineStr">
+        <is>
+          <t>부산진해경자청, 동북아 콜드체인 허브 구축 본격화…Sea&amp;Air 물류전략 착수</t>
+        </is>
+      </c>
+      <c r="E682" s="4" t="inlineStr">
+        <is>
+          <t>부산진해경제자유구역청이 부산항과 가덕도신공항을 연계하여 동북아 콜드체인 물류 허브 구축 전략을 본격 추진한다.</t>
+        </is>
+      </c>
+      <c r="F682" s="4" t="inlineStr">
+        <is>
+          <t>콜드체인 물류 허브 구축은 장기적인 인프라 개선으로, 당장 우리 회사의 배터리/전자부품 물류에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G682" s="4" t="n"/>
+      <c r="H682" s="4" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I682" s="4" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260709-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J682" s="4" t="inlineStr"/>
+    </row>
+    <row r="683">
+      <c r="A683" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B683" s="4" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C683" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D683" s="4" t="inlineStr">
+        <is>
+          <t>이란·카타르 해상 교역 재개…'5개월 중단' 알</t>
+        </is>
+      </c>
+      <c r="E683" s="4" t="inlineStr">
+        <is>
+          <t>이란과 카타르 간 해상 교역이 5개월 만에 재개되어 중동 지역 내 일부 교역 관계가 정상화되었다.</t>
+        </is>
+      </c>
+      <c r="F683" s="4" t="inlineStr">
+        <is>
+          <t>이란-카타르 간 해상 교역 재개는 지역적인 이슈로, 우리 회사의 글로벌 물류 운영에 직접적인 영향은 미미하다.</t>
+        </is>
+      </c>
+      <c r="G683" s="4" t="n"/>
+      <c r="H683" s="4" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I683" s="4" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260706-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J683" s="4" t="inlineStr"/>
+    </row>
+    <row r="684">
+      <c r="A684" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B684" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C684" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D684" s="4" t="inlineStr">
+        <is>
+          <t>두핸즈 XFC 센터 / AI 기반 모듈형 자동화 물류거점 ‘XFC 센터’ 본격 가동</t>
+        </is>
+      </c>
+      <c r="E684" s="4" t="inlineStr">
+        <is>
+          <t>풀필먼트 서비스 '품고'를 운영하는 두핸즈가 AI 기반 모듈형 자동화 물류거점 'XFC 센터'를 개소하고 포장 자동화부터 휴머노이드까지 차세대 풀필먼트 기술 실증에 나섰다.</t>
+        </is>
+      </c>
+      <c r="F684" s="4" t="inlineStr">
+        <is>
+          <t>특정 풀필먼트 업체의 AI 기반 자동화 물류센터 가동은 물류 기술 트렌드를 보여주지만, 당장 우리 회사의 물류 운영에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G684" s="4" t="n"/>
+      <c r="H684" s="4" t="inlineStr">
+        <is>
+          <t>ulogistics</t>
+        </is>
+      </c>
+      <c r="I684" s="4" t="inlineStr">
+        <is>
+          <t>http://www.ulogistics.co.kr/test/board.php?board=all2&amp;command=body&amp;no=5203</t>
+        </is>
+      </c>
+      <c r="J684" s="4" t="inlineStr"/>
+    </row>
+    <row r="685">
+      <c r="A685" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B685" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C685" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D685" s="4" t="inlineStr">
+        <is>
+          <t>Explainer: What the UK’s new Supply Chain Centre means for logistics</t>
+        </is>
+      </c>
+      <c r="E685" s="4" t="inlineStr">
+        <is>
+          <t>영국 정부가 지정학적 불안정, 기후 관련 혼란 등에 대응하여 공급망 복원력을 강화하고 핵심 산업 투입재 접근성을 개선하기 위한 공급망 센터를 설립했다.</t>
+        </is>
+      </c>
+      <c r="F685" s="4" t="inlineStr">
+        <is>
+          <t>영국 정부의 공급망 센터 설립은 국가 차원의 공급망 복원력 강화 노력으로, 우리 회사의 직접적인 물류 운영에 당장 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G685" s="4" t="n"/>
+      <c r="H685" s="4" t="inlineStr">
+        <is>
+          <t>Logistics Manager</t>
+        </is>
+      </c>
+      <c r="I685" s="4" t="inlineStr">
+        <is>
+          <t>https://logisticsmanager.com/explainer-what-the-uks-new-supply-chain-centre-means-for-logistics</t>
+        </is>
+      </c>
+      <c r="J685" s="4" t="inlineStr"/>
+    </row>
+    <row r="686">
+      <c r="A686" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B686" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C686" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D686" s="4" t="inlineStr">
+        <is>
+          <t>Beating the Hours-of-Service (HOS) Clock: How Smart Route Planning Keeps Your Long-Haul OTR Freight Moving</t>
+        </is>
+      </c>
+      <c r="E686" s="4" t="inlineStr">
+        <is>
+          <t>장거리 육상 운송에서 운전자의 운행 시간 규제(HOS)를 준수하며 화물을 효율적으로 운송하기 위한 스마트 경로 계획의 중요성을 강조한다.</t>
+        </is>
+      </c>
+      <c r="F686" s="4" t="inlineStr">
+        <is>
+          <t>미국 내 육상 운송 규제 및 효율화 방안은 우리 회사의 글로벌 해상/항공 운송 중심의 물류 운영에 직접적인 영향은 미미하다.</t>
+        </is>
+      </c>
+      <c r="G686" s="4" t="n"/>
+      <c r="H686" s="4" t="inlineStr">
+        <is>
+          <t>Jansson LLC</t>
+        </is>
+      </c>
+      <c r="I686" s="4" t="inlineStr">
+        <is>
+          <t>https://janssonllc.com/logbook/beating-the-hours-of-service-hos-clock-how-smart-route-planning-keeps-your-long-haul-otr-freight-moving</t>
+        </is>
+      </c>
+      <c r="J686" s="4" t="inlineStr"/>
+    </row>
+    <row r="687">
+      <c r="A687" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B687" s="4" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C687" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D687" s="4" t="inlineStr">
+        <is>
+          <t>"공급 부족에 가격 급등"… 올해 글로벌 천연가스 수요 역성장 전망</t>
+        </is>
+      </c>
+      <c r="E687" s="4" t="inlineStr">
+        <is>
+          <t>중동 지정학적 갈등으로 글로벌 천연가스 공급 부족과 가격 급등이 예상되며, 이는 전 세계 천연가스 소비량 역성장으로 이어질 전망이다.</t>
+        </is>
+      </c>
+      <c r="F687" s="4" t="inlineStr">
+        <is>
+          <t>천연가스 가격 변동은 배터리 제조 공정의 에너지 비용에 간접적인 영향을 줄 수 있으나, 당사 물류 운영에 직접적인 영향은 미미하다.</t>
+        </is>
+      </c>
+      <c r="G687" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H687" s="4" t="inlineStr">
+        <is>
+          <t>ESG비즈니스리뷰</t>
+        </is>
+      </c>
+      <c r="I687" s="4" t="inlineStr">
+        <is>
+          <t>https://esgbusinessreview.kr/news/articleView.html?idxno=6760</t>
+        </is>
+      </c>
+      <c r="J687" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -31298,7 +32986,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -31904,6 +33592,49 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>3326.87</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>+87 (+2.7%)</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>+1,457 (+77.9%)</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>4330</v>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>+410 (+10.5%)</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>+1,619 (+59.7%)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -31916,7 +33647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I111"/>
+  <dimension ref="A1:I121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -35827,6 +37558,356 @@
       </c>
       <c r="I111" s="6" t="inlineStr"/>
     </row>
+    <row r="112">
+      <c r="A112" s="6" t="inlineStr">
+        <is>
+          <t>RSK-111</t>
+        </is>
+      </c>
+      <c r="B112" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C112" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D112" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E112" s="6" t="inlineStr">
+        <is>
+          <t>"다시 강력 공격" 트럼프 예고대로…미군, 연이틀 이란 공습</t>
+        </is>
+      </c>
+      <c r="F112" s="6" t="inlineStr"/>
+      <c r="G112" s="6" t="inlineStr"/>
+      <c r="H112" s="6" t="inlineStr">
+        <is>
+          <t>유가 및 해상 운임 변동 추이를 면밀히 모니터링하고, 중동 경유 항로의 잠재적 지연 또는 중단 가능성에 대비하여 대체 운송 경로 및 비상 계획을 수립한다.</t>
+        </is>
+      </c>
+      <c r="I112" s="6" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="6" t="inlineStr">
+        <is>
+          <t>RSK-112</t>
+        </is>
+      </c>
+      <c r="B113" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C113" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D113" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E113" s="6" t="inlineStr">
+        <is>
+          <t>현대글로비스, 일시적 충격에도 본질은 견조</t>
+        </is>
+      </c>
+      <c r="F113" s="6" t="inlineStr"/>
+      <c r="G113" s="6" t="inlineStr"/>
+      <c r="H113" s="6" t="inlineStr">
+        <is>
+          <t>유가 및 벙커유 가격 변동을 면밀히 모니터링하고, BAF 적용 시차에 따른 물류비 상승에 대비하여 운송 계약 조건을 재검토하거나 대체 운송 방안을 고려한다.</t>
+        </is>
+      </c>
+      <c r="I113" s="6" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="6" t="inlineStr">
+        <is>
+          <t>RSK-113</t>
+        </is>
+      </c>
+      <c r="B114" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C114" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D114" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E114" s="6" t="inlineStr">
+        <is>
+          <t>미군, 이란 공습 시작 및 원유 제재 면제 철회로 호르무즈 해협 긴장 최고조</t>
+        </is>
+      </c>
+      <c r="F114" s="6" t="inlineStr"/>
+      <c r="G114" s="6" t="inlineStr"/>
+      <c r="H114" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 상황을 실시간으로 모니터링하고, 비상시 대체 운송 경로(육상/항공) 및 재고 확보, 선사와의 긴밀한 소통을 통한 운송 계획 조정을 준비한다.</t>
+        </is>
+      </c>
+      <c r="I114" s="6" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="6" t="inlineStr">
+        <is>
+          <t>RSK-114</t>
+        </is>
+      </c>
+      <c r="B115" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C115" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D115" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E115" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈 선박 피격에 국제유가 급등…브렌트유 3%↑</t>
+        </is>
+      </c>
+      <c r="F115" s="6" t="inlineStr"/>
+      <c r="G115" s="6" t="inlineStr"/>
+      <c r="H115" s="6" t="inlineStr">
+        <is>
+          <t>유가 변동에 따른 물류비용 상승을 예측하고, 운송 계약 조건(유류할증료 등)을 검토하며, 필요시 재고 수준 조정 및 운송 방식 다변화를 고려한다.</t>
+        </is>
+      </c>
+      <c r="I115" s="6" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="6" t="inlineStr">
+        <is>
+          <t>RSK-115</t>
+        </is>
+      </c>
+      <c r="B116" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C116" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D116" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E116" s="6" t="inlineStr">
+        <is>
+          <t>산업硏 "호르무즈 봉쇄로 한국 제조업 생산비 4.7% 뛰어"</t>
+        </is>
+      </c>
+      <c r="F116" s="6" t="inlineStr"/>
+      <c r="G116" s="6" t="inlineStr"/>
+      <c r="H116" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 봉쇄 시나리오에 대비하여 대체 운송 경로 및 운송 수단 확보 방안을 구체화하고, 비상 재고 수준을 검토하며, 물류비용 상승에 대한 재무적 영향을 분석한다.</t>
+        </is>
+      </c>
+      <c r="I116" s="6" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="6" t="inlineStr">
+        <is>
+          <t>RSK-116</t>
+        </is>
+      </c>
+      <c r="B117" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C117" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D117" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E117" s="6" t="inlineStr">
+        <is>
+          <t>전쟁 리스크에 출렁이는 해운시장…중동 항로 운임 변동성 80% 급증</t>
+        </is>
+      </c>
+      <c r="F117" s="6" t="inlineStr"/>
+      <c r="G117" s="6" t="inlineStr"/>
+      <c r="H117" s="6" t="inlineStr">
+        <is>
+          <t>중동 항로 운임 변동성 추이를 면밀히 주시하고, 대체 항로 및 운송 수단 확보 방안을 검토하며, 운송 계약 시 위험 분산 조항을 강화한다.</t>
+        </is>
+      </c>
+      <c r="I117" s="6" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="6" t="inlineStr">
+        <is>
+          <t>RSK-117</t>
+        </is>
+      </c>
+      <c r="B118" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C118" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D118" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E118" s="6" t="inlineStr">
+        <is>
+          <t>이란發 인플레 악몽 되살아나나…세계 공급망 다시 긴장</t>
+        </is>
+      </c>
+      <c r="F118" s="6" t="inlineStr"/>
+      <c r="G118" s="6" t="inlineStr"/>
+      <c r="H118" s="6" t="inlineStr">
+        <is>
+          <t>유가 및 해상 운임 변동성 모니터링 강화, 운송 계약 조건 재검토, 잠재적 비용 상승에 대비한 예산 조정 및 재고 전략 검토.</t>
+        </is>
+      </c>
+      <c r="I118" s="6" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="6" t="inlineStr">
+        <is>
+          <t>RSK-118</t>
+        </is>
+      </c>
+      <c r="B119" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C119" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D119" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E119" s="6" t="inlineStr">
+        <is>
+          <t>IMF, 美 경제 진단... “이란 전쟁 여파로 인플레 충격, 2027년까지 지속”</t>
+        </is>
+      </c>
+      <c r="F119" s="6" t="inlineStr"/>
+      <c r="G119" s="6" t="inlineStr"/>
+      <c r="H119" s="6" t="inlineStr">
+        <is>
+          <t>장기적인 물류비용 상승 시나리오 분석, 미국 시장 수출 시 관세 및 운임 변동성 고려한 가격 및 공급망 전략 수립.</t>
+        </is>
+      </c>
+      <c r="I119" s="6" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="6" t="inlineStr">
+        <is>
+          <t>RSK-119</t>
+        </is>
+      </c>
+      <c r="B120" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C120" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D120" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E120" s="6" t="inlineStr">
+        <is>
+          <t>“중국산 막히면 서방 제조업 올스톱”…G2 전장, 칩에서 광물로 [텅스텐 War ②]</t>
+        </is>
+      </c>
+      <c r="F120" s="6" t="inlineStr"/>
+      <c r="G120" s="6" t="inlineStr"/>
+      <c r="H120" s="6" t="inlineStr">
+        <is>
+          <t>핵심 광물 재고 수준 점검, 중국 외 대체 공급처 발굴 및 다변화 전략 수립, 공급망 리스크 시나리오별 대응 계획 마련.</t>
+        </is>
+      </c>
+      <c r="I120" s="6" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="6" t="inlineStr">
+        <is>
+          <t>RSK-120</t>
+        </is>
+      </c>
+      <c r="B121" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C121" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D121" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E121" s="6" t="inlineStr">
+        <is>
+          <t>정부, WTO서 해외 기술규제 8건 제기…수출 애로 해소 나선다</t>
+        </is>
+      </c>
+      <c r="F121" s="6" t="inlineStr"/>
+      <c r="G121" s="6" t="inlineStr"/>
+      <c r="H121" s="6" t="inlineStr">
+        <is>
+          <t>현재 수출 중인 제품에 대한 각국의 기술규제 현황을 파악하고, 잠재적 영향을 분석하여 필요시 제품 설계 변경 또는 인증 획득 계획을 수립해야 한다.</t>
+        </is>
+      </c>
+      <c r="I121" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
📰 뉴스 데이터 2026-07-13_08:53
</commit_message>
<xml_diff>
--- a/data/SCM_물류_브리핑.xlsx
+++ b/data/SCM_물류_브리핑.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J687"/>
+  <dimension ref="A1:J712"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -32974,6 +32974,1154 @@
       </c>
       <c r="J687" s="4" t="inlineStr"/>
     </row>
+    <row r="688">
+      <c r="A688" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B688" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C688" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D688" s="2" t="inlineStr">
+        <is>
+          <t>20260713 경제·물류 주요뉴스 (데일리스크랩)</t>
+        </is>
+      </c>
+      <c r="E688" s="2" t="inlineStr">
+        <is>
+          <t>유가 급등 경고와 함께 미-이란 간 호르무즈 해협 통제권 갈등이 재점화되어 오만이 남북 2개 항로를 제안하는 등 중동 정세 불안이 고조되고 있다.</t>
+        </is>
+      </c>
+      <c r="F688" s="2" t="inlineStr">
+        <is>
+          <t>주요 해상 운송로인 호르무즈 해협의 지정학적 갈등은 즉각적인 운송 지연, 운임 상승 및 공급망 불안정을 야기할 수 있으며, 유가 급등은 물류비에 직접적인 영향을 미친다.</t>
+        </is>
+      </c>
+      <c r="G688" s="2" t="inlineStr">
+        <is>
+          <t>중동 항로 이용 시 대체 항로 및 운송 수단 검토, 선사와의 비상 계획 수립 논의, 유가 변동 추이 모니터링 및 운임 계약 조건 재검토.</t>
+        </is>
+      </c>
+      <c r="H688" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I688" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260713-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J688" s="2" t="inlineStr">
+        <is>
+          <t>RSK-121</t>
+        </is>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B689" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C689" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D689" s="2" t="inlineStr">
+        <is>
+          <t>이란 "호르무즈 해협 봉쇄하겠다"</t>
+        </is>
+      </c>
+      <c r="E689" s="2" t="inlineStr">
+        <is>
+          <t>이란이 호르무즈 해협 봉쇄를 위협하며, 이는 글로벌 에너지 공급망과 물류에 심각한 파급 효과를 미칠 수 있는 중요한 지정학적 사안입니다.</t>
+        </is>
+      </c>
+      <c r="F689" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 봉쇄는 글로벌 해상 운송 경로와 유가에 직접적인 영향을 미쳐 우리 물류 운영 및 비용에 즉각적인 차질을 초래할 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G689" s="2" t="inlineStr">
+        <is>
+          <t>대체 운송 경로 및 운송사 옵션 검토, 유가 변동에 따른 물류비 상승 시나리오 분석, 재고 수준 및 리드타임 영향 평가.</t>
+        </is>
+      </c>
+      <c r="H689" s="2" t="inlineStr">
+        <is>
+          <t>매일경제</t>
+        </is>
+      </c>
+      <c r="I689" s="2" t="inlineStr">
+        <is>
+          <t>https://mk.co.kr/news/world/12096599</t>
+        </is>
+      </c>
+      <c r="J689" s="2" t="inlineStr">
+        <is>
+          <t>RSK-122</t>
+        </is>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B690" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C690" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D690" s="3" t="inlineStr">
+        <is>
+          <t>Air Cargo Demand Up 6.0% in May</t>
+        </is>
+      </c>
+      <c r="E690" s="3" t="inlineStr">
+        <is>
+          <t>2026년 5월 글로벌 항공 화물 수요가 전년 동기 대비 6.0% 증가했다.</t>
+        </is>
+      </c>
+      <c r="F690" s="3" t="inlineStr">
+        <is>
+          <t>항공 화물 수요 증가는 향후 항공 운임 상승 압력으로 작용하거나, 특정 노선에서 공간 확보에 어려움을 줄 수 있으므로 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G690" s="3" t="n"/>
+      <c r="H690" s="3" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I690" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-29-air-cargo-demand-up-may/</t>
+        </is>
+      </c>
+      <c r="J690" s="3" t="inlineStr"/>
+    </row>
+    <row r="691">
+      <c r="A691" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B691" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C691" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D691" s="3" t="inlineStr">
+        <is>
+          <t>글로벌 정기선사들 항만 연결성 적극적으로 재편</t>
+        </is>
+      </c>
+      <c r="E691" s="3" t="inlineStr">
+        <is>
+          <t>글로벌 정기선사들이 기존 주요 환적 허브 중심의 항로를 축소하고 인도 및 중동 등 지역 중계항으로 네트워크를 분산 및 재편하고 있다.</t>
+        </is>
+      </c>
+      <c r="F691" s="3" t="inlineStr">
+        <is>
+          <t>주요 항만의 연결성 변화는 우리 회사의 해상 운송 경로 및 리드타임에 영향을 줄 수 있으므로, 주요 항로의 변화를 모니터링하고 필요시 운송 전략을 재검토해야 한다.</t>
+        </is>
+      </c>
+      <c r="G691" s="3" t="inlineStr">
+        <is>
+          <t>주요 항로 및 환적 허브 변화 모니터링, 운송 리드타임 및 비용 영향 분석 준비</t>
+        </is>
+      </c>
+      <c r="H691" s="3" t="inlineStr">
+        <is>
+          <t>kita</t>
+        </is>
+      </c>
+      <c r="I691" s="3" t="inlineStr">
+        <is>
+          <t>https://www.kita.net/shippers/board/newsView.do?morgueCode=2&amp;dataCls=B&amp;dataSeq=8160</t>
+        </is>
+      </c>
+      <c r="J691" s="3" t="inlineStr"/>
+    </row>
+    <row r="692">
+      <c r="A692" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B692" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C692" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D692" s="3" t="inlineStr">
+        <is>
+          <t>Structural Contraction of Global Liner Networks</t>
+        </is>
+      </c>
+      <c r="E692" s="3" t="inlineStr">
+        <is>
+          <t>2012년 이후 글로벌 정기선 네트워크가 구조적으로 축소되어, 선사들이 지리적 범위는 유지하나 서비스 빈도를 줄이고 있다.</t>
+        </is>
+      </c>
+      <c r="F692" s="3" t="inlineStr">
+        <is>
+          <t>선사들의 서비스 빈도 감소는 특정 노선의 운송 옵션 감소 및 리드타임 증가로 이어질 수 있으므로, 주요 노선의 서비스 변화를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G692" s="3" t="inlineStr">
+        <is>
+          <t>주요 해상 운송 노선의 서비스 빈도 및 운송 옵션 변화 모니터링</t>
+        </is>
+      </c>
+      <c r="H692" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I692" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/397-structural-contraction-of-global-liner-networks</t>
+        </is>
+      </c>
+      <c r="J692" s="3" t="inlineStr"/>
+    </row>
+    <row r="693">
+      <c r="A693" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B693" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C693" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D693" s="3" t="inlineStr">
+        <is>
+          <t>PLSCI Data Indicates Mega-Hub Retrenchment</t>
+        </is>
+      </c>
+      <c r="E693" s="3" t="inlineStr">
+        <is>
+          <t>UNCTAD의 PLSCI 데이터 분석 결과, 최근 선사들의 네트워크 재편이 메가 허브 항만의 연결성 축소로 이어지고 있음을 시사한다.</t>
+        </is>
+      </c>
+      <c r="F693" s="3" t="inlineStr">
+        <is>
+          <t>주요 메가 허브 항만의 연결성 축소는 우리 회사의 해상 운송 경로 및 환적 효율성에 영향을 줄 수 있으므로, 주요 항만의 연결성 변화를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G693" s="3" t="inlineStr">
+        <is>
+          <t>주요 메가 허브 항만의 연결성 변화 모니터링 및 잠재적 운송 경로 영향 분석</t>
+        </is>
+      </c>
+      <c r="H693" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I693" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/396-plsci-data-indicates-mega-hub-retrenchment</t>
+        </is>
+      </c>
+      <c r="J693" s="3" t="inlineStr"/>
+    </row>
+    <row r="694">
+      <c r="A694" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B694" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C694" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D694" s="3" t="inlineStr">
+        <is>
+          <t>Tracking True Vessel Delay</t>
+        </is>
+      </c>
+      <c r="E694" s="3" t="inlineStr">
+        <is>
+          <t>선사들이 운송 시간을 늘려 스케줄 버퍼링에 의존하는 경향이 증가하고 있으며, 이는 실제 선박 지연과 스케줄 정시성 간의 관계를 분석하는 데 중요하다.</t>
+        </is>
+      </c>
+      <c r="F694" s="3" t="inlineStr">
+        <is>
+          <t>선사들의 스케줄 버퍼링 증가는 겉으로는 정시성이 개선된 것처럼 보일 수 있으나, 실제 운송 리드타임이 길어질 수 있음을 의미하므로, 우리 회사의 운송 계획에 미치는 영향을 면밀히 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G694" s="3" t="inlineStr">
+        <is>
+          <t>실제 운송 리드타임과 선사 제공 스케줄 간의 차이 분석 및 모니터링 강화</t>
+        </is>
+      </c>
+      <c r="H694" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I694" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/394-tracking-true-vessel-delay</t>
+        </is>
+      </c>
+      <c r="J694" s="3" t="inlineStr"/>
+    </row>
+    <row r="695">
+      <c r="A695" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B695" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C695" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D695" s="3" t="inlineStr">
+        <is>
+          <t>Transpacific: Ripe for new non-alliance services</t>
+        </is>
+      </c>
+      <c r="E695" s="3" t="inlineStr">
+        <is>
+          <t>태평양 횡단 노선에서 비동맹 선사들의 신규 서비스가 증가할 가능성이 있으며, 이는 운임 경쟁 심화로 이어질 수 있다.</t>
+        </is>
+      </c>
+      <c r="F695" s="3" t="inlineStr">
+        <is>
+          <t>태평양 횡단 노선은 우리 회사의 주요 운송 경로 중 하나일 수 있으며, 신규 서비스 증가는 운임 하락 압력으로 작용할 수 있으므로 시장 동향을 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G695" s="3" t="inlineStr">
+        <is>
+          <t>태평양 횡단 노선 운임 및 서비스 공급 변화 모니터링</t>
+        </is>
+      </c>
+      <c r="H695" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I695" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/393-transpacific-ripe-for-new-non-alliance-services</t>
+        </is>
+      </c>
+      <c r="J695" s="3" t="inlineStr"/>
+    </row>
+    <row r="696">
+      <c r="A696" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B696" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C696" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D696" s="3" t="inlineStr">
+        <is>
+          <t>20260710 경제·물류 주요뉴스 (데일리스크랩)</t>
+        </is>
+      </c>
+      <c r="E696" s="3" t="inlineStr">
+        <is>
+          <t>해운시장은 수에즈 운하 정상화와 우회 선복 복귀 속도가 핵심 변수로 작용할 것이며, 부산항만공사는 친환경 북극항로 포럼을 개최하며 관련 논의를 본격화했다.</t>
+        </is>
+      </c>
+      <c r="F696" s="3" t="inlineStr">
+        <is>
+          <t>수에즈 운하 정상화는 긍정적이나 해운 시장의 변동성이 지속될 수 있어 선복 공급 및 운임 추이를 모니터링할 필요가 있으며, 북극항로는 장기적인 논의 단계이다.</t>
+        </is>
+      </c>
+      <c r="G696" s="3" t="inlineStr">
+        <is>
+          <t>해운 시장 동향 및 선복 공급 변화 지속 모니터링.</t>
+        </is>
+      </c>
+      <c r="H696" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I696" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260710-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J696" s="3" t="inlineStr"/>
+    </row>
+    <row r="697">
+      <c r="A697" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B697" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C697" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D697" s="3" t="inlineStr">
+        <is>
+          <t>아시아역내 '컨' 운임, 7주 만에 1000달러선 붕괴</t>
+        </is>
+      </c>
+      <c r="E697" s="3" t="inlineStr">
+        <is>
+          <t>아시아 역내 컨테이너 운임지수가 3주 연속 하락하며 7주 만에 처음으로 FEU당 1,000달러 아래로 떨어졌다.</t>
+        </is>
+      </c>
+      <c r="F697" s="3" t="inlineStr">
+        <is>
+          <t>운임 하락은 긍정적 신호이나, 아시아 역내 운임에 국한되며 장거리 운송에 미치는 영향과 추세 지속 여부를 모니터링할 필요가 있다.</t>
+        </is>
+      </c>
+      <c r="G697" s="3" t="inlineStr">
+        <is>
+          <t>운임 변동 추이 지속 모니터링 및 향후 운임 협상 시 참고.</t>
+        </is>
+      </c>
+      <c r="H697" s="3" t="inlineStr">
+        <is>
+          <t>해양통신</t>
+        </is>
+      </c>
+      <c r="I697" s="3" t="inlineStr">
+        <is>
+          <t>https://oceanpress.co.kr/news/article.html?no=30582</t>
+        </is>
+      </c>
+      <c r="J697" s="3" t="inlineStr"/>
+    </row>
+    <row r="698">
+      <c r="A698" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B698" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C698" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D698" s="3" t="inlineStr">
+        <is>
+          <t>이스라엘 점령지와 무역 어쩌나…유럽 골머리</t>
+        </is>
+      </c>
+      <c r="E698" s="3" t="inlineStr">
+        <is>
+          <t>유럽연합이 이스라엘의 팔레스타인 점령지 정착촌과의 무역 문제로 고심하고 있으며, 이는 향후 무역 정책 변화로 이어질 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="F698" s="3" t="inlineStr">
+        <is>
+          <t>이스라엘 점령지와의 무역 관련 유럽의 고민은 향후 무역 정책 변화나 공급망 리스크로 이어질 수 있어 추이를 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G698" s="3" t="n"/>
+      <c r="H698" s="3" t="inlineStr">
+        <is>
+          <t>연합뉴스</t>
+        </is>
+      </c>
+      <c r="I698" s="3" t="inlineStr">
+        <is>
+          <t>https://yna.co.kr/view/AKR20260712050900085</t>
+        </is>
+      </c>
+      <c r="J698" s="3" t="inlineStr"/>
+    </row>
+    <row r="699">
+      <c r="A699" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B699" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C699" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D699" s="3" t="inlineStr">
+        <is>
+          <t>현대화된 EU-멕시코 협정에 대한 경제 분석: 대서양 무역 구조의 재편</t>
+        </is>
+      </c>
+      <c r="E699" s="3" t="inlineStr">
+        <is>
+          <t>현대화된 EU-멕시코 협정은 유럽 기업에 새로운 수출 기회를 제공하고 대서양 무역 구조를 재편할 잠재력이 있습니다.</t>
+        </is>
+      </c>
+      <c r="F699" s="3" t="inlineStr">
+        <is>
+          <t>EU-멕시코 무역 협정은 대서양 무역 구조에 변화를 가져와 향후 우리 기업의 수출입 전략 및 물류 경로에 영향을 줄 수 있으므로 추이를 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G699" s="3" t="n"/>
+      <c r="H699" s="3" t="inlineStr">
+        <is>
+          <t>xpert.digital</t>
+        </is>
+      </c>
+      <c r="I699" s="3" t="inlineStr">
+        <is>
+          <t>https://xpert.digital/ko/eu-%EB%A9%95%EC%8B%9C%EC%BD%94-%ED%98%91%EC%A0%95</t>
+        </is>
+      </c>
+      <c r="J699" s="3" t="inlineStr"/>
+    </row>
+    <row r="700">
+      <c r="A700" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B700" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C700" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D700" s="3" t="inlineStr">
+        <is>
+          <t>주유소 기름값 8주 연속 하락…전국 휘발유 가격 1893원 [포토로그]</t>
+        </is>
+      </c>
+      <c r="E700" s="3" t="inlineStr">
+        <is>
+          <t>전국 주유소 기름값이 8주 연속 하락세를 이어가며 휘발유 가격이 1800원대를 기록했습니다.</t>
+        </is>
+      </c>
+      <c r="F700" s="3" t="inlineStr">
+        <is>
+          <t>국내 유가 하락세는 육상 운송 비용에 긍정적인 영향을 미칠 수 있으나, 국제 유가 및 해상/항공 운임에 미치는 영향은 지속적으로 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G700" s="3" t="n"/>
+      <c r="H700" s="3" t="inlineStr">
+        <is>
+          <t>이투데이</t>
+        </is>
+      </c>
+      <c r="I700" s="3" t="inlineStr">
+        <is>
+          <t>https://etoday.co.kr/news/view/2602777</t>
+        </is>
+      </c>
+      <c r="J700" s="3" t="inlineStr"/>
+    </row>
+    <row r="701">
+      <c r="A701" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B701" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C701" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D701" s="3" t="inlineStr">
+        <is>
+          <t>미·이란 충돌 격화에 국제 유가 3% 이상 상승</t>
+        </is>
+      </c>
+      <c r="E701" s="3" t="inlineStr">
+        <is>
+          <t>미국과 이란의 호르무즈 해협을 둘러싼 갈등이 격화되면서 국제 유가가 3% 이상 상승하여 해상 및 항공 운임의 유류할증료 인상 압박이 커지고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F701" s="3" t="inlineStr">
+        <is>
+          <t>국제 유가 상승은 배터리/전자부품 운송에 필수적인 해상 및 항공 운임의 유류할증료에 직접적인 영향을 미쳐 물류비용 증가 가능성을 높이므로 지속적인 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G701" s="3" t="inlineStr">
+        <is>
+          <t>국제 유가 및 해상/항공 운임 추이를 면밀히 모니터링하고, 잠재적인 물류비용 상승에 대비하여 운송 계약 조건 및 예산 계획을 검토해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H701" s="3" t="inlineStr">
+        <is>
+          <t>이데일리</t>
+        </is>
+      </c>
+      <c r="I701" s="3" t="inlineStr">
+        <is>
+          <t>https://edaily.co.kr/News/Read?mediaCodeNo=257&amp;newsId=02043446645514192</t>
+        </is>
+      </c>
+      <c r="J701" s="3" t="inlineStr"/>
+    </row>
+    <row r="702">
+      <c r="A702" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B702" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C702" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D702" s="4" t="inlineStr">
+        <is>
+          <t>러 철도 ‘컨’ 물동량 상반기 '13% 증가'</t>
+        </is>
+      </c>
+      <c r="E702" s="4" t="inlineStr">
+        <is>
+          <t>러시아 철도 컨테이너 물동량이 상반기 3.7%, 6월 13% 증가했으며, 특히 극동철도 물동량이 크게 늘었다.</t>
+        </is>
+      </c>
+      <c r="F702" s="4" t="inlineStr">
+        <is>
+          <t>우리 회사의 주요 운송 경로가 러시아 철도에 크게 의존하지 않는 한 직접적인 영향은 낮으며, 글로벌 물류 흐름의 참고 자료로 활용 가능하다.</t>
+        </is>
+      </c>
+      <c r="G702" s="4" t="n"/>
+      <c r="H702" s="4" t="inlineStr">
+        <is>
+          <t>cargonews</t>
+        </is>
+      </c>
+      <c r="I702" s="4" t="inlineStr">
+        <is>
+          <t>https://www.cargonews.co.kr/news/articleView.html?idxno=60507</t>
+        </is>
+      </c>
+      <c r="J702" s="4" t="inlineStr"/>
+    </row>
+    <row r="703">
+      <c r="A703" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B703" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C703" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D703" s="4" t="inlineStr">
+        <is>
+          <t>IATA Outlines Four Priorities to Strengthen the Aviation Supply Chain</t>
+        </is>
+      </c>
+      <c r="E703" s="4" t="inlineStr">
+        <is>
+          <t>IATA가 항공 공급망 강화를 위한 네 가지 우선순위를 제시했으며, 이는 항공 화물 운송의 안정성 및 효율성 개선에 기여할 수 있다.</t>
+        </is>
+      </c>
+      <c r="F703" s="4" t="inlineStr">
+        <is>
+          <t>장기적인 관점에서 긍정적일 수 있으나, 당장 우리 회사의 물류 운영에 직접적인 영향을 미치지는 않는다.</t>
+        </is>
+      </c>
+      <c r="G703" s="4" t="n"/>
+      <c r="H703" s="4" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I703" s="4" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-24-iata-outlines-four-priorities-to-strengthen-aviation-supply-chain/</t>
+        </is>
+      </c>
+      <c r="J703" s="4" t="inlineStr"/>
+    </row>
+    <row r="704">
+      <c r="A704" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B704" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C704" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D704" s="4" t="inlineStr">
+        <is>
+          <t>‘40년만의 귀환’ 흥아해운, 부산 간다…국내해운 4번째</t>
+        </is>
+      </c>
+      <c r="E704" s="4" t="inlineStr">
+        <is>
+          <t>흥아해운이 40년 만에 본사를 부산으로 이전하며, 친환경 대형선 중심의 글로벌 특수선 해운기업으로 도약할 계획이다.</t>
+        </is>
+      </c>
+      <c r="F704" s="4" t="inlineStr">
+        <is>
+          <t>국내 해운사의 본사 이전은 우리 회사의 물류 운영에 직접적인 영향을 주지 않는다.</t>
+        </is>
+      </c>
+      <c r="G704" s="4" t="n"/>
+      <c r="H704" s="4" t="inlineStr">
+        <is>
+          <t>ksg</t>
+        </is>
+      </c>
+      <c r="I704" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksg.co.kr/news/main_newsView.jsp?pNum=147583</t>
+        </is>
+      </c>
+      <c r="J704" s="4" t="inlineStr"/>
+    </row>
+    <row r="705">
+      <c r="A705" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B705" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C705" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D705" s="4" t="inlineStr">
+        <is>
+          <t>Global Schedule Reliability for May 2026 the Highest of the Year</t>
+        </is>
+      </c>
+      <c r="E705" s="4" t="inlineStr">
+        <is>
+          <t>2026년 5월 글로벌 정기선 스케줄 신뢰도가 올해 최고치를 기록하며, 해상 운송의 정시성이 개선되고 있음을 나타낸다.</t>
+        </is>
+      </c>
+      <c r="F705" s="4" t="inlineStr">
+        <is>
+          <t>스케줄 신뢰도 개선은 긍정적인 신호이나, 일회성 데이터일 수 있으며, 여전히 변동성이 존재하므로 당장 높은 영향으로 보기는 어렵다. 지속적인 추이 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G705" s="4" t="n"/>
+      <c r="H705" s="4" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I705" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/395-global-schedule-reliability-for-may-2026-the-highest-of-the-year</t>
+        </is>
+      </c>
+      <c r="J705" s="4" t="inlineStr"/>
+    </row>
+    <row r="706">
+      <c r="A706" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B706" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C706" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D706" s="4" t="inlineStr">
+        <is>
+          <t>20260712 경제·물류 주요뉴스 (데일리스크랩)</t>
+        </is>
+      </c>
+      <c r="E706" s="4" t="inlineStr">
+        <is>
+          <t>일본 JAPEX가 미국 내 석유·가스 생산을 확대하여 아시아 운송을 추진하며, 물류 현장에 휴머노이드 로봇 도입이 확산되는 등 물류 자동화 기술 동향이 나타나고 있다.</t>
+        </is>
+      </c>
+      <c r="F706" s="4" t="inlineStr">
+        <is>
+          <t>JAPEX의 석유·가스 생산 확대는 장기적인 에너지 공급망 안정화에 기여할 수 있으나 단기 유가나 물류비에 직접 영향은 미미하며, 로봇 도입은 물류 기술 동향으로 당장 우리 운영에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G706" s="4" t="n"/>
+      <c r="H706" s="4" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I706" s="4" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260712-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J706" s="4" t="inlineStr"/>
+    </row>
+    <row r="707">
+      <c r="A707" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B707" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C707" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D707" s="4" t="inlineStr">
+        <is>
+          <t>20260709 경제·물류 주요뉴스 (데일리스크랩)</t>
+        </is>
+      </c>
+      <c r="E707" s="4" t="inlineStr">
+        <is>
+          <t>부산진해경자청이 부산항과 가덕도신공항을 연계한 동북아 콜드체인 물류허브 구축 전략을 추진하며, 대우건설은 중동~유럽 해상·육상 물류 전환을 통해 운송 기간 단축 및 공급망 리스크를 완화했다.</t>
+        </is>
+      </c>
+      <c r="F707" s="4" t="inlineStr">
+        <is>
+          <t>지역 물류 인프라 강화 및 타사 공급망 전략 사례로, 당장 우리 기업의 물류 운영에 직접적인 영향은 없으며 참고할 만한 수준이다.</t>
+        </is>
+      </c>
+      <c r="G707" s="4" t="n"/>
+      <c r="H707" s="4" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I707" s="4" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260709-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J707" s="4" t="inlineStr"/>
+    </row>
+    <row r="708">
+      <c r="A708" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B708" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C708" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D708" s="4" t="inlineStr">
+        <is>
+          <t>이베코코리아 / 연비·안전·주행 편의성 향상 대형 트랙터 ‘올 뉴 S-Way’ 출시</t>
+        </is>
+      </c>
+      <c r="E708" s="4" t="inlineStr">
+        <is>
+          <t>이베코코리아가 연비, 안전, 주행 편의성을 향상시킨 대형 트랙터 ‘올 뉴 S-Way’를 국내 시장에 출시하여 육상 운송 효율성 개선에 기여할 것으로 보인다.</t>
+        </is>
+      </c>
+      <c r="F708" s="4" t="inlineStr">
+        <is>
+          <t>운송 장비 기술 발전 동향으로, 장기적으로는 운송 서비스 품질에 영향을 줄 수 있으나 당장 우리 기업의 물류 운영에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G708" s="4" t="n"/>
+      <c r="H708" s="4" t="inlineStr">
+        <is>
+          <t>ulogistics</t>
+        </is>
+      </c>
+      <c r="I708" s="4" t="inlineStr">
+        <is>
+          <t>http://www.ulogistics.co.kr/test/board.php?board=all2&amp;command=body&amp;no=5212</t>
+        </is>
+      </c>
+      <c r="J708" s="4" t="inlineStr"/>
+    </row>
+    <row r="709">
+      <c r="A709" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B709" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C709" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D709" s="4" t="inlineStr">
+        <is>
+          <t>'바다의 테슬라'… HMM, 전 선단에 AI 자율운항 도입-경제ㅣ한국일보</t>
+        </is>
+      </c>
+      <c r="E709" s="4" t="inlineStr">
+        <is>
+          <t>HMM이 전 선박에 AI 기반 자율운항 시스템을 도입하여 운항 안전성과 효율을 높이고, 친환경 선박 기술로 탄소 절감 목표 달성을 추진한다.</t>
+        </is>
+      </c>
+      <c r="F709" s="4" t="inlineStr">
+        <is>
+          <t>주요 선사의 기술 도입 동향으로, 장기적으로 해상 운송 서비스 품질에 영향을 줄 수 있으나 당장 우리 기업의 물류 운영에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G709" s="4" t="n"/>
+      <c r="H709" s="4" t="inlineStr">
+        <is>
+          <t>한국일보</t>
+        </is>
+      </c>
+      <c r="I709" s="4" t="inlineStr">
+        <is>
+          <t>https://hankookilbo.com/news/article/A2026070911050004516</t>
+        </is>
+      </c>
+      <c r="J709" s="4" t="inlineStr"/>
+    </row>
+    <row r="710">
+      <c r="A710" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B710" s="4" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C710" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D710" s="4" t="inlineStr">
+        <is>
+          <t>돈바스 지역으로 불법 휘발?? 를 운반하던 차량 운? ?자가 로스?? 프 지역에서 체포되었습니다</t>
+        </is>
+      </c>
+      <c r="E710" s="4" t="inlineStr">
+        <is>
+          <t>러시아 로스토프 지역에서 루간스크 인민공화국(LPR)과 도네츠크 인민공화국(DPR)으로 불법 연료를 운송하던 운전자가 체포되었습니다.</t>
+        </is>
+      </c>
+      <c r="F710" s="4" t="inlineStr">
+        <is>
+          <t>개인의 불법 연료 운송 적발 사례로, 기업의 합법적인 물류 운영이나 위험물 규제에 직접적인 영향을 미치지 않습니다.</t>
+        </is>
+      </c>
+      <c r="G710" s="4" t="n"/>
+      <c r="H710" s="4" t="inlineStr">
+        <is>
+          <t>Pravda 한국</t>
+        </is>
+      </c>
+      <c r="I710" s="4" t="inlineStr">
+        <is>
+          <t>https://korea.news-pravda.com/dprk/2026/07/11/69403.html</t>
+        </is>
+      </c>
+      <c r="J710" s="4" t="inlineStr"/>
+    </row>
+    <row r="711">
+      <c r="A711" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B711" s="4" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C711" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D711" s="4" t="inlineStr">
+        <is>
+          <t>블랙록, 지정학적 10대 위험 요인 발표</t>
+        </is>
+      </c>
+      <c r="E711" s="4" t="inlineStr">
+        <is>
+          <t>블랙록이 10대 지정학적 위험 요인을 발표했으나, 구체적인 내용이 없어 우리 물류 운영에 미치는 즉각적인 영향은 파악하기 어렵습니다.</t>
+        </is>
+      </c>
+      <c r="F711" s="4" t="inlineStr">
+        <is>
+          <t>특정 위험 요인에 대한 구체적인 내용이 없어 당장 우리 물류 운영에 미치는 직접적인 영향은 낮지만, 전반적인 지정학적 리스크 인식을 위해 참고할 만합니다.</t>
+        </is>
+      </c>
+      <c r="G711" s="4" t="n"/>
+      <c r="H711" s="4" t="inlineStr">
+        <is>
+          <t>Investing.com</t>
+        </is>
+      </c>
+      <c r="I711" s="4" t="inlineStr">
+        <is>
+          <t>https://kr.investing.com/news/economy-news/article-2012470</t>
+        </is>
+      </c>
+      <c r="J711" s="4" t="inlineStr"/>
+    </row>
+    <row r="712">
+      <c r="A712" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B712" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C712" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D712" s="4" t="inlineStr">
+        <is>
+          <t>제주공항 결항 105편·지연 85편… 휴가철 주말 하늘길 멈췄다</t>
+        </is>
+      </c>
+      <c r="E712" s="4" t="inlineStr">
+        <is>
+          <t>태풍 '바비'의 영향으로 제주국제공항 항공편 100편 이상이 결항 및 지연되어 휴가철 여행객들의 이동에 차질이 발생했습니다.</t>
+        </is>
+      </c>
+      <c r="F712" s="4" t="inlineStr">
+        <is>
+          <t>태풍으로 인한 제주공항 결항은 국내 특정 지역의 항공 운송 지연 사례로, 우리 기업의 주요 국제 물류 운영에 직접적인 영향은 낮지만, 기상 악화 시 운송 리스크를 상기시킵니다.</t>
+        </is>
+      </c>
+      <c r="G712" s="4" t="n"/>
+      <c r="H712" s="4" t="inlineStr">
+        <is>
+          <t>파이낸셜뉴스</t>
+        </is>
+      </c>
+      <c r="I712" s="4" t="inlineStr">
+        <is>
+          <t>https://fnnews.com/news/202607121548077480</t>
+        </is>
+      </c>
+      <c r="J712" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -32986,7 +34134,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -33635,6 +34783,49 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>3184.82</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>-142 (-4.3%)</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>+1,323 (+71.1%)</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>4330</v>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>+410 (+10.5%)</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>+1,619 (+59.7%)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -33647,7 +34838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I121"/>
+  <dimension ref="A1:I123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -37908,6 +39099,76 @@
       </c>
       <c r="I121" s="6" t="inlineStr"/>
     </row>
+    <row r="122">
+      <c r="A122" s="6" t="inlineStr">
+        <is>
+          <t>RSK-121</t>
+        </is>
+      </c>
+      <c r="B122" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="C122" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D122" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E122" s="6" t="inlineStr">
+        <is>
+          <t>20260713 경제·물류 주요뉴스 (데일리스크랩)</t>
+        </is>
+      </c>
+      <c r="F122" s="6" t="inlineStr"/>
+      <c r="G122" s="6" t="inlineStr"/>
+      <c r="H122" s="6" t="inlineStr">
+        <is>
+          <t>중동 항로 이용 시 대체 항로 및 운송 수단 검토, 선사와의 비상 계획 수립 논의, 유가 변동 추이 모니터링 및 운임 계약 조건 재검토.</t>
+        </is>
+      </c>
+      <c r="I122" s="6" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="6" t="inlineStr">
+        <is>
+          <t>RSK-122</t>
+        </is>
+      </c>
+      <c r="B123" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="C123" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D123" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E123" s="6" t="inlineStr">
+        <is>
+          <t>이란 "호르무즈 해협 봉쇄하겠다"</t>
+        </is>
+      </c>
+      <c r="F123" s="6" t="inlineStr"/>
+      <c r="G123" s="6" t="inlineStr"/>
+      <c r="H123" s="6" t="inlineStr">
+        <is>
+          <t>대체 운송 경로 및 운송사 옵션 검토, 유가 변동에 따른 물류비 상승 시나리오 분석, 재고 수준 및 리드타임 영향 평가.</t>
+        </is>
+      </c>
+      <c r="I123" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
📰 뉴스 데이터 2026-07-14_08:54
</commit_message>
<xml_diff>
--- a/data/SCM_물류_브리핑.xlsx
+++ b/data/SCM_물류_브리핑.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J712"/>
+  <dimension ref="A1:J746"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -34122,6 +34122,1638 @@
       </c>
       <c r="J712" s="4" t="inlineStr"/>
     </row>
+    <row r="713">
+      <c r="A713" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B713" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C713" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D713" s="2" t="inlineStr">
+        <is>
+          <t>美, 중국 항만 파나마 선박 억류 증가에 대해 경고</t>
+        </is>
+      </c>
+      <c r="E713" s="2" t="inlineStr">
+        <is>
+          <t>미국 연방해사위원회(FMC)가 중국 항만 내 파나마 선적 선박에 대한 보복성 억류 조치를 공급망 위협으로 규정하고 중국 선사에 대한 시정 조치를 경고했다.</t>
+        </is>
+      </c>
+      <c r="F713" s="2" t="inlineStr">
+        <is>
+          <t>주요 무역국인 미국과 중국 간의 해운 관련 지정학적 갈등 심화는 우리 회사의 중국 발/착 해상 운송에 직접적인 지연 및 비용 증가 위험을 초래할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G713" s="2" t="inlineStr">
+        <is>
+          <t>중국 항만 이용 시 선박 억류 가능성 및 운송 지연 위험을 면밀히 모니터링하고, 비상 운송 계획 수립을 검토한다.</t>
+        </is>
+      </c>
+      <c r="H713" s="2" t="inlineStr">
+        <is>
+          <t>kita</t>
+        </is>
+      </c>
+      <c r="I713" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kita.net/shippers/board/newsView.do?morgueCode=2&amp;dataCls=B&amp;dataSeq=8162</t>
+        </is>
+      </c>
+      <c r="J713" s="2" t="inlineStr">
+        <is>
+          <t>RSK-123</t>
+        </is>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B714" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C714" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D714" s="2" t="inlineStr">
+        <is>
+          <t>미·이란 전면전 위기…국제유가 9%↑, 한달만에 최고치</t>
+        </is>
+      </c>
+      <c r="E714" s="2" t="inlineStr">
+        <is>
+          <t>미-이란 간 전면전 위기 고조로 호르무즈 해협 인근의 공급 차질 우려가 커지면서 국제유가가 한 달 만에 최고치로 9% 급등했으며, 오만은 해협의 남북 2개 항로 분리 관리 방안을 제안했습니다.</t>
+        </is>
+      </c>
+      <c r="F714" s="2" t="inlineStr">
+        <is>
+          <t>국제유가 급등은 해상 및 항공 운임에 직접적인 영향을 미쳐 물류비용을 증가시키며, 호르무즈 해협의 불안정은 주요 운송로의 차질을 야기할 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G714" s="2" t="inlineStr">
+        <is>
+          <t>유가 변동성 모니터링 강화, 비상 운송 계획(대체 항로, 운송 수단) 검토, 물류비 상승에 대비한 예산 확보.</t>
+        </is>
+      </c>
+      <c r="H714" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I714" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260714-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J714" s="2" t="inlineStr">
+        <is>
+          <t>RSK-124</t>
+        </is>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B715" s="2" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C715" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D715" s="2" t="inlineStr">
+        <is>
+          <t>BUSINESSES CONTINUE BUILDING BUFFER STOCKS IN ANTICIPATION OF FURTHER DISRUPTION AS SUPPLY SHORTAGES PERSIST: GEP GLOBAL SUPPLY CHAIN VOLATILITY INDEX</t>
+        </is>
+      </c>
+      <c r="E715" s="2" t="inlineStr">
+        <is>
+          <t>공급 부족이 지속되고 추가적인 공급망 혼란이 예상됨에 따라 기업들이 완충 재고를 계속 구축하고 있으며, 공급망 병목 현상이 최소 3분기까지 이어질 것으로 전망됩니다.</t>
+        </is>
+      </c>
+      <c r="F715" s="2" t="inlineStr">
+        <is>
+          <t>공급망 병목 현상 지속은 원자재 및 부품 수급에 차질을 줄 수 있으며, 운송 지연 및 비용 상승으로 이어져 생산 계획에 직접적인 영향을 미칩니다.</t>
+        </is>
+      </c>
+      <c r="G715" s="2" t="inlineStr">
+        <is>
+          <t>재고 수준 재검토 및 적정 재고 확보, 공급망 다변화 전략 강화, 운송 파트너와 긴밀한 협력으로 운송 스케줄 사전 확보.</t>
+        </is>
+      </c>
+      <c r="H715" s="2" t="inlineStr">
+        <is>
+          <t>The Manila Times</t>
+        </is>
+      </c>
+      <c r="I715" s="2" t="inlineStr">
+        <is>
+          <t>https://manilatimes.net/2026/07/13/tmt-newswire/pr-newswire/businesses-continue-building-buffer-stocks-in-anticipation-of-further-disruption-as-supply-shortages-persist-gep-global-supply-chain-volatility-index/2383367</t>
+        </is>
+      </c>
+      <c r="J715" s="2" t="inlineStr">
+        <is>
+          <t>RSK-125</t>
+        </is>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B716" s="2" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C716" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D716" s="2" t="inlineStr">
+        <is>
+          <t>Key European shipping corridor hit by river and rail freight ‘double whammy’</t>
+        </is>
+      </c>
+      <c r="E716" s="2" t="inlineStr">
+        <is>
+          <t>독일 라인강의 수위 급락으로 바지선 운송 역량 부족이 심화되어 유럽의 주요 운송 회랑에서 심각한 공급망 혼란이 발생할 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="F716" s="2" t="inlineStr">
+        <is>
+          <t>라인강 운송 차질은 유럽 내륙 운송에 의존하는 원자재 및 완제품의 이동에 직접적인 영향을 미쳐 생산 및 배송 계획에 지연을 발생시킬 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G716" s="2" t="inlineStr">
+        <is>
+          <t>유럽향/유럽발 물량의 운송 경로 및 모드 재검토, 대체 운송 수단(철도, 도로) 활용 가능성 타진, 운송 파트너와 긴밀한 소통으로 상황 모니터링.</t>
+        </is>
+      </c>
+      <c r="H716" s="2" t="inlineStr">
+        <is>
+          <t>AJOT.COM</t>
+        </is>
+      </c>
+      <c r="I716" s="2" t="inlineStr">
+        <is>
+          <t>https://ajot.com/insights/full/ai-key-european-shipping-corridor-hit-by-river-and-rail-freight-double-whammy</t>
+        </is>
+      </c>
+      <c r="J716" s="2" t="inlineStr">
+        <is>
+          <t>RSK-126</t>
+        </is>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B717" s="2" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C717" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D717" s="2" t="inlineStr">
+        <is>
+          <t>배터리 갈아끼우는 애플펜슬 나오나…EU 규제 대응[모닝폰]</t>
+        </is>
+      </c>
+      <c r="E717" s="2" t="inlineStr">
+        <is>
+          <t>애플이 내년부터 적용되는 유럽연합(EU)의 사용자 교체 가능 배터리 규제에 대응하여 차세대 애플펜슬에 배터리 교체 기능을 도입할 가능성이 제기되었습니다. 이는 배터리 제품 설계 및 생산 방식에 직접적인 영향을 미칩니다.</t>
+        </is>
+      </c>
+      <c r="F717" s="2" t="inlineStr">
+        <is>
+          <t>EU의 사용자 교체 가능 배터리 규제는 우리 회사의 배터리 제품 설계 및 생산, 그리고 향후 역물류(수리/교체) 프로세스에 직접적인 영향을 미치므로 즉각적인 대응이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G717" s="2" t="inlineStr">
+        <is>
+          <t>EU 배터리 규제 상세 내용을 파악하고, 해당 규제에 부합하는 제품 설계 및 생산 공정 변경 가능성을 검토하며, 관련 물류 프로세스(예: 교체용 배터리 유통, 폐배터리 회수)에 대한 계획 수립</t>
+        </is>
+      </c>
+      <c r="H717" s="2" t="inlineStr">
+        <is>
+          <t>이데일리</t>
+        </is>
+      </c>
+      <c r="I717" s="2" t="inlineStr">
+        <is>
+          <t>https://edaily.co.kr/News/Read?mediaCodeNo=257&amp;newsId=01905686645514192</t>
+        </is>
+      </c>
+      <c r="J717" s="2" t="inlineStr">
+        <is>
+          <t>RSK-127</t>
+        </is>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B718" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C718" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D718" s="2" t="inlineStr">
+        <is>
+          <t>중, 호르무즈 재봉쇄 직전 헬륨 수출 금지···‘자국 우선’ 수출 통제</t>
+        </is>
+      </c>
+      <c r="E718" s="2" t="inlineStr">
+        <is>
+          <t>중국이 이란과 미국의 분쟁 재개로 호르무즈 해협이 재봉쇄되기 직전 헬륨 수출을 일시적으로 금지하며 자국 산업 보호를 위한 수출 통제 조치를 시행했습니다. 이는 지정학적 리스크가 원자재 공급망에 미치는 직접적인 영향을 보여줍니다.</t>
+        </is>
+      </c>
+      <c r="F718" s="2" t="inlineStr">
+        <is>
+          <t>특정 원자재에 대한 국가의 수출 통제는 배터리/전자부품 제조에 필요한 핵심 광물 및 부품의 공급망 안정성에 심각한 위협이 될 수 있으므로 즉각적인 공급망 리스크 분석이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G718" s="2" t="inlineStr">
+        <is>
+          <t>핵심 원자재 및 부품의 공급망 리스크를 재평가하고, 특정 국가 의존도를 낮추기 위한 공급처 다변화 전략을 적극적으로 모색하며, 비상 재고 확보 방안 검토</t>
+        </is>
+      </c>
+      <c r="H718" s="2" t="inlineStr">
+        <is>
+          <t>경향신문</t>
+        </is>
+      </c>
+      <c r="I718" s="2" t="inlineStr">
+        <is>
+          <t>https://khan.co.kr/article/202607121536001</t>
+        </is>
+      </c>
+      <c r="J718" s="2" t="inlineStr">
+        <is>
+          <t>RSK-128</t>
+        </is>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B719" s="2" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C719" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D719" s="2" t="inlineStr">
+        <is>
+          <t>보일하이츠 리니지 물류창고 화재 수습 지연…파리 떼 극성과 악취로 주민 고통 심화</t>
+        </is>
+      </c>
+      <c r="E719" s="2" t="inlineStr">
+        <is>
+          <t>보일하이츠 리니지 로지스틱스 물류창고 화재 수습이 한 달 가까이 지연되며 악취와 파리 떼로 주민 고통이 심화되고 있습니다. 이는 물류창고의 안전 관리 및 화재 대응 능력의 중요성을 강조합니다.</t>
+        </is>
+      </c>
+      <c r="F719" s="2" t="inlineStr">
+        <is>
+          <t>대형 물류창고 화재는 우리 회사의 보관 중인 제품 손실, 물류 운영 중단, 그리고 향후 창고 안전 규제 강화로 이어질 수 있으므로 즉각적인 내부 점검 및 대비가 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G719" s="2" t="inlineStr">
+        <is>
+          <t>현재 사용 중인 물류창고의 화재 안전 시스템 및 비상 대응 계획을 즉시 점검하고, 위험물 보관 규정 준수 여부를 재확인하며, 비상시 대체 보관 및 운송 계획 수립</t>
+        </is>
+      </c>
+      <c r="H719" s="2" t="inlineStr">
+        <is>
+          <t>Radio Seoul</t>
+        </is>
+      </c>
+      <c r="I719" s="2" t="inlineStr">
+        <is>
+          <t>https://radioseoul1650.com/archives/146958</t>
+        </is>
+      </c>
+      <c r="J719" s="2" t="inlineStr">
+        <is>
+          <t>RSK-129</t>
+        </is>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B720" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C720" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D720" s="2" t="inlineStr">
+        <is>
+          <t>이란 "호르무즈 해협 봉쇄하겠다"</t>
+        </is>
+      </c>
+      <c r="E720" s="2" t="inlineStr">
+        <is>
+          <t>이란이 호르무즈 해협 봉쇄를 위협하며, 이는 국제유가 급등 및 글로벌 에너지 공급망과 물류에 심각한 파급 효과를 초래할 수 있다.</t>
+        </is>
+      </c>
+      <c r="F720" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협은 주요 에너지 수송로이자 글로벌 해상 운송의 핵심 길목으로, 봉쇄 시 유가 및 해상 운임 폭등, 운송 지연 등 우리 물류 운영에 치명적인 영향을 미친다.</t>
+        </is>
+      </c>
+      <c r="G720" s="2" t="inlineStr">
+        <is>
+          <t>중동발 원자재 및 부품의 재고 수준을 즉시 점검하고, 대체 운송 경로 및 운송 수단 확보 방안을 긴급 검토하며, 유가 및 운임 변동에 대한 헤징 전략을 수립.</t>
+        </is>
+      </c>
+      <c r="H720" s="2" t="inlineStr">
+        <is>
+          <t>매일경제</t>
+        </is>
+      </c>
+      <c r="I720" s="2" t="inlineStr">
+        <is>
+          <t>https://mk.co.kr/news/world/12096599</t>
+        </is>
+      </c>
+      <c r="J720" s="2" t="inlineStr">
+        <is>
+          <t>RSK-130</t>
+        </is>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B721" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C721" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D721" s="2" t="inlineStr">
+        <is>
+          <t>다시 막힌 호르무즈 해협…국내 원유 수급 문제 없나</t>
+        </is>
+      </c>
+      <c r="E721" s="2" t="inlineStr">
+        <is>
+          <t>미국과 이란의 무력 충돌 격화로 호르무즈 해협 봉쇄 가능성이 다시 제기되며, 중동발 원유 공급망 리스크가 고조되어 국내 원유 수급 및 유가에 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="F721" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 봉쇄는 유가 급등을 야기하여 항공/해상/육상 운송 비용을 직접적으로 상승시키고, 물류 운영 전반에 심각한 영향을 미친다.</t>
+        </is>
+      </c>
+      <c r="G721" s="2" t="inlineStr">
+        <is>
+          <t>유가 변동에 따른 물류비 상승 시나리오를 수립하고, 운송 계약의 유류할증료 조항을 검토하며, 대체 에너지원 또는 운송 수단 활용 가능성을 모색.</t>
+        </is>
+      </c>
+      <c r="H721" s="2" t="inlineStr">
+        <is>
+          <t>연합뉴스</t>
+        </is>
+      </c>
+      <c r="I721" s="2" t="inlineStr">
+        <is>
+          <t>https://yna.co.kr/view/AKR20260713060200003</t>
+        </is>
+      </c>
+      <c r="J721" s="2" t="inlineStr">
+        <is>
+          <t>RSK-131</t>
+        </is>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B722" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C722" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D722" s="3" t="inlineStr">
+        <is>
+          <t>U.S.-EU Trade Agreement Eliminates Duties on Most U.S. Goods Starting July 1; TPEB Rates Rise as July Capacity Hits Three-Year High</t>
+        </is>
+      </c>
+      <c r="E722" s="3" t="inlineStr">
+        <is>
+          <t>미국-EU 무역 협정으로 7월 1일부터 대부분의 미국 상품에 대한 관세가 철폐되었으며, 동시에 태평양 횡단 동향(TPEB) 해상 운임이 상승하고 7월 선복량이 3년 내 최고치를 기록했다.</t>
+        </is>
+      </c>
+      <c r="F722" s="3" t="inlineStr">
+        <is>
+          <t>미국-EU 관세 철폐는 긍정적이나 TPEB 운임 상승 및 선복량 증가는 향후 운송 비용 및 가용성에 영향을 미칠 수 있어 추이를 지켜봐야 한다.</t>
+        </is>
+      </c>
+      <c r="G722" s="3" t="inlineStr">
+        <is>
+          <t>TPEB 노선 이용 시 운임 변동 추이 및 선복량 상황을 지속 모니터링하고, 관세 철폐의 우리 회사 제품 수출입 영향 여부를 확인한다.</t>
+        </is>
+      </c>
+      <c r="H722" s="3" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I722" s="3" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/july-02-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J722" s="3" t="inlineStr"/>
+    </row>
+    <row r="723">
+      <c r="A723" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B723" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C723" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D723" s="3" t="inlineStr">
+        <is>
+          <t>Structural Contraction of Global Liner Networks</t>
+        </is>
+      </c>
+      <c r="E723" s="3" t="inlineStr">
+        <is>
+          <t>2012년 이후 글로벌 정기선 네트워크 데이터 분석 결과, 선사들이 지리적 범위는 유지하면서도 서비스 빈도를 줄이는 등 네트워크 관리 방식에 근본적인 변화가 있음을 보여준다.</t>
+        </is>
+      </c>
+      <c r="F723" s="3" t="inlineStr">
+        <is>
+          <t>선사들의 서비스 빈도 감소는 장기적으로 특정 노선의 선복량 감소 및 운송 시간 증가로 이어질 수 있어, 향후 운송 계획에 잠재적 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G723" s="3" t="inlineStr">
+        <is>
+          <t>주요 운송 노선의 선사 서비스 빈도 및 네트워크 변화를 지속적으로 모니터링하여 잠재적 운송 지연 또는 비용 증가에 대비한다.</t>
+        </is>
+      </c>
+      <c r="H723" s="3" t="inlineStr">
+        <is>
+          <t>sea-intelligence</t>
+        </is>
+      </c>
+      <c r="I723" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/397-structural-contraction-of-global-liner-networks</t>
+        </is>
+      </c>
+      <c r="J723" s="3" t="inlineStr"/>
+    </row>
+    <row r="724">
+      <c r="A724" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B724" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C724" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D724" s="3" t="inlineStr">
+        <is>
+          <t>Transpacific: Ripe for new non-alliance services</t>
+        </is>
+      </c>
+      <c r="E724" s="3" t="inlineStr">
+        <is>
+          <t>아시아-북미 서안 항로에서 컨테이너 스팟 운임과 비동맹 선사 선복량 간의 관계를 분석하며, 새로운 비동맹 서비스의 출현 가능성을 시사합니다.</t>
+        </is>
+      </c>
+      <c r="F724" s="3" t="inlineStr">
+        <is>
+          <t>비동맹 선사 서비스 증가는 장기적으로 운송 옵션 확대 및 운임 안정화에 기여할 수 있으나, 즉각적인 영향은 미미합니다.</t>
+        </is>
+      </c>
+      <c r="G724" s="3" t="n"/>
+      <c r="H724" s="3" t="inlineStr">
+        <is>
+          <t>sea-intelligence</t>
+        </is>
+      </c>
+      <c r="I724" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/393-transpacific-ripe-for-new-non-alliance-services</t>
+        </is>
+      </c>
+      <c r="J724" s="3" t="inlineStr"/>
+    </row>
+    <row r="725">
+      <c r="A725" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B725" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C725" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D725" s="3" t="inlineStr">
+        <is>
+          <t>예상 밖 길어진 해운 호황···HMM 몸값 키우나</t>
+        </is>
+      </c>
+      <c r="E725" s="3" t="inlineStr">
+        <is>
+          <t>해상운임 강세가 예상보다 길어지면서 HMM의 기업가치에 대한 관심이 다시 쏠리고 있으며, 이는 컨테이너 운임 상승 추세가 지속되고 있음을 시사합니다.</t>
+        </is>
+      </c>
+      <c r="F725" s="3" t="inlineStr">
+        <is>
+          <t>컨테이너 운임 강세는 해상 운송 비용 증가로 직결되어 물류 예산에 영향을 미칠 수 있으므로 지속적인 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G725" s="3" t="inlineStr">
+        <is>
+          <t>해상 운임 지수 및 시장 동향 지속 모니터링, 운송 계약 조건 재검토 준비.</t>
+        </is>
+      </c>
+      <c r="H725" s="3" t="inlineStr">
+        <is>
+          <t>시사저널e</t>
+        </is>
+      </c>
+      <c r="I725" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sisajournal-e.com/news/articleView.html?idxno=422402</t>
+        </is>
+      </c>
+      <c r="J725" s="3" t="inlineStr"/>
+    </row>
+    <row r="726">
+      <c r="A726" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B726" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C726" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D726" s="3" t="inlineStr">
+        <is>
+          <t>해진공 "해운시장 예측보다 외부 충격 신속 대응이 중요해질 것"</t>
+        </is>
+      </c>
+      <c r="E726" s="3" t="inlineStr">
+        <is>
+          <t>한국해양진흥공사는 수에즈 운하 정상화 및 우회 선복 복귀 속도가 글로벌 컨테이너 시장의 핵심 변수라며, 해운시장 예측보다 외부 충격에 대한 신속한 대응이 중요하다고 진단했습니다.</t>
+        </is>
+      </c>
+      <c r="F726" s="3" t="inlineStr">
+        <is>
+          <t>수에즈 운하의 안정화는 긍정적이나, 해운 시장의 불확실성이 상존하므로 외부 충격에 대한 대응 전략을 지속적으로 검토해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G726" s="3" t="inlineStr">
+        <is>
+          <t>글로벌 해운 시장 동향 및 주요 운하 상황 지속 모니터링, 비상 운송 계획 정기적 검토.</t>
+        </is>
+      </c>
+      <c r="H726" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I726" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260710-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J726" s="3" t="inlineStr"/>
+    </row>
+    <row r="727">
+      <c r="A727" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B727" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C727" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D727" s="3" t="inlineStr">
+        <is>
+          <t>From Deluges to Dry Beds: How Extreme Weather is Rewriting Logistics Strategy</t>
+        </is>
+      </c>
+      <c r="E727" s="3" t="inlineStr">
+        <is>
+          <t>극심한 기상 이변이 더 이상 고립된 사건이 아닌 시스템적이고 복합적인 위험으로 작용하며 전 세계 물류 전략을 근본적으로 재편하고 있습니다. 이는 기후 변화가 공급망에 미치는 영향이 심화되고 있음을 시사합니다.</t>
+        </is>
+      </c>
+      <c r="F727" s="3" t="inlineStr">
+        <is>
+          <t>기후 변화로 인한 극심한 기상 이변이 전 세계 물류 시스템에 구조적인 지연 및 혼란을 야기할 수 있어 지속적인 모니터링과 대비책 마련이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G727" s="3" t="inlineStr">
+        <is>
+          <t>주요 운송 경로의 기상 예측 시스템 강화 및 비상 운송 계획 수립 검토</t>
+        </is>
+      </c>
+      <c r="H727" s="3" t="inlineStr">
+        <is>
+          <t>Logistics Viewpoints</t>
+        </is>
+      </c>
+      <c r="I727" s="3" t="inlineStr">
+        <is>
+          <t>https://logisticsviewpoints.com/2026/07/13/from-deluges-to-dry-beds-how-extreme-weather-is-rewriting-logistics-strategy</t>
+        </is>
+      </c>
+      <c r="J727" s="3" t="inlineStr"/>
+    </row>
+    <row r="728">
+      <c r="A728" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B728" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C728" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D728" s="3" t="inlineStr">
+        <is>
+          <t>미국, 한국산 탄소강·합금강 선재와 절단 강판(CTL), 대구경 용접관에 대한 반덤핑 관세(AD) 및 상계관세(CVD) 조사 실시</t>
+        </is>
+      </c>
+      <c r="E728" s="3" t="inlineStr">
+        <is>
+          <t>미국이 한국산 철강 제품에 대한 반덤핑 및 상계관세 조사를 실시하며, 한국의 산업용 전기요금과 탄소배출권을 정부 보조금으로 간주하고 있습니다. 이는 무역 분쟁의 확대를 시사하며, 다른 산업에도 유사한 조치가 적용될 가능성이 있습니다.</t>
+        </is>
+      </c>
+      <c r="F728" s="3" t="inlineStr">
+        <is>
+          <t>철강 제품에 대한 관세 조치이지만, 한국 정부의 보조금 정책에 대한 문제 제기는 향후 배터리/전자부품 산업에도 유사한 무역 규제가 적용될 수 있음을 시사합니다.</t>
+        </is>
+      </c>
+      <c r="G728" s="3" t="inlineStr">
+        <is>
+          <t>주요 수출국과의 무역 정책 동향을 면밀히 모니터링하고, 잠재적 관세 부과 시나리오에 대비한 공급망 다변화 전략을 검토</t>
+        </is>
+      </c>
+      <c r="H728" s="3" t="inlineStr">
+        <is>
+          <t>더구루(the guru)</t>
+        </is>
+      </c>
+      <c r="I728" s="3" t="inlineStr">
+        <is>
+          <t>https://theguru.co.kr/news/article.html?no=104299</t>
+        </is>
+      </c>
+      <c r="J728" s="3" t="inlineStr"/>
+    </row>
+    <row r="729">
+      <c r="A729" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B729" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C729" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D729" s="3" t="inlineStr">
+        <is>
+          <t>기후부, 미생물 활용해 폐배터리 속 리튬 90% 회수</t>
+        </is>
+      </c>
+      <c r="E729" s="3" t="inlineStr">
+        <is>
+          <t>기후에너지환경부 산하 국립낙동강생물자원관이 담수 미생물을 이용해 이차전지 폐기물에서 리튬을 90% 회수하는 기술을 개발했습니다. 이는 폐배터리 재활용 효율을 높여 원자재 수급 안정화와 환경 규제 대응에 기여할 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="F729" s="3" t="inlineStr">
+        <is>
+          <t>폐배터리 재활용 기술 발전은 장기적으로 원자재 수급 안정화 및 폐배터리 회수/처리 물류 전략에 영향을 미칠 수 있으므로 기술 상용화 추이를 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G729" s="3" t="inlineStr">
+        <is>
+          <t>폐배터리 회수 및 재활용 관련 기술 동향을 지속적으로 파악하고, 향후 관련 규제 변화 및 역물류 시스템 구축 가능성을 검토</t>
+        </is>
+      </c>
+      <c r="H729" s="3" t="inlineStr">
+        <is>
+          <t>아시아투데이</t>
+        </is>
+      </c>
+      <c r="I729" s="3" t="inlineStr">
+        <is>
+          <t>https://asiatoday.co.kr/kn/view.php?key=20260713010004556</t>
+        </is>
+      </c>
+      <c r="J729" s="3" t="inlineStr"/>
+    </row>
+    <row r="730">
+      <c r="A730" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B730" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C730" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D730" s="3" t="inlineStr">
+        <is>
+          <t>충남, 화학사고 예방부터 초동 대응까지 아우르는 지역 맞춤형 화학안전 정책 지속 추진</t>
+        </is>
+      </c>
+      <c r="E730" s="3" t="inlineStr">
+        <is>
+          <t>충남도가 화학사고 예방부터 초동 대응까지 아우르는 지역 맞춤형 화학안전 정책을 지속 추진하며 화학안전 관리체계를 강화합니다. 이는 화학물질 취급 및 보관에 대한 안전 규제 강화 추세를 반영합니다.</t>
+        </is>
+      </c>
+      <c r="F730" s="3" t="inlineStr">
+        <is>
+          <t>화학물질 안전 관리 강화는 배터리 제조 과정 및 위험물 운송/보관에 대한 규제 강화로 이어질 수 있으므로, 관련 법규 변화 및 지역별 정책 동향을 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G730" s="3" t="inlineStr">
+        <is>
+          <t>사업장이 위치한 지역 및 주요 운송 경로의 화학물질 안전 관리 규제 동향을 지속적으로 파악하고, 내부 안전 관리 절차 및 교육 강화</t>
+        </is>
+      </c>
+      <c r="H730" s="3" t="inlineStr">
+        <is>
+          <t>세계환경신문</t>
+        </is>
+      </c>
+      <c r="I730" s="3" t="inlineStr">
+        <is>
+          <t>https://e-newsp.com/news/article.html?no=89441</t>
+        </is>
+      </c>
+      <c r="J730" s="3" t="inlineStr"/>
+    </row>
+    <row r="731">
+      <c r="A731" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B731" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C731" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D731" s="3" t="inlineStr">
+        <is>
+          <t>[영상] 파주 전자제품 창고서 '화재'…건물 4개 동 번져 '대응 1단계'</t>
+        </is>
+      </c>
+      <c r="E731" s="3" t="inlineStr">
+        <is>
+          <t>파주 전자제품 창고에서 대형 화재가 발생하여 건물 4개 동이 불에 탔으며, 인명 피해는 없으나 전자제품 창고 화재는 배터리/전자부품 물류에 잠재적 위험을 시사한다.</t>
+        </is>
+      </c>
+      <c r="F731" s="3" t="inlineStr">
+        <is>
+          <t>전자제품 창고 화재는 배터리/전자부품 취급 창고의 안전 규제 강화 및 보험료 인상 가능성을 시사하며, 유사 사고 발생 시 우리 물류 운영에 직접적인 영향을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="G731" s="3" t="inlineStr">
+        <is>
+          <t>국내 전자제품 창고 화재 사례 분석 및 우리 창고의 화재 예방 시스템, 비상 대응 계획, 위험물(배터리) 보관 규정 준수 여부 점검.</t>
+        </is>
+      </c>
+      <c r="H731" s="3" t="inlineStr">
+        <is>
+          <t>뉴스1</t>
+        </is>
+      </c>
+      <c r="I731" s="3" t="inlineStr">
+        <is>
+          <t>https://www.news1.kr/local/gyeonggi/6226913</t>
+        </is>
+      </c>
+      <c r="J731" s="3" t="inlineStr"/>
+    </row>
+    <row r="732">
+      <c r="A732" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B732" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C732" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D732" s="3" t="inlineStr">
+        <is>
+          <t>“2027년 반도체 역사상 최악의 공급절벽…삼전 목표가 60만원” [오늘나온보고서]</t>
+        </is>
+      </c>
+      <c r="E732" s="3" t="inlineStr">
+        <is>
+          <t>2027년 반도체 공급절벽이 예상되며, 이는 AI 기술 확산과 맞물려 반도체 수요 증가 대비 공급 부족이 심화될 수 있음을 시사한다.</t>
+        </is>
+      </c>
+      <c r="F732" s="3" t="inlineStr">
+        <is>
+          <t>2027년 예상되는 반도체 공급 부족은 우리 제품 생산에 필요한 핵심 부품 수급에 장기적인 영향을 미쳐 생산 계획 및 원가에 중대한 리스크를 초래할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G732" s="3" t="inlineStr">
+        <is>
+          <t>장기적인 반도체 수급 전망을 면밀히 분석하고, 주요 반도체 부품의 재고 전략 및 다중 공급처 확보 방안을 검토.</t>
+        </is>
+      </c>
+      <c r="H732" s="3" t="inlineStr">
+        <is>
+          <t>매일경제</t>
+        </is>
+      </c>
+      <c r="I732" s="3" t="inlineStr">
+        <is>
+          <t>https://mk.co.kr/news/stock/12096709</t>
+        </is>
+      </c>
+      <c r="J732" s="3" t="inlineStr"/>
+    </row>
+    <row r="733">
+      <c r="A733" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B733" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C733" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D733" s="3" t="inlineStr">
+        <is>
+          <t>‘반도체 고점론’ 머쓱하게 만든 한은 “내년까지 공급 부족 지속”</t>
+        </is>
+      </c>
+      <c r="E733" s="3" t="inlineStr">
+        <is>
+          <t>한국은행은 AI 기술 확산으로 반도체 공급 부족이 내년까지 지속될 것으로 전망하며, 이는 공급망 불안정 및 기술 규제 강화와 같은 지정학적 리스크와 연관될 수 있다.</t>
+        </is>
+      </c>
+      <c r="F733" s="3" t="inlineStr">
+        <is>
+          <t>반도체 공급 부족 지속은 우리 제품 생산에 필요한 핵심 부품 조달에 어려움을 가중시키고, 생산 계획 및 원가에 영향을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="G733" s="3" t="inlineStr">
+        <is>
+          <t>주요 반도체 부품의 장기 수급 계획을 재검토하고, 공급망 다변화 및 재고 확보 전략을 강화.</t>
+        </is>
+      </c>
+      <c r="H733" s="3" t="inlineStr">
+        <is>
+          <t>매일경제</t>
+        </is>
+      </c>
+      <c r="I733" s="3" t="inlineStr">
+        <is>
+          <t>https://mk.co.kr/news/economy/12096743</t>
+        </is>
+      </c>
+      <c r="J733" s="3" t="inlineStr"/>
+    </row>
+    <row r="734">
+      <c r="A734" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B734" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C734" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D734" s="3" t="inlineStr">
+        <is>
+          <t>SCFI 11주 만에 하락 전환…글로벌 컨운임 상승세 '숨 고르기'</t>
+        </is>
+      </c>
+      <c r="E734" s="3" t="inlineStr">
+        <is>
+          <t>SCFI가 11주 만에 하락 전환하며 글로벌 컨테이너 운임 상승세가 주춤했으나, 미주, 유럽 등 전 항로에서 일제히 하락했고 홍해 우회 수요는 여전히 변수로 남아있다.</t>
+        </is>
+      </c>
+      <c r="F734" s="3" t="inlineStr">
+        <is>
+          <t>컨테이너 운임 하락은 물류비 절감에 긍정적이나, 홍해 사태 등 불안정한 요인이 상존하여 언제든 운임이 다시 상승할 수 있으므로 지속적인 관찰이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G734" s="3" t="inlineStr">
+        <is>
+          <t>해상 운임 변동 추이를 면밀히 주시하고, 장기 운송 계약 조건 및 단기 스팟 운임 시장 동향을 분석하여 최적의 운송 전략을 수립.</t>
+        </is>
+      </c>
+      <c r="H734" s="3" t="inlineStr">
+        <is>
+          <t>해사신문</t>
+        </is>
+      </c>
+      <c r="I734" s="3" t="inlineStr">
+        <is>
+          <t>https://haesanews.com/news/articleView.html?idxno=149253</t>
+        </is>
+      </c>
+      <c r="J734" s="3" t="inlineStr"/>
+    </row>
+    <row r="735">
+      <c r="A735" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B735" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C735" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D735" s="4" t="inlineStr">
+        <is>
+          <t>FRA, 亞 5.5% 증가…中東 15.7% 감소</t>
+        </is>
+      </c>
+      <c r="E735" s="4" t="inlineStr">
+        <is>
+          <t>프랑크푸르트 공항의 6월 항공화물 물동량이 아시아 노선 성장에 힘입어 전년 대비 2% 증가했으며, 상반기 전체적으로도 1% 증가했다.</t>
+        </is>
+      </c>
+      <c r="F735" s="4" t="inlineStr">
+        <is>
+          <t>특정 공항의 항공화물 물동량 증가는 전반적인 항공 화물 시장의 미미한 개선을 시사하지만, 우리 회사의 특정 운송 계획에 즉각적인 영향을 미치지는 않는다.</t>
+        </is>
+      </c>
+      <c r="G735" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H735" s="4" t="inlineStr">
+        <is>
+          <t>cargonews</t>
+        </is>
+      </c>
+      <c r="I735" s="4" t="inlineStr">
+        <is>
+          <t>https://www.cargonews.co.kr/news/articleView.html?idxno=60518</t>
+        </is>
+      </c>
+      <c r="J735" s="4" t="inlineStr"/>
+    </row>
+    <row r="736">
+      <c r="A736" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B736" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C736" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D736" s="4" t="inlineStr">
+        <is>
+          <t>Air Cargo Demand Up 6.0% in May</t>
+        </is>
+      </c>
+      <c r="E736" s="4" t="inlineStr">
+        <is>
+          <t>2026년 5월 전 세계 항공 화물 수요가 전년 동기 대비 6.0% 증가하여, 항공 화물 시장의 지속적인 회복세를 나타냈다.</t>
+        </is>
+      </c>
+      <c r="F736" s="4" t="inlineStr">
+        <is>
+          <t>전 세계 항공 화물 수요 증가는 시장의 긍정적인 신호이나, 특정 노선이나 운임에 대한 즉각적인 영향보다는 전반적인 시장 동향을 파악하는 참고 자료이다.</t>
+        </is>
+      </c>
+      <c r="G736" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H736" s="4" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I736" s="4" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-29-air-cargo-demand-up-may/</t>
+        </is>
+      </c>
+      <c r="J736" s="4" t="inlineStr"/>
+    </row>
+    <row r="737">
+      <c r="A737" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B737" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C737" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D737" s="4" t="inlineStr">
+        <is>
+          <t>HMM, 스페인-서아프리카항로 뱃고동…ONE과 제휴</t>
+        </is>
+      </c>
+      <c r="E737" s="4" t="inlineStr">
+        <is>
+          <t>HMM이 스페인 알헤시라스를 허브로 서아프리카 주요 항만을 연결하는 신규 컨테이너선 서비스 MA2를 개설했으며, 이는 허브 앤드 스포크 전략의 일환이다.</t>
+        </is>
+      </c>
+      <c r="F737" s="4" t="inlineStr">
+        <is>
+          <t>스페인-서아프리카 노선 신설은 해당 지역의 운송 옵션을 확대하지만, 우리 회사의 주요 운송 경로가 아닐 가능성이 높으므로 즉각적인 영향은 낮다.</t>
+        </is>
+      </c>
+      <c r="G737" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H737" s="4" t="inlineStr">
+        <is>
+          <t>ksg</t>
+        </is>
+      </c>
+      <c r="I737" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksg.co.kr/news/main_newsView.jsp?pNum=147571</t>
+        </is>
+      </c>
+      <c r="J737" s="4" t="inlineStr"/>
+    </row>
+    <row r="738">
+      <c r="A738" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B738" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C738" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D738" s="4" t="inlineStr">
+        <is>
+          <t>Global Schedule Reliability for May 2026 the Highest of the Year</t>
+        </is>
+      </c>
+      <c r="E738" s="4" t="inlineStr">
+        <is>
+          <t>2026년 5월 전 세계 해상 스케줄 정시성이 올해 최고치를 기록하며, 해상 운송의 안정성이 개선되고 있음을 나타냈다.</t>
+        </is>
+      </c>
+      <c r="F738" s="4" t="inlineStr">
+        <is>
+          <t>전반적인 해상 스케줄 정시성 개선은 긍정적인 신호이나, 특정 노선이나 항만의 상황은 다를 수 있으며, 우리 회사의 운송 계획에 즉각적인 큰 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G738" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H738" s="4" t="inlineStr">
+        <is>
+          <t>sea-intelligence</t>
+        </is>
+      </c>
+      <c r="I738" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/395-global-schedule-reliability-for-may-2026-the-highest-of-the-year</t>
+        </is>
+      </c>
+      <c r="J738" s="4" t="inlineStr"/>
+    </row>
+    <row r="739">
+      <c r="A739" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B739" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C739" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D739" s="4" t="inlineStr">
+        <is>
+          <t>항공화물운송 상장기업 브랜드 7월 빅데이터 분석결과...1위 현대글로비스, 2위 CJ대한통운, (주)한진</t>
+        </is>
+      </c>
+      <c r="E739" s="4" t="inlineStr">
+        <is>
+          <t>2026년 7월 항공화물운송 상장기업 브랜드 평판 분석 결과, 현대글로비스, CJ대한통운, (주)한진이 상위권을 차지했습니다.</t>
+        </is>
+      </c>
+      <c r="F739" s="4" t="inlineStr">
+        <is>
+          <t>기업의 브랜드 평판 순위는 물류 서비스 선택 시 참고 자료가 될 수 있으나, 당사의 물류 운영이나 생산 계획에 즉각적인 영향을 미치지 않습니다.</t>
+        </is>
+      </c>
+      <c r="G739" s="4" t="n"/>
+      <c r="H739" s="4" t="inlineStr">
+        <is>
+          <t>shippingnewsnet</t>
+        </is>
+      </c>
+      <c r="I739" s="4" t="inlineStr">
+        <is>
+          <t>https://www.shippingnewsnet.com/news/articleView.html?idxno=71162</t>
+        </is>
+      </c>
+      <c r="J739" s="4" t="inlineStr"/>
+    </row>
+    <row r="740">
+      <c r="A740" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B740" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C740" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D740" s="4" t="inlineStr">
+        <is>
+          <t>상하이, 런던 제치고 세계 2위 해운 중심지 등극… ‘물동량’ 넘어 ‘...</t>
+        </is>
+      </c>
+      <c r="E740" s="4" t="inlineStr">
+        <is>
+          <t>상하이가 컨테이너 물동량뿐만 아니라 금융, 법률, 조선 등 해운 관련 서비스 분야에서도 발전하며 세계 2위 해운 중심지로 부상했습니다.</t>
+        </is>
+      </c>
+      <c r="F740" s="4" t="inlineStr">
+        <is>
+          <t>특정 항만의 위상 변화는 장기적인 관점에서 물류 네트워크 전략 수립 시 참고할 수 있으나, 즉각적인 운영 영향은 없습니다.</t>
+        </is>
+      </c>
+      <c r="G740" s="4" t="n"/>
+      <c r="H740" s="4" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I740" s="4" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260714-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J740" s="4" t="inlineStr"/>
+    </row>
+    <row r="741">
+      <c r="A741" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B741" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C741" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D741" s="4" t="inlineStr">
+        <is>
+          <t>BPA, '제3회 친환경 북극항로 포럼' 성황리에 개최</t>
+        </is>
+      </c>
+      <c r="E741" s="4" t="inlineStr">
+        <is>
+          <t>부산항만공사가 친환경 북극항로 포럼을 개최하며 북극항로 활용 가능성과 관련 논의를 본격화했습니다.</t>
+        </is>
+      </c>
+      <c r="F741" s="4" t="inlineStr">
+        <is>
+          <t>북극항로는 아직 상용화 단계가 아니며, 우리 회사의 주요 운송 경로에 즉각적인 변화를 가져오지 않습니다.</t>
+        </is>
+      </c>
+      <c r="G741" s="4" t="n"/>
+      <c r="H741" s="4" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I741" s="4" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260710-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J741" s="4" t="inlineStr"/>
+    </row>
+    <row r="742">
+      <c r="A742" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B742" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C742" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D742" s="4" t="inlineStr">
+        <is>
+          <t>이베코코리아 / 연비·안전·주행 편의성 향상 대형 트랙터 ‘올 뉴 S-Way’ 출시</t>
+        </is>
+      </c>
+      <c r="E742" s="4" t="inlineStr">
+        <is>
+          <t>이베코코리아가 연비, 안전, 주행 편의성을 대폭 향상시킨 대형 트랙터 '올 뉴 S-Way'를 국내 시장에 출시했습니다.</t>
+        </is>
+      </c>
+      <c r="F742" s="4" t="inlineStr">
+        <is>
+          <t>주로 3PL을 이용하는 우리 회사의 경우, 운송 파트너사의 차량 교체에 따른 간접적인 영향만 있을 뿐 직접적인 운영 변화는 없습니다.</t>
+        </is>
+      </c>
+      <c r="G742" s="4" t="n"/>
+      <c r="H742" s="4" t="inlineStr">
+        <is>
+          <t>ulogistics</t>
+        </is>
+      </c>
+      <c r="I742" s="4" t="inlineStr">
+        <is>
+          <t>http://www.ulogistics.co.kr/test/board.php?board=all2&amp;command=body&amp;no=5212</t>
+        </is>
+      </c>
+      <c r="J742" s="4" t="inlineStr"/>
+    </row>
+    <row r="743">
+      <c r="A743" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B743" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C743" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D743" s="4" t="inlineStr">
+        <is>
+          <t>글로벌 은행 선박금융 3,006억달러로 6% 성장</t>
+        </is>
+      </c>
+      <c r="E743" s="4" t="inlineStr">
+        <is>
+          <t>글로벌 신조선 발주 확대와 선박 자산가치 상승에 힘입어 지난해 글로벌 은행권의 선박금융 규모가 3,006억 달러로 6% 성장했습니다.</t>
+        </is>
+      </c>
+      <c r="F743" s="4" t="inlineStr">
+        <is>
+          <t>선박금융은 해운 산업의 장기적인 투자 동향을 보여주지만, 우리 회사의 단기적인 물류 운영이나 비용에 직접적인 영향을 미치지 않습니다.</t>
+        </is>
+      </c>
+      <c r="G743" s="4" t="n"/>
+      <c r="H743" s="4" t="inlineStr">
+        <is>
+          <t>해양통신</t>
+        </is>
+      </c>
+      <c r="I743" s="4" t="inlineStr">
+        <is>
+          <t>https://oceanpress.co.kr/news/article.html?no=30583</t>
+        </is>
+      </c>
+      <c r="J743" s="4" t="inlineStr"/>
+    </row>
+    <row r="744">
+      <c r="A744" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B744" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C744" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D744" s="4" t="inlineStr">
+        <is>
+          <t>항만·독, 해상 인프라 뒷받침할 기반 설비로 부각</t>
+        </is>
+      </c>
+      <c r="E744" s="4" t="inlineStr">
+        <is>
+          <t>AI 인프라 확대로 인한 전력 수요 증가와 육상 부지 부족으로 항만 및 대형 도크 등 해상 기반 시설이 친환경 연료 공급 체계와 함께 새로운 대안으로 부상하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F744" s="4" t="inlineStr">
+        <is>
+          <t>항만 인프라 개발은 장기적인 관점에서 물류 네트워크 효율성을 높일 수 있지만, 즉각적인 운영 변화나 비용 영향은 없습니다.</t>
+        </is>
+      </c>
+      <c r="G744" s="4" t="n"/>
+      <c r="H744" s="4" t="inlineStr">
+        <is>
+          <t>매일일보</t>
+        </is>
+      </c>
+      <c r="I744" s="4" t="inlineStr">
+        <is>
+          <t>https://m-i.kr/news/articleView.html?idxno=1390376</t>
+        </is>
+      </c>
+      <c r="J744" s="4" t="inlineStr"/>
+    </row>
+    <row r="745">
+      <c r="A745" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B745" s="4" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C745" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D745" s="4" t="inlineStr">
+        <is>
+          <t>中하이난, 2030년부터 내연기관차 판매 금지 정책 재확인</t>
+        </is>
+      </c>
+      <c r="E745" s="4" t="inlineStr">
+        <is>
+          <t>중국 하이난성이 2030년부터 휘발유·경유 등 내연기관 자동차 판매를 전면 금지하는 정책을 재확인했습니다. 이는 전기차 전환 가속화를 의미하며, 장기적으로 배터리 수요 증가에 영향을 미칠 것입니다.</t>
+        </is>
+      </c>
+      <c r="F745" s="4" t="inlineStr">
+        <is>
+          <t>2030년 시행되는 정책으로 당장 물류 운영에 직접적인 영향은 없으나, 장기적인 배터리 수요 증가 추세를 시사합니다.</t>
+        </is>
+      </c>
+      <c r="G745" s="4" t="n"/>
+      <c r="H745" s="4" t="inlineStr">
+        <is>
+          <t>연합뉴스</t>
+        </is>
+      </c>
+      <c r="I745" s="4" t="inlineStr">
+        <is>
+          <t>https://yna.co.kr/view/AKR20260713144900083</t>
+        </is>
+      </c>
+      <c r="J745" s="4" t="inlineStr"/>
+    </row>
+    <row r="746">
+      <c r="A746" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B746" s="4" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C746" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D746" s="4" t="inlineStr">
+        <is>
+          <t>[속보] 7월 초 수출, 또 최대치 경신…반도체 3배로 늘었다</t>
+        </is>
+      </c>
+      <c r="E746" s="4" t="inlineStr">
+        <is>
+          <t>7월 초 한국 수출액이 반도체 호황에 힘입어 53.9% 증가하며 역대 최대치를 경신, 반도체 산업의 강한 수요를 보여준다.</t>
+        </is>
+      </c>
+      <c r="F746" s="4" t="inlineStr">
+        <is>
+          <t>반도체 수출 호조는 산업 전반의 긍정적 신호이나, 우리 회사의 특정 물류 운영에 즉각적인 영향을 주기보다는 시장 상황 참고 자료로 활용된다.</t>
+        </is>
+      </c>
+      <c r="G746" s="4" t="n"/>
+      <c r="H746" s="4" t="inlineStr">
+        <is>
+          <t>디지털타임스</t>
+        </is>
+      </c>
+      <c r="I746" s="4" t="inlineStr">
+        <is>
+          <t>https://dt.co.kr/article/12072521</t>
+        </is>
+      </c>
+      <c r="J746" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -34134,7 +35766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -34826,6 +36458,49 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>3184.82</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>-142 (-4.3%)</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>+1,323 (+71.1%)</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>4318</v>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>-12 (-0.3%)</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>+1,728 (+66.7%)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -34838,7 +36513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I123"/>
+  <dimension ref="A1:I132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -39169,6 +40844,321 @@
       </c>
       <c r="I123" s="6" t="inlineStr"/>
     </row>
+    <row r="124">
+      <c r="A124" s="6" t="inlineStr">
+        <is>
+          <t>RSK-123</t>
+        </is>
+      </c>
+      <c r="B124" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C124" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D124" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E124" s="6" t="inlineStr">
+        <is>
+          <t>美, 중국 항만 파나마 선박 억류 증가에 대해 경고</t>
+        </is>
+      </c>
+      <c r="F124" s="6" t="inlineStr"/>
+      <c r="G124" s="6" t="inlineStr"/>
+      <c r="H124" s="6" t="inlineStr">
+        <is>
+          <t>중국 항만 이용 시 선박 억류 가능성 및 운송 지연 위험을 면밀히 모니터링하고, 비상 운송 계획 수립을 검토한다.</t>
+        </is>
+      </c>
+      <c r="I124" s="6" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="6" t="inlineStr">
+        <is>
+          <t>RSK-124</t>
+        </is>
+      </c>
+      <c r="B125" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C125" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D125" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E125" s="6" t="inlineStr">
+        <is>
+          <t>미·이란 전면전 위기…국제유가 9%↑, 한달만에 최고치</t>
+        </is>
+      </c>
+      <c r="F125" s="6" t="inlineStr"/>
+      <c r="G125" s="6" t="inlineStr"/>
+      <c r="H125" s="6" t="inlineStr">
+        <is>
+          <t>유가 변동성 모니터링 강화, 비상 운송 계획(대체 항로, 운송 수단) 검토, 물류비 상승에 대비한 예산 확보.</t>
+        </is>
+      </c>
+      <c r="I125" s="6" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="6" t="inlineStr">
+        <is>
+          <t>RSK-125</t>
+        </is>
+      </c>
+      <c r="B126" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C126" s="6" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="D126" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E126" s="6" t="inlineStr">
+        <is>
+          <t>BUSINESSES CONTINUE BUILDING BUFFER STOCKS IN ANTICIPATION OF FURTHER DISRUPTION AS SUPPLY SHORTAGES PERSIST: GEP GLOBAL SUPPLY CHAIN VOLATILITY INDEX</t>
+        </is>
+      </c>
+      <c r="F126" s="6" t="inlineStr"/>
+      <c r="G126" s="6" t="inlineStr"/>
+      <c r="H126" s="6" t="inlineStr">
+        <is>
+          <t>재고 수준 재검토 및 적정 재고 확보, 공급망 다변화 전략 강화, 운송 파트너와 긴밀한 협력으로 운송 스케줄 사전 확보.</t>
+        </is>
+      </c>
+      <c r="I126" s="6" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="6" t="inlineStr">
+        <is>
+          <t>RSK-126</t>
+        </is>
+      </c>
+      <c r="B127" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C127" s="6" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="D127" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E127" s="6" t="inlineStr">
+        <is>
+          <t>Key European shipping corridor hit by river and rail freight ‘double whammy’</t>
+        </is>
+      </c>
+      <c r="F127" s="6" t="inlineStr"/>
+      <c r="G127" s="6" t="inlineStr"/>
+      <c r="H127" s="6" t="inlineStr">
+        <is>
+          <t>유럽향/유럽발 물량의 운송 경로 및 모드 재검토, 대체 운송 수단(철도, 도로) 활용 가능성 타진, 운송 파트너와 긴밀한 소통으로 상황 모니터링.</t>
+        </is>
+      </c>
+      <c r="I127" s="6" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="6" t="inlineStr">
+        <is>
+          <t>RSK-127</t>
+        </is>
+      </c>
+      <c r="B128" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C128" s="6" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="D128" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E128" s="6" t="inlineStr">
+        <is>
+          <t>배터리 갈아끼우는 애플펜슬 나오나…EU 규제 대응[모닝폰]</t>
+        </is>
+      </c>
+      <c r="F128" s="6" t="inlineStr"/>
+      <c r="G128" s="6" t="inlineStr"/>
+      <c r="H128" s="6" t="inlineStr">
+        <is>
+          <t>EU 배터리 규제 상세 내용을 파악하고, 해당 규제에 부합하는 제품 설계 및 생산 공정 변경 가능성을 검토하며, 관련 물류 프로세스(예: 교체용 배터리 유통, 폐배터리 회수)에 대한 계획 수립</t>
+        </is>
+      </c>
+      <c r="I128" s="6" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="6" t="inlineStr">
+        <is>
+          <t>RSK-128</t>
+        </is>
+      </c>
+      <c r="B129" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C129" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D129" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E129" s="6" t="inlineStr">
+        <is>
+          <t>중, 호르무즈 재봉쇄 직전 헬륨 수출 금지···‘자국 우선’ 수출 통제</t>
+        </is>
+      </c>
+      <c r="F129" s="6" t="inlineStr"/>
+      <c r="G129" s="6" t="inlineStr"/>
+      <c r="H129" s="6" t="inlineStr">
+        <is>
+          <t>핵심 원자재 및 부품의 공급망 리스크를 재평가하고, 특정 국가 의존도를 낮추기 위한 공급처 다변화 전략을 적극적으로 모색하며, 비상 재고 확보 방안 검토</t>
+        </is>
+      </c>
+      <c r="I129" s="6" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="6" t="inlineStr">
+        <is>
+          <t>RSK-129</t>
+        </is>
+      </c>
+      <c r="B130" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C130" s="6" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="D130" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E130" s="6" t="inlineStr">
+        <is>
+          <t>보일하이츠 리니지 물류창고 화재 수습 지연…파리 떼 극성과 악취로 주민 고통 심화</t>
+        </is>
+      </c>
+      <c r="F130" s="6" t="inlineStr"/>
+      <c r="G130" s="6" t="inlineStr"/>
+      <c r="H130" s="6" t="inlineStr">
+        <is>
+          <t>현재 사용 중인 물류창고의 화재 안전 시스템 및 비상 대응 계획을 즉시 점검하고, 위험물 보관 규정 준수 여부를 재확인하며, 비상시 대체 보관 및 운송 계획 수립</t>
+        </is>
+      </c>
+      <c r="I130" s="6" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="6" t="inlineStr">
+        <is>
+          <t>RSK-130</t>
+        </is>
+      </c>
+      <c r="B131" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C131" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D131" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E131" s="6" t="inlineStr">
+        <is>
+          <t>이란 "호르무즈 해협 봉쇄하겠다"</t>
+        </is>
+      </c>
+      <c r="F131" s="6" t="inlineStr"/>
+      <c r="G131" s="6" t="inlineStr"/>
+      <c r="H131" s="6" t="inlineStr">
+        <is>
+          <t>중동발 원자재 및 부품의 재고 수준을 즉시 점검하고, 대체 운송 경로 및 운송 수단 확보 방안을 긴급 검토하며, 유가 및 운임 변동에 대한 헤징 전략을 수립.</t>
+        </is>
+      </c>
+      <c r="I131" s="6" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="6" t="inlineStr">
+        <is>
+          <t>RSK-131</t>
+        </is>
+      </c>
+      <c r="B132" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C132" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D132" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E132" s="6" t="inlineStr">
+        <is>
+          <t>다시 막힌 호르무즈 해협…국내 원유 수급 문제 없나</t>
+        </is>
+      </c>
+      <c r="F132" s="6" t="inlineStr"/>
+      <c r="G132" s="6" t="inlineStr"/>
+      <c r="H132" s="6" t="inlineStr">
+        <is>
+          <t>유가 변동에 따른 물류비 상승 시나리오를 수립하고, 운송 계약의 유류할증료 조항을 검토하며, 대체 에너지원 또는 운송 수단 활용 가능성을 모색.</t>
+        </is>
+      </c>
+      <c r="I132" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
📰 뉴스 데이터 2026-07-15_08:53
</commit_message>
<xml_diff>
--- a/data/SCM_물류_브리핑.xlsx
+++ b/data/SCM_물류_브리핑.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J746"/>
+  <dimension ref="A1:J783"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -35754,6 +35754,1734 @@
       </c>
       <c r="J746" s="4" t="inlineStr"/>
     </row>
+    <row r="747">
+      <c r="A747" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B747" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C747" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D747" s="2" t="inlineStr">
+        <is>
+          <t>[26.07.03] 글로벌 공급망 인사이트 175호</t>
+        </is>
+      </c>
+      <c r="E747" s="2" t="inlineStr">
+        <is>
+          <t>코트라 글로벌 공급망 인사이트 175호에 따르면, 미국-중국 간 수출통제 및 제재, 콩고의 코발트 수출 쿼터 회수, 중국의 인듐/갈륨 수출 검사 강화 등 주요 원자재 및 무역 관련 지정학적 리스크가 부각되고 있다.</t>
+        </is>
+      </c>
+      <c r="F747" s="2" t="inlineStr">
+        <is>
+          <t>배터리/전자부품 제조기업으로서 코발트, 인듐, 갈륨 등 핵심 원자재의 수출 규제 및 쿼터 변동은 생산 계획 및 공급망 안정성에 직접적인 영향을 미치므로 즉시 대응이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G747" s="2" t="inlineStr">
+        <is>
+          <t>코발트, 인듐, 갈륨 등 핵심 원자재의 공급망 다변화 및 재고 확보 방안 검토, 관련 규제 변화 모니터링 강화.</t>
+        </is>
+      </c>
+      <c r="H747" s="2" t="inlineStr">
+        <is>
+          <t>kotra</t>
+        </is>
+      </c>
+      <c r="I747" s="2" t="inlineStr">
+        <is>
+          <t>https://dream.kotra.or.kr/kotranews/cms/news/actionKotraBoardDetail.do?SITE_NO=3&amp;MENU_ID=70&amp;CONTENTS_NO=1&amp;pNttSn=242590</t>
+        </is>
+      </c>
+      <c r="J747" s="2" t="inlineStr">
+        <is>
+          <t>RSK-132</t>
+        </is>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B748" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C748" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D748" s="2" t="inlineStr">
+        <is>
+          <t>이란의 VLCC 연쇄 공격에 원유시장 '원점 회귀'</t>
+        </is>
+      </c>
+      <c r="E748" s="2" t="inlineStr">
+        <is>
+          <t>이란이 중동 해역에서 초대형 원유운반선(VLCC)을 연쇄 공격하여 글로벌 원유시장과 유조선 시장의 불확실성이 커졌으며, 이는 유가 상승 압력으로 작용할 수 있다.</t>
+        </is>
+      </c>
+      <c r="F748" s="2" t="inlineStr">
+        <is>
+          <t>중동 지역의 지정학적 불안정 심화는 유가 상승을 유발하여 해상 운임 및 물류비에 직접적인 영향을 미치며, 해당 지역 운송 안전성에도 위험을 초래할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G748" s="2" t="inlineStr">
+        <is>
+          <t>유가 변동 추이 면밀히 모니터링, 해상 운송 보험 조건 및 중동 항로 이용 시 대체 경로 또는 운송 방식 검토.</t>
+        </is>
+      </c>
+      <c r="H748" s="2" t="inlineStr">
+        <is>
+          <t>oceanpress</t>
+        </is>
+      </c>
+      <c r="I748" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oceanpress.co.kr/news/article.html?no=30615</t>
+        </is>
+      </c>
+      <c r="J748" s="2" t="inlineStr">
+        <is>
+          <t>RSK-133</t>
+        </is>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B749" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C749" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D749" s="2" t="inlineStr">
+        <is>
+          <t>미-이란, 호르무즈 통제권 놓고 또 충돌…오만, 남북 2개 항로 제안</t>
+        </is>
+      </c>
+      <c r="E749" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 통제권을 둘러싼 미-이란 갈등이 재점화되었으며, 오만이 남북 2개 항로 분리 방안을 제안했다.</t>
+        </is>
+      </c>
+      <c r="F749" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협은 주요 해상 운송로로, 갈등 심화 시 운송 지연, 운임 급등, 보험료 인상 등 우리 물류 운영에 즉각적이고 직접적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G749" s="2" t="inlineStr">
+        <is>
+          <t>중동 지역 정세 변화를 실시간으로 모니터링하고, 주요 항로의 대체 경로 및 비상 운송 계획을 수립하며, 포워더와 긴밀히 소통하여 선박 스케줄 변경 가능성에 대비한다.</t>
+        </is>
+      </c>
+      <c r="H749" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I749" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260713-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J749" s="2" t="inlineStr">
+        <is>
+          <t>RSK-134</t>
+        </is>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B750" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C750" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D750" s="2" t="inlineStr">
+        <is>
+          <t>트럼프 '호르무즈 통행료' 하루 만에 철회…해협 불확실성은 여전</t>
+        </is>
+      </c>
+      <c r="E750" s="2" t="inlineStr">
+        <is>
+          <t>트럼프 대통령이 호르무즈 해협 통행료 부과 구상을 하루 만에 철회했으나, 해협을 둘러싼 불확실성은 여전히 높다.</t>
+        </is>
+      </c>
+      <c r="F750" s="2" t="inlineStr">
+        <is>
+          <t>통행료 부과 철회는 긍정적이나, 언제든 유사한 정책이 재추진될 수 있어 호르무즈 해협의 지정학적 리스크가 우리 물류 비용 및 안정성에 직접적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G750" s="2" t="inlineStr">
+        <is>
+          <t>중동 지역의 정치적 발언 및 정책 변화를 면밀히 주시하고, 운송 계약 시 지정학적 리스크 관련 조항을 검토하며, 비상시 대체 운송 방안을 재점검한다.</t>
+        </is>
+      </c>
+      <c r="H750" s="2" t="inlineStr">
+        <is>
+          <t>뉴스핌</t>
+        </is>
+      </c>
+      <c r="I750" s="2" t="inlineStr">
+        <is>
+          <t>https://www.newspim.com/news/view/20260715000027</t>
+        </is>
+      </c>
+      <c r="J750" s="2" t="inlineStr">
+        <is>
+          <t>RSK-135</t>
+        </is>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B751" s="2" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C751" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D751" s="2" t="inlineStr">
+        <is>
+          <t>[테크 차이나] 中 전기차 배터리 안전기준 대폭 강화…산업 재편 본격화</t>
+        </is>
+      </c>
+      <c r="E751" s="2" t="inlineStr">
+        <is>
+          <t>중국이 7월 1일부터 전기차 배터리 안전 국가표준을 대폭 강화하여, 관련 산업 전반에 걸쳐 재편이 예상됩니다.</t>
+        </is>
+      </c>
+      <c r="F751" s="2" t="inlineStr">
+        <is>
+          <t>중국으로 수출되는 배터리 제품에 대한 안전 규제 강화는 우리 회사의 제품 설계, 생산, 그리고 중국향 물류 프로세스에 직접적인 영향을 미칠 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G751" s="2" t="inlineStr">
+        <is>
+          <t>중국 수출 제품의 배터리 안전 기준(GB 38031-2025) 준수 여부 즉시 확인 및 필요 시 제품/포장/운송 방식 변경 검토.</t>
+        </is>
+      </c>
+      <c r="H751" s="2" t="inlineStr">
+        <is>
+          <t>전자신문</t>
+        </is>
+      </c>
+      <c r="I751" s="2" t="inlineStr">
+        <is>
+          <t>https://etnews.com/20260714000143</t>
+        </is>
+      </c>
+      <c r="J751" s="2" t="inlineStr">
+        <is>
+          <t>RSK-136</t>
+        </is>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B752" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C752" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D752" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 충돌에 국제유가 80달러 육박…정부 “7~8월 물량 차질 없어”</t>
+        </is>
+      </c>
+      <c r="E752" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 충돌 격화로 국제유가가 배럴당 80달러에 육박하며 급등했으나, 정부는 7~8월 물량 차질은 없을 것이라고 밝혔다.</t>
+        </is>
+      </c>
+      <c r="F752" s="2" t="inlineStr">
+        <is>
+          <t>주요 해상 운송로인 호르무즈 해협의 지정학적 리스크로 인한 국제유가 급등은 모든 운송 모드의 유류할증료 및 물류비용에 즉각적이고 직접적인 상승 압력을 가한다.</t>
+        </is>
+      </c>
+      <c r="G752" s="2" t="inlineStr">
+        <is>
+          <t>국제유가 및 중동 정세 변화를 실시간으로 모니터링하고, 유류할증료 변동에 따른 물류 예산 재검토 및 운송 계약의 유류할증료 조항을 확인한다.</t>
+        </is>
+      </c>
+      <c r="H752" s="2" t="inlineStr">
+        <is>
+          <t>동아일보</t>
+        </is>
+      </c>
+      <c r="I752" s="2" t="inlineStr">
+        <is>
+          <t>https://www.donga.com/news/Economy/article/all/20260713/134288100/1</t>
+        </is>
+      </c>
+      <c r="J752" s="2" t="inlineStr">
+        <is>
+          <t>RSK-137</t>
+        </is>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B753" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C753" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D753" s="3" t="inlineStr">
+        <is>
+          <t>Air Cargo Demand Up 6.0% in May</t>
+        </is>
+      </c>
+      <c r="E753" s="3" t="inlineStr">
+        <is>
+          <t>2026년 5월 전 세계 항공 화물 수요가 전년 대비 6.0% 증가하여 항공 화물 시장의 성장세를 보였다.</t>
+        </is>
+      </c>
+      <c r="F753" s="3" t="inlineStr">
+        <is>
+          <t>항공 화물 수요 증가는 향후 항공 운임 상승 압력으로 작용할 수 있으므로 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G753" s="3" t="n"/>
+      <c r="H753" s="3" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I753" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-29-air-cargo-demand-up-may/</t>
+        </is>
+      </c>
+      <c r="J753" s="3" t="inlineStr"/>
+    </row>
+    <row r="754">
+      <c r="A754" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B754" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C754" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D754" s="3" t="inlineStr">
+        <is>
+          <t>Urgent Action Needed to Ease Engine MRO Bottlenecks</t>
+        </is>
+      </c>
+      <c r="E754" s="3" t="inlineStr">
+        <is>
+          <t>항공기 엔진 유지보수(MRO) 병목 현상 완화를 위한 긴급 조치가 필요하며, 이는 항공기 가동률에 영향을 미쳐 항공 화물 운송 능력에 부담을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="F754" s="3" t="inlineStr">
+        <is>
+          <t>엔진 MRO 병목 현상은 항공 화물 운송 능력 감소로 이어져 운임 상승 및 스케줄 지연을 유발할 수 있으므로 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G754" s="3" t="n"/>
+      <c r="H754" s="3" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I754" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-24-urgent-action-needed-to-ease-engine-mro-bottlenecks/</t>
+        </is>
+      </c>
+      <c r="J754" s="3" t="inlineStr"/>
+    </row>
+    <row r="755">
+      <c r="A755" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B755" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C755" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D755" s="3" t="inlineStr">
+        <is>
+          <t>고려해운, 한일항로 개편…부산-규슈 통합</t>
+        </is>
+      </c>
+      <c r="E755" s="3" t="inlineStr">
+        <is>
+          <t>고려해운이 한일항로 컨테이너선 네트워크를 개편하여 부산-규슈 노선을 통합하고 운항 선박을 대형화하며, 나가사키항 기항을 중단한다.</t>
+        </is>
+      </c>
+      <c r="F755" s="3" t="inlineStr">
+        <is>
+          <t>한일 항로를 이용하는 경우, 노선 통합 및 기항지 변경이 운송 리드타임 및 비용에 영향을 줄 수 있으므로 확인이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G755" s="3" t="inlineStr">
+        <is>
+          <t>한일 항로 이용 시 변경된 노선 및 기항지 확인, 운송 스케줄 및 비용 영향 분석.</t>
+        </is>
+      </c>
+      <c r="H755" s="3" t="inlineStr">
+        <is>
+          <t>ksg</t>
+        </is>
+      </c>
+      <c r="I755" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ksg.co.kr/news/main_newsView.jsp?pNum=147572</t>
+        </is>
+      </c>
+      <c r="J755" s="3" t="inlineStr"/>
+    </row>
+    <row r="756">
+      <c r="A756" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B756" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C756" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D756" s="3" t="inlineStr">
+        <is>
+          <t>Structural Contraction of Global Liner Networks</t>
+        </is>
+      </c>
+      <c r="E756" s="3" t="inlineStr">
+        <is>
+          <t>2012년 이후 글로벌 정기선 네트워크가 구조적으로 축소되고 있으며, 이는 지리적 범위는 유지되나 서비스 빈도가 감소하는 경향을 보인다.</t>
+        </is>
+      </c>
+      <c r="F756" s="3" t="inlineStr">
+        <is>
+          <t>정기선 서비스 빈도 감소는 특정 항로의 운송 리드타임 증가 또는 스케줄 유연성 저하로 이어질 수 있으므로 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G756" s="3" t="n"/>
+      <c r="H756" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I756" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/397-structural-contraction-of-global-liner-networks</t>
+        </is>
+      </c>
+      <c r="J756" s="3" t="inlineStr"/>
+    </row>
+    <row r="757">
+      <c r="A757" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B757" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C757" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D757" s="3" t="inlineStr">
+        <is>
+          <t>Transpacific: Ripe for new non-alliance services</t>
+        </is>
+      </c>
+      <c r="E757" s="3" t="inlineStr">
+        <is>
+          <t>태평양 횡단 항로에서 비동맹 선사들의 새로운 서비스가 증가할 가능성이 있으며, 이는 컨테이너 스팟 운임과 관련이 있다.</t>
+        </is>
+      </c>
+      <c r="F757" s="3" t="inlineStr">
+        <is>
+          <t>태평양 횡단 항로의 비동맹 선사 서비스 증가는 운임 경쟁을 심화시켜 운임 하락 압력으로 작용할 수 있으므로 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G757" s="3" t="n"/>
+      <c r="H757" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I757" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/393-transpacific-ripe-for-new-non-alliance-services</t>
+        </is>
+      </c>
+      <c r="J757" s="3" t="inlineStr"/>
+    </row>
+    <row r="758">
+      <c r="A758" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B758" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C758" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D758" s="3" t="inlineStr">
+        <is>
+          <t>미·이란 전면전 위기…국제유가 9%↑, 한달만에 최고치</t>
+        </is>
+      </c>
+      <c r="E758" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 인근 긴장으로 공급 차질 우려가 커지며 국제유가가 한 달 만에 최고치로 9% 급등했다.</t>
+        </is>
+      </c>
+      <c r="F758" s="3" t="inlineStr">
+        <is>
+          <t>국제유가 급등은 해상/항공/육상 운송비용에 직접적인 영향을 미치므로, 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G758" s="3" t="inlineStr">
+        <is>
+          <t>유가 추이 및 유류할증료 변동을 주시하고, 운송 계약 시 유가 변동 조항을 검토한다.</t>
+        </is>
+      </c>
+      <c r="H758" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I758" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260714-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J758" s="3" t="inlineStr"/>
+    </row>
+    <row r="759">
+      <c r="A759" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B759" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C759" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D759" s="3" t="inlineStr">
+        <is>
+          <t>유가 150달러 경고! 세계 경제 뒤흔들 최악의 시나리오</t>
+        </is>
+      </c>
+      <c r="E759" s="3" t="inlineStr">
+        <is>
+          <t>유가가 150달러까지 급등할 수 있다는 경고가 나왔으나, 대체 운송로 확보와 전략비축유 방출 등으로 가격이 안정될 수 있다는 전망도 함께 제시되었다.</t>
+        </is>
+      </c>
+      <c r="F759" s="3" t="inlineStr">
+        <is>
+          <t>극심한 유가 변동 가능성은 물류비용에 막대한 영향을 줄 수 있으나, 안정화 요인도 있어 추이를 지켜봐야 한다.</t>
+        </is>
+      </c>
+      <c r="G759" s="3" t="inlineStr">
+        <is>
+          <t>글로벌 유가 시장 동향 및 중동 정세 변화를 면밀히 모니터링하고, 비상시 물류비용 상승에 대비한 예산을 검토한다.</t>
+        </is>
+      </c>
+      <c r="H759" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I759" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260713-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J759" s="3" t="inlineStr"/>
+    </row>
+    <row r="760">
+      <c r="A760" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B760" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C760" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D760" s="3" t="inlineStr">
+        <is>
+          <t>봉쇄 위기 넘긴 호르무즈 해협…"오만 '남북 항로 분리' 제안"</t>
+        </is>
+      </c>
+      <c r="E760" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협의 봉쇄 위기는 일단 넘겼으나, 오만이 선박 통항을 남북 2개 분리 항로로 관리하는 방안을 제안했다.</t>
+        </is>
+      </c>
+      <c r="F760" s="3" t="inlineStr">
+        <is>
+          <t>즉각적인 봉쇄 위기는 넘겼지만, 항로 분리 제안은 향후 운항 절차, 시간, 비용에 영향을 줄 수 있어 지속적인 관찰이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G760" s="3" t="inlineStr">
+        <is>
+          <t>오만의 항로 분리 제안에 대한 국제사회의 논의와 실제 적용 여부를 주시하고, 잠재적인 운송 시간 및 비용 변화를 예측한다.</t>
+        </is>
+      </c>
+      <c r="H760" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I760" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260712-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J760" s="3" t="inlineStr"/>
+    </row>
+    <row r="761">
+      <c r="A761" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B761" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C761" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D761" s="3" t="inlineStr">
+        <is>
+          <t>11주 만에 꺾인 해상운임 '숨고르기'… HMM·팬오션 실적은 '청신호'</t>
+        </is>
+      </c>
+      <c r="E761" s="3" t="inlineStr">
+        <is>
+          <t>고공행진을 이어가던 글로벌 해상운임이 11주 만에 하락세로 전환하며 숨고르기에 들어갔다.</t>
+        </is>
+      </c>
+      <c r="F761" s="3" t="inlineStr">
+        <is>
+          <t>해상운임 하락은 물류비용 절감 기회가 될 수 있으나, 일시적 현상일 수 있으므로 장기적인 추이를 모니터링하여 운송 계약 전략에 반영해야 한다.</t>
+        </is>
+      </c>
+      <c r="G761" s="3" t="inlineStr">
+        <is>
+          <t>주요 해상운임 지수(SCFI, FBX 등)를 지속적으로 모니터링하고, 포워더와 협상 시 운임 하락 추세를 반영하여 비용 절감 방안을 모색한다.</t>
+        </is>
+      </c>
+      <c r="H761" s="3" t="inlineStr">
+        <is>
+          <t>파이낸셜뉴스</t>
+        </is>
+      </c>
+      <c r="I761" s="3" t="inlineStr">
+        <is>
+          <t>https://fnnews.com/news/202607140822416437</t>
+        </is>
+      </c>
+      <c r="J761" s="3" t="inlineStr"/>
+    </row>
+    <row r="762">
+      <c r="A762" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B762" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C762" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D762" s="3" t="inlineStr">
+        <is>
+          <t>“호르무즈 의존도 ‘0’으로”···UAE의 ‘결단’ 새 항만 건설 ‘돌파구’</t>
+        </is>
+      </c>
+      <c r="E762" s="3" t="inlineStr">
+        <is>
+          <t>아랍에미리트(UAE) 두바이 소유 물류기업 DP월드가 호르무즈 해협 의존도를 낮추기 위해 UAE 동쪽 해안에 새로운 항구와 컨테이너 터미널을 건설할 계획이다.</t>
+        </is>
+      </c>
+      <c r="F762" s="3" t="inlineStr">
+        <is>
+          <t>UAE의 신항만 건설은 장기적으로 호르무즈 해협 우회 경로를 제공하여 중동 지역 물류의 안정성을 높일 수 있으나, 완공까지 시간이 소요되므로 지속적인 관찰이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G762" s="3" t="inlineStr">
+        <is>
+          <t>신항만 건설 진행 상황을 주시하고, 완공 시 우리 회사의 중동 지역 물류 네트워크 및 운송 경로 다변화에 활용 가능성을 검토한다.</t>
+        </is>
+      </c>
+      <c r="H762" s="3" t="inlineStr">
+        <is>
+          <t>경향신문</t>
+        </is>
+      </c>
+      <c r="I762" s="3" t="inlineStr">
+        <is>
+          <t>https://www.khan.co.kr/article/202607140711001</t>
+        </is>
+      </c>
+      <c r="J762" s="3" t="inlineStr"/>
+    </row>
+    <row r="763">
+      <c r="A763" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B763" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C763" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D763" s="3" t="inlineStr">
+        <is>
+          <t>From Deluges to Dry Beds: How Extreme Weather is Rewriting Logistics Strategy</t>
+        </is>
+      </c>
+      <c r="E763" s="3" t="inlineStr">
+        <is>
+          <t>극심한 기후 변화가 물류 전략을 재편하고 있으며, 기후 관련 물류 중단이 고립된 사건이 아닌 시스템적이고 복합적인 위험으로 인식되고 있다.</t>
+        </is>
+      </c>
+      <c r="F763" s="3" t="inlineStr">
+        <is>
+          <t>기후 변화로 인한 물류 중단은 운송 지연, 창고 손상 등 우리 공급망 전반에 걸쳐 예측 불가능한 위험을 증가시키므로, 장기적인 관점에서 물류 전략에 반영해야 한다.</t>
+        </is>
+      </c>
+      <c r="G763" s="3" t="inlineStr">
+        <is>
+          <t>기후 변화에 따른 물류 리스크를 평가하고, 운송 경로 다변화, 재고 관리 전략 조정, 비상 계획 수립 등 공급망 회복력 강화 방안을 검토한다.</t>
+        </is>
+      </c>
+      <c r="H763" s="3" t="inlineStr">
+        <is>
+          <t>Logistics Viewpoints</t>
+        </is>
+      </c>
+      <c r="I763" s="3" t="inlineStr">
+        <is>
+          <t>https://logisticsviewpoints.com/2026/07/13/from-deluges-to-dry-beds-how-extreme-weather-is-rewriting-logistics-strategy</t>
+        </is>
+      </c>
+      <c r="J763" s="3" t="inlineStr"/>
+    </row>
+    <row r="764">
+      <c r="A764" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B764" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C764" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D764" s="3" t="inlineStr">
+        <is>
+          <t>Geopolitical disruption and AI demand reshape cargo markets</t>
+        </is>
+      </c>
+      <c r="E764" s="3" t="inlineStr">
+        <is>
+          <t>항공 화물 시장이 지정학적 불확실성과 높은 유가에도 불구하고 상대적 안정기에 접어들었으며, AI 수요가 시장을 재편하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F764" s="3" t="inlineStr">
+        <is>
+          <t>항공 화물 시장의 전반적인 안정화 추세는 긍정적이나, 지정학적 불확실성과 AI 수요로 인한 시장 재편 가능성은 지속적인 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G764" s="3" t="n"/>
+      <c r="H764" s="3" t="inlineStr">
+        <is>
+          <t>Air Cargo Week</t>
+        </is>
+      </c>
+      <c r="I764" s="3" t="inlineStr">
+        <is>
+          <t>https://aircargoweek.com/geopolitical-disruption-and-ai-demand-reshape-cargo-markets</t>
+        </is>
+      </c>
+      <c r="J764" s="3" t="inlineStr"/>
+    </row>
+    <row r="765">
+      <c r="A765" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B765" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C765" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D765" s="3" t="inlineStr">
+        <is>
+          <t>이란도 조롱할 만큼 터무니없는 20% 통항료···실현 가능성 낮지만, 점점 멀어지는 자유통항 원칙</t>
+        </is>
+      </c>
+      <c r="E765" s="3" t="inlineStr">
+        <is>
+          <t>도널드 트럼프 전 미국 대통령이 호르무즈 해협 통항료 20% 부과를 언급하며 원유 운송 비용 급증 우려를 낳았으나, 실현 가능성은 낮게 평가됩니다.</t>
+        </is>
+      </c>
+      <c r="F765" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협은 주요 원유 수송로로, 통항료 부과가 현실화될 경우 유가 상승을 유발하여 해상 운임 및 물류비에 간접적인 영향을 줄 수 있으므로 추이를 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G765" s="3" t="n"/>
+      <c r="H765" s="3" t="inlineStr">
+        <is>
+          <t>경향신문</t>
+        </is>
+      </c>
+      <c r="I765" s="3" t="inlineStr">
+        <is>
+          <t>https://khan.co.kr/article/202607141419001</t>
+        </is>
+      </c>
+      <c r="J765" s="3" t="inlineStr"/>
+    </row>
+    <row r="766">
+      <c r="A766" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B766" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C766" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D766" s="3" t="inlineStr">
+        <is>
+          <t>중국산 걷어내려면 비용이 무려…“미국·유럽 탈중국에 3.5경원 든다”</t>
+        </is>
+      </c>
+      <c r="E766" s="3" t="inlineStr">
+        <is>
+          <t>컨설팅업체 분석에 따르면 미국과 유럽이 중국 공급망에서 부분적으로 벗어나기 위해 막대한 비용이 들 것으로 예상되며, 이는 현실적인 탈중국 전략의 어려움을 시사한다.</t>
+        </is>
+      </c>
+      <c r="F766" s="3" t="inlineStr">
+        <is>
+          <t>주요 시장의 탈중국 공급망 재편 움직임은 장기적인 관점에서 우리 회사의 생산 및 물류 거점 전략, 원자재 조달처 다변화에 영향을 미칠 수 있으므로 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G766" s="3" t="inlineStr">
+        <is>
+          <t>글로벌 공급망 재편 동향을 지속적으로 모니터링하고, 잠재적인 공급망 다변화 전략 및 비용 영향을 평가한다.</t>
+        </is>
+      </c>
+      <c r="H766" s="3" t="inlineStr">
+        <is>
+          <t>매일경제</t>
+        </is>
+      </c>
+      <c r="I766" s="3" t="inlineStr">
+        <is>
+          <t>https://mk.co.kr/news/world/12097543</t>
+        </is>
+      </c>
+      <c r="J766" s="3" t="inlineStr"/>
+    </row>
+    <row r="767">
+      <c r="A767" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B767" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C767" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D767" s="3" t="inlineStr">
+        <is>
+          <t>[하반기 성장전략] 중동전 교훈에 공급망 4단계 정비…5대업종 탈탄소 전환 시동</t>
+        </is>
+      </c>
+      <c r="E767" s="3" t="inlineStr">
+        <is>
+          <t>정부가 중동전 교훈을 바탕으로 국내 생산, 해외 생산, 수입선 다변화 등 4단계 공급망 재편 전략을 추진하고, 5대 업종의 탈탄소 전환을 시작한다.</t>
+        </is>
+      </c>
+      <c r="F767" s="3" t="inlineStr">
+        <is>
+          <t>정부의 공급망 재편 및 탈탄소 전환 정책은 우리 회사의 국내외 생산 및 조달 전략, 그리고 ESG 물류 전환에 중장기적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G767" s="3" t="inlineStr">
+        <is>
+          <t>정부의 공급망 정책 및 지원 방안을 면밀히 검토하고, 우리 회사의 공급망 다변화 및 탈탄소 물류 전략에 반영할 방안을 모색한다.</t>
+        </is>
+      </c>
+      <c r="H767" s="3" t="inlineStr">
+        <is>
+          <t>연합뉴스</t>
+        </is>
+      </c>
+      <c r="I767" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20260713154800002</t>
+        </is>
+      </c>
+      <c r="J767" s="3" t="inlineStr"/>
+    </row>
+    <row r="768">
+      <c r="A768" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B768" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C768" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D768" s="3" t="inlineStr">
+        <is>
+          <t>EU "중국 의존 탈피에는 막대한 자금 필요"…공급망 다변화 지원기금 추진</t>
+        </is>
+      </c>
+      <c r="E768" s="3" t="inlineStr">
+        <is>
+          <t>유럽연합(EU)이 중국 공급망 의존도를 낮추기 위해 역내 기업에 대한 재정적 지원을 확대하고 공급망 다변화 지원기금을 추진할 계획이다.</t>
+        </is>
+      </c>
+      <c r="F768" s="3" t="inlineStr">
+        <is>
+          <t>EU의 공급망 다변화 지원 정책은 유럽 내 사업을 운영하거나 유럽 시장에 제품을 공급하는 우리 회사에 잠재적인 기회 또는 규제 변화로 작용할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G768" s="3" t="inlineStr">
+        <is>
+          <t>EU의 공급망 지원 정책 및 기금 추진 동향을 주시하고, 유럽 내 공급망 전략 및 파트너십 구축에 활용 가능성을 검토한다.</t>
+        </is>
+      </c>
+      <c r="H768" s="3" t="inlineStr">
+        <is>
+          <t>더구루</t>
+        </is>
+      </c>
+      <c r="I768" s="3" t="inlineStr">
+        <is>
+          <t>https://theguru.co.kr/news/article.html?no=104293</t>
+        </is>
+      </c>
+      <c r="J768" s="3" t="inlineStr"/>
+    </row>
+    <row r="769">
+      <c r="A769" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B769" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C769" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D769" s="3" t="inlineStr">
+        <is>
+          <t>예상 밖 길어진 해운 호황···HMM 몸값 키우나</t>
+        </is>
+      </c>
+      <c r="E769" s="3" t="inlineStr">
+        <is>
+          <t>해상운임 강세가 예상보다 길어지면서 HMM의 기업가치가 상승하고 있으며, 2분기와 하반기에도 호실적이 기대된다.</t>
+        </is>
+      </c>
+      <c r="F769" s="3" t="inlineStr">
+        <is>
+          <t>해상운임 강세가 지속될 것으로 예상되어 우리 회사의 해상 물류 비용 부담이 계속될 것이며, 이는 물류 예산 및 운송 계획에 영향을 미친다.</t>
+        </is>
+      </c>
+      <c r="G769" s="3" t="inlineStr">
+        <is>
+          <t>해상운임 동향을 지속적으로 모니터링하고, 장기 계약 검토 및 운송 모드 최적화 등 비용 절감 방안을 모색한다.</t>
+        </is>
+      </c>
+      <c r="H769" s="3" t="inlineStr">
+        <is>
+          <t>시사저널e</t>
+        </is>
+      </c>
+      <c r="I769" s="3" t="inlineStr">
+        <is>
+          <t>https://sisajournal-e.com/news/articleView.html?idxno=422402</t>
+        </is>
+      </c>
+      <c r="J769" s="3" t="inlineStr"/>
+    </row>
+    <row r="770">
+      <c r="A770" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B770" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C770" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D770" s="3" t="inlineStr">
+        <is>
+          <t>"대한항공, 목표가 4.1만↑…고유가에도 화물·국제선 호조"-하나</t>
+        </is>
+      </c>
+      <c r="E770" s="3" t="inlineStr">
+        <is>
+          <t>고유가에도 불구하고 항공화물 및 국제선 수요 호조로 대한항공의 실적이 개선될 것으로 예상되며, 이는 비탄력적인 항공 수요를 반영한다.</t>
+        </is>
+      </c>
+      <c r="F770" s="3" t="inlineStr">
+        <is>
+          <t>고유가에도 불구하고 항공화물 수요가 견조하여 항공운임이 높은 수준을 유지할 가능성이 크므로, 항공 운송을 이용하는 우리 회사의 물류 비용에 지속적인 영향을 미칠 것이다.</t>
+        </is>
+      </c>
+      <c r="G770" s="3" t="inlineStr">
+        <is>
+          <t>항공운임 및 유류할증료 동향을 면밀히 주시하고, 긴급 화물 외에는 해상 운송 전환 또는 운송 계획 최적화를 검토하여 비용 효율성을 확보한다.</t>
+        </is>
+      </c>
+      <c r="H770" s="3" t="inlineStr">
+        <is>
+          <t>머니투데이</t>
+        </is>
+      </c>
+      <c r="I770" s="3" t="inlineStr">
+        <is>
+          <t>https://mt.co.kr/stock/2026/07/14/2026071408053868162</t>
+        </is>
+      </c>
+      <c r="J770" s="3" t="inlineStr"/>
+    </row>
+    <row r="771">
+      <c r="A771" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B771" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C771" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D771" s="3" t="inlineStr">
+        <is>
+          <t>변화하는 물류 환경, 어떻게 준비하고 계십니까?</t>
+        </is>
+      </c>
+      <c r="E771" s="3" t="inlineStr">
+        <is>
+          <t>이커머스 성장과 다품종 소량 생산으로 인한 SKU 복잡성 증가, 물류 거점 부지 및 인건비 상승, 인력 부족 등 국내외 물류 현장의 다양한 도전 과제들이 제기되고 있다.</t>
+        </is>
+      </c>
+      <c r="F771" s="3" t="inlineStr">
+        <is>
+          <t>물류 현장의 SKU 복잡성, 비용 상승, 인력 부족 등은 우리 회사의 창고 운영 효율성, 물류 거점 전략, 인력 수급에 직접적인 영향을 미칠 수 있는 장기적인 과제이다.</t>
+        </is>
+      </c>
+      <c r="G771" s="3" t="inlineStr">
+        <is>
+          <t>물류 자동화 및 디지털 전환 투자 계획을 검토하고, 물류 거점 최적화 및 인력 운영 효율화 방안을 수립하여 변화하는 물류 환경에 선제적으로 대응한다.</t>
+        </is>
+      </c>
+      <c r="H771" s="3" t="inlineStr">
+        <is>
+          <t>헬로티 HelloT</t>
+        </is>
+      </c>
+      <c r="I771" s="3" t="inlineStr">
+        <is>
+          <t>https://hellot.net/news/article.html?no=113750</t>
+        </is>
+      </c>
+      <c r="J771" s="3" t="inlineStr"/>
+    </row>
+    <row r="772">
+      <c r="A772" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B772" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C772" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D772" s="4" t="inlineStr">
+        <is>
+          <t>Global Schedule Reliability for May 2026 the Highest of the Year</t>
+        </is>
+      </c>
+      <c r="E772" s="4" t="inlineStr">
+        <is>
+          <t>2026년 5월 전 세계 정기선 스케줄 신뢰도가 올해 최고치를 기록하여 해상 운송의 정시성이 개선되고 있음을 나타낸다.</t>
+        </is>
+      </c>
+      <c r="F772" s="4" t="inlineStr">
+        <is>
+          <t>스케줄 신뢰도 개선은 긍정적인 신호이나, 일회성 데이터일 수 있으며 당장 우리 물류 운영에 직접적인 영향은 낮다.</t>
+        </is>
+      </c>
+      <c r="G772" s="4" t="n"/>
+      <c r="H772" s="4" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I772" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/395-global-schedule-reliability-for-may-2026-the-highest-of-the-year</t>
+        </is>
+      </c>
+      <c r="J772" s="4" t="inlineStr"/>
+    </row>
+    <row r="773">
+      <c r="A773" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B773" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C773" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D773" s="4" t="inlineStr">
+        <is>
+          <t>영남이공대, '교육 넘어 채용까지'…쿠팡과 손잡고 AI 물류인재 키운다</t>
+        </is>
+      </c>
+      <c r="E773" s="4" t="inlineStr">
+        <is>
+          <t>영남이공대학교가 쿠팡풀필먼트서비스와 협력하여 AI 기반 물류 전문교육과 취업을 연계하는 현장형 인재 양성에 나선다.</t>
+        </is>
+      </c>
+      <c r="F773" s="4" t="inlineStr">
+        <is>
+          <t>물류 산업의 인재 양성 동향을 보여주는 뉴스이나, 우리 회사의 당면한 물류 운영이나 비용에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G773" s="4" t="n"/>
+      <c r="H773" s="4" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I773" s="4" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260715-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J773" s="4" t="inlineStr"/>
+    </row>
+    <row r="774">
+      <c r="A774" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B774" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C774" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D774" s="4" t="inlineStr">
+        <is>
+          <t>상하이, 런던 제치고 세계 2위 해운 중심지 등극… ‘물동량’ 넘어 ‘...</t>
+        </is>
+      </c>
+      <c r="E774" s="4" t="inlineStr">
+        <is>
+          <t>상하이가 컨테이너 물동량뿐 아니라 금융, 법률, 조선 등 종합적인 해운 역량을 바탕으로 세계 2위 해운 중심지로 부상했다.</t>
+        </is>
+      </c>
+      <c r="F774" s="4" t="inlineStr">
+        <is>
+          <t>주요 항만의 위상 변화는 장기적인 물류 네트워크 계획에 참고할 수 있으나, 당장 우리 회사의 물류 운영에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G774" s="4" t="n"/>
+      <c r="H774" s="4" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I774" s="4" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260714-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J774" s="4" t="inlineStr"/>
+    </row>
+    <row r="775">
+      <c r="A775" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B775" s="4" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C775" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D775" s="4" t="inlineStr">
+        <is>
+          <t>선사가 다른 선사를 인수할 때 정부가 나서는 이유 : 해운업과 국가안보의 경계 (Week 28, 2026)</t>
+        </is>
+      </c>
+      <c r="E775" s="4" t="inlineStr">
+        <is>
+          <t>해운 산업은 국가 기간 산업으로, 선사 간 인수합병 시 항만, 선박, 물류 데이터 등 핵심 인프라가 이전되므로 여러 나라가 국가안보 심사 절차를 두고 있다.</t>
+        </is>
+      </c>
+      <c r="F775" s="4" t="inlineStr">
+        <is>
+          <t>해운 산업의 국가안보적 중요성을 설명하는 정책적 내용으로, 우리 회사의 당면한 물류 운영에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G775" s="4" t="n"/>
+      <c r="H775" s="4" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I775" s="4" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/선사가-다른-선사를-인수할-때-정부가-나서는-이유-해운업과-국가안보의-경계-week-28-2026</t>
+        </is>
+      </c>
+      <c r="J775" s="4" t="inlineStr"/>
+    </row>
+    <row r="776">
+      <c r="A776" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B776" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C776" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D776" s="4" t="inlineStr">
+        <is>
+          <t>이베코코리아 / 연비·안전·주행 편의성 향상 대형 트랙터 ‘올 뉴 S-Way’ 출시</t>
+        </is>
+      </c>
+      <c r="E776" s="4" t="inlineStr">
+        <is>
+          <t>이베코코리아가 연비, 안전, 주행 편의성을 향상시킨 플래그십 대형 트랙터 ‘올 뉴 S-Way’를 국내 시장에 공식 출시했다.</t>
+        </is>
+      </c>
+      <c r="F776" s="4" t="inlineStr">
+        <is>
+          <t>신형 트럭 출시 소식은 운송 효율성 개선의 잠재력을 시사하지만, 당장 우리 회사의 물류 운영이나 비용에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G776" s="4" t="n"/>
+      <c r="H776" s="4" t="inlineStr">
+        <is>
+          <t>ulogistics</t>
+        </is>
+      </c>
+      <c r="I776" s="4" t="inlineStr">
+        <is>
+          <t>http://www.ulogistics.co.kr/test/board.php?board=all2&amp;command=body&amp;no=5212</t>
+        </is>
+      </c>
+      <c r="J776" s="4" t="inlineStr"/>
+    </row>
+    <row r="777">
+      <c r="A777" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B777" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C777" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D777" s="4" t="inlineStr">
+        <is>
+          <t>Freight Distress Report: Carrier, logistics closures erase over 245 jobs</t>
+        </is>
+      </c>
+      <c r="E777" s="4" t="inlineStr">
+        <is>
+          <t>화물 운송 및 물류 기업들의 폐업과 파산으로 245개 이상의 일자리가 사라졌다는 보고서가 나왔다.</t>
+        </is>
+      </c>
+      <c r="F777" s="4" t="inlineStr">
+        <is>
+          <t>일부 운송 및 물류 기업의 어려움을 보여주지만, 우리 회사의 주요 운송 파트너나 전체 물류 네트워크에 즉각적인 영향을 미칠 정도의 광범위한 위기는 아니다.</t>
+        </is>
+      </c>
+      <c r="G777" s="4" t="n"/>
+      <c r="H777" s="4" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="I777" s="4" t="inlineStr">
+        <is>
+          <t>https://finance.yahoo.com/economy/articles/freight-distress-report-carrier-logistics-144420684.html</t>
+        </is>
+      </c>
+      <c r="J777" s="4" t="inlineStr"/>
+    </row>
+    <row r="778">
+      <c r="A778" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B778" s="4" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C778" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D778" s="4" t="inlineStr">
+        <is>
+          <t>삼성SDI UPS 배터리…글로벌 화재시험 통과</t>
+        </is>
+      </c>
+      <c r="E778" s="4" t="inlineStr">
+        <is>
+          <t>삼성SDI의 UPS용 배터리가 글로벌 안전 인증기관 UL솔루션스의 옥내 대형 화재 테스트를 통과하며 높은 안전성을 입증했습니다.</t>
+        </is>
+      </c>
+      <c r="F778" s="4" t="inlineStr">
+        <is>
+          <t>경쟁사 제품의 안전성 강화 소식으로, 우리 회사의 직접적인 물류 운영에 미치는 영향은 낮지만, 시장의 안전 기준 강화 추세를 보여줍니다.</t>
+        </is>
+      </c>
+      <c r="G778" s="4" t="n"/>
+      <c r="H778" s="4" t="inlineStr">
+        <is>
+          <t>매일경제</t>
+        </is>
+      </c>
+      <c r="I778" s="4" t="inlineStr">
+        <is>
+          <t>https://mk.co.kr/news/business/12098616</t>
+        </is>
+      </c>
+      <c r="J778" s="4" t="inlineStr"/>
+    </row>
+    <row r="779">
+      <c r="A779" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B779" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C779" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D779" s="4" t="inlineStr">
+        <is>
+          <t>中하이난, 2030년부터 내연기관차 판매 금지 정책 재확인</t>
+        </is>
+      </c>
+      <c r="E779" s="4" t="inlineStr">
+        <is>
+          <t>중국 하이난성이 2030년부터 내연기관차 판매를 전면 금지하는 정책을 재확인하여 전기차 시장 확대에 기여할 것으로 보입니다.</t>
+        </is>
+      </c>
+      <c r="F779" s="4" t="inlineStr">
+        <is>
+          <t>장기적인 전기차 시장 확대 가능성을 시사하지만, 당장 우리 회사의 물류 운영에 직접적인 영향을 미치지는 않습니다.</t>
+        </is>
+      </c>
+      <c r="G779" s="4" t="n"/>
+      <c r="H779" s="4" t="inlineStr">
+        <is>
+          <t>연합뉴스</t>
+        </is>
+      </c>
+      <c r="I779" s="4" t="inlineStr">
+        <is>
+          <t>https://yna.co.kr/view/AKR20260713144900083</t>
+        </is>
+      </c>
+      <c r="J779" s="4" t="inlineStr"/>
+    </row>
+    <row r="780">
+      <c r="A780" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B780" s="4" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C780" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D780" s="4" t="inlineStr">
+        <is>
+          <t>서울교통공사, 대용량 리튬배터리 반입 제한 집중 캠페인</t>
+        </is>
+      </c>
+      <c r="E780" s="4" t="inlineStr">
+        <is>
+          <t>서울교통공사가 대용량 리튬배터리 및 개인형 이동장치(PM)의 지하철 반입 제한 제도 정착을 위한 캠페인을 진행 중입니다.</t>
+        </is>
+      </c>
+      <c r="F780" s="4" t="inlineStr">
+        <is>
+          <t>대중교통 내 개인 휴대품 규제로, 우리 회사의 제품 운송이나 물류 운영에 직접적인 영향은 없습니다.</t>
+        </is>
+      </c>
+      <c r="G780" s="4" t="n"/>
+      <c r="H780" s="4" t="inlineStr">
+        <is>
+          <t>헤럴드경제</t>
+        </is>
+      </c>
+      <c r="I780" s="4" t="inlineStr">
+        <is>
+          <t>https://biz.heraldcorp.com/article/10808357</t>
+        </is>
+      </c>
+      <c r="J780" s="4" t="inlineStr"/>
+    </row>
+    <row r="781">
+      <c r="A781" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B781" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C781" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D781" s="4" t="inlineStr">
+        <is>
+          <t>기후부, 미생물 활용해 폐배터리 속 리튬 90% 회수</t>
+        </is>
+      </c>
+      <c r="E781" s="4" t="inlineStr">
+        <is>
+          <t>기후에너지환경부가 담수 미생물을 이용해 폐배터리에서 리튬을 90% 회수하는 기술을 개발하여 자원 재활용 가능성을 높였습니다.</t>
+        </is>
+      </c>
+      <c r="F781" s="4" t="inlineStr">
+        <is>
+          <t>폐배터리 재활용 기술 개발 소식으로, 장기적으로 원자재 수급 및 역물류 전략에 영향을 줄 수 있으나 당장 물류 운영에 미치는 영향은 낮습니다.</t>
+        </is>
+      </c>
+      <c r="G781" s="4" t="n"/>
+      <c r="H781" s="4" t="inlineStr">
+        <is>
+          <t>아시아투데이</t>
+        </is>
+      </c>
+      <c r="I781" s="4" t="inlineStr">
+        <is>
+          <t>https://asiatoday.co.kr/kn/view.php?key=20260713010004556</t>
+        </is>
+      </c>
+      <c r="J781" s="4" t="inlineStr"/>
+    </row>
+    <row r="782">
+      <c r="A782" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B782" s="4" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C782" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D782" s="4" t="inlineStr">
+        <is>
+          <t>보일하이츠 리니지 물류창고 화재 수습 지연…파리 떼 극성과 악취로 주민 고통 심화</t>
+        </is>
+      </c>
+      <c r="E782" s="4" t="inlineStr">
+        <is>
+          <t>보일하이츠 지역의 리니지 로지스틱스 물류창고 화재 수습이 지연되면서 악취와 파리 떼로 인근 주민들이 고통받고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F782" s="4" t="inlineStr">
+        <is>
+          <t>특정 지역 물류창고 화재 소식으로, 우리 회사의 물류 운영에 직접적인 영향은 없으나 창고 안전 관리의 중요성을 상기시킵니다.</t>
+        </is>
+      </c>
+      <c r="G782" s="4" t="n"/>
+      <c r="H782" s="4" t="inlineStr">
+        <is>
+          <t>Radio Seoul</t>
+        </is>
+      </c>
+      <c r="I782" s="4" t="inlineStr">
+        <is>
+          <t>https://radioseoul1650.com/archives/146958</t>
+        </is>
+      </c>
+      <c r="J782" s="4" t="inlineStr"/>
+    </row>
+    <row r="783">
+      <c r="A783" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B783" s="4" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C783" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D783" s="4" t="inlineStr">
+        <is>
+          <t>[영상] 파주 전자제품 창고서 '화재'…건물 4개 동 번져 '대응 1단계'</t>
+        </is>
+      </c>
+      <c r="E783" s="4" t="inlineStr">
+        <is>
+          <t>경기 파주시 전자제품 창고에서 화재가 발생하여 건물 4개 동으로 번졌으며, 인명 피해는 없는 것으로 확인되었습니다.</t>
+        </is>
+      </c>
+      <c r="F783" s="4" t="inlineStr">
+        <is>
+          <t>국내 특정 지역 전자제품 창고 화재 소식으로, 우리 회사의 물류 운영에 직접적인 영향은 없으나 창고 안전 관리의 중요성을 상기시킵니다.</t>
+        </is>
+      </c>
+      <c r="G783" s="4" t="n"/>
+      <c r="H783" s="4" t="inlineStr">
+        <is>
+          <t>뉴스1</t>
+        </is>
+      </c>
+      <c r="I783" s="4" t="inlineStr">
+        <is>
+          <t>https://www.news1.kr/local/gyeonggi/6226913</t>
+        </is>
+      </c>
+      <c r="J783" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -35766,7 +37494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -36501,6 +38229,35 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n"/>
+      <c r="C18" s="5" t="inlineStr"/>
+      <c r="D18" s="5" t="inlineStr"/>
+      <c r="E18" s="5" t="inlineStr"/>
+      <c r="F18" s="5" t="n">
+        <v>4318</v>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>-12 (-0.3%)</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>+1,728 (+66.7%)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -36513,7 +38270,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I132"/>
+  <dimension ref="A1:I138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -41159,6 +42916,216 @@
       </c>
       <c r="I132" s="6" t="inlineStr"/>
     </row>
+    <row r="133">
+      <c r="A133" s="6" t="inlineStr">
+        <is>
+          <t>RSK-132</t>
+        </is>
+      </c>
+      <c r="B133" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C133" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D133" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E133" s="6" t="inlineStr">
+        <is>
+          <t>[26.07.03] 글로벌 공급망 인사이트 175호</t>
+        </is>
+      </c>
+      <c r="F133" s="6" t="inlineStr"/>
+      <c r="G133" s="6" t="inlineStr"/>
+      <c r="H133" s="6" t="inlineStr">
+        <is>
+          <t>코발트, 인듐, 갈륨 등 핵심 원자재의 공급망 다변화 및 재고 확보 방안 검토, 관련 규제 변화 모니터링 강화.</t>
+        </is>
+      </c>
+      <c r="I133" s="6" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="6" t="inlineStr">
+        <is>
+          <t>RSK-133</t>
+        </is>
+      </c>
+      <c r="B134" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C134" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D134" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E134" s="6" t="inlineStr">
+        <is>
+          <t>이란의 VLCC 연쇄 공격에 원유시장 '원점 회귀'</t>
+        </is>
+      </c>
+      <c r="F134" s="6" t="inlineStr"/>
+      <c r="G134" s="6" t="inlineStr"/>
+      <c r="H134" s="6" t="inlineStr">
+        <is>
+          <t>유가 변동 추이 면밀히 모니터링, 해상 운송 보험 조건 및 중동 항로 이용 시 대체 경로 또는 운송 방식 검토.</t>
+        </is>
+      </c>
+      <c r="I134" s="6" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="6" t="inlineStr">
+        <is>
+          <t>RSK-134</t>
+        </is>
+      </c>
+      <c r="B135" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C135" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D135" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E135" s="6" t="inlineStr">
+        <is>
+          <t>미-이란, 호르무즈 통제권 놓고 또 충돌…오만, 남북 2개 항로 제안</t>
+        </is>
+      </c>
+      <c r="F135" s="6" t="inlineStr"/>
+      <c r="G135" s="6" t="inlineStr"/>
+      <c r="H135" s="6" t="inlineStr">
+        <is>
+          <t>중동 지역 정세 변화를 실시간으로 모니터링하고, 주요 항로의 대체 경로 및 비상 운송 계획을 수립하며, 포워더와 긴밀히 소통하여 선박 스케줄 변경 가능성에 대비한다.</t>
+        </is>
+      </c>
+      <c r="I135" s="6" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="6" t="inlineStr">
+        <is>
+          <t>RSK-135</t>
+        </is>
+      </c>
+      <c r="B136" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C136" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D136" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E136" s="6" t="inlineStr">
+        <is>
+          <t>트럼프 '호르무즈 통행료' 하루 만에 철회…해협 불확실성은 여전</t>
+        </is>
+      </c>
+      <c r="F136" s="6" t="inlineStr"/>
+      <c r="G136" s="6" t="inlineStr"/>
+      <c r="H136" s="6" t="inlineStr">
+        <is>
+          <t>중동 지역의 정치적 발언 및 정책 변화를 면밀히 주시하고, 운송 계약 시 지정학적 리스크 관련 조항을 검토하며, 비상시 대체 운송 방안을 재점검한다.</t>
+        </is>
+      </c>
+      <c r="I136" s="6" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="6" t="inlineStr">
+        <is>
+          <t>RSK-136</t>
+        </is>
+      </c>
+      <c r="B137" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C137" s="6" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="D137" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E137" s="6" t="inlineStr">
+        <is>
+          <t>[테크 차이나] 中 전기차 배터리 안전기준 대폭 강화…산업 재편 본격화</t>
+        </is>
+      </c>
+      <c r="F137" s="6" t="inlineStr"/>
+      <c r="G137" s="6" t="inlineStr"/>
+      <c r="H137" s="6" t="inlineStr">
+        <is>
+          <t>중국 수출 제품의 배터리 안전 기준(GB 38031-2025) 준수 여부 즉시 확인 및 필요 시 제품/포장/운송 방식 변경 검토.</t>
+        </is>
+      </c>
+      <c r="I137" s="6" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="6" t="inlineStr">
+        <is>
+          <t>RSK-137</t>
+        </is>
+      </c>
+      <c r="B138" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C138" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D138" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E138" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈 충돌에 국제유가 80달러 육박…정부 “7~8월 물량 차질 없어”</t>
+        </is>
+      </c>
+      <c r="F138" s="6" t="inlineStr"/>
+      <c r="G138" s="6" t="inlineStr"/>
+      <c r="H138" s="6" t="inlineStr">
+        <is>
+          <t>국제유가 및 중동 정세 변화를 실시간으로 모니터링하고, 유류할증료 변동에 따른 물류 예산 재검토 및 운송 계약의 유류할증료 조항을 확인한다.</t>
+        </is>
+      </c>
+      <c r="I138" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
📰 뉴스 데이터 2026-07-16_08:59
</commit_message>
<xml_diff>
--- a/data/SCM_물류_브리핑.xlsx
+++ b/data/SCM_물류_브리핑.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J783"/>
+  <dimension ref="A1:J826"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -37482,6 +37482,2050 @@
       </c>
       <c r="J783" s="4" t="inlineStr"/>
     </row>
+    <row r="784">
+      <c r="A784" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B784" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C784" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D784" s="2" t="inlineStr">
+        <is>
+          <t>DOJ Appeals CIT's IEEPA Refund Injunction as CAPE Phase 2 Targets June 29; TPEB Rates Surge 30% Into Peak</t>
+        </is>
+      </c>
+      <c r="E784" s="2" t="inlineStr">
+        <is>
+          <t>법무부가 IEEPA 환급 금지 명령에 항소했으며, TPEB(Trans-Pacific Eastbound) 운임이 성수기를 맞아 30% 급등했다.</t>
+        </is>
+      </c>
+      <c r="F784" s="2" t="inlineStr">
+        <is>
+          <t>TPEB 운임의 30% 급등은 북미향 물류 비용에 즉각적이고 심각한 영향을 미치며, IEEPA 환급 관련 법적 분쟁은 관세 비용에 대한 불확실성을 높인다.</t>
+        </is>
+      </c>
+      <c r="G784" s="2" t="inlineStr">
+        <is>
+          <t>TPEB 운임 급등에 대한 즉각적인 비용 절감 방안(예: 선적 계획 조정, 운송사 협상)을 모색하고, IEEPA 환급 관련 소송 진행 상황을 면밀히 주시하여 잠재적 관세 비용 영향을 평가한다.</t>
+        </is>
+      </c>
+      <c r="H784" s="2" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I784" s="2" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/june-11-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J784" s="2" t="inlineStr">
+        <is>
+          <t>RSK-138</t>
+        </is>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B785" s="2" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C785" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D785" s="2" t="inlineStr">
+        <is>
+          <t>CPSC Mandatory eFiling Takes Effect July 8; TPEB Rates Surge ~10% as Peak Season Demand Outpaces Capacity</t>
+        </is>
+      </c>
+      <c r="E785" s="2" t="inlineStr">
+        <is>
+          <t>CPSC의 의무 전자 신고가 7월 8일 발효되고, CBP는 강제 노동 관련 지침을 발표하여 미국 수출 제품의 규제 준수 부담이 증가했다.</t>
+        </is>
+      </c>
+      <c r="F785" s="2" t="inlineStr">
+        <is>
+          <t>CPSC 전자 신고 의무는 미국 수출 제품의 통관 절차에 직접 영향을 미치며, CBP의 강제 노동 지침은 공급망 실사 및 규제 준수 리스크를 높인다.</t>
+        </is>
+      </c>
+      <c r="G785" s="2" t="inlineStr">
+        <is>
+          <t>CPSC 전자 신고 의무 사항을 즉시 확인하고 관련 시스템 및 절차를 준비하며, CBP의 강제 노동 지침에 따라 공급망 내 강제 노동 리스크를 재평가하고 필요한 조치를 취한다.</t>
+        </is>
+      </c>
+      <c r="H785" s="2" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I785" s="2" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/june-18-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J785" s="2" t="inlineStr">
+        <is>
+          <t>RSK-139</t>
+        </is>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B786" s="2" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C786" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D786" s="2" t="inlineStr">
+        <is>
+          <t>CBP Rejects Warehouse Entries on CAPE Declarations, Risking IEEPA Refunds; TPEB Rates Climb as Panama Canal Restrictions Tighten Capacity</t>
+        </is>
+      </c>
+      <c r="E786" s="2" t="inlineStr">
+        <is>
+          <t>CBP가 CAPE 선언에 대한 창고 입고를 거부하여 IEEPA 환급 위험이 있으며, 파나마 운하 제한으로 아시아-미국 동부 해상 운송에 지연이 예상된다.</t>
+        </is>
+      </c>
+      <c r="F786" s="2" t="inlineStr">
+        <is>
+          <t>파나마 운하의 운송량 제한은 아시아-미국 동부 해상 운송에 직접적인 지연 및 운임 상승을 유발하며, CBP의 CAPE 관련 조치는 관세 환급에 영향을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="G786" s="2" t="inlineStr">
+        <is>
+          <t>파나마 운하를 이용하는 운송 경로의 지연 및 운임 상승에 대비하여 대체 경로(예: 수에즈 운하, 미 서안 육상 운송)를 검토하고, IEEPA 환급 관련 CBP 지침을 확인하여 관세 비용 영향을 최소화한다.</t>
+        </is>
+      </c>
+      <c r="H786" s="2" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I786" s="2" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/july-09-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J786" s="2" t="inlineStr">
+        <is>
+          <t>RSK-140</t>
+        </is>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B787" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C787" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D787" s="2" t="inlineStr">
+        <is>
+          <t>유가 150달러 경고! 세계 경제 뒤흔들 최악의 시나리오</t>
+        </is>
+      </c>
+      <c r="E787" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 긴장 등으로 국제유가가 급등할 수 있다는 경고가 나왔으나, 대체 운송로 확보 및 수요 둔화로 안정될 가능성도 제기됩니다.</t>
+        </is>
+      </c>
+      <c r="F787" s="2" t="inlineStr">
+        <is>
+          <t>유가 급등은 해상 및 항공 운임 상승으로 직결되어 물류비에 즉각적인 영향을 미치며, 생산 원가에도 부담을 줄 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G787" s="2" t="inlineStr">
+        <is>
+          <t>유가 및 운임 변동 추이를 면밀히 모니터링하고, 운송 계약 시 유가 연동 조항 검토 및 장기 계약을 통한 리스크 헤지 방안을 모색합니다.</t>
+        </is>
+      </c>
+      <c r="H787" s="2" t="inlineStr">
+        <is>
+          <t>Surff</t>
+        </is>
+      </c>
+      <c r="I787" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260713-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J787" s="2" t="inlineStr">
+        <is>
+          <t>RSK-141</t>
+        </is>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B788" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C788" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D788" s="2" t="inlineStr">
+        <is>
+          <t>미-이란, 호르무즈 통제권 놓고 또 충돌…오만, 남북 2개 항로 제안</t>
+        </is>
+      </c>
+      <c r="E788" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 통제권을 둘러싼 미-이란 갈등이 재점화되었으며, 오만이 대체 항로를 제안하는 등 긴장이 고조되고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F788" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협은 주요 원유 및 가스 수송로이자 글로벌 해운의 핵심 길목으로, 봉쇄 시 운송 지연, 운임 급등, 에너지 공급망 교란 등 직접적인 물류 대란을 초래할 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G788" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 상황을 실시간으로 모니터링하고, 비상시 대체 운송 경로 및 운송 수단(항공 등) 확보 계획을 수립하며, 주요 원자재 재고 수준을 점검합니다.</t>
+        </is>
+      </c>
+      <c r="H788" s="2" t="inlineStr">
+        <is>
+          <t>Surff</t>
+        </is>
+      </c>
+      <c r="I788" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260713-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J788" s="2" t="inlineStr">
+        <is>
+          <t>RSK-142</t>
+        </is>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B789" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C789" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D789" s="2" t="inlineStr">
+        <is>
+          <t>트럼프 '호르무즈 통행료' 하루 만에 철회…해협 불확실성은 여전</t>
+        </is>
+      </c>
+      <c r="E789" s="2" t="inlineStr">
+        <is>
+          <t>트럼프 전 대통령이 호르무즈 해협 통행료 부과 구상을 하루 만에 철회했으나, 해협을 둘러싼 불확실성은 여전히 남아있습니다.</t>
+        </is>
+      </c>
+      <c r="F789" s="2" t="inlineStr">
+        <is>
+          <t>통행료 부과 가능성은 철회되었으나, 호르무즈 해협의 지정학적 불안정성은 언제든 운송 지연 및 운임 상승을 유발할 수 있는 직접적인 리스크입니다.</t>
+        </is>
+      </c>
+      <c r="G789" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 관련 정치적 발언 및 동향을 예의주시하고, 비상시 운송 계획을 재점검합니다.</t>
+        </is>
+      </c>
+      <c r="H789" s="2" t="inlineStr">
+        <is>
+          <t>뉴스핌</t>
+        </is>
+      </c>
+      <c r="I789" s="2" t="inlineStr">
+        <is>
+          <t>https://www.newspim.com/news/view/20260715000027</t>
+        </is>
+      </c>
+      <c r="J789" s="2" t="inlineStr">
+        <is>
+          <t>RSK-143</t>
+        </is>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B790" s="2" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C790" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D790" s="2" t="inlineStr">
+        <is>
+          <t>상하이항 태풍으로 운영 중단, 수십 척 컨테이너선 입항 지연</t>
+        </is>
+      </c>
+      <c r="E790" s="2" t="inlineStr">
+        <is>
+          <t>태풍으로 인해 상하이항이 컨테이너 하역 작업을 전면 중단했으며, 수십  척의 컨테이너선 입항이 48시간 이상 지연되고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F790" s="2" t="inlineStr">
+        <is>
+          <t>상하이항은 주요 수출입 허브 항만으로, 운영 중단 및 선박 지연은 우리 회사의 아시아발/착 해상 운송 스케줄 및 리드타임에 직접적인 차질을 발생시킵니다.</t>
+        </is>
+      </c>
+      <c r="G790" s="2" t="inlineStr">
+        <is>
+          <t>상하이항을 경유하는 모든 선적의 현황을 즉시 파악하고, 지연 예상 물량에 대한 고객 및 생산 부서에 통보하며, 필요시 대체 항만 또는 항공 운송 전환을 검토합니다.</t>
+        </is>
+      </c>
+      <c r="H790" s="2" t="inlineStr">
+        <is>
+          <t>해양통신</t>
+        </is>
+      </c>
+      <c r="I790" s="2" t="inlineStr">
+        <is>
+          <t>https://oceanpress.co.kr/news/article.html?no=30614</t>
+        </is>
+      </c>
+      <c r="J790" s="2" t="inlineStr">
+        <is>
+          <t>RSK-144</t>
+        </is>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B791" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C791" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D791" s="3" t="inlineStr">
+        <is>
+          <t>LA港 118년 역사상 최대 물동량 기록</t>
+        </is>
+      </c>
+      <c r="E791" s="3" t="inlineStr">
+        <is>
+          <t>LA항이 6월 컨테이너 물동량 100만 TEU를 돌파하며 118년 역사상 최대치를 기록, 수입 컨테이너가 크게 증가했다.</t>
+        </is>
+      </c>
+      <c r="F791" s="3" t="inlineStr">
+        <is>
+          <t>LA항의 기록적인 물동량 증가는 항만 적체와 운송 지연으로 이어질 수 있어 북미향 물류에 잠재적 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G791" s="3" t="inlineStr">
+        <is>
+          <t>북미향 선적 스케줄 및 리드타임 변동 가능성을 지속 모니터링하고, 필요 시 대체 운송 방안을 검토한다.</t>
+        </is>
+      </c>
+      <c r="H791" s="3" t="inlineStr">
+        <is>
+          <t>cargonews</t>
+        </is>
+      </c>
+      <c r="I791" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cargonews.co.kr/news/articleView.html?idxno=60531</t>
+        </is>
+      </c>
+      <c r="J791" s="3" t="inlineStr"/>
+    </row>
+    <row r="792">
+      <c r="A792" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B792" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C792" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D792" s="3" t="inlineStr">
+        <is>
+          <t>U.S.-EU Trade Agreement Eliminates Duties on Most U.S. Goods Starting July 1; TPEB Rates Rise as July Capacity Hits Three-Year High</t>
+        </is>
+      </c>
+      <c r="E792" s="3" t="inlineStr">
+        <is>
+          <t>미국-EU 무역 협정이 7월 1일부터 대부분의 미국산 제품에 대한 관세를 철폐하여 글로벌 무역 환경에 변화가 예상된다.</t>
+        </is>
+      </c>
+      <c r="F792" s="3" t="inlineStr">
+        <is>
+          <t>미국-EU 무역 협정은 우리 회사에 직접적인 관세 영향을 주지는 않지만, 글로벌 무역 흐름 및 경쟁 환경에 장기적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G792" s="3" t="inlineStr">
+        <is>
+          <t>미국-EU 무역 협정이 글로벌 공급망 및 경쟁 환경에 미칠 장기적인 영향을 모니터링하고, 잠재적 기회 또는 위협 요소를 분석한다.</t>
+        </is>
+      </c>
+      <c r="H792" s="3" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I792" s="3" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/july-02-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J792" s="3" t="inlineStr"/>
+    </row>
+    <row r="793">
+      <c r="A793" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B793" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C793" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D793" s="3" t="inlineStr">
+        <is>
+          <t>Air Cargo Demand Up 6.0% in May</t>
+        </is>
+      </c>
+      <c r="E793" s="3" t="inlineStr">
+        <is>
+          <t>IATA에 따르면 2026년 5월 전 세계 항공 화물 수요가 전년 동기 대비 6.0% 증가했다.</t>
+        </is>
+      </c>
+      <c r="F793" s="3" t="inlineStr">
+        <is>
+          <t>항공 화물 수요 증가는 항공 운임 상승 압력으로 작용할 수 있으며, 이는 긴급 운송 또는 고가 제품 운송 비용에 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G793" s="3" t="inlineStr">
+        <is>
+          <t>항공 화물 운임 추이를 지속적으로 모니터링하고, 필요 시 항공 운송 계약 조건 재검토 및 대체 운송 수단(해상)과의 비용 효율성을 비교 검토한다.</t>
+        </is>
+      </c>
+      <c r="H793" s="3" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I793" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-29-air-cargo-demand-up-may/</t>
+        </is>
+      </c>
+      <c r="J793" s="3" t="inlineStr"/>
+    </row>
+    <row r="794">
+      <c r="A794" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B794" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C794" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D794" s="3" t="inlineStr">
+        <is>
+          <t>Urgent Action Needed to Ease Engine MRO Bottlenecks</t>
+        </is>
+      </c>
+      <c r="E794" s="3" t="inlineStr">
+        <is>
+          <t>IATA가 항공기 엔진 유지보수(MRO) 병목 현상 완화를 위한 긴급 조치를 촉구했다.</t>
+        </is>
+      </c>
+      <c r="F794" s="3" t="inlineStr">
+        <is>
+          <t>항공기 엔진 MRO 병목 현상은 장기적으로 항공기 가동률에 영향을 주어 항공 화물 운송 능력에 간접적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G794" s="3" t="inlineStr">
+        <is>
+          <t>항공기 가동률 및 항공 화물 운송 능력에 미칠 잠재적 영향을 장기적으로 모니터링하고, 항공 운송 시장의 공급 측면 변화를 주시한다.</t>
+        </is>
+      </c>
+      <c r="H794" s="3" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I794" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-24-urgent-action-needed-to-ease-engine-mro-bottlenecks/</t>
+        </is>
+      </c>
+      <c r="J794" s="3" t="inlineStr"/>
+    </row>
+    <row r="795">
+      <c r="A795" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B795" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C795" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D795" s="3" t="inlineStr">
+        <is>
+          <t>Structural Contraction of Global Liner Networks</t>
+        </is>
+      </c>
+      <c r="E795" s="3" t="inlineStr">
+        <is>
+          <t>IMF의 세계 경제 전망 보고서에 따르면 2026년 글로벌 무역량 성장률이 3.5%로 둔화될 것으로 예상되며, 이는 글로벌 정기선 네트워크의 구조적 축소로 이어질 수 있다.</t>
+        </is>
+      </c>
+      <c r="F795" s="3" t="inlineStr">
+        <is>
+          <t>글로벌 무역량 성장 둔화와 정기선 네트워크 축소는 장기적으로 해상 운송 서비스의 가용성 및 운임에 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G795" s="3" t="inlineStr">
+        <is>
+          <t>글로벌 무역 동향 및 해상 운송 시장의 구조적 변화를 지속적으로 모니터링하고, 장기적인 운송 전략 수립 시 이를 반영한다.</t>
+        </is>
+      </c>
+      <c r="H795" s="3" t="inlineStr">
+        <is>
+          <t>sea-intelligence</t>
+        </is>
+      </c>
+      <c r="I795" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/398-structural-contraction-of-global-liner-network</t>
+        </is>
+      </c>
+      <c r="J795" s="3" t="inlineStr"/>
+    </row>
+    <row r="796">
+      <c r="A796" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B796" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C796" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D796" s="3" t="inlineStr">
+        <is>
+          <t>Structural Contraction of Global Liner Networks</t>
+        </is>
+      </c>
+      <c r="E796" s="3" t="inlineStr">
+        <is>
+          <t>2012년 이후 글로벌 선사 네트워크가 구조적으로 축소되고 있으며, 지리적 범위는 유지되나 서비스 빈도가 감소하는 추세입니다.</t>
+        </is>
+      </c>
+      <c r="F796" s="3" t="inlineStr">
+        <is>
+          <t>선사 네트워크 축소 및 서비스 빈도 감소는 장기적으로 특정 노선의 운송 용량 및 스케줄 신뢰성에 영향을 미칠 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G796" s="3" t="inlineStr">
+        <is>
+          <t>주요 노선의 선사 서비스 빈도 변화를 지속적으로 모니터링하고, 필요시 대체 운송 옵션을 검토합니다.</t>
+        </is>
+      </c>
+      <c r="H796" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I796" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/397-structural-contraction-of-global-liner-networks</t>
+        </is>
+      </c>
+      <c r="J796" s="3" t="inlineStr"/>
+    </row>
+    <row r="797">
+      <c r="A797" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B797" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C797" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D797" s="3" t="inlineStr">
+        <is>
+          <t>PLSCI Data Indicates Mega-Hub Retrenchment</t>
+        </is>
+      </c>
+      <c r="E797" s="3" t="inlineStr">
+        <is>
+          <t>UNCTAD의 PLSCI 데이터에 따르면, 최근 선사 네트워크 재조정으로 메가 허브 항만의 연결성이 축소되는 경향을 보입니다.</t>
+        </is>
+      </c>
+      <c r="F797" s="3" t="inlineStr">
+        <is>
+          <t>주요 허브 항만의 연결성 축소는 환적 효율성 저하 및 운송 시간 증가로 이어질 수 있어 장기적인 물류 계획에 영향을 줄 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G797" s="3" t="inlineStr">
+        <is>
+          <t>주요 수출입 항만의 PLSCI 지수 변화를 주시하고, 허브 항만 의존도를 재평가하여 다변화 전략을 고려합니다.</t>
+        </is>
+      </c>
+      <c r="H797" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I797" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/396-plsci-data-indicates-mega-hub-retrenchment</t>
+        </is>
+      </c>
+      <c r="J797" s="3" t="inlineStr"/>
+    </row>
+    <row r="798">
+      <c r="A798" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B798" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C798" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D798" s="3" t="inlineStr">
+        <is>
+          <t>Tracking True Vessel Delay</t>
+        </is>
+      </c>
+      <c r="E798" s="3" t="inlineStr">
+        <is>
+          <t>선사들이 운송 시간을 늘리는 '스케줄 버퍼링'을 통해 실제 선박 지연을 관리하고 있으며, 이는 조기 도착 선박 증가로 이어지고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F798" s="3" t="inlineStr">
+        <is>
+          <t>스케줄 버퍼링은 겉보기에는 정시성을 높이지만, 실제 운송 시간 증가를 의미하므로 리드타임 예측 및 재고 관리에 영향을 줄 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G798" s="3" t="inlineStr">
+        <is>
+          <t>선사별 실제 운송 리드타임 데이터를 면밀히 분석하여 물류 계획에 반영하고, 운송 계약 시 리드타임 조건을 명확히 합니다.</t>
+        </is>
+      </c>
+      <c r="H798" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I798" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/394-tracking-true-vessel-delay</t>
+        </is>
+      </c>
+      <c r="J798" s="3" t="inlineStr"/>
+    </row>
+    <row r="799">
+      <c r="A799" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B799" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C799" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D799" s="3" t="inlineStr">
+        <is>
+          <t>HMM 주가 힘 못 받는 이유</t>
+        </is>
+      </c>
+      <c r="E799" s="3" t="inlineStr">
+        <is>
+          <t>해상 운임 흐름이 우호적이지 않아 대규모 투자에도 불구하고 HMM 주가가 탄력을 받기 어렵다는 분석이 나왔습니다.</t>
+        </is>
+      </c>
+      <c r="F799" s="3" t="inlineStr">
+        <is>
+          <t>해상 운임 시장의 약세는 단기적으로 운송비 절감 기회가 될 수 있으나, 장기적으로 선사들의 서비스 축소로 이어질 가능성도 있습니다.</t>
+        </is>
+      </c>
+      <c r="G799" s="3" t="inlineStr">
+        <is>
+          <t>해상 운임 지수를 지속적으로 모니터링하고, 운임 계약 시 시장 상황을 반영한 협상 전략을 수립합니다.</t>
+        </is>
+      </c>
+      <c r="H799" s="3" t="inlineStr">
+        <is>
+          <t>Surff</t>
+        </is>
+      </c>
+      <c r="I799" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260716-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J799" s="3" t="inlineStr"/>
+    </row>
+    <row r="800">
+      <c r="A800" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B800" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C800" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D800" s="3" t="inlineStr">
+        <is>
+          <t>"비싸도 지금 산다"...호르무즈 장기화에 VLCC 발주 사상 최대</t>
+        </is>
+      </c>
+      <c r="E800" s="3" t="inlineStr">
+        <is>
+          <t>중동 사태 장기화로 호르무즈 해협 불확실성이 커지면서 글로벌 선주들이 초대형 원유운반선(VLCC) 확보에 속도를 내고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F800" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 리스크에 대한 선주들의 대응은 장기적으로 해운 시장의 선박 공급 및 운임 구조에 영향을 미칠 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G800" s="3" t="inlineStr">
+        <is>
+          <t>중동 정세 변화에 따른 해운 시장의 구조적 변화 가능성을 지속적으로 모니터링합니다.</t>
+        </is>
+      </c>
+      <c r="H800" s="3" t="inlineStr">
+        <is>
+          <t>이비엔(EBN)뉴스센터</t>
+        </is>
+      </c>
+      <c r="I800" s="3" t="inlineStr">
+        <is>
+          <t>https://ebn.co.kr/news/articleView.html?idxno=1716474</t>
+        </is>
+      </c>
+      <c r="J800" s="3" t="inlineStr"/>
+    </row>
+    <row r="801">
+      <c r="A801" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B801" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C801" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D801" s="3" t="inlineStr">
+        <is>
+          <t>美재무부, 이란 해운 거물 샴카니 겨냥 추가 제재</t>
+        </is>
+      </c>
+      <c r="E801" s="3" t="inlineStr">
+        <is>
+          <t>미국 재무부가 이란의 해운 거물을 겨냥해 추가 제재를 단행하여 이란 해운 부문에 대한 압박을 강화했습니다.</t>
+        </is>
+      </c>
+      <c r="F801" s="3" t="inlineStr">
+        <is>
+          <t>이란 해운 부문에 대한 제재 강화는 중동 지역의 해운 활동에 간접적인 영향을 미칠 수 있으며, 향후 제재 범위 확대 시 물류 운영에 영향을 줄 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G801" s="3" t="inlineStr">
+        <is>
+          <t>중동 지역 관련 제재 동향을 지속적으로 모니터링하고, 해당 지역을 경유하는 운송에 대한 잠재적 리스크를 평가합니다.</t>
+        </is>
+      </c>
+      <c r="H801" s="3" t="inlineStr">
+        <is>
+          <t>연합뉴스</t>
+        </is>
+      </c>
+      <c r="I801" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20260715009800071</t>
+        </is>
+      </c>
+      <c r="J801" s="3" t="inlineStr"/>
+    </row>
+    <row r="802">
+      <c r="A802" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B802" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C802" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D802" s="3" t="inlineStr">
+        <is>
+          <t>"두바이, 호르무즈 우회 동해안 신항만 건설 추진"</t>
+        </is>
+      </c>
+      <c r="E802" s="3" t="inlineStr">
+        <is>
+          <t>두바이가 호르무즈 해협 의존도를 낮추기 위해 UAE 동해안에 신항만과 컨테이너 터미널 건설을 추진하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F802" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 리스크에 대한 장기적인 대응책으로, 새로운 항만 개발은 미래 중동 지역 물류 흐름에 변화를 가져올 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G802" s="3" t="inlineStr">
+        <is>
+          <t>중동 지역의 신규 항만 개발 동향을 주시하고, 장기적인 공급망 다변화 전략 수립 시 해당 정보를 참고합니다.</t>
+        </is>
+      </c>
+      <c r="H802" s="3" t="inlineStr">
+        <is>
+          <t>뉴스핌</t>
+        </is>
+      </c>
+      <c r="I802" s="3" t="inlineStr">
+        <is>
+          <t>https://www.newspim.com/news/view/20260714000218</t>
+        </is>
+      </c>
+      <c r="J802" s="3" t="inlineStr"/>
+    </row>
+    <row r="803">
+      <c r="A803" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B803" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C803" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D803" s="3" t="inlineStr">
+        <is>
+          <t>UAE, 호르무즈 우회 신규 항만·터미널 건설 추진</t>
+        </is>
+      </c>
+      <c r="E803" s="3" t="inlineStr">
+        <is>
+          <t>UAE가 중동 지역의 지정학적 위기에 대응하여 호르무즈 해협을 우회할 수 있는 신규 항만 및 컨테이너 터미널 건설을 추진 중이며, 이는 해상 운송 경로의 안정성 확보를 위한 장기적인 인프라 투자이다.</t>
+        </is>
+      </c>
+      <c r="F803" s="3" t="inlineStr">
+        <is>
+          <t>중동 지역의 지정학적 리스크로 인한 해상 운송 지연 가능성에 대비하는 장기적인 인프라 투자로, 당장 직접적인 영향은 없으나 향후 운송 경로 다변화에 기여할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G803" s="3" t="inlineStr">
+        <is>
+          <t>중동 지역 해상 운송 경로의 지정학적 리스크 변화 및 신규 항만 건설 진행 상황을 지속적으로 모니터링하고, 필요시 대체 운송 경로 확보 방안을 검토한다.</t>
+        </is>
+      </c>
+      <c r="H803" s="3" t="inlineStr">
+        <is>
+          <t>아시아투데이</t>
+        </is>
+      </c>
+      <c r="I803" s="3" t="inlineStr">
+        <is>
+          <t>https://www.asiatoday.co.kr/kn/view.php?key=20260714010005326</t>
+        </is>
+      </c>
+      <c r="J803" s="3" t="inlineStr"/>
+    </row>
+    <row r="804">
+      <c r="A804" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B804" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C804" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D804" s="3" t="inlineStr">
+        <is>
+          <t>Warehouse Capacity Squeeze Tightens as Tariffs Loom</t>
+        </is>
+      </c>
+      <c r="E804" s="3" t="inlineStr">
+        <is>
+          <t>소매업체들이 새로운 관세 부과에 앞서 재고를 미리 확보하려 하면서 창고 용량이 부족해지고 있으며, 이는 화주들에게 창고 네트워크 준비의 중요성을 시사한다.</t>
+        </is>
+      </c>
+      <c r="F804" s="3" t="inlineStr">
+        <is>
+          <t>관세 부과에 대한 선제적 재고 확보 움직임으로 창고 용량 부족 현상이 심화될 수 있으며, 이는 우리 회사의 재고 보관 및 유통 전략에 간접적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G804" s="3" t="inlineStr">
+        <is>
+          <t>주요 시장의 창고 가용성 및 비용 추이를 모니터링하고, 필요시 재고 전략 및 창고 네트워크 운영 효율화 방안을 검토한다.</t>
+        </is>
+      </c>
+      <c r="H804" s="3" t="inlineStr">
+        <is>
+          <t>Inbound Logistics</t>
+        </is>
+      </c>
+      <c r="I804" s="3" t="inlineStr">
+        <is>
+          <t>https://inboundlogistics.com/articles/retailers-are-racing-to-beat-tariffs-is-your-warehouse-network-ready</t>
+        </is>
+      </c>
+      <c r="J804" s="3" t="inlineStr"/>
+    </row>
+    <row r="805">
+      <c r="A805" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B805" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C805" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D805" s="3" t="inlineStr">
+        <is>
+          <t>유용 폐자원의 위장수출 막고 순환자원 수입 문턱 낮춘다</t>
+        </is>
+      </c>
+      <c r="E805" s="3" t="inlineStr">
+        <is>
+          <t>기후에너지환경부가 국내 핵심광물 공급망 안정화 및 유용 폐자원 국내 순환 이용 촉진을 위해 폐기물 수출입 관리 고시 개정을 추진한다.</t>
+        </is>
+      </c>
+      <c r="F805" s="3" t="inlineStr">
+        <is>
+          <t>폐기물 수출입 관리 고시 개정은 배터리 재활용 및 핵심 광물 공급망과 연관될 수 있어, 향후 우리 회사의 원자재 조달 및 폐배터리 처리 전략에 영향을 미칠 가능성이 있다.</t>
+        </is>
+      </c>
+      <c r="G805" s="3" t="inlineStr">
+        <is>
+          <t>폐기물 수출입 관리 고시 개정안의 구체적인 내용을 확인하고, 폐배터리 재활용 및 핵심 광물 공급망에 미칠 영향을 분석하여 대응 방안을 마련한다.</t>
+        </is>
+      </c>
+      <c r="H805" s="3" t="inlineStr">
+        <is>
+          <t>세계환경신문</t>
+        </is>
+      </c>
+      <c r="I805" s="3" t="inlineStr">
+        <is>
+          <t>https://e-newsp.com/news/article.html?no=89561</t>
+        </is>
+      </c>
+      <c r="J805" s="3" t="inlineStr"/>
+    </row>
+    <row r="806">
+      <c r="A806" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B806" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C806" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D806" s="3" t="inlineStr">
+        <is>
+          <t>관세청, 위해물품 불법 반입 차단 강화...5851개 품목 관리</t>
+        </is>
+      </c>
+      <c r="E806" s="3" t="inlineStr">
+        <is>
+          <t>관세청이 국민 건강 및 산업 안전을 위협하는 위해물품의 불법 반입을 막기 위해 통관 단계에서 5851개 품목에 대한 요건 확인을 강화한다.</t>
+        </is>
+      </c>
+      <c r="F806" s="3" t="inlineStr">
+        <is>
+          <t>배터리/전자부품 제조 과정에서 사용되거나 생산되는 특정 물질이 위해물품으로 분류될 경우 통관 절차가 복잡해지거나 지연될 수 있어 지속적인 확인이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G806" s="3" t="inlineStr">
+        <is>
+          <t>우리 회사 제품 또는 원자재 중 해당 품목에 포함될 가능성이 있는 물질이 있는지 확인하고, 관련 규제 변화를 지속적으로 모니터링하여 통관 지연을 예방해야 한다.</t>
+        </is>
+      </c>
+      <c r="H806" s="3" t="inlineStr">
+        <is>
+          <t>뉴스핌</t>
+        </is>
+      </c>
+      <c r="I806" s="3" t="inlineStr">
+        <is>
+          <t>https://newspim.com/news/view/20260715001262</t>
+        </is>
+      </c>
+      <c r="J806" s="3" t="inlineStr"/>
+    </row>
+    <row r="807">
+      <c r="A807" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B807" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C807" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D807" s="3" t="inlineStr">
+        <is>
+          <t>대형 화학물질 화재사고 대비 비상대응체계 강화한다</t>
+        </is>
+      </c>
+      <c r="E807" s="3" t="inlineStr">
+        <is>
+          <t>화학물질안전원이 대형 화학물질 화재사고에 효과적으로 대비하기 위해 화학사고예방관리계획서 상의 비상대응계획을 강화한다.</t>
+        </is>
+      </c>
+      <c r="F807" s="3" t="inlineStr">
+        <is>
+          <t>배터리/전자부품 제조 과정에서 위험 화학물질을 취급할 가능성이 높으므로, 관련 비상대응체계 강화는 우리 회사의 안전 관리 및 물류 창고 운영에 잠재적 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G807" s="3" t="inlineStr">
+        <is>
+          <t>우리 회사의 화학물질 취급 및 보관 관련 안전 규정 및 비상대응계획을 점검하고, 강화되는 정부 지침에 맞춰 업데이트할 필요가 있는지 검토한다.</t>
+        </is>
+      </c>
+      <c r="H807" s="3" t="inlineStr">
+        <is>
+          <t>헤럴드경제</t>
+        </is>
+      </c>
+      <c r="I807" s="3" t="inlineStr">
+        <is>
+          <t>https://biz.heraldcorp.com/article/10810366</t>
+        </is>
+      </c>
+      <c r="J807" s="3" t="inlineStr"/>
+    </row>
+    <row r="808">
+      <c r="A808" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B808" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C808" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D808" s="3" t="inlineStr">
+        <is>
+          <t>美 상원, 中·印 등 러산 원유 수입국에 최대 100% 관세 추진...500%에서 ↓</t>
+        </is>
+      </c>
+      <c r="E808" s="3" t="inlineStr">
+        <is>
+          <t>미국 상원이 러시아산 원유 수입국인 중국과 인도 등에 최대 100%의 관세를 부과하는 대러 제재 방안을 추진 중이며, 이는 당초 500%에서 완화된 수준이다.</t>
+        </is>
+      </c>
+      <c r="F808" s="3" t="inlineStr">
+        <is>
+          <t>국제 유가 변동에 영향을 미쳐 물류비 상승으로 이어질 수 있으며, 주요 교역국인 중국과의 관계에도 간접적인 영향을 미칠 수 있어 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G808" s="3" t="inlineStr">
+        <is>
+          <t>국제 유가 및 해상/항공 운임 변동 추이를 지속적으로 모니터링하고, 필요시 물류비용 예측 및 예산 계획에 반영한다.</t>
+        </is>
+      </c>
+      <c r="H808" s="3" t="inlineStr">
+        <is>
+          <t>뉴스핌</t>
+        </is>
+      </c>
+      <c r="I808" s="3" t="inlineStr">
+        <is>
+          <t>https://newspim.com/news/view/20260715000838</t>
+        </is>
+      </c>
+      <c r="J808" s="3" t="inlineStr"/>
+    </row>
+    <row r="809">
+      <c r="A809" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B809" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C809" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D809" s="3" t="inlineStr">
+        <is>
+          <t>[유럽 특징주] ASML, 생산능력 확대와 중국 수출 제한 과제 주목</t>
+        </is>
+      </c>
+      <c r="E809" s="3" t="inlineStr">
+        <is>
+          <t>ASML이 생산능력 확대와 함께 중국 수출 제한이라는 과제에 직면해 있으며, 이는 반도체 산업 전반의 공급망에 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="F809" s="3" t="inlineStr">
+        <is>
+          <t>반도체 장비 공급망의 불안정성은 전자부품 생산에 영향을 미칠 수 있으며, 이는 우리 회사의 생산 계획 및 원자재 수급에 간접적인 영향을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="G809" s="3" t="inlineStr">
+        <is>
+          <t>반도체 산업 공급망 동향을 지속적으로 모니터링하고, 우리 회사 제품에 사용되는 전자부품의 수급 안정성을 주기적으로 점검한다.</t>
+        </is>
+      </c>
+      <c r="H809" s="3" t="inlineStr">
+        <is>
+          <t>뉴스핌</t>
+        </is>
+      </c>
+      <c r="I809" s="3" t="inlineStr">
+        <is>
+          <t>https://www.newspim.com/news/view/20260715000016</t>
+        </is>
+      </c>
+      <c r="J809" s="3" t="inlineStr"/>
+    </row>
+    <row r="810">
+      <c r="A810" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B810" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C810" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D810" s="3" t="inlineStr">
+        <is>
+          <t>[하반기 성장전략] 중동전 교훈에 공급망 4단계 정비…5대업종 탈탄소 전환 시동</t>
+        </is>
+      </c>
+      <c r="E810" s="3" t="inlineStr">
+        <is>
+          <t>정부가 중동전 교훈을 바탕으로 국내 생산·비축, 해외 생산, 수입선 다변화 등 4단계로 공급망을 재편하고 5대 업종의 탈탄소 전환을 추진한다.</t>
+        </is>
+      </c>
+      <c r="F810" s="3" t="inlineStr">
+        <is>
+          <t>정부의 공급망 재편 전략은 우리 회사의 원자재 수급 및 생산 계획에 장기적인 영향을 미칠 수 있으며, 탈탄소 전환은 물류 운영 방식에도 변화를 요구할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G810" s="3" t="inlineStr">
+        <is>
+          <t>정부의 공급망 정책 변화를 면밀히 주시하고, 우리 회사의 공급망 다변화 전략 및 탈탄소 물류 전환 계획에 반영할 방안을 검토한다.</t>
+        </is>
+      </c>
+      <c r="H810" s="3" t="inlineStr">
+        <is>
+          <t>연합뉴스</t>
+        </is>
+      </c>
+      <c r="I810" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20260713154800002</t>
+        </is>
+      </c>
+      <c r="J810" s="3" t="inlineStr"/>
+    </row>
+    <row r="811">
+      <c r="A811" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B811" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C811" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D811" s="3" t="inlineStr">
+        <is>
+          <t>신한증권 "대한항공, 유류할증료 완화로 여행 수요 회복…목표가↑"</t>
+        </is>
+      </c>
+      <c r="E811" s="3" t="inlineStr">
+        <is>
+          <t>신한투자증권은 대한항공의 유류할증료 완화로 여행 수요가 회복되고 항공화물 운임 강세와 아시아나 합병 효과가 기대되어 목표가를 상향 조정했다.</t>
+        </is>
+      </c>
+      <c r="F811" s="3" t="inlineStr">
+        <is>
+          <t>유류할증료 완화는 항공 운임에 긍정적인 영향을 줄 수 있으나, 항공화물 운임 강세는 물류비 상승 요인이 될 수 있어 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G811" s="3" t="inlineStr">
+        <is>
+          <t>항공화물 운임 동향을 지속적으로 모니터링하고, 유류할증료 변동이 우리 회사의 항공 물류 비용에 미치는 영향을 분석하여 운송 계획에 반영한다.</t>
+        </is>
+      </c>
+      <c r="H811" s="3" t="inlineStr">
+        <is>
+          <t>연합뉴스</t>
+        </is>
+      </c>
+      <c r="I811" s="3" t="inlineStr">
+        <is>
+          <t>https://yna.co.kr/amp/view/AKR20260715028200008</t>
+        </is>
+      </c>
+      <c r="J811" s="3" t="inlineStr"/>
+    </row>
+    <row r="812">
+      <c r="A812" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B812" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C812" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D812" s="3" t="inlineStr">
+        <is>
+          <t>국제유가 하락에 수입물가 4.4%↓…3년6개월 만에 최대 낙폭</t>
+        </is>
+      </c>
+      <c r="E812" s="3" t="inlineStr">
+        <is>
+          <t>한국은행 발표에 따르면 지난달 국제유가가 하락하면서 수입물가가 3년 6개월 만에 가장 큰 폭인 4.4% 떨어졌다.</t>
+        </is>
+      </c>
+      <c r="F812" s="3" t="inlineStr">
+        <is>
+          <t>국제 유가 하락은 해상/항공 운임 및 물류비용 하락으로 이어질 수 있어 우리 회사의 물류비 절감에 긍정적인 영향을 미칠 수 있으므로 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G812" s="3" t="inlineStr">
+        <is>
+          <t>국제 유가 및 운임 변동 추이를 지속적으로 모니터링하고, 물류비용 절감 기회를 모색하며 운송 계약 조건 검토 시 반영한다.</t>
+        </is>
+      </c>
+      <c r="H812" s="3" t="inlineStr">
+        <is>
+          <t>헤럴드경제</t>
+        </is>
+      </c>
+      <c r="I812" s="3" t="inlineStr">
+        <is>
+          <t>https://biz.heraldcorp.com/article/10808720</t>
+        </is>
+      </c>
+      <c r="J812" s="3" t="inlineStr"/>
+    </row>
+    <row r="813">
+      <c r="A813" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B813" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C813" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D813" s="3" t="inlineStr">
+        <is>
+          <t>[국제유가] 미-이란 공방 속 0.3% 안팎 상승</t>
+        </is>
+      </c>
+      <c r="E813" s="3" t="inlineStr">
+        <is>
+          <t>국제 유가가 미-이란 공방 속에서 소폭(0.3%) 상승했으나, 전반적으로 관망세를 보이며 배럴당 84.95달러 수준을 유지했다.</t>
+        </is>
+      </c>
+      <c r="F813" s="3" t="inlineStr">
+        <is>
+          <t>유가가 소폭 상승했으나 큰 변동은 아니며, 물류비에 직접적인 영향을 미치기까지는 추이를 지켜봐야 한다.</t>
+        </is>
+      </c>
+      <c r="G813" s="3" t="inlineStr">
+        <is>
+          <t>유가 변동 추이 및 유류할증료 변화를 지속적으로 모니터링하여 물류비 예측에 반영.</t>
+        </is>
+      </c>
+      <c r="H813" s="3" t="inlineStr">
+        <is>
+          <t>파이낸셜뉴스</t>
+        </is>
+      </c>
+      <c r="I813" s="3" t="inlineStr">
+        <is>
+          <t>https://www.fnnews.com/news/202607160424534831</t>
+        </is>
+      </c>
+      <c r="J813" s="3" t="inlineStr"/>
+    </row>
+    <row r="814">
+      <c r="A814" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B814" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C814" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D814" s="3" t="inlineStr">
+        <is>
+          <t>한국 수입물가, 3년 6개월 만의 최대 하락...국제유가 급락 영향</t>
+        </is>
+      </c>
+      <c r="E814" s="3" t="inlineStr">
+        <is>
+          <t>국제 유가 급락의 영향으로 지난달 한국의 수입 물가가 3년 6개월 만에 최대 폭으로 하락했으며, 이는 중동 전쟁 안정화로 인한 유가 안정세에 기인한다.</t>
+        </is>
+      </c>
+      <c r="F814" s="3" t="inlineStr">
+        <is>
+          <t>국제 유가 하락은 해상/항공 운임의 유류할증료 인하로 이어져 물류비 절감에 긍정적인 영향을 미칠 수 있으므로 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G814" s="3" t="inlineStr">
+        <is>
+          <t>유가 하락 추세가 지속될 경우, 운송 계약 시 유류할증료 조건 재검토 및 물류비 절감 방안 모색.</t>
+        </is>
+      </c>
+      <c r="H814" s="3" t="inlineStr">
+        <is>
+          <t>M이코노미뉴스</t>
+        </is>
+      </c>
+      <c r="I814" s="3" t="inlineStr">
+        <is>
+          <t>https://www.m-economynews.com/news/article.html?no=68767</t>
+        </is>
+      </c>
+      <c r="J814" s="3" t="inlineStr"/>
+    </row>
+    <row r="815">
+      <c r="A815" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B815" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C815" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D815" s="4" t="inlineStr">
+        <is>
+          <t>Global Schedule Reliability for May 2026 the Highest of the Year</t>
+        </is>
+      </c>
+      <c r="E815" s="4" t="inlineStr">
+        <is>
+          <t>2026년 5월 글로벌 선박 스케줄 신뢰도가 연중 최고치를 기록하여 해운 서비스의 안정성이 개선되고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F815" s="4" t="inlineStr">
+        <is>
+          <t>스케줄 신뢰도 개선은 긍정적인 소식이지만, 일시적일 수 있으며 장기적인 추이를 더 지켜봐야 합니다.</t>
+        </is>
+      </c>
+      <c r="G815" s="4" t="n"/>
+      <c r="H815" s="4" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I815" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/395-global-liner-performance-glp-report-issue-178</t>
+        </is>
+      </c>
+      <c r="J815" s="4" t="inlineStr"/>
+    </row>
+    <row r="816">
+      <c r="A816" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B816" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C816" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D816" s="4" t="inlineStr">
+        <is>
+          <t>글로벌 LNG선 선대 중 선령 20년 이상 스팀터빈 선박 총 120척 규모...향후 5년 내 폐선 가능성 높아</t>
+        </is>
+      </c>
+      <c r="E816" s="4" t="inlineStr">
+        <is>
+          <t>글로벌 LNG선 선대 중 노후 선박의 폐선 가능성이 높아 향후 5년간 LNG선 발주 수요가 증가할 것으로 전망됩니다.</t>
+        </is>
+      </c>
+      <c r="F816" s="4" t="inlineStr">
+        <is>
+          <t>LNG선 시장 동향은 배터리/전자부품 운송에 직접적인 영향이 적으며, 일반 컨테이너선 시장과는 별개입니다.</t>
+        </is>
+      </c>
+      <c r="G816" s="4" t="n"/>
+      <c r="H816" s="4" t="inlineStr">
+        <is>
+          <t>쉬핑뉴스넷</t>
+        </is>
+      </c>
+      <c r="I816" s="4" t="inlineStr">
+        <is>
+          <t>https://www.shippingnewsnet.com/news/articleView.html?idxno=71197</t>
+        </is>
+      </c>
+      <c r="J816" s="4" t="inlineStr"/>
+    </row>
+    <row r="817">
+      <c r="A817" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B817" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C817" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D817" s="4" t="inlineStr">
+        <is>
+          <t>영남이공대, '교육 넘어 채용까지'…쿠팡과 손잡고 AI 물류인재 키운다</t>
+        </is>
+      </c>
+      <c r="E817" s="4" t="inlineStr">
+        <is>
+          <t>영남이공대학교가 쿠팡과 협력하여 AI 기반 물류 전문 교육 및 취업 연계 프로그램을 통해 현장형 인재 양성에 나섭니다.</t>
+        </is>
+      </c>
+      <c r="F817" s="4" t="inlineStr">
+        <is>
+          <t>물류 인재 양성 소식은 긍정적이나, 우리 회사의 당면한 물류 운영에 직접적인 영향은 없습니다.</t>
+        </is>
+      </c>
+      <c r="G817" s="4" t="n"/>
+      <c r="H817" s="4" t="inlineStr">
+        <is>
+          <t>Surff</t>
+        </is>
+      </c>
+      <c r="I817" s="4" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260715-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J817" s="4" t="inlineStr"/>
+    </row>
+    <row r="818">
+      <c r="A818" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B818" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C818" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D818" s="4" t="inlineStr">
+        <is>
+          <t>현대LNG해운 매각, 산기위·공정위 심</t>
+        </is>
+      </c>
+      <c r="E818" s="4" t="inlineStr">
+        <is>
+          <t>현대LNG해운 매각이 산업통상자원부와 공정거래위원회의 심사를 받고 있으며, 이는 해운 산업의 국가 안보적 중요성을 반영합니다.</t>
+        </is>
+      </c>
+      <c r="F818" s="4" t="inlineStr">
+        <is>
+          <t>LNG선사의 매각은 우리 회사의 배터리/전자부품 운송에 직접적인 영향이 없으며, 일반 해운 시장에 미치는 영향도 제한적입니다.</t>
+        </is>
+      </c>
+      <c r="G818" s="4" t="n"/>
+      <c r="H818" s="4" t="inlineStr">
+        <is>
+          <t>Surff</t>
+        </is>
+      </c>
+      <c r="I818" s="4" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260713-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J818" s="4" t="inlineStr"/>
+    </row>
+    <row r="819">
+      <c r="A819" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B819" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C819" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D819" s="4" t="inlineStr">
+        <is>
+          <t>선사가 다른 선사를 인수할 때 정부가 나서는 이유 : 해운업과 국가안보의 경계 (Week 28, 2026)</t>
+        </is>
+      </c>
+      <c r="E819" s="4" t="inlineStr">
+        <is>
+          <t>해운 산업은 국가 기간 산업으로 인식되어 선사 간 M&amp;A 시 항만, 선박 등 핵심 인프라 이전을 이유로 여러 국가가 국가안보 심사 절차를 두고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F819" s="4" t="inlineStr">
+        <is>
+          <t>해운 M&amp;A에 대한 정부의 개입은 장기적인 산업 구조에 영향을 미칠 수 있으나, 우리 회사의 단기 물류 운영에 직접적인 영향은 없습니다.</t>
+        </is>
+      </c>
+      <c r="G819" s="4" t="n"/>
+      <c r="H819" s="4" t="inlineStr">
+        <is>
+          <t>Surff</t>
+        </is>
+      </c>
+      <c r="I819" s="4" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/선사가-다른-선사를-인수할-때-정부가-나서는-이유-해운업과-국가안보의-경계-week-28-2026</t>
+        </is>
+      </c>
+      <c r="J819" s="4" t="inlineStr"/>
+    </row>
+    <row r="820">
+      <c r="A820" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B820" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C820" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D820" s="4" t="inlineStr">
+        <is>
+          <t>Freight Distress Report: Carrier, logistics closures erase over 245 jobs</t>
+        </is>
+      </c>
+      <c r="E820" s="4" t="inlineStr">
+        <is>
+          <t>운송 및 물류 기업들의 폐업과 파산으로 245개 이상의 일자리가 사라지는 등 화물 운송 산업의 어려움이 지속되고 있으며, 이는 트럭 운송, 물류, 복합 운송 등 전반적인 분야에 걸쳐 나타나고 있다.</t>
+        </is>
+      </c>
+      <c r="F820" s="4" t="inlineStr">
+        <is>
+          <t>물류 산업 전반의 어려움을 보여주지만, 특정 운송 지연이나 규제 변화와 같이 우리 회사에 직접적인 영향을 미칠 정도는 아니다.</t>
+        </is>
+      </c>
+      <c r="G820" s="4" t="n"/>
+      <c r="H820" s="4" t="inlineStr">
+        <is>
+          <t>FreightWaves</t>
+        </is>
+      </c>
+      <c r="I820" s="4" t="inlineStr">
+        <is>
+          <t>https://finance.yahoo.com/economy/articles/freight-distress-report-carrier-logistics-144420684.html</t>
+        </is>
+      </c>
+      <c r="J820" s="4" t="inlineStr"/>
+    </row>
+    <row r="821">
+      <c r="A821" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B821" s="4" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C821" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D821" s="4" t="inlineStr">
+        <is>
+          <t>US tariff talks, West Asia tensions cloud outlook for Indian textile exporters | Mint</t>
+        </is>
+      </c>
+      <c r="E821" s="4" t="inlineStr">
+        <is>
+          <t>미국 관세 협상과 서아시아(중동) 지역의 긴장이 인도 섬유 수출업자들의 전망을 불확실하게 만들고 있으며, 이는 원자재 가격 변동과 함께 수출 환경에 영향을 미치고 있다.</t>
+        </is>
+      </c>
+      <c r="F821" s="4" t="inlineStr">
+        <is>
+          <t>인도 섬유 산업에 대한 관세 및 중동 긴장 관련 뉴스이며, 우리 회사의 배터리/전자부품 물류에 직접적인 영향은 미미하다.</t>
+        </is>
+      </c>
+      <c r="G821" s="4" t="n"/>
+      <c r="H821" s="4" t="inlineStr">
+        <is>
+          <t>Mint</t>
+        </is>
+      </c>
+      <c r="I821" s="4" t="inlineStr">
+        <is>
+          <t>https://livemint.com/industry/india-textile-exporters-us-tariffs-cotton-prices-west-asia-11784099967570.html</t>
+        </is>
+      </c>
+      <c r="J821" s="4" t="inlineStr"/>
+    </row>
+    <row r="822">
+      <c r="A822" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B822" s="4" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C822" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D822" s="4" t="inlineStr">
+        <is>
+          <t>삼성SDI UPS용 배터리, 글로벌 ‘화재 안전’ 테스트 통과</t>
+        </is>
+      </c>
+      <c r="E822" s="4" t="inlineStr">
+        <is>
+          <t>삼성SDI의 UPS(무정전전원장치)용 배터리가 글로벌 안전 인증기관 UL 솔루션즈의 옥내 대형 화재 차단 테스트를 통과하며 높은 안전성 기술을 인정받았다.</t>
+        </is>
+      </c>
+      <c r="F822" s="4" t="inlineStr">
+        <is>
+          <t>경쟁사의 배터리 안전성 인증 소식으로, 우리 회사의 제품 안전성 강화 및 규제 준수 노력에 긍정적인 참고 자료가 될 수 있으나 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G822" s="4" t="n"/>
+      <c r="H822" s="4" t="inlineStr">
+        <is>
+          <t>울산매일</t>
+        </is>
+      </c>
+      <c r="I822" s="4" t="inlineStr">
+        <is>
+          <t>https://iusm.co.kr/news/articleView.html?idxno=1065347</t>
+        </is>
+      </c>
+      <c r="J822" s="4" t="inlineStr"/>
+    </row>
+    <row r="823">
+      <c r="A823" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B823" s="4" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C823" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D823" s="4" t="inlineStr">
+        <is>
+          <t>서울교통공사, 대용량 리튬배터리 반입 제한 집중 캠페인</t>
+        </is>
+      </c>
+      <c r="E823" s="4" t="inlineStr">
+        <is>
+          <t>서울교통공사가 지난 1일부터 시행 중인 대용량 리튬배터리 및 개인형 이동장치(PM) 휴대 제한 제도의 안정적인 정착과 시민 인지도 제고를 위한 집중 캠페인을 진행하고 있다.</t>
+        </is>
+      </c>
+      <c r="F823" s="4" t="inlineStr">
+        <is>
+          <t>대중교통 내 리튬배터리 반입 제한은 주로 개인 소비자에게 영향을 미치며, 우리 회사의 물류 운송 방식에는 직접적인 영향이 없다.</t>
+        </is>
+      </c>
+      <c r="G823" s="4" t="n"/>
+      <c r="H823" s="4" t="inlineStr">
+        <is>
+          <t>헤럴드경제</t>
+        </is>
+      </c>
+      <c r="I823" s="4" t="inlineStr">
+        <is>
+          <t>https://biz.heraldcorp.com/article/10808357</t>
+        </is>
+      </c>
+      <c r="J823" s="4" t="inlineStr"/>
+    </row>
+    <row r="824">
+      <c r="A824" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B824" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C824" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D824" s="4" t="inlineStr">
+        <is>
+          <t>국토부, 2028년 UAM 초기 서비스 기준 마련…조종사·정비사 양성 착수</t>
+        </is>
+      </c>
+      <c r="E824" s="4" t="inlineStr">
+        <is>
+          <t>국토부가 2028년 도심항공교통(UAM) 초기 시범서비스 개시를 위한 구체적인 운항 기준을 마련하고 조종사 및 정비사 양성에 착수했다.</t>
+        </is>
+      </c>
+      <c r="F824" s="4" t="inlineStr">
+        <is>
+          <t>UAM 서비스 기준 마련은 미래 운송 기술 동향에 대한 정보이며, 현재 우리 회사의 배터리/전자부품 물류 운영에는 직접적인 영향이 없다.</t>
+        </is>
+      </c>
+      <c r="G824" s="4" t="n"/>
+      <c r="H824" s="4" t="inlineStr">
+        <is>
+          <t>IDSN</t>
+        </is>
+      </c>
+      <c r="I824" s="4" t="inlineStr">
+        <is>
+          <t>https://idsn.co.kr/news/view/1065579269817032</t>
+        </is>
+      </c>
+      <c r="J824" s="4" t="inlineStr"/>
+    </row>
+    <row r="825">
+      <c r="A825" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B825" s="4" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C825" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D825" s="4" t="inlineStr">
+        <is>
+          <t>폐배터리 속 리튬, 미생물로 90% 이상 회수</t>
+        </is>
+      </c>
+      <c r="E825" s="4" t="inlineStr">
+        <is>
+          <t>국립낙동강생물자원관이 담수 미생물을 활용하여 폐배터리에서 핵심 원료인 리튬을 90% 이상 회수할 수 있는 친환경 기술을 개발했다.</t>
+        </is>
+      </c>
+      <c r="F825" s="4" t="inlineStr">
+        <is>
+          <t>폐배터리 재활용 기술 개발 소식으로, 장기적으로 친환경 원료 확보에 기여할 수 있으나, 현재 우리 회사의 물류 운영에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G825" s="4" t="n"/>
+      <c r="H825" s="4" t="inlineStr">
+        <is>
+          <t>데일리대구경북뉴스</t>
+        </is>
+      </c>
+      <c r="I825" s="4" t="inlineStr">
+        <is>
+          <t>https://dailydgnews.com/news/article.html?no=257442</t>
+        </is>
+      </c>
+      <c r="J825" s="4" t="inlineStr"/>
+    </row>
+    <row r="826">
+      <c r="A826" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B826" s="4" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C826" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D826" s="4" t="inlineStr">
+        <is>
+          <t>반도체공장 방화구획 기준 완화…건축 화재안전 규제 합리화</t>
+        </is>
+      </c>
+      <c r="E826" s="4" t="inlineStr">
+        <is>
+          <t>국토교통부가 반도체 공장의 현장 여건을 반영하여 층간 방화구획 기준을 완화하고 건축 화재안전 자재의 신제품 품질인정 범위를 확대하는 등 건축 관련 규제를 합리화한다.</t>
+        </is>
+      </c>
+      <c r="F826" s="4" t="inlineStr">
+        <is>
+          <t>이 뉴스는 주로 반도체 공장의 건축 화재안전 규제 완화에 관한 것으로, 배터리/전자부품 제조기업의 물류 운영에 직접적인 영향은 미미하다.</t>
+        </is>
+      </c>
+      <c r="G826" s="4" t="inlineStr"/>
+      <c r="H826" s="4" t="inlineStr">
+        <is>
+          <t>전기신문</t>
+        </is>
+      </c>
+      <c r="I826" s="4" t="inlineStr">
+        <is>
+          <t>https://electimes.com/news/articleView.html?idxno=370349</t>
+        </is>
+      </c>
+      <c r="J826" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -37494,7 +39538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -38258,6 +40302,49 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>3184.82</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>-142 (-4.3%)</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>+1,323 (+71.1%)</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>4318</v>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>-12 (-0.3%)</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>+1,728 (+66.7%)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -38270,7 +40357,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I138"/>
+  <dimension ref="A1:I145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -43126,6 +45213,251 @@
       </c>
       <c r="I138" s="6" t="inlineStr"/>
     </row>
+    <row r="139">
+      <c r="A139" s="6" t="inlineStr">
+        <is>
+          <t>RSK-138</t>
+        </is>
+      </c>
+      <c r="B139" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C139" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D139" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E139" s="6" t="inlineStr">
+        <is>
+          <t>DOJ Appeals CIT's IEEPA Refund Injunction as CAPE Phase 2 Targets June 29; TPEB Rates Surge 30% Into Peak</t>
+        </is>
+      </c>
+      <c r="F139" s="6" t="inlineStr"/>
+      <c r="G139" s="6" t="inlineStr"/>
+      <c r="H139" s="6" t="inlineStr">
+        <is>
+          <t>TPEB 운임 급등에 대한 즉각적인 비용 절감 방안(예: 선적 계획 조정, 운송사 협상)을 모색하고, IEEPA 환급 관련 소송 진행 상황을 면밀히 주시하여 잠재적 관세 비용 영향을 평가한다.</t>
+        </is>
+      </c>
+      <c r="I139" s="6" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="6" t="inlineStr">
+        <is>
+          <t>RSK-139</t>
+        </is>
+      </c>
+      <c r="B140" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C140" s="6" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="D140" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E140" s="6" t="inlineStr">
+        <is>
+          <t>CPSC Mandatory eFiling Takes Effect July 8; TPEB Rates Surge ~10% as Peak Season Demand Outpaces Capacity</t>
+        </is>
+      </c>
+      <c r="F140" s="6" t="inlineStr"/>
+      <c r="G140" s="6" t="inlineStr"/>
+      <c r="H140" s="6" t="inlineStr">
+        <is>
+          <t>CPSC 전자 신고 의무 사항을 즉시 확인하고 관련 시스템 및 절차를 준비하며, CBP의 강제 노동 지침에 따라 공급망 내 강제 노동 리스크를 재평가하고 필요한 조치를 취한다.</t>
+        </is>
+      </c>
+      <c r="I140" s="6" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="6" t="inlineStr">
+        <is>
+          <t>RSK-140</t>
+        </is>
+      </c>
+      <c r="B141" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C141" s="6" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="D141" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E141" s="6" t="inlineStr">
+        <is>
+          <t>CBP Rejects Warehouse Entries on CAPE Declarations, Risking IEEPA Refunds; TPEB Rates Climb as Panama Canal Restrictions Tighten Capacity</t>
+        </is>
+      </c>
+      <c r="F141" s="6" t="inlineStr"/>
+      <c r="G141" s="6" t="inlineStr"/>
+      <c r="H141" s="6" t="inlineStr">
+        <is>
+          <t>파나마 운하를 이용하는 운송 경로의 지연 및 운임 상승에 대비하여 대체 경로(예: 수에즈 운하, 미 서안 육상 운송)를 검토하고, IEEPA 환급 관련 CBP 지침을 확인하여 관세 비용 영향을 최소화한다.</t>
+        </is>
+      </c>
+      <c r="I141" s="6" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="6" t="inlineStr">
+        <is>
+          <t>RSK-141</t>
+        </is>
+      </c>
+      <c r="B142" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C142" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D142" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E142" s="6" t="inlineStr">
+        <is>
+          <t>유가 150달러 경고! 세계 경제 뒤흔들 최악의 시나리오</t>
+        </is>
+      </c>
+      <c r="F142" s="6" t="inlineStr"/>
+      <c r="G142" s="6" t="inlineStr"/>
+      <c r="H142" s="6" t="inlineStr">
+        <is>
+          <t>유가 및 운임 변동 추이를 면밀히 모니터링하고, 운송 계약 시 유가 연동 조항 검토 및 장기 계약을 통한 리스크 헤지 방안을 모색합니다.</t>
+        </is>
+      </c>
+      <c r="I142" s="6" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="6" t="inlineStr">
+        <is>
+          <t>RSK-142</t>
+        </is>
+      </c>
+      <c r="B143" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C143" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D143" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E143" s="6" t="inlineStr">
+        <is>
+          <t>미-이란, 호르무즈 통제권 놓고 또 충돌…오만, 남북 2개 항로 제안</t>
+        </is>
+      </c>
+      <c r="F143" s="6" t="inlineStr"/>
+      <c r="G143" s="6" t="inlineStr"/>
+      <c r="H143" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 상황을 실시간으로 모니터링하고, 비상시 대체 운송 경로 및 운송 수단(항공 등) 확보 계획을 수립하며, 주요 원자재 재고 수준을 점검합니다.</t>
+        </is>
+      </c>
+      <c r="I143" s="6" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="6" t="inlineStr">
+        <is>
+          <t>RSK-143</t>
+        </is>
+      </c>
+      <c r="B144" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C144" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D144" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E144" s="6" t="inlineStr">
+        <is>
+          <t>트럼프 '호르무즈 통행료' 하루 만에 철회…해협 불확실성은 여전</t>
+        </is>
+      </c>
+      <c r="F144" s="6" t="inlineStr"/>
+      <c r="G144" s="6" t="inlineStr"/>
+      <c r="H144" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 관련 정치적 발언 및 동향을 예의주시하고, 비상시 운송 계획을 재점검합니다.</t>
+        </is>
+      </c>
+      <c r="I144" s="6" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="6" t="inlineStr">
+        <is>
+          <t>RSK-144</t>
+        </is>
+      </c>
+      <c r="B145" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C145" s="6" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="D145" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E145" s="6" t="inlineStr">
+        <is>
+          <t>상하이항 태풍으로 운영 중단, 수십 척 컨테이너선 입항 지연</t>
+        </is>
+      </c>
+      <c r="F145" s="6" t="inlineStr"/>
+      <c r="G145" s="6" t="inlineStr"/>
+      <c r="H145" s="6" t="inlineStr">
+        <is>
+          <t>상하이항을 경유하는 모든 선적의 현황을 즉시 파악하고, 지연 예상 물량에 대한 고객 및 생산 부서에 통보하며, 필요시 대체 항만 또는 항공 운송 전환을 검토합니다.</t>
+        </is>
+      </c>
+      <c r="I145" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
📰 뉴스 데이터 2026-07-17_08:58
</commit_message>
<xml_diff>
--- a/data/SCM_물류_브리핑.xlsx
+++ b/data/SCM_물류_브리핑.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J826"/>
+  <dimension ref="A1:J872"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -39526,6 +39526,2186 @@
       </c>
       <c r="J826" s="4" t="inlineStr"/>
     </row>
+    <row r="827">
+      <c r="A827" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B827" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C827" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D827" s="2" t="inlineStr">
+        <is>
+          <t>Section 301 Tariffs on Brazil Take Effect July 22, Stacking with Section 122 Duties; Strait of Hormuz Closure Restricts 200K TEU of Ocean Capacity</t>
+        </is>
+      </c>
+      <c r="E827" s="2" t="inlineStr">
+        <is>
+          <t>7월 22일부터 브라질에 대한 Section 301 관세가 발효되며, 러시아 제재 법안은 중국과 인도에 대한 2차 관세 부과 가능성을 언급한다. 또한 호르무즈 해협 폐쇄로 20만 TEU의 해상 운송 용량이 제한될 수 있다.</t>
+        </is>
+      </c>
+      <c r="F827" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 폐쇄는 중동발 원자재 및 유럽향/아시아향 해상 운송에 심각한 지연과 비용 상승을 초래할 수 있으며, 브라질 및 러시아 관련 관세는 특정 원자재 수급 및 비용에 직접적인 영향을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="G827" s="2" t="inlineStr">
+        <is>
+          <t>중동발 원자재 및 유럽/아시아향 해상 운송 경로 다변화 및 대체 운송 수단 검토, 브라질 및 러시아 관련 공급망 점검 및 관세 영향 분석.</t>
+        </is>
+      </c>
+      <c r="H827" s="2" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I827" s="2" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/july-16-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J827" s="2" t="inlineStr">
+        <is>
+          <t>RSK-145</t>
+        </is>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B828" s="2" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C828" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D828" s="2" t="inlineStr">
+        <is>
+          <t>CBP Rejects Warehouse Entries on CAPE Declarations, Risking IEEPA Refunds; TPEB Rates Climb as Panama Canal Restrictions Tighten Capacity</t>
+        </is>
+      </c>
+      <c r="E828" s="2" t="inlineStr">
+        <is>
+          <t>CBP가 CAPE 신고에 대한 창고 입고를 거부하여 IEEPA 환급에 위험을 초래하고 있으며, 파나마 운하 통행 제한으로 인해 태평양 횡단 동향(TPEB) 운임이 상승하고 있다.</t>
+        </is>
+      </c>
+      <c r="F828" s="2" t="inlineStr">
+        <is>
+          <t>파나마 운하 통행 제한은 미주향 운송 지연 및 운임 상승에 직접적인 영향을 미치며, CBP의 창고 입고 거부는 통관 및 재고 관리에 즉각적인 문제를 야기할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G828" s="2" t="inlineStr">
+        <is>
+          <t>파나마 운하 대체 경로 및 운송 수단 검토, CBP 통관 절차 및 CAPE 관련 규정 준수 여부 재확인 및 대응 방안 마련.</t>
+        </is>
+      </c>
+      <c r="H828" s="2" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I828" s="2" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/july-09-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J828" s="2" t="inlineStr">
+        <is>
+          <t>RSK-146</t>
+        </is>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B829" s="2" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C829" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D829" s="2" t="inlineStr">
+        <is>
+          <t>CPSC Mandatory eFiling Takes Effect July 8; TPEB Rates Surge ~10% as Peak Season Demand Outpaces Capacity</t>
+        </is>
+      </c>
+      <c r="E829" s="2" t="inlineStr">
+        <is>
+          <t>7월 8일부터 CPSC의 의무적인 전자 신고가 발효되었고, CBP는 강제 노동 관련 지침을 통합 발표했으며, 성수기 수요가 공급을 초과하면서 태평양 횡단 동향(TPEB) 운임이 약 10% 급등했다.</t>
+        </is>
+      </c>
+      <c r="F829" s="2" t="inlineStr">
+        <is>
+          <t>CPSC 전자 신고 의무화는 미국 수출 시 통관 절차에 직접적인 영향을 미치며, CBP의 강제 노동 지침은 공급망 실사에 대한 부담을 가중시키고, TPEB 운임 급등은 미주향 물류 비용에 즉각적인 영향을 준다.</t>
+        </is>
+      </c>
+      <c r="G829" s="2" t="inlineStr">
+        <is>
+          <t>CPSC 전자 신고 시스템 및 강제 노동 지침 준수 여부 확인 및 내부 프로세스 업데이트, TPEB 운임 급등에 대한 단기 및 장기 운송 전략 재검토.</t>
+        </is>
+      </c>
+      <c r="H829" s="2" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I829" s="2" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/june-18-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J829" s="2" t="inlineStr">
+        <is>
+          <t>RSK-147</t>
+        </is>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B830" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C830" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D830" s="2" t="inlineStr">
+        <is>
+          <t>끝나지 않은 중동 사태…'호르무즈 없는 시나리오' 짜는 산업계</t>
+        </is>
+      </c>
+      <c r="E830" s="2" t="inlineStr">
+        <is>
+          <t>중동 사태 장기화로 해상 운송 의존도가 높은 산업계가 운임 상승과 물류 지연에 대비해 '호르무즈 없는 시나리오'를 포함한 비상 계획을 수립하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F830" s="2" t="inlineStr">
+        <is>
+          <t>주요 산업계가 호르무즈 사태 장기화에 대비하는 것은 우리 기업 또한 유사한 리스크에 노출되어 있음을 의미하며, 선제적인 대응이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G830" s="2" t="inlineStr">
+        <is>
+          <t>중동 리스크에 대한 비상 계획 구체화, 대체 운송 경로 및 운송 수단 다변화 검토, 재고 수준 조정.</t>
+        </is>
+      </c>
+      <c r="H830" s="2" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I830" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260717-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J830" s="2" t="inlineStr">
+        <is>
+          <t>RSK-148</t>
+        </is>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B831" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C831" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D831" s="2" t="inlineStr">
+        <is>
+          <t>미·이란 전면전 위기…국제유가 9%↑, 한달만에 최고치</t>
+        </is>
+      </c>
+      <c r="E831" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 인근 긴장으로 공급 차질 우려가 커지며 국제유가가 한 달 만에 최고치로 급등했으며, 유가 150달러 경고까지 나오고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F831" s="2" t="inlineStr">
+        <is>
+          <t>국제유가 급등은 해상 및 항공 운송 비용에 즉각적인 영향을 미쳐 우리 물류비 상승으로 이어지므로 즉시 대응이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G831" s="2" t="inlineStr">
+        <is>
+          <t>유가 변동성 모니터링 강화, 운송 계약 조건(유류할증료 등) 재검토, 비용 절감 방안 모색.</t>
+        </is>
+      </c>
+      <c r="H831" s="2" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I831" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260714-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J831" s="2" t="inlineStr">
+        <is>
+          <t>RSK-149</t>
+        </is>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B832" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C832" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D832" s="2" t="inlineStr">
+        <is>
+          <t>봉쇄된 호르무즈의 ‘숨통’ 셔틀선도 이란 공격 위협 직면</t>
+        </is>
+      </c>
+      <c r="E832" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협의 군사적 긴장이 고조되면서 해협을 오가던 셔틀선 운항마저 이란의 공격 위협에 직면하여 운항이 위축될 전망입니다.</t>
+        </is>
+      </c>
+      <c r="F832" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협은 주요 에너지 및 물류 동맥으로, 이곳의 군사적 긴장 고조와 셔틀선 운항 위축은 유가 상승 및 해상 운송 지연을 야기하여 우리 물류 운영에 직접적인 영향을 미칩니다.</t>
+        </is>
+      </c>
+      <c r="G832" s="2" t="inlineStr">
+        <is>
+          <t>중동 경유 노선 및 유가 변동성 모니터링 강화, 대체 운송 경로 및 재고 확보 방안 검토, 비상 계획 수립.</t>
+        </is>
+      </c>
+      <c r="H832" s="2" t="inlineStr">
+        <is>
+          <t>khan.co.kr</t>
+        </is>
+      </c>
+      <c r="I832" s="2" t="inlineStr">
+        <is>
+          <t>https://khan.co.kr/article/202607151023001</t>
+        </is>
+      </c>
+      <c r="J832" s="2" t="inlineStr">
+        <is>
+          <t>RSK-150</t>
+        </is>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B833" s="2" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C833" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D833" s="2" t="inlineStr">
+        <is>
+          <t>‘화재 철통 관리’ BIFC 지하에서 화재 발생… 소형 이동 장치 ‘안전 사각’ - 부산일보</t>
+        </is>
+      </c>
+      <c r="E833" s="2" t="inlineStr">
+        <is>
+          <t>국내 최고 수준의 소방관리 기준이 적용되는 부산국제금융센터(BIFC) 지하에서 충전 중이던 청소용 전동카트 배터리에 불이 나, 소형 이동 장치의 배터리 안전 관리 사각지대 문제가 부각되었다.</t>
+        </is>
+      </c>
+      <c r="F833" s="2" t="inlineStr">
+        <is>
+          <t>배터리 화재 사고는 당사 제품의 안전성 및 운송/보관 규제 강화로 이어질 수 있어 즉각적인 내부 안전 점검 및 규제 변화 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G833" s="2" t="inlineStr">
+        <is>
+          <t>배터리 제품의 운송 및 보관, 충전 관련 안전 지침을 재검토하고, 관련 규제 동향을 면밀히 모니터링하며, 창고 및 물류센터 내 배터리 취급 안전 교육을 강화한다.</t>
+        </is>
+      </c>
+      <c r="H833" s="2" t="inlineStr">
+        <is>
+          <t>부산일보</t>
+        </is>
+      </c>
+      <c r="I833" s="2" t="inlineStr">
+        <is>
+          <t>https://busan.com/view/busan/view.php?code=2026071612315555568</t>
+        </is>
+      </c>
+      <c r="J833" s="2" t="inlineStr">
+        <is>
+          <t>RSK-151</t>
+        </is>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B834" s="2" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C834" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D834" s="2" t="inlineStr">
+        <is>
+          <t>대형 화학물질 화재사고 대비 비상대응체계 강화한다 - 헤럴드경제</t>
+        </is>
+      </c>
+      <c r="E834" s="2" t="inlineStr">
+        <is>
+          <t>기후에너지환경부 소속 화학물질안전원은 대형 화학물질 화재사고에 효과적으로 대비하기 위해 화학사고예방관리계획서 상의 비상대응계획을 강화한다.</t>
+        </is>
+      </c>
+      <c r="F834" s="2" t="inlineStr">
+        <is>
+          <t>화학물질 화재사고 비상대응체계 강화는 당사의 위험물(배터리) 취급 및 보관 규제에 직접적인 영향을 미치므로 즉각적인 내부 지침 검토가 필요하다.</t>
+        </is>
+      </c>
+      <c r="G834" s="2" t="inlineStr">
+        <is>
+          <t>당사 물류센터 및 창고의 위험물(배터리) 보관 및 취급 관련 비상대응계획을 재검토하고, 관련 규제 변화에 맞춰 안전 관리 시스템을 강화한다.</t>
+        </is>
+      </c>
+      <c r="H834" s="2" t="inlineStr">
+        <is>
+          <t>헤럴드경제</t>
+        </is>
+      </c>
+      <c r="I834" s="2" t="inlineStr">
+        <is>
+          <t>https://biz.heraldcorp.com/article/10810366</t>
+        </is>
+      </c>
+      <c r="J834" s="2" t="inlineStr">
+        <is>
+          <t>RSK-152</t>
+        </is>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B835" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C835" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D835" s="2" t="inlineStr">
+        <is>
+          <t>Micron Technology Inc (MU) 주식 움직였습니다 하락 6.96%에 7월15일: 어떤 신호인가요?</t>
+        </is>
+      </c>
+      <c r="E835" s="2" t="inlineStr">
+        <is>
+          <t>마이크론 주가가 미국의 메모리 제품 수출 규제 가능성 및 수요 둔화로 하락했으며, 이는 반도체 시장 불균형을 시사한다.</t>
+        </is>
+      </c>
+      <c r="F835" s="2" t="inlineStr">
+        <is>
+          <t>주요 전자부품인 메모리 제품에 대한 미국의 수출 규제 가능성은 우리 회사의 부품 조달 및 생산 계획에 직접적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G835" s="2" t="inlineStr">
+        <is>
+          <t>주요 메모리 부품 공급망 현황 점검 및 대체 공급처 확보 가능성 검토.</t>
+        </is>
+      </c>
+      <c r="H835" s="2" t="inlineStr">
+        <is>
+          <t>TradingKey</t>
+        </is>
+      </c>
+      <c r="I835" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tradingkey.com/kr/news/market-movers/262032480-market-movers-mu-20260715</t>
+        </is>
+      </c>
+      <c r="J835" s="2" t="inlineStr">
+        <is>
+          <t>RSK-153</t>
+        </is>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B836" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C836" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D836" s="2" t="inlineStr">
+        <is>
+          <t>대통령 그 입 어떻게 안됩니까…‘호르무즈 통행료’ 번복한 트럼프</t>
+        </is>
+      </c>
+      <c r="E836" s="2" t="inlineStr">
+        <is>
+          <t>트럼프 전 대통령이 호르무즈 해협 통행료 부과 및 이란에 대한 해상 봉쇄 가능성을 언급하며 중동 원유 수출 전면 봉쇄를 예고했다.</t>
+        </is>
+      </c>
+      <c r="F836" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협은 주요 원유 수송로이자 글로벌 해상 물류의 핵심 통로로, 봉쇄 시 국제 유가 급등 및 해상 운송 지연/차질이 발생하여 물류 운영에 심각한 영향을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="G836" s="2" t="inlineStr">
+        <is>
+          <t>중동 정세 및 호르무즈 해협 관련 뉴스 실시간 모니터링, 해상 운송 경로 다변화 및 비상 운송 계획 수립 검토.</t>
+        </is>
+      </c>
+      <c r="H836" s="2" t="inlineStr">
+        <is>
+          <t>매일경제</t>
+        </is>
+      </c>
+      <c r="I836" s="2" t="inlineStr">
+        <is>
+          <t>https://mk.co.kr/news/world/12099613</t>
+        </is>
+      </c>
+      <c r="J836" s="2" t="inlineStr">
+        <is>
+          <t>RSK-154</t>
+        </is>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B837" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C837" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D837" s="2" t="inlineStr">
+        <is>
+          <t>유가 85달러 재돌파···항공사 실적 '비상'</t>
+        </is>
+      </c>
+      <c r="E837" s="2" t="inlineStr">
+        <is>
+          <t>미국과 이란 간 갈등 재점화로 국제유가가 85달러를 재돌파하며 항공사들의 유류비 부담이 커져 하반기 실적에 비상이 걸렸다.</t>
+        </is>
+      </c>
+      <c r="F837" s="2" t="inlineStr">
+        <is>
+          <t>국제유가 급등은 항공 운임 및 해상 운임의 유류할증료 상승으로 직결되어 우리 회사의 물류비용에 즉각적이고 직접적인 영향을 미친다.</t>
+        </is>
+      </c>
+      <c r="G837" s="2" t="inlineStr">
+        <is>
+          <t>항공/해상 운임 변동성 분석 및 물류비 예산 재조정, 운송사와의 계약 조건 재협상 검토.</t>
+        </is>
+      </c>
+      <c r="H837" s="2" t="inlineStr">
+        <is>
+          <t>뉴스웨이</t>
+        </is>
+      </c>
+      <c r="I837" s="2" t="inlineStr">
+        <is>
+          <t>https://newsway.co.kr/news/view?ud=2026071513415045833</t>
+        </is>
+      </c>
+      <c r="J837" s="2" t="inlineStr">
+        <is>
+          <t>RSK-155</t>
+        </is>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B838" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C838" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D838" s="3" t="inlineStr">
+        <is>
+          <t>U.S.-EU Trade Agreement Eliminates Duties on Most U.S. Goods Starting July 1; TPEB Rates Rise as July Capacity Hits Three-Year High</t>
+        </is>
+      </c>
+      <c r="E838" s="3" t="inlineStr">
+        <is>
+          <t>7월 1일부터 미국-EU 무역 협정 발효로 대부분의 미국산 공산품에 대한 관세가 철폐되었으며, 7월 운송 용량이 3년 내 최고치를 기록했음에도 태평양 횡단 동향(TPEB) 운임은 상승하고 있다.</t>
+        </is>
+      </c>
+      <c r="F838" s="3" t="inlineStr">
+        <is>
+          <t>미국-EU 관세 철폐는 해당 지역으로의 수출입 비용 절감 기회를 제공하지만, 우리 회사의 주요 교역국이 아니거나 품목에 따라 영향이 제한적일 수 있다. TPEB 운임 상승은 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G838" s="3" t="inlineStr">
+        <is>
+          <t>미국-EU 무역 협정의 세부 내용을 검토하여 우리 제품의 관세 혜택 여부 확인, TPEB 운임 추이 지속 모니터링.</t>
+        </is>
+      </c>
+      <c r="H838" s="3" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I838" s="3" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/july-02-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J838" s="3" t="inlineStr"/>
+    </row>
+    <row r="839">
+      <c r="A839" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B839" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C839" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D839" s="3" t="inlineStr">
+        <is>
+          <t>CAPE Phase 2 Launches June 29 for Reconciliation-Flagged Entries; TPEB Rates Rise 10% for Sixth Consecutive Week</t>
+        </is>
+      </c>
+      <c r="E839" s="3" t="inlineStr">
+        <is>
+          <t>CBP의 CAPE IEEPA 관세 환급 시스템 2단계가 6월 29일 발효되어 적용 대상이 확대되었으며, 태평양 횡단 동향(TPEB) 운임이 6주 연속 10% 상승했다.</t>
+        </is>
+      </c>
+      <c r="F839" s="3" t="inlineStr">
+        <is>
+          <t>CAPE 시스템 확장은 관세 환급 기회를 제공할 수 있으나, TPEB 운임의 지속적인 상승은 미주향 물류 비용에 부담을 줄 수 있어 추이를 면밀히 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G839" s="3" t="inlineStr">
+        <is>
+          <t>CAPE 2단계 적용 가능성 검토 및 관세 환급 기회 모색, TPEB 운임 상승에 대비한 운송 계약 및 예산 재검토.</t>
+        </is>
+      </c>
+      <c r="H839" s="3" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I839" s="3" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/june-25-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J839" s="3" t="inlineStr"/>
+    </row>
+    <row r="840">
+      <c r="A840" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B840" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C840" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D840" s="3" t="inlineStr">
+        <is>
+          <t>Air Cargo Demand Up 6.0% in May</t>
+        </is>
+      </c>
+      <c r="E840" s="3" t="inlineStr">
+        <is>
+          <t>IATA가 2026년 5월 전 세계 항공 화물 수요가 전년 동월 대비 6.0% 증가했다고 발표했다.</t>
+        </is>
+      </c>
+      <c r="F840" s="3" t="inlineStr">
+        <is>
+          <t>항공 화물 수요 증가는 향후 항공 운임 상승 압력으로 작용할 수 있으므로 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G840" s="3" t="inlineStr">
+        <is>
+          <t>항공 화물 운임 추이 및 공급망 상황 지속 모니터링.</t>
+        </is>
+      </c>
+      <c r="H840" s="3" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I840" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-29-air-cargo-demand-up-may/</t>
+        </is>
+      </c>
+      <c r="J840" s="3" t="inlineStr"/>
+    </row>
+    <row r="841">
+      <c r="A841" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B841" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C841" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D841" s="3" t="inlineStr">
+        <is>
+          <t>Structural Contraction of Global Liner Networks</t>
+        </is>
+      </c>
+      <c r="E841" s="3" t="inlineStr">
+        <is>
+          <t>IMF의 최신 보고서에 따르면 2026년 전 세계 무역량 성장률이 3.5%로 크게 둔화될 것으로 예상되며, 이는 글로벌 정기선 네트워크의 구조적 축소로 이어질 수 있다.</t>
+        </is>
+      </c>
+      <c r="F841" s="3" t="inlineStr">
+        <is>
+          <t>글로벌 무역량 성장 둔화와 정기선 네트워크 축소는 향후 해상 운송 용량 감소 및 운임 변동성 증가로 이어질 수 있어 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G841" s="3" t="inlineStr">
+        <is>
+          <t>글로벌 해상 운송 시장 동향 및 선사들의 운항 계획 변화 지속 모니터링.</t>
+        </is>
+      </c>
+      <c r="H841" s="3" t="inlineStr">
+        <is>
+          <t>sea-intelligence</t>
+        </is>
+      </c>
+      <c r="I841" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/398-structural-contraction-of-global-liner-network</t>
+        </is>
+      </c>
+      <c r="J841" s="3" t="inlineStr"/>
+    </row>
+    <row r="842">
+      <c r="A842" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B842" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C842" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D842" s="3" t="inlineStr">
+        <is>
+          <t>Structural Contraction of Global Liner Networks</t>
+        </is>
+      </c>
+      <c r="E842" s="3" t="inlineStr">
+        <is>
+          <t>글로벌 선사들이 네트워크를 관리하는 방식에 근본적인 변화가 있으며, 지리적 범위는 유지하지만 서비스 빈도가 감소하는 구조적 축소가 나타나고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F842" s="3" t="inlineStr">
+        <is>
+          <t>선사들의 서비스 빈도 감소는 장기적으로 운송 옵션 및 스케줄 유연성에 영향을 미칠 수 있으므로 추이를 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G842" s="3" t="n"/>
+      <c r="H842" s="3" t="inlineStr">
+        <is>
+          <t>sea-intelligence.com</t>
+        </is>
+      </c>
+      <c r="I842" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/397-structural-contraction-of-global-liner-networks</t>
+        </is>
+      </c>
+      <c r="J842" s="3" t="inlineStr"/>
+    </row>
+    <row r="843">
+      <c r="A843" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B843" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C843" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D843" s="3" t="inlineStr">
+        <is>
+          <t>PLSCI Data Indicates Mega-Hub Retrenchment</t>
+        </is>
+      </c>
+      <c r="E843" s="3" t="inlineStr">
+        <is>
+          <t>UNCTAD의 PLSCI 데이터 분석 결과, 최근 해운 네트워크 재조정이 메가 허브 항만의 연결성 후퇴로 이어지고 있음을 시사합니다.</t>
+        </is>
+      </c>
+      <c r="F843" s="3" t="inlineStr">
+        <is>
+          <t>주요 허브 항만의 연결성 변화는 우리 물류 경로 및 환적 효율성에 영향을 줄 수 있으므로 지속적인 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G843" s="3" t="n"/>
+      <c r="H843" s="3" t="inlineStr">
+        <is>
+          <t>sea-intelligence.com</t>
+        </is>
+      </c>
+      <c r="I843" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/396-plsci-data-indicates-mega-hub-retrenchment</t>
+        </is>
+      </c>
+      <c r="J843" s="3" t="inlineStr"/>
+    </row>
+    <row r="844">
+      <c r="A844" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B844" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C844" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D844" s="3" t="inlineStr">
+        <is>
+          <t>Tracking True Vessel Delay</t>
+        </is>
+      </c>
+      <c r="E844" s="3" t="inlineStr">
+        <is>
+          <t>선사들이 운송 시간을 늘리는 스케줄 버퍼링을 통해 선박의 조기 도착을 관리하고 있으며, 이는 실제 지연과 다르게 나타날 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="F844" s="3" t="inlineStr">
+        <is>
+          <t>선사들의 스케줄 버퍼링 전략은 공시된 운송 시간과 실제 도착 시간 간의 괴리를 발생시켜 운송 계획 수립에 영향을 줄 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G844" s="3" t="inlineStr">
+        <is>
+          <t>선사별 스케줄 버퍼링 경향을 파악하여 운송 리드타임 예측 정확도를 높이는 방안 검토.</t>
+        </is>
+      </c>
+      <c r="H844" s="3" t="inlineStr">
+        <is>
+          <t>sea-intelligence.com</t>
+        </is>
+      </c>
+      <c r="I844" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/394-tracking-true-vessel-delay</t>
+        </is>
+      </c>
+      <c r="J844" s="3" t="inlineStr"/>
+    </row>
+    <row r="845">
+      <c r="A845" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B845" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C845" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D845" s="3" t="inlineStr">
+        <is>
+          <t>23조 원 투자도 상황 바꾸긴 어렵다? HMM 주가 힘 못 받는 이유</t>
+        </is>
+      </c>
+      <c r="E845" s="3" t="inlineStr">
+        <is>
+          <t>해상 운임 흐름이 우호적이지 않아 대규모 투자에도 HMM 주가가 탄력을 받기 어렵다는 분석이 나왔습니다.</t>
+        </is>
+      </c>
+      <c r="F845" s="3" t="inlineStr">
+        <is>
+          <t>해상 운임 흐름이 불우호적이라는 분석은 전반적인 해상 운임 시장의 약세를 시사하며, 향후 우리 운송 비용에 영향을 줄 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G845" s="3" t="inlineStr">
+        <is>
+          <t>해상 운임 지수 및 시장 동향을 지속적으로 모니터링하고, 운송 계약 시 운임 협상 전략을 검토합니다.</t>
+        </is>
+      </c>
+      <c r="H845" s="3" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I845" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260716-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J845" s="3" t="inlineStr"/>
+    </row>
+    <row r="846">
+      <c r="A846" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B846" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C846" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D846" s="3" t="inlineStr">
+        <is>
+          <t>"비싸도 지금 산다"...호르무즈 장기화에 VLCC 발주 사상 최대</t>
+        </is>
+      </c>
+      <c r="E846" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 불확실성 장기화에 대비하여 글로벌 선주들이 초대형 원유운반선(VLCC) 확보에 속도를 내며 발주량이 사상 최대를 기록하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F846" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 사태 장기화에 대한 시장의 대응으로, 유조선 시장에 영향을 주지만 우리 배터리/전자부품 운송에는 간접적인 영향이므로 추이를 모니터링합니다.</t>
+        </is>
+      </c>
+      <c r="G846" s="3" t="n"/>
+      <c r="H846" s="3" t="inlineStr">
+        <is>
+          <t>ebn.co.kr</t>
+        </is>
+      </c>
+      <c r="I846" s="3" t="inlineStr">
+        <is>
+          <t>https://ebn.co.kr/news/articleView.html?idxno=1716474</t>
+        </is>
+      </c>
+      <c r="J846" s="3" t="inlineStr"/>
+    </row>
+    <row r="847">
+      <c r="A847" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B847" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C847" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D847" s="3" t="inlineStr">
+        <is>
+          <t>FedEx CEO says we are in the middle of the biggest supply chain shift he’s seen in 35 years: ‘We are the referendum’</t>
+        </is>
+      </c>
+      <c r="E847" s="3" t="inlineStr">
+        <is>
+          <t>FedEx CEO는 예측 불가능한 관세와 글로벌 공급망의 변화 속에서 지난 35년간 가장 큰 공급망 변화의 한가운데에 있다고 언급하며, 기업들이 공급망 재편에 집중하고 있음을 시사했습니다.</t>
+        </is>
+      </c>
+      <c r="F847" s="3" t="inlineStr">
+        <is>
+          <t>글로벌 공급망의 구조적 변화는 장기적으로 우리 물류 전략에 영향을 미칠 수 있으므로, 변화의 방향과 주요 동인을 지속적으로 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G847" s="3" t="inlineStr">
+        <is>
+          <t>글로벌 공급망 재편 동향 분석 및 우리 기업의 공급망 탄력성 강화 방안 검토.</t>
+        </is>
+      </c>
+      <c r="H847" s="3" t="inlineStr">
+        <is>
+          <t>fortune.com</t>
+        </is>
+      </c>
+      <c r="I847" s="3" t="inlineStr">
+        <is>
+          <t>https://fortune.com/2026/07/15/fedex-ceo-raj-subramaniam-tariffs-supply-chain-shipping-fortune-500-titans-and-disruptors-of-industry</t>
+        </is>
+      </c>
+      <c r="J847" s="3" t="inlineStr"/>
+    </row>
+    <row r="848">
+      <c r="A848" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B848" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C848" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D848" s="3" t="inlineStr">
+        <is>
+          <t>Distribution and supply chain under pressure: how the channel is rewriting the rules</t>
+        </is>
+      </c>
+      <c r="E848" s="3" t="inlineStr">
+        <is>
+          <t>기업들이 제3자 공급업체에 대한 과도한 의존을 줄이고 공급망을 단축하며 리쇼어링을 통해 공급망 탄력성을 강화하는 데 집중하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F848" s="3" t="inlineStr">
+        <is>
+          <t>공급망 탄력성 강화 및 리쇼어링 추세는 우리 기업의 생산 및 물류 네트워크 전략에 중장기적인 영향을 미칠 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G848" s="3" t="inlineStr">
+        <is>
+          <t>공급망 리스크 분산 및 지역화 전략 검토, 핵심 부품의 재고 정책 재평가.</t>
+        </is>
+      </c>
+      <c r="H848" s="3" t="inlineStr">
+        <is>
+          <t>eenewseurope.com</t>
+        </is>
+      </c>
+      <c r="I848" s="3" t="inlineStr">
+        <is>
+          <t>https://www.eenewseurope.com/en/distribution-and-supply-chain-under-pressure-how-the-channel-is-rewriting-the-rules/</t>
+        </is>
+      </c>
+      <c r="J848" s="3" t="inlineStr"/>
+    </row>
+    <row r="849">
+      <c r="A849" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B849" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C849" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D849" s="3" t="inlineStr">
+        <is>
+          <t>KFC Faces Supply Chain Disruption in Japan Due to Cyberattack</t>
+        </is>
+      </c>
+      <c r="E849" s="3" t="inlineStr">
+        <is>
+          <t>KFC Japan은 물류 파트너의 시스템 장애로 인해 전국 매장으로의 식품 공급이 중단되는 공급망 차질을 겪고 있다고 발표했다.</t>
+        </is>
+      </c>
+      <c r="F849" s="3" t="inlineStr">
+        <is>
+          <t>물류 파트너에 대한 사이버 공격은 공급망을 심각하게 교란할 수 있으므로, 당사 물류 네트워크 내 사이버 보안 위험에 대한 경계가 필요하다.</t>
+        </is>
+      </c>
+      <c r="G849" s="3" t="inlineStr">
+        <is>
+          <t>당사 물류 파트너들의 사이버 보안 역량을 점검하고, 잠재적 위험에 대비한 비상 계획을 수립한다.</t>
+        </is>
+      </c>
+      <c r="H849" s="3" t="inlineStr">
+        <is>
+          <t>Gurufocus</t>
+        </is>
+      </c>
+      <c r="I849" s="3" t="inlineStr">
+        <is>
+          <t>https://www.gurufocus.com/news/8959056/kfc-faces-supply-chain-disruption-in-japan-due-to-cyberattack</t>
+        </is>
+      </c>
+      <c r="J849" s="3" t="inlineStr"/>
+    </row>
+    <row r="850">
+      <c r="A850" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B850" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C850" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D850" s="3" t="inlineStr">
+        <is>
+          <t>위생용품·의료기기·보호장비 수입요건 확인 강화 &lt; 경제 일반 &lt; 경제 &lt; 기사본문 - 시사저널</t>
+        </is>
+      </c>
+      <c r="E850" s="3" t="inlineStr">
+        <is>
+          <t>관세청이 국민 건강과 산업 안전, 생태계를 위협하는 물품에 대한 수입 요건 확인을 강화하여, 위생용품, 의료기기, 보호장비 등의 수입 절차가 엄격해진다.</t>
+        </is>
+      </c>
+      <c r="F850" s="3" t="inlineStr">
+        <is>
+          <t>'산업 안전 물품'에 대한 수입 요건 강화 추세는 배터리 등 당사 제품에도 확대 적용될 가능성이 있어, 향후 규제 변화를 주시해야 한다.</t>
+        </is>
+      </c>
+      <c r="G850" s="3" t="inlineStr">
+        <is>
+          <t>당사 제품의 수입 요건에 대한 최신 정보를 지속적으로 확인하고, 관련 규제 변화 시 선제적으로 대응할 준비를 한다.</t>
+        </is>
+      </c>
+      <c r="H850" s="3" t="inlineStr">
+        <is>
+          <t>시사저널</t>
+        </is>
+      </c>
+      <c r="I850" s="3" t="inlineStr">
+        <is>
+          <t>https://sisajournal.com/news/articleView.html?idxno=380007</t>
+        </is>
+      </c>
+      <c r="J850" s="3" t="inlineStr"/>
+    </row>
+    <row r="851">
+      <c r="A851" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B851" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C851" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D851" s="3" t="inlineStr">
+        <is>
+          <t>美상원, 중국 등 러시아 원유 구매국에 최대 100% 관세 추진</t>
+        </is>
+      </c>
+      <c r="E851" s="3" t="inlineStr">
+        <is>
+          <t>미국 상원이 러시아 에너지 수입국(중국 등)에 최대 100% 관세를 부과하는 대러 제재안을 추진 중이다.</t>
+        </is>
+      </c>
+      <c r="F851" s="3" t="inlineStr">
+        <is>
+          <t>러시아 원유 구매국에 대한 관세 부과는 국제 유가 및 에너지 시장에 간접적인 영향을 미쳐 물류비 변동 가능성을 높이지만, 배터리/전자부품 물류에 직접적인 영향은 낮다.</t>
+        </is>
+      </c>
+      <c r="G851" s="3" t="inlineStr">
+        <is>
+          <t>없음</t>
+        </is>
+      </c>
+      <c r="H851" s="3" t="inlineStr">
+        <is>
+          <t>연합뉴스</t>
+        </is>
+      </c>
+      <c r="I851" s="3" t="inlineStr">
+        <is>
+          <t>https://yna.co.kr/view/AKR20260715037300009</t>
+        </is>
+      </c>
+      <c r="J851" s="3" t="inlineStr"/>
+    </row>
+    <row r="852">
+      <c r="A852" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B852" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C852" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D852" s="3" t="inlineStr">
+        <is>
+          <t>반도체 규제 완화 ‘선물 보따리’ 받은 UAE···전쟁서 미국 편에 선 대가?</t>
+        </is>
+      </c>
+      <c r="E852" s="3" t="inlineStr">
+        <is>
+          <t>미국이 이란과의 분쟁에서 미국 편에 선 아랍에미리트(UAE)에 인공지능(AI) 반도체 수출 규제를 완화했다.</t>
+        </is>
+      </c>
+      <c r="F852" s="3" t="inlineStr">
+        <is>
+          <t>미국의 반도체 수출 규제 정책이 지정학적 상황에 따라 유동적으로 변화함을 보여주며, 향후 우리 회사의 수출입 전략에 영향을 줄 수 있어 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G852" s="3" t="inlineStr">
+        <is>
+          <t>없음</t>
+        </is>
+      </c>
+      <c r="H852" s="3" t="inlineStr">
+        <is>
+          <t>경향신문</t>
+        </is>
+      </c>
+      <c r="I852" s="3" t="inlineStr">
+        <is>
+          <t>https://www.khan.co.kr/article/202607151422011/</t>
+        </is>
+      </c>
+      <c r="J852" s="3" t="inlineStr"/>
+    </row>
+    <row r="853">
+      <c r="A853" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B853" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C853" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D853" s="3" t="inlineStr">
+        <is>
+          <t>엔비디아, H200 중국 출하 시작…美 “수량은 매우 적다”</t>
+        </is>
+      </c>
+      <c r="E853" s="3" t="inlineStr">
+        <is>
+          <t>엔비디아의 첨단 AI 칩 H200이 중국으로 출하되기 시작했으나, 미국은 수량이 매우 적다고 밝혀 대중 수출 통제의 실효성에 대한 논의가 지속되고 있다.</t>
+        </is>
+      </c>
+      <c r="F853" s="3" t="inlineStr">
+        <is>
+          <t>주요 전자부품의 대중국 수출 규제 및 그 실효성 논란은 글로벌 전자부품 공급망의 불확실성을 높이며, 향후 규제 강화 시 우리 회사의 중국향 수출 또는 중국 내 생산에 영향을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="G853" s="3" t="inlineStr">
+        <is>
+          <t>없음</t>
+        </is>
+      </c>
+      <c r="H853" s="3" t="inlineStr">
+        <is>
+          <t>시사저널</t>
+        </is>
+      </c>
+      <c r="I853" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sisajournal.com/news/articleView.html?idxno=379878</t>
+        </is>
+      </c>
+      <c r="J853" s="3" t="inlineStr"/>
+    </row>
+    <row r="854">
+      <c r="A854" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B854" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C854" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D854" s="3" t="inlineStr">
+        <is>
+          <t>韓총리 "국제유가 공급망 불안 상수로 보고 장단기 대책 추진해야"</t>
+        </is>
+      </c>
+      <c r="E854" s="3" t="inlineStr">
+        <is>
+          <t>한 총리는 미국-이란 무력 충돌 재반복 등 국제유가 공급망 불안을 상수로 보고 장단기 대책을 추진해야 한다고 강조했다.</t>
+        </is>
+      </c>
+      <c r="F854" s="3" t="inlineStr">
+        <is>
+          <t>국제유가 불안정은 해상/항공 운임 상승으로 이어져 물류비용에 직접적인 영향을 미치므로, 장기적인 관점에서 유가 변동에 대한 대비책 마련이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G854" s="3" t="inlineStr">
+        <is>
+          <t>유가 변동에 따른 물류비 예산 영향 분석 및 운송 계약 조건 재검토.</t>
+        </is>
+      </c>
+      <c r="H854" s="3" t="inlineStr">
+        <is>
+          <t>파이낸셜뉴스</t>
+        </is>
+      </c>
+      <c r="I854" s="3" t="inlineStr">
+        <is>
+          <t>https://fnnews.com/news/202607151018319744</t>
+        </is>
+      </c>
+      <c r="J854" s="3" t="inlineStr"/>
+    </row>
+    <row r="855">
+      <c r="A855" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B855" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C855" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D855" s="3" t="inlineStr">
+        <is>
+          <t>대한항공, 8월 유류할증료 25%↓…미·이란 갈등에 9월은 불투명</t>
+        </is>
+      </c>
+      <c r="E855" s="3" t="inlineStr">
+        <is>
+          <t>대한항공의 8월 국제선 유류할증료가 25% 하향 조정되었으나, 미국-이란 갈등으로 9월 이후 유류할증료는 불투명하다.</t>
+        </is>
+      </c>
+      <c r="F855" s="3" t="inlineStr">
+        <is>
+          <t>단기적으로 항공 운임 부담이 완화되지만, 중동 지정학적 리스크로 인한 유가 변동성이 커 9월 이후 항공 운임 상승 가능성이 높아 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G855" s="3" t="inlineStr">
+        <is>
+          <t>항공 운송 비중 및 비용 재검토, 9월 이후 유류할증료 변동 추이 주시.</t>
+        </is>
+      </c>
+      <c r="H855" s="3" t="inlineStr">
+        <is>
+          <t>머니투데이</t>
+        </is>
+      </c>
+      <c r="I855" s="3" t="inlineStr">
+        <is>
+          <t>https://mt.co.kr/industry/2026/07/16/2026071613284167931</t>
+        </is>
+      </c>
+      <c r="J855" s="3" t="inlineStr"/>
+    </row>
+    <row r="856">
+      <c r="A856" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B856" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C856" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D856" s="3" t="inlineStr">
+        <is>
+          <t>8월에 사면 '최대 17만 원' 절약…대한항공 국제선 유류할증료 또 내린다 | 위키트리</t>
+        </is>
+      </c>
+      <c r="E856" s="3" t="inlineStr">
+        <is>
+          <t>국제 항공유 가격 하락으로 8월 국제선 유류할증료가 3개월 연속 인하되며, 장거리 노선에서 최대 17만 원의 비용 절감이 예상됩니다.</t>
+        </is>
+      </c>
+      <c r="F856" s="3" t="inlineStr">
+        <is>
+          <t>항공 운송 비용의 주요 구성 요소인 유류할증료 인하는 물류비 절감 기회로 작용할 수 있으므로 지속적인 추이 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G856" s="3" t="inlineStr">
+        <is>
+          <t>항공 운송 비용 절감 기회를 파악하고, 운송사와의 계약 조건 검토 및 향후 항공 운송 계획에 반영을 고려합니다.</t>
+        </is>
+      </c>
+      <c r="H856" s="3" t="inlineStr">
+        <is>
+          <t>위키트리</t>
+        </is>
+      </c>
+      <c r="I856" s="3" t="inlineStr">
+        <is>
+          <t>https://wikitree.co.kr/articles/1146870</t>
+        </is>
+      </c>
+      <c r="J856" s="3" t="inlineStr"/>
+    </row>
+    <row r="857">
+      <c r="A857" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B857" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C857" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D857" s="4" t="inlineStr">
+        <is>
+          <t>SV, 11월 RUH-NRT노선 주3편 운항</t>
+        </is>
+      </c>
+      <c r="E857" s="4" t="inlineStr">
+        <is>
+          <t>사우디아라비아항공이 11월 17일부터 리야드-나리타 노선에 주 3회 B787-9 화물기를 운항할 예정이다.</t>
+        </is>
+      </c>
+      <c r="F857" s="4" t="inlineStr">
+        <is>
+          <t>우리 회사의 주요 운송 경로와 직접적인 관련이 없으며, 추가적인 항공 화물 노선은 전반적인 운송 옵션 증가에 기여할 수 있으나 당장 큰 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G857" s="4" t="inlineStr"/>
+      <c r="H857" s="4" t="inlineStr">
+        <is>
+          <t>cargonews</t>
+        </is>
+      </c>
+      <c r="I857" s="4" t="inlineStr">
+        <is>
+          <t>https://www.cargonews.co.kr/news/articleView.html?idxno=60534</t>
+        </is>
+      </c>
+      <c r="J857" s="4" t="inlineStr"/>
+    </row>
+    <row r="858">
+      <c r="A858" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B858" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C858" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D858" s="4" t="inlineStr">
+        <is>
+          <t>IATA Releases 2025 World Air Transport Statistics</t>
+        </is>
+      </c>
+      <c r="E858" s="4" t="inlineStr">
+        <is>
+          <t>IATA가 2025년까지의 전 세계 항공 운송 통계를 담은 최신 보고서를 발표했다.</t>
+        </is>
+      </c>
+      <c r="F858" s="4" t="inlineStr">
+        <is>
+          <t>과거 데이터 및 통계 보고서 발표는 현재 물류 운영에 직접적인 영향을 미치지 않으며, 참고 자료 수준이다.</t>
+        </is>
+      </c>
+      <c r="G858" s="4" t="inlineStr"/>
+      <c r="H858" s="4" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I858" s="4" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/07-16-iata-releases-2025-world-air-transport-statistics-report/</t>
+        </is>
+      </c>
+      <c r="J858" s="4" t="inlineStr"/>
+    </row>
+    <row r="859">
+      <c r="A859" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B859" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C859" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D859" s="4" t="inlineStr">
+        <is>
+          <t>IATA Guidance Supports Clearer and More Consistent In-Cabin Pet Travel</t>
+        </is>
+      </c>
+      <c r="E859" s="4" t="inlineStr">
+        <is>
+          <t>IATA가 기내 반려동물 운송에 대한 명확하고 일관된 운영 지침을 발표했다.</t>
+        </is>
+      </c>
+      <c r="F859" s="4" t="inlineStr">
+        <is>
+          <t>반려동물 운송 지침은 우리 회사의 화물 운송과는 무관하다.</t>
+        </is>
+      </c>
+      <c r="G859" s="4" t="inlineStr"/>
+      <c r="H859" s="4" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I859" s="4" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/07-15-iata-guidance-supports-clearer-more-consistent-in-cabin-pet-travel/</t>
+        </is>
+      </c>
+      <c r="J859" s="4" t="inlineStr"/>
+    </row>
+    <row r="860">
+      <c r="A860" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B860" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C860" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D860" s="4" t="inlineStr">
+        <is>
+          <t>Air Passenger Demand Falls 2.2% in May</t>
+        </is>
+      </c>
+      <c r="E860" s="4" t="inlineStr">
+        <is>
+          <t>IATA가 2026년 5월 전 세계 항공 여객 수요가 전년 동월 대비 2.2% 감소했다고 발표했다.</t>
+        </is>
+      </c>
+      <c r="F860" s="4" t="inlineStr">
+        <is>
+          <t>여객 수요 감소는 항공 화물 운송에 간접적인 영향을 줄 수 있으나, 직접적인 화물 운송 수요나 비용에 대한 정보가 아니므로 당장 큰 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G860" s="4" t="inlineStr"/>
+      <c r="H860" s="4" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I860" s="4" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-30-air-passenger-demand-falls-may/</t>
+        </is>
+      </c>
+      <c r="J860" s="4" t="inlineStr"/>
+    </row>
+    <row r="861">
+      <c r="A861" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B861" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C861" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D861" s="4" t="inlineStr">
+        <is>
+          <t>IATA and IATP Collaborate to Support Airline Supply Chain Resilience</t>
+        </is>
+      </c>
+      <c r="E861" s="4" t="inlineStr">
+        <is>
+          <t>IATA와 IATP가 항공기 부품 가시성 및 접근성 개선을 통해 항공사 공급망 복원력 강화를 위해 협력하기로 합의했다.</t>
+        </is>
+      </c>
+      <c r="F861" s="4" t="inlineStr">
+        <is>
+          <t>항공사 자체의 공급망 복원력 강화는 간접적으로 항공 화물 서비스 안정성에 기여할 수 있으나, 우리 회사의 직접적인 물류 운영에 미치는 영향은 미미하다.</t>
+        </is>
+      </c>
+      <c r="G861" s="4" t="inlineStr"/>
+      <c r="H861" s="4" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I861" s="4" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-25-iata-iatp-collaborate-support-airline-supply-chain-resilience/</t>
+        </is>
+      </c>
+      <c r="J861" s="4" t="inlineStr"/>
+    </row>
+    <row r="862">
+      <c r="A862" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B862" s="4" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C862" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D862" s="4" t="inlineStr">
+        <is>
+          <t>트럼프 “지역 밖에서 만들어진 선박도 구매…한국기업 살펴볼 것”</t>
+        </is>
+      </c>
+      <c r="E862" s="4" t="inlineStr">
+        <is>
+          <t>트럼프 전 대통령이 미 해군력 강화를 위해 한국 등 우방국 조선업계와의 협력 확대를 시사했다.</t>
+        </is>
+      </c>
+      <c r="F862" s="4" t="inlineStr">
+        <is>
+          <t>조선업계 협력은 장기적인 산업 정책에 해당하며, 우리 회사의 단기 물류 운영에 직접적인 영향을 미치지 않는다.</t>
+        </is>
+      </c>
+      <c r="G862" s="4" t="inlineStr"/>
+      <c r="H862" s="4" t="inlineStr">
+        <is>
+          <t>kita</t>
+        </is>
+      </c>
+      <c r="I862" s="4" t="inlineStr">
+        <is>
+          <t>https://www.kita.net/shippers/board/newsView.do?morgueCode=2&amp;dataCls=B&amp;dataSeq=8168</t>
+        </is>
+      </c>
+      <c r="J862" s="4" t="inlineStr"/>
+    </row>
+    <row r="863">
+      <c r="A863" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B863" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C863" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D863" s="4" t="inlineStr">
+        <is>
+          <t>여수광양항, 북극항로 연계 에너지 물류 허브 구축</t>
+        </is>
+      </c>
+      <c r="E863" s="4" t="inlineStr">
+        <is>
+          <t>여수광양항만공사가 포스코플로우 등과 협력하여 북극항로 시대에 대비한 에너지 물류 허브 구축을 위한 업무협약을 체결했다.</t>
+        </is>
+      </c>
+      <c r="F863" s="4" t="inlineStr">
+        <is>
+          <t>북극항로 연계 에너지 물류 허브 구축은 장기적인 국가 및 지역 물류 인프라 계획으로, 우리 회사의 현재 배터리/전자부품 물류 운영에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G863" s="4" t="inlineStr"/>
+      <c r="H863" s="4" t="inlineStr">
+        <is>
+          <t>ksg</t>
+        </is>
+      </c>
+      <c r="I863" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksg.co.kr/news/main_newsView.jsp?pNum=147647</t>
+        </is>
+      </c>
+      <c r="J863" s="4" t="inlineStr"/>
+    </row>
+    <row r="864">
+      <c r="A864" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B864" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C864" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D864" s="4" t="inlineStr">
+        <is>
+          <t>Global Schedule Reliability for May 2026 the Highest of the Year</t>
+        </is>
+      </c>
+      <c r="E864" s="4" t="inlineStr">
+        <is>
+          <t>2026년 5월 글로벌 선박 스케줄 신뢰도가 올해 최고치를 기록하며 전반적인 해운 서비스의 정시성이 개선되고 있음을 보여줍니다.</t>
+        </is>
+      </c>
+      <c r="F864" s="4" t="inlineStr">
+        <is>
+          <t>스케줄 신뢰도 개선은 긍정적인 신호이나, 단기적인 수치이며 우리 물류 운영에 즉각적인 큰 영향은 없습니다.</t>
+        </is>
+      </c>
+      <c r="G864" s="4" t="n"/>
+      <c r="H864" s="4" t="inlineStr">
+        <is>
+          <t>sea-intelligence.com</t>
+        </is>
+      </c>
+      <c r="I864" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/395-global-schedule-reliability-for-may-2026-the-highest-of-the-year</t>
+        </is>
+      </c>
+      <c r="J864" s="4" t="inlineStr"/>
+    </row>
+    <row r="865">
+      <c r="A865" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B865" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C865" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D865" s="4" t="inlineStr">
+        <is>
+          <t>한국해양대, ‘디지털조선소 전문인력양성사업’ 선정…5년간 180억 원 투입</t>
+        </is>
+      </c>
+      <c r="E865" s="4" t="inlineStr">
+        <is>
+          <t>한국해양대학교가 산업통상자원부의 디지털 조선소 전문인력 양성사업에 선정되어 5년간 180억 원을 투입, AI 기반 해운·물류 분야 인재를 양성합니다.</t>
+        </is>
+      </c>
+      <c r="F865" s="4" t="inlineStr">
+        <is>
+          <t>장기적인 산업 인프라 강화 소식이지만, 우리 기업의 단기 물류 운영에 직접적인 영향은 없습니다.</t>
+        </is>
+      </c>
+      <c r="G865" s="4" t="n"/>
+      <c r="H865" s="4" t="inlineStr">
+        <is>
+          <t>shippingnewsnet.com</t>
+        </is>
+      </c>
+      <c r="I865" s="4" t="inlineStr">
+        <is>
+          <t>https://www.shippingnewsnet.com/news/articleView.html?idxno=71212</t>
+        </is>
+      </c>
+      <c r="J865" s="4" t="inlineStr"/>
+    </row>
+    <row r="866">
+      <c r="A866" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B866" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C866" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D866" s="4" t="inlineStr">
+        <is>
+          <t>광양시, 농식품 수출 경쟁력 강화에 4,200만 원 지원</t>
+        </is>
+      </c>
+      <c r="E866" s="4" t="inlineStr">
+        <is>
+          <t>광양시가 농식품 수출 경쟁력 강화를 위해 수출 컨테이너 내륙 운임, 포장재, 해외 인증 등 6개 사업에 총 4,200만 원을 지원합니다.</t>
+        </is>
+      </c>
+      <c r="F866" s="4" t="inlineStr">
+        <is>
+          <t>지역 농식품 수출 지원 정책으로, 우리 기업의 물류 운영에 직접적인 영향은 없습니다.</t>
+        </is>
+      </c>
+      <c r="G866" s="4" t="n"/>
+      <c r="H866" s="4" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I866" s="4" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260717-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J866" s="4" t="inlineStr"/>
+    </row>
+    <row r="867">
+      <c r="A867" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B867" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C867" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D867" s="4" t="inlineStr">
+        <is>
+          <t>‘AI 시대, 해양의 미래’…제7회 인천국제해양포럼 개막</t>
+        </is>
+      </c>
+      <c r="E867" s="4" t="inlineStr">
+        <is>
+          <t>인천국제해양포럼에서 AI 기반 해상운송과 물류 네트워크 최적화 등 해운·물류 분야의 미래 전략이 논의되었습니다.</t>
+        </is>
+      </c>
+      <c r="F867" s="4" t="inlineStr">
+        <is>
+          <t>AI 기반 물류 기술 논의는 장기적인 관점에서 중요하나, 당장 우리 물류 운영에 직접적인 영향은 없습니다.</t>
+        </is>
+      </c>
+      <c r="G867" s="4" t="n"/>
+      <c r="H867" s="4" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I867" s="4" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260716-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J867" s="4" t="inlineStr"/>
+    </row>
+    <row r="868">
+      <c r="A868" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B868" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C868" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D868" s="4" t="inlineStr">
+        <is>
+          <t>광양항이 증명한 국가전략, 이제는 '영일만항'</t>
+        </is>
+      </c>
+      <c r="E868" s="4" t="inlineStr">
+        <is>
+          <t>물류비 절감과 화물 흐름 재편이 항만산업 판도를 바꿀 수 있어 영일만항의 중요성이 부각되고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F868" s="4" t="inlineStr">
+        <is>
+          <t>국내 항만 경쟁력 강화 및 화물 흐름 재편 논의는 장기적인 관점에서 중요하나, 우리 기업의 단기 물류 운영에 직접적인 영향은 없습니다.</t>
+        </is>
+      </c>
+      <c r="G868" s="4" t="n"/>
+      <c r="H868" s="4" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I868" s="4" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260716-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J868" s="4" t="inlineStr"/>
+    </row>
+    <row r="869">
+      <c r="A869" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B869" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C869" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D869" s="4" t="inlineStr">
+        <is>
+          <t>영남이공대, '교육 넘어 채용까지'…쿠팡과 손잡고 AI 물류인재 키운다</t>
+        </is>
+      </c>
+      <c r="E869" s="4" t="inlineStr">
+        <is>
+          <t>영남이공대학교가 쿠팡풀필먼트서비스와 협력하여 AI 기반 물류 전문 교육과 취업을 연계하는 현장형 인재 양성에 나섭니다.</t>
+        </is>
+      </c>
+      <c r="F869" s="4" t="inlineStr">
+        <is>
+          <t>AI 물류 인재 양성은 산업 전반에 긍정적이나, 우리 기업의 단기 물류 운영에 직접적인 영향은 없습니다.</t>
+        </is>
+      </c>
+      <c r="G869" s="4" t="n"/>
+      <c r="H869" s="4" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I869" s="4" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260715-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J869" s="4" t="inlineStr"/>
+    </row>
+    <row r="870">
+      <c r="A870" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B870" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C870" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D870" s="4" t="inlineStr">
+        <is>
+          <t>상하이, 런던 제치고 세계 2위 해운 중심지 등극… ‘물동량’ 넘어 ‘...</t>
+        </is>
+      </c>
+      <c r="E870" s="4" t="inlineStr">
+        <is>
+          <t>상하이가 컨테이너 물동량뿐 아니라 금융·법률·조선 등 해운 관련 서비스 분야에서도 성장하며 세계 2위 해운 중심지로 등극했습니다.</t>
+        </is>
+      </c>
+      <c r="F870" s="4" t="inlineStr">
+        <is>
+          <t>상하이의 해운 중심지 위상 강화는 아시아 지역 물류 인프라에 긍정적이나, 우리 기업의 단기 물류 운영에 직접적인 영향은 없습니다.</t>
+        </is>
+      </c>
+      <c r="G870" s="4" t="n"/>
+      <c r="H870" s="4" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I870" s="4" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260714-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J870" s="4" t="inlineStr"/>
+    </row>
+    <row r="871">
+      <c r="A871" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B871" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C871" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D871" s="4" t="inlineStr">
+        <is>
+          <t>올 상반기 PCTC 발주량 29척, 전년 동기 2척에서 '급반등'</t>
+        </is>
+      </c>
+      <c r="E871" s="4" t="inlineStr">
+        <is>
+          <t>중국 자동차 수출 증가에 힘입어 자동차운반선(PCTC) 신조 발주량이 올해 상반기 급증하며 선복 확보 경쟁이 심화되고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F871" s="4" t="inlineStr">
+        <is>
+          <t>자동차 운반선 발주 증가는 특정 산업 분야의 선복 수요 증가를 나타내며, 우리 배터리/전자부품 물류에는 직접적인 영향이 없습니다.</t>
+        </is>
+      </c>
+      <c r="G871" s="4" t="n"/>
+      <c r="H871" s="4" t="inlineStr">
+        <is>
+          <t>oceanpress.co.kr</t>
+        </is>
+      </c>
+      <c r="I871" s="4" t="inlineStr">
+        <is>
+          <t>https://oceanpress.co.kr/news/article.html?no=30625</t>
+        </is>
+      </c>
+      <c r="J871" s="4" t="inlineStr"/>
+    </row>
+    <row r="872">
+      <c r="A872" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B872" s="4" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C872" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D872" s="4" t="inlineStr">
+        <is>
+          <t>장금마리타임, 그리스서 유조선 1년 용선…VLCC 선대 확장</t>
+        </is>
+      </c>
+      <c r="E872" s="4" t="inlineStr">
+        <is>
+          <t>장금마리타임이 미국-이란 갈등 장기화로 인한 고운임에 대응하여 그리스에서 초대형 유조선(VLCC)을 1년 용선하며 선대를 확장하고 있다.</t>
+        </is>
+      </c>
+      <c r="F872" s="4" t="inlineStr">
+        <is>
+          <t>유조선 용선은 주로 원유 운송 시장에 영향을 미치며, 우리 회사의 배터리/전자부품 운송에는 직접적인 영향이 적다. 다만, 고운임 추세는 전반적인 해운 시장에 영향을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="G872" s="4" t="inlineStr">
+        <is>
+          <t>없음</t>
+        </is>
+      </c>
+      <c r="H872" s="4" t="inlineStr">
+        <is>
+          <t>더구루</t>
+        </is>
+      </c>
+      <c r="I872" s="4" t="inlineStr">
+        <is>
+          <t>https://view.mk.co.kr/car-tech/article/250149</t>
+        </is>
+      </c>
+      <c r="J872" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -39538,7 +41718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -40345,6 +42525,49 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>3184.82</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>-142 (-4.3%)</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>+1,323 (+71.1%)</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="n">
+        <v>4318</v>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>-12 (-0.3%)</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>+1,728 (+66.7%)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -40357,7 +42580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I145"/>
+  <dimension ref="A1:I156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -45458,6 +47681,391 @@
       </c>
       <c r="I145" s="6" t="inlineStr"/>
     </row>
+    <row r="146">
+      <c r="A146" s="6" t="inlineStr">
+        <is>
+          <t>RSK-145</t>
+        </is>
+      </c>
+      <c r="B146" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C146" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D146" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E146" s="6" t="inlineStr">
+        <is>
+          <t>Section 301 Tariffs on Brazil Take Effect July 22, Stacking with Section 122 Duties; Strait of Hormuz Closure Restricts 200K TEU of Ocean Capacity</t>
+        </is>
+      </c>
+      <c r="F146" s="6" t="inlineStr"/>
+      <c r="G146" s="6" t="inlineStr"/>
+      <c r="H146" s="6" t="inlineStr">
+        <is>
+          <t>중동발 원자재 및 유럽/아시아향 해상 운송 경로 다변화 및 대체 운송 수단 검토, 브라질 및 러시아 관련 공급망 점검 및 관세 영향 분석.</t>
+        </is>
+      </c>
+      <c r="I146" s="6" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="6" t="inlineStr">
+        <is>
+          <t>RSK-146</t>
+        </is>
+      </c>
+      <c r="B147" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C147" s="6" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="D147" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E147" s="6" t="inlineStr">
+        <is>
+          <t>CBP Rejects Warehouse Entries on CAPE Declarations, Risking IEEPA Refunds; TPEB Rates Climb as Panama Canal Restrictions Tighten Capacity</t>
+        </is>
+      </c>
+      <c r="F147" s="6" t="inlineStr"/>
+      <c r="G147" s="6" t="inlineStr"/>
+      <c r="H147" s="6" t="inlineStr">
+        <is>
+          <t>파나마 운하 대체 경로 및 운송 수단 검토, CBP 통관 절차 및 CAPE 관련 규정 준수 여부 재확인 및 대응 방안 마련.</t>
+        </is>
+      </c>
+      <c r="I147" s="6" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="6" t="inlineStr">
+        <is>
+          <t>RSK-147</t>
+        </is>
+      </c>
+      <c r="B148" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C148" s="6" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="D148" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E148" s="6" t="inlineStr">
+        <is>
+          <t>CPSC Mandatory eFiling Takes Effect July 8; TPEB Rates Surge ~10% as Peak Season Demand Outpaces Capacity</t>
+        </is>
+      </c>
+      <c r="F148" s="6" t="inlineStr"/>
+      <c r="G148" s="6" t="inlineStr"/>
+      <c r="H148" s="6" t="inlineStr">
+        <is>
+          <t>CPSC 전자 신고 시스템 및 강제 노동 지침 준수 여부 확인 및 내부 프로세스 업데이트, TPEB 운임 급등에 대한 단기 및 장기 운송 전략 재검토.</t>
+        </is>
+      </c>
+      <c r="I148" s="6" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="6" t="inlineStr">
+        <is>
+          <t>RSK-148</t>
+        </is>
+      </c>
+      <c r="B149" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C149" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D149" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E149" s="6" t="inlineStr">
+        <is>
+          <t>끝나지 않은 중동 사태…'호르무즈 없는 시나리오' 짜는 산업계</t>
+        </is>
+      </c>
+      <c r="F149" s="6" t="inlineStr"/>
+      <c r="G149" s="6" t="inlineStr"/>
+      <c r="H149" s="6" t="inlineStr">
+        <is>
+          <t>중동 리스크에 대한 비상 계획 구체화, 대체 운송 경로 및 운송 수단 다변화 검토, 재고 수준 조정.</t>
+        </is>
+      </c>
+      <c r="I149" s="6" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="6" t="inlineStr">
+        <is>
+          <t>RSK-149</t>
+        </is>
+      </c>
+      <c r="B150" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C150" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D150" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E150" s="6" t="inlineStr">
+        <is>
+          <t>미·이란 전면전 위기…국제유가 9%↑, 한달만에 최고치</t>
+        </is>
+      </c>
+      <c r="F150" s="6" t="inlineStr"/>
+      <c r="G150" s="6" t="inlineStr"/>
+      <c r="H150" s="6" t="inlineStr">
+        <is>
+          <t>유가 변동성 모니터링 강화, 운송 계약 조건(유류할증료 등) 재검토, 비용 절감 방안 모색.</t>
+        </is>
+      </c>
+      <c r="I150" s="6" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="6" t="inlineStr">
+        <is>
+          <t>RSK-150</t>
+        </is>
+      </c>
+      <c r="B151" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C151" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D151" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E151" s="6" t="inlineStr">
+        <is>
+          <t>봉쇄된 호르무즈의 ‘숨통’ 셔틀선도 이란 공격 위협 직면</t>
+        </is>
+      </c>
+      <c r="F151" s="6" t="inlineStr"/>
+      <c r="G151" s="6" t="inlineStr"/>
+      <c r="H151" s="6" t="inlineStr">
+        <is>
+          <t>중동 경유 노선 및 유가 변동성 모니터링 강화, 대체 운송 경로 및 재고 확보 방안 검토, 비상 계획 수립.</t>
+        </is>
+      </c>
+      <c r="I151" s="6" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="6" t="inlineStr">
+        <is>
+          <t>RSK-151</t>
+        </is>
+      </c>
+      <c r="B152" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C152" s="6" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="D152" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E152" s="6" t="inlineStr">
+        <is>
+          <t>‘화재 철통 관리’ BIFC 지하에서 화재 발생… 소형 이동 장치 ‘안전 사각’ - 부산일보</t>
+        </is>
+      </c>
+      <c r="F152" s="6" t="inlineStr"/>
+      <c r="G152" s="6" t="inlineStr"/>
+      <c r="H152" s="6" t="inlineStr">
+        <is>
+          <t>배터리 제품의 운송 및 보관, 충전 관련 안전 지침을 재검토하고, 관련 규제 동향을 면밀히 모니터링하며, 창고 및 물류센터 내 배터리 취급 안전 교육을 강화한다.</t>
+        </is>
+      </c>
+      <c r="I152" s="6" t="inlineStr"/>
+    </row>
+    <row r="153">
+      <c r="A153" s="6" t="inlineStr">
+        <is>
+          <t>RSK-152</t>
+        </is>
+      </c>
+      <c r="B153" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C153" s="6" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="D153" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E153" s="6" t="inlineStr">
+        <is>
+          <t>대형 화학물질 화재사고 대비 비상대응체계 강화한다 - 헤럴드경제</t>
+        </is>
+      </c>
+      <c r="F153" s="6" t="inlineStr"/>
+      <c r="G153" s="6" t="inlineStr"/>
+      <c r="H153" s="6" t="inlineStr">
+        <is>
+          <t>당사 물류센터 및 창고의 위험물(배터리) 보관 및 취급 관련 비상대응계획을 재검토하고, 관련 규제 변화에 맞춰 안전 관리 시스템을 강화한다.</t>
+        </is>
+      </c>
+      <c r="I153" s="6" t="inlineStr"/>
+    </row>
+    <row r="154">
+      <c r="A154" s="6" t="inlineStr">
+        <is>
+          <t>RSK-153</t>
+        </is>
+      </c>
+      <c r="B154" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C154" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D154" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E154" s="6" t="inlineStr">
+        <is>
+          <t>Micron Technology Inc (MU) 주식 움직였습니다 하락 6.96%에 7월15일: 어떤 신호인가요?</t>
+        </is>
+      </c>
+      <c r="F154" s="6" t="inlineStr"/>
+      <c r="G154" s="6" t="inlineStr"/>
+      <c r="H154" s="6" t="inlineStr">
+        <is>
+          <t>주요 메모리 부품 공급망 현황 점검 및 대체 공급처 확보 가능성 검토.</t>
+        </is>
+      </c>
+      <c r="I154" s="6" t="inlineStr"/>
+    </row>
+    <row r="155">
+      <c r="A155" s="6" t="inlineStr">
+        <is>
+          <t>RSK-154</t>
+        </is>
+      </c>
+      <c r="B155" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C155" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D155" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E155" s="6" t="inlineStr">
+        <is>
+          <t>대통령 그 입 어떻게 안됩니까…‘호르무즈 통행료’ 번복한 트럼프</t>
+        </is>
+      </c>
+      <c r="F155" s="6" t="inlineStr"/>
+      <c r="G155" s="6" t="inlineStr"/>
+      <c r="H155" s="6" t="inlineStr">
+        <is>
+          <t>중동 정세 및 호르무즈 해협 관련 뉴스 실시간 모니터링, 해상 운송 경로 다변화 및 비상 운송 계획 수립 검토.</t>
+        </is>
+      </c>
+      <c r="I155" s="6" t="inlineStr"/>
+    </row>
+    <row r="156">
+      <c r="A156" s="6" t="inlineStr">
+        <is>
+          <t>RSK-155</t>
+        </is>
+      </c>
+      <c r="B156" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C156" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D156" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E156" s="6" t="inlineStr">
+        <is>
+          <t>유가 85달러 재돌파···항공사 실적 '비상'</t>
+        </is>
+      </c>
+      <c r="F156" s="6" t="inlineStr"/>
+      <c r="G156" s="6" t="inlineStr"/>
+      <c r="H156" s="6" t="inlineStr">
+        <is>
+          <t>항공/해상 운임 변동성 분석 및 물류비 예산 재조정, 운송사와의 계약 조건 재협상 검토.</t>
+        </is>
+      </c>
+      <c r="I156" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
📰 뉴스 데이터 2026-07-20_08:56
</commit_message>
<xml_diff>
--- a/data/SCM_물류_브리핑.xlsx
+++ b/data/SCM_물류_브리핑.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J872"/>
+  <dimension ref="A1:J912"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -41706,6 +41706,1922 @@
       </c>
       <c r="J872" s="4" t="inlineStr"/>
     </row>
+    <row r="873">
+      <c r="A873" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B873" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C873" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D873" s="2" t="inlineStr">
+        <is>
+          <t>Section 301 Tariffs on Brazil Take Effect July 22, Stacking with Section 122 Duties; Strait of Hormuz Closure Restricts 200K TEU of Ocean Capacity</t>
+        </is>
+      </c>
+      <c r="E873" s="2" t="inlineStr">
+        <is>
+          <t>미국의 브라질에 대한 Section 301 관세가 7월 22일 발효되며, 호르무즈 해협 폐쇄로 인해 20만 TEU의 해상 운송 용량이 제한됩니다.</t>
+        </is>
+      </c>
+      <c r="F873" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 폐쇄는 주요 해상 운송 경로의 용량을 크게 제한하여 운송 지연 및 비용 상승을 유발할 수 있으며, 새로운 관세는 원자재 및 부품 조달 비용에 직접적인 영향을 미칠 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G873" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 경유 노선 확인 및 대체 경로/운송 계획 수립, 브라질 및 러시아 관련 공급망 내 관세 영향 분석 및 대응 전략 마련.</t>
+        </is>
+      </c>
+      <c r="H873" s="2" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I873" s="2" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/july-16-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J873" s="2" t="inlineStr">
+        <is>
+          <t>RSK-156</t>
+        </is>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B874" s="2" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C874" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D874" s="2" t="inlineStr">
+        <is>
+          <t>CBP Rejects Warehouse Entries on CAPE Declarations, Risking IEEPA Refunds; TPEB Rates Climb as Panama Canal Restrictions Tighten Capacity</t>
+        </is>
+      </c>
+      <c r="E874" s="2" t="inlineStr">
+        <is>
+          <t>CBP가 CAPE 선언에 대한 창고 입고를 거부하여 IEEPA 환급에 위험을 초래하고 있으며, 파나마 운하 제한으로 용량이 줄어들면서 TPEB(태평양 횡단 동향) 운임이 상승하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F874" s="2" t="inlineStr">
+        <is>
+          <t>파나마 운하의 용량 제한은 아시아-미주 노선의 운송 지연과 운임 상승을 직접적으로 유발하며, CBP의 창고 입고 거부는 통관 및 환급 절차에 혼란을 줄 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G874" s="2" t="inlineStr">
+        <is>
+          <t>파나마 운하 경유 노선에 대한 운송 계획 재검토 및 대체 경로/운송 수단 고려, CBP의 CAPE 선언 관련 지침 확인 및 통관 절차 준수 강화.</t>
+        </is>
+      </c>
+      <c r="H874" s="2" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I874" s="2" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/july-09-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J874" s="2" t="inlineStr">
+        <is>
+          <t>RSK-157</t>
+        </is>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B875" s="2" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C875" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D875" s="2" t="inlineStr">
+        <is>
+          <t>CPSC Mandatory eFiling Takes Effect July 8; TPEB Rates Surge ~10% as Peak Season Demand Outpaces Capacity</t>
+        </is>
+      </c>
+      <c r="E875" s="2" t="inlineStr">
+        <is>
+          <t>CPSC의 의무 전자 신고가 7월 8일 발효되어 특정 제품에 대한 규정 준수가 필요하며, 성수기 수요가 용량을 초과하면서 TPEB 운임이 약 10% 급등했습니다.</t>
+        </is>
+      </c>
+      <c r="F875" s="2" t="inlineStr">
+        <is>
+          <t>CPSC의 의무 전자 신고는 우리 제품의 미국 수출 시 필수적인 규제 준수 사항이며, TPEB 운임의 급등은 주요 운송 비용에 직접적인 영향을 미칩니다.</t>
+        </is>
+      </c>
+      <c r="G875" s="2" t="inlineStr">
+        <is>
+          <t>CPSC eFiling 요건 확인 및 시스템 구축/준비, TPEB 운임 상승에 대비한 운송 계획 및 예산 재조정, 운송사와의 협상 강화.</t>
+        </is>
+      </c>
+      <c r="H875" s="2" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I875" s="2" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/june-18-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J875" s="2" t="inlineStr">
+        <is>
+          <t>RSK-158</t>
+        </is>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B876" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C876" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D876" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 이어 홍해 봉쇄 위기... 다시 희망봉 돌아야 하나</t>
+        </is>
+      </c>
+      <c r="E876" s="2" t="inlineStr">
+        <is>
+          <t>홍해 봉쇄 우려가 커지면서 아시아-유럽 항로가 희망봉 우회로 전환될 가능성이 제기되며, 이는 운송기간, 연료비, 운임 상승 및 선복 부족을 야기할 수 있다.</t>
+        </is>
+      </c>
+      <c r="F876" s="2" t="inlineStr">
+        <is>
+          <t>홍해 봉쇄 및 희망봉 우회는 아시아-유럽 주요 항로의 운송 지연, 운임 급등, 선복 부족을 초래하여 우리 물류 운영에 즉각적이고 심각한 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G876" s="2" t="inlineStr">
+        <is>
+          <t>아시아-유럽 항로의 운송 계획 재검토, 대체 경로 및 운송 수단 옵션 분석, 선사와의 긴밀한 소통을 통한 선복 확보 노력.</t>
+        </is>
+      </c>
+      <c r="H876" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I876" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260720-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J876" s="2" t="inlineStr">
+        <is>
+          <t>RSK-159</t>
+        </is>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B877" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C877" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D877" s="2" t="inlineStr">
+        <is>
+          <t>머스크, 극동아시아-북유럽·지중해 노선 성수기할증료 인상</t>
+        </is>
+      </c>
+      <c r="E877" s="2" t="inlineStr">
+        <is>
+          <t>머스크가 극동아시아발 북유럽·지중해 노선에 성수기 할증료(PSS)를 인상한다고 발표했다.</t>
+        </is>
+      </c>
+      <c r="F877" s="2" t="inlineStr">
+        <is>
+          <t>주요 선사의 성수기 할증료 인상은 해당 노선을 이용하는 우리 물류의 운송 비용에 직접적인 영향을 미치므로 즉시 대응이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G877" s="2" t="inlineStr">
+        <is>
+          <t>해당 노선 운송 계획 및 예산 재검토, 선사와의 운임 협상 또는 대체 운송 방안 모색.</t>
+        </is>
+      </c>
+      <c r="H877" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I877" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/vol132-주간-선사별-동향-week-29-2026</t>
+        </is>
+      </c>
+      <c r="J877" s="2" t="inlineStr">
+        <is>
+          <t>RSK-160</t>
+        </is>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B878" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C878" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D878" s="2" t="inlineStr">
+        <is>
+          <t>끝나지 않은 중동 사태…'호르무즈 없는 시나리오' 짜는 산업계</t>
+        </is>
+      </c>
+      <c r="E878" s="2" t="inlineStr">
+        <is>
+          <t>중동 사태 장기화에 대비하여 산업계가 운임 상승과 물류 지연에 대비한 비상 시나리오를 마련하고 있다.</t>
+        </is>
+      </c>
+      <c r="F878" s="2" t="inlineStr">
+        <is>
+          <t>중동 사태는 주요 해상 운송 경로에 지속적인 불확실성을 제공하며, 운임 상승 및 물류 지연 가능성이 높아 우리 물류 운영에 직접적인 영향을 미친다.</t>
+        </is>
+      </c>
+      <c r="G878" s="2" t="inlineStr">
+        <is>
+          <t>중동 경유 항로의 잠재적 위험 평가 및 대체 운송 방안 검토, 운임 변동성 대비 예산 계획 수립, 비상 시나리오 구체화.</t>
+        </is>
+      </c>
+      <c r="H878" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I878" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260717-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J878" s="2" t="inlineStr">
+        <is>
+          <t>RSK-161</t>
+        </is>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B879" s="2" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C879" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D879" s="2" t="inlineStr">
+        <is>
+          <t>쿠팡, 아직도 불 못껐다…급기야 굴삭기로 ‘건물 파괴’ 초강수</t>
+        </is>
+      </c>
+      <c r="E879" s="2" t="inlineStr">
+        <is>
+          <t>인천 쿠팡 물류센터 화재가 이틀째 지속되자 소방당국이 굴삭기를 동원한 건물 파괴 작업으로 진화에 총력을 기울이고 있다.</t>
+        </is>
+      </c>
+      <c r="F879" s="2" t="inlineStr">
+        <is>
+          <t>대형 물류센터 화재는 창고 안전 규제 강화 논의로 이어질 수 있으며, 유사 시설을 이용하는 우리 물류 운영 및 위험물 보관 규정에 직접적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G879" s="2" t="inlineStr">
+        <is>
+          <t>국내 물류센터 안전 관리 현황 점검 및 비상 계획 재검토, 위험물 보관 시설의 안전 규정 준수 여부 확인.</t>
+        </is>
+      </c>
+      <c r="H879" s="2" t="inlineStr">
+        <is>
+          <t>중앙일보</t>
+        </is>
+      </c>
+      <c r="I879" s="2" t="inlineStr">
+        <is>
+          <t>https://joongang.co.kr/article/25446240</t>
+        </is>
+      </c>
+      <c r="J879" s="2" t="inlineStr">
+        <is>
+          <t>RSK-162</t>
+        </is>
+      </c>
+    </row>
+    <row r="880">
+      <c r="A880" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B880" s="2" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C880" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D880" s="2" t="inlineStr">
+        <is>
+          <t>국가소방동원령에도 쿠팡물류센터 불길 이틀째 안 잡힌 이유는</t>
+        </is>
+      </c>
+      <c r="E880" s="2" t="inlineStr">
+        <is>
+          <t>인천 쿠팡 물류센터에서 이틀째 대형 화재가 진압되지 않고 있으며, 이는 물류센터의 구조적 문제와 보관 물품의 특성 때문으로 분석된다.</t>
+        </is>
+      </c>
+      <c r="F880" s="2" t="inlineStr">
+        <is>
+          <t>대형 물류센터 화재는 물류 네트워크 전반의 안전 점검 및 비상 계획의 중요성을 부각시키며, 우리 회사의 창고 운영 및 재고 관리에 대한 잠재적 위험을 시사한다.</t>
+        </is>
+      </c>
+      <c r="G880" s="2" t="inlineStr">
+        <is>
+          <t>자체 물류센터 및 협력사 창고의 화재 안전 점검 강화, 위험물 보관 규정 준수 여부 재확인, 비상 재고 확보 및 대체 물류 경로 검토.</t>
+        </is>
+      </c>
+      <c r="H880" s="2" t="inlineStr">
+        <is>
+          <t>연합뉴스</t>
+        </is>
+      </c>
+      <c r="I880" s="2" t="inlineStr">
+        <is>
+          <t>https://yna.co.kr/view/AKR20260719034200065</t>
+        </is>
+      </c>
+      <c r="J880" s="2" t="inlineStr">
+        <is>
+          <t>RSK-163</t>
+        </is>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B881" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C881" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D881" s="2" t="inlineStr">
+        <is>
+          <t>이란 혁명수비대 "호르무즈 배 2척 멈춰…美에 속아 진입하면 사고"</t>
+        </is>
+      </c>
+      <c r="E881" s="2" t="inlineStr">
+        <is>
+          <t>이란 혁명수비대가 호르무즈 해협에서 선박 2척을 멈춰 세우고 허가 없는 통과 시 사고를 경고하며 해협 통행에 대한 긴장을 고조시켰다.</t>
+        </is>
+      </c>
+      <c r="F881" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협은 주요 해상 운송 경로로, 이곳의 통행 제한이나 분쟁은 유가 상승 및 해상 운임 변동, 운송 지연 등 우리 회사의 물류 비용과 공급망 안정성에 직접적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G881" s="2" t="inlineStr">
+        <is>
+          <t>중동 항로를 이용하는 선박의 운항 상황 실시간 모니터링, 대체 항로 및 운송 수단 검토, 유가 및 운임 변동에 대한 헤징 전략 고려.</t>
+        </is>
+      </c>
+      <c r="H881" s="2" t="inlineStr">
+        <is>
+          <t>이데일리</t>
+        </is>
+      </c>
+      <c r="I881" s="2" t="inlineStr">
+        <is>
+          <t>https://edaily.co.kr/News/Read?mediaCodeNo=257&amp;newsId=02007366645516160</t>
+        </is>
+      </c>
+      <c r="J881" s="2" t="inlineStr">
+        <is>
+          <t>RSK-164</t>
+        </is>
+      </c>
+    </row>
+    <row r="882">
+      <c r="A882" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B882" s="2" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C882" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D882" s="2" t="inlineStr">
+        <is>
+          <t>창고 가득한 생활용품이 ‘땔감’ 역할… 불 났다하면 대형 화재</t>
+        </is>
+      </c>
+      <c r="E882" s="2" t="inlineStr">
+        <is>
+          <t>인천 쿠팡 물류센터 화재는 물류창고의 구조적 문제와 보관 물품의 가연성으로 인해 대형 화재로 번졌으며, 이는 물류창고의 안전 관리 중요성을 부각시킨다.</t>
+        </is>
+      </c>
+      <c r="F882" s="2" t="inlineStr">
+        <is>
+          <t>물류센터의 구조적 문제와 보관 물품의 특성이 대형 화재로 이어질 수 있음을 보여주며, 우리 회사의 물류센터 및 협력사 창고의 화재 안전 규정 및 위험물 보관 기준 준수 여부를 재점검할 필요가 있다.</t>
+        </is>
+      </c>
+      <c r="G882" s="2" t="inlineStr">
+        <is>
+          <t>자체 물류센터 및 협력사 창고의 화재 안전 점검 강화, 위험물 보관 규정 준수 여부 재확인, 비상 재고 확보 및 대체 물류 경로 검토.</t>
+        </is>
+      </c>
+      <c r="H882" s="2" t="inlineStr">
+        <is>
+          <t>국민일보</t>
+        </is>
+      </c>
+      <c r="I882" s="2" t="inlineStr">
+        <is>
+          <t>https://kmib.co.kr/article/view.asp?arcid=1784452963&amp;code=11131100&amp;sid1=soc</t>
+        </is>
+      </c>
+      <c r="J882" s="2" t="inlineStr">
+        <is>
+          <t>RSK-165</t>
+        </is>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B883" s="2" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C883" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D883" s="2" t="inlineStr">
+        <is>
+          <t>24시간 넘게 불타는 쿠팡 물류센터…“피해 수천억원 될 수도”</t>
+        </is>
+      </c>
+      <c r="E883" s="2" t="inlineStr">
+        <is>
+          <t>인천 쿠팡 물류센터 화재가 24시간 넘게 지속되며 수천억 원에 달하는 막대한 피해가 예상되어, 대형 물류센터 화재의 경제적 파급력을 보여준다.</t>
+        </is>
+      </c>
+      <c r="F883" s="2" t="inlineStr">
+        <is>
+          <t>대형 물류센터 화재로 인한 막대한 재산 및 영업 손실은 우리 회사의 물류 운영 중단 시 발생할 수 있는 잠재적 피해 규모를 가늠하게 하며, 비상 계획의 중요성을 강조한다.</t>
+        </is>
+      </c>
+      <c r="G883" s="2" t="inlineStr">
+        <is>
+          <t>자체 물류센터 및 협력사 창고의 화재 안전 점검 강화, 위험물 보관 규정 준수 여부 재확인, 비상 재고 확보 및 대체 물류 경로 검토, 물류 보험 커버리지 재검토.</t>
+        </is>
+      </c>
+      <c r="H883" s="2" t="inlineStr">
+        <is>
+          <t>중앙일보</t>
+        </is>
+      </c>
+      <c r="I883" s="2" t="inlineStr">
+        <is>
+          <t>https://joongang.co.kr/article/25446154</t>
+        </is>
+      </c>
+      <c r="J883" s="2" t="inlineStr">
+        <is>
+          <t>RSK-166</t>
+        </is>
+      </c>
+    </row>
+    <row r="884">
+      <c r="A884" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B884" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C884" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D884" s="2" t="inlineStr">
+        <is>
+          <t>[기획] 세계경제 흔드는 ‘호르무즈’… 유가 넘어 글로벌 공급망 재충격</t>
+        </is>
+      </c>
+      <c r="E884" s="2" t="inlineStr">
+        <is>
+          <t>중동 지역의 군사적 긴장이 고조되면서 호르무즈 해협 리스크가 다시 부각되고 있으며, 이는 유가 상승을 넘어 글로벌 공급망 전반에 재충격을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="F884" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협은 주요 원유 및 가스 운송 경로이자 글로벌 해상 운송의 핵심 길목으로, 긴장 고조는 유가 및 해상 운임 급등, 운송 지연 등 우리 회사의 물류 운영에 직접적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G884" s="2" t="inlineStr">
+        <is>
+          <t>중동 항로를 이용하는 선박의 운항 상황 및 유가, 해상 운임 변동 추이 실시간 모니터링, 비상 운송 계획 및 재고 수준 점검</t>
+        </is>
+      </c>
+      <c r="H884" s="2" t="inlineStr">
+        <is>
+          <t>매일일보</t>
+        </is>
+      </c>
+      <c r="I884" s="2" t="inlineStr">
+        <is>
+          <t>https://m-i.kr/news/articleView.html?idxno=1392251</t>
+        </is>
+      </c>
+      <c r="J884" s="2" t="inlineStr">
+        <is>
+          <t>RSK-167</t>
+        </is>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B885" s="2" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C885" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D885" s="2" t="inlineStr">
+        <is>
+          <t>연기 가득, 진화 난항…쿠팡 물류센터 화재 국가소방동원령 4차 발령</t>
+        </is>
+      </c>
+      <c r="E885" s="2" t="inlineStr">
+        <is>
+          <t>인천 쿠팡 물류센터에서 대형 화재가 발생하여 15시간째 진압에 난항을 겪고 있으며, 소방청이 국가소방동원령을 4차까지 발령했다.</t>
+        </is>
+      </c>
+      <c r="F885" s="2" t="inlineStr">
+        <is>
+          <t>대형 물류센터 화재는 창고 안전 규제 강화 및 물류 운영 안정성 점검의 필요성을 높이며, 우리 회사의 창고 운영 및 재고 전략에 직접적인 영향을 미칠 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G885" s="2" t="inlineStr">
+        <is>
+          <t>우리 회사 물류센터 및 협력사 창고의 화재 안전 점검 강화, 배터리/전자부품 등 위험물 보관 규정 준수 여부 재확인, 비상 계획 수립 및 훈련.</t>
+        </is>
+      </c>
+      <c r="H885" s="2" t="inlineStr">
+        <is>
+          <t>머니투데이</t>
+        </is>
+      </c>
+      <c r="I885" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mt.co.kr/society/2026/07/18/2026071820405851539</t>
+        </is>
+      </c>
+      <c r="J885" s="2" t="inlineStr">
+        <is>
+          <t>RSK-168</t>
+        </is>
+      </c>
+    </row>
+    <row r="886">
+      <c r="A886" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B886" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C886" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D886" s="3" t="inlineStr">
+        <is>
+          <t>올 세계 항공시장 ‘에상보다 더 낙관적’</t>
+        </is>
+      </c>
+      <c r="E886" s="3" t="inlineStr">
+        <is>
+          <t>글로벌 항공화물 운임이 중동 전쟁으로 인한 공급망 혼란과 긴급 수요 확대로 인해 2026년 5~15% 상승할 것으로 전망됩니다.</t>
+        </is>
+      </c>
+      <c r="F886" s="3" t="inlineStr">
+        <is>
+          <t>항공 운임 상승은 배터리/전자부품과 같은 고부가가치 제품의 운송 비용에 직접적인 영향을 미치므로 지속적인 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G886" s="3" t="inlineStr">
+        <is>
+          <t>항공 운송 계약 조건 재검토, 대체 운송 수단(해상 등) 활용 가능성 검토, 운송비 예산 재조정.</t>
+        </is>
+      </c>
+      <c r="H886" s="3" t="inlineStr">
+        <is>
+          <t>cargonews</t>
+        </is>
+      </c>
+      <c r="I886" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cargonews.co.kr/news/articleView.html?idxno=60543</t>
+        </is>
+      </c>
+      <c r="J886" s="3" t="inlineStr"/>
+    </row>
+    <row r="887">
+      <c r="A887" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B887" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C887" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D887" s="3" t="inlineStr">
+        <is>
+          <t>U.S.-EU Trade Agreement Eliminates Duties on Most U.S. Goods Starting July 1; TPEB Rates Rise as July Capacity Hits Three-Year High</t>
+        </is>
+      </c>
+      <c r="E887" s="3" t="inlineStr">
+        <is>
+          <t>미국-EU 무역 협정이 7월 1일부터 대부분의 미국산 공산품에 대한 관세를 철폐했으며, 7월 용량이 3년 만에 최고치를 기록했음에도 불구하고 TPEB 운임은 상승하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F887" s="3" t="inlineStr">
+        <is>
+          <t>미-EU 무역 협정은 해당 지역으로의 수출입 비용을 절감할 잠재력이 있으나, TPEB 운임 상승은 주요 운송 비용 증가 추세를 나타내므로 지속적인 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G887" s="3" t="inlineStr">
+        <is>
+          <t>미-EU 무역 협정의 세부 내용 검토 및 해당 제품에 대한 관세 혜택 활용 방안 모색, TPEB 운임 추이 모니터링 및 운송 계약 조건 재검토.</t>
+        </is>
+      </c>
+      <c r="H887" s="3" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I887" s="3" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/july-02-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J887" s="3" t="inlineStr"/>
+    </row>
+    <row r="888">
+      <c r="A888" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B888" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C888" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D888" s="3" t="inlineStr">
+        <is>
+          <t>CAPE Phase 2 Launches June 29 for Reconciliation-Flagged Entries; TPEB Rates Rise 10% for Sixth Consecutive Week</t>
+        </is>
+      </c>
+      <c r="E888" s="3" t="inlineStr">
+        <is>
+          <t>CBP의 CAPE Phase 2가 6월 29일 조정 대상 항목에 대해 시작되었으며, TPEB 운임은 6주 연속 10% 상승했습니다.</t>
+        </is>
+      </c>
+      <c r="F888" s="3" t="inlineStr">
+        <is>
+          <t>TPEB 운임의 지속적인 상승은 주요 운송 비용 증가를 의미하며, CAPE Phase 2는 통관 절차에 영향을 줄 수 있으므로 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G888" s="3" t="inlineStr">
+        <is>
+          <t>TPEB 운임 상승 추이 모니터링 및 운송 계약 조건 재검토, CAPE Phase 2 관련 CBP 지침 확인 및 통관 절차에 미치는 영향 분석.</t>
+        </is>
+      </c>
+      <c r="H888" s="3" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I888" s="3" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/june-25-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J888" s="3" t="inlineStr"/>
+    </row>
+    <row r="889">
+      <c r="A889" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B889" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C889" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D889" s="3" t="inlineStr">
+        <is>
+          <t>Statement on EU Commission Revision of the EU Emissions Trading System</t>
+        </is>
+      </c>
+      <c r="E889" s="3" t="inlineStr">
+        <is>
+          <t>IATA는 EU 배출권 거래 시스템(ETS)의 유럽 외 지역 확장 제안에 대해 깊은 불만을 표하며 부정적인 결과를 경고했습니다.</t>
+        </is>
+      </c>
+      <c r="F889" s="3" t="inlineStr">
+        <is>
+          <t>EU ETS의 확장 논의는 항공 운송 비용 증가 및 규제 준수 부담으로 이어질 수 있으므로, 향후 우리 항공 물류 운영에 미칠 영향을 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G889" s="3" t="inlineStr">
+        <is>
+          <t>EU ETS 확장 논의 진행 상황 주시, 항공 운송 비용에 미칠 잠재적 영향 분석, 탄소 배출량 관리 및 저감 방안 검토.</t>
+        </is>
+      </c>
+      <c r="H889" s="3" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I889" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/07-17-statement-eu-commission-revision-emissions-trading-system/</t>
+        </is>
+      </c>
+      <c r="J889" s="3" t="inlineStr"/>
+    </row>
+    <row r="890">
+      <c r="A890" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B890" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C890" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D890" s="3" t="inlineStr">
+        <is>
+          <t>Air Cargo Demand Up 6.0% in May</t>
+        </is>
+      </c>
+      <c r="E890" s="3" t="inlineStr">
+        <is>
+          <t>2026년 5월 글로벌 항공 화물 수요가 전년 대비 6.0% 증가하여 시장의 강세를 나타냈습니다.</t>
+        </is>
+      </c>
+      <c r="F890" s="3" t="inlineStr">
+        <is>
+          <t>항공 화물 수요 증가는 운임 상승 압력으로 작용할 수 있으며, 이는 우리 제품의 항공 운송 비용에 영향을 미칠 수 있으므로 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G890" s="3" t="inlineStr">
+        <is>
+          <t>항공 운임 추이와 항공사 용량 확보 상황 지속 모니터링.</t>
+        </is>
+      </c>
+      <c r="H890" s="3" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I890" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-29-air-cargo-demand-up-may/</t>
+        </is>
+      </c>
+      <c r="J890" s="3" t="inlineStr"/>
+    </row>
+    <row r="891">
+      <c r="A891" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B891" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C891" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D891" s="3" t="inlineStr">
+        <is>
+          <t>Structural Contraction of Global Liner Networks</t>
+        </is>
+      </c>
+      <c r="E891" s="3" t="inlineStr">
+        <is>
+          <t>IMF는 2026년 글로벌 무역량 성장률이 3.5%로 크게 둔화될 것으로 전망하며, 이는 글로벌 선사 네트워크의 구조적 축소로 이어질 것이라고 분석했습니다.</t>
+        </is>
+      </c>
+      <c r="F891" s="3" t="inlineStr">
+        <is>
+          <t>글로벌 무역량 둔화와 선사 네트워크 축소는 해상 운송 용량 감소 및 서비스 빈도 변화로 이어져 우리 제품의 해상 운송 계획에 영향을 미칠 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G891" s="3" t="inlineStr">
+        <is>
+          <t>주요 해상 운송 노선의 선사 서비스 변화 모니터링, 장기 운송 계약 조건 재검토, 운송 파트너와의 긴밀한 소통 유지.</t>
+        </is>
+      </c>
+      <c r="H891" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I891" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/398-structural-contraction-of-global-liner-network</t>
+        </is>
+      </c>
+      <c r="J891" s="3" t="inlineStr"/>
+    </row>
+    <row r="892">
+      <c r="A892" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B892" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C892" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D892" s="3" t="inlineStr">
+        <is>
+          <t>Structural Contraction of Global Liner Networks</t>
+        </is>
+      </c>
+      <c r="E892" s="3" t="inlineStr">
+        <is>
+          <t>글로벌 선사들이 네트워크를 구조적으로 축소하고 있으며, 지리적 범위는 유지하나 서비스 빈도가 감소하는 추세이다.</t>
+        </is>
+      </c>
+      <c r="F892" s="3" t="inlineStr">
+        <is>
+          <t>선사들의 서비스 빈도 감소는 장기적으로 우리 물류의 운송 옵션 및 스케줄 유연성에 영향을 줄 수 있으므로 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G892" s="3" t="n"/>
+      <c r="H892" s="3" t="inlineStr">
+        <is>
+          <t>sea-intelligence</t>
+        </is>
+      </c>
+      <c r="I892" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/397-structural-contraction-of-global-liner-networks</t>
+        </is>
+      </c>
+      <c r="J892" s="3" t="inlineStr"/>
+    </row>
+    <row r="893">
+      <c r="A893" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B893" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C893" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D893" s="3" t="inlineStr">
+        <is>
+          <t>PLSCI Data Indicates Mega-Hub Retrenchment</t>
+        </is>
+      </c>
+      <c r="E893" s="3" t="inlineStr">
+        <is>
+          <t>UNCTAD의 PLSCI 데이터에 따르면 메가 허브 항만의 연결성이 재조정되고 있으며, 이는 선사들의 네트워크 전략 변화를 반영한다.</t>
+        </is>
+      </c>
+      <c r="F893" s="3" t="inlineStr">
+        <is>
+          <t>주요 허브 항만의 연결성 변화는 향후 우리 물류의 주요 환적 경로 및 리드타임에 영향을 미칠 수 있어 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G893" s="3" t="n"/>
+      <c r="H893" s="3" t="inlineStr">
+        <is>
+          <t>sea-intelligence</t>
+        </is>
+      </c>
+      <c r="I893" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/396-plsci-data-indicates-mega-hub-retrenchment</t>
+        </is>
+      </c>
+      <c r="J893" s="3" t="inlineStr"/>
+    </row>
+    <row r="894">
+      <c r="A894" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B894" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C894" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D894" s="3" t="inlineStr">
+        <is>
+          <t>Tracking True Vessel Delay</t>
+        </is>
+      </c>
+      <c r="E894" s="3" t="inlineStr">
+        <is>
+          <t>선사들이 운송 시간을 늘리는 스케줄 버퍼링을 통해 선박 지연을 관리하고 있으며, 이는 실제 지연과 조기 도착 간의 관계를 분석한 결과이다.</t>
+        </is>
+      </c>
+      <c r="F894" s="3" t="inlineStr">
+        <is>
+          <t>선사들의 스케줄 버퍼링은 명목상 운송 시간 증가로 이어져 우리 물류의 리드타임 예측에 영향을 줄 수 있으므로 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G894" s="3" t="n"/>
+      <c r="H894" s="3" t="inlineStr">
+        <is>
+          <t>sea-intelligence</t>
+        </is>
+      </c>
+      <c r="I894" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/394-tracking-true-vessel-delay</t>
+        </is>
+      </c>
+      <c r="J894" s="3" t="inlineStr"/>
+    </row>
+    <row r="895">
+      <c r="A895" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B895" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C895" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D895" s="3" t="inlineStr">
+        <is>
+          <t>해진공 "중동불안 장기화 속 국제물류 구조 재편...효율성→안정성·유..."</t>
+        </is>
+      </c>
+      <c r="E895" s="3" t="inlineStr">
+        <is>
+          <t>중동 불안이 장기화되면서 국제 물류 구조가 효율성보다는 안정성 및 유연성을 중시하는 방향으로 재편될 수 있다는 분석이다.</t>
+        </is>
+      </c>
+      <c r="F895" s="3" t="inlineStr">
+        <is>
+          <t>중동 불안으로 인한 국제 물류 구조 재편은 장기적으로 우리 SCM 전략에 영향을 미칠 수 있으므로 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G895" s="3" t="n"/>
+      <c r="H895" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I895" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260718-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J895" s="3" t="inlineStr"/>
+    </row>
+    <row r="896">
+      <c r="A896" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B896" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C896" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D896" s="3" t="inlineStr">
+        <is>
+          <t>머스크, 홍해 복귀 속도…WAF15도 수에즈 전환</t>
+        </is>
+      </c>
+      <c r="E896" s="3" t="inlineStr">
+        <is>
+          <t>머스크가 서아프리카 지선 서비스 WAF15를 희망봉 우회에서 수에즈·홍해 항로로 전환하며 홍해 복귀에 속도를 내고 있다.</t>
+        </is>
+      </c>
+      <c r="F896" s="3" t="inlineStr">
+        <is>
+          <t>주요 선사의 홍해/수에즈 운하 복귀는 해당 항로의 안정성 회복 가능성을 시사하나, 중동 리스크가 상존하므로 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G896" s="3" t="n"/>
+      <c r="H896" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I896" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/vol132-주간-선사별-동향-week-29-2026</t>
+        </is>
+      </c>
+      <c r="J896" s="3" t="inlineStr"/>
+    </row>
+    <row r="897">
+      <c r="A897" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B897" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C897" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D897" s="3" t="inlineStr">
+        <is>
+          <t>머스크, 인도·중동-미국 동안 항로 수에즈운하 복귀…동항 운송일수 14일 단축</t>
+        </is>
+      </c>
+      <c r="E897" s="3" t="inlineStr">
+        <is>
+          <t>머스크가 인도·중동-미국 동안 서비스 MECL을 수에즈운하 경유로 전환하여 운송 일수를 14일 단축했다.</t>
+        </is>
+      </c>
+      <c r="F897" s="3" t="inlineStr">
+        <is>
+          <t>주요 항로의 운송일수 단축은 긍정적인 신호이나, 중동 리스크로 인한 재우회 가능성이 있어 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G897" s="3" t="n"/>
+      <c r="H897" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I897" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/vol132-주간-선사별-동향-week-29-2026</t>
+        </is>
+      </c>
+      <c r="J897" s="3" t="inlineStr"/>
+    </row>
+    <row r="898">
+      <c r="A898" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B898" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C898" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D898" s="3" t="inlineStr">
+        <is>
+          <t>The GAFG Connectivity Doctrine: From Corridors to Governance Ecosystems</t>
+        </is>
+      </c>
+      <c r="E898" s="3" t="inlineStr">
+        <is>
+          <t>지정학적 불안정성과 공급망 혼란 속에서 북극 항로, 미들 코리더 등 다양한 대체 무역 경로의 중요성과 거버넌스 생태계 구축의 필요성을 강조한다.</t>
+        </is>
+      </c>
+      <c r="F898" s="3" t="inlineStr">
+        <is>
+          <t>장기적인 관점에서 공급망 다변화 및 대체 운송 경로 개발의 중요성을 시사하며, 우리 회사의 미래 물류 전략 수립에 참고할 만한 정보이다.</t>
+        </is>
+      </c>
+      <c r="G898" s="3" t="inlineStr">
+        <is>
+          <t>없음</t>
+        </is>
+      </c>
+      <c r="H898" s="3" t="inlineStr">
+        <is>
+          <t>Morocco World News</t>
+        </is>
+      </c>
+      <c r="I898" s="3" t="inlineStr">
+        <is>
+          <t>https://www.moroccoworldnews.com/2026/07/330231/the-gafg-connectivity-doctrine-from-corridors-to-governance-ecosystems/</t>
+        </is>
+      </c>
+      <c r="J898" s="3" t="inlineStr"/>
+    </row>
+    <row r="899">
+      <c r="A899" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B899" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C899" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D899" s="3" t="inlineStr">
+        <is>
+          <t>Asia’s renewable energy expansion faces rising project risks</t>
+        </is>
+      </c>
+      <c r="E899" s="3" t="inlineStr">
+        <is>
+          <t>아시아의 재생에너지 확장이 지정학적 긴장, 무역 정책 변화, 물류 혼란, 공급업체 집중 등으로 인해 공급망 회복력 측면에서 프로젝트 위험에 직면하고 있다.</t>
+        </is>
+      </c>
+      <c r="F899" s="3" t="inlineStr">
+        <is>
+          <t>지정학적 긴장, 무역 정책 변화, 물류 혼란 등은 우리 회사의 공급망에도 유사한 위험을 초래할 수 있으므로, 아시아 지역의 공급망 리스크 추이를 지속적으로 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G899" s="3" t="inlineStr">
+        <is>
+          <t>없음</t>
+        </is>
+      </c>
+      <c r="H899" s="3" t="inlineStr">
+        <is>
+          <t>Asian Power</t>
+        </is>
+      </c>
+      <c r="I899" s="3" t="inlineStr">
+        <is>
+          <t>https://asian-power.com/in-focus/asias-renewable-energy-expansion-faces-rising-project-risks</t>
+        </is>
+      </c>
+      <c r="J899" s="3" t="inlineStr"/>
+    </row>
+    <row r="900">
+      <c r="A900" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B900" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C900" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D900" s="3" t="inlineStr">
+        <is>
+          <t>한번 터지면 장기화·대형화재···반복되는 ‘물류센터 화재’ 막을 방법 없나</t>
+        </is>
+      </c>
+      <c r="E900" s="3" t="inlineStr">
+        <is>
+          <t>인천 쿠팡 물류센터에서 대형 화재가 발생하여 물류센터 안전 관리 문제가 다시 부각되었으며, 이는 대형화·장기화되는 물류센터 화재에 대한 근본적인 대책 마련의 필요성을 제기한다.</t>
+        </is>
+      </c>
+      <c r="F900" s="3" t="inlineStr">
+        <is>
+          <t>물류센터 화재가 반복되면서 안전 규제 강화 논의가 시작될 수 있으며, 이는 향후 우리 회사의 물류센터 운영 및 보관 비용에 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G900" s="3" t="inlineStr">
+        <is>
+          <t>물류센터 안전 관리 현황 점검 및 관련 규제 동향 지속 모니터링</t>
+        </is>
+      </c>
+      <c r="H900" s="3" t="inlineStr">
+        <is>
+          <t>경향신문</t>
+        </is>
+      </c>
+      <c r="I900" s="3" t="inlineStr">
+        <is>
+          <t>https://www.khan.co.kr/article/202607191506001/</t>
+        </is>
+      </c>
+      <c r="J900" s="3" t="inlineStr"/>
+    </row>
+    <row r="901">
+      <c r="A901" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B901" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C901" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D901" s="3" t="inlineStr">
+        <is>
+          <t>"中메모리칩 사지 말라"...美공화당‧민주당,상무부에 CXMT·YMTC 구매 제한 촉구</t>
+        </is>
+      </c>
+      <c r="E901" s="3" t="inlineStr">
+        <is>
+          <t>미국 공화당과 민주당이 상무부에 중국 D램 및 낸드플래시 제조업체인 CXMT와 YMTC에 대한 구매 제한을 촉구하며, 이는 미중 반도체 기술 경쟁 심화와 공급망 분리 압력을 보여준다.</t>
+        </is>
+      </c>
+      <c r="F901" s="3" t="inlineStr">
+        <is>
+          <t>중국 메모리칩에 대한 미국의 추가 제재 가능성은 우리 회사의 부품 조달 및 공급망 전략에 간접적인 영향을 미칠 수 있으므로 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G901" s="3" t="inlineStr">
+        <is>
+          <t>중국산 반도체 부품 사용 현황 점검 및 대체 공급처 확보 가능성 검토</t>
+        </is>
+      </c>
+      <c r="H901" s="3" t="inlineStr">
+        <is>
+          <t>더퍼블릭</t>
+        </is>
+      </c>
+      <c r="I901" s="3" t="inlineStr">
+        <is>
+          <t>https://thepublic.kr/news/articleView.html?idxno=311695</t>
+        </is>
+      </c>
+      <c r="J901" s="3" t="inlineStr"/>
+    </row>
+    <row r="902">
+      <c r="A902" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B902" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C902" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D902" s="3" t="inlineStr">
+        <is>
+          <t>8월 국제선 유류할증료 또 내린다</t>
+        </is>
+      </c>
+      <c r="E902" s="3" t="inlineStr">
+        <is>
+          <t>국제유가 안정세가 이어지면서 대한항공의 국제선 유류할증료가 8월에도 큰 폭으로 인하되어 3개월 연속 하락한다.</t>
+        </is>
+      </c>
+      <c r="F902" s="3" t="inlineStr">
+        <is>
+          <t>국제선 유류할증료 인하는 항공 운송 비용 절감에 긍정적이나, 유가 변동성에 따라 언제든 다시 상승할 수 있어 지속적인 추이 관찰이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G902" s="3" t="inlineStr">
+        <is>
+          <t>항공 운송 비용 절감 기회 모색 및 장기적인 운임 추이 모니터링.</t>
+        </is>
+      </c>
+      <c r="H902" s="3" t="inlineStr">
+        <is>
+          <t>트래블데일리</t>
+        </is>
+      </c>
+      <c r="I902" s="3" t="inlineStr">
+        <is>
+          <t>https://www.traveldaily.co.kr/news/articleView.html?idxno=71556</t>
+        </is>
+      </c>
+      <c r="J902" s="3" t="inlineStr"/>
+    </row>
+    <row r="903">
+      <c r="A903" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B903" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C903" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D903" s="3" t="inlineStr">
+        <is>
+          <t>뉴스스페이스</t>
+        </is>
+      </c>
+      <c r="E903" s="3" t="inlineStr">
+        <is>
+          <t>이란 고위 군사 고문이 미국 공습 지속 시 보복 작전을 경고하며 중동 지역의 지정학적 긴장이 고조되고 있다.</t>
+        </is>
+      </c>
+      <c r="F903" s="3" t="inlineStr">
+        <is>
+          <t>중동 지역의 지정학적 긴장은 국제 유가 및 주요 해상 운송로의 안정성에 영향을 미칠 수 있으므로, 에너지 비용 및 운송 리스크 관점에서 추이를 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G903" s="3" t="inlineStr">
+        <is>
+          <t>국제 유가 및 중동 지역 정세 변화 모니터링, 비상 운송 경로 및 재고 확보 전략 검토.</t>
+        </is>
+      </c>
+      <c r="H903" s="3" t="inlineStr">
+        <is>
+          <t>뉴스스페이스</t>
+        </is>
+      </c>
+      <c r="I903" s="3" t="inlineStr">
+        <is>
+          <t>https://newsspace.kr/news/article.html?no=14861</t>
+        </is>
+      </c>
+      <c r="J903" s="3" t="inlineStr"/>
+    </row>
+    <row r="904">
+      <c r="A904" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B904" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C904" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D904" s="4" t="inlineStr">
+        <is>
+          <t>Global Schedule Reliability for May 2026 the Highest of the Year</t>
+        </is>
+      </c>
+      <c r="E904" s="4" t="inlineStr">
+        <is>
+          <t>2026년 5월 글로벌 선박 스케줄 신뢰도가 올해 최고치를 기록하여 전반적인 해운 서비스의 정시성이 개선되었다.</t>
+        </is>
+      </c>
+      <c r="F904" s="4" t="inlineStr">
+        <is>
+          <t>스케줄 신뢰도 개선은 긍정적이나, 단기적인 수치이며 우리 물류 운영에 즉각적인 변화를 요구하지는 않는다.</t>
+        </is>
+      </c>
+      <c r="G904" s="4" t="n"/>
+      <c r="H904" s="4" t="inlineStr">
+        <is>
+          <t>sea-intelligence</t>
+        </is>
+      </c>
+      <c r="I904" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/395-global-schedule-reliability-for-may-2026-the-highest-of-the-year</t>
+        </is>
+      </c>
+      <c r="J904" s="4" t="inlineStr"/>
+    </row>
+    <row r="905">
+      <c r="A905" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B905" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C905" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D905" s="4" t="inlineStr">
+        <is>
+          <t>"한화 필리조선소, 신규 수주로 MASGA 투자 과실 증명"...골든 디펜더급 MRIV 수주로 미 골든 돔 정책 참여</t>
+        </is>
+      </c>
+      <c r="E905" s="4" t="inlineStr">
+        <is>
+          <t>한화 필리조선소가 미사일 방어 프로젝트 관련 신규 수주를 확보하며 미국 현지 조선 투자 성과를 입증했다.</t>
+        </is>
+      </c>
+      <c r="F905" s="4" t="inlineStr">
+        <is>
+          <t>조선업 관련 뉴스이나, 우리 회사의 배터리/전자부품 물류 운영에 직접적인 영향은 없으며 참고 수준이다.</t>
+        </is>
+      </c>
+      <c r="G905" s="4" t="n"/>
+      <c r="H905" s="4" t="inlineStr">
+        <is>
+          <t>shippingnewsnet</t>
+        </is>
+      </c>
+      <c r="I905" s="4" t="inlineStr">
+        <is>
+          <t>https://www.shippingnewsnet.com/news/articleView.html?idxno=71225</t>
+        </is>
+      </c>
+      <c r="J905" s="4" t="inlineStr"/>
+    </row>
+    <row r="906">
+      <c r="A906" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B906" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C906" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D906" s="4" t="inlineStr">
+        <is>
+          <t>이베코코리아 / 연비·안전·주행 편의성 향상 대형 트랙터 ‘올 뉴 S-Way’ 출시</t>
+        </is>
+      </c>
+      <c r="E906" s="4" t="inlineStr">
+        <is>
+          <t>이베코코리아가 연비, 안전, 주행 편의성을 향상시킨 대형 트랙터 '올 뉴 S-Way'를 국내에 출시하여 운송 사업자의 운영 효율을 높일 것으로 기대된다.</t>
+        </is>
+      </c>
+      <c r="F906" s="4" t="inlineStr">
+        <is>
+          <t>신형 트랙터 출시는 육상 운송 효율성 개선에 기여할 수 있으나, 우리 물류 운영에 직접적인 영향은 없으며 참고 수준이다.</t>
+        </is>
+      </c>
+      <c r="G906" s="4" t="n"/>
+      <c r="H906" s="4" t="inlineStr">
+        <is>
+          <t>ulogistics</t>
+        </is>
+      </c>
+      <c r="I906" s="4" t="inlineStr">
+        <is>
+          <t>http://www.ulogistics.co.kr/test/board.php?board=all2&amp;command=body&amp;no=5212</t>
+        </is>
+      </c>
+      <c r="J906" s="4" t="inlineStr"/>
+    </row>
+    <row r="907">
+      <c r="A907" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B907" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C907" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D907" s="4" t="inlineStr">
+        <is>
+          <t>[해양통신] LNGBV 시장 급성장… "중국 가세, 대형화가 특징"</t>
+        </is>
+      </c>
+      <c r="E907" s="4" t="inlineStr">
+        <is>
+          <t>LNG 벙커링 시장이 급성장하며 전 세계 LNG 벙커링선 선단이 확대될 전망이며, 중국 기업의 투자와 대형화가 특징이다.</t>
+        </is>
+      </c>
+      <c r="F907" s="4" t="inlineStr">
+        <is>
+          <t>LNG 벙커링 시장 성장은 장기적인 해운 연료 동향에 영향을 줄 수 있으나, 우리 물류 운영에 당장 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G907" s="4" t="n"/>
+      <c r="H907" s="4" t="inlineStr">
+        <is>
+          <t>oceanpress.co.kr</t>
+        </is>
+      </c>
+      <c r="I907" s="4" t="inlineStr">
+        <is>
+          <t>https://oceanpress.co.kr/news/article.html?no=30653</t>
+        </is>
+      </c>
+      <c r="J907" s="4" t="inlineStr"/>
+    </row>
+    <row r="908">
+      <c r="A908" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B908" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C908" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D908" s="4" t="inlineStr">
+        <is>
+          <t>의사 원격진료 없이도 일반의약품 투여 가능…선내 안전보건 기준 손질</t>
+        </is>
+      </c>
+      <c r="E908" s="4" t="inlineStr">
+        <is>
+          <t>선박 건강담당자의 일반의약품 투여 절차가 간소화되고 안전대표자 선정 방식에 임명제가 포함되는 등 선박 내 안전·보건 기준이 개선된다.</t>
+        </is>
+      </c>
+      <c r="F908" s="4" t="inlineStr">
+        <is>
+          <t>선박 내 의료 및 안전보건 기준에 대한 내용으로, 우리 회사의 배터리/전자부품 물류 운영에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G908" s="4" t="inlineStr">
+        <is>
+          <t>없음</t>
+        </is>
+      </c>
+      <c r="H908" s="4" t="inlineStr">
+        <is>
+          <t>아주경제</t>
+        </is>
+      </c>
+      <c r="I908" s="4" t="inlineStr">
+        <is>
+          <t>https://ajunews.com/view/20260719143613531</t>
+        </is>
+      </c>
+      <c r="J908" s="4" t="inlineStr"/>
+    </row>
+    <row r="909">
+      <c r="A909" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B909" s="4" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C909" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D909" s="4" t="inlineStr">
+        <is>
+          <t>정부, 석유 매점매석 금지 9월까지 연장…최고가격제와 '동반 유지'</t>
+        </is>
+      </c>
+      <c r="E909" s="4" t="inlineStr">
+        <is>
+          <t>정부가 석유제품 매점매석 금지 조치를 9월 12일까지 연장하여 유가 상승 압력 속에서 국내 석유 공급 가격을 안정화하려 한다.</t>
+        </is>
+      </c>
+      <c r="F909" s="4" t="inlineStr">
+        <is>
+          <t>국내 석유제품 가격 안정화 조치로, 우리 회사의 직접적인 물류 운임이나 유가 변동에 미치는 영향은 제한적이다.</t>
+        </is>
+      </c>
+      <c r="G909" s="4" t="n"/>
+      <c r="H909" s="4" t="inlineStr">
+        <is>
+          <t>뉴스1</t>
+        </is>
+      </c>
+      <c r="I909" s="4" t="inlineStr">
+        <is>
+          <t>https://news1.kr/economy/trend/6230794</t>
+        </is>
+      </c>
+      <c r="J909" s="4" t="inlineStr"/>
+    </row>
+    <row r="910">
+      <c r="A910" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B910" s="4" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C910" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D910" s="4" t="inlineStr">
+        <is>
+          <t>“러, 침대 밑에 돈 쌓아둬”…군시설 대신 물류센터 때린 우크라</t>
+        </is>
+      </c>
+      <c r="E910" s="4" t="inlineStr">
+        <is>
+          <t>우크라이나가 러시아의 주요 전자상거래 물류센터를 타격하여 8명의 사망자를 발생시켰으며, 이는 러시아 국민의 일상에 전쟁의 대가를 실감케 하는 전략의 일환이다.</t>
+        </is>
+      </c>
+      <c r="F910" s="4" t="inlineStr">
+        <is>
+          <t>러시아-우크라이나 전쟁 관련 소식으로, 우리 회사의 주요 물류 경로 및 공급망에 직접적인 영향은 현재로서는 낮다.</t>
+        </is>
+      </c>
+      <c r="G910" s="4" t="n"/>
+      <c r="H910" s="4" t="inlineStr">
+        <is>
+          <t>중앙일보</t>
+        </is>
+      </c>
+      <c r="I910" s="4" t="inlineStr">
+        <is>
+          <t>https://joongang.co.kr/article/25446189</t>
+        </is>
+      </c>
+      <c r="J910" s="4" t="inlineStr"/>
+    </row>
+    <row r="911">
+      <c r="A911" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B911" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C911" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D911" s="4" t="inlineStr">
+        <is>
+          <t>에베레스트 오른 DJI, 허가 막힌 美… 세계 최고봉서 맞붙은 미중 드론 경쟁-국제ㅣ한국일보</t>
+        </is>
+      </c>
+      <c r="E911" s="4" t="inlineStr">
+        <is>
+          <t>중국 드론 기업 DJI가 에베레스트에서 화물 드론 시험 비행에 성공하며 미래 드론 산업의 가능성을 입증했으나, 미국에서는 허가 문제로 미중 드론 경쟁이 심화되고 있다.</t>
+        </is>
+      </c>
+      <c r="F911" s="4" t="inlineStr">
+        <is>
+          <t>드론 기술 발전 및 미중 경쟁에 대한 소식으로, 우리 회사의 현재 물류 운영에 직접적인 영향은 없으며 장기적인 기술 동향 참고 수준이다.</t>
+        </is>
+      </c>
+      <c r="G911" s="4" t="n"/>
+      <c r="H911" s="4" t="inlineStr">
+        <is>
+          <t>한국일보</t>
+        </is>
+      </c>
+      <c r="I911" s="4" t="inlineStr">
+        <is>
+          <t>https://www.hankookilbo.com/news/article/A2026070910250000193</t>
+        </is>
+      </c>
+      <c r="J911" s="4" t="inlineStr"/>
+    </row>
+    <row r="912">
+      <c r="A912" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B912" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C912" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D912" s="4" t="inlineStr">
+        <is>
+          <t>통합 대한항공, 제대로 비상할 수 있을까&amp;hellip;마일리지&amp;middot;계열사 '난제' 수두룩</t>
+        </is>
+      </c>
+      <c r="E912" s="4" t="inlineStr">
+        <is>
+          <t>대한항공과 아시아나항공의 통합 항공사 출범이 12월로 예정되어 있으나, 마일리지 및 계열사 문제 등 해결해야 할 난제가 많다.</t>
+        </is>
+      </c>
+      <c r="F912" s="4" t="inlineStr">
+        <is>
+          <t>국내 주요 항공사의 통합 소식으로, 장기적으로 항공 화물 운임 구조에 영향을 줄 수 있으나 당장 우리 회사의 물류 운영에 미치는 직접적인 영향은 낮다.</t>
+        </is>
+      </c>
+      <c r="G912" s="4" t="n"/>
+      <c r="H912" s="4" t="inlineStr">
+        <is>
+          <t>디지털데일리</t>
+        </is>
+      </c>
+      <c r="I912" s="4" t="inlineStr">
+        <is>
+          <t>https://ddaily.co.kr/page/view/2026071517053448483</t>
+        </is>
+      </c>
+      <c r="J912" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -41718,7 +43634,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -42568,6 +44484,49 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>3080.31</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>-105 (-3.3%)</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>+1,317 (+74.7%)</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="n">
+        <v>4318</v>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>-12 (-0.3%)</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>+1,728 (+66.7%)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -42580,7 +44539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I156"/>
+  <dimension ref="A1:I169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -48066,6 +50025,461 @@
       </c>
       <c r="I156" s="6" t="inlineStr"/>
     </row>
+    <row r="157">
+      <c r="A157" s="6" t="inlineStr">
+        <is>
+          <t>RSK-156</t>
+        </is>
+      </c>
+      <c r="B157" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C157" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D157" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E157" s="6" t="inlineStr">
+        <is>
+          <t>Section 301 Tariffs on Brazil Take Effect July 22, Stacking with Section 122 Duties; Strait of Hormuz Closure Restricts 200K TEU of Ocean Capacity</t>
+        </is>
+      </c>
+      <c r="F157" s="6" t="inlineStr"/>
+      <c r="G157" s="6" t="inlineStr"/>
+      <c r="H157" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 경유 노선 확인 및 대체 경로/운송 계획 수립, 브라질 및 러시아 관련 공급망 내 관세 영향 분석 및 대응 전략 마련.</t>
+        </is>
+      </c>
+      <c r="I157" s="6" t="inlineStr"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="6" t="inlineStr">
+        <is>
+          <t>RSK-157</t>
+        </is>
+      </c>
+      <c r="B158" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C158" s="6" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="D158" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E158" s="6" t="inlineStr">
+        <is>
+          <t>CBP Rejects Warehouse Entries on CAPE Declarations, Risking IEEPA Refunds; TPEB Rates Climb as Panama Canal Restrictions Tighten Capacity</t>
+        </is>
+      </c>
+      <c r="F158" s="6" t="inlineStr"/>
+      <c r="G158" s="6" t="inlineStr"/>
+      <c r="H158" s="6" t="inlineStr">
+        <is>
+          <t>파나마 운하 경유 노선에 대한 운송 계획 재검토 및 대체 경로/운송 수단 고려, CBP의 CAPE 선언 관련 지침 확인 및 통관 절차 준수 강화.</t>
+        </is>
+      </c>
+      <c r="I158" s="6" t="inlineStr"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="6" t="inlineStr">
+        <is>
+          <t>RSK-158</t>
+        </is>
+      </c>
+      <c r="B159" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C159" s="6" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="D159" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E159" s="6" t="inlineStr">
+        <is>
+          <t>CPSC Mandatory eFiling Takes Effect July 8; TPEB Rates Surge ~10% as Peak Season Demand Outpaces Capacity</t>
+        </is>
+      </c>
+      <c r="F159" s="6" t="inlineStr"/>
+      <c r="G159" s="6" t="inlineStr"/>
+      <c r="H159" s="6" t="inlineStr">
+        <is>
+          <t>CPSC eFiling 요건 확인 및 시스템 구축/준비, TPEB 운임 상승에 대비한 운송 계획 및 예산 재조정, 운송사와의 협상 강화.</t>
+        </is>
+      </c>
+      <c r="I159" s="6" t="inlineStr"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="6" t="inlineStr">
+        <is>
+          <t>RSK-159</t>
+        </is>
+      </c>
+      <c r="B160" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C160" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D160" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E160" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈 이어 홍해 봉쇄 위기... 다시 희망봉 돌아야 하나</t>
+        </is>
+      </c>
+      <c r="F160" s="6" t="inlineStr"/>
+      <c r="G160" s="6" t="inlineStr"/>
+      <c r="H160" s="6" t="inlineStr">
+        <is>
+          <t>아시아-유럽 항로의 운송 계획 재검토, 대체 경로 및 운송 수단 옵션 분석, 선사와의 긴밀한 소통을 통한 선복 확보 노력.</t>
+        </is>
+      </c>
+      <c r="I160" s="6" t="inlineStr"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="6" t="inlineStr">
+        <is>
+          <t>RSK-160</t>
+        </is>
+      </c>
+      <c r="B161" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C161" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D161" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E161" s="6" t="inlineStr">
+        <is>
+          <t>머스크, 극동아시아-북유럽·지중해 노선 성수기할증료 인상</t>
+        </is>
+      </c>
+      <c r="F161" s="6" t="inlineStr"/>
+      <c r="G161" s="6" t="inlineStr"/>
+      <c r="H161" s="6" t="inlineStr">
+        <is>
+          <t>해당 노선 운송 계획 및 예산 재검토, 선사와의 운임 협상 또는 대체 운송 방안 모색.</t>
+        </is>
+      </c>
+      <c r="I161" s="6" t="inlineStr"/>
+    </row>
+    <row r="162">
+      <c r="A162" s="6" t="inlineStr">
+        <is>
+          <t>RSK-161</t>
+        </is>
+      </c>
+      <c r="B162" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C162" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D162" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E162" s="6" t="inlineStr">
+        <is>
+          <t>끝나지 않은 중동 사태…'호르무즈 없는 시나리오' 짜는 산업계</t>
+        </is>
+      </c>
+      <c r="F162" s="6" t="inlineStr"/>
+      <c r="G162" s="6" t="inlineStr"/>
+      <c r="H162" s="6" t="inlineStr">
+        <is>
+          <t>중동 경유 항로의 잠재적 위험 평가 및 대체 운송 방안 검토, 운임 변동성 대비 예산 계획 수립, 비상 시나리오 구체화.</t>
+        </is>
+      </c>
+      <c r="I162" s="6" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="6" t="inlineStr">
+        <is>
+          <t>RSK-162</t>
+        </is>
+      </c>
+      <c r="B163" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C163" s="6" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="D163" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E163" s="6" t="inlineStr">
+        <is>
+          <t>쿠팡, 아직도 불 못껐다…급기야 굴삭기로 ‘건물 파괴’ 초강수</t>
+        </is>
+      </c>
+      <c r="F163" s="6" t="inlineStr"/>
+      <c r="G163" s="6" t="inlineStr"/>
+      <c r="H163" s="6" t="inlineStr">
+        <is>
+          <t>국내 물류센터 안전 관리 현황 점검 및 비상 계획 재검토, 위험물 보관 시설의 안전 규정 준수 여부 확인.</t>
+        </is>
+      </c>
+      <c r="I163" s="6" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="6" t="inlineStr">
+        <is>
+          <t>RSK-163</t>
+        </is>
+      </c>
+      <c r="B164" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C164" s="6" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="D164" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E164" s="6" t="inlineStr">
+        <is>
+          <t>국가소방동원령에도 쿠팡물류센터 불길 이틀째 안 잡힌 이유는</t>
+        </is>
+      </c>
+      <c r="F164" s="6" t="inlineStr"/>
+      <c r="G164" s="6" t="inlineStr"/>
+      <c r="H164" s="6" t="inlineStr">
+        <is>
+          <t>자체 물류센터 및 협력사 창고의 화재 안전 점검 강화, 위험물 보관 규정 준수 여부 재확인, 비상 재고 확보 및 대체 물류 경로 검토.</t>
+        </is>
+      </c>
+      <c r="I164" s="6" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="6" t="inlineStr">
+        <is>
+          <t>RSK-164</t>
+        </is>
+      </c>
+      <c r="B165" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C165" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D165" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E165" s="6" t="inlineStr">
+        <is>
+          <t>이란 혁명수비대 "호르무즈 배 2척 멈춰…美에 속아 진입하면 사고"</t>
+        </is>
+      </c>
+      <c r="F165" s="6" t="inlineStr"/>
+      <c r="G165" s="6" t="inlineStr"/>
+      <c r="H165" s="6" t="inlineStr">
+        <is>
+          <t>중동 항로를 이용하는 선박의 운항 상황 실시간 모니터링, 대체 항로 및 운송 수단 검토, 유가 및 운임 변동에 대한 헤징 전략 고려.</t>
+        </is>
+      </c>
+      <c r="I165" s="6" t="inlineStr"/>
+    </row>
+    <row r="166">
+      <c r="A166" s="6" t="inlineStr">
+        <is>
+          <t>RSK-165</t>
+        </is>
+      </c>
+      <c r="B166" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C166" s="6" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="D166" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E166" s="6" t="inlineStr">
+        <is>
+          <t>창고 가득한 생활용품이 ‘땔감’ 역할… 불 났다하면 대형 화재</t>
+        </is>
+      </c>
+      <c r="F166" s="6" t="inlineStr"/>
+      <c r="G166" s="6" t="inlineStr"/>
+      <c r="H166" s="6" t="inlineStr">
+        <is>
+          <t>자체 물류센터 및 협력사 창고의 화재 안전 점검 강화, 위험물 보관 규정 준수 여부 재확인, 비상 재고 확보 및 대체 물류 경로 검토.</t>
+        </is>
+      </c>
+      <c r="I166" s="6" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="6" t="inlineStr">
+        <is>
+          <t>RSK-166</t>
+        </is>
+      </c>
+      <c r="B167" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C167" s="6" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="D167" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E167" s="6" t="inlineStr">
+        <is>
+          <t>24시간 넘게 불타는 쿠팡 물류센터…“피해 수천억원 될 수도”</t>
+        </is>
+      </c>
+      <c r="F167" s="6" t="inlineStr"/>
+      <c r="G167" s="6" t="inlineStr"/>
+      <c r="H167" s="6" t="inlineStr">
+        <is>
+          <t>자체 물류센터 및 협력사 창고의 화재 안전 점검 강화, 위험물 보관 규정 준수 여부 재확인, 비상 재고 확보 및 대체 물류 경로 검토, 물류 보험 커버리지 재검토.</t>
+        </is>
+      </c>
+      <c r="I167" s="6" t="inlineStr"/>
+    </row>
+    <row r="168">
+      <c r="A168" s="6" t="inlineStr">
+        <is>
+          <t>RSK-167</t>
+        </is>
+      </c>
+      <c r="B168" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C168" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D168" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E168" s="6" t="inlineStr">
+        <is>
+          <t>[기획] 세계경제 흔드는 ‘호르무즈’… 유가 넘어 글로벌 공급망 재충격</t>
+        </is>
+      </c>
+      <c r="F168" s="6" t="inlineStr"/>
+      <c r="G168" s="6" t="inlineStr"/>
+      <c r="H168" s="6" t="inlineStr">
+        <is>
+          <t>중동 항로를 이용하는 선박의 운항 상황 및 유가, 해상 운임 변동 추이 실시간 모니터링, 비상 운송 계획 및 재고 수준 점검</t>
+        </is>
+      </c>
+      <c r="I168" s="6" t="inlineStr"/>
+    </row>
+    <row r="169">
+      <c r="A169" s="6" t="inlineStr">
+        <is>
+          <t>RSK-168</t>
+        </is>
+      </c>
+      <c r="B169" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C169" s="6" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="D169" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E169" s="6" t="inlineStr">
+        <is>
+          <t>연기 가득, 진화 난항…쿠팡 물류센터 화재 국가소방동원령 4차 발령</t>
+        </is>
+      </c>
+      <c r="F169" s="6" t="inlineStr"/>
+      <c r="G169" s="6" t="inlineStr"/>
+      <c r="H169" s="6" t="inlineStr">
+        <is>
+          <t>우리 회사 물류센터 및 협력사 창고의 화재 안전 점검 강화, 배터리/전자부품 등 위험물 보관 규정 준수 여부 재확인, 비상 계획 수립 및 훈련.</t>
+        </is>
+      </c>
+      <c r="I169" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
📰 뉴스 데이터 2026-07-21_08:57
</commit_message>
<xml_diff>
--- a/data/SCM_물류_브리핑.xlsx
+++ b/data/SCM_물류_브리핑.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J912"/>
+  <dimension ref="A1:J939"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -43622,6 +43622,1298 @@
       </c>
       <c r="J912" s="4" t="inlineStr"/>
     </row>
+    <row r="913">
+      <c r="A913" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B913" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C913" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D913" s="2" t="inlineStr">
+        <is>
+          <t>수요공급으로 설명되던 컨시장은 끝났다</t>
+        </is>
+      </c>
+      <c r="E913" s="2" t="inlineStr">
+        <is>
+          <t>지정학적 리스크 장기화로 글로벌 컨테이너선 시장이 비용 절감 중심에서 안정성과 회복탄력성을 중시하는 방향으로 전환되고 있다.</t>
+        </is>
+      </c>
+      <c r="F913" s="2" t="inlineStr">
+        <is>
+          <t>글로벌 컨테이너 시장의 전략적 전환은 우리 회사의 해상 운송 전략 및 공급망 회복탄력성 구축에 직접적인 영향을 미친다.</t>
+        </is>
+      </c>
+      <c r="G913" s="2" t="inlineStr">
+        <is>
+          <t>해상 운송 파트너십 재검토, 다중 운송 경로 및 운송사 확보 전략 수립, 재고 수준 및 안전 재고 정책 재평가.</t>
+        </is>
+      </c>
+      <c r="H913" s="2" t="inlineStr">
+        <is>
+          <t>kita</t>
+        </is>
+      </c>
+      <c r="I913" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kita.net/shippers/board/newsView.do?morgueCode=2&amp;dataCls=B&amp;dataSeq=8169</t>
+        </is>
+      </c>
+      <c r="J913" s="2" t="inlineStr">
+        <is>
+          <t>RSK-169</t>
+        </is>
+      </c>
+    </row>
+    <row r="914">
+      <c r="A914" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B914" s="2" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C914" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D914" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 이어 홍해 봉쇄 위기... 다시 희망봉 돌아야 하나 - surff</t>
+        </is>
+      </c>
+      <c r="E914" s="2" t="inlineStr">
+        <is>
+          <t>홍해 봉쇄 우려가 커지면서 아시아-유럽 항로가 희망봉 우회로 전환될 경우 운송기간과 연료비가 증가하고 선복 부족 및 운임 상승이 재현될 수 있다는 분석이 나왔다.</t>
+        </is>
+      </c>
+      <c r="F914" s="2" t="inlineStr">
+        <is>
+          <t>주요 해상 운송로 봉쇄는 아시아-유럽 항로의 운송 지연 및 비용 급증으로 이어져 우리 회사의 물류 운영 및 생산 계획에 직접적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G914" s="2" t="inlineStr">
+        <is>
+          <t>비상 운송 계획 수립, 대체 항로 및 운송 수단 검토, 주요 선사와의 긴밀한 소통을 통한 상황 변화 모니터링.</t>
+        </is>
+      </c>
+      <c r="H914" s="2" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I914" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260720-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J914" s="2" t="inlineStr">
+        <is>
+          <t>RSK-170</t>
+        </is>
+      </c>
+    </row>
+    <row r="915">
+      <c r="A915" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B915" s="2" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C915" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D915" s="2" t="inlineStr">
+        <is>
+          <t>쿠팡 화재 사흘째…‘전기차 20대분’ 로봇 배터리 불길 방어 총력 - ZDNet korea</t>
+        </is>
+      </c>
+      <c r="E915" s="2" t="inlineStr">
+        <is>
+          <t>인천 쿠팡 물류센터 화재가 사흘째 이어지는 가운데, 소방당국이 전기차 20대 분량의 리튬 배터리가 탑재된 물류 로봇이 있는 5층으로의 불길 확산을 막는 데 총력을 기울이고 있다.</t>
+        </is>
+      </c>
+      <c r="F915" s="2" t="inlineStr">
+        <is>
+          <t>배터리 제조기업으로서 물류센터 내 배터리 보관 및 취급 안전에 대한 경각심을 높이고, 유사 사고 발생 시 심각한 물류 운영 중단 및 인명 피해로 이어질 수 있음을 보여주는 사례이다.</t>
+        </is>
+      </c>
+      <c r="G915" s="2" t="inlineStr">
+        <is>
+          <t>자사 물류센터 및 협력사 물류센터의 배터리 보관 규정 및 화재 안전 시스템(소화 설비, 방화 구획 등) 점검, 위험물 취급 교육 강화, 비상 대응 계획 재검토.</t>
+        </is>
+      </c>
+      <c r="H915" s="2" t="inlineStr">
+        <is>
+          <t>ZDNet korea</t>
+        </is>
+      </c>
+      <c r="I915" s="2" t="inlineStr">
+        <is>
+          <t>https://zdnet.co.kr/view/?no=20260720152826</t>
+        </is>
+      </c>
+      <c r="J915" s="2" t="inlineStr">
+        <is>
+          <t>RSK-171</t>
+        </is>
+      </c>
+    </row>
+    <row r="916">
+      <c r="A916" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B916" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C916" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D916" s="2" t="inlineStr">
+        <is>
+          <t>[기획]관세發 K-수출 하반기 불확실성 더 커진다 - 매일일보</t>
+        </is>
+      </c>
+      <c r="E916" s="2" t="inlineStr">
+        <is>
+          <t>미국 무역대표부(USTR)가 한국산 제품에 12.5%의 추가 관세 부과 방안을 제안하면서 국내 수출기업의 하반기 경영 불확실성이 커지고 있다.</t>
+        </is>
+      </c>
+      <c r="F916" s="2" t="inlineStr">
+        <is>
+          <t>한국산 제품에 대한 추가 관세 부과는 배터리/전자부품 제조기업의 수출 물류 비용 및 전략에 직접적이고 즉각적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G916" s="2" t="inlineStr">
+        <is>
+          <t>관세 부과 동향 면밀히 모니터링, 관세 부과 시나리오별 수출 가격 및 물류 비용 영향 분석, 대체 운송 경로 또는 생산지 다변화 등 대응 전략 검토.</t>
+        </is>
+      </c>
+      <c r="H916" s="2" t="inlineStr">
+        <is>
+          <t>매일일보</t>
+        </is>
+      </c>
+      <c r="I916" s="2" t="inlineStr">
+        <is>
+          <t>https://m-i.kr/news/articleView.html?idxno=1392969</t>
+        </is>
+      </c>
+      <c r="J916" s="2" t="inlineStr">
+        <is>
+          <t>RSK-172</t>
+        </is>
+      </c>
+    </row>
+    <row r="917">
+      <c r="A917" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B917" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C917" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D917" s="2" t="inlineStr">
+        <is>
+          <t>글로벌 10% 관세 만료 눈앞…트럼프 무역장벽 더 높이나 | 한국경제</t>
+        </is>
+      </c>
+      <c r="E917" s="2" t="inlineStr">
+        <is>
+          <t>미국이 무역법 122조에 따른 글로벌 10% 관세 만료를 앞두고 무역법 301조를 근거로 한국, 중국 등 60개국에 대한 관세 부과를 준비하고 있어 무역장벽이 더 높아질 수 있다.</t>
+        </is>
+      </c>
+      <c r="F917" s="2" t="inlineStr">
+        <is>
+          <t>미국발 관세 정책 변화는 배터리/전자부품 제조기업의 글로벌 수출 전략 및 물류 비용에 직접적인 영향을 미치므로 즉각적인 대응이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G917" s="2" t="inlineStr">
+        <is>
+          <t>미국 관세 정책 변화 동향 면밀히 모니터링, 잠재적 관세 부과 대상 품목 및 세율 확인, 수출 시장 다변화 및 공급망 재편 가능성 검토.</t>
+        </is>
+      </c>
+      <c r="H917" s="2" t="inlineStr">
+        <is>
+          <t>한국경제</t>
+        </is>
+      </c>
+      <c r="I917" s="2" t="inlineStr">
+        <is>
+          <t>https://hankyung.com/article/2026071928891</t>
+        </is>
+      </c>
+      <c r="J917" s="2" t="inlineStr">
+        <is>
+          <t>RSK-173</t>
+        </is>
+      </c>
+    </row>
+    <row r="918">
+      <c r="A918" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B918" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C918" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D918" s="2" t="inlineStr">
+        <is>
+          <t>이란 원전 건설현장 때린 美 … 국제유가 90弗 재돌파</t>
+        </is>
+      </c>
+      <c r="E918" s="2" t="inlineStr">
+        <is>
+          <t>미국이 이란 원전 건설 현장을 공격하면서 국제유가가 배럴당 90달러를 재돌파했으며, 이는 중동 긴장 고조로 인한 공급망 불안과 인플레이션 압력 가중으로 이어질 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="F918" s="2" t="inlineStr">
+        <is>
+          <t>국제유가 상승은 해상 및 항공 운임의 유류할증료 인상으로 직결되어 우리 회사의 물류비용에 즉각적인 영향을 미치며, 중동 리스크는 주요 해상 운송로의 불안정성을 높일 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G918" s="2" t="inlineStr">
+        <is>
+          <t>유가 변동에 따른 운임 인상 가능성을 예측하고, 운송 계약 조건 재검토 및 대체 운송 경로/방안을 사전에 검토하며, 재고 수준 및 운송 스케줄 조정 가능성을 평가합니다.</t>
+        </is>
+      </c>
+      <c r="H918" s="2" t="inlineStr">
+        <is>
+          <t>매일경제</t>
+        </is>
+      </c>
+      <c r="I918" s="2" t="inlineStr">
+        <is>
+          <t>https://mk.co.kr/news/world/12102616</t>
+        </is>
+      </c>
+      <c r="J918" s="2" t="inlineStr">
+        <is>
+          <t>RSK-174</t>
+        </is>
+      </c>
+    </row>
+    <row r="919">
+      <c r="A919" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B919" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C919" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D919" s="2" t="inlineStr">
+        <is>
+          <t>대한항공 2분기 매출 늘었지만 유가·환율 탓 이익 급감, 조원태 글로벌 불확실성 '통제'와 아시아나항공 안정적 '통합' 이중 과제</t>
+        </is>
+      </c>
+      <c r="E919" s="2" t="inlineStr">
+        <is>
+          <t>대한항공의 2분기 매출은 여객 및 화물 수요 증가로 늘었으나, 크게 오른 유가와 환율 영향으로 영업이익이 급감하며 수익성이 악화되었습니다.</t>
+        </is>
+      </c>
+      <c r="F919" s="2" t="inlineStr">
+        <is>
+          <t>항공사의 수익성 악화는 유가 및 환율 변동이 항공 운임에 직접적으로 반영될 가능성을 높이며, 이는 우리 회사의 항공 운송 비용 증가로 이어질 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G919" s="2" t="inlineStr">
+        <is>
+          <t>유가 및 환율 변동 추이를 면밀히 모니터링하고, 항공 운임 인상 가능성에 대비하여 운송 계약 조건을 재검토하며, 필요시 해상 운송 등 대체 운송 수단 활용을 고려합니다.</t>
+        </is>
+      </c>
+      <c r="H919" s="2" t="inlineStr">
+        <is>
+          <t>허프포스트코리아</t>
+        </is>
+      </c>
+      <c r="I919" s="2" t="inlineStr">
+        <is>
+          <t>https://huffingtonpost.kr/article/258847</t>
+        </is>
+      </c>
+      <c r="J919" s="2" t="inlineStr">
+        <is>
+          <t>RSK-175</t>
+        </is>
+      </c>
+    </row>
+    <row r="920">
+      <c r="A920" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B920" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C920" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D920" s="3" t="inlineStr">
+        <is>
+          <t>Statement on EU Commission Revision of the EU Emissions Trading System</t>
+        </is>
+      </c>
+      <c r="E920" s="3" t="inlineStr">
+        <is>
+          <t>IATA는 EU ETS(배출권 거래 시스템)의 유럽 국경 외 확장 제안에 대해 깊은 불만을 표명하며, 이는 항공 운송 비용 증가로 이어질 수 있다고 경고했다.</t>
+        </is>
+      </c>
+      <c r="F920" s="3" t="inlineStr">
+        <is>
+          <t>EU ETS의 유럽 국경 외 확장은 항공 운송 비용 증가로 이어져 항공 화물 운임 상승 압력으로 작용할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G920" s="3" t="inlineStr">
+        <is>
+          <t>항공 운송 비용 변화 추이 모니터링 및 잠재적 운임 인상에 대비한 예산 검토.</t>
+        </is>
+      </c>
+      <c r="H920" s="3" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I920" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/07-17-statement-eu-commission-revision-emissions-trading-system/</t>
+        </is>
+      </c>
+      <c r="J920" s="3" t="inlineStr"/>
+    </row>
+    <row r="921">
+      <c r="A921" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B921" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C921" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D921" s="3" t="inlineStr">
+        <is>
+          <t>Air Cargo Demand Up 6.0% in May</t>
+        </is>
+      </c>
+      <c r="E921" s="3" t="inlineStr">
+        <is>
+          <t>2026년 5월 전 세계 항공 화물 수요가 전년 대비 6.0% 증가하여 항공 운송 시장의 활황세를 보였다.</t>
+        </is>
+      </c>
+      <c r="F921" s="3" t="inlineStr">
+        <is>
+          <t>항공 화물 수요 증가는 항공 운송 공간 확보 경쟁을 심화시키고 운임 상승으로 이어질 수 있어 물류 비용에 직접적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G921" s="3" t="inlineStr">
+        <is>
+          <t>항공 운임 추이 및 가용성 지속 모니터링, 필요시 운송 계획 조정 검토.</t>
+        </is>
+      </c>
+      <c r="H921" s="3" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I921" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-29-air-cargo-demand-up-may/</t>
+        </is>
+      </c>
+      <c r="J921" s="3" t="inlineStr"/>
+    </row>
+    <row r="922">
+      <c r="A922" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B922" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C922" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D922" s="3" t="inlineStr">
+        <is>
+          <t>Structural Contraction of Global Liner Networks</t>
+        </is>
+      </c>
+      <c r="E922" s="3" t="inlineStr">
+        <is>
+          <t>2012년 이후 글로벌 라이너 네트워크 데이터 분석 결과, 선사들이 지리적 범위는 유지하면서도 서비스 빈도를 줄이는 등 네트워크 관리 방식에 근본적인 변화가 있음을 보여준다.</t>
+        </is>
+      </c>
+      <c r="F922" s="3" t="inlineStr">
+        <is>
+          <t>해상 운송 네트워크의 서비스 빈도 감소는 운송 리드타임 증가 및 스케줄 유연성 저하로 이어질 수 있다.</t>
+        </is>
+      </c>
+      <c r="G922" s="3" t="inlineStr">
+        <is>
+          <t>해상 운송 스케줄 및 서비스 빈도 변화 모니터링, 운송 리드타임 증가에 대비한 재고 및 생산 계획 조정 검토.</t>
+        </is>
+      </c>
+      <c r="H922" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I922" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/397-structural-contraction-of-global-liner-networks</t>
+        </is>
+      </c>
+      <c r="J922" s="3" t="inlineStr"/>
+    </row>
+    <row r="923">
+      <c r="A923" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B923" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C923" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D923" s="3" t="inlineStr">
+        <is>
+          <t>PLSCI Data Indicates Mega-Hub Retrenchment</t>
+        </is>
+      </c>
+      <c r="E923" s="3" t="inlineStr">
+        <is>
+          <t>2026년 2분기 PLSCI(항만 라이너 선박 연결성 지수) 분석 결과, 최근 네트워크 재조정이 반응적 대응에서 선제적 대응으로 전환되며 메가 허브 항만들이 축소되는 경향을 보인다.</t>
+        </is>
+      </c>
+      <c r="F923" s="3" t="inlineStr">
+        <is>
+          <t>주요 메가 허브 항만의 연결성 변화는 우리 회사의 해상 운송 경로 및 환적 효율성에 영향을 미쳐 잠재적으로 운송 시간 증가나 비용 상승을 초래할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G923" s="3" t="inlineStr">
+        <is>
+          <t>주요 항만 연결성 지표 및 운송 경로 변화 모니터링, 필요시 대체 항만 및 운송 경로 검토.</t>
+        </is>
+      </c>
+      <c r="H923" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I923" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/396-plsci-data-indicates-mega-hub-retrenchment</t>
+        </is>
+      </c>
+      <c r="J923" s="3" t="inlineStr"/>
+    </row>
+    <row r="924">
+      <c r="A924" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B924" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C924" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D924" s="3" t="inlineStr">
+        <is>
+          <t>Tracking True Vessel Delay</t>
+        </is>
+      </c>
+      <c r="E924" s="3" t="inlineStr">
+        <is>
+          <t>선사들이 운송 시간을 늘리는 '스케줄 버퍼링'에 의존하면서 실제 선박 지연과 스케줄 버퍼링 간의 관계를 분석하여 운송 리드타임 예측의 중요성을 강조했다.</t>
+        </is>
+      </c>
+      <c r="F924" s="3" t="inlineStr">
+        <is>
+          <t>선사들이 스케줄 버퍼링을 통해 운송 시간을 늘리는 경향은 우리 회사의 운송 리드타임 예측 및 재고 계획에 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G924" s="3" t="inlineStr">
+        <is>
+          <t>운송사별 실제 운송 리드타임과 공시된 스케줄 간의 차이 분석, 재고 및 생산 계획에 반영.</t>
+        </is>
+      </c>
+      <c r="H924" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I924" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/394-tracking-true-vessel-delay</t>
+        </is>
+      </c>
+      <c r="J924" s="3" t="inlineStr"/>
+    </row>
+    <row r="925">
+      <c r="A925" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B925" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C925" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D925" s="3" t="inlineStr">
+        <is>
+          <t>VLCC 13.7% 하락한 118,483달러...8만4000cbm급 LPG운반선 운임 중 미주-동아시아 운임은 13.8% 상승</t>
+        </is>
+      </c>
+      <c r="E925" s="3" t="inlineStr">
+        <is>
+          <t>VLCC 운임은 하락하고 LPG 운반선 운임은 상승하는 등 선종별 운임 변동이 있었으며, 컨테이너 정기선 운임은 성수기 강세 기조를 유지했다.</t>
+        </is>
+      </c>
+      <c r="F925" s="3" t="inlineStr">
+        <is>
+          <t>우리 회사는 배터리/전자부품 제조기업이므로 컨테이너 운임이 가장 중요하며, 컨테이너 운임 강세 기조는 물류비 상승 압박으로 작용할 수 있어 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G925" s="3" t="inlineStr">
+        <is>
+          <t>컨테이너 운임 추이 지속 모니터링 및 운송 계약 조건 검토.</t>
+        </is>
+      </c>
+      <c r="H925" s="3" t="inlineStr">
+        <is>
+          <t>shippingnews</t>
+        </is>
+      </c>
+      <c r="I925" s="3" t="inlineStr">
+        <is>
+          <t>https://www.shippingnewsnet.com/news/articleView.html?idxno=71245</t>
+        </is>
+      </c>
+      <c r="J925" s="3" t="inlineStr"/>
+    </row>
+    <row r="926">
+      <c r="A926" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B926" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C926" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D926" s="3" t="inlineStr">
+        <is>
+          <t>진입 힘든 내부에 가연성 생활용품 빼곡 … 창문도 없어 진화 어려워 - 매일경제</t>
+        </is>
+      </c>
+      <c r="E926" s="3" t="inlineStr">
+        <is>
+          <t>인천 쿠팡 물류센터 화재가 장기화되는 가운데, 메자닌 복층 구조와 가연성 생활용품, 5층의 리튬 배터리 로봇이 진화를 어렵게 하고 있으며, 2024년 이전 허가 물류창고의 안전기준 미흡 문제가 제기되었다.</t>
+        </is>
+      </c>
+      <c r="F926" s="3" t="inlineStr">
+        <is>
+          <t>물류창고 화재 시 리튬 배터리의 위험성이 다시 부각되었고, 기존 물류창고의 안전 기준 미흡 문제가 제기되어 향후 배터리 보관 및 위험물 창고 규제 강화 논의로 이어질 수 있으므로 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G926" s="3" t="inlineStr">
+        <is>
+          <t>사내 위험물 보관 창고의 안전 점검 및 규제 동향 주시.</t>
+        </is>
+      </c>
+      <c r="H926" s="3" t="inlineStr">
+        <is>
+          <t>매일경제</t>
+        </is>
+      </c>
+      <c r="I926" s="3" t="inlineStr">
+        <is>
+          <t>https://mk.co.kr/news/society/12102656</t>
+        </is>
+      </c>
+      <c r="J926" s="3" t="inlineStr"/>
+    </row>
+    <row r="927">
+      <c r="A927" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B927" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C927" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D927" s="3" t="inlineStr">
+        <is>
+          <t>Vol132. 주간 선사별 동향 (Week 29, 2026) (주간 선사 동향)</t>
+        </is>
+      </c>
+      <c r="E927" s="3" t="inlineStr">
+        <is>
+          <t>머스크가 서아프리카 및 인도·중동-미국 동안 항로를 희망봉 우회에서 수에즈·홍해 항로로 전환하며 운송 일수를 단축하고 있으나, 극동아시아-북유럽·지중해 노선에 성수기 할증료를 인상했다.</t>
+        </is>
+      </c>
+      <c r="F927" s="3" t="inlineStr">
+        <is>
+          <t>주요 선사의 홍해/수에즈 복귀는 긍정적이나, 여전히 성수기 할증료 인상이 발생하고 있어 운임 변동 가능성을 지속적으로 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G927" s="3" t="inlineStr">
+        <is>
+          <t>주요 선사의 항로 운영 및 운임 정책 변화 지속 모니터링.</t>
+        </is>
+      </c>
+      <c r="H927" s="3" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I927" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/vol132-주간-선사별-동향-week-29-2026</t>
+        </is>
+      </c>
+      <c r="J927" s="3" t="inlineStr"/>
+    </row>
+    <row r="928">
+      <c r="A928" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B928" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C928" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D928" s="3" t="inlineStr">
+        <is>
+          <t>반복되는 물류센터 화재…강화된 기준에도 기존시설은 사각지대 - 파이낸셜뉴스</t>
+        </is>
+      </c>
+      <c r="E928" s="3" t="inlineStr">
+        <is>
+          <t>반복되는 물류센터 화재에도 불구하고 2024년부터 강화된 스프링클러 기준이 기존 시설에는 적용되지 않아 안전 사각지대가 발생하고 있으며, 전문가들은 기존 시설의 안전성 보완 대책 마련을 촉구하고 있다.</t>
+        </is>
+      </c>
+      <c r="F928" s="3" t="inlineStr">
+        <is>
+          <t>현재는 기존 시설에 대한 규제 강화가 없지만, 쿠팡 화재와 같은 대형 사고가 반복되면 기존 물류센터에 대한 안전 규제 강화 논의가 시작될 수 있어 향후 물류 운영에 영향을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="G928" s="3" t="inlineStr">
+        <is>
+          <t>물류센터 화재 관련 규제 동향 지속 모니터링, 자사 및 협력사 물류센터의 안전 기준 준수 여부 선제적 점검 및 개선 방안 검토.</t>
+        </is>
+      </c>
+      <c r="H928" s="3" t="inlineStr">
+        <is>
+          <t>파이낸셜뉴스</t>
+        </is>
+      </c>
+      <c r="I928" s="3" t="inlineStr">
+        <is>
+          <t>https://fnnews.com/news/202607201229505639</t>
+        </is>
+      </c>
+      <c r="J928" s="3" t="inlineStr"/>
+    </row>
+    <row r="929">
+      <c r="A929" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B929" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C929" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D929" s="3" t="inlineStr">
+        <is>
+          <t>中 자동차 부품기업 태국 인니 동남아 공장 진출 가속</t>
+        </is>
+      </c>
+      <c r="E929" s="3" t="inlineStr">
+        <is>
+          <t>중국 자동차 부품 기업들이 글로벌 경쟁력 강화와 공급망 다변화를 위해 태국, 인도네시아 등 동남아시아로 공장 진출을 가속화하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F929" s="3" t="inlineStr">
+        <is>
+          <t>동남아시아 지역의 물류 인프라 및 공급망 환경 변화 가능성을 시사하며, 장기적으로 우리 회사의 부품 조달 또는 생산 거점 전략에 영향을 줄 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G929" s="3" t="inlineStr">
+        <is>
+          <t>동남아시아 지역의 물류 인프라 개발 동향 및 잠재적 공급망 파트너 변화를 지속적으로 모니터링하고, 필요시 공급망 다변화 전략을 검토합니다.</t>
+        </is>
+      </c>
+      <c r="H929" s="3" t="inlineStr">
+        <is>
+          <t>뉴스핌</t>
+        </is>
+      </c>
+      <c r="I929" s="3" t="inlineStr">
+        <is>
+          <t>https://www.newspim.com/news/view/20260720000762</t>
+        </is>
+      </c>
+      <c r="J929" s="3" t="inlineStr"/>
+    </row>
+    <row r="930">
+      <c r="A930" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B930" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C930" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D930" s="3" t="inlineStr">
+        <is>
+          <t>코트라, 디트로이트서 韓자동차 부품사 포드·스텔란티스 공급망 연결</t>
+        </is>
+      </c>
+      <c r="E930" s="3" t="inlineStr">
+        <is>
+          <t>KOTRA가 미국발 관세와 전기차 전환, 현지화 확대에 대응하여 한국 자동차 부품사들이 포드, 스텔란티스 등 글로벌 완성차 공급망에 진입하도록 지원하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F930" s="3" t="inlineStr">
+        <is>
+          <t>미국 시장의 현지화 및 관세 정책은 우리 회사의 북미 지역 공급망 전략 및 고객사와의 관계에 간접적인 영향을 미칠 수 있으며, 특히 EV 부품 공급 시 중요하게 고려해야 할 요소입니다.</t>
+        </is>
+      </c>
+      <c r="G930" s="3" t="inlineStr">
+        <is>
+          <t>북미 시장의 무역 정책 및 현지화 동향을 지속적으로 모니터링하고, 주요 고객사의 공급망 현지화 전략 변화에 대한 정보를 수집하여 잠재적 기회 또는 리스크를 평가합니다.</t>
+        </is>
+      </c>
+      <c r="H930" s="3" t="inlineStr">
+        <is>
+          <t>서울경제</t>
+        </is>
+      </c>
+      <c r="I930" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sedaily.com/article/20069033</t>
+        </is>
+      </c>
+      <c r="J930" s="3" t="inlineStr"/>
+    </row>
+    <row r="931">
+      <c r="A931" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B931" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C931" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D931" s="4" t="inlineStr">
+        <is>
+          <t>삼영물류-SF익스프레스, 크로스보더 물류 협력</t>
+        </is>
+      </c>
+      <c r="E931" s="4" t="inlineStr">
+        <is>
+          <t>삼영물류와 SF익스프레스코리아가 크로스보더 이커머스 물류사업을 공동 추진하기 위해 협력하여 국내외 물류 인프라와 운송 네트워크를 결합한 엔드투엔드 서비스를 제공한다.</t>
+        </is>
+      </c>
+      <c r="F931" s="4" t="inlineStr">
+        <is>
+          <t>국내외 물류 기업 간 협력은 시장 경쟁을 촉진할 수 있으나, 우리 회사의 B2B 중심 물류 운영에 직접적인 영향은 미미하다.</t>
+        </is>
+      </c>
+      <c r="G931" s="4" t="n"/>
+      <c r="H931" s="4" t="inlineStr">
+        <is>
+          <t>ksg</t>
+        </is>
+      </c>
+      <c r="I931" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksg.co.kr/news/main_newsView.jsp?pNum=147654</t>
+        </is>
+      </c>
+      <c r="J931" s="4" t="inlineStr"/>
+    </row>
+    <row r="932">
+      <c r="A932" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B932" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C932" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D932" s="4" t="inlineStr">
+        <is>
+          <t>Global Schedule Reliability for May 2026 the Highest of the Year</t>
+        </is>
+      </c>
+      <c r="E932" s="4" t="inlineStr">
+        <is>
+          <t>2026년 5월 글로벌 선박 스케줄 신뢰도가 올해 최고치를 기록하여 해상 운송의 정시성이 개선되었다.</t>
+        </is>
+      </c>
+      <c r="F932" s="4" t="inlineStr">
+        <is>
+          <t>해상 운송 스케줄 신뢰도 개선은 운송 계획 수립에 긍정적이나, 이는 단기적인 지표일 수 있으며 지속적인 개선 여부를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G932" s="4" t="inlineStr">
+        <is>
+          <t>해상 운송 스케줄 신뢰도 추이 지속 모니터링.</t>
+        </is>
+      </c>
+      <c r="H932" s="4" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I932" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/395-global-schedule-reliability-for-may-2026-the-highest-of-the-year</t>
+        </is>
+      </c>
+      <c r="J932" s="4" t="inlineStr"/>
+    </row>
+    <row r="933">
+      <c r="A933" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B933" s="4" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C933" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D933" s="4" t="inlineStr">
+        <is>
+          <t>러시아, 우크라 오데사 항구 화물선에 미사일 공격, 10명 사망 - surff</t>
+        </is>
+      </c>
+      <c r="E933" s="4" t="inlineStr">
+        <is>
+          <t>러시아가 우크라이나 오데사 항구의 화물선을 미사일로 공격하여 10명이 사망하는 사건이 발생했다.</t>
+        </is>
+      </c>
+      <c r="F933" s="4" t="inlineStr">
+        <is>
+          <t>우크라이나 항구 공격은 해당 지역의 물류에 직접적인 영향을 미치지만, 우리 회사의 주요 운송 경로와는 거리가 있어 당장 직접적인 영향은 낮다.</t>
+        </is>
+      </c>
+      <c r="G933" s="4" t="n"/>
+      <c r="H933" s="4" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I933" s="4" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260721-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J933" s="4" t="inlineStr"/>
+    </row>
+    <row r="934">
+      <c r="A934" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B934" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C934" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D934" s="4" t="inlineStr">
+        <is>
+          <t>중동 불안에 닻 올린 중국 조선…전 세계 주문 싹쓸이 - surff</t>
+        </is>
+      </c>
+      <c r="E934" s="4" t="inlineStr">
+        <is>
+          <t>중동 불안으로 운송 거리가 늘어나면서 선복 부족 우려가 커지자 중국 조선업이 전 세계 선박 주문을 싹쓸이하며 선복 공급 확대에 기여할 것으로 예상된다.</t>
+        </is>
+      </c>
+      <c r="F934" s="4" t="inlineStr">
+        <is>
+          <t>장기적으로 선복 공급 확대에 긍정적일 수 있으나, 단기적인 우리 물류 운영에는 직접적인 영향이 낮다.</t>
+        </is>
+      </c>
+      <c r="G934" s="4" t="n"/>
+      <c r="H934" s="4" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I934" s="4" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260720-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J934" s="4" t="inlineStr"/>
+    </row>
+    <row r="935">
+      <c r="A935" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B935" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C935" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D935" s="4" t="inlineStr">
+        <is>
+          <t>이베코코리아 / 연비·안전·주행 편의성 향상 대형 트랙터 ‘올 뉴 S-Way’ 출시</t>
+        </is>
+      </c>
+      <c r="E935" s="4" t="inlineStr">
+        <is>
+          <t>이베코코리아가 연비, 안전, 주행 편의성을 향상시킨 대형 트랙터 '올 뉴 S-Way'를 출시하여 운송 사업자의 운영 효율을 높이고 운전자에게 안전하고 편안한 환경을 제공할 것으로 기대된다.</t>
+        </is>
+      </c>
+      <c r="F935" s="4" t="inlineStr">
+        <is>
+          <t>신형 트랙터 출시는 장기적으로 육상 운송 효율 개선에 기여할 수 있으나, 당장 우리 회사의 물류 운영에 직접적인 영향은 낮다.</t>
+        </is>
+      </c>
+      <c r="G935" s="4" t="n"/>
+      <c r="H935" s="4" t="inlineStr">
+        <is>
+          <t>ulogistics</t>
+        </is>
+      </c>
+      <c r="I935" s="4" t="inlineStr">
+        <is>
+          <t>http://www.ulogistics.co.kr/test/board.php?board=all2&amp;command=body&amp;no=5212</t>
+        </is>
+      </c>
+      <c r="J935" s="4" t="inlineStr"/>
+    </row>
+    <row r="936">
+      <c r="A936" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B936" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C936" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D936" s="4" t="inlineStr">
+        <is>
+          <t>Hyperlocal Supply Chains Are Emerging As Hospitality’s Next Big Asset</t>
+        </is>
+      </c>
+      <c r="E936" s="4" t="inlineStr">
+        <is>
+          <t>기후 변화로 인한 공급망 교란에 대응하기 위해 호텔 산업에서 효율성보다는 회복탄력성을 강조하는 하이퍼로컬 공급망이 부상하고 있다.</t>
+        </is>
+      </c>
+      <c r="F936" s="4" t="inlineStr">
+        <is>
+          <t>호텔 산업의 공급망 변화에 대한 내용으로, 배터리/전자부품 제조기업의 직접적인 물류 운영에 당장 영향을 미치지는 않는다.</t>
+        </is>
+      </c>
+      <c r="G936" s="4" t="inlineStr"/>
+      <c r="H936" s="4" t="inlineStr">
+        <is>
+          <t>Forbes</t>
+        </is>
+      </c>
+      <c r="I936" s="4" t="inlineStr">
+        <is>
+          <t>https://forbes.com/sites/indrabatilahiri/2026/07/19/hyperlocal-supply-chains-are-emerging-as-hospitalitys-next-big-asset</t>
+        </is>
+      </c>
+      <c r="J936" s="4" t="inlineStr"/>
+    </row>
+    <row r="937">
+      <c r="A937" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B937" s="4" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C937" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D937" s="4" t="inlineStr">
+        <is>
+          <t>화물차·지게차·작업자 동선 색으로 구분…CJ제일제당 안전 강화 | 한국경제</t>
+        </is>
+      </c>
+      <c r="E937" s="4" t="inlineStr">
+        <is>
+          <t>CJ제일제당이 식품업계 최초로 CUD(Color Universal Design)를 적용하여 화물차, 지게차, 작업자 동선을 색으로 구분하는 등 물류센터 안전을 강화하고 있다.</t>
+        </is>
+      </c>
+      <c r="F937" s="4" t="inlineStr">
+        <is>
+          <t>물류센터 안전 강화 노력의 일환으로 참고할 만한 사례이나, 배터리/전자부품 제조기업의 물류 운영에 직접적인 영향을 미치는 규제나 위험물 관련 이슈는 아니다.</t>
+        </is>
+      </c>
+      <c r="G937" s="4" t="inlineStr"/>
+      <c r="H937" s="4" t="inlineStr">
+        <is>
+          <t>한국경제</t>
+        </is>
+      </c>
+      <c r="I937" s="4" t="inlineStr">
+        <is>
+          <t>https://hankyung.com/article/202607203490g</t>
+        </is>
+      </c>
+      <c r="J937" s="4" t="inlineStr"/>
+    </row>
+    <row r="938">
+      <c r="A938" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B938" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C938" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D938" s="4" t="inlineStr">
+        <is>
+          <t>재활용업계 "정부 자원순환정책 사각지대 해소해야" &lt; 신재생.환경 &lt; 기사본문 - 에너지데일리</t>
+        </is>
+      </c>
+      <c r="E938" s="4" t="inlineStr">
+        <is>
+          <t>재활용업계가 탄소중립 및 순환경제 전환 정책 속에서 미신고 사업장 난립 등 정부 자원순환정책의 사각지대 해소를 요구하고 있다.</t>
+        </is>
+      </c>
+      <c r="F938" s="4" t="inlineStr">
+        <is>
+          <t>재활용 산업의 정책적 이슈로, 배터리/전자부품 제조기업의 물류 운영에 직접적인 영향을 미치는 위험물 규제나 안전 문제와는 거리가 있다.</t>
+        </is>
+      </c>
+      <c r="G938" s="4" t="inlineStr"/>
+      <c r="H938" s="4" t="inlineStr">
+        <is>
+          <t>에너지데일리</t>
+        </is>
+      </c>
+      <c r="I938" s="4" t="inlineStr">
+        <is>
+          <t>https://energydaily.co.kr/news/articleView.html?idxno=201524</t>
+        </is>
+      </c>
+      <c r="J938" s="4" t="inlineStr"/>
+    </row>
+    <row r="939">
+      <c r="A939" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B939" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C939" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D939" s="4" t="inlineStr">
+        <is>
+          <t>"고맙다, 외국인 환승특수"…항공사 실적 버팀목으로</t>
+        </is>
+      </c>
+      <c r="E939" s="4" t="inlineStr">
+        <is>
+          <t>중동전 여파로 두바이공항 대체 수요가 인천공항으로 몰리면서 외국인 환승객이 증가하여 항공사 실적에 긍정적인 영향을 미치고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F939" s="4" t="inlineStr">
+        <is>
+          <t>주로 여객 환승 특수에 대한 내용으로, 우리 회사의 항공 화물 운송에 직접적인 영향은 미미하며, 오히려 항공사 실적 개선은 장기적으로 항공 화물 서비스 안정화에 기여할 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G939" s="4" t="inlineStr"/>
+      <c r="H939" s="4" t="inlineStr">
+        <is>
+          <t>매일경제</t>
+        </is>
+      </c>
+      <c r="I939" s="4" t="inlineStr">
+        <is>
+          <t>https://mk.co.kr/news/business/12102636</t>
+        </is>
+      </c>
+      <c r="J939" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -43634,7 +44926,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -44527,6 +45819,49 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>3080.31</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>-105 (-3.3%)</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>+1,317 (+74.7%)</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="n">
+        <v>4204</v>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>-114 (-2.6%)</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>+1,755 (+71.7%)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -44539,7 +45874,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I169"/>
+  <dimension ref="A1:I176"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -50480,6 +51815,251 @@
       </c>
       <c r="I169" s="6" t="inlineStr"/>
     </row>
+    <row r="170">
+      <c r="A170" s="6" t="inlineStr">
+        <is>
+          <t>RSK-169</t>
+        </is>
+      </c>
+      <c r="B170" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C170" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D170" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E170" s="6" t="inlineStr">
+        <is>
+          <t>수요공급으로 설명되던 컨시장은 끝났다</t>
+        </is>
+      </c>
+      <c r="F170" s="6" t="inlineStr"/>
+      <c r="G170" s="6" t="inlineStr"/>
+      <c r="H170" s="6" t="inlineStr">
+        <is>
+          <t>해상 운송 파트너십 재검토, 다중 운송 경로 및 운송사 확보 전략 수립, 재고 수준 및 안전 재고 정책 재평가.</t>
+        </is>
+      </c>
+      <c r="I170" s="6" t="inlineStr"/>
+    </row>
+    <row r="171">
+      <c r="A171" s="6" t="inlineStr">
+        <is>
+          <t>RSK-170</t>
+        </is>
+      </c>
+      <c r="B171" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C171" s="6" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="D171" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E171" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈 이어 홍해 봉쇄 위기... 다시 희망봉 돌아야 하나 - surff</t>
+        </is>
+      </c>
+      <c r="F171" s="6" t="inlineStr"/>
+      <c r="G171" s="6" t="inlineStr"/>
+      <c r="H171" s="6" t="inlineStr">
+        <is>
+          <t>비상 운송 계획 수립, 대체 항로 및 운송 수단 검토, 주요 선사와의 긴밀한 소통을 통한 상황 변화 모니터링.</t>
+        </is>
+      </c>
+      <c r="I171" s="6" t="inlineStr"/>
+    </row>
+    <row r="172">
+      <c r="A172" s="6" t="inlineStr">
+        <is>
+          <t>RSK-171</t>
+        </is>
+      </c>
+      <c r="B172" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C172" s="6" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="D172" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E172" s="6" t="inlineStr">
+        <is>
+          <t>쿠팡 화재 사흘째…‘전기차 20대분’ 로봇 배터리 불길 방어 총력 - ZDNet korea</t>
+        </is>
+      </c>
+      <c r="F172" s="6" t="inlineStr"/>
+      <c r="G172" s="6" t="inlineStr"/>
+      <c r="H172" s="6" t="inlineStr">
+        <is>
+          <t>자사 물류센터 및 협력사 물류센터의 배터리 보관 규정 및 화재 안전 시스템(소화 설비, 방화 구획 등) 점검, 위험물 취급 교육 강화, 비상 대응 계획 재검토.</t>
+        </is>
+      </c>
+      <c r="I172" s="6" t="inlineStr"/>
+    </row>
+    <row r="173">
+      <c r="A173" s="6" t="inlineStr">
+        <is>
+          <t>RSK-172</t>
+        </is>
+      </c>
+      <c r="B173" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C173" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D173" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E173" s="6" t="inlineStr">
+        <is>
+          <t>[기획]관세發 K-수출 하반기 불확실성 더 커진다 - 매일일보</t>
+        </is>
+      </c>
+      <c r="F173" s="6" t="inlineStr"/>
+      <c r="G173" s="6" t="inlineStr"/>
+      <c r="H173" s="6" t="inlineStr">
+        <is>
+          <t>관세 부과 동향 면밀히 모니터링, 관세 부과 시나리오별 수출 가격 및 물류 비용 영향 분석, 대체 운송 경로 또는 생산지 다변화 등 대응 전략 검토.</t>
+        </is>
+      </c>
+      <c r="I173" s="6" t="inlineStr"/>
+    </row>
+    <row r="174">
+      <c r="A174" s="6" t="inlineStr">
+        <is>
+          <t>RSK-173</t>
+        </is>
+      </c>
+      <c r="B174" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C174" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D174" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E174" s="6" t="inlineStr">
+        <is>
+          <t>글로벌 10% 관세 만료 눈앞…트럼프 무역장벽 더 높이나 | 한국경제</t>
+        </is>
+      </c>
+      <c r="F174" s="6" t="inlineStr"/>
+      <c r="G174" s="6" t="inlineStr"/>
+      <c r="H174" s="6" t="inlineStr">
+        <is>
+          <t>미국 관세 정책 변화 동향 면밀히 모니터링, 잠재적 관세 부과 대상 품목 및 세율 확인, 수출 시장 다변화 및 공급망 재편 가능성 검토.</t>
+        </is>
+      </c>
+      <c r="I174" s="6" t="inlineStr"/>
+    </row>
+    <row r="175">
+      <c r="A175" s="6" t="inlineStr">
+        <is>
+          <t>RSK-174</t>
+        </is>
+      </c>
+      <c r="B175" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C175" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D175" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E175" s="6" t="inlineStr">
+        <is>
+          <t>이란 원전 건설현장 때린 美 … 국제유가 90弗 재돌파</t>
+        </is>
+      </c>
+      <c r="F175" s="6" t="inlineStr"/>
+      <c r="G175" s="6" t="inlineStr"/>
+      <c r="H175" s="6" t="inlineStr">
+        <is>
+          <t>유가 변동에 따른 운임 인상 가능성을 예측하고, 운송 계약 조건 재검토 및 대체 운송 경로/방안을 사전에 검토하며, 재고 수준 및 운송 스케줄 조정 가능성을 평가합니다.</t>
+        </is>
+      </c>
+      <c r="I175" s="6" t="inlineStr"/>
+    </row>
+    <row r="176">
+      <c r="A176" s="6" t="inlineStr">
+        <is>
+          <t>RSK-175</t>
+        </is>
+      </c>
+      <c r="B176" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C176" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D176" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E176" s="6" t="inlineStr">
+        <is>
+          <t>대한항공 2분기 매출 늘었지만 유가·환율 탓 이익 급감, 조원태 글로벌 불확실성 '통제'와 아시아나항공 안정적 '통합' 이중 과제</t>
+        </is>
+      </c>
+      <c r="F176" s="6" t="inlineStr"/>
+      <c r="G176" s="6" t="inlineStr"/>
+      <c r="H176" s="6" t="inlineStr">
+        <is>
+          <t>유가 및 환율 변동 추이를 면밀히 모니터링하고, 항공 운임 인상 가능성에 대비하여 운송 계약 조건을 재검토하며, 필요시 해상 운송 등 대체 운송 수단 활용을 고려합니다.</t>
+        </is>
+      </c>
+      <c r="I176" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
📰 뉴스 데이터 2026-07-22_08:57
</commit_message>
<xml_diff>
--- a/data/SCM_물류_브리핑.xlsx
+++ b/data/SCM_물류_브리핑.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J939"/>
+  <dimension ref="A1:J977"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -44914,6 +44914,1806 @@
       </c>
       <c r="J939" s="4" t="inlineStr"/>
     </row>
+    <row r="940">
+      <c r="A940" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B940" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C940" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D940" s="2" t="inlineStr">
+        <is>
+          <t>Section 301 Tariffs on Brazil Take Effect July 22, Stacking with Section 122 Duties; Strait of Hormuz Closure Restricts 200K TEU of Ocean Capacity</t>
+        </is>
+      </c>
+      <c r="E940" s="2" t="inlineStr">
+        <is>
+          <t>브라질에 대한 Section 301 관세가 7월 22일 발효되며, 호르무즈 해협 폐쇄로 20만 TEU의 해상 운송 용량이 제한될 수 있다. 또한 러시아 제재 법안이 중국, 인도에 2차 관세를 부과할 가능성도 언급되었다.</t>
+        </is>
+      </c>
+      <c r="F940" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 폐쇄는 중동 항로를 이용하는 선박의 운항에 직접적인 영향을 주어 해상 운송 지연 및 비용 상승을 유발할 수 있으며, 브라질 및 러시아 관련 관세는 특정 지역과의 무역 비용에 즉각적인 영향을 미친다.</t>
+        </is>
+      </c>
+      <c r="G940" s="2" t="inlineStr">
+        <is>
+          <t>중동 항로 이용 여부 및 대체 경로 검토, 브라질 및 러시아 관련 무역 거래에 대한 관세 영향 분석 및 대응 방안 마련.</t>
+        </is>
+      </c>
+      <c r="H940" s="2" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I940" s="2" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/july-16-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J940" s="2" t="inlineStr">
+        <is>
+          <t>RSK-176</t>
+        </is>
+      </c>
+    </row>
+    <row r="941">
+      <c r="A941" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B941" s="2" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C941" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D941" s="2" t="inlineStr">
+        <is>
+          <t>홍해 봉쇄 위기 고조, 아시아-유럽 항로 희망봉 우회 가능성</t>
+        </is>
+      </c>
+      <c r="E941" s="2" t="inlineStr">
+        <is>
+          <t>홍해 봉쇄 우려가 커지면서 아시아-유럽 항로가 희망봉 우회로 전환될 경우 운송기간과 연료비 증가, 선복 부족 및 운임 상승이 재현될 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="F941" s="2" t="inlineStr">
+        <is>
+          <t>아시아-유럽 항로는 우리 회사의 주요 수출입 경로 중 하나로, 홍해 봉쇄로 인한 희망봉 우회는 운송 리드타임 및 물류비용에 직접적이고 심각한 영향을 미칠 것입니다.</t>
+        </is>
+      </c>
+      <c r="G941" s="2" t="inlineStr">
+        <is>
+          <t>아시아-유럽 노선 운송 계획 재검토, 대체 운송 경로 및 운송 수단(항공 등) 비상 계획 수립, 선사와의 긴밀한 소통을 통한 상황 변화 주시.</t>
+        </is>
+      </c>
+      <c r="H941" s="2" t="inlineStr">
+        <is>
+          <t>Surff (데일리스크랩)</t>
+        </is>
+      </c>
+      <c r="I941" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260720-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J941" s="2" t="inlineStr">
+        <is>
+          <t>RSK-177</t>
+        </is>
+      </c>
+    </row>
+    <row r="942">
+      <c r="A942" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B942" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C942" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D942" s="2" t="inlineStr">
+        <is>
+          <t>홍해 봉쇄 위기, 중동 원유 수송 차질로 유가 120달러 재돌파 우려</t>
+        </is>
+      </c>
+      <c r="E942" s="2" t="inlineStr">
+        <is>
+          <t>친이란 후티 반군의 홍해 봉쇄 선언으로 중동 원유 수송에 차질이 발생할 경우, 유가가 120달러를 재돌파하며 한국 등 아시아 지역에 에너지 쇼크가 발생할 수 있다는 우려가 제기됩니다.</t>
+        </is>
+      </c>
+      <c r="F942" s="2" t="inlineStr">
+        <is>
+          <t>유가 급등은 해상 및 항공 운송의 연료비 상승으로 직결되어 우리 회사의 물류비용에 직접적이고 심각한 영향을 미칠 것이며, 이는 제품 원가 상승으로 이어질 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G942" s="2" t="inlineStr">
+        <is>
+          <t>유가 변동 추이 및 물류비에 미치는 영향 분석, 운송 계약 시 유류할증료 조건 재검토, 에너지 효율적인 운송 방안 모색.</t>
+        </is>
+      </c>
+      <c r="H942" s="2" t="inlineStr">
+        <is>
+          <t>매일경제</t>
+        </is>
+      </c>
+      <c r="I942" s="2" t="inlineStr">
+        <is>
+          <t>https://mk.co.kr/news/world/12103585</t>
+        </is>
+      </c>
+      <c r="J942" s="2" t="inlineStr">
+        <is>
+          <t>RSK-178</t>
+        </is>
+      </c>
+    </row>
+    <row r="943">
+      <c r="A943" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B943" s="2" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C943" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D943" s="2" t="inlineStr">
+        <is>
+          <t>쿠팡 4·5층 모두 '화약고'였다… "리튬배터리 로봇 수백 대·포장비닐 빼곡"-사회ㅣ한국일보</t>
+        </is>
+      </c>
+      <c r="E943" s="2" t="inlineStr">
+        <is>
+          <t>인천 쿠팡 물류센터 화재 진압 과정에서 4, 5층에 리튬 배터리 로봇 수백 대와 가연성 포장재가 대량 적재되어 화재 확산 및 폭발 위험이 컸으며, 이는 물류센터의 화재 안전관리 및 방재 체계 강화의 필요성을 부각시키고 있다.</t>
+        </is>
+      </c>
+      <c r="F943" s="2" t="inlineStr">
+        <is>
+          <t>우리 회사가 취급하는 리튬 배터리의 물류센터 내 보관 안전성 문제와 직결되며, 향후 위험물 보관 규제 강화 및 물류센터 안전 인허가 기준 변화로 이어질 가능성이 매우 높아 즉각적인 대응이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G943" s="2" t="inlineStr">
+        <is>
+          <t>현재 물류센터 내 리튬 배터리 보관 현황 및 안전 관리 절차를 점검하고, 협력 물류센터의 화재 안전 시스템 및 위험물 취급 규정 준수 여부를 확인한다. 관련 규제 동향을 모니터링하고 선제적 대응 방안 및 비상 계획을 마련한다.</t>
+        </is>
+      </c>
+      <c r="H943" s="2" t="inlineStr">
+        <is>
+          <t>한국일보</t>
+        </is>
+      </c>
+      <c r="I943" s="2" t="inlineStr">
+        <is>
+          <t>https://hankookilbo.com/news/article/A2026072114280001860</t>
+        </is>
+      </c>
+      <c r="J943" s="2" t="inlineStr">
+        <is>
+          <t>RSK-179</t>
+        </is>
+      </c>
+    </row>
+    <row r="944">
+      <c r="A944" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B944" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C944" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D944" s="2" t="inlineStr">
+        <is>
+          <t>철강은 “산 넘어 산”…배터리는 소재비 긴장 [관세 리셋, 美 301조의 경고] - 이투데이</t>
+        </is>
+      </c>
+      <c r="E944" s="2" t="inlineStr">
+        <is>
+          <t>미국이 10% 글로벌 관세 종료 후 무역법 301조에 따른 추가 관세를 예고하며, 특히 배터리 산업은 현지 생산에도 수입 소재 관세 변수로 인해 소재비 긴장이 고조되고 있다.</t>
+        </is>
+      </c>
+      <c r="F944" s="2" t="inlineStr">
+        <is>
+          <t>배터리 소재 수입 관세 부과는 우리 제품의 원가 상승 및 가격 경쟁력 약화로 이어져 생산 계획 및 공급망 전략에 직접적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G944" s="2" t="inlineStr">
+        <is>
+          <t>미국향 수출 제품 및 소재의 원산지 규정 준수 여부를 재검토하고, 관세 부과 시나리오별 원가 영향 분석 및 공급망 다변화 전략을 수립해야 함.</t>
+        </is>
+      </c>
+      <c r="H944" s="2" t="inlineStr">
+        <is>
+          <t>이투데이</t>
+        </is>
+      </c>
+      <c r="I944" s="2" t="inlineStr">
+        <is>
+          <t>https://etoday.co.kr/news/view/2605699</t>
+        </is>
+      </c>
+      <c r="J944" s="2" t="inlineStr">
+        <is>
+          <t>RSK-180</t>
+        </is>
+      </c>
+    </row>
+    <row r="945">
+      <c r="A945" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B945" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C945" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D945" s="2" t="inlineStr">
+        <is>
+          <t>중동 긴장 재고조…항공·해운 비용 부담에 '초긴장' - 매일일보</t>
+        </is>
+      </c>
+      <c r="E945" s="2" t="inlineStr">
+        <is>
+          <t>중동 지역의 군사적 긴장이 재고조되면서 국제유가가 급등하고, 이로 인해 국내 항공·해운 업계의 운임 상승 및 물류 비용 부담이 커질 것으로 예상된다.</t>
+        </is>
+      </c>
+      <c r="F945" s="2" t="inlineStr">
+        <is>
+          <t>유가 상승은 해상 및 항공 운임에 직접적인 영향을 미쳐 우리 회사의 물류비용을 증가시키고, 이는 제품 원가 및 수익성에 즉각적인 악영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G945" s="2" t="inlineStr">
+        <is>
+          <t>중동 정세 및 국제 유가 동향을 면밀히 주시하고, 물류비 상승에 대비하여 운송 계약 조건 재검토, 운송 모드 전환 검토, 재고 수준 조정 등 비상 계획을 수립해야 함.</t>
+        </is>
+      </c>
+      <c r="H945" s="2" t="inlineStr">
+        <is>
+          <t>매일일보</t>
+        </is>
+      </c>
+      <c r="I945" s="2" t="inlineStr">
+        <is>
+          <t>https://m-i.kr/news/articleView.html?idxno=1392973</t>
+        </is>
+      </c>
+      <c r="J945" s="2" t="inlineStr">
+        <is>
+          <t>RSK-181</t>
+        </is>
+      </c>
+    </row>
+    <row r="946">
+      <c r="A946" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B946" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C946" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D946" s="3" t="inlineStr">
+        <is>
+          <t>CBP Rejects Warehouse Entries on CAPE Declarations, Risking IEEPA Refunds; TPEB Rates Climb as Panama Canal Restrictions Tighten Capacity</t>
+        </is>
+      </c>
+      <c r="E946" s="3" t="inlineStr">
+        <is>
+          <t>CBP가 CAPE 신고에 대한 창고 입고를 거부하여 IEEPA 환급에 위험을 초래하고 있으며, 파나마 운하의 통행 제한 강화로 태평양 횡단 동향(TPEB) 운임이 상승하고 있다. CPSC의 eFiling 의무화 기한도 7월 8일 발효되었다.</t>
+        </is>
+      </c>
+      <c r="F946" s="3" t="inlineStr">
+        <is>
+          <t>파나마 운하 통행 제한 강화는 태평양 횡단 운송에 영향을 미쳐 운임 상승 및 운송 지연을 야기할 수 있으며, CBP의 새로운 규정은 통관 절차에 영향을 줄 수 있으므로 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G946" s="3" t="inlineStr">
+        <is>
+          <t>파나마 운하를 이용하는 운송 경로 및 스케줄에 대한 영향 분석, CBP의 CAPE 및 CPSC eFiling 규정 준수 여부 확인 및 필요 시 프로세스 업데이트.</t>
+        </is>
+      </c>
+      <c r="H946" s="3" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I946" s="3" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/july-09-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J946" s="3" t="inlineStr"/>
+    </row>
+    <row r="947">
+      <c r="A947" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B947" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C947" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D947" s="3" t="inlineStr">
+        <is>
+          <t>U.S.-EU Trade Agreement Eliminates Duties on Most U.S. Goods Starting July 1; TPEB Rates Rise as July Capacity Hits Three-Year High</t>
+        </is>
+      </c>
+      <c r="E947" s="3" t="inlineStr">
+        <is>
+          <t>미국-EU 무역 협정이 7월 1일부터 발효되어 대부분의 미국산 공산품에 대한 관세가 철폐되었으며, 7월 태평양 횡단 동향(TPEB) 운임이 상승하고 용량은 3년 만에 최고치를 기록했다.</t>
+        </is>
+      </c>
+      <c r="F947" s="3" t="inlineStr">
+        <is>
+          <t>미국-EU 무역 협정은 해당 지역으로의 수출입 관세에 긍정적인 영향을 줄 수 있으나, TPEB 운임 상승은 전체 물류 비용에 영향을 미칠 수 있어 지속적인 추이 관찰이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G947" s="3" t="inlineStr">
+        <is>
+          <t>미국-EU 무역 협정으로 인한 관세 절감 효과 분석 및 활용 방안 검토, TPEB 운임 변동에 따른 운송 계획 및 예산 재검토.</t>
+        </is>
+      </c>
+      <c r="H947" s="3" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I947" s="3" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/july-02-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J947" s="3" t="inlineStr"/>
+    </row>
+    <row r="948">
+      <c r="A948" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B948" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C948" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D948" s="3" t="inlineStr">
+        <is>
+          <t>CAPE Phase 2 Launches June 29 for Reconciliation-Flagged Entries; TPEB Rates Rise 10% for Sixth Consecutive Week</t>
+        </is>
+      </c>
+      <c r="E948" s="3" t="inlineStr">
+        <is>
+          <t>CBP의 CAPE IEEPA 관세 환급 시스템 2단계가 6월 29일 시작되어 환급 대상이 확대되었으며, 태평양 횡단 동향(TPEB) 운임이 6주 연속 10% 상승했다.</t>
+        </is>
+      </c>
+      <c r="F948" s="3" t="inlineStr">
+        <is>
+          <t>CAPE 시스템 확장은 관세 환급 기회를 제공할 수 있으나, TPEB 운임의 지속적인 상승은 물류 비용에 직접적인 영향을 미치므로 면밀한 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G948" s="3" t="inlineStr">
+        <is>
+          <t>CAPE 시스템을 통한 관세 환급 가능성 검토, TPEB 운임 상승에 대비한 운송 계약 및 예산 조정 검토.</t>
+        </is>
+      </c>
+      <c r="H948" s="3" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I948" s="3" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/june-25-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J948" s="3" t="inlineStr"/>
+    </row>
+    <row r="949">
+      <c r="A949" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B949" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C949" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D949" s="3" t="inlineStr">
+        <is>
+          <t>CPSC Mandatory eFiling Takes Effect July 8; TPEB Rates Surge ~10% as Peak Season Demand Outpaces Capacity</t>
+        </is>
+      </c>
+      <c r="E949" s="3" t="inlineStr">
+        <is>
+          <t>CPSC의 의무적인 eFiling이 7월 8일 발효되었으며, 성수기 수요가 공급을 초과하면서 태평양 횡단 동향(TPEB) 운임이 약 10% 급등했다. CBP는 강제 노동 관련 통합 지침을 발표했다.</t>
+        </is>
+      </c>
+      <c r="F949" s="3" t="inlineStr">
+        <is>
+          <t>CPSC eFiling 의무화는 미국 수출 제품의 통관 절차에 영향을 주며, TPEB 운임 급등은 물류 비용 상승을 야기하고, 강제 노동 지침은 공급망 실사에 영향을 미치므로 지속적인 모니터링과 대비가 필요하다.</t>
+        </is>
+      </c>
+      <c r="G949" s="3" t="inlineStr">
+        <is>
+          <t>CPSC eFiling 규정 준수 여부 확인 및 시스템 준비, TPEB 운임 상승에 따른 운송 전략 및 예산 재검토, CBP의 강제 노동 지침에 대한 공급망 실사 강화.</t>
+        </is>
+      </c>
+      <c r="H949" s="3" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I949" s="3" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/june-18-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J949" s="3" t="inlineStr"/>
+    </row>
+    <row r="950">
+      <c r="A950" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B950" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C950" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D950" s="3" t="inlineStr">
+        <is>
+          <t>Statement on EU Commission Revision of the EU Emissions Trading System</t>
+        </is>
+      </c>
+      <c r="E950" s="3" t="inlineStr">
+        <is>
+          <t>IATA는 EU 배출권 거래 시스템(ETS)의 유럽 국경 외 확장 제안에 대해 깊은 우려를 표명하며, 이는 항공 운송 비용 증가로 이어질 수 있다고 밝혔다.</t>
+        </is>
+      </c>
+      <c r="F950" s="3" t="inlineStr">
+        <is>
+          <t>EU ETS의 확장 적용은 항공 운송 비용 증가로 이어져 우리 회사의 항공 물류 비용에 영향을 미칠 수 있으므로, 관련 논의 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G950" s="3" t="inlineStr">
+        <is>
+          <t>EU ETS 확장 적용 시 항공 운송 비용 변화 시뮬레이션 및 잠재적 영향 분석.</t>
+        </is>
+      </c>
+      <c r="H950" s="3" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I950" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/07-17-statement-eu-commission-revision-emissions-trading-system/</t>
+        </is>
+      </c>
+      <c r="J950" s="3" t="inlineStr"/>
+    </row>
+    <row r="951">
+      <c r="A951" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B951" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C951" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D951" s="3" t="inlineStr">
+        <is>
+          <t>고유가에도 웃는 항공 화물… 위기 겪는 LCC도 앞다퉈 진출</t>
+        </is>
+      </c>
+      <c r="E951" s="3" t="inlineStr">
+        <is>
+          <t>반도체 특수와 해상 운송 불안정으로 항공 화물 수요와 운임이 상승세를 보이며, 대한항공 등 화물 사업 중심 항공사들이 실적 호조를 기록하고 있다.</t>
+        </is>
+      </c>
+      <c r="F951" s="3" t="inlineStr">
+        <is>
+          <t>해상 운송 불안정으로 인한 항공 화물 수요 및 운임 상승은 우리 회사의 항공 운송 비용 증가로 이어질 수 있으므로 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G951" s="3" t="inlineStr">
+        <is>
+          <t>항공 운송 시장 동향 및 운임 추이 면밀히 관찰, 해상 운송 지연 시 항공 운송 전환 비용 효율성 분석.</t>
+        </is>
+      </c>
+      <c r="H951" s="3" t="inlineStr">
+        <is>
+          <t>kita</t>
+        </is>
+      </c>
+      <c r="I951" s="3" t="inlineStr">
+        <is>
+          <t>https://www.kita.net/shippers/board/newsView.do?morgueCode=2&amp;dataCls=C&amp;dataSeq=2861</t>
+        </is>
+      </c>
+      <c r="J951" s="3" t="inlineStr"/>
+    </row>
+    <row r="952">
+      <c r="A952" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B952" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C952" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D952" s="3" t="inlineStr">
+        <is>
+          <t>Structural Contraction of Global Liner Networks</t>
+        </is>
+      </c>
+      <c r="E952" s="3" t="inlineStr">
+        <is>
+          <t>IMF 보고서에 따르면 2026년 글로벌 무역량 성장률이 3.5%로 급격히 둔화될 것으로 예상되며, 이는 글로벌 선사 네트워크의 구조적 축소를 야기할 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="F952" s="3" t="inlineStr">
+        <is>
+          <t>글로벌 무역량 둔화는 해운 수요 감소로 이어져 장기적으로 운임 안정화에 기여할 수 있으나, 선사들의 네트워크 축소는 특정 노선의 선복 감소나 서비스 빈도 저하로 이어질 수 있어 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G952" s="3" t="inlineStr">
+        <is>
+          <t>주요 운송 노선의 선복 공급 및 서비스 빈도 변화 추이 모니터링.</t>
+        </is>
+      </c>
+      <c r="H952" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I952" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/398-structural-contraction-of-global-liner-network</t>
+        </is>
+      </c>
+      <c r="J952" s="3" t="inlineStr"/>
+    </row>
+    <row r="953">
+      <c r="A953" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B953" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C953" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D953" s="3" t="inlineStr">
+        <is>
+          <t>Structural Contraction of Global Liner Networks</t>
+        </is>
+      </c>
+      <c r="E953" s="3" t="inlineStr">
+        <is>
+          <t>글로벌 선사 네트워크 데이터 분석 결과, 선사들이 지리적 거점은 유지하면서도 서비스 빈도를 줄이는 방식으로 네트워크를 관리하는 근본적인 변화가 나타나고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F953" s="3" t="inlineStr">
+        <is>
+          <t>선사들의 서비스 빈도 감소는 우리 제품의 운송 리드타임 증가나 스케줄 유연성 저하로 이어질 수 있으므로, 주요 노선의 서비스 변화를 지속적으로 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G953" s="3" t="inlineStr">
+        <is>
+          <t>주요 운송 노선의 선사별 서비스 빈도 및 스케줄 변화 추이 모니터링.</t>
+        </is>
+      </c>
+      <c r="H953" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I953" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/397-structural-contraction-of-global-liner-networks</t>
+        </is>
+      </c>
+      <c r="J953" s="3" t="inlineStr"/>
+    </row>
+    <row r="954">
+      <c r="A954" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B954" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C954" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D954" s="3" t="inlineStr">
+        <is>
+          <t>PLSCI Data Indicates Mega-Hub Retrenchment</t>
+        </is>
+      </c>
+      <c r="E954" s="3" t="inlineStr">
+        <is>
+          <t>UNCTAD의 2026년 2분기 항만 선박 연결성 지수(PLSCI) 분석 결과, 최근 네트워크 재조정이 메가 허브 항만에서의 서비스 축소로 전환되고 있음을 시사합니다.</t>
+        </is>
+      </c>
+      <c r="F954" s="3" t="inlineStr">
+        <is>
+          <t>메가 허브 항만에서의 서비스 축소는 주요 환적 항만에서의 연결성 저하 및 운송 지연을 야기할 수 있으므로, 우리 제품의 주요 경유 항만 변화를 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G954" s="3" t="inlineStr">
+        <is>
+          <t>주요 환적 항만 및 경유 항만의 연결성 지수 변화 추이 모니터링 및 대체 항만 옵션 검토.</t>
+        </is>
+      </c>
+      <c r="H954" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I954" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/396-plsci-data-indicates-mega-hub-retrenchment</t>
+        </is>
+      </c>
+      <c r="J954" s="3" t="inlineStr"/>
+    </row>
+    <row r="955">
+      <c r="A955" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B955" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C955" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D955" s="3" t="inlineStr">
+        <is>
+          <t>Tracking True Vessel Delay</t>
+        </is>
+      </c>
+      <c r="E955" s="3" t="inlineStr">
+        <is>
+          <t>선사들이 운송 시간을 늘려 스케줄 버퍼링을 활용함으로써 실제 선박 지연을 완화하고 있으나, 이는 명목상 운송 기간 증가로 이어질 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="F955" s="3" t="inlineStr">
+        <is>
+          <t>선사들의 스케줄 버퍼링 전략은 겉으로는 정시성 개선처럼 보일 수 있으나, 실제 운송 리드타임이 길어질 수 있어 생산 계획 및 재고 관리에 영향을 줄 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G955" s="3" t="inlineStr">
+        <is>
+          <t>주요 운송 노선의 실제 운송 리드타임 변화를 면밀히 분석하고, 선사와의 계약 시 명목상 스케줄 외 실제 운송 기간 확인.</t>
+        </is>
+      </c>
+      <c r="H955" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I955" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/394-tracking-true-vessel-delay</t>
+        </is>
+      </c>
+      <c r="J955" s="3" t="inlineStr"/>
+    </row>
+    <row r="956">
+      <c r="A956" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B956" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C956" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D956" s="3" t="inlineStr">
+        <is>
+          <t>트럼프, 캐나다에 관세 폭탄… 북미 무역협정 균열 조짐</t>
+        </is>
+      </c>
+      <c r="E956" s="3" t="inlineStr">
+        <is>
+          <t>트럼프 전 대통령이 캐나다에 관세 부과를 시사하며 북미 무역협정에 균열 조짐이 보이고 있어, 북미 지역의 무역 환경 불확실성이 증가하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F956" s="3" t="inlineStr">
+        <is>
+          <t>북미 지역에 대한 관세 부과 및 무역 분쟁은 해당 지역으로의 수출입 비용 증가 및 공급망 재편을 야기할 수 있으므로, 관련 동향을 주시해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G956" s="3" t="inlineStr">
+        <is>
+          <t>북미 지역 수출입 비중 및 해당 지역 공급망 현황 점검, 관세 부과 시나리오별 영향 분석 준비.</t>
+        </is>
+      </c>
+      <c r="H956" s="3" t="inlineStr">
+        <is>
+          <t>Surff (데일리스크랩)</t>
+        </is>
+      </c>
+      <c r="I956" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260722-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J956" s="3" t="inlineStr"/>
+    </row>
+    <row r="957">
+      <c r="A957" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B957" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C957" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D957" s="3" t="inlineStr">
+        <is>
+          <t>인천 쿠팡 물류센터 대형 화재, 붕괴 위험 속 진화 장기화</t>
+        </is>
+      </c>
+      <c r="E957" s="3" t="inlineStr">
+        <is>
+          <t>인천 쿠팡 물류센터에서 대형 화재가 사흘째 이어지며 붕괴 위험 속에 진화에 어려움을 겪고 있어 물류창고 안전 및 규제에 대한 관심이 높아지고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F957" s="3" t="inlineStr">
+        <is>
+          <t>대형 물류센터 화재는 배터리 등 위험물을 취급하는 우리 회사의 창고 안전 규제 강화 논의로 이어질 수 있으며, 유사 사고 발생 시 물류 운영에 심각한 차질을 초래할 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G957" s="3" t="inlineStr">
+        <is>
+          <t>국내외 물류창고 안전 규제 동향 모니터링, 자사 창고의 화재 예방 및 비상 대응 시스템 점검, 위험물 보관 규정 준수 여부 재확인.</t>
+        </is>
+      </c>
+      <c r="H957" s="3" t="inlineStr">
+        <is>
+          <t>Surff (데일리스크랩)</t>
+        </is>
+      </c>
+      <c r="I957" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260720-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J957" s="3" t="inlineStr"/>
+    </row>
+    <row r="958">
+      <c r="A958" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B958" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C958" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D958" s="3" t="inlineStr">
+        <is>
+          <t>항만 물동량 증가 속 터미널 처리능력 병목 현상 심화</t>
+        </is>
+      </c>
+      <c r="E958" s="3" t="inlineStr">
+        <is>
+          <t>미국 로스앤젤레스·롱비치 항만 등에서 관세 인상에 따른 조기 선적으로 역대급 물동량을 기록 중이며, 선박 입항보다 터미널의 선석·야드·게이트 처리능력이 병목으로 작용하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F958" s="3" t="inlineStr">
+        <is>
+          <t>주요 항만의 터미널 처리능력 병목은 항만 적체와 운송 지연을 야기할 수 있으며, 이는 우리 제품의 수출입 일정에 영향을 미칠 수 있으므로 주요 항만의 상황을 주시해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G958" s="3" t="inlineStr">
+        <is>
+          <t>주요 수출입 항만의 터미널 혼잡도 및 처리 능력 모니터링, 필요시 대체 항만 또는 운송 방식 검토.</t>
+        </is>
+      </c>
+      <c r="H958" s="3" t="inlineStr">
+        <is>
+          <t>Surff (물류101)</t>
+        </is>
+      </c>
+      <c r="I958" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/항만이-역대급-물동량을-소화하는-법-터미널-처리능력이라는-숨은-병목-week-29-2026-</t>
+        </is>
+      </c>
+      <c r="J958" s="3" t="inlineStr"/>
+    </row>
+    <row r="959">
+      <c r="A959" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B959" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C959" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D959" s="3" t="inlineStr">
+        <is>
+          <t>Will the Bab el-Mandeb Blockade Impact Oil and Shipping Prices?</t>
+        </is>
+      </c>
+      <c r="E959" s="3" t="inlineStr">
+        <is>
+          <t>바브엘만데브 해협 봉쇄가 유가 및 해운 운임에 미칠 영향에 대한 분석으로, 호르무즈 해협과 동시 봉쇄 시 더 큰 위험을 초래할 수 있다고 경고한다.</t>
+        </is>
+      </c>
+      <c r="F959" s="3" t="inlineStr">
+        <is>
+          <t>주요 해협 봉쇄는 해상 운송 경로 변경 및 운임 상승으로 이어져, 우리 회사의 글로벌 물류 비용과 리드타임에 잠재적 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G959" s="3" t="inlineStr">
+        <is>
+          <t>해협 상황 및 주요 선사들의 우회 경로, 운임 인상 동향을 지속적으로 모니터링하고 비상 운송 계획을 검토한다.</t>
+        </is>
+      </c>
+      <c r="H959" s="3" t="inlineStr">
+        <is>
+          <t>Northeastern Global News</t>
+        </is>
+      </c>
+      <c r="I959" s="3" t="inlineStr">
+        <is>
+          <t>https://news.northeastern.edu/2026/07/21/houthi-blockade-bab-el-mandeb-strait</t>
+        </is>
+      </c>
+      <c r="J959" s="3" t="inlineStr"/>
+    </row>
+    <row r="960">
+      <c r="A960" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B960" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C960" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D960" s="3" t="inlineStr">
+        <is>
+          <t>EU 알리익스프레스, 불법·위험상품 판매 조장…9300억 과징금 부과 | 한국경제</t>
+        </is>
+      </c>
+      <c r="E960" s="3" t="inlineStr">
+        <is>
+          <t>EU가 알리익스프레스에 불법 및 위험 상품 판매를 조장한 혐의로 9300억 원의 과징금을 부과했으며, 소액 관세 면제 제도 철폐 및 수수료 부과 논의도 진행 중이다.</t>
+        </is>
+      </c>
+      <c r="F960" s="3" t="inlineStr">
+        <is>
+          <t>EU의 '위험상품' 판매 조장 규제는 향후 배터리/전자부품의 온라인 판매 및 통관 규제 강화로 이어질 가능성이 있으며, 소액관세면제제도 철폐는 B2C 물량의 관세 부담을 증가시킬 수 있어 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G960" s="3" t="inlineStr">
+        <is>
+          <t>EU의 온라인 플랫폼 규제 및 위험물 관련 상품 판매 규제 동향, 그리고 소액 관세 면제 제도 변경 사항을 지속적으로 모니터링한다.</t>
+        </is>
+      </c>
+      <c r="H960" s="3" t="inlineStr">
+        <is>
+          <t>한국경제</t>
+        </is>
+      </c>
+      <c r="I960" s="3" t="inlineStr">
+        <is>
+          <t>https://hankyung.com/article/202607205430i</t>
+        </is>
+      </c>
+      <c r="J960" s="3" t="inlineStr"/>
+    </row>
+    <row r="961">
+      <c r="A961" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B961" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C961" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D961" s="3" t="inlineStr">
+        <is>
+          <t>[단독] 3년 전에도 12시간 불…인천 쿠팡, 불났다 하면 대형 화재 왜 | 중앙일보</t>
+        </is>
+      </c>
+      <c r="E961" s="3" t="inlineStr">
+        <is>
+          <t>물류센터 화재가 잇따르면서 소방 당국이 물류시설 화재 원인 및 현행 화재 안전 관련 제도와 규제의 적정성을 점검할 계획이다.</t>
+        </is>
+      </c>
+      <c r="F961" s="3" t="inlineStr">
+        <is>
+          <t>물류센터 화재 안전 규제 강화 논의는 배터리/전자부품 보관 및 운송 관련 창고 운영에 잠재적 비용 증가나 운영 방식 변경을 초래할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G961" s="3" t="inlineStr">
+        <is>
+          <t>국내외 물류센터 화재 안전 규제 동향을 지속 모니터링하고, 우리 물류센터의 안전 관리 현황을 점검하여 선제적 대응 방안을 마련해야 함.</t>
+        </is>
+      </c>
+      <c r="H961" s="3" t="inlineStr">
+        <is>
+          <t>중앙일보</t>
+        </is>
+      </c>
+      <c r="I961" s="3" t="inlineStr">
+        <is>
+          <t>https://www.joongang.co.kr/article/25446743</t>
+        </is>
+      </c>
+      <c r="J961" s="3" t="inlineStr"/>
+    </row>
+    <row r="962">
+      <c r="A962" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B962" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C962" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D962" s="3" t="inlineStr">
+        <is>
+          <t>FT "중국, AI·반도체 기술 수출통제 강화 검토" | 연합뉴스</t>
+        </is>
+      </c>
+      <c r="E962" s="3" t="inlineStr">
+        <is>
+          <t>중국이 AI 및 반도체 기술에 대한 수출통제를 강화하는 방안을 검토 중이며, 과거 리튬이온 배터리 제조 기술도 수출 금지·제한 목록에 추가된 바 있어 관련 기술 수출에 대한 불확실성이 커지고 있다.</t>
+        </is>
+      </c>
+      <c r="F962" s="3" t="inlineStr">
+        <is>
+          <t>중국의 기술 수출통제 강화는 배터리 제조 관련 핵심 기술 및 장비 도입에 영향을 미칠 수 있으며, 장기적으로는 생산 및 연구개발 전략에 변수로 작용할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G962" s="3" t="inlineStr">
+        <is>
+          <t>중국의 수출통제 대상 기술 목록 개정 동향을 면밀히 주시하고, 관련 기술 및 장비의 대체 공급처 확보 가능성을 검토해야 함.</t>
+        </is>
+      </c>
+      <c r="H962" s="3" t="inlineStr">
+        <is>
+          <t>연합뉴스</t>
+        </is>
+      </c>
+      <c r="I962" s="3" t="inlineStr">
+        <is>
+          <t>https://yna.co.kr/view/AKR20260721130100009</t>
+        </is>
+      </c>
+      <c r="J962" s="3" t="inlineStr"/>
+    </row>
+    <row r="963">
+      <c r="A963" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B963" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C963" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D963" s="3" t="inlineStr">
+        <is>
+          <t>영풍, ESG 정공법으로 글로벌 공급망 장벽 정면 돌파 &lt; 산업일반 &lt; 경제 &lt; 기사본문 - 굿모닝경제</t>
+        </is>
+      </c>
+      <c r="E963" s="3" t="inlineStr">
+        <is>
+          <t>유럽연합(EU)의 공급망 실사 의무화 등 글로벌 무역 규제가 친환경 및 공급망 실사 확대로 이동하면서 비철금속 제련 업계의 생존 패러다임이 재편되고 있다.</t>
+        </is>
+      </c>
+      <c r="F963" s="3" t="inlineStr">
+        <is>
+          <t>EU의 공급망 실사 의무화는 우리 회사의 원자재 조달 및 생산 과정 전반에 대한 투명성 요구를 높여, 공급망 관리 시스템 개선 및 추가 비용 발생 가능성이 있다.</t>
+        </is>
+      </c>
+      <c r="G963" s="3" t="inlineStr">
+        <is>
+          <t>EU 공급망 실사 규제 내용을 상세히 파악하고, 우리 공급망 내 ESG 리스크를 평가하여 선제적인 대응 방안(예: 공급망 실사 시스템 구축, 협력사 ESG 평가 강화)을 준비해야 함.</t>
+        </is>
+      </c>
+      <c r="H963" s="3" t="inlineStr">
+        <is>
+          <t>굿모닝경제</t>
+        </is>
+      </c>
+      <c r="I963" s="3" t="inlineStr">
+        <is>
+          <t>https://www.goodkyung.com/news/articleView.html?idxno=289363</t>
+        </is>
+      </c>
+      <c r="J963" s="3" t="inlineStr"/>
+    </row>
+    <row r="964">
+      <c r="A964" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B964" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C964" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D964" s="3" t="inlineStr">
+        <is>
+          <t>[사설]국제유가 90달러 돌파, 선제적 물가대응 나서야</t>
+        </is>
+      </c>
+      <c r="E964" s="3" t="inlineStr">
+        <is>
+          <t>미국과 이란의 군사적 충돌 재개로 국제유가(브렌트유)가 배럴당 90달러를 돌파하며 급등했다.</t>
+        </is>
+      </c>
+      <c r="F964" s="3" t="inlineStr">
+        <is>
+          <t>국제유가 급등은 해상/항공/육상 운송의 유류할증료 인상으로 이어져 물류비용 증가에 직접적인 영향을 미치므로 추이를 면밀히 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G964" s="3" t="inlineStr">
+        <is>
+          <t>물류비용 변동 추이 분석 및 운송사와의 유류할증료 협상 준비</t>
+        </is>
+      </c>
+      <c r="H964" s="3" t="inlineStr">
+        <is>
+          <t>경향신문</t>
+        </is>
+      </c>
+      <c r="I964" s="3" t="inlineStr">
+        <is>
+          <t>https://www.khan.co.kr/article/202607201810001/</t>
+        </is>
+      </c>
+      <c r="J964" s="3" t="inlineStr"/>
+    </row>
+    <row r="965">
+      <c r="A965" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B965" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C965" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D965" s="4" t="inlineStr">
+        <is>
+          <t>페덱스, ‘페덱스 라이프 사이언스’ 출범</t>
+        </is>
+      </c>
+      <c r="E965" s="4" t="inlineStr">
+        <is>
+          <t>페덱스가 의약품, 의료기기 등 헬스케어 화물 운송을 전문적으로 지원하는 '페덱스 라이프 사이언스' 조직을 출범하여 글로벌 네트워크와 첨단 모니터링 역량을 결합한다.</t>
+        </is>
+      </c>
+      <c r="F965" s="4" t="inlineStr">
+        <is>
+          <t>우리 회사는 배터리/전자부품 제조기업으로, 헬스케어 물류 전문 서비스 출범은 직접적인 영향이 적다.</t>
+        </is>
+      </c>
+      <c r="G965" s="4" t="inlineStr"/>
+      <c r="H965" s="4" t="inlineStr">
+        <is>
+          <t>cargonews</t>
+        </is>
+      </c>
+      <c r="I965" s="4" t="inlineStr">
+        <is>
+          <t>https://www.cargonews.co.kr/news/articleView.html?idxno=60565</t>
+        </is>
+      </c>
+      <c r="J965" s="4" t="inlineStr"/>
+    </row>
+    <row r="966">
+      <c r="A966" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B966" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C966" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D966" s="4" t="inlineStr">
+        <is>
+          <t>IATA Releases 2025 World Air Transport Statistics</t>
+        </is>
+      </c>
+      <c r="E966" s="4" t="inlineStr">
+        <is>
+          <t>IATA가 2025년까지의 포괄적인 통계 데이터를 담은 최신 세계 항공 운송 통계(WATS) 보고서를 발표했다.</t>
+        </is>
+      </c>
+      <c r="F966" s="4" t="inlineStr">
+        <is>
+          <t>항공 운송 시장의 전반적인 동향을 파악하는 데 참고할 수 있는 자료이나, 당사의 물류 운영에 직접적인 영향을 미치지 않는다.</t>
+        </is>
+      </c>
+      <c r="G966" s="4" t="inlineStr"/>
+      <c r="H966" s="4" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I966" s="4" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/07-16-iata-releases-2025-world-air-transport-statistics-report/</t>
+        </is>
+      </c>
+      <c r="J966" s="4" t="inlineStr"/>
+    </row>
+    <row r="967">
+      <c r="A967" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B967" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C967" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D967" s="4" t="inlineStr">
+        <is>
+          <t>SCIA 2026참관기 - 모로코 자동차산업, 하청기지 넘어 ‘전기차·배터리·스마트 제조’ 허브로 도약</t>
+        </is>
+      </c>
+      <c r="E967" s="4" t="inlineStr">
+        <is>
+          <t>모로코 자동차 산업이 전기차, 배터리, 스마트 제조 허브로 전환을 추진하며, 한국 기업에게 자동차 부품, 배터리 소재·장비, 자동화 설비 등 분야에서 진출 기회를 제공하고 있다.</t>
+        </is>
+      </c>
+      <c r="F967" s="4" t="inlineStr">
+        <is>
+          <t>모로코의 산업 전환은 장기적인 공급망 다변화 관점에서 참고할 수 있으나, 당장 우리 회사의 물류 운영에 직접적인 영향을 미치지 않는다.</t>
+        </is>
+      </c>
+      <c r="G967" s="4" t="inlineStr"/>
+      <c r="H967" s="4" t="inlineStr">
+        <is>
+          <t>kotra</t>
+        </is>
+      </c>
+      <c r="I967" s="4" t="inlineStr">
+        <is>
+          <t>https://dream.kotra.or.kr/kotranews/cms/news/actionKotraBoardDetail.do?SITE_NO=3&amp;MENU_ID=70&amp;CONTENTS_NO=1&amp;pNttSn=242652</t>
+        </is>
+      </c>
+      <c r="J967" s="4" t="inlineStr"/>
+    </row>
+    <row r="968">
+      <c r="A968" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B968" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C968" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D968" s="4" t="inlineStr">
+        <is>
+          <t>브라질 발레, 3중연료 초대형선 30척 도입…HMM·폴라리스쉬핑 신조</t>
+        </is>
+      </c>
+      <c r="E968" s="4" t="inlineStr">
+        <is>
+          <t>브라질 광산 대기업 발레가 HMM, 폴라리스쉬핑 등과 협력하여 3중 연료를 사용하는 21만t급 친환경 신조 벌크선 20척을 25년간 장기 임차하는 계약을 추진 중이다.</t>
+        </is>
+      </c>
+      <c r="F968" s="4" t="inlineStr">
+        <is>
+          <t>벌크선 신조는 장기적인 해상 운송 시장의 친환경 전환 및 용량 변화를 시사하지만, 우리 회사의 컨테이너 기반 물류 운영에 직접적인 영향은 미미하다.</t>
+        </is>
+      </c>
+      <c r="G968" s="4" t="inlineStr"/>
+      <c r="H968" s="4" t="inlineStr">
+        <is>
+          <t>ksg</t>
+        </is>
+      </c>
+      <c r="I968" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksg.co.kr/news/main_newsView.jsp?pNum=147628</t>
+        </is>
+      </c>
+      <c r="J968" s="4" t="inlineStr"/>
+    </row>
+    <row r="969">
+      <c r="A969" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B969" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C969" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D969" s="4" t="inlineStr">
+        <is>
+          <t>케이조선, 풍력보조추진 MR 탱커 개발 본격화</t>
+        </is>
+      </c>
+      <c r="E969" s="4" t="inlineStr">
+        <is>
+          <t>케이조선이 그리스 선주사 및 로이드선급과 협력하여 풍력보조추진 기술을 적용한 차세대 MR 탱커 개발에 착수했으며, 이는 5만 DWT급 MR 탱커에 대한 상업적 적용 가능성을 검증하는 프로젝트이다.</t>
+        </is>
+      </c>
+      <c r="F969" s="4" t="inlineStr">
+        <is>
+          <t>풍력보조추진 기술 개발은 해운 산업의 친환경 전환 노력의 일환이나, MR 탱커에 대한 기술 개발이 우리 회사의 배터리/전자부품 물류 운영에 직접적인 영향을 미치지는 않는다.</t>
+        </is>
+      </c>
+      <c r="G969" s="4" t="inlineStr"/>
+      <c r="H969" s="4" t="inlineStr">
+        <is>
+          <t>oceanpress</t>
+        </is>
+      </c>
+      <c r="I969" s="4" t="inlineStr">
+        <is>
+          <t>https://www.oceanpress.co.kr/news/article.html?no=30687</t>
+        </is>
+      </c>
+      <c r="J969" s="4" t="inlineStr"/>
+    </row>
+    <row r="970">
+      <c r="A970" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B970" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C970" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D970" s="4" t="inlineStr">
+        <is>
+          <t>Global Schedule Reliability for May 2026 the Highest of the Year</t>
+        </is>
+      </c>
+      <c r="E970" s="4" t="inlineStr">
+        <is>
+          <t>2026년 5월 글로벌 선박 스케줄 정시성이 연중 최고치를 기록하며 해운 서비스의 안정성이 개선되고 있음을 보여줍니다.</t>
+        </is>
+      </c>
+      <c r="F970" s="4" t="inlineStr">
+        <is>
+          <t>스케줄 정시성 개선은 긍정적인 신호이나, 일시적인 개선일 수 있으며, 우리 물류 운영에 즉각적인 큰 영향보다는 장기적인 안정화 추세로 판단됩니다.</t>
+        </is>
+      </c>
+      <c r="G970" s="4" t="n"/>
+      <c r="H970" s="4" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I970" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/395-global-schedule-reliability-for-may-2026-the-highest-of-the-year</t>
+        </is>
+      </c>
+      <c r="J970" s="4" t="inlineStr"/>
+    </row>
+    <row r="971">
+      <c r="A971" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B971" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C971" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D971" s="4" t="inlineStr">
+        <is>
+          <t>유통업계, 해외 팝업·역직구 결합 수출 플랫폼 사업 확대</t>
+        </is>
+      </c>
+      <c r="E971" s="4" t="inlineStr">
+        <is>
+          <t>유통업계가 해외 팝업과 역직구를 결합하여 통관 및 물류 지원까지 제공하는 K-패션 등 수출 플랫폼 사업을 확대하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F971" s="4" t="inlineStr">
+        <is>
+          <t>이는 주로 소비재 유통업계의 수출 전략으로, 배터리/전자부품 제조기업의 B2B 물류 운영에 직접적인 영향은 낮으나, 향후 B2C 또는 소량 다품종 수출 시 참고할 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G971" s="4" t="n"/>
+      <c r="H971" s="4" t="inlineStr">
+        <is>
+          <t>Surff (데일리스크랩)</t>
+        </is>
+      </c>
+      <c r="I971" s="4" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260722-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J971" s="4" t="inlineStr"/>
+    </row>
+    <row r="972">
+      <c r="A972" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B972" s="4" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C972" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D972" s="4" t="inlineStr">
+        <is>
+          <t>러시아, 우크라 오데사 항구 화물선에 미사일 공격</t>
+        </is>
+      </c>
+      <c r="E972" s="4" t="inlineStr">
+        <is>
+          <t>러시아가 우크라이나 오데사 항구의 화물선에 미사일 공격을 가해 10명이 사망하는 사건이 발생했습니다.</t>
+        </is>
+      </c>
+      <c r="F972" s="4" t="inlineStr">
+        <is>
+          <t>오데사 항구는 우리 회사의 주요 운송 경로가 아니며, 해당 지역의 지정학적 리스크는 이미 인지된 상황으로, 직접적인 물류 운영 영향은 낮습니다.</t>
+        </is>
+      </c>
+      <c r="G972" s="4" t="n"/>
+      <c r="H972" s="4" t="inlineStr">
+        <is>
+          <t>Surff (데일리스크랩)</t>
+        </is>
+      </c>
+      <c r="I972" s="4" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260721-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J972" s="4" t="inlineStr"/>
+    </row>
+    <row r="973">
+      <c r="A973" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B973" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C973" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D973" s="4" t="inlineStr">
+        <is>
+          <t>중동 불안으로 운송거리 증가, 중국 조선업 선박 주문 싹쓸이</t>
+        </is>
+      </c>
+      <c r="E973" s="4" t="inlineStr">
+        <is>
+          <t>중동 지정학적 불안으로 운송 거리가 늘어나면서 선복 수요가 증가하고 있으며, 이에 따라 중국 조선업이 전 세계 선박 주문을 싹쓸이하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F973" s="4" t="inlineStr">
+        <is>
+          <t>이는 장기적인 선복 공급 증가로 이어질 수 있으나, 단기적인 우리 물류 운영에 직접적인 영향은 낮으며, 선박 건조는 수년이 소요되므로 참고 수준입니다.</t>
+        </is>
+      </c>
+      <c r="G973" s="4" t="n"/>
+      <c r="H973" s="4" t="inlineStr">
+        <is>
+          <t>Surff (데일리스크랩)</t>
+        </is>
+      </c>
+      <c r="I973" s="4" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260720-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J973" s="4" t="inlineStr"/>
+    </row>
+    <row r="974">
+      <c r="A974" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B974" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C974" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D974" s="4" t="inlineStr">
+        <is>
+          <t>Comment: Supply chain disruption on land, sea, and in the air is the new norm – how agentic AI with data movement in real time is helping businesses tackle this global reality head on | The AI Journal</t>
+        </is>
+      </c>
+      <c r="E974" s="4" t="inlineStr">
+        <is>
+          <t>육상, 해상, 항공을 아우르는 공급망 혼란이 뉴노멀이 되었으며, 실시간 데이터 이동을 활용하는 AI가 기업들이 이러한 글로벌 현실에 대처하는 데 도움을 주고 있다는 분석이다.</t>
+        </is>
+      </c>
+      <c r="F974" s="4" t="inlineStr">
+        <is>
+          <t>공급망 혼란이 일반화되고 AI 솔루션이 부상한다는 일반적인 분석으로, 당장 우리 회사의 물류 운영에 직접적인 영향을 미치기보다는 장기적인 관점의 참고 자료이다.</t>
+        </is>
+      </c>
+      <c r="G974" s="4" t="n"/>
+      <c r="H974" s="4" t="inlineStr">
+        <is>
+          <t>The AI Journal</t>
+        </is>
+      </c>
+      <c r="I974" s="4" t="inlineStr">
+        <is>
+          <t>https://aijourn.com/comment-supply-chain-disruption-on-land-sea-and-in-the-air-is-the-new-norm-how-agentic-ai-with-data-movement-in-real-time-is-helping-businesses-tackle-this-global-reality-head-on/</t>
+        </is>
+      </c>
+      <c r="J974" s="4" t="inlineStr"/>
+    </row>
+    <row r="975">
+      <c r="A975" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B975" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C975" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D975" s="4" t="inlineStr">
+        <is>
+          <t>Hyperlocal Supply Chains Are Emerging As Hospitality’s Next Big Asset</t>
+        </is>
+      </c>
+      <c r="E975" s="4" t="inlineStr">
+        <is>
+          <t>기후 변화 등으로 인해 효율성 위주였던 호텔 산업의 공급망이 회복탄력성을 위해 하이퍼로컬 공급망으로 전환되고 있다는 내용이다.</t>
+        </is>
+      </c>
+      <c r="F975" s="4" t="inlineStr">
+        <is>
+          <t>호텔 산업의 특정 공급망 변화에 대한 내용으로, 배터리/전자부품 제조기업의 물류 운영에 직접적인 관련성은 낮다.</t>
+        </is>
+      </c>
+      <c r="G975" s="4" t="n"/>
+      <c r="H975" s="4" t="inlineStr">
+        <is>
+          <t>Forbes</t>
+        </is>
+      </c>
+      <c r="I975" s="4" t="inlineStr">
+        <is>
+          <t>https://forbes.com/sites/indrabatilahiri/2026/07/19/hyperlocal-supply-chains-are-emerging-as-hospitalitys-next-big-asset</t>
+        </is>
+      </c>
+      <c r="J975" s="4" t="inlineStr"/>
+    </row>
+    <row r="976">
+      <c r="A976" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B976" s="4" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C976" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D976" s="4" t="inlineStr">
+        <is>
+          <t>울산소방본부, 에쓰오일·샤힌프로젝트 현장 점검 &lt; 사회일반 &lt; 사회 &lt; 뉴스 &lt; 기사본문 - 울산매일 - 울산최초, 최고의 조간신문</t>
+        </is>
+      </c>
+      <c r="E976" s="4" t="inlineStr">
+        <is>
+          <t>울산소방본부가 에쓰오일 울산공장 및 샤힌 프로젝트 공사현장을 방문하여 위험물 중점관리대상에 대한 화재예방 지도점검을 실시했다.</t>
+        </is>
+      </c>
+      <c r="F976" s="4" t="inlineStr">
+        <is>
+          <t>특정 지역의 특정 산업(정유/화학) 시설에 대한 정기적인 위험물 안전 점검 소식으로, 우리 회사의 물류 운영에 직접적인 영향은 낮다.</t>
+        </is>
+      </c>
+      <c r="G976" s="4" t="n"/>
+      <c r="H976" s="4" t="inlineStr">
+        <is>
+          <t>울산매일</t>
+        </is>
+      </c>
+      <c r="I976" s="4" t="inlineStr">
+        <is>
+          <t>https://www.iusm.co.kr/news/articleView.html?idxno=1065629</t>
+        </is>
+      </c>
+      <c r="J976" s="4" t="inlineStr"/>
+    </row>
+    <row r="977">
+      <c r="A977" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B977" s="4" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C977" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D977" s="4" t="inlineStr">
+        <is>
+          <t>中 자동차 부품기업 태국 인니 동남아 공장 진출 가속</t>
+        </is>
+      </c>
+      <c r="E977" s="4" t="inlineStr">
+        <is>
+          <t>중국 자동차 부품 기업들이 글로벌 시장 경쟁력 강화와 공급망 다변화를 위해 태국, 인도네시아 등 동남아시아 시장 진출을 가속화하고 있다.</t>
+        </is>
+      </c>
+      <c r="F977" s="4" t="inlineStr">
+        <is>
+          <t>중국 기업의 동남아 진출은 해당 지역의 물류 인프라 및 노동 시장에 영향을 줄 수 있으나, 당사 배터리/전자부품 공급망에 직접적인 영향은 아직 미미하다.</t>
+        </is>
+      </c>
+      <c r="G977" s="4" t="inlineStr">
+        <is>
+          <t>동남아시아 지역의 물류 인프라 변화 및 경쟁 환경 동향을 참고 수준으로 모니터링.</t>
+        </is>
+      </c>
+      <c r="H977" s="4" t="inlineStr">
+        <is>
+          <t>뉴스핌</t>
+        </is>
+      </c>
+      <c r="I977" s="4" t="inlineStr">
+        <is>
+          <t>https://www.newspim.com/news/view/20260720000762</t>
+        </is>
+      </c>
+      <c r="J977" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -44926,7 +46726,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -45862,6 +47662,49 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>3080.31</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>-105 (-3.3%)</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>+1,317 (+74.7%)</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="n">
+        <v>4204</v>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>-114 (-2.6%)</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="inlineStr">
+        <is>
+          <t>+1,755 (+71.7%)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -45874,7 +47717,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I176"/>
+  <dimension ref="A1:I182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -52060,6 +53903,216 @@
       </c>
       <c r="I176" s="6" t="inlineStr"/>
     </row>
+    <row r="177">
+      <c r="A177" s="6" t="inlineStr">
+        <is>
+          <t>RSK-176</t>
+        </is>
+      </c>
+      <c r="B177" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C177" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D177" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E177" s="6" t="inlineStr">
+        <is>
+          <t>Section 301 Tariffs on Brazil Take Effect July 22, Stacking with Section 122 Duties; Strait of Hormuz Closure Restricts 200K TEU of Ocean Capacity</t>
+        </is>
+      </c>
+      <c r="F177" s="6" t="inlineStr"/>
+      <c r="G177" s="6" t="inlineStr"/>
+      <c r="H177" s="6" t="inlineStr">
+        <is>
+          <t>중동 항로 이용 여부 및 대체 경로 검토, 브라질 및 러시아 관련 무역 거래에 대한 관세 영향 분석 및 대응 방안 마련.</t>
+        </is>
+      </c>
+      <c r="I177" s="6" t="inlineStr"/>
+    </row>
+    <row r="178">
+      <c r="A178" s="6" t="inlineStr">
+        <is>
+          <t>RSK-177</t>
+        </is>
+      </c>
+      <c r="B178" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C178" s="6" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="D178" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E178" s="6" t="inlineStr">
+        <is>
+          <t>홍해 봉쇄 위기 고조, 아시아-유럽 항로 희망봉 우회 가능성</t>
+        </is>
+      </c>
+      <c r="F178" s="6" t="inlineStr"/>
+      <c r="G178" s="6" t="inlineStr"/>
+      <c r="H178" s="6" t="inlineStr">
+        <is>
+          <t>아시아-유럽 노선 운송 계획 재검토, 대체 운송 경로 및 운송 수단(항공 등) 비상 계획 수립, 선사와의 긴밀한 소통을 통한 상황 변화 주시.</t>
+        </is>
+      </c>
+      <c r="I178" s="6" t="inlineStr"/>
+    </row>
+    <row r="179">
+      <c r="A179" s="6" t="inlineStr">
+        <is>
+          <t>RSK-178</t>
+        </is>
+      </c>
+      <c r="B179" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C179" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D179" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E179" s="6" t="inlineStr">
+        <is>
+          <t>홍해 봉쇄 위기, 중동 원유 수송 차질로 유가 120달러 재돌파 우려</t>
+        </is>
+      </c>
+      <c r="F179" s="6" t="inlineStr"/>
+      <c r="G179" s="6" t="inlineStr"/>
+      <c r="H179" s="6" t="inlineStr">
+        <is>
+          <t>유가 변동 추이 및 물류비에 미치는 영향 분석, 운송 계약 시 유류할증료 조건 재검토, 에너지 효율적인 운송 방안 모색.</t>
+        </is>
+      </c>
+      <c r="I179" s="6" t="inlineStr"/>
+    </row>
+    <row r="180">
+      <c r="A180" s="6" t="inlineStr">
+        <is>
+          <t>RSK-179</t>
+        </is>
+      </c>
+      <c r="B180" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C180" s="6" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="D180" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E180" s="6" t="inlineStr">
+        <is>
+          <t>쿠팡 4·5층 모두 '화약고'였다… "리튬배터리 로봇 수백 대·포장비닐 빼곡"-사회ㅣ한국일보</t>
+        </is>
+      </c>
+      <c r="F180" s="6" t="inlineStr"/>
+      <c r="G180" s="6" t="inlineStr"/>
+      <c r="H180" s="6" t="inlineStr">
+        <is>
+          <t>현재 물류센터 내 리튬 배터리 보관 현황 및 안전 관리 절차를 점검하고, 협력 물류센터의 화재 안전 시스템 및 위험물 취급 규정 준수 여부를 확인한다. 관련 규제 동향을 모니터링하고 선제적 대응 방안 및 비상 계획을 마련한다.</t>
+        </is>
+      </c>
+      <c r="I180" s="6" t="inlineStr"/>
+    </row>
+    <row r="181">
+      <c r="A181" s="6" t="inlineStr">
+        <is>
+          <t>RSK-180</t>
+        </is>
+      </c>
+      <c r="B181" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C181" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D181" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E181" s="6" t="inlineStr">
+        <is>
+          <t>철강은 “산 넘어 산”…배터리는 소재비 긴장 [관세 리셋, 美 301조의 경고] - 이투데이</t>
+        </is>
+      </c>
+      <c r="F181" s="6" t="inlineStr"/>
+      <c r="G181" s="6" t="inlineStr"/>
+      <c r="H181" s="6" t="inlineStr">
+        <is>
+          <t>미국향 수출 제품 및 소재의 원산지 규정 준수 여부를 재검토하고, 관세 부과 시나리오별 원가 영향 분석 및 공급망 다변화 전략을 수립해야 함.</t>
+        </is>
+      </c>
+      <c r="I181" s="6" t="inlineStr"/>
+    </row>
+    <row r="182">
+      <c r="A182" s="6" t="inlineStr">
+        <is>
+          <t>RSK-181</t>
+        </is>
+      </c>
+      <c r="B182" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C182" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D182" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E182" s="6" t="inlineStr">
+        <is>
+          <t>중동 긴장 재고조…항공·해운 비용 부담에 '초긴장' - 매일일보</t>
+        </is>
+      </c>
+      <c r="F182" s="6" t="inlineStr"/>
+      <c r="G182" s="6" t="inlineStr"/>
+      <c r="H182" s="6" t="inlineStr">
+        <is>
+          <t>중동 정세 및 국제 유가 동향을 면밀히 주시하고, 물류비 상승에 대비하여 운송 계약 조건 재검토, 운송 모드 전환 검토, 재고 수준 조정 등 비상 계획을 수립해야 함.</t>
+        </is>
+      </c>
+      <c r="I182" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
📰 뉴스 데이터 2026-07-23_09:07
</commit_message>
<xml_diff>
--- a/data/SCM_물류_브리핑.xlsx
+++ b/data/SCM_물류_브리핑.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J977"/>
+  <dimension ref="A1:J1007"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -46714,6 +46714,1410 @@
       </c>
       <c r="J977" s="4" t="inlineStr"/>
     </row>
+    <row r="978">
+      <c r="A978" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B978" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C978" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D978" s="2" t="inlineStr">
+        <is>
+          <t>미·이란 충돌 격화에 홍해 봉쇄 위협까지…국제유가 2%↑</t>
+        </is>
+      </c>
+      <c r="E978" s="2" t="inlineStr">
+        <is>
+          <t>미국-이란 충돌 격화와 홍해 봉쇄 위협, 카스피해 송유관 피격 등 중동발 지정학적 리스크가 고조되면서 국제유가가 2% 이상 상승했다.</t>
+        </is>
+      </c>
+      <c r="F978" s="2" t="inlineStr">
+        <is>
+          <t>중동 지정학적 리스크는 홍해 항로의 불안정성을 높여 해상 운송 지연 및 운임 상승을 유발하고, 국제유가 상승은 해상/항공 운송 비용 전반에 직접적인 영향을 미치므로 즉각적인 대응이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G978" s="2" t="inlineStr">
+        <is>
+          <t>홍해 항로 이용 현황 점검 및 대체 항로(희망봉 우회 등) 검토, 운송사와의 비상 계획 수립, 유가 변동에 따른 물류비 예산 재검토.</t>
+        </is>
+      </c>
+      <c r="H978" s="2" t="inlineStr">
+        <is>
+          <t>kita</t>
+        </is>
+      </c>
+      <c r="I978" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kita.net/shippers/board/newsView.do?morgueCode=2&amp;dataCls=A&amp;dataSeq=2537</t>
+        </is>
+      </c>
+      <c r="J978" s="2" t="inlineStr">
+        <is>
+          <t>RSK-182</t>
+        </is>
+      </c>
+    </row>
+    <row r="979">
+      <c r="A979" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B979" s="2" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C979" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D979" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 이어 홍해 봉쇄 위기... 다시 희망봉 돌아야 하나</t>
+        </is>
+      </c>
+      <c r="E979" s="2" t="inlineStr">
+        <is>
+          <t>예멘 후티 반군의 홍해 봉쇄 위협이 커지면서 아시아-유럽 항로가 희망봉 우회로 전환될 가능성이 있으며, 이는 운송기간과 연료비 증가, 선복 부족 및 운임 상승을 재현시킬 수 있다. 또한 사우디 봉쇄 현실화 시 세계 원유 공급의 25%가 타격받을 수 있다는 전망도 나왔다.</t>
+        </is>
+      </c>
+      <c r="F979" s="2" t="inlineStr">
+        <is>
+          <t>주요 해상 운송로인 홍해 및 호르무즈 해협의 봉쇄 위협은 아시아-유럽 항로의 장기 우회, 운송 기간 및 비용 급증, 선복 부족 심화로 이어져 우리 물류 운영 및 생산 계획에 즉각적이고 직접적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G979" s="2" t="inlineStr">
+        <is>
+          <t>대체 항로 및 운송 수단 검토, 비상 재고 확보, 운임 변동성 분석 및 계약 조건 재검토, 공급망 리스크 평가 및 대응 계획 수립</t>
+        </is>
+      </c>
+      <c r="H979" s="2" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I979" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260720-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J979" s="2" t="inlineStr">
+        <is>
+          <t>RSK-183</t>
+        </is>
+      </c>
+    </row>
+    <row r="980">
+      <c r="A980" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B980" s="2" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C980" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D980" s="2" t="inlineStr">
+        <is>
+          <t>[단독] ‘덕평 악몽’ 5년 만에 또…쿠팡, 全물류센터 안전시스템 전면 재정비[물류센터의 경고] - 이투데이</t>
+        </is>
+      </c>
+      <c r="E980" s="2" t="inlineStr">
+        <is>
+          <t>쿠팡 인천 물류센터 화재 이후, 쿠팡이 모든 물류센터의 안전 시스템을 전면 재정비하고 가드포스트 강화, 출입 통제 재정비, 소방당국 협력 체계 구축 등 재난 대응 훈련을 정례화할 계획이다.</t>
+        </is>
+      </c>
+      <c r="F980" s="2" t="inlineStr">
+        <is>
+          <t>대형 물류센터 화재는 위험물(배터리 등) 보관 및 취급 규제 강화로 이어질 수 있으며, 우리 회사의 물류센터 안전 관리 및 비상 대응 계획에 즉각적인 점검이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G980" s="2" t="inlineStr">
+        <is>
+          <t>우리 회사의 물류센터 안전 점검 및 위험물 보관 규정 준수 여부 확인, 비상 대응 훈련 강화, 물류 파트너사의 안전 관리 현황 확인.</t>
+        </is>
+      </c>
+      <c r="H980" s="2" t="inlineStr">
+        <is>
+          <t>이투데이</t>
+        </is>
+      </c>
+      <c r="I980" s="2" t="inlineStr">
+        <is>
+          <t>https://etoday.co.kr/news/view/2606169</t>
+        </is>
+      </c>
+      <c r="J980" s="2" t="inlineStr">
+        <is>
+          <t>RSK-184</t>
+        </is>
+      </c>
+    </row>
+    <row r="981">
+      <c r="A981" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B981" s="2" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C981" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D981" s="2" t="inlineStr">
+        <is>
+          <t>[데일리연합 (SNSJTV)] 리튬 배터리 수백대와 충격적인 붕괴 위험</t>
+        </is>
+      </c>
+      <c r="E981" s="2" t="inlineStr">
+        <is>
+          <t>리튬 배터리 수백 대와 관련된 충격적인 붕괴 위험을 경고하는 내용으로, 리튬 배터리 보관 및 취급의 안전 문제에 대한 주의를 요한다.</t>
+        </is>
+      </c>
+      <c r="F981" s="2" t="inlineStr">
+        <is>
+          <t>리튬 배터리 보관 및 취급과 관련된 붕괴 위험 경고는 우리 회사의 핵심 제품과 직결되는 안전 문제로, 즉각적인 주의와 점검이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G981" s="2" t="inlineStr">
+        <is>
+          <t>리튬 배터리 보관 시설의 안전성 재점검, 취급 절차 준수 여부 확인, 관련 안전 교육 강화.</t>
+        </is>
+      </c>
+      <c r="H981" s="2" t="inlineStr">
+        <is>
+          <t>데일리연합 (SNSJTV)</t>
+        </is>
+      </c>
+      <c r="I981" s="2" t="inlineStr">
+        <is>
+          <t>https://dailyan.com/news/article.html?no=773791</t>
+        </is>
+      </c>
+      <c r="J981" s="2" t="inlineStr">
+        <is>
+          <t>RSK-185</t>
+        </is>
+      </c>
+    </row>
+    <row r="982">
+      <c r="A982" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B982" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C982" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D982" s="3" t="inlineStr">
+        <is>
+          <t>U.S.-EU Trade Agreement Eliminates Duties on Most U.S. Goods Starting July 1; TPEB Rates Rise as July Capacity Hits Three-Year High</t>
+        </is>
+      </c>
+      <c r="E982" s="3" t="inlineStr">
+        <is>
+          <t>미국-EU 무역 협정으로 7월 1일부터 대부분의 미국 상품에 대한 관세가 철폐되며, 동시에 태평양 횡단 동향(TPEB) 운임이 상승하고 7월 선복량이 3년 내 최고치를 기록했다.</t>
+        </is>
+      </c>
+      <c r="F982" s="3" t="inlineStr">
+        <is>
+          <t>미국-EU 간 관세 철폐는 해당 지역으로의 수출입 비용에 직접적인 영향을 미칠 수 있으며, TPEB 운임 상승은 아시아발 미주/유럽 운송 비용 증가로 이어질 수 있어 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G982" s="3" t="inlineStr">
+        <is>
+          <t>미국-EU 간 수출입 품목 및 물량 확인, 관세 철폐 적용 여부 및 비용 절감 효과 분석. TPEB 운임 추이 및 선복량 변동 모니터링.</t>
+        </is>
+      </c>
+      <c r="H982" s="3" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I982" s="3" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/july-02-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J982" s="3" t="inlineStr"/>
+    </row>
+    <row r="983">
+      <c r="A983" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B983" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C983" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D983" s="3" t="inlineStr">
+        <is>
+          <t>Statement on EU Commission Revision of the EU Emissions Trading System</t>
+        </is>
+      </c>
+      <c r="E983" s="3" t="inlineStr">
+        <is>
+          <t>IATA는 EU 배출권 거래 시스템(ETS)의 유럽 외 확장 제안에 대해 깊은 우려를 표명하며, 이는 항공 운송 비용 증가로 이어질 수 있다고 밝혔다.</t>
+        </is>
+      </c>
+      <c r="F983" s="3" t="inlineStr">
+        <is>
+          <t>EU ETS의 확장 적용은 항공 운송 비용을 증가시키고 항공사들의 운항 전략에 영향을 미쳐, 우리 제품의 유럽향 항공 운송 비용 상승으로 이어질 수 있으므로 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G983" s="3" t="inlineStr">
+        <is>
+          <t>EU ETS 확장 논의 진행 상황 및 항공 운임에 미칠 잠재적 영향 지속 모니터링.</t>
+        </is>
+      </c>
+      <c r="H983" s="3" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I983" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/07-17-statement-eu-commission-revision-emissions-trading-system/</t>
+        </is>
+      </c>
+      <c r="J983" s="3" t="inlineStr"/>
+    </row>
+    <row r="984">
+      <c r="A984" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B984" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C984" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D984" s="3" t="inlineStr">
+        <is>
+          <t>Air Cargo Demand Up 6.0% in May</t>
+        </is>
+      </c>
+      <c r="E984" s="3" t="inlineStr">
+        <is>
+          <t>2026년 5월 전 세계 항공 화물 수요가 전년 동기 대비 6.0% 증가했으며, 이는 항공 화물 시장의 견조한 성장을 나타낸다.</t>
+        </is>
+      </c>
+      <c r="F984" s="3" t="inlineStr">
+        <is>
+          <t>항공 화물 수요 증가는 향후 항공 운임 상승 압력으로 작용할 수 있으며, 우리 제품의 항공 운송 비용에 영향을 미칠 수 있으므로 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G984" s="3" t="inlineStr">
+        <is>
+          <t>항공 화물 운임 및 선복량 추이 지속 모니터링, 필요시 운송 계획 조정 검토.</t>
+        </is>
+      </c>
+      <c r="H984" s="3" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I984" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/06-29-air-cargo-demand-up-may/</t>
+        </is>
+      </c>
+      <c r="J984" s="3" t="inlineStr"/>
+    </row>
+    <row r="985">
+      <c r="A985" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B985" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C985" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D985" s="3" t="inlineStr">
+        <is>
+          <t>DP월드, 푸자이라 신항 50년 운영권 확보</t>
+        </is>
+      </c>
+      <c r="E985" s="3" t="inlineStr">
+        <is>
+          <t>DP월드가 UAE 푸자이라 신항의 50년 운영권을 확보하며 호르무즈 해협 의존도를 낮추기 위한 전략적 물류망 구축에 나섰다.</t>
+        </is>
+      </c>
+      <c r="F985" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협의 지정학적 긴장 고조에 대응하여 대체 물류망이 구축되는 것은 장기적으로 중동 지역 운송 리스크 완화에 기여할 수 있으므로 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G985" s="3" t="inlineStr">
+        <is>
+          <t>중동 지역 운송 경로 및 리스크 분석 시 푸자이라 신항 개발 동향 참고.</t>
+        </is>
+      </c>
+      <c r="H985" s="3" t="inlineStr">
+        <is>
+          <t>oceanpress</t>
+        </is>
+      </c>
+      <c r="I985" s="3" t="inlineStr">
+        <is>
+          <t>https://www.oceanpress.co.kr/news/article.html?no=30703</t>
+        </is>
+      </c>
+      <c r="J985" s="3" t="inlineStr"/>
+    </row>
+    <row r="986">
+      <c r="A986" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B986" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C986" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D986" s="3" t="inlineStr">
+        <is>
+          <t>Structural Contraction of Global Liner Networks</t>
+        </is>
+      </c>
+      <c r="E986" s="3" t="inlineStr">
+        <is>
+          <t>IMF의 최신 전망에 따르면 2026년 글로벌 무역량 성장률이 둔화될 것으로 예상됨에 따라, 글로벌 정기선 네트워크의 구조적 축소가 진행되고 있다.</t>
+        </is>
+      </c>
+      <c r="F986" s="3" t="inlineStr">
+        <is>
+          <t>글로벌 무역량 둔화와 정기선 네트워크 축소는 해상 운송 선복량 감소 및 서비스 빈도 저하로 이어져, 향후 운송 스케줄 및 비용에 영향을 미칠 수 있으므로 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G986" s="3" t="inlineStr">
+        <is>
+          <t>주요 항로의 선복량 및 서비스 빈도 변화 추이 모니터링, 운송사와의 정보 공유 강화.</t>
+        </is>
+      </c>
+      <c r="H986" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I986" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/398-structural-contraction-of-global-liner-network</t>
+        </is>
+      </c>
+      <c r="J986" s="3" t="inlineStr"/>
+    </row>
+    <row r="987">
+      <c r="A987" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B987" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C987" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D987" s="3" t="inlineStr">
+        <is>
+          <t>PLSCI Data Indicates Mega-Hub Retrenchment</t>
+        </is>
+      </c>
+      <c r="E987" s="3" t="inlineStr">
+        <is>
+          <t>UNCTAD의 2026년 2분기 항만 정기선 연결성 지수(PLSCI) 분석 결과, 최근 네트워크 재조정이 메가 허브 항만의 후퇴를 시사하는 것으로 나타났다.</t>
+        </is>
+      </c>
+      <c r="F987" s="3" t="inlineStr">
+        <is>
+          <t>메가 허브 항만의 연결성 변화는 주요 항만 이용 전략 및 운송 경로 재검토 필요성을 야기할 수 있으므로, 우리 물류 운영에 미칠 영향을 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G987" s="3" t="inlineStr">
+        <is>
+          <t>주요 수출입 항만의 PLSCI 변화 추이 모니터링, 운송 경로 및 허브 전략 재검토 필요성 분석.</t>
+        </is>
+      </c>
+      <c r="H987" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I987" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/396-plsci-data-indicates-mega-hub-retrenchment</t>
+        </is>
+      </c>
+      <c r="J987" s="3" t="inlineStr"/>
+    </row>
+    <row r="988">
+      <c r="A988" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B988" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C988" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D988" s="3" t="inlineStr">
+        <is>
+          <t>Tracking True Vessel Delay</t>
+        </is>
+      </c>
+      <c r="E988" s="3" t="inlineStr">
+        <is>
+          <t>해운사들이 선박 스케줄 버퍼를 늘려 공시된 운송 시간을 연장하고 있으며, 이는 실제 선박 지연과 조기 도착 간의 관계를 분석한 결과이다.</t>
+        </is>
+      </c>
+      <c r="F988" s="3" t="inlineStr">
+        <is>
+          <t>해운사들의 스케줄 버퍼 증가는 공시된 운송 시간 증가로 이어져 우리 물류 계획에 간접적인 영향을 줄 수 있으므로 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G988" s="3" t="n"/>
+      <c r="H988" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I988" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/394-tracking-true-vessel-delay</t>
+        </is>
+      </c>
+      <c r="J988" s="3" t="inlineStr"/>
+    </row>
+    <row r="989">
+      <c r="A989" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B989" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C989" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D989" s="3" t="inlineStr">
+        <is>
+          <t>쿠팡화재, 빽빽한 구조가 진화 발목 잡았다</t>
+        </is>
+      </c>
+      <c r="E989" s="3" t="inlineStr">
+        <is>
+          <t>인천 쿠팡 물류센터에서 대형 화재가 발생하여 진화에 어려움을 겪었으며, 빽빽한 물류센터 구조가 진화를 방해한 것으로 분석되었다.</t>
+        </is>
+      </c>
+      <c r="F989" s="3" t="inlineStr">
+        <is>
+          <t>대형 물류센터 화재는 물류창고 안전 규제 강화 논의로 이어질 수 있으며, 이는 배터리/전자부품과 같은 위험물 취급 시 우리 물류센터 운영 및 보관 비용에 잠재적 영향을 미칠 수 있으므로 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G989" s="3" t="n"/>
+      <c r="H989" s="3" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I989" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260721-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J989" s="3" t="inlineStr"/>
+    </row>
+    <row r="990">
+      <c r="A990" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B990" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C990" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D990" s="3" t="inlineStr">
+        <is>
+          <t>트럼프, 캐나다에 관세 폭탄… 북미 무역협정 균열 조짐</t>
+        </is>
+      </c>
+      <c r="E990" s="3" t="inlineStr">
+        <is>
+          <t>트럼프 전 대통령이 캐나다에 관세 부과를 시사하며 북미 무역협정의 균열 조짐이 보이고 있다.</t>
+        </is>
+      </c>
+      <c r="F990" s="3" t="inlineStr">
+        <is>
+          <t>북미 지역의 무역 분쟁 및 관세 부과는 해당 지역으로의 수출입 물류 비용 증가 및 공급망 재편을 야기할 수 있으므로 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G990" s="3" t="n"/>
+      <c r="H990" s="3" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I990" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260722-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J990" s="3" t="inlineStr"/>
+    </row>
+    <row r="991">
+      <c r="A991" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B991" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C991" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D991" s="3" t="inlineStr">
+        <is>
+          <t>러시아, 우크라 오데사 항구 화물선에 미사일 공격, 10명 사망</t>
+        </is>
+      </c>
+      <c r="E991" s="3" t="inlineStr">
+        <is>
+          <t>러시아가 우크라이나 오데사 항구의 화물선에 미사일 공격을 가해 10명이 사망하는 사건이 발생했다.</t>
+        </is>
+      </c>
+      <c r="F991" s="3" t="inlineStr">
+        <is>
+          <t>전쟁 지역 항구에 대한 공격은 해당 지역의 해상 운송을 불안정하게 만들고, 글로벌 해상 보험료 인상 및 항로 변경 가능성을 높여 간접적인 영향을 미칠 수 있으므로 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G991" s="3" t="n"/>
+      <c r="H991" s="3" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I991" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260721-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J991" s="3" t="inlineStr"/>
+    </row>
+    <row r="992">
+      <c r="A992" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B992" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C992" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D992" s="3" t="inlineStr">
+        <is>
+          <t>항만이 '역대급 물동량'을 소화하는 법 - 터미널 처리능력이라는 숨은 병목</t>
+        </is>
+      </c>
+      <c r="E992" s="3" t="inlineStr">
+        <is>
+          <t>미국 LA/롱비치 항만이 관세 인상 전 조기 선적으로 역대급 물동량을 기록 중이며, 실제 병목은 선박 입항보다 터미널의 처리 능력(선석, 야드, 게이트)에서 발생하고 있다.</t>
+        </is>
+      </c>
+      <c r="F992" s="3" t="inlineStr">
+        <is>
+          <t>주요 항만의 터미널 처리 능력 부족은 물동량 증가 시 항만 적체와 운송 지연을 유발할 수 있어 우리 수출입 물류에 잠재적 영향을 미치므로 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G992" s="3" t="n"/>
+      <c r="H992" s="3" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I992" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/항만이-역대급-물동량을-소화하는-법-터미널-처리능력이라는-숨은-병목-week-29-2026-</t>
+        </is>
+      </c>
+      <c r="J992" s="3" t="inlineStr"/>
+    </row>
+    <row r="993">
+      <c r="A993" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B993" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C993" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D993" s="3" t="inlineStr">
+        <is>
+          <t>Carriers roll out hefty surcharges as demand rises in 'hot' Indian markets</t>
+        </is>
+      </c>
+      <c r="E993" s="3" t="inlineStr">
+        <is>
+          <t>인도 시장의 높은 수요로 인해 해운사들이 상당한 할증료를 부과하고 있으며, 이는 현지 수출업자들의 대규모 선복 수요를 이용하는 것이다.</t>
+        </is>
+      </c>
+      <c r="F993" s="3" t="inlineStr">
+        <is>
+          <t>특정 지역(인도)의 해상 운임 할증료 부과는 글로벌 운임 시장의 상승 압력을 시사하며, 우리 수출입 물류 비용에 잠재적 영향을 줄 수 있으므로 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G993" s="3" t="n"/>
+      <c r="H993" s="3" t="inlineStr">
+        <is>
+          <t>The Loadstar</t>
+        </is>
+      </c>
+      <c r="I993" s="3" t="inlineStr">
+        <is>
+          <t>https://theloadstar.com/carriers-roll-out-hefty-surcharges-as-demand-rises-in-hot-indian-markets</t>
+        </is>
+      </c>
+      <c r="J993" s="3" t="inlineStr"/>
+    </row>
+    <row r="994">
+      <c r="A994" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B994" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C994" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D994" s="3" t="inlineStr">
+        <is>
+          <t>윤진식 무협 회장, 부·울·경 수출기업 애로 청취</t>
+        </is>
+      </c>
+      <c r="E994" s="3" t="inlineStr">
+        <is>
+          <t>수출기업들이 해상운임 급등에 따른 컨테이너 확보 대책을 건의했으며, 유조선 입항에도 관련 비용 부담은 여전한 것으로 나타났다.</t>
+        </is>
+      </c>
+      <c r="F994" s="3" t="inlineStr">
+        <is>
+          <t>해상운임 급등 및 컨테이너 확보의 어려움은 지속적인 물류비 상승 압력으로 작용하여 우리 수출입 물류 비용에 직접적인 영향을 미칠 수 있으므로 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G994" s="3" t="n"/>
+      <c r="H994" s="3" t="inlineStr">
+        <is>
+          <t>surff.kr</t>
+        </is>
+      </c>
+      <c r="I994" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260723-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J994" s="3" t="inlineStr"/>
+    </row>
+    <row r="995">
+      <c r="A995" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B995" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C995" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D995" s="3" t="inlineStr">
+        <is>
+          <t>Cyber Attack on Major Japanese Refrigerated Logistics Provider Disrupts KFC and Other Food Chains - CPO Magazine</t>
+        </is>
+      </c>
+      <c r="E995" s="3" t="inlineStr">
+        <is>
+          <t>일본의 주요 냉장 물류 제공업체가 사이버 공격을 받아 KFC 등 식품 체인에 차질이 발생했으며, 과거 나고야 항구도 랜섬웨어 공격으로 화물 유통이 중단된 사례가 있다.</t>
+        </is>
+      </c>
+      <c r="F995" s="3" t="inlineStr">
+        <is>
+          <t>물류 시스템에 대한 사이버 공격은 운송 지연 및 운영 중단을 초래할 수 있어, 우리 회사의 물류 파트너 및 시스템 보안 강화 필요성을 시사한다.</t>
+        </is>
+      </c>
+      <c r="G995" s="3" t="inlineStr">
+        <is>
+          <t>주요 물류 파트너사의 사이버 보안 현황 점검 및 비상 계획 수립 여부 확인.</t>
+        </is>
+      </c>
+      <c r="H995" s="3" t="inlineStr">
+        <is>
+          <t>CPO Magazine</t>
+        </is>
+      </c>
+      <c r="I995" s="3" t="inlineStr">
+        <is>
+          <t>https://cpomagazine.com/cyber-security/cyber-attack-on-major-japanese-refrigerated-logistics-provider-disrupts-kfc-and-other-food-chains</t>
+        </is>
+      </c>
+      <c r="J995" s="3" t="inlineStr"/>
+    </row>
+    <row r="996">
+      <c r="A996" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B996" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C996" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D996" s="3" t="inlineStr">
+        <is>
+          <t>Global Supply Chain Disruption And Middle East Tensions Showing Up On Shelves - KamCity</t>
+        </is>
+      </c>
+      <c r="E996" s="3" t="inlineStr">
+        <is>
+          <t>중동의 지정학적 불안정으로 인한 글로벌 공급망 및 국제 해운 경로의 혼란이 진열대 상품 부족으로 이어지고 있다는 연구 결과가 나왔다.</t>
+        </is>
+      </c>
+      <c r="F996" s="3" t="inlineStr">
+        <is>
+          <t>중동 지역의 지정학적 리스크가 해운 경로에 지속적인 영향을 미쳐 운송 지연 및 비용 상승을 유발할 수 있으므로 추이를 주시해야 한다.</t>
+        </is>
+      </c>
+      <c r="G996" s="3" t="inlineStr">
+        <is>
+          <t>중동 항로 의존도 점검 및 대체 운송 경로/방안 사전 검토.</t>
+        </is>
+      </c>
+      <c r="H996" s="3" t="inlineStr">
+        <is>
+          <t>KamCity</t>
+        </is>
+      </c>
+      <c r="I996" s="3" t="inlineStr">
+        <is>
+          <t>https://www.kamcity.com/namnews/uk-and-ireland/manufacturers/global-supply-chain-disruption-and-middle-east-tensions-showing-up-on-shelves/</t>
+        </is>
+      </c>
+      <c r="J996" s="3" t="inlineStr"/>
+    </row>
+    <row r="997">
+      <c r="A997" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B997" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C997" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D997" s="3" t="inlineStr">
+        <is>
+          <t>한여름 활주로는 거대한 가마솥, '폭염안전 수칙' 의무화 절실 - 오마이뉴스</t>
+        </is>
+      </c>
+      <c r="E997" s="3" t="inlineStr">
+        <is>
+          <t>공항과 항만 노동자들이 폭염에 상시 노출되어 있으며, 폭염일수 증가에 따라 이들의 안전을 위한 폭염 안전 수칙 의무화가 절실하다는 내용이다.</t>
+        </is>
+      </c>
+      <c r="F997" s="3" t="inlineStr">
+        <is>
+          <t>폭염으로 인한 항만/공항 작업자의 안전 문제는 작업 지연이나 인력 운영에 영향을 줄 수 있으므로, 물류 파트너사의 대응 현황을 모니터링할 필요가 있다.</t>
+        </is>
+      </c>
+      <c r="G997" s="3" t="inlineStr">
+        <is>
+          <t>물류 파트너사의 폭염 대비 작업 환경 및 안전 수칙 준수 여부 확인.</t>
+        </is>
+      </c>
+      <c r="H997" s="3" t="inlineStr">
+        <is>
+          <t>오마이뉴스</t>
+        </is>
+      </c>
+      <c r="I997" s="3" t="inlineStr">
+        <is>
+          <t>https://ohmynews.com/NWS_Web/View/at_pg.aspx?CMPT_CD=M0117&amp;CNTN_CD=A0003253020&amp;PAGE_CD=N0002</t>
+        </is>
+      </c>
+      <c r="J997" s="3" t="inlineStr"/>
+    </row>
+    <row r="998">
+      <c r="A998" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B998" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C998" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D998" s="3" t="inlineStr">
+        <is>
+          <t>[한국세정신문] 한미 관세당국, 마약 등 신종 무역범죄 공조 확대</t>
+        </is>
+      </c>
+      <c r="E998" s="3" t="inlineStr">
+        <is>
+          <t>한미 관세당국이 컨테이너 안전구상 부칙 제정 서명식을 통해 마약 등 신종 무역범죄 공조를 확대하기로 합의했다.</t>
+        </is>
+      </c>
+      <c r="F998" s="3" t="inlineStr">
+        <is>
+          <t>관세 당국의 무역 범죄 공조 확대는 컨테이너 검사 강화로 이어져 통관 지연 가능성을 높일 수 있으므로, 관련 동향을 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G998" s="3" t="inlineStr">
+        <is>
+          <t>통관 절차 지연 가능성에 대비하여 리드타임 점검 및 필요 시 통관 대행사와 협의.</t>
+        </is>
+      </c>
+      <c r="H998" s="3" t="inlineStr">
+        <is>
+          <t>한국세정신문</t>
+        </is>
+      </c>
+      <c r="I998" s="3" t="inlineStr">
+        <is>
+          <t>https://taxtimes.co.kr/news/article.html?no=276101</t>
+        </is>
+      </c>
+      <c r="J998" s="3" t="inlineStr"/>
+    </row>
+    <row r="999">
+      <c r="A999" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B999" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C999" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D999" s="3" t="inlineStr">
+        <is>
+          <t>위성락 “美, 한국에 추가 관세 부과 가능성”</t>
+        </is>
+      </c>
+      <c r="E999" s="3" t="inlineStr">
+        <is>
+          <t>미국이 한국에 추가 관세를 부과할 가능성이 있으며, 한미 합의 15% 세율을 넘지 않을 것으로 예상되나 정부는 미국과 협의하며 대응 중이다.</t>
+        </is>
+      </c>
+      <c r="F999" s="3" t="inlineStr">
+        <is>
+          <t>배터리/전자부품 수출 시 관세가 부과될 경우 물류비용 및 가격 경쟁력에 직접적인 영향을 미칠 수 있으므로 추이를 면밀히 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G999" s="3" t="inlineStr">
+        <is>
+          <t>미국 무역 정책 동향 및 한국 정부의 대응을 지속적으로 주시하고, 잠재적 관세 부과 시나리오별 물류 비용 및 공급망 영향 분석을 준비해야 함.</t>
+        </is>
+      </c>
+      <c r="H999" s="3" t="inlineStr">
+        <is>
+          <t>서울신문</t>
+        </is>
+      </c>
+      <c r="I999" s="3" t="inlineStr">
+        <is>
+          <t>https://seoul.co.kr/news/politics/2026/07/23/20260723008004</t>
+        </is>
+      </c>
+      <c r="J999" s="3" t="inlineStr"/>
+    </row>
+    <row r="1000">
+      <c r="A1000" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B1000" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C1000" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1000" s="3" t="inlineStr">
+        <is>
+          <t>홍해서 유조선 줄줄이 회항…원유 ‘마지막 우회로’도 흔들</t>
+        </is>
+      </c>
+      <c r="E1000" s="3" t="inlineStr">
+        <is>
+          <t>홍해에서 후티 반군의 위협으로 유조선들이 회항하면서, 우회 항로 장기화 시 운임 및 보험료가 추가 상승할 수 있다.</t>
+        </is>
+      </c>
+      <c r="F1000" s="3" t="inlineStr">
+        <is>
+          <t>유가 상승은 항공 및 해상 운임에 직접적인 영향을 미쳐 물류비용 증가로 이어질 수 있으므로 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G1000" s="3" t="inlineStr">
+        <is>
+          <t>유가 및 해상 운임 변동 추이를 면밀히 주시하고, 잠재적 물류비용 상승에 대비한 예산 계획을 검토해야 함.</t>
+        </is>
+      </c>
+      <c r="H1000" s="3" t="inlineStr">
+        <is>
+          <t>이투데이</t>
+        </is>
+      </c>
+      <c r="I1000" s="3" t="inlineStr">
+        <is>
+          <t>https://etoday.co.kr/news/view/2606309</t>
+        </is>
+      </c>
+      <c r="J1000" s="3" t="inlineStr"/>
+    </row>
+    <row r="1001">
+      <c r="A1001" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B1001" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C1001" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1001" s="3" t="inlineStr">
+        <is>
+          <t>뉴욕증시 반등 하루만에 약세...미국, 11일 연속 공습에 유가 $95 터치도 [월가월부]</t>
+        </is>
+      </c>
+      <c r="E1001" s="3" t="inlineStr">
+        <is>
+          <t>미국 공습 지속으로 뉴욕 증시가 약세를 보이며 유가가 배럴당 95달러를 기록하는 등 상승 압력을 받고 있다.</t>
+        </is>
+      </c>
+      <c r="F1001" s="3" t="inlineStr">
+        <is>
+          <t>유가 상승은 항공 및 해상 운임에 직접적인 영향을 미쳐 물류비용 증가로 이어질 수 있으므로 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G1001" s="3" t="inlineStr">
+        <is>
+          <t>유가 변동 추이를 면밀히 주시하고, 잠재적 물류비용 상승에 대비한 예산 계획을 검토해야 함.</t>
+        </is>
+      </c>
+      <c r="H1001" s="3" t="inlineStr">
+        <is>
+          <t>매일경제</t>
+        </is>
+      </c>
+      <c r="I1001" s="3" t="inlineStr">
+        <is>
+          <t>https://mk.co.kr/news/stock/12104991</t>
+        </is>
+      </c>
+      <c r="J1001" s="3" t="inlineStr"/>
+    </row>
+    <row r="1002">
+      <c r="A1002" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B1002" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C1002" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D1002" s="4" t="inlineStr">
+        <is>
+          <t>해운·물류 공급망 협력 위해 협력구축</t>
+        </is>
+      </c>
+      <c r="E1002" s="4" t="inlineStr">
+        <is>
+          <t>한국해양수산개발원과 한국해양진흥공사가 해운·물류 공급망 협력을 위한 업무협약을 체결했으며, AI 기반 해상공급망 조기경보 시스템 구축을 목표로 한다.</t>
+        </is>
+      </c>
+      <c r="F1002" s="4" t="inlineStr">
+        <is>
+          <t>장기적인 관점에서 공급망 가시성 개선에 기여할 수 있으나, 당장 우리 물류 운영에 직접적인 영향을 미치지는 않는다.</t>
+        </is>
+      </c>
+      <c r="G1002" s="4" t="n"/>
+      <c r="H1002" s="4" t="inlineStr">
+        <is>
+          <t>cargonews</t>
+        </is>
+      </c>
+      <c r="I1002" s="4" t="inlineStr">
+        <is>
+          <t>https://www.cargonews.co.kr/news/articleView.html?idxno=60573</t>
+        </is>
+      </c>
+      <c r="J1002" s="4" t="inlineStr"/>
+    </row>
+    <row r="1003">
+      <c r="A1003" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B1003" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C1003" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D1003" s="4" t="inlineStr">
+        <is>
+          <t>벌크선 시장, 全 선형서 숨고르기…선복 증가 추세 이어져</t>
+        </is>
+      </c>
+      <c r="E1003" s="4" t="inlineStr">
+        <is>
+          <t>7월 중순 벌크선 시장은 모든 선형에서 운임 하락세를 보였으며, 특히 태평양 수역에서 중국 항만 체선 해소로 선복 증가 효과가 발생했다.</t>
+        </is>
+      </c>
+      <c r="F1003" s="4" t="inlineStr">
+        <is>
+          <t>벌크선 시장 동향은 컨테이너 운송에 직접적인 영향은 적지만, 중국 항만 체선 해소는 전반적인 항만 운영 효율성 개선 가능성을 시사하므로 참고할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G1003" s="4" t="n"/>
+      <c r="H1003" s="4" t="inlineStr">
+        <is>
+          <t>ksg</t>
+        </is>
+      </c>
+      <c r="I1003" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksg.co.kr/news/main_newsView.jsp?pNum=147666</t>
+        </is>
+      </c>
+      <c r="J1003" s="4" t="inlineStr"/>
+    </row>
+    <row r="1004">
+      <c r="A1004" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B1004" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C1004" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D1004" s="4" t="inlineStr">
+        <is>
+          <t>‘2만4000TEU’에서 멈춘 이유…초대형 ‘컨선의 경제학’</t>
+        </is>
+      </c>
+      <c r="E1004" s="4" t="inlineStr">
+        <is>
+          <t>컨테이너선 대형화가 2만4000TEU급에서 사실상 멈춘 이유를 분석하며, 초대형 컨테이너선의 경제성과 한계에 대해 다루고 있다.</t>
+        </is>
+      </c>
+      <c r="F1004" s="4" t="inlineStr">
+        <is>
+          <t>컨테이너선 대형화 추세에 대한 분석으로, 현재 우리 물류 운영에 직접적인 영향을 미치기보다는 장기적인 해운 시장 동향을 이해하는 데 참고할 만한 수준이다.</t>
+        </is>
+      </c>
+      <c r="G1004" s="4" t="n"/>
+      <c r="H1004" s="4" t="inlineStr">
+        <is>
+          <t>아시아투데이</t>
+        </is>
+      </c>
+      <c r="I1004" s="4" t="inlineStr">
+        <is>
+          <t>https://asiatoday.co.kr/kn/view.php?key=20260722010008106</t>
+        </is>
+      </c>
+      <c r="J1004" s="4" t="inlineStr"/>
+    </row>
+    <row r="1005">
+      <c r="A1005" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B1005" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C1005" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D1005" s="4" t="inlineStr">
+        <is>
+          <t>관세청, 2026년 상반기 마약류 총 767건, 1,007kg 적발</t>
+        </is>
+      </c>
+      <c r="E1005" s="4" t="inlineStr">
+        <is>
+          <t>관세청이 2026년 상반기 마약류 밀수 단속 현황을 발표하며 총 767건, 1,007kg의 마약류를 적발했다고 밝혔다.</t>
+        </is>
+      </c>
+      <c r="F1005" s="4" t="inlineStr">
+        <is>
+          <t>마약 밀수 단속 강화는 일반 화물 운송에 직접적인 영향을 미치지 않으며, 우리 회사의 물류 운영과는 무관하다.</t>
+        </is>
+      </c>
+      <c r="G1005" s="4" t="inlineStr"/>
+      <c r="H1005" s="4" t="inlineStr">
+        <is>
+          <t>localsegye.co.kr</t>
+        </is>
+      </c>
+      <c r="I1005" s="4" t="inlineStr">
+        <is>
+          <t>https://localsegye.co.kr/news/view/1065593432351077</t>
+        </is>
+      </c>
+      <c r="J1005" s="4" t="inlineStr"/>
+    </row>
+    <row r="1006">
+      <c r="A1006" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B1006" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C1006" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D1006" s="4" t="inlineStr">
+        <is>
+          <t>日 완성차 업계, 2028년 공동수송 도입…운전기사 부족 대응 | 연합뉴스</t>
+        </is>
+      </c>
+      <c r="E1006" s="4" t="inlineStr">
+        <is>
+          <t>일본 완성차 업계가 운전기사 부족 문제에 대응하기 위해 2028년까지 완성차 공동 수송 시스템을 도입할 계획이다.</t>
+        </is>
+      </c>
+      <c r="F1006" s="4" t="inlineStr">
+        <is>
+          <t>일본 완성차 업계의 공동 수송 도입은 장기적인 물류 효율화 방안으로 참고할 만하나, 우리 회사의 현재 물류 운영에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G1006" s="4" t="inlineStr"/>
+      <c r="H1006" s="4" t="inlineStr">
+        <is>
+          <t>연합뉴스</t>
+        </is>
+      </c>
+      <c r="I1006" s="4" t="inlineStr">
+        <is>
+          <t>https://yna.co.kr/view/AKR20260722067300009</t>
+        </is>
+      </c>
+      <c r="J1006" s="4" t="inlineStr"/>
+    </row>
+    <row r="1007">
+      <c r="A1007" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B1007" s="4" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1007" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D1007" s="4" t="inlineStr">
+        <is>
+          <t>[테크 차이나] 아세안은 생산, 중동은 자본, 유럽은 규칙…중국 공급망 세계지도 〈하〉 [박지민의 비욘드 차이나]</t>
+        </is>
+      </c>
+      <c r="E1007" s="4" t="inlineStr">
+        <is>
+          <t>중국의 글로벌 공급망 전략은 현지화, 규제 대응, 미국 영향력 관리를 포함하며, 한국과 일본은 반도체, 배터리 소재·장비 등 첨단 부품 협력 파트너로 인식된다.</t>
+        </is>
+      </c>
+      <c r="F1007" s="4" t="inlineStr">
+        <is>
+          <t>중국의 장기적인 공급망 전략에 대한 분석으로, 우리 회사의 직접적인 물류 운영에 당장 영향을 미치기보다는 참고할 만한 거시적 동향이다.</t>
+        </is>
+      </c>
+      <c r="G1007" s="4" t="inlineStr"/>
+      <c r="H1007" s="4" t="inlineStr">
+        <is>
+          <t>전자신문</t>
+        </is>
+      </c>
+      <c r="I1007" s="4" t="inlineStr">
+        <is>
+          <t>https://etnews.com/20260721000272</t>
+        </is>
+      </c>
+      <c r="J1007" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -46726,7 +48130,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -47705,6 +49109,49 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>3080.31</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>-105 (-3.3%)</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>+1,317 (+74.7%)</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="n">
+        <v>4204</v>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>-114 (-2.6%)</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>+1,755 (+71.7%)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -47717,7 +49164,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I182"/>
+  <dimension ref="A1:I186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -54113,6 +55560,146 @@
       </c>
       <c r="I182" s="6" t="inlineStr"/>
     </row>
+    <row r="183">
+      <c r="A183" s="6" t="inlineStr">
+        <is>
+          <t>RSK-182</t>
+        </is>
+      </c>
+      <c r="B183" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="C183" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D183" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E183" s="6" t="inlineStr">
+        <is>
+          <t>미·이란 충돌 격화에 홍해 봉쇄 위협까지…국제유가 2%↑</t>
+        </is>
+      </c>
+      <c r="F183" s="6" t="inlineStr"/>
+      <c r="G183" s="6" t="inlineStr"/>
+      <c r="H183" s="6" t="inlineStr">
+        <is>
+          <t>홍해 항로 이용 현황 점검 및 대체 항로(희망봉 우회 등) 검토, 운송사와의 비상 계획 수립, 유가 변동에 따른 물류비 예산 재검토.</t>
+        </is>
+      </c>
+      <c r="I183" s="6" t="inlineStr"/>
+    </row>
+    <row r="184">
+      <c r="A184" s="6" t="inlineStr">
+        <is>
+          <t>RSK-183</t>
+        </is>
+      </c>
+      <c r="B184" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="C184" s="6" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="D184" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E184" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈 이어 홍해 봉쇄 위기... 다시 희망봉 돌아야 하나</t>
+        </is>
+      </c>
+      <c r="F184" s="6" t="inlineStr"/>
+      <c r="G184" s="6" t="inlineStr"/>
+      <c r="H184" s="6" t="inlineStr">
+        <is>
+          <t>대체 항로 및 운송 수단 검토, 비상 재고 확보, 운임 변동성 분석 및 계약 조건 재검토, 공급망 리스크 평가 및 대응 계획 수립</t>
+        </is>
+      </c>
+      <c r="I184" s="6" t="inlineStr"/>
+    </row>
+    <row r="185">
+      <c r="A185" s="6" t="inlineStr">
+        <is>
+          <t>RSK-184</t>
+        </is>
+      </c>
+      <c r="B185" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="C185" s="6" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="D185" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E185" s="6" t="inlineStr">
+        <is>
+          <t>[단독] ‘덕평 악몽’ 5년 만에 또…쿠팡, 全물류센터 안전시스템 전면 재정비[물류센터의 경고] - 이투데이</t>
+        </is>
+      </c>
+      <c r="F185" s="6" t="inlineStr"/>
+      <c r="G185" s="6" t="inlineStr"/>
+      <c r="H185" s="6" t="inlineStr">
+        <is>
+          <t>우리 회사의 물류센터 안전 점검 및 위험물 보관 규정 준수 여부 확인, 비상 대응 훈련 강화, 물류 파트너사의 안전 관리 현황 확인.</t>
+        </is>
+      </c>
+      <c r="I185" s="6" t="inlineStr"/>
+    </row>
+    <row r="186">
+      <c r="A186" s="6" t="inlineStr">
+        <is>
+          <t>RSK-185</t>
+        </is>
+      </c>
+      <c r="B186" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="C186" s="6" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="D186" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E186" s="6" t="inlineStr">
+        <is>
+          <t>[데일리연합 (SNSJTV)] 리튬 배터리 수백대와 충격적인 붕괴 위험</t>
+        </is>
+      </c>
+      <c r="F186" s="6" t="inlineStr"/>
+      <c r="G186" s="6" t="inlineStr"/>
+      <c r="H186" s="6" t="inlineStr">
+        <is>
+          <t>리튬 배터리 보관 시설의 안전성 재점검, 취급 절차 준수 여부 확인, 관련 안전 교육 강화.</t>
+        </is>
+      </c>
+      <c r="I186" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
📰 뉴스 데이터 2026-07-24_09:04
</commit_message>
<xml_diff>
--- a/data/SCM_물류_브리핑.xlsx
+++ b/data/SCM_물류_브리핑.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1007"/>
+  <dimension ref="A1:J1036"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -48118,6 +48118,1394 @@
       </c>
       <c r="J1007" s="4" t="inlineStr"/>
     </row>
+    <row r="1008">
+      <c r="A1008" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B1008" s="2" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C1008" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D1008" s="2" t="inlineStr">
+        <is>
+          <t>파나마 운하 관리청, ‘3차 기간’ 슬롯경매 일시중단</t>
+        </is>
+      </c>
+      <c r="E1008" s="2" t="inlineStr">
+        <is>
+          <t>파나마 운하 관리청이 수자원 관리 및 엘니뇨 대비를 위해 '3차 기간' 슬롯 경매를 일시 중단하여 대기 시간 연장이 우려됩니다.</t>
+        </is>
+      </c>
+      <c r="F1008" s="2" t="inlineStr">
+        <is>
+          <t>파나마 운하 통항 제한은 주요 동서 무역로의 운송 시간과 비용에 직접적인 영향을 미치므로 즉각적인 대체 경로 또는 일정 평가가 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G1008" s="2" t="inlineStr">
+        <is>
+          <t>파나마 운하를 이용하는 현재 및 계획된 선적을 평가하고, 대체 경로(예: 수에즈 운하, 철도, 복합운송)를 모색하며, 잠재적 지연을 내부 이해관계자에게 전달해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H1008" s="2" t="inlineStr">
+        <is>
+          <t>kita</t>
+        </is>
+      </c>
+      <c r="I1008" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kita.net/shippers/board/newsView.do?morgueCode=2&amp;dataCls=B&amp;dataSeq=8175</t>
+        </is>
+      </c>
+      <c r="J1008" s="2" t="inlineStr">
+        <is>
+          <t>RSK-186</t>
+        </is>
+      </c>
+    </row>
+    <row r="1009">
+      <c r="A1009" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B1009" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1009" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D1009" s="2" t="inlineStr">
+        <is>
+          <t>“돌아가면 30일, 얀부 막히면 그마저도 못한다”</t>
+        </is>
+      </c>
+      <c r="E1009" s="2" t="inlineStr">
+        <is>
+          <t>예멘 후티 반군의 홍해 봉쇄로 국제유가가 배럴당 100달러를 돌파했으며, 사우디아라비아의 주요 홍해 원유 수출항인 얀부까지 위협이 확대될 가능성에 대한 우려가 커지고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F1009" s="2" t="inlineStr">
+        <is>
+          <t>홍해 봉쇄와 얀부 항구로의 위협 확대 가능성은 글로벌 해운 경로, 운송 시간 및 연료 비용에 심각한 위험을 초래하므로 즉각적인 비상 계획이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G1009" s="2" t="inlineStr">
+        <is>
+          <t>홍해 지역을 통과하거나 영향을 받을 수 있는 모든 선적을 검토하고, 대체 경로를 평가하며, 유가 변동을 모니터링하고, 잠재적 혼란에 대비한 비상 계획을 수립해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H1009" s="2" t="inlineStr">
+        <is>
+          <t>oceanpress</t>
+        </is>
+      </c>
+      <c r="I1009" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oceanpress.co.kr/news/article.html?no=30718</t>
+        </is>
+      </c>
+      <c r="J1009" s="2" t="inlineStr">
+        <is>
+          <t>RSK-187</t>
+        </is>
+      </c>
+    </row>
+    <row r="1010">
+      <c r="A1010" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B1010" s="2" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C1010" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D1010" s="2" t="inlineStr">
+        <is>
+          <t>[해양통신] 머스크, 우크라이나 초르노모르스크항 기항 중단</t>
+        </is>
+      </c>
+      <c r="E1010" s="2" t="inlineStr">
+        <is>
+          <t>러시아와 우크라이나 간 공격 격화로 머스크가 우크라이나 초르노모르스크항 기항 서비스를 중단하여 흑해 해상 수출망이 다시 위협받고 있다.</t>
+        </is>
+      </c>
+      <c r="F1010" s="2" t="inlineStr">
+        <is>
+          <t>주요 선사의 특정 항만 기항 중단은 해당 지역으로의 운송 경로를 완전히 차단하여 우리 회사의 물류 계획 및 공급망에 직접적인 차질을 발생시킬 수 있다.</t>
+        </is>
+      </c>
+      <c r="G1010" s="2" t="inlineStr">
+        <is>
+          <t>흑해 지역을 경유하는 운송 경로가 있는지 즉시 확인하고, 해당 지역으로의 운송이 필요한 경우 대체 경로 및 운송 수단을 긴급히 검토해야 한다.</t>
+        </is>
+      </c>
+      <c r="H1010" s="2" t="inlineStr">
+        <is>
+          <t>해양통신</t>
+        </is>
+      </c>
+      <c r="I1010" s="2" t="inlineStr">
+        <is>
+          <t>https://oceanpress.co.kr/news/article.html?no=30704</t>
+        </is>
+      </c>
+      <c r="J1010" s="2" t="inlineStr">
+        <is>
+          <t>RSK-188</t>
+        </is>
+      </c>
+    </row>
+    <row r="1011">
+      <c r="A1011" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B1011" s="2" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C1011" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D1011" s="2" t="inlineStr">
+        <is>
+          <t>61시간 사투가 남긴 경고...물류 로봇 ‘리튬 배터리’ 화재 취약성[스마트 물류의 그늘]</t>
+        </is>
+      </c>
+      <c r="E1011" s="2" t="inlineStr">
+        <is>
+          <t>물류 로봇에 사용되는 리튬 배터리의 화재 취약성이 부각되며, 물류창고 내 배터리 포함 소방체계 및 이차전지 규제 강화의 필요성이 제기되고 있다.</t>
+        </is>
+      </c>
+      <c r="F1011" s="2" t="inlineStr">
+        <is>
+          <t>배터리 제조사로서 물류센터 내 배터리 화재 위험성 및 관련 규제 강화 논의는 보관, 운송, 안전 관리 프로세스에 즉각적인 변경을 요구할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G1011" s="2" t="inlineStr">
+        <is>
+          <t>물류센터 내 배터리 보관 및 취급 안전 절차 전면 재검토, 관련 법규 및 규제 동향 상시 모니터링, 비상 대응 계획 강화.</t>
+        </is>
+      </c>
+      <c r="H1011" s="2" t="inlineStr">
+        <is>
+          <t>이투데이</t>
+        </is>
+      </c>
+      <c r="I1011" s="2" t="inlineStr">
+        <is>
+          <t>https://www.etoday.co.kr/news/view/2606640</t>
+        </is>
+      </c>
+      <c r="J1011" s="2" t="inlineStr">
+        <is>
+          <t>RSK-189</t>
+        </is>
+      </c>
+    </row>
+    <row r="1012">
+      <c r="A1012" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B1012" s="2" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C1012" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D1012" s="2" t="inlineStr">
+        <is>
+          <t>[사회]쿠팡 물류센터 화재 109시간 만에 완진...다른 센터에 또 불</t>
+        </is>
+      </c>
+      <c r="E1012" s="2" t="inlineStr">
+        <is>
+          <t>인천 석남동 쿠팡 물류센터 화재가 완진된 후, 항동의 또 다른 물류센터에서 화재가 발생하여 물류센터 화재 안전에 대한 경각심이 높아지고 있다.</t>
+        </is>
+      </c>
+      <c r="F1012" s="2" t="inlineStr">
+        <is>
+          <t>물류센터 화재 발생은 배터리/전자부품 보관 및 취급 안전에 대한 경각심을 높이고, 향후 물류센터 규제 강화로 이어질 수 있다.</t>
+        </is>
+      </c>
+      <c r="G1012" s="2" t="inlineStr">
+        <is>
+          <t>물류센터 내 화재 예방 및 진압 시스템 점검, 비상 대응 계획 재검토, 배터리 보관 시설 안전성 강화 방안 모색.</t>
+        </is>
+      </c>
+      <c r="H1012" s="2" t="inlineStr">
+        <is>
+          <t>YTN</t>
+        </is>
+      </c>
+      <c r="I1012" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ytn.co.kr/_ln/0103_202607230938138586</t>
+        </is>
+      </c>
+      <c r="J1012" s="2" t="inlineStr">
+        <is>
+          <t>RSK-190</t>
+        </is>
+      </c>
+    </row>
+    <row r="1013">
+      <c r="A1013" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B1013" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1013" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D1013" s="2" t="inlineStr">
+        <is>
+          <t>[속보] 미국 USTR, 무역법 301조 '강제노동 관세' 부과</t>
+        </is>
+      </c>
+      <c r="E1013" s="2" t="inlineStr">
+        <is>
+          <t>미국 USTR이 무역법 301조에 의거하여 '강제노동 관세'를 부과할 예정으로, 특정 지역/국가에서 생산된 제품의 수입에 영향을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="F1013" s="2" t="inlineStr">
+        <is>
+          <t>강제노동 관세 부과는 우리 회사의 특정 공급망(특히 중국 등)에서 생산되는 부품/제품의 수입 비용 및 공급망 전략에 직접적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G1013" s="2" t="inlineStr">
+        <is>
+          <t>공급망 내 강제노동 관련 리스크 점검, 해당 관세 부과 대상 품목 및 지역 확인, 공급망 다변화 또는 대체 소싱 방안 검토.</t>
+        </is>
+      </c>
+      <c r="H1013" s="2" t="inlineStr">
+        <is>
+          <t>이투데이</t>
+        </is>
+      </c>
+      <c r="I1013" s="2" t="inlineStr">
+        <is>
+          <t>https://etoday.co.kr/news/view/2606896</t>
+        </is>
+      </c>
+      <c r="J1013" s="2" t="inlineStr">
+        <is>
+          <t>RSK-191</t>
+        </is>
+      </c>
+    </row>
+    <row r="1014">
+      <c r="A1014" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B1014" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1014" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D1014" s="2" t="inlineStr">
+        <is>
+          <t>트럼프 '관세 재건'…韓 강제노동 12.5%에 남은 '2.5%p'에 협상 성패 달렸다</t>
+        </is>
+      </c>
+      <c r="E1014" s="2" t="inlineStr">
+        <is>
+          <t>미국 정부가 강제노동으로 생산된 제품 수입을 금지하지 않은 60개 경제권에 10% 또는 12.5%의 관세를 부과할 예정이며, 한국은 12.5% 관세 부과 대상에 포함될 가능성이 있다.</t>
+        </is>
+      </c>
+      <c r="F1014" s="2" t="inlineStr">
+        <is>
+          <t>미국이 한국산 제품에 강제노동 관세를 부과할 경우, 우리 회사의 대미 수출 제품에 직접적인 비용 상승을 초래하여 물류 및 가격 전략에 즉각적인 영향을 미친다.</t>
+        </is>
+      </c>
+      <c r="G1014" s="2" t="inlineStr">
+        <is>
+          <t>대미 수출 제품의 원산지 증명 및 공급망 내 강제노동 리스크 점검 강화, 관세 부과 시나리오별 비용 분석 및 대응 방안 마련.</t>
+        </is>
+      </c>
+      <c r="H1014" s="2" t="inlineStr">
+        <is>
+          <t>이데일리</t>
+        </is>
+      </c>
+      <c r="I1014" s="2" t="inlineStr">
+        <is>
+          <t>https://edaily.co.kr/News/Read?mediaCodeNo=257&amp;newsId=02722406645517800</t>
+        </is>
+      </c>
+      <c r="J1014" s="2" t="inlineStr">
+        <is>
+          <t>RSK-192</t>
+        </is>
+      </c>
+    </row>
+    <row r="1015">
+      <c r="A1015" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B1015" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C1015" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D1015" s="2" t="inlineStr">
+        <is>
+          <t>[속보] 브렌트유 배럴당 100달러 재돌파…5월 26일 이후 처음 - 매일경제</t>
+        </is>
+      </c>
+      <c r="E1015" s="2" t="inlineStr">
+        <is>
+          <t>중동 긴장 고조로 국제유가 기준인 브렌트유 가격이 약 두 달 만에 배럴당 100달러를 재돌파했다.</t>
+        </is>
+      </c>
+      <c r="F1015" s="2" t="inlineStr">
+        <is>
+          <t>국제유가 급등은 해상 및 항공 운임 상승, 육상 운송 비용 증가로 이어져 우리 회사의 전체 물류 비용에 즉각적이고 직접적인 영향을 미친다.</t>
+        </is>
+      </c>
+      <c r="G1015" s="2" t="inlineStr">
+        <is>
+          <t>유가 변동에 따른 물류비용 증가분 분석, 운송 계약 조건 재검토, 연료 효율 개선 방안 모색, 비상 운송 계획 수립.</t>
+        </is>
+      </c>
+      <c r="H1015" s="2" t="inlineStr">
+        <is>
+          <t>매일경제</t>
+        </is>
+      </c>
+      <c r="I1015" s="2" t="inlineStr">
+        <is>
+          <t>https://mk.co.kr/news/economy/12106036</t>
+        </is>
+      </c>
+      <c r="J1015" s="2" t="inlineStr">
+        <is>
+          <t>RSK-193</t>
+        </is>
+      </c>
+    </row>
+    <row r="1016">
+      <c r="A1016" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B1016" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1016" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1016" s="3" t="inlineStr">
+        <is>
+          <t>U.S.-EU Trade Agreement Eliminates Duties on Most U.S. Goods Starting July 1; TPEB Rates Rise as July Capacity Hits Three-Year High</t>
+        </is>
+      </c>
+      <c r="E1016" s="3" t="inlineStr">
+        <is>
+          <t>미국-EU 무역 협정으로 7월 1일부터 대부분의 미국 상품에 대한 관세가 철폐되는 반면, 태평양 동향(TPEB) 운임은 7월 선복량이 3년 만에 최고치를 기록하며 상승하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F1016" s="3" t="inlineStr">
+        <is>
+          <t>미국-EU 관세 철폐는 관련 무역로의 비용을 절감할 수 있지만, TPEB 운임 상승은 태평양 횡단 운송 비용을 증가시킬 것입니다.</t>
+        </is>
+      </c>
+      <c r="G1016" s="3" t="inlineStr">
+        <is>
+          <t>TPEB 운임 추이를 모니터링하고, 미국-EU 관세 철폐로 인한 관련 제품 흐름의 잠재적 비용 절감 효과를 평가해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H1016" s="3" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I1016" s="3" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/july-02-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J1016" s="3" t="inlineStr"/>
+    </row>
+    <row r="1017">
+      <c r="A1017" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B1017" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1017" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1017" s="3" t="inlineStr">
+        <is>
+          <t>Statement on EU Commission Revision of the EU Emissions Trading System</t>
+        </is>
+      </c>
+      <c r="E1017" s="3" t="inlineStr">
+        <is>
+          <t>국제항공운송협회(IATA)는 유럽연합(EU) 배출권거래제(ETS)를 유럽 국경 너머로 확대하려는 제안에 대해 깊은 불만을 표명하며 부정적인 결과를 경고했습니다.</t>
+        </is>
+      </c>
+      <c r="F1017" s="3" t="inlineStr">
+        <is>
+          <t>EU ETS 확대는 EU 관련 항공 화물 운송 비용을 크게 증가시키고 운영 복잡성을 가중시킬 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G1017" s="3" t="inlineStr">
+        <is>
+          <t>EU ETS 개정 진행 상황을 모니터링하고, EU를 오가는 항공 화물 운송의 잠재적 비용 증가를 평가해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H1017" s="3" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I1017" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/07-17-statement-eu-commission-revision-emissions-trading-system/</t>
+        </is>
+      </c>
+      <c r="J1017" s="3" t="inlineStr"/>
+    </row>
+    <row r="1018">
+      <c r="A1018" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B1018" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C1018" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1018" s="3" t="inlineStr">
+        <is>
+          <t>Structural Contraction of Global Liner Networks</t>
+        </is>
+      </c>
+      <c r="E1018" s="3" t="inlineStr">
+        <is>
+          <t>IMF의 최신 보고서에 따르면 2025년 5.0%에서 2026년 3.5%로 글로벌 무역량 증가율이 급격히 둔화될 것으로 예상되며, 이는 글로벌 정기선 네트워크의 구조적 축소로 이어질 것입니다.</t>
+        </is>
+      </c>
+      <c r="F1018" s="3" t="inlineStr">
+        <is>
+          <t>글로벌 무역 둔화와 정기선 네트워크 축소는 중기적으로 해운 옵션 감소 및 잠재적 비용 상승 또는 리드 타임 증가로 이어질 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G1018" s="3" t="inlineStr">
+        <is>
+          <t>글로벌 무역 전망과 선사 서비스 발표를 모니터링하여 해운 선복량 및 서비스 빈도의 잠재적 변화를 예측해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H1018" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I1018" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/398-structural-contraction-of-global-liner-network</t>
+        </is>
+      </c>
+      <c r="J1018" s="3" t="inlineStr"/>
+    </row>
+    <row r="1019">
+      <c r="A1019" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B1019" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C1019" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1019" s="3" t="inlineStr">
+        <is>
+          <t>PLSCI Data Indicates Mega-Hub Retrenchment</t>
+        </is>
+      </c>
+      <c r="E1019" s="3" t="inlineStr">
+        <is>
+          <t>2026년 2분기 항만 정기선 연결성 지수(PLSCI) 분석 결과, 최근 네트워크 재조정이 메가 허브의 축소로 이어졌음을 시사합니다.</t>
+        </is>
+      </c>
+      <c r="F1019" s="3" t="inlineStr">
+        <is>
+          <t>항만 연결성 및 메가 허브 전략의 변화는 현재의 항만 선택 및 환적 전략에 영향을 미치고 특정 경로의 리드 타임을 증가시킬 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G1019" s="3" t="inlineStr">
+        <is>
+          <t>잠재적인 메가 허브 축소에 대비하여 현재 항만 사용 및 환적 전략을 검토하고 대체 항만 옵션을 평가해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H1019" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I1019" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/396-plsci-data-indicates-mega-hub-retrenchment</t>
+        </is>
+      </c>
+      <c r="J1019" s="3" t="inlineStr"/>
+    </row>
+    <row r="1020">
+      <c r="A1020" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B1020" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C1020" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1020" s="3" t="inlineStr">
+        <is>
+          <t>[sea] Tracking True Vessel Delay</t>
+        </is>
+      </c>
+      <c r="E1020" s="3" t="inlineStr">
+        <is>
+          <t>해운사들이 스케줄 버퍼링을 늘려 겉으로는 정시 도착률을 높이지만 실제 운송 리드타임은 길어지고 있어 진정한 선박 지연 추적이 중요해지고 있다.</t>
+        </is>
+      </c>
+      <c r="F1020" s="3" t="inlineStr">
+        <is>
+          <t>선박 스케줄 버퍼링 증가는 겉보기 정시성을 높이나 실제 운송 리드타임을 증가시켜 우리 물류 계획에 잠재적 영향을 미칠 수 있으므로 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G1020" s="3" t="inlineStr">
+        <is>
+          <t>정기 선박 스케줄 및 실제 운송 리드타임 데이터를 지속적으로 분석하여 운송 계획에 반영할 필요가 있다.</t>
+        </is>
+      </c>
+      <c r="H1020" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I1020" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/394-tracking-true-vessel-delay</t>
+        </is>
+      </c>
+      <c r="J1020" s="3" t="inlineStr"/>
+    </row>
+    <row r="1021">
+      <c r="A1021" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B1021" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C1021" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1021" s="3" t="inlineStr">
+        <is>
+          <t>[surff] 20260724 경제·물류 주요뉴스 (데일리스크랩)</t>
+        </is>
+      </c>
+      <c r="E1021" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 긴장에도 해상 운임(SCFI)이 하락세를 보였으나, 해운업계의 시선이 홍해로 옮겨가며 지정학적 리스크에 따른 운임 변동성이 커질 수 있다.</t>
+        </is>
+      </c>
+      <c r="F1021" s="3" t="inlineStr">
+        <is>
+          <t>해상 운임의 변동성과 주요 해협의 지정학적 리스크는 우리 회사의 해상 운송 비용 및 리드타임에 잠재적 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G1021" s="3" t="inlineStr">
+        <is>
+          <t>주요 해상 운임 지수(SCFI, CCFI) 및 유가 추이를 면밀히 모니터링하고, 홍해, 호르무즈 등 주요 해협의 지정학적 상황 변화에 대한 비상 계획을 수립해야 한다.</t>
+        </is>
+      </c>
+      <c r="H1021" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I1021" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260724-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J1021" s="3" t="inlineStr"/>
+    </row>
+    <row r="1022">
+      <c r="A1022" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B1022" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C1022" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1022" s="3" t="inlineStr">
+        <is>
+          <t>[surff] Vol133. 주간 선사별 동향 (Week 30, 2026) (주간 선사 동향)</t>
+        </is>
+      </c>
+      <c r="E1022" s="3" t="inlineStr">
+        <is>
+          <t>머스크가 수에즈운하 경유 노선을 확대하고 북유럽-미국, 아시아-인도 등 다수 항로에 성수기 할증료(PSS) 인상을 발표했다.</t>
+        </is>
+      </c>
+      <c r="F1022" s="3" t="inlineStr">
+        <is>
+          <t>주요 선사의 특정 항로 할증료 인상은 해당 노선을 이용하는 우리 회사의 운송 비용에 직접적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G1022" s="3" t="inlineStr">
+        <is>
+          <t>머스크를 포함한 주요 선사들의 운임 및 할증료 인상 공지를 주시하고, 해당 노선 이용 시 운송 비용 변화를 예측하여 운송 계획 및 예산에 반영해야 한다.</t>
+        </is>
+      </c>
+      <c r="H1022" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I1022" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/vol133-주간-선사별-동향-week-30-2026</t>
+        </is>
+      </c>
+      <c r="J1022" s="3" t="inlineStr"/>
+    </row>
+    <row r="1023">
+      <c r="A1023" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B1023" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C1023" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1023" s="3" t="inlineStr">
+        <is>
+          <t>[surff] 20260722 경제·물류 주요뉴스 (데일리스크랩)</t>
+        </is>
+      </c>
+      <c r="E1023" s="3" t="inlineStr">
+        <is>
+          <t>인천 서구 쿠팡 물류센터에서 대형 화재가 발생하여 진화에 어려움을 겪었으며, 빽빽한 구조가 진화를 방해했다는 분석이 나왔다.</t>
+        </is>
+      </c>
+      <c r="F1023" s="3" t="inlineStr">
+        <is>
+          <t>대형 물류센터 화재는 물류창고 안전 규제 강화 논의로 이어질 수 있으며, 이는 우리 회사의 물류센터 운영 및 보관 비용에 잠재적 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G1023" s="3" t="inlineStr">
+        <is>
+          <t>물류센터 화재 관련 조사 결과 및 향후 안전 규제 강화 동향을 주시하고, 우리 물류센터의 화재 예방 및 비상 대응 시스템을 점검하여 개선 방안을 모색해야 한다.</t>
+        </is>
+      </c>
+      <c r="H1023" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I1023" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260722-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J1023" s="3" t="inlineStr"/>
+    </row>
+    <row r="1024">
+      <c r="A1024" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B1024" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C1024" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1024" s="3" t="inlineStr">
+        <is>
+          <t>물류센터 화재 때마다 도마 에오르는 ‘메자닌 구조’... 정부는 설치 현황도 모른다</t>
+        </is>
+      </c>
+      <c r="E1024" s="3" t="inlineStr">
+        <is>
+          <t>물류센터 화재 시 복층 적재 구조인 메자닌의 안전성 논란이 지속되지만, 정부는 설치 현황조차 파악하지 못하고 있어 규제 사각지대에 놓여있다.</t>
+        </is>
+      </c>
+      <c r="F1024" s="3" t="inlineStr">
+        <is>
+          <t>물류센터 화재 안전 규제 강화 논의는 향후 물류센터 설계 및 운영 방식에 영향을 미칠 수 있으므로 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G1024" s="3" t="n"/>
+      <c r="H1024" s="3" t="inlineStr">
+        <is>
+          <t>인사이트</t>
+        </is>
+      </c>
+      <c r="I1024" s="3" t="inlineStr">
+        <is>
+          <t>https://www.insight.co.kr/news/564327</t>
+        </is>
+      </c>
+      <c r="J1024" s="3" t="inlineStr"/>
+    </row>
+    <row r="1025">
+      <c r="A1025" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B1025" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C1025" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1025" s="3" t="inlineStr">
+        <is>
+          <t>동해·묵호항 물동량 3.6% 증가…동해해수청, 위험물 안전관리와 항만 경쟁력 강화 '두 축' 추진</t>
+        </is>
+      </c>
+      <c r="E1025" s="3" t="inlineStr">
+        <is>
+          <t>동해·묵호항의 물동량이 증가하는 가운데, 동해해양수산청이 위험물 안전관리와 항만 경쟁력 강화를 동시에 추진하고 있다.</t>
+        </is>
+      </c>
+      <c r="F1025" s="3" t="inlineStr">
+        <is>
+          <t>국내 항만의 위험물 안전관리 강화는 향후 위험물 운송 절차 및 비용에 영향을 미칠 수 있으므로 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G1025" s="3" t="n"/>
+      <c r="H1025" s="3" t="inlineStr">
+        <is>
+          <t>아주경제</t>
+        </is>
+      </c>
+      <c r="I1025" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ajunews.com/view/20260723145153185</t>
+        </is>
+      </c>
+      <c r="J1025" s="3" t="inlineStr"/>
+    </row>
+    <row r="1026">
+      <c r="A1026" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B1026" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1026" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1026" s="3" t="inlineStr">
+        <is>
+          <t>中상무부 "미중, '관세 인하' 의견 수렴 중…조속 시행"</t>
+        </is>
+      </c>
+      <c r="E1026" s="3" t="inlineStr">
+        <is>
+          <t>미중 양국이 300억 달러 규모의 관세 인하에 대해 의견을 수렴 중이며 조속한 시행을 기대하고 있다.</t>
+        </is>
+      </c>
+      <c r="F1026" s="3" t="inlineStr">
+        <is>
+          <t>미중 관세 인하는 우리 회사의 대중국 수출입 비용에 긍정적인 영향을 미칠 수 있으므로 진행 상황을 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G1026" s="3" t="n"/>
+      <c r="H1026" s="3" t="inlineStr">
+        <is>
+          <t>연합뉴스</t>
+        </is>
+      </c>
+      <c r="I1026" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20260723177100089</t>
+        </is>
+      </c>
+      <c r="J1026" s="3" t="inlineStr"/>
+    </row>
+    <row r="1027">
+      <c r="A1027" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B1027" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1027" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1027" s="3" t="inlineStr">
+        <is>
+          <t>정의는 공급망을 바로 세우는 데서 시작된다 - 오마이뉴스</t>
+        </is>
+      </c>
+      <c r="E1027" s="3" t="inlineStr">
+        <is>
+          <t>아프리카와 아시아 일부 국가에서 불법 벌목된 목재가 국경을 넘어 합법적으로 세탁되어 수출되는 사례를 통해 공급망 투명성의 중요성을 강조한다.</t>
+        </is>
+      </c>
+      <c r="F1027" s="3" t="inlineStr">
+        <is>
+          <t>강제노동 관세와 유사하게 공급망 내 윤리적, 환경적 이슈는 향후 규제 강화로 이어질 수 있으며, 우리 회사의 공급망 투명성 및 ESG 경영 측면에서 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G1027" s="3" t="inlineStr">
+        <is>
+          <t>공급망 내 원자재 조달 과정의 투명성 및 윤리적 기준 준수 여부 점검, ESG 리스크 관리 강화.</t>
+        </is>
+      </c>
+      <c r="H1027" s="3" t="inlineStr">
+        <is>
+          <t>오마이뉴스</t>
+        </is>
+      </c>
+      <c r="I1027" s="3" t="inlineStr">
+        <is>
+          <t>https://ohmynews.com/NWS_Web/View/at_pg.aspx?CNTN_CD=A0003253607</t>
+        </is>
+      </c>
+      <c r="J1027" s="3" t="inlineStr"/>
+    </row>
+    <row r="1028">
+      <c r="A1028" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B1028" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C1028" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1028" s="3" t="inlineStr">
+        <is>
+          <t>중동 리스크로 운임 ↑…해운업계, 2분기 `호실적` 전망 - 디지털데일리</t>
+        </is>
+      </c>
+      <c r="E1028" s="3" t="inlineStr">
+        <is>
+          <t>중동 지정학적 리스크로 인한 해상운임 상승으로 국내 해운업계가 2분기 호실적을 거둘 것으로 전망된다.</t>
+        </is>
+      </c>
+      <c r="F1028" s="3" t="inlineStr">
+        <is>
+          <t>중동 리스크로 인한 해상운임 상승은 우리 회사의 물류 비용 증가로 이어질 수 있으므로, 운임 추이를 지속적으로 모니터링하고 운송 계약 전략을 검토해야 한다.</t>
+        </is>
+      </c>
+      <c r="G1028" s="3" t="inlineStr">
+        <is>
+          <t>해상운임 변동 추이 모니터링, 장기 운송 계약 조건 재검토, 대체 운송 경로 및 방식 검토.</t>
+        </is>
+      </c>
+      <c r="H1028" s="3" t="inlineStr">
+        <is>
+          <t>디지털데일리</t>
+        </is>
+      </c>
+      <c r="I1028" s="3" t="inlineStr">
+        <is>
+          <t>https://ddaily.co.kr/page/view/2026072215373082351</t>
+        </is>
+      </c>
+      <c r="J1028" s="3" t="inlineStr"/>
+    </row>
+    <row r="1029">
+      <c r="A1029" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B1029" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C1029" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1029" s="3" t="inlineStr">
+        <is>
+          <t>베트남 휘발유·경유 가격, 국제 유가 상승으로 리터당 880~2,440 동 인상</t>
+        </is>
+      </c>
+      <c r="E1029" s="3" t="inlineStr">
+        <is>
+          <t>미국-이란 갈등 고조와 후티 반군의 홍해 봉쇄 선언으로 국제 유가가 상승함에 따라 베트남의 휘발유 및 경유 가격이 인상되었다.</t>
+        </is>
+      </c>
+      <c r="F1029" s="3" t="inlineStr">
+        <is>
+          <t>국제유가 상승으로 인한 베트남 내 연료 가격 인상은 베트남 현지 물류 비용(육상 운송 등)에 영향을 줄 수 있으므로, 현지 물류 운영에 대한 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G1029" s="3" t="inlineStr">
+        <is>
+          <t>베트남 현지 물류 파트너와 비용 변동 논의, 현지 운송 비용 증가분 분석.</t>
+        </is>
+      </c>
+      <c r="H1029" s="3" t="inlineStr">
+        <is>
+          <t>굿모닝베트남미디어</t>
+        </is>
+      </c>
+      <c r="I1029" s="3" t="inlineStr">
+        <is>
+          <t>https://www.goodmorningvietnam.co.kr/news/article.html?no=82771</t>
+        </is>
+      </c>
+      <c r="J1029" s="3" t="inlineStr"/>
+    </row>
+    <row r="1030">
+      <c r="A1030" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B1030" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C1030" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D1030" s="4" t="inlineStr">
+        <is>
+          <t>Global Schedule Reliability for May 2026 the Highest of the Year</t>
+        </is>
+      </c>
+      <c r="E1030" s="4" t="inlineStr">
+        <is>
+          <t>2026년 5월 글로벌 컨테이너 해운의 스케줄 신뢰도가 올해 최고치를 기록했습니다.</t>
+        </is>
+      </c>
+      <c r="F1030" s="4" t="inlineStr">
+        <is>
+          <t>스케줄 신뢰도 향상은 긍정적인 추세이지만, 한 달간의 데이터만으로는 지속적인 개선을 보장하거나 즉각적인 조치를 요구하지 않습니다.</t>
+        </is>
+      </c>
+      <c r="G1030" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H1030" s="4" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I1030" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/395-global-schedule-reliability-for-may-2026-the-highest-of-the-year</t>
+        </is>
+      </c>
+      <c r="J1030" s="4" t="inlineStr"/>
+    </row>
+    <row r="1031">
+      <c r="A1031" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B1031" s="4" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1031" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D1031" s="4" t="inlineStr">
+        <is>
+          <t>EU, 그리스 해운사에 러 가스 수송 허용 예정</t>
+        </is>
+      </c>
+      <c r="E1031" s="4" t="inlineStr">
+        <is>
+          <t>유럽연합(EU)이 러시아에 대한 신규 제재를 추진하면서도 EU 기업들이 러시아산 액화천연가스(LNG)를 제3국으로 수송하는 것을 허용할 예정이다.</t>
+        </is>
+      </c>
+      <c r="F1031" s="4" t="inlineStr">
+        <is>
+          <t>러시아 LNG 수송 관련 뉴스로, 우리 회사의 배터리/전자부품 물류 운영에 직접적인 영향이 없다.</t>
+        </is>
+      </c>
+      <c r="G1031" s="4" t="n"/>
+      <c r="H1031" s="4" t="inlineStr">
+        <is>
+          <t>연합뉴스</t>
+        </is>
+      </c>
+      <c r="I1031" s="4" t="inlineStr">
+        <is>
+          <t>https://yna.co.kr/view/AKR20260723092800009</t>
+        </is>
+      </c>
+      <c r="J1031" s="4" t="inlineStr"/>
+    </row>
+    <row r="1032">
+      <c r="A1032" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B1032" s="4" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1032" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D1032" s="4" t="inlineStr">
+        <is>
+          <t>[쇼츠] 우크라, 러 최대 유통업체 물류창고 또 공격</t>
+        </is>
+      </c>
+      <c r="E1032" s="4" t="inlineStr">
+        <is>
+          <t>우크라이나가 러시아 최대 유통업체 와일드베리스의 물류창고를 또다시 공격했다는 소식.</t>
+        </is>
+      </c>
+      <c r="F1032" s="4" t="inlineStr">
+        <is>
+          <t>러시아-우크라이나 전쟁 관련 뉴스로, 우리 회사의 주요 물류 경로 및 운영에 직접적인 영향이 없다.</t>
+        </is>
+      </c>
+      <c r="G1032" s="4" t="n"/>
+      <c r="H1032" s="4" t="inlineStr">
+        <is>
+          <t>연합뉴스</t>
+        </is>
+      </c>
+      <c r="I1032" s="4" t="inlineStr">
+        <is>
+          <t>https://yna.co.kr/view/AKR20260723102900704</t>
+        </is>
+      </c>
+      <c r="J1032" s="4" t="inlineStr"/>
+    </row>
+    <row r="1033">
+      <c r="A1033" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B1033" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C1033" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D1033" s="4" t="inlineStr">
+        <is>
+          <t>정부, 공직자 소극행정·혐오표현 징계기준 강화</t>
+        </is>
+      </c>
+      <c r="E1033" s="4" t="inlineStr">
+        <is>
+          <t>정부가 공직자의 직무태만이나 소극행정 등 정당한 이유 없이 업무를 처리하지 않는 행위에 대한 징계 기준을 강화할 예정이다.</t>
+        </is>
+      </c>
+      <c r="F1033" s="4" t="inlineStr">
+        <is>
+          <t>공직자 징계 기준 강화는 우리 회사의 물류 운영에 직접적인 영향이 없다.</t>
+        </is>
+      </c>
+      <c r="G1033" s="4" t="n"/>
+      <c r="H1033" s="4" t="inlineStr">
+        <is>
+          <t>연합뉴스</t>
+        </is>
+      </c>
+      <c r="I1033" s="4" t="inlineStr">
+        <is>
+          <t>https://yna.co.kr/view/AKR20260723035700001</t>
+        </is>
+      </c>
+      <c r="J1033" s="4" t="inlineStr"/>
+    </row>
+    <row r="1034">
+      <c r="A1034" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B1034" s="4" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1034" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D1034" s="4" t="inlineStr">
+        <is>
+          <t>LG에너지솔루션, 미국서 中 EVE에너지 상대 특허소송 - 이투데이</t>
+        </is>
+      </c>
+      <c r="E1034" s="4" t="inlineStr">
+        <is>
+          <t>LG에너지솔루션이 중국 배터리 기업 EVE에너지를 상대로 미국에서 특허침해소송을 제기했다.</t>
+        </is>
+      </c>
+      <c r="F1034" s="4" t="inlineStr">
+        <is>
+          <t>경쟁사 간의 특허 소송은 우리 회사의 직접적인 물류 운영에 당장 영향을 미치지 않으며, 시장 경쟁 구도 변화는 장기적인 관점에서 모니터링할 사안이다.</t>
+        </is>
+      </c>
+      <c r="G1034" s="4" t="n"/>
+      <c r="H1034" s="4" t="inlineStr">
+        <is>
+          <t>이투데이</t>
+        </is>
+      </c>
+      <c r="I1034" s="4" t="inlineStr">
+        <is>
+          <t>https://etoday.co.kr/news/view/2606525</t>
+        </is>
+      </c>
+      <c r="J1034" s="4" t="inlineStr"/>
+    </row>
+    <row r="1035">
+      <c r="A1035" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B1035" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C1035" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D1035" s="4" t="inlineStr">
+        <is>
+          <t>재경부, 런던·싱가포르서 투자설명회…글로벌 협의체 가동 계획 | 연합뉴스</t>
+        </is>
+      </c>
+      <c r="E1035" s="4" t="inlineStr">
+        <is>
+          <t>정부가 글로벌 투자자와 국내 유관기관이 참여하는 '글로벌 핵심 투자자 협의체'를 가동하고 런던, 싱가포르에서 투자설명회를 개최할 계획이다.</t>
+        </is>
+      </c>
+      <c r="F1035" s="4" t="inlineStr">
+        <is>
+          <t>정부의 투자 유치 활동은 거시 경제 환경에 긍정적 영향을 줄 수 있으나, 우리 회사의 물류 운영에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G1035" s="4" t="n"/>
+      <c r="H1035" s="4" t="inlineStr">
+        <is>
+          <t>연합뉴스</t>
+        </is>
+      </c>
+      <c r="I1035" s="4" t="inlineStr">
+        <is>
+          <t>https://yna.co.kr/view/AKR20260723115100002</t>
+        </is>
+      </c>
+      <c r="J1035" s="4" t="inlineStr"/>
+    </row>
+    <row r="1036">
+      <c r="A1036" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B1036" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C1036" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D1036" s="4" t="inlineStr">
+        <is>
+          <t>[기획∙한중교류] 中∙韓 잇는 '황금 해상 통로'...단둥~인천 항로, 양국 교류 확대 견인 &lt; 국제 &lt; 기사본문 - 동방일보</t>
+        </is>
+      </c>
+      <c r="E1036" s="4" t="inlineStr">
+        <is>
+          <t>단둥-인천 국제 여객·화물선 항로의 이용객 및 운항 횟수가 증가하며 한중 교류 확대에 기여하고 있다.</t>
+        </is>
+      </c>
+      <c r="F1036" s="4" t="inlineStr">
+        <is>
+          <t>특정 항로의 활성화 소식은 긍정적이나, 우리 회사의 주요 물류 경로와 직접적인 관련이 없으며 운임 변동 등 즉각적인 물류 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G1036" s="4" t="n"/>
+      <c r="H1036" s="4" t="inlineStr">
+        <is>
+          <t>동방일보</t>
+        </is>
+      </c>
+      <c r="I1036" s="4" t="inlineStr">
+        <is>
+          <t>https://dongbangilbo.co.kr/news/articleView.html?idxno=98837</t>
+        </is>
+      </c>
+      <c r="J1036" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -48130,7 +49518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -49152,6 +50540,49 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>3080.31</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>-105 (-3.3%)</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>+1,317 (+74.7%)</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="n">
+        <v>4204</v>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>-114 (-2.6%)</t>
+        </is>
+      </c>
+      <c r="I25" s="5" t="inlineStr">
+        <is>
+          <t>+1,755 (+71.7%)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -49164,7 +50595,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I186"/>
+  <dimension ref="A1:I194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -55700,6 +57131,286 @@
       </c>
       <c r="I186" s="6" t="inlineStr"/>
     </row>
+    <row r="187">
+      <c r="A187" s="6" t="inlineStr">
+        <is>
+          <t>RSK-186</t>
+        </is>
+      </c>
+      <c r="B187" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C187" s="6" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="D187" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E187" s="6" t="inlineStr">
+        <is>
+          <t>파나마 운하 관리청, ‘3차 기간’ 슬롯경매 일시중단</t>
+        </is>
+      </c>
+      <c r="F187" s="6" t="inlineStr"/>
+      <c r="G187" s="6" t="inlineStr"/>
+      <c r="H187" s="6" t="inlineStr">
+        <is>
+          <t>파나마 운하를 이용하는 현재 및 계획된 선적을 평가하고, 대체 경로(예: 수에즈 운하, 철도, 복합운송)를 모색하며, 잠재적 지연을 내부 이해관계자에게 전달해야 합니다.</t>
+        </is>
+      </c>
+      <c r="I187" s="6" t="inlineStr"/>
+    </row>
+    <row r="188">
+      <c r="A188" s="6" t="inlineStr">
+        <is>
+          <t>RSK-187</t>
+        </is>
+      </c>
+      <c r="B188" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C188" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D188" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E188" s="6" t="inlineStr">
+        <is>
+          <t>“돌아가면 30일, 얀부 막히면 그마저도 못한다”</t>
+        </is>
+      </c>
+      <c r="F188" s="6" t="inlineStr"/>
+      <c r="G188" s="6" t="inlineStr"/>
+      <c r="H188" s="6" t="inlineStr">
+        <is>
+          <t>홍해 지역을 통과하거나 영향을 받을 수 있는 모든 선적을 검토하고, 대체 경로를 평가하며, 유가 변동을 모니터링하고, 잠재적 혼란에 대비한 비상 계획을 수립해야 합니다.</t>
+        </is>
+      </c>
+      <c r="I188" s="6" t="inlineStr"/>
+    </row>
+    <row r="189">
+      <c r="A189" s="6" t="inlineStr">
+        <is>
+          <t>RSK-188</t>
+        </is>
+      </c>
+      <c r="B189" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C189" s="6" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="D189" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E189" s="6" t="inlineStr">
+        <is>
+          <t>[해양통신] 머스크, 우크라이나 초르노모르스크항 기항 중단</t>
+        </is>
+      </c>
+      <c r="F189" s="6" t="inlineStr"/>
+      <c r="G189" s="6" t="inlineStr"/>
+      <c r="H189" s="6" t="inlineStr">
+        <is>
+          <t>흑해 지역을 경유하는 운송 경로가 있는지 즉시 확인하고, 해당 지역으로의 운송이 필요한 경우 대체 경로 및 운송 수단을 긴급히 검토해야 한다.</t>
+        </is>
+      </c>
+      <c r="I189" s="6" t="inlineStr"/>
+    </row>
+    <row r="190">
+      <c r="A190" s="6" t="inlineStr">
+        <is>
+          <t>RSK-189</t>
+        </is>
+      </c>
+      <c r="B190" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C190" s="6" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="D190" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E190" s="6" t="inlineStr">
+        <is>
+          <t>61시간 사투가 남긴 경고...물류 로봇 ‘리튬 배터리’ 화재 취약성[스마트 물류의 그늘]</t>
+        </is>
+      </c>
+      <c r="F190" s="6" t="inlineStr"/>
+      <c r="G190" s="6" t="inlineStr"/>
+      <c r="H190" s="6" t="inlineStr">
+        <is>
+          <t>물류센터 내 배터리 보관 및 취급 안전 절차 전면 재검토, 관련 법규 및 규제 동향 상시 모니터링, 비상 대응 계획 강화.</t>
+        </is>
+      </c>
+      <c r="I190" s="6" t="inlineStr"/>
+    </row>
+    <row r="191">
+      <c r="A191" s="6" t="inlineStr">
+        <is>
+          <t>RSK-190</t>
+        </is>
+      </c>
+      <c r="B191" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C191" s="6" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="D191" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E191" s="6" t="inlineStr">
+        <is>
+          <t>[사회]쿠팡 물류센터 화재 109시간 만에 완진...다른 센터에 또 불</t>
+        </is>
+      </c>
+      <c r="F191" s="6" t="inlineStr"/>
+      <c r="G191" s="6" t="inlineStr"/>
+      <c r="H191" s="6" t="inlineStr">
+        <is>
+          <t>물류센터 내 화재 예방 및 진압 시스템 점검, 비상 대응 계획 재검토, 배터리 보관 시설 안전성 강화 방안 모색.</t>
+        </is>
+      </c>
+      <c r="I191" s="6" t="inlineStr"/>
+    </row>
+    <row r="192">
+      <c r="A192" s="6" t="inlineStr">
+        <is>
+          <t>RSK-191</t>
+        </is>
+      </c>
+      <c r="B192" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C192" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D192" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E192" s="6" t="inlineStr">
+        <is>
+          <t>[속보] 미국 USTR, 무역법 301조 '강제노동 관세' 부과</t>
+        </is>
+      </c>
+      <c r="F192" s="6" t="inlineStr"/>
+      <c r="G192" s="6" t="inlineStr"/>
+      <c r="H192" s="6" t="inlineStr">
+        <is>
+          <t>공급망 내 강제노동 관련 리스크 점검, 해당 관세 부과 대상 품목 및 지역 확인, 공급망 다변화 또는 대체 소싱 방안 검토.</t>
+        </is>
+      </c>
+      <c r="I192" s="6" t="inlineStr"/>
+    </row>
+    <row r="193">
+      <c r="A193" s="6" t="inlineStr">
+        <is>
+          <t>RSK-192</t>
+        </is>
+      </c>
+      <c r="B193" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C193" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D193" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E193" s="6" t="inlineStr">
+        <is>
+          <t>트럼프 '관세 재건'…韓 강제노동 12.5%에 남은 '2.5%p'에 협상 성패 달렸다</t>
+        </is>
+      </c>
+      <c r="F193" s="6" t="inlineStr"/>
+      <c r="G193" s="6" t="inlineStr"/>
+      <c r="H193" s="6" t="inlineStr">
+        <is>
+          <t>대미 수출 제품의 원산지 증명 및 공급망 내 강제노동 리스크 점검 강화, 관세 부과 시나리오별 비용 분석 및 대응 방안 마련.</t>
+        </is>
+      </c>
+      <c r="I193" s="6" t="inlineStr"/>
+    </row>
+    <row r="194">
+      <c r="A194" s="6" t="inlineStr">
+        <is>
+          <t>RSK-193</t>
+        </is>
+      </c>
+      <c r="B194" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C194" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D194" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E194" s="6" t="inlineStr">
+        <is>
+          <t>[속보] 브렌트유 배럴당 100달러 재돌파…5월 26일 이후 처음 - 매일경제</t>
+        </is>
+      </c>
+      <c r="F194" s="6" t="inlineStr"/>
+      <c r="G194" s="6" t="inlineStr"/>
+      <c r="H194" s="6" t="inlineStr">
+        <is>
+          <t>유가 변동에 따른 물류비용 증가분 분석, 운송 계약 조건 재검토, 연료 효율 개선 방안 모색, 비상 운송 계획 수립.</t>
+        </is>
+      </c>
+      <c r="I194" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
📰 뉴스 데이터 2026-07-27_09:01
</commit_message>
<xml_diff>
--- a/data/SCM_물류_브리핑.xlsx
+++ b/data/SCM_물류_브리핑.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1036"/>
+  <dimension ref="A1:J1074"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -49506,6 +49506,1818 @@
       </c>
       <c r="J1036" s="4" t="inlineStr"/>
     </row>
+    <row r="1037">
+      <c r="A1037" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B1037" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1037" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D1037" s="2" t="inlineStr">
+        <is>
+          <t>Section 122 Tariffs' July 24 Expiration Thrown Into Doubt as U.S. Appeals CIT Ruling; Strait of Hormuz Reverts to War Conditions, Transits Down 66%</t>
+        </is>
+      </c>
+      <c r="E1037" s="2" t="inlineStr">
+        <is>
+          <t>미국이 Section 122 관세 만료에 대한 항소를 제기하여 관세 불확실성이 커지고 있으며, 호르무즈 해협이 전쟁 상황으로 회귀하여 통행량이 66% 감소했습니다.</t>
+        </is>
+      </c>
+      <c r="F1037" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협의 통행량 급감은 중동 발 물류에 즉각적인 차질을 야기하며, Section 122 관세의 불확실성은 무역 비용에 직접적인 영향을 미칠 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G1037" s="2" t="inlineStr">
+        <is>
+          <t>중동 항로를 이용하는 물량에 대한 대체 운송 경로 및 운송사 확보 검토, 관세 관련 동향 지속 모니터링 및 필요 시 무역팀과 협의.</t>
+        </is>
+      </c>
+      <c r="H1037" s="2" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I1037" s="2" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/july-23-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J1037" s="2" t="inlineStr">
+        <is>
+          <t>RSK-194</t>
+        </is>
+      </c>
+    </row>
+    <row r="1038">
+      <c r="A1038" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B1038" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1038" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D1038" s="2" t="inlineStr">
+        <is>
+          <t>Section 301 Tariffs on Brazil Take Effect July 22, Stacking with Section 122 Duties; Strait of Hormuz Closure Restricts 200K TEU of Ocean Capacity</t>
+        </is>
+      </c>
+      <c r="E1038" s="2" t="inlineStr">
+        <is>
+          <t>브라질에 대한 Section 301 관세가 발효되고 러시아 제재 법안이 중국, 인도에 대한 2차 관세를 부과할 수 있으며, 호르무즈 해협 폐쇄로 20만 TEU의 해상 운송 역량이 제한됩니다.</t>
+        </is>
+      </c>
+      <c r="F1038" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 폐쇄는 중동 및 유럽 항로에 심각한 운송 지연과 비용 상승을 초래하며, 새로운 관세 부과는 무역 비용에 직접적인 영향을 미칩니다.</t>
+        </is>
+      </c>
+      <c r="G1038" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협을 경유하는 물량에 대한 비상 계획 수립, 대체 항로 및 운송 수단 검토, 브라질 및 러시아 관련 무역 정책 변화 모니터링 및 무역팀과 협의.</t>
+        </is>
+      </c>
+      <c r="H1038" s="2" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I1038" s="2" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/july-16-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J1038" s="2" t="inlineStr">
+        <is>
+          <t>RSK-195</t>
+        </is>
+      </c>
+    </row>
+    <row r="1039">
+      <c r="A1039" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B1039" s="2" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C1039" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D1039" s="2" t="inlineStr">
+        <is>
+          <t>CBP Rejects Warehouse Entries on CAPE Declarations, Risking IEEPA Refunds; TPEB Rates Climb as Panama Canal Restrictions Tighten Capacity</t>
+        </is>
+      </c>
+      <c r="E1039" s="2" t="inlineStr">
+        <is>
+          <t>CBP가 CAPE 신고에 대한 창고 입고를 거부하여 IEEPA 환급 위험이 발생하고 있으며, 파나마 운하 통행 제한으로 인해 태평양 횡단 동향(TPEB) 운임이 상승하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F1039" s="2" t="inlineStr">
+        <is>
+          <t>파나마 운하 통행 제한은 미주향 물류의 운송 지연과 운임 상승을 직접적으로 야기하며, CBP의 창고 입고 거부는 통관 및 비용에 영향을 줄 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G1039" s="2" t="inlineStr">
+        <is>
+          <t>파나마 운하를 이용하는 미주향 물량에 대한 운송 계획 재검토, 대체 경로 및 운송 수단(예: 철도, 육상) 고려, CBP 통관 절차 변화에 대한 무역팀과 협의 및 대응 방안 마련.</t>
+        </is>
+      </c>
+      <c r="H1039" s="2" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I1039" s="2" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/july-09-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J1039" s="2" t="inlineStr">
+        <is>
+          <t>RSK-196</t>
+        </is>
+      </c>
+    </row>
+    <row r="1040">
+      <c r="A1040" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B1040" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1040" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D1040" s="2" t="inlineStr">
+        <is>
+          <t>'꼼수 관세' 꺼낸 트럼프, 강제노동 관세 60개국 부과...한국 12.5%</t>
+        </is>
+      </c>
+      <c r="E1040" s="2" t="inlineStr">
+        <is>
+          <t>미국이 무역법 301조를 근거로 한국을 포함한 60개 교역국에 최대 12.5%의 강제노동 관세를 부과할 예정이며, 이는 한국 기업의 수출 비용에 직접적인 영향을 미칠 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="F1040" s="2" t="inlineStr">
+        <is>
+          <t>한국에 대한 12.5% 관세 부과는 우리 회사의 미국 수출 비용을 직접적으로 증가시키고 경쟁력에 영향을 줄 수 있으므로 즉각적인 대응이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G1040" s="2" t="inlineStr">
+        <is>
+          <t>무역팀과 협의하여 강제노동 관세 부과 대상 품목 및 적용 시기 확인, 관세 회피 또는 최소화 방안 검토 (예: 원산지 증명, 생산지 다변화).</t>
+        </is>
+      </c>
+      <c r="H1040" s="2" t="inlineStr">
+        <is>
+          <t>kita</t>
+        </is>
+      </c>
+      <c r="I1040" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kita.net/shippers/board/newsView.do?morgueCode=2&amp;dataCls=A&amp;dataSeq=2539</t>
+        </is>
+      </c>
+      <c r="J1040" s="2" t="inlineStr">
+        <is>
+          <t>RSK-197</t>
+        </is>
+      </c>
+    </row>
+    <row r="1041">
+      <c r="A1041" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B1041" s="2" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C1041" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D1041" s="2" t="inlineStr">
+        <is>
+          <t>중동 물류 혼란으로 항만 대기 및 내륙 운송비 급증, 인도 지연</t>
+        </is>
+      </c>
+      <c r="E1041" s="2" t="inlineStr">
+        <is>
+          <t>중동 지역의 물류 혼란으로 항만 대기 및 내륙 운송비가 급증하고, 최종 인도까지 한 달 이상 지연되는 사례가 증가하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F1041" s="2" t="inlineStr">
+        <is>
+          <t>중동 지역은 당사의 잠재적 또는 현재 시장일 수 있으며, 물류 지연 및 비용 증가는 해당 지역으로의 수출에 직접적인 타격을 줄 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G1041" s="2" t="inlineStr">
+        <is>
+          <t>중동향 물량의 운송 경로 및 리드타임 재검토, 대체 운송 수단 및 파트너사 협의, 고객사와의 납기 조율.</t>
+        </is>
+      </c>
+      <c r="H1041" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I1041" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260727-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J1041" s="2" t="inlineStr">
+        <is>
+          <t>RSK-198</t>
+        </is>
+      </c>
+    </row>
+    <row r="1042">
+      <c r="A1042" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B1042" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C1042" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D1042" s="2" t="inlineStr">
+        <is>
+          <t>유가 급등, 금리·관세·환율 변수 겹치며 대외무역 불확실성 확대</t>
+        </is>
+      </c>
+      <c r="E1042" s="2" t="inlineStr">
+        <is>
+          <t>유가 급등과 함께 금리, 관세, 환율 변수까지 겹치며 물가 및 대외 무역 불확실성이 확대되고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F1042" s="2" t="inlineStr">
+        <is>
+          <t>유가 급등은 직접적인 물류비 상승을 야기하며, 관세 및 환율 변동은 수출입 비용에 큰 영향을 미치므로 즉각적인 대응이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G1042" s="2" t="inlineStr">
+        <is>
+          <t>유가 및 환율 변동에 따른 물류비 및 원가 상승 시나리오 분석, 관세 변동 가능성 대비 수출입 전략 검토.</t>
+        </is>
+      </c>
+      <c r="H1042" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I1042" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260726-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J1042" s="2" t="inlineStr">
+        <is>
+          <t>RSK-199</t>
+        </is>
+      </c>
+    </row>
+    <row r="1043">
+      <c r="A1043" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B1043" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1043" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D1043" s="2" t="inlineStr">
+        <is>
+          <t>중국, EU 대러 제재 보복으로 유럽 기업 14곳 수출 통제</t>
+        </is>
+      </c>
+      <c r="E1043" s="2" t="inlineStr">
+        <is>
+          <t>중국이 EU의 대러 제재에 대한 보복으로 유럽 기업 14곳에 수출 통제를 가하며 중국과 유럽 간 무역 갈등이 격화되고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F1043" s="2" t="inlineStr">
+        <is>
+          <t>중국-EU 무역 갈등 심화 및 수출 통제는 해당 지역으로의 부품 조달 또는 완제품 수출에 직접적인 차질을 발생시킬 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G1043" s="2" t="inlineStr">
+        <is>
+          <t>중국 및 EU 지역 공급망 리스크 점검, 대체 공급처 및 시장 확보 방안 검토, 무역 분쟁 추이 모니터링.</t>
+        </is>
+      </c>
+      <c r="H1043" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I1043" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260726-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J1043" s="2" t="inlineStr">
+        <is>
+          <t>RSK-200</t>
+        </is>
+      </c>
+    </row>
+    <row r="1044">
+      <c r="A1044" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B1044" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1044" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D1044" s="2" t="inlineStr">
+        <is>
+          <t>미국 무역법 301조, 강제노동 관련 관세 12.5% 확정</t>
+        </is>
+      </c>
+      <c r="E1044" s="2" t="inlineStr">
+        <is>
+          <t>미국 무역법 301조 조사에서 강제노동 관련 관세 12.5%가 확정되었으며, 과잉생산 관련 관세 논의도 진행 중입니다.</t>
+        </is>
+      </c>
+      <c r="F1044" s="2" t="inlineStr">
+        <is>
+          <t>미국의 강제노동 관련 관세 부과는 해당 지역으로부터의 부품 조달 또는 완제품 수출에 직접적인 비용 상승을 야기할 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G1044" s="2" t="inlineStr">
+        <is>
+          <t>강제노동 관련 관세 적용 대상 품목 및 지역 확인, 공급망 내 강제노동 리스크 점검 및 대응 방안 마련.</t>
+        </is>
+      </c>
+      <c r="H1044" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I1044" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260725-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J1044" s="2" t="inlineStr">
+        <is>
+          <t>RSK-201</t>
+        </is>
+      </c>
+    </row>
+    <row r="1045">
+      <c r="A1045" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B1045" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1045" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D1045" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 이어 홍해까지…글로벌 공급망 '이중 봉쇄' 공포</t>
+        </is>
+      </c>
+      <c r="E1045" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협에 이어 홍해 항로마저 막힐 가능성이 커지면서 중동 원유 및 원자재 의존도가 높은 국내 산업계의 글로벌 공급망 '이중 봉쇄' 공포가 커지고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F1045" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 및 홍해 항로 봉쇄는 주요 해상 운송로의 마비를 의미하며, 이는 원자재 수급난과 운송 지연을 야기하여 당사의 생산 및 물류 운영에 치명적인 영향을 미칠 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G1045" s="2" t="inlineStr">
+        <is>
+          <t>중동 및 유럽향/발 물량의 운송 경로 및 리드타임 재검토, 대체 운송 수단 및 파트너사 협의, 비축 재고 수준 점검, 고객사와의 납기 조율.</t>
+        </is>
+      </c>
+      <c r="H1045" s="2" t="inlineStr">
+        <is>
+          <t>파이낸셜뉴스</t>
+        </is>
+      </c>
+      <c r="I1045" s="2" t="inlineStr">
+        <is>
+          <t>https://fnnews.com/news/202607251300396182</t>
+        </is>
+      </c>
+      <c r="J1045" s="2" t="inlineStr">
+        <is>
+          <t>RSK-202</t>
+        </is>
+      </c>
+    </row>
+    <row r="1046">
+      <c r="A1046" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B1046" s="2" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C1046" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D1046" s="2" t="inlineStr">
+        <is>
+          <t>미·이란 충돌에 뱃길 꽉 막힌 중동…코트라, 우회 물류비 최대 8400만원 쏜다</t>
+        </is>
+      </c>
+      <c r="E1046" s="2" t="inlineStr">
+        <is>
+          <t>미·이란 충돌로 인한 홍해 봉쇄로 중동 항만 물류 대란이 심화되고 있으며, 코트라가 우회 물류비 지원을 확대하여 기업들의 부담을 덜어주고 있다.</t>
+        </is>
+      </c>
+      <c r="F1046" s="2" t="inlineStr">
+        <is>
+          <t>홍해 봉쇄로 인한 중동 항만 적체 및 우회 항로 사용은 해상 운송 지연과 물류비 급증을 야기하여 우리 회사의 생산 및 물류 계획에 직접적인 영향을 미칠 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G1046" s="2" t="inlineStr">
+        <is>
+          <t>중동 및 유럽향/발 해상 운송 경로 및 리드타임 재검토, 대체 운송 수단 및 항로(예: 희망봉 우회, 항공 운송) 비용 및 가용성 분석, 코트라 지원 프로그램 활용 검토.</t>
+        </is>
+      </c>
+      <c r="H1046" s="2" t="inlineStr">
+        <is>
+          <t>매일경제</t>
+        </is>
+      </c>
+      <c r="I1046" s="2" t="inlineStr">
+        <is>
+          <t>https://mk.co.kr/news/business/12107600</t>
+        </is>
+      </c>
+      <c r="J1046" s="2" t="inlineStr">
+        <is>
+          <t>RSK-203</t>
+        </is>
+      </c>
+    </row>
+    <row r="1047">
+      <c r="A1047" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B1047" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C1047" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D1047" s="2" t="inlineStr">
+        <is>
+          <t>"바이어 뺏길라"...물류비 급등에도 수출기업 3곳 중 1곳 '비용 전가 0%'</t>
+        </is>
+      </c>
+      <c r="E1047" s="2" t="inlineStr">
+        <is>
+          <t>중동 전쟁 이후 국제 유가 상승으로 물류비 부담이 확대되었으나, 국내 수출기업 3곳 중 1곳은 바이어 이탈 우려로 늘어난 비용을 제품 가격에 전혀 반영하지 못하고 있다.</t>
+        </is>
+      </c>
+      <c r="F1047" s="2" t="inlineStr">
+        <is>
+          <t>국제 유가 상승으로 인한 물류비 급등은 우리 회사의 수출 수익성에 직접적인 악영향을 미치며, 경쟁력 유지를 위해 비용 전가 여부와 관계없이 물류 효율화가 시급합니다.</t>
+        </is>
+      </c>
+      <c r="G1047" s="2" t="inlineStr">
+        <is>
+          <t>운송 계약 재협상, 운송 모드 최적화(예: 해상/항공 운송 비율 조정), 물류 파트너와의 협력 강화, 물류비 절감 방안(예: 컨테이너 활용률 증대, 라우팅 최적화) 모색, 물류비 변동에 따른 가격 정책 유연성 검토.</t>
+        </is>
+      </c>
+      <c r="H1047" s="2" t="inlineStr">
+        <is>
+          <t>파이낸셜뉴스</t>
+        </is>
+      </c>
+      <c r="I1047" s="2" t="inlineStr">
+        <is>
+          <t>https://fnnews.com/news/202607261036055758</t>
+        </is>
+      </c>
+      <c r="J1047" s="2" t="inlineStr">
+        <is>
+          <t>RSK-204</t>
+        </is>
+      </c>
+    </row>
+    <row r="1048">
+      <c r="A1048" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B1048" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1048" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D1048" s="2" t="inlineStr">
+        <is>
+          <t>[기획]다시 불거진 관세리스크…수출기업 부담 커진다</t>
+        </is>
+      </c>
+      <c r="E1048" s="2" t="inlineStr">
+        <is>
+          <t>미국이 한국에 12.5%의 강제노동 관세를 적용하면서 국내 수출기업의 물류비 부담이 가중될 것으로 예상되며, 이는 기존 10% 글로벌 관세에 2.5%포인트가 추가되는 수준이다.</t>
+        </is>
+      </c>
+      <c r="F1048" s="2" t="inlineStr">
+        <is>
+          <t>우리 기업의 미국 수출 시 추가 관세가 부과되어 제품 가격 경쟁력 하락 및 물류비 부담이 직접적으로 증가할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G1048" s="2" t="inlineStr">
+        <is>
+          <t>미국 수출 품목에 대한 관세 영향 분석 및 가격 정책 재검토, 강제노동 관련 공급망 실사 강화.</t>
+        </is>
+      </c>
+      <c r="H1048" s="2" t="inlineStr">
+        <is>
+          <t>매일일보</t>
+        </is>
+      </c>
+      <c r="I1048" s="2" t="inlineStr">
+        <is>
+          <t>https://m-i.kr/news/articleView.html?idxno=1395028</t>
+        </is>
+      </c>
+      <c r="J1048" s="2" t="inlineStr">
+        <is>
+          <t>RSK-205</t>
+        </is>
+      </c>
+    </row>
+    <row r="1049">
+      <c r="A1049" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B1049" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C1049" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D1049" s="2" t="inlineStr">
+        <is>
+          <t>유가·운임 급등에 수출기업 '이중 부담'…물류비 쇼크 현실화</t>
+        </is>
+      </c>
+      <c r="E1049" s="2" t="inlineStr">
+        <is>
+          <t>중동 정세 불안으로 국제유가와 해상운임이 동반 상승하여 국내 수출기업의 물류비 부담이 크게 확대되고 있으며, 이는 물류비 쇼크로 이어질 수 있다.</t>
+        </is>
+      </c>
+      <c r="F1049" s="2" t="inlineStr">
+        <is>
+          <t>국제유가 및 해상운임 급등은 우리 기업의 물류비용을 직접적으로 증가시켜 수익성에 즉각적인 악영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G1049" s="2" t="inlineStr">
+        <is>
+          <t>운송 계약 조건 재검토, 대체 운송 수단 및 경로 검토, 물류비 상승분 제품 가격 반영 여부 논의, 유가 및 운임 변동성 모니터링 강화.</t>
+        </is>
+      </c>
+      <c r="H1049" s="2" t="inlineStr">
+        <is>
+          <t>이비엔(EBN)뉴스센터</t>
+        </is>
+      </c>
+      <c r="I1049" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ebn.co.kr/news/articleView.html?idxno=1717809</t>
+        </is>
+      </c>
+      <c r="J1049" s="2" t="inlineStr">
+        <is>
+          <t>RSK-206</t>
+        </is>
+      </c>
+    </row>
+    <row r="1050">
+      <c r="A1050" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B1050" s="2" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C1050" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D1050" s="2" t="inlineStr">
+        <is>
+          <t>“호르무즈 정상화 후에도 수출 물류 회복까지 6개월 이상 소요”</t>
+        </is>
+      </c>
+      <c r="E1050" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 통항 차질이 장기화되고 대체 항만 적체 및 홍해 해상 봉쇄 가능성까지 더해져, 수출 물류 회복까지 6개월 이상 상당한 시간이 소요될 것으로 전망된다.</t>
+        </is>
+      </c>
+      <c r="F1050" s="2" t="inlineStr">
+        <is>
+          <t>주요 해상 운송로의 장기적인 불안정은 우리 기업의 원자재 수급 및 완제품 수출에 심각한 지연을 초래하여 생산 및 판매 계획에 직접적인 차질을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="G1050" s="2" t="inlineStr">
+        <is>
+          <t>대체 운송 경로 및 운송 수단 확보 방안 검토, 재고 수준 조정, 고객 및 공급업체와 소통 강화, 비상 계획 수립.</t>
+        </is>
+      </c>
+      <c r="H1050" s="2" t="inlineStr">
+        <is>
+          <t>국민일보</t>
+        </is>
+      </c>
+      <c r="I1050" s="2" t="inlineStr">
+        <is>
+          <t>https://kmib.co.kr/article/view.asp?arcid=1785053911&amp;code=11151400&amp;sid1=eco</t>
+        </is>
+      </c>
+      <c r="J1050" s="2" t="inlineStr">
+        <is>
+          <t>RSK-207</t>
+        </is>
+      </c>
+    </row>
+    <row r="1051">
+      <c r="A1051" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B1051" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1051" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1051" s="3" t="inlineStr">
+        <is>
+          <t>U.S.-EU Trade Agreement Eliminates Duties on Most U.S. Goods Starting July 1; TPEB Rates Rise as July Capacity Hits Three-Year High</t>
+        </is>
+      </c>
+      <c r="E1051" s="3" t="inlineStr">
+        <is>
+          <t>미국-EU 무역 협정이 7월 1일부터 대부분의 미국산 제품에 대한 관세를 철폐했으며, 7월 운송 역량이 3년 만에 최고치를 기록했음에도 불구하고 태평양 횡단 동향(TPEB) 운임이 상승하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F1051" s="3" t="inlineStr">
+        <is>
+          <t>미국-EU 무역 협정은 장기적으로 관세 비용 절감 기회를 제공하지만, 당장 우리 회사의 물류 운영에 직접적인 영향을 주지는 않으며, TPEB 운임 상승은 지속적인 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G1051" s="3" t="inlineStr">
+        <is>
+          <t>미국-EU 무역 협정의 세부 내용을 검토하여 우리 제품에 대한 관세 혜택 여부 확인, TPEB 운임 추이 지속 모니터링 및 운송 계약 조건 검토.</t>
+        </is>
+      </c>
+      <c r="H1051" s="3" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I1051" s="3" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/july-02-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J1051" s="3" t="inlineStr"/>
+    </row>
+    <row r="1052">
+      <c r="A1052" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B1052" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C1052" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1052" s="3" t="inlineStr">
+        <is>
+          <t>Statement on EU Commission Revision of the EU Emissions Trading System</t>
+        </is>
+      </c>
+      <c r="E1052" s="3" t="inlineStr">
+        <is>
+          <t>IATA는 유럽연합 배출권 거래 시스템(EU ETS)의 유럽 외 확장 제안에 대해 깊은 우려를 표명하며, 이는 항공 운송 비용 증가로 이어질 수 있다고 밝혔습니다.</t>
+        </is>
+      </c>
+      <c r="F1052" s="3" t="inlineStr">
+        <is>
+          <t>EU ETS의 확장은 항공 운송 비용에 영향을 미칠 수 있으나, 아직 제안 단계이며 즉각적인 비용 상승으로 이어지지는 않으므로 추이를 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G1052" s="3" t="inlineStr">
+        <is>
+          <t>EU ETS 확장 논의 동향을 지속적으로 모니터링하고, 항공 운송 비용에 미칠 잠재적 영향 분석 및 필요 시 운송사와의 협의 준비.</t>
+        </is>
+      </c>
+      <c r="H1052" s="3" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I1052" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/07-17-statement-eu-commission-revision-emissions-trading-system/</t>
+        </is>
+      </c>
+      <c r="J1052" s="3" t="inlineStr"/>
+    </row>
+    <row r="1053">
+      <c r="A1053" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B1053" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C1053" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1053" s="3" t="inlineStr">
+        <is>
+          <t>현대글로비스, 中 제조기업 운송 물량 잇따라 수주</t>
+        </is>
+      </c>
+      <c r="E1053" s="3" t="inlineStr">
+        <is>
+          <t>현대글로비스가 중국 배터리 선도 기업 및 전기차 제조 기업과 잇따라 운송 계약을 체결하며, 중국에서 유럽으로의 전기차 배터리 해상 운송 물량을 확대하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F1053" s="3" t="inlineStr">
+        <is>
+          <t>주요 물류 기업이 배터리 운송 시장에서 경쟁력을 강화하고 있음을 보여주며, 이는 향후 운송 서비스 선택 및 계약 조건에 영향을 미칠 수 있으므로 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G1053" s="3" t="inlineStr">
+        <is>
+          <t>배터리 운송 시장의 경쟁 동향 및 주요 운송사의 서비스 포트폴리오 변화를 지속적으로 모니터링하고, 필요 시 현재 운송 파트너와의 계약 조건 재검토.</t>
+        </is>
+      </c>
+      <c r="H1053" s="3" t="inlineStr">
+        <is>
+          <t>oceanpress</t>
+        </is>
+      </c>
+      <c r="I1053" s="3" t="inlineStr">
+        <is>
+          <t>https://www.oceanpress.co.kr/news/article.html?no=30741</t>
+        </is>
+      </c>
+      <c r="J1053" s="3" t="inlineStr"/>
+    </row>
+    <row r="1054">
+      <c r="A1054" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B1054" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C1054" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1054" s="3" t="inlineStr">
+        <is>
+          <t>Structural Shift in Blank Sailing Strategies</t>
+        </is>
+      </c>
+      <c r="E1054" s="3" t="inlineStr">
+        <is>
+          <t>2026년 상반기 주요 동서항로에서 선박 결항(blank sailing)으로 인한 공급 감소가 전체 선복량 증가보다 빠르게 나타나, 선사들이 적극적으로 공급을 조절하고 있음을 보여줍니다.</t>
+        </is>
+      </c>
+      <c r="F1054" s="3" t="inlineStr">
+        <is>
+          <t>Blank sailing 증가는 선박 스케줄 불확실성을 높여 운송 지연을 유발할 수 있으므로 지속적인 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G1054" s="3" t="n"/>
+      <c r="H1054" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I1054" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/399-structural-shift-in-blank-sailing-strategies</t>
+        </is>
+      </c>
+      <c r="J1054" s="3" t="inlineStr"/>
+    </row>
+    <row r="1055">
+      <c r="A1055" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B1055" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C1055" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1055" s="3" t="inlineStr">
+        <is>
+          <t>Structural Contraction of Global Liner Networks (Service Frequencies)</t>
+        </is>
+      </c>
+      <c r="E1055" s="3" t="inlineStr">
+        <is>
+          <t>2012년 이후 글로벌 정기선 네트워크 분석 결과, 선사들이 지리적 범위는 유지하면서도 서비스 빈도를 조정하는 등 네트워크 관리 방식에 근본적인 변화가 있음을 보여줍니다.</t>
+        </is>
+      </c>
+      <c r="F1055" s="3" t="inlineStr">
+        <is>
+          <t>선사들의 서비스 빈도 조정은 운송 리드타임 및 스케줄 신뢰성에 영향을 줄 수 있으므로 주요 항로의 서비스 변화를 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G1055" s="3" t="n"/>
+      <c r="H1055" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I1055" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/397-structural-contraction-of-global-liner-networks</t>
+        </is>
+      </c>
+      <c r="J1055" s="3" t="inlineStr"/>
+    </row>
+    <row r="1056">
+      <c r="A1056" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B1056" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C1056" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1056" s="3" t="inlineStr">
+        <is>
+          <t>PLSCI Data Indicates Mega-Hub Retrenchment</t>
+        </is>
+      </c>
+      <c r="E1056" s="3" t="inlineStr">
+        <is>
+          <t>2026년 2분기 항만 정기선 연결성 지수(PLSCI) 분석 결과, 최근 네트워크 재조정이 메가 허브 항만의 연결성 변화를 나타내고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F1056" s="3" t="inlineStr">
+        <is>
+          <t>주요 허브 항만의 연결성 변화는 운송 경로 및 리드타임에 영향을 줄 수 있으므로, 당사 주요 수출입 항만의 연결성 변화를 주시해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G1056" s="3" t="n"/>
+      <c r="H1056" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I1056" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/396-plsci-data-indicates-mega-hub-retrenchment</t>
+        </is>
+      </c>
+      <c r="J1056" s="3" t="inlineStr"/>
+    </row>
+    <row r="1057">
+      <c r="A1057" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B1057" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C1057" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1057" s="3" t="inlineStr">
+        <is>
+          <t>SCFI 상승 및 유가 부담 회수 전망, 하반기 해운 실적 영향</t>
+        </is>
+      </c>
+      <c r="E1057" s="3" t="inlineStr">
+        <is>
+          <t>상하이컨테이너운임지수(SCFI) 상승과 유가 부담 회수 전망이 맞물려 하반기 컨테이너 관련 매출 및 물류 처리 실적에 긍정적 영향이 예상됩니다.</t>
+        </is>
+      </c>
+      <c r="F1057" s="3" t="inlineStr">
+        <is>
+          <t>SCFI 상승은 해상 운임 상승 압력으로 작용하여 당사의 물류비에 영향을 줄 수 있으므로 추이를 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G1057" s="3" t="n"/>
+      <c r="H1057" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I1057" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260726-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J1057" s="3" t="inlineStr"/>
+    </row>
+    <row r="1058">
+      <c r="A1058" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B1058" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C1058" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1058" s="3" t="inlineStr">
+        <is>
+          <t>운임지수 상승 등 외부 환경 호조, LX인터내셔널 실적 기대</t>
+        </is>
+      </c>
+      <c r="E1058" s="3" t="inlineStr">
+        <is>
+          <t>석탄 가격과 운임지수 상승 등 외부 환경 호조가 LX인터내셔널의 실적 개선 기대를 키우고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F1058" s="3" t="inlineStr">
+        <is>
+          <t>운임지수 상승은 해상 운임 상승 압력으로 작용하여 당사의 물류비에 영향을 줄 수 있으므로 추이를 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G1058" s="3" t="n"/>
+      <c r="H1058" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I1058" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260725-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J1058" s="3" t="inlineStr"/>
+    </row>
+    <row r="1059">
+      <c r="A1059" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B1059" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C1059" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1059" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 위기에도 해상운임 하락, 해운 시황 변화 주목</t>
+        </is>
+      </c>
+      <c r="E1059" s="3" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 긴장에도 불구하고 상하이컨테이너운임지수(SCFI)가 하락하여 해운 시황 변화가 주목됩니다.</t>
+        </is>
+      </c>
+      <c r="F1059" s="3" t="inlineStr">
+        <is>
+          <t>SCFI 하락은 단기적으로 긍정적이나, 지정학적 리스크와 상반되는 추세이므로 운임 변동성 확대 가능성을 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G1059" s="3" t="n"/>
+      <c r="H1059" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I1059" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260724-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J1059" s="3" t="inlineStr"/>
+    </row>
+    <row r="1060">
+      <c r="A1060" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B1060" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C1060" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1060" s="3" t="inlineStr">
+        <is>
+          <t>SCFI·CCFI 상승 및 관세 변경 전 선적 수요로 하반기 해운 시황 기대</t>
+        </is>
+      </c>
+      <c r="E1060" s="3" t="inlineStr">
+        <is>
+          <t>상하이컨테이너운임지수(SCFI) 및 컨테이너선운임지수(CCFI) 상승과 관세 변경 전 선적 수요 등으로 하반기 해운 시황에 대한 기대감이 커지고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F1060" s="3" t="inlineStr">
+        <is>
+          <t>운임지수 상승은 해상 운임 상승 압력으로 작용하여 당사의 물류비에 영향을 줄 수 있으므로 추이를 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G1060" s="3" t="n"/>
+      <c r="H1060" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I1060" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260724-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J1060" s="3" t="inlineStr"/>
+    </row>
+    <row r="1061">
+      <c r="A1061" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B1061" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C1061" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1061" s="3" t="inlineStr">
+        <is>
+          <t>中 조선소, 상반기 수주 173% 급증…"사실상 독주 체제"</t>
+        </is>
+      </c>
+      <c r="E1061" s="3" t="inlineStr">
+        <is>
+          <t>중국 조선업계가 2026년 상반기 역대 최대 규모의 신조선 주문을 확보하며 벌크선, 컨테이너선, 유조선 등 주요 선종 전반에서 수주가 급증했습니다.</t>
+        </is>
+      </c>
+      <c r="F1061" s="3" t="inlineStr">
+        <is>
+          <t>중국 조선소의 수주 급증은 장기적으로 선복량 증가로 이어져 운임 안정화에 기여할 수 있으나, 건조 기간을 고려할 때 단기적인 영향은 제한적입니다.</t>
+        </is>
+      </c>
+      <c r="G1061" s="3" t="n"/>
+      <c r="H1061" s="3" t="inlineStr">
+        <is>
+          <t>해양통신</t>
+        </is>
+      </c>
+      <c r="I1061" s="3" t="inlineStr">
+        <is>
+          <t>https://oceanpress.co.kr/news/article.html?no=30732</t>
+        </is>
+      </c>
+      <c r="J1061" s="3" t="inlineStr"/>
+    </row>
+    <row r="1062">
+      <c r="A1062" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B1062" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C1062" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1062" s="3" t="inlineStr">
+        <is>
+          <t>반복되는 창고 화재 "쿠팡만의 문제(?)"...최근 5년간 창고 화재건수 "7천300여건"</t>
+        </is>
+      </c>
+      <c r="E1062" s="3" t="inlineStr">
+        <is>
+          <t>인천 쿠팡 물류센터 화재를 계기로 물류센터 화재의 반복적인 발생과 이에 대한 안전 관리 시스템 및 규제 강화 필요성이 제기되고 있으며, 이는 물류 창고 운영에 대한 전반적인 재검토를 요구하고 있다.</t>
+        </is>
+      </c>
+      <c r="F1062" s="3" t="inlineStr">
+        <is>
+          <t>대형 물류센터 화재가 반복됨에 따라 향후 물류 창고의 안전 규제(특히 위험물 취급 관련)가 강화될 가능성이 높으며, 이는 우리 회사의 보관 및 물류 운영 비용과 절차에 영향을 줄 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G1062" s="3" t="inlineStr">
+        <is>
+          <t>국내외 물류센터 화재 관련 규제 동향 지속 모니터링, 현재 운영 중인 창고의 화재 안전 시스템 및 위험물 보관 규정 준수 여부 점검, 비상 계획 및 대응 훈련 강화.</t>
+        </is>
+      </c>
+      <c r="H1062" s="3" t="inlineStr">
+        <is>
+          <t>청년일보</t>
+        </is>
+      </c>
+      <c r="I1062" s="3" t="inlineStr">
+        <is>
+          <t>https://youthdaily.co.kr/news/article.html?no=223709</t>
+        </is>
+      </c>
+      <c r="J1062" s="3" t="inlineStr"/>
+    </row>
+    <row r="1063">
+      <c r="A1063" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B1063" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1063" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1063" s="3" t="inlineStr">
+        <is>
+          <t>美 무역법 '301조·232조'가 뭐길래…韓 산업 전방위 긴장</t>
+        </is>
+      </c>
+      <c r="E1063" s="3" t="inlineStr">
+        <is>
+          <t>미국이 무역법 301조를 근거로 한국산 제품에 관세를 부과하면서 국내 산업계의 긴장감이 고조되고 있으며, 이는 기존 232조에 이어 통상 압박 수단으로 활용되고 있다.</t>
+        </is>
+      </c>
+      <c r="F1063" s="3" t="inlineStr">
+        <is>
+          <t>미국 무역법 301조 및 232조 적용 확대는 한국산 배터리/전자부품에 대한 관세 부과로 이어질 수 있어, 대미 수출 가격 경쟁력 및 공급망 전략에 잠재적 영향을 미칠 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G1063" s="3" t="inlineStr">
+        <is>
+          <t>미국 무역법 관련 동향 및 한국산 배터리/전자부품에 대한 관세 부과 가능성 지속 모니터링, 관세 부과 시나리오별 대응 전략(예: 생산 기지 다변화, 가격 정책 조정) 사전 검토.</t>
+        </is>
+      </c>
+      <c r="H1063" s="3" t="inlineStr">
+        <is>
+          <t>ZDNet korea</t>
+        </is>
+      </c>
+      <c r="I1063" s="3" t="inlineStr">
+        <is>
+          <t>https://zdnet.co.kr/view/?no=20260724170832</t>
+        </is>
+      </c>
+      <c r="J1063" s="3" t="inlineStr"/>
+    </row>
+    <row r="1064">
+      <c r="A1064" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B1064" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1064" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1064" s="3" t="inlineStr">
+        <is>
+          <t>[분석] 기후가 무역을 바꾼다…GEPA 참여, 한국 통상전략의 새 전환점 될까</t>
+        </is>
+      </c>
+      <c r="E1064" s="3" t="inlineStr">
+        <is>
+          <t>세계 무역 질서의 중심축이 관세에서 기후로 이동함에 따라, 한국의 통상 전략도 기후 관련 무역 정책에 대한 참여를 통해 새로운 전환점을 맞이할 필요가 있다.</t>
+        </is>
+      </c>
+      <c r="F1064" s="3" t="inlineStr">
+        <is>
+          <t>기후 관련 무역 규제(예: 탄소국경조정제도)는 향후 우리 회사의 수출입 물류 비용 및 절차에 영향을 미칠 수 있으므로, 관련 정책 변화를 지속적으로 주시해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G1064" s="3" t="inlineStr">
+        <is>
+          <t>주요 수출 대상국의 기후 관련 무역 정책(예: EU 탄소국경조정제도) 동향 모니터링, 공급망 내 탄소 배출량 측정 및 관리 방안 검토, 친환경 물류 솔루션 도입 가능성 탐색.</t>
+        </is>
+      </c>
+      <c r="H1064" s="3" t="inlineStr">
+        <is>
+          <t>에너지데일리</t>
+        </is>
+      </c>
+      <c r="I1064" s="3" t="inlineStr">
+        <is>
+          <t>https://energydaily.co.kr/news/articleView.html?idxno=201740</t>
+        </is>
+      </c>
+      <c r="J1064" s="3" t="inlineStr"/>
+    </row>
+    <row r="1065">
+      <c r="A1065" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B1065" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1065" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1065" s="3" t="inlineStr">
+        <is>
+          <t>“트럼프 대체 관세, 기존 상호관세 손실분 60%도 대체 못 해”</t>
+        </is>
+      </c>
+      <c r="E1065" s="3" t="inlineStr">
+        <is>
+          <t>트럼프 전 대통령의 대체 관세 정책이 기존 상호 관세의 손실분을 충분히 대체하지 못할 것이라는 분석이 나오며, 이는 향후 미국의 통상 정책 변화에 대한 불확실성을 시사한다.</t>
+        </is>
+      </c>
+      <c r="F1065" s="3" t="inlineStr">
+        <is>
+          <t>트럼프 전 대통령의 대체 관세 정책은 향후 미국의 통상 정책 방향에 대한 불확실성을 높이며, 이는 우리 회사의 수출입 관세 및 공급망 전략에 잠재적 영향을 미칠 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G1065" s="3" t="inlineStr">
+        <is>
+          <t>미국 대선 결과 및 통상 정책 변화 동향 지속 모니터링, 다양한 관세 시나리오에 따른 공급망 리스크 분석 및 대응 방안(예: 생산 기지 다변화, 원산지 관리 강화) 사전 준비.</t>
+        </is>
+      </c>
+      <c r="H1065" s="3" t="inlineStr">
+        <is>
+          <t>이투데이</t>
+        </is>
+      </c>
+      <c r="I1065" s="3" t="inlineStr">
+        <is>
+          <t>https://etoday.co.kr/news/view/2607504</t>
+        </is>
+      </c>
+      <c r="J1065" s="3" t="inlineStr"/>
+    </row>
+    <row r="1066">
+      <c r="A1066" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B1066" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1066" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1066" s="3" t="inlineStr">
+        <is>
+          <t>[fn광장] 공급망 재편 시대, 한국의 생존 전략</t>
+        </is>
+      </c>
+      <c r="E1066" s="3" t="inlineStr">
+        <is>
+          <t>팬데믹과 미중 전략경쟁 등으로 인해 세계 경제의 패러다임이 효율 중심에서 공급망 안정 중심으로 재편되고 있으며, 이에 대한 한국의 생존 전략 마련이 중요해지고 있다.</t>
+        </is>
+      </c>
+      <c r="F1066" s="3" t="inlineStr">
+        <is>
+          <t>공급망 안정성 강화는 장기적인 관점에서 우리 기업의 물류 및 생산 전략에 중요한 영향을 미치므로, 관련 동향을 지속적으로 주시해야 한다.</t>
+        </is>
+      </c>
+      <c r="G1066" s="3" t="n"/>
+      <c r="H1066" s="3" t="inlineStr">
+        <is>
+          <t>파이낸셜뉴스</t>
+        </is>
+      </c>
+      <c r="I1066" s="3" t="inlineStr">
+        <is>
+          <t>https://fnnews.com/news/202607261827516230</t>
+        </is>
+      </c>
+      <c r="J1066" s="3" t="inlineStr"/>
+    </row>
+    <row r="1067">
+      <c r="A1067" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B1067" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C1067" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D1067" s="4" t="inlineStr">
+        <is>
+          <t>“2040년까지 반도체 장비물량 꽉 찼어요”</t>
+        </is>
+      </c>
+      <c r="E1067" s="4" t="inlineStr">
+        <is>
+          <t>팬스타그룹이 반도체 시장 활황에 힘입어 2040년까지 한일 간 반도체 장비 수송 물량을 확보했으며, 이는 고부가가치 산업 물류 수요 증가를 보여줍니다.</t>
+        </is>
+      </c>
+      <c r="F1067" s="4" t="inlineStr">
+        <is>
+          <t>반도체 장비 운송 계약은 우리 회사의 배터리/전자부품 물류에 직접적인 영향을 주지는 않지만, 고부가가치 산업 물류 시장의 전반적인 동향을 파악하는 데 참고할 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G1067" s="4" t="n"/>
+      <c r="H1067" s="4" t="inlineStr">
+        <is>
+          <t>ksg</t>
+        </is>
+      </c>
+      <c r="I1067" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksg.co.kr/news/main_newsView.jsp?pNum=147678</t>
+        </is>
+      </c>
+      <c r="J1067" s="4" t="inlineStr"/>
+    </row>
+    <row r="1068">
+      <c r="A1068" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B1068" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C1068" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D1068" s="4" t="inlineStr">
+        <is>
+          <t>Structural Contraction of Global Liner Networks (IMF Projections)</t>
+        </is>
+      </c>
+      <c r="E1068" s="4" t="inlineStr">
+        <is>
+          <t>IMF의 2026년 세계 경제 전망 보고서에 따르면 글로벌 무역량 성장률이 2025년 5.0%에서 2026년 3.5%로 크게 둔화될 것으로 예상됩니다.</t>
+        </is>
+      </c>
+      <c r="F1068" s="4" t="inlineStr">
+        <is>
+          <t>글로벌 무역량 성장 둔화는 장기적인 물류 수요에 영향을 미칠 수 있으나, 당사의 단기 물류 운영에 직접적인 영향은 낮습니다.</t>
+        </is>
+      </c>
+      <c r="G1068" s="4" t="n"/>
+      <c r="H1068" s="4" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I1068" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/398-structural-contraction-of-global-liner-network</t>
+        </is>
+      </c>
+      <c r="J1068" s="4" t="inlineStr"/>
+    </row>
+    <row r="1069">
+      <c r="A1069" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B1069" s="4" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C1069" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D1069" s="4" t="inlineStr">
+        <is>
+          <t>Global Schedule Reliability for May 2026 the Highest of the Year</t>
+        </is>
+      </c>
+      <c r="E1069" s="4" t="inlineStr">
+        <is>
+          <t>2026년 5월 글로벌 선박 스케줄 정시성이 올해 최고치를 기록했습니다.</t>
+        </is>
+      </c>
+      <c r="F1069" s="4" t="inlineStr">
+        <is>
+          <t>스케줄 정시성 개선은 긍정적인 신호이나, 단일 월 데이터이므로 장기적인 추세 변화를 판단하기에는 이릅니다.</t>
+        </is>
+      </c>
+      <c r="G1069" s="4" t="n"/>
+      <c r="H1069" s="4" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I1069" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/395-global-schedule-reliability-for-may-2026-the-highest-of-the-year</t>
+        </is>
+      </c>
+      <c r="J1069" s="4" t="inlineStr"/>
+    </row>
+    <row r="1070">
+      <c r="A1070" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B1070" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C1070" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D1070" s="4" t="inlineStr">
+        <is>
+          <t>현대글로비스, 중국 제조 기업 운송 물량 잇따라 수주</t>
+        </is>
+      </c>
+      <c r="E1070" s="4" t="inlineStr">
+        <is>
+          <t>현대글로비스가 중국 배터리 선도 기업을 포함한 주요 제조 기업으로부터 전기차 배터리, 자동차 반조립 부품 등의 유럽 및 중앙아시아향 운송 물량을 잇따라 수주했습니다.</t>
+        </is>
+      </c>
+      <c r="F1070" s="4" t="inlineStr">
+        <is>
+          <t>특정 물류 기업의 수주 소식으로, 당사의 물류 운영에 직접적인 영향은 없으나 배터리 운송 시장의 동향을 참고할 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G1070" s="4" t="n"/>
+      <c r="H1070" s="4" t="inlineStr">
+        <is>
+          <t>shippingnewsnet</t>
+        </is>
+      </c>
+      <c r="I1070" s="4" t="inlineStr">
+        <is>
+          <t>https://www.shippingnewsnet.com/news/articleView.html?idxno=71321</t>
+        </is>
+      </c>
+      <c r="J1070" s="4" t="inlineStr"/>
+    </row>
+    <row r="1071">
+      <c r="A1071" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B1071" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C1071" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D1071" s="4" t="inlineStr">
+        <is>
+          <t>전국 항만공사 통합 논의, 지역 이해관계 충돌 우려</t>
+        </is>
+      </c>
+      <c r="E1071" s="4" t="inlineStr">
+        <is>
+          <t>전국 항만공사 통합 논의가 항만별 특화 투자 필요성 및 지역 이해관계 충돌로 인한 갈등 확대 우려를 낳고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F1071" s="4" t="inlineStr">
+        <is>
+          <t>국내 항만 운영 정책 변화 논의로, 당사의 국제 물류 운영에 직접적인 영향은 낮습니다.</t>
+        </is>
+      </c>
+      <c r="G1071" s="4" t="n"/>
+      <c r="H1071" s="4" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I1071" s="4" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260725-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J1071" s="4" t="inlineStr"/>
+    </row>
+    <row r="1072">
+      <c r="A1072" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B1072" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C1072" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D1072" s="4" t="inlineStr">
+        <is>
+          <t>이베코코리아 / 연비·안전·주행 편의성 향상 대형 트랙터 ‘올 뉴 S-Way’ 출시</t>
+        </is>
+      </c>
+      <c r="E1072" s="4" t="inlineStr">
+        <is>
+          <t>이베코코리아가 연비, 안전, 주행 편의성을 향상시킨 대형 트랙터 '올 뉴 S-Way'를 국내에 출시했으며, 신형 엔진과 공기역학 설계 개선을 통해 최대 10%의 연료 효율 개선을 제공합니다.</t>
+        </is>
+      </c>
+      <c r="F1072" s="4" t="inlineStr">
+        <is>
+          <t>신형 트랙터 출시는 장기적으로 육상 운송 효율 개선에 기여할 수 있으나, 당사의 현재 물류 운영에 직접적인 영향은 낮습니다.</t>
+        </is>
+      </c>
+      <c r="G1072" s="4" t="n"/>
+      <c r="H1072" s="4" t="inlineStr">
+        <is>
+          <t>ulogistics</t>
+        </is>
+      </c>
+      <c r="I1072" s="4" t="inlineStr">
+        <is>
+          <t>http://www.ulogistics.co.kr/test/board.php?board=all2&amp;command=body&amp;no=5212</t>
+        </is>
+      </c>
+      <c r="J1072" s="4" t="inlineStr"/>
+    </row>
+    <row r="1073">
+      <c r="A1073" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B1073" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C1073" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D1073" s="4" t="inlineStr">
+        <is>
+          <t>배 만들 조선소도 사람도 없다…미국이 K-조선을 찾는 이유</t>
+        </is>
+      </c>
+      <c r="E1073" s="4" t="inlineStr">
+        <is>
+          <t>미국 해사청이 한화오션과 '해상 미사일 시험 계측선' 건조 계약을 체결하며, 미국 내 조선 역량 부족으로 한국 조선업을 찾는 경향을 보여줍니다.</t>
+        </is>
+      </c>
+      <c r="F1073" s="4" t="inlineStr">
+        <is>
+          <t>특정 국가의 조선 산업 동향으로, 당사의 물류 운영에 직접적인 영향은 낮습니다.</t>
+        </is>
+      </c>
+      <c r="G1073" s="4" t="n"/>
+      <c r="H1073" s="4" t="inlineStr">
+        <is>
+          <t>디지털데일리</t>
+        </is>
+      </c>
+      <c r="I1073" s="4" t="inlineStr">
+        <is>
+          <t>https://ddaily.co.kr/page/view/2026072116170018482</t>
+        </is>
+      </c>
+      <c r="J1073" s="4" t="inlineStr"/>
+    </row>
+    <row r="1074">
+      <c r="A1074" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B1074" s="4" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1074" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D1074" s="4" t="inlineStr">
+        <is>
+          <t>日, 제조업 경쟁력 회복 정책 강화…韓 기업 진출 기회 확대</t>
+        </is>
+      </c>
+      <c r="E1074" s="4" t="inlineStr">
+        <is>
+          <t>일본이 제조업 경쟁력 회복을 위한 지원 정책을 강화하고 있어, 한국 기업의 일본 시장 진출 기회가 확대될 것으로 기대된다.</t>
+        </is>
+      </c>
+      <c r="F1074" s="4" t="inlineStr">
+        <is>
+          <t>일본 시장 진출 기회 확대는 장기적인 사업 전략에 영향을 줄 수 있으나, 당장 우리 물류 운영이나 생산 계획에 직접적인 영향은 없다.</t>
+        </is>
+      </c>
+      <c r="G1074" s="4" t="n"/>
+      <c r="H1074" s="4" t="inlineStr">
+        <is>
+          <t>더구루</t>
+        </is>
+      </c>
+      <c r="I1074" s="4" t="inlineStr">
+        <is>
+          <t>https://view.mk.co.kr/car-tech/article/253322/</t>
+        </is>
+      </c>
+      <c r="J1074" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -49518,7 +51330,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -50583,6 +52395,49 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>3062.95</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>-17 (-0.6%)</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>+1,330 (+76.7%)</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="n">
+        <v>4204</v>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>-114 (-2.6%)</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>+1,755 (+71.7%)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -50595,7 +52450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I194"/>
+  <dimension ref="A1:I208"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -57411,6 +59266,496 @@
       </c>
       <c r="I194" s="6" t="inlineStr"/>
     </row>
+    <row r="195">
+      <c r="A195" s="6" t="inlineStr">
+        <is>
+          <t>RSK-194</t>
+        </is>
+      </c>
+      <c r="B195" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C195" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D195" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E195" s="6" t="inlineStr">
+        <is>
+          <t>Section 122 Tariffs' July 24 Expiration Thrown Into Doubt as U.S. Appeals CIT Ruling; Strait of Hormuz Reverts to War Conditions, Transits Down 66%</t>
+        </is>
+      </c>
+      <c r="F195" s="6" t="inlineStr"/>
+      <c r="G195" s="6" t="inlineStr"/>
+      <c r="H195" s="6" t="inlineStr">
+        <is>
+          <t>중동 항로를 이용하는 물량에 대한 대체 운송 경로 및 운송사 확보 검토, 관세 관련 동향 지속 모니터링 및 필요 시 무역팀과 협의.</t>
+        </is>
+      </c>
+      <c r="I195" s="6" t="inlineStr"/>
+    </row>
+    <row r="196">
+      <c r="A196" s="6" t="inlineStr">
+        <is>
+          <t>RSK-195</t>
+        </is>
+      </c>
+      <c r="B196" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C196" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D196" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E196" s="6" t="inlineStr">
+        <is>
+          <t>Section 301 Tariffs on Brazil Take Effect July 22, Stacking with Section 122 Duties; Strait of Hormuz Closure Restricts 200K TEU of Ocean Capacity</t>
+        </is>
+      </c>
+      <c r="F196" s="6" t="inlineStr"/>
+      <c r="G196" s="6" t="inlineStr"/>
+      <c r="H196" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈 해협을 경유하는 물량에 대한 비상 계획 수립, 대체 항로 및 운송 수단 검토, 브라질 및 러시아 관련 무역 정책 변화 모니터링 및 무역팀과 협의.</t>
+        </is>
+      </c>
+      <c r="I196" s="6" t="inlineStr"/>
+    </row>
+    <row r="197">
+      <c r="A197" s="6" t="inlineStr">
+        <is>
+          <t>RSK-196</t>
+        </is>
+      </c>
+      <c r="B197" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C197" s="6" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="D197" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E197" s="6" t="inlineStr">
+        <is>
+          <t>CBP Rejects Warehouse Entries on CAPE Declarations, Risking IEEPA Refunds; TPEB Rates Climb as Panama Canal Restrictions Tighten Capacity</t>
+        </is>
+      </c>
+      <c r="F197" s="6" t="inlineStr"/>
+      <c r="G197" s="6" t="inlineStr"/>
+      <c r="H197" s="6" t="inlineStr">
+        <is>
+          <t>파나마 운하를 이용하는 미주향 물량에 대한 운송 계획 재검토, 대체 경로 및 운송 수단(예: 철도, 육상) 고려, CBP 통관 절차 변화에 대한 무역팀과 협의 및 대응 방안 마련.</t>
+        </is>
+      </c>
+      <c r="I197" s="6" t="inlineStr"/>
+    </row>
+    <row r="198">
+      <c r="A198" s="6" t="inlineStr">
+        <is>
+          <t>RSK-197</t>
+        </is>
+      </c>
+      <c r="B198" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C198" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D198" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E198" s="6" t="inlineStr">
+        <is>
+          <t>'꼼수 관세' 꺼낸 트럼프, 강제노동 관세 60개국 부과...한국 12.5%</t>
+        </is>
+      </c>
+      <c r="F198" s="6" t="inlineStr"/>
+      <c r="G198" s="6" t="inlineStr"/>
+      <c r="H198" s="6" t="inlineStr">
+        <is>
+          <t>무역팀과 협의하여 강제노동 관세 부과 대상 품목 및 적용 시기 확인, 관세 회피 또는 최소화 방안 검토 (예: 원산지 증명, 생산지 다변화).</t>
+        </is>
+      </c>
+      <c r="I198" s="6" t="inlineStr"/>
+    </row>
+    <row r="199">
+      <c r="A199" s="6" t="inlineStr">
+        <is>
+          <t>RSK-198</t>
+        </is>
+      </c>
+      <c r="B199" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C199" s="6" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="D199" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E199" s="6" t="inlineStr">
+        <is>
+          <t>중동 물류 혼란으로 항만 대기 및 내륙 운송비 급증, 인도 지연</t>
+        </is>
+      </c>
+      <c r="F199" s="6" t="inlineStr"/>
+      <c r="G199" s="6" t="inlineStr"/>
+      <c r="H199" s="6" t="inlineStr">
+        <is>
+          <t>중동향 물량의 운송 경로 및 리드타임 재검토, 대체 운송 수단 및 파트너사 협의, 고객사와의 납기 조율.</t>
+        </is>
+      </c>
+      <c r="I199" s="6" t="inlineStr"/>
+    </row>
+    <row r="200">
+      <c r="A200" s="6" t="inlineStr">
+        <is>
+          <t>RSK-199</t>
+        </is>
+      </c>
+      <c r="B200" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C200" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D200" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E200" s="6" t="inlineStr">
+        <is>
+          <t>유가 급등, 금리·관세·환율 변수 겹치며 대외무역 불확실성 확대</t>
+        </is>
+      </c>
+      <c r="F200" s="6" t="inlineStr"/>
+      <c r="G200" s="6" t="inlineStr"/>
+      <c r="H200" s="6" t="inlineStr">
+        <is>
+          <t>유가 및 환율 변동에 따른 물류비 및 원가 상승 시나리오 분석, 관세 변동 가능성 대비 수출입 전략 검토.</t>
+        </is>
+      </c>
+      <c r="I200" s="6" t="inlineStr"/>
+    </row>
+    <row r="201">
+      <c r="A201" s="6" t="inlineStr">
+        <is>
+          <t>RSK-200</t>
+        </is>
+      </c>
+      <c r="B201" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C201" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D201" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E201" s="6" t="inlineStr">
+        <is>
+          <t>중국, EU 대러 제재 보복으로 유럽 기업 14곳 수출 통제</t>
+        </is>
+      </c>
+      <c r="F201" s="6" t="inlineStr"/>
+      <c r="G201" s="6" t="inlineStr"/>
+      <c r="H201" s="6" t="inlineStr">
+        <is>
+          <t>중국 및 EU 지역 공급망 리스크 점검, 대체 공급처 및 시장 확보 방안 검토, 무역 분쟁 추이 모니터링.</t>
+        </is>
+      </c>
+      <c r="I201" s="6" t="inlineStr"/>
+    </row>
+    <row r="202">
+      <c r="A202" s="6" t="inlineStr">
+        <is>
+          <t>RSK-201</t>
+        </is>
+      </c>
+      <c r="B202" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C202" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D202" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E202" s="6" t="inlineStr">
+        <is>
+          <t>미국 무역법 301조, 강제노동 관련 관세 12.5% 확정</t>
+        </is>
+      </c>
+      <c r="F202" s="6" t="inlineStr"/>
+      <c r="G202" s="6" t="inlineStr"/>
+      <c r="H202" s="6" t="inlineStr">
+        <is>
+          <t>강제노동 관련 관세 적용 대상 품목 및 지역 확인, 공급망 내 강제노동 리스크 점검 및 대응 방안 마련.</t>
+        </is>
+      </c>
+      <c r="I202" s="6" t="inlineStr"/>
+    </row>
+    <row r="203">
+      <c r="A203" s="6" t="inlineStr">
+        <is>
+          <t>RSK-202</t>
+        </is>
+      </c>
+      <c r="B203" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C203" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D203" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E203" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈 이어 홍해까지…글로벌 공급망 '이중 봉쇄' 공포</t>
+        </is>
+      </c>
+      <c r="F203" s="6" t="inlineStr"/>
+      <c r="G203" s="6" t="inlineStr"/>
+      <c r="H203" s="6" t="inlineStr">
+        <is>
+          <t>중동 및 유럽향/발 물량의 운송 경로 및 리드타임 재검토, 대체 운송 수단 및 파트너사 협의, 비축 재고 수준 점검, 고객사와의 납기 조율.</t>
+        </is>
+      </c>
+      <c r="I203" s="6" t="inlineStr"/>
+    </row>
+    <row r="204">
+      <c r="A204" s="6" t="inlineStr">
+        <is>
+          <t>RSK-203</t>
+        </is>
+      </c>
+      <c r="B204" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C204" s="6" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="D204" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E204" s="6" t="inlineStr">
+        <is>
+          <t>미·이란 충돌에 뱃길 꽉 막힌 중동…코트라, 우회 물류비 최대 8400만원 쏜다</t>
+        </is>
+      </c>
+      <c r="F204" s="6" t="inlineStr"/>
+      <c r="G204" s="6" t="inlineStr"/>
+      <c r="H204" s="6" t="inlineStr">
+        <is>
+          <t>중동 및 유럽향/발 해상 운송 경로 및 리드타임 재검토, 대체 운송 수단 및 항로(예: 희망봉 우회, 항공 운송) 비용 및 가용성 분석, 코트라 지원 프로그램 활용 검토.</t>
+        </is>
+      </c>
+      <c r="I204" s="6" t="inlineStr"/>
+    </row>
+    <row r="205">
+      <c r="A205" s="6" t="inlineStr">
+        <is>
+          <t>RSK-204</t>
+        </is>
+      </c>
+      <c r="B205" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C205" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D205" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E205" s="6" t="inlineStr">
+        <is>
+          <t>"바이어 뺏길라"...물류비 급등에도 수출기업 3곳 중 1곳 '비용 전가 0%'</t>
+        </is>
+      </c>
+      <c r="F205" s="6" t="inlineStr"/>
+      <c r="G205" s="6" t="inlineStr"/>
+      <c r="H205" s="6" t="inlineStr">
+        <is>
+          <t>운송 계약 재협상, 운송 모드 최적화(예: 해상/항공 운송 비율 조정), 물류 파트너와의 협력 강화, 물류비 절감 방안(예: 컨테이너 활용률 증대, 라우팅 최적화) 모색, 물류비 변동에 따른 가격 정책 유연성 검토.</t>
+        </is>
+      </c>
+      <c r="I205" s="6" t="inlineStr"/>
+    </row>
+    <row r="206">
+      <c r="A206" s="6" t="inlineStr">
+        <is>
+          <t>RSK-205</t>
+        </is>
+      </c>
+      <c r="B206" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C206" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D206" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E206" s="6" t="inlineStr">
+        <is>
+          <t>[기획]다시 불거진 관세리스크…수출기업 부담 커진다</t>
+        </is>
+      </c>
+      <c r="F206" s="6" t="inlineStr"/>
+      <c r="G206" s="6" t="inlineStr"/>
+      <c r="H206" s="6" t="inlineStr">
+        <is>
+          <t>미국 수출 품목에 대한 관세 영향 분석 및 가격 정책 재검토, 강제노동 관련 공급망 실사 강화.</t>
+        </is>
+      </c>
+      <c r="I206" s="6" t="inlineStr"/>
+    </row>
+    <row r="207">
+      <c r="A207" s="6" t="inlineStr">
+        <is>
+          <t>RSK-206</t>
+        </is>
+      </c>
+      <c r="B207" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C207" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D207" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E207" s="6" t="inlineStr">
+        <is>
+          <t>유가·운임 급등에 수출기업 '이중 부담'…물류비 쇼크 현실화</t>
+        </is>
+      </c>
+      <c r="F207" s="6" t="inlineStr"/>
+      <c r="G207" s="6" t="inlineStr"/>
+      <c r="H207" s="6" t="inlineStr">
+        <is>
+          <t>운송 계약 조건 재검토, 대체 운송 수단 및 경로 검토, 물류비 상승분 제품 가격 반영 여부 논의, 유가 및 운임 변동성 모니터링 강화.</t>
+        </is>
+      </c>
+      <c r="I207" s="6" t="inlineStr"/>
+    </row>
+    <row r="208">
+      <c r="A208" s="6" t="inlineStr">
+        <is>
+          <t>RSK-207</t>
+        </is>
+      </c>
+      <c r="B208" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C208" s="6" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="D208" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E208" s="6" t="inlineStr">
+        <is>
+          <t>“호르무즈 정상화 후에도 수출 물류 회복까지 6개월 이상 소요”</t>
+        </is>
+      </c>
+      <c r="F208" s="6" t="inlineStr"/>
+      <c r="G208" s="6" t="inlineStr"/>
+      <c r="H208" s="6" t="inlineStr">
+        <is>
+          <t>대체 운송 경로 및 운송 수단 확보 방안 검토, 재고 수준 조정, 고객 및 공급업체와 소통 강화, 비상 계획 수립.</t>
+        </is>
+      </c>
+      <c r="I208" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
📰 뉴스 데이터 2026-07-28_09:04
</commit_message>
<xml_diff>
--- a/data/SCM_물류_브리핑.xlsx
+++ b/data/SCM_물류_브리핑.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1074"/>
+  <dimension ref="A1:J1111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -51318,6 +51318,1790 @@
       </c>
       <c r="J1074" s="4" t="inlineStr"/>
     </row>
+    <row r="1075">
+      <c r="A1075" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B1075" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1075" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D1075" s="2" t="inlineStr">
+        <is>
+          <t>Section 301 Tariffs on Brazil Take Effect July 22, Stacking with Section 122 Duties; Strait of Hormuz Closure Restricts 200K TEU of Ocean Capacity</t>
+        </is>
+      </c>
+      <c r="E1075" s="2" t="inlineStr">
+        <is>
+          <t>브라질에 대한 Section 301 관세가 발효되고 호르무즈 해협 폐쇄로 20만 TEU의 해상 운송 용량이 제한되었으며, 러시아 제재 관련 중국/인도에 대한 2차 관세 부과 가능성도 제기되었다.</t>
+        </is>
+      </c>
+      <c r="F1075" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 폐쇄는 중동발 원자재 수급 및 유럽향/중동향 해상 운송에 즉각적인 차질을 유발하며, 관세 부과는 무역 비용에 직접적인 영향을 미친다.</t>
+        </is>
+      </c>
+      <c r="G1075" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 경유 노선 및 대체 운송 경로 검토, 중동발 원자재 재고 수준 점검, 브라질 및 러시아 관련 무역 동향 지속 모니터링 및 무역팀과 협의.</t>
+        </is>
+      </c>
+      <c r="H1075" s="2" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I1075" s="2" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/july-16-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J1075" s="2" t="inlineStr">
+        <is>
+          <t>RSK-208</t>
+        </is>
+      </c>
+    </row>
+    <row r="1076">
+      <c r="A1076" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B1076" s="2" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C1076" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D1076" s="2" t="inlineStr">
+        <is>
+          <t>미·이란, 공습·보복 이틀째 중단…'호르무즈 협상' 재개 분수령</t>
+        </is>
+      </c>
+      <c r="E1076" s="2" t="inlineStr">
+        <is>
+          <t>이란의 호르무즈 해협 사실상 봉쇄로 유조선·화물선 운항에 차질이 발생하고 국제유가가 급등했으며, 미-이란 간 공습 중단으로 협상 재개 여부가 주목된다.</t>
+        </is>
+      </c>
+      <c r="F1076" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협은 주요 해상 운송로이며, 봉쇄는 해상 운송 지연 및 유가 급등으로 이어져 물류비 상승과 운송 리드타임 증가에 직접적인 영향을 미친다.</t>
+        </is>
+      </c>
+      <c r="G1076" s="2" t="inlineStr">
+        <is>
+          <t>중동 항로 이용 시 대체 경로 및 운송 수단 검토, 유가 변동에 따른 물류비 상승분 예측 및 대응 계획 수립.</t>
+        </is>
+      </c>
+      <c r="H1076" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I1076" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260727-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J1076" s="2" t="inlineStr">
+        <is>
+          <t>RSK-209</t>
+        </is>
+      </c>
+    </row>
+    <row r="1077">
+      <c r="A1077" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B1077" s="2" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C1077" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D1077" s="2" t="inlineStr">
+        <is>
+          <t>코트라, 중동 수출길 확보 총력 및 요르단서 'K-이니셔티브 판촉전' 개최</t>
+        </is>
+      </c>
+      <c r="E1077" s="2" t="inlineStr">
+        <is>
+          <t>중동 지역의 물류 혼란으로 항만 대기 및 내륙 운송비가 급증하고 최종 인도까지 한 달 이상 지연되는 사례가 증가하고 있다.</t>
+        </is>
+      </c>
+      <c r="F1077" s="2" t="inlineStr">
+        <is>
+          <t>중동 지역으로의 수출 또는 해당 지역을 경유하는 운송 시 항만 적체 및 운송 지연, 비용 증가가 발생하여 당사의 물류 운영에 직접적인 차질을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="G1077" s="2" t="inlineStr">
+        <is>
+          <t>중동 지역 수출입 물량에 대한 운송 경로 및 리드타임 재검토, 현지 물류 파트너와 비상 계획 수립.</t>
+        </is>
+      </c>
+      <c r="H1077" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I1077" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260727-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J1077" s="2" t="inlineStr">
+        <is>
+          <t>RSK-210</t>
+        </is>
+      </c>
+    </row>
+    <row r="1078">
+      <c r="A1078" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B1078" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C1078" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D1078" s="2" t="inlineStr">
+        <is>
+          <t>뛰는 유가에 물가 불안 우려…금리·관세·환율도 '경고등'</t>
+        </is>
+      </c>
+      <c r="E1078" s="2" t="inlineStr">
+        <is>
+          <t>유가 급등과 함께 금리, 관세, 환율 변수까지 겹치면서 물가 및 대외무역의 불확실성이 확대되고 있다.</t>
+        </is>
+      </c>
+      <c r="F1078" s="2" t="inlineStr">
+        <is>
+          <t>유가 급등은 운송비에 직접적인 영향을 미치고, 관세 및 환율 변동은 수입 부품 원가 및 수출 경쟁력에 영향을 주어 전반적인 SCM 비용 및 계획에 높은 불확실성을 야기한다.</t>
+        </is>
+      </c>
+      <c r="G1078" s="2" t="inlineStr">
+        <is>
+          <t>유가, 환율, 주요 관세 변동 추이 면밀히 모니터링, 물류비 및 원가 상승 시나리오별 대응 계획 수립, 헤징 전략 검토.</t>
+        </is>
+      </c>
+      <c r="H1078" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I1078" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260726-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J1078" s="2" t="inlineStr">
+        <is>
+          <t>RSK-211</t>
+        </is>
+      </c>
+    </row>
+    <row r="1079">
+      <c r="A1079" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B1079" s="2" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C1079" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D1079" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 긴장에도 운임 하락… 해운업계 시선은 홍해로</t>
+        </is>
+      </c>
+      <c r="E1079" s="2" t="inlineStr">
+        <is>
+          <t>상하이컨테이너운임지수(SCFI)가 2주 연속 하락했으나, 지정학적 리스크의 초점이 홍해로 옮겨가면서 향후 운임 변동성이 커질 수 있다.</t>
+        </is>
+      </c>
+      <c r="F1079" s="2" t="inlineStr">
+        <is>
+          <t>홍해는 주요 해상 운송로이며, 해당 지역의 지정학적 리스크 증가는 운송 지연, 운임 급등, 선박 우회 등으로 이어져 당사의 물류 운영에 직접적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G1079" s="2" t="inlineStr">
+        <is>
+          <t>홍해 지역 지정학적 상황 및 해상 운임 변동 추이 면밀히 모니터링, 필요 시 대체 항로 및 운송 수단 검토.</t>
+        </is>
+      </c>
+      <c r="H1079" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I1079" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260724-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J1079" s="2" t="inlineStr">
+        <is>
+          <t>RSK-212</t>
+        </is>
+      </c>
+    </row>
+    <row r="1080">
+      <c r="A1080" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B1080" s="2" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C1080" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D1080" s="2" t="inlineStr">
+        <is>
+          <t>홍해 길목 지나는 화물선 하루 11척 불과...후티-사우디 충돌에 운항 '뚝'</t>
+        </is>
+      </c>
+      <c r="E1080" s="2" t="inlineStr">
+        <is>
+          <t>후티 반군과 사우디아라비아의 무력 충돌로 홍해의 바브엘만데브 해협을 지나는 화물선 통항이 수개월 만에 최저 수준으로 감소했다.</t>
+        </is>
+      </c>
+      <c r="F1080" s="2" t="inlineStr">
+        <is>
+          <t>홍해 해협의 화물선 통항 감소는 중동 및 유럽향 해상 운송의 심각한 지연을 초래하며, 이는 당사의 물류 리드타임 및 비용에 직접적인 영향을 미친다.</t>
+        </is>
+      </c>
+      <c r="G1080" s="2" t="inlineStr">
+        <is>
+          <t>홍해 항로 이용 시 대체 경로 및 운송 수단 검토, 중동/유럽향 물량의 운송 일정 재조정 및 고객사/협력사와의 소통 강화.</t>
+        </is>
+      </c>
+      <c r="H1080" s="2" t="inlineStr">
+        <is>
+          <t>뉴스핌</t>
+        </is>
+      </c>
+      <c r="I1080" s="2" t="inlineStr">
+        <is>
+          <t>https://www.newspim.com/news/view/20260727000630</t>
+        </is>
+      </c>
+      <c r="J1080" s="2" t="inlineStr">
+        <is>
+          <t>RSK-213</t>
+        </is>
+      </c>
+    </row>
+    <row r="1081">
+      <c r="A1081" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B1081" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C1081" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1081" s="3" t="inlineStr">
+        <is>
+          <t>CBP Rejects Warehouse Entries on CAPE Declarations, Risking IEEPA Refunds; TPEB Rates Climb as Panama Canal Restrictions Tighten Capacity</t>
+        </is>
+      </c>
+      <c r="E1081" s="3" t="inlineStr">
+        <is>
+          <t>CBP가 CAPE 신고에 대한 창고 입고를 거부하여 IEEPA 환급 위험이 발생했으며, 파나마 운하의 통행 제한으로 태평양 횡단 동향(TPEB) 운임이 상승하고 용량이 타이트해졌다.</t>
+        </is>
+      </c>
+      <c r="F1081" s="3" t="inlineStr">
+        <is>
+          <t>파나마 운하 통행 제한은 미주향 운송에 영향을 미치며 운임 상승을 유발할 수 있고, CBP의 창고 입고 거부는 관세 환급 절차에 복잡성을 더할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G1081" s="3" t="inlineStr">
+        <is>
+          <t>파나마 운하 경유 미주향 운송 스케줄 및 운임 변동 추이 모니터링, 관세 환급 절차 관련 무역팀과 협의.</t>
+        </is>
+      </c>
+      <c r="H1081" s="3" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I1081" s="3" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/july-09-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J1081" s="3" t="inlineStr"/>
+    </row>
+    <row r="1082">
+      <c r="A1082" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B1082" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C1082" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1082" s="3" t="inlineStr">
+        <is>
+          <t>CAPE Phase 2 Launches June 29 for Reconciliation-Flagged Entries; TPEB Rates Rise 10% for Sixth Consecutive Week</t>
+        </is>
+      </c>
+      <c r="E1082" s="3" t="inlineStr">
+        <is>
+          <t>CBP의 CAPE IEEPA 관세 환급 시스템 2단계가 시작되어 환급 대상이 확대되었으며, 태평양 횡단 동향(TPEB) 운임이 6주 연속 10% 상승했다.</t>
+        </is>
+      </c>
+      <c r="F1082" s="3" t="inlineStr">
+        <is>
+          <t>TPEB 운임의 지속적인 상승은 미주향 운송 비용 증가로 이어지며, CAPE 시스템 확장은 관세 환급 절차에 영향을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="G1082" s="3" t="inlineStr">
+        <is>
+          <t>TPEB 운임 추이 및 장기 계약 조건 재검토, 관세 환급 절차 관련 무역팀과 협의.</t>
+        </is>
+      </c>
+      <c r="H1082" s="3" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I1082" s="3" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/june-25-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J1082" s="3" t="inlineStr"/>
+    </row>
+    <row r="1083">
+      <c r="A1083" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B1083" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C1083" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1083" s="3" t="inlineStr">
+        <is>
+          <t>Statement on EU Commission Revision of the EU Emissions Trading System</t>
+        </is>
+      </c>
+      <c r="E1083" s="3" t="inlineStr">
+        <is>
+          <t>IATA는 EU 배출권 거래 시스템(ETS)의 유럽 외 확장 제안에 깊은 우려를 표명하며, 이는 항공 운송 비용 증가로 이어질 수 있다고 경고했다.</t>
+        </is>
+      </c>
+      <c r="F1083" s="3" t="inlineStr">
+        <is>
+          <t>EU ETS의 확장은 항공 운송 비용을 증가시켜 유럽향/유럽발 항공 화물 운임에 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G1083" s="3" t="inlineStr">
+        <is>
+          <t>EU ETS 관련 규제 동향 및 항공 운임 변동 추이 모니터링, 항공 운송 비용 증가 시 대체 운송 방안 검토.</t>
+        </is>
+      </c>
+      <c r="H1083" s="3" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I1083" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/07-17-statement-eu-commission-revision-emissions-trading-system/</t>
+        </is>
+      </c>
+      <c r="J1083" s="3" t="inlineStr"/>
+    </row>
+    <row r="1084">
+      <c r="A1084" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B1084" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C1084" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1084" s="3" t="inlineStr">
+        <is>
+          <t>북미항로/ ‘수요둔화 대응’ HMM·코스코, 내달 운임회복 시동</t>
+        </is>
+      </c>
+      <c r="E1084" s="3" t="inlineStr">
+        <is>
+          <t>북미항로 운임 상승세가 둔화되었으나, HMM과 코스코 등 선사들이 운임 인상 및 할증료 부과를 통해 운임 회복을 시도하며 여전히 높은 수준을 유지하고 있다.</t>
+        </is>
+      </c>
+      <c r="F1084" s="3" t="inlineStr">
+        <is>
+          <t>북미항로 운임이 높은 수준을 유지하고 선사들이 추가 인상을 시도하고 있어, 북미향 운송 비용에 지속적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G1084" s="3" t="inlineStr">
+        <is>
+          <t>북미항로 운임 추이 지속 모니터링, 장기 운송 계약 조건 재검토 및 선사와의 협상 준비.</t>
+        </is>
+      </c>
+      <c r="H1084" s="3" t="inlineStr">
+        <is>
+          <t>kita</t>
+        </is>
+      </c>
+      <c r="I1084" s="3" t="inlineStr">
+        <is>
+          <t>https://www.kita.net/shippers/board/newsView.do?morgueCode=2&amp;dataCls=B&amp;dataSeq=8179</t>
+        </is>
+      </c>
+      <c r="J1084" s="3" t="inlineStr"/>
+    </row>
+    <row r="1085">
+      <c r="A1085" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B1085" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C1085" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1085" s="3" t="inlineStr">
+        <is>
+          <t>Global Schedule Reliability drops to 62.6% in June 2026</t>
+        </is>
+      </c>
+      <c r="E1085" s="3" t="inlineStr">
+        <is>
+          <t>2026년 6월 글로벌 선박 스케줄 신뢰도가 62.6%로 하락하여 해상 운송의 지연 가능성이 증가하고 있음을 보여준다.</t>
+        </is>
+      </c>
+      <c r="F1085" s="3" t="inlineStr">
+        <is>
+          <t>선박 스케줄 신뢰도 하락은 해상 운송 지연으로 이어져 부품 및 완제품의 입출고 일정에 영향을 줄 수 있으므로 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G1085" s="3" t="inlineStr">
+        <is>
+          <t>주요 항로의 선박 스케줄 변동성 추이 모니터링 및 비상 재고 수준 검토.</t>
+        </is>
+      </c>
+      <c r="H1085" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I1085" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/400-global-schedule-reliability-drops-to-62-6-in-june-2026</t>
+        </is>
+      </c>
+      <c r="J1085" s="3" t="inlineStr"/>
+    </row>
+    <row r="1086">
+      <c r="A1086" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B1086" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C1086" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1086" s="3" t="inlineStr">
+        <is>
+          <t>Structural Shift in Blank Sailing Strategies</t>
+        </is>
+      </c>
+      <c r="E1086" s="3" t="inlineStr">
+        <is>
+          <t>2026년 상반기 선사들의 결항(Blank Sailing) 전략이 전체 선복량 증가보다 빠르게 늘어나고 있어 주요 동서 항로의 운송 공급에 구조적 변화가 있음을 시사한다.</t>
+        </is>
+      </c>
+      <c r="F1086" s="3" t="inlineStr">
+        <is>
+          <t>결항 증가는 선복량 감소로 이어져 운송 공간 확보에 어려움을 주거나 운임 상승 압력으로 작용할 수 있으므로 추이를 주시해야 한다.</t>
+        </is>
+      </c>
+      <c r="G1086" s="3" t="inlineStr">
+        <is>
+          <t>주요 항로의 선복량 및 결항률 변화 모니터링, 장기 운송 계약 조건 검토.</t>
+        </is>
+      </c>
+      <c r="H1086" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I1086" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/399-structural-shift-in-blank-sailing-strategies</t>
+        </is>
+      </c>
+      <c r="J1086" s="3" t="inlineStr"/>
+    </row>
+    <row r="1087">
+      <c r="A1087" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B1087" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C1087" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1087" s="3" t="inlineStr">
+        <is>
+          <t>Structural Contraction of Global Liner Networks (Shipping lines network management)</t>
+        </is>
+      </c>
+      <c r="E1087" s="3" t="inlineStr">
+        <is>
+          <t>2012년 이후 글로벌 정기선 네트워크 데이터 분석 결과, 선사들이 지리적 범위는 유지하면서도 서비스 빈도를 줄이는 등 네트워크 관리 방식에 근본적인 변화가 나타나고 있다.</t>
+        </is>
+      </c>
+      <c r="F1087" s="3" t="inlineStr">
+        <is>
+          <t>선사들의 서비스 빈도 감소는 특정 항로의 운송 옵션 축소 및 리드타임 증가로 이어질 수 있어 잠재적 영향에 대한 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G1087" s="3" t="inlineStr">
+        <is>
+          <t>주요 항로의 선사 서비스 빈도 변화 모니터링 및 대체 운송 옵션 검토.</t>
+        </is>
+      </c>
+      <c r="H1087" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I1087" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/397-structural-contraction-of-global-liner-networks</t>
+        </is>
+      </c>
+      <c r="J1087" s="3" t="inlineStr"/>
+    </row>
+    <row r="1088">
+      <c r="A1088" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B1088" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C1088" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1088" s="3" t="inlineStr">
+        <is>
+          <t>PLSCI Data Indicates Mega-Hub Retrenchment</t>
+        </is>
+      </c>
+      <c r="E1088" s="3" t="inlineStr">
+        <is>
+          <t>UNCTAD의 2026년 2분기 항만 정기선 연결성 지수(PLSCI) 분석에 따르면, 최근 네트워크 재조정이 메가 허브 항만에서의 서비스 축소로 이어지고 있다.</t>
+        </is>
+      </c>
+      <c r="F1088" s="3" t="inlineStr">
+        <is>
+          <t>주요 허브 항만의 연결성 축소는 환적 지연이나 특정 지역으로의 운송 경로 변경을 야기할 수 있어 물류 효율성에 영향을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="G1088" s="3" t="inlineStr">
+        <is>
+          <t>주요 환적 항만의 연결성 변화 모니터링 및 대체 항만 활용 가능성 검토.</t>
+        </is>
+      </c>
+      <c r="H1088" s="3" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I1088" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/396-plsci-data-indicates-mega-hub-retrenchment</t>
+        </is>
+      </c>
+      <c r="J1088" s="3" t="inlineStr"/>
+    </row>
+    <row r="1089">
+      <c r="A1089" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B1089" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1089" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1089" s="3" t="inlineStr">
+        <is>
+          <t>중, EU의 대러 제재에 보복… 라인메탈 등 유럽 기업 14곳 수출 통제</t>
+        </is>
+      </c>
+      <c r="E1089" s="3" t="inlineStr">
+        <is>
+          <t>중국이 EU의 대러 제재에 대한 보복으로 라인메탈 등 유럽 기업 14곳에 대해 수출 통제를 가하며 중국과 유럽 간 무역 갈등이 격화되고 있다.</t>
+        </is>
+      </c>
+      <c r="F1089" s="3" t="inlineStr">
+        <is>
+          <t>중국과 유럽 간 무역 갈등 격화 및 수출 통제는 해당 지역의 공급망 안정성에 영향을 줄 수 있으며, 당사의 유럽 또는 중국향 물류에 간접적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G1089" s="3" t="inlineStr">
+        <is>
+          <t>중국-EU 간 무역 갈등 추이 및 추가 제재 가능성 모니터링, 해당 지역 공급망 리스크 평가.</t>
+        </is>
+      </c>
+      <c r="H1089" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I1089" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260726-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J1089" s="3" t="inlineStr"/>
+    </row>
+    <row r="1090">
+      <c r="A1090" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B1090" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1090" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1090" s="3" t="inlineStr">
+        <is>
+          <t>미 301조 강제노동 관세 12.5% 매듭…과잉생산 관세는?</t>
+        </is>
+      </c>
+      <c r="E1090" s="3" t="inlineStr">
+        <is>
+          <t>미국의 무역법 301조 조사에서 강제노동 관련 관세가 12.5%로 확정되었으며, 과잉생산 관련 관세 부과 여부가 주목된다.</t>
+        </is>
+      </c>
+      <c r="F1090" s="3" t="inlineStr">
+        <is>
+          <t>미국의 강제노동 관련 관세 부과는 특정 지역에서 생산되는 부품 및 제품의 수입 비용을 증가시킬 수 있으며, 향후 과잉생산 관세 부과 여부에 따라 공급망 전략 재검토가 필요할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G1090" s="3" t="inlineStr">
+        <is>
+          <t>미국 무역 정책 변화 및 추가 관세 부과 가능성 모니터링, 공급망 내 강제노동 관련 리스크 점검.</t>
+        </is>
+      </c>
+      <c r="H1090" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I1090" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260725-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J1090" s="3" t="inlineStr"/>
+    </row>
+    <row r="1091">
+      <c r="A1091" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B1091" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C1091" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1091" s="3" t="inlineStr">
+        <is>
+          <t>HMM 주목하는 증권가...하반기 더 기대되는 이유는?</t>
+        </is>
+      </c>
+      <c r="E1091" s="3" t="inlineStr">
+        <is>
+          <t>상하이컨테이너운임지수(SCFI) 및 컨테이너선운임지수(CCFI) 상승과 관세 변경 전 선적 수요 증가로 하반기 해운 시황 개선 및 HMM 실적 기대감이 커지고 있다.</t>
+        </is>
+      </c>
+      <c r="F1091" s="3" t="inlineStr">
+        <is>
+          <t>운임 지수 상승은 해상 운임 상승 압력으로 작용하여 당사의 물류비 증가로 이어질 수 있으며, 관세 변경 전 선적 수요는 일시적인 운송 병목 현상을 유발할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G1091" s="3" t="inlineStr">
+        <is>
+          <t>SCFI/CCFI 및 주요 항로 운임 지수 변화 모니터링, 관세 변경 예정 품목의 선적 일정 사전 조율.</t>
+        </is>
+      </c>
+      <c r="H1091" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I1091" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260724-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J1091" s="3" t="inlineStr"/>
+    </row>
+    <row r="1092">
+      <c r="A1092" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B1092" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C1092" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1092" s="3" t="inlineStr">
+        <is>
+          <t>Supply Chain Disruptions and Operational Vulnerabilities</t>
+        </is>
+      </c>
+      <c r="E1092" s="3" t="inlineStr">
+        <is>
+          <t>공급망 중단이 지연된 송장, 비용 상승, 재고 불일치 등으로 나타나며, 팬데믹 이후에도 지연, 부족, 예측 불가능한 물류 문제가 지속되고 있다. 기업들은 공급망 취약성에 대한 대비가 필요하다.</t>
+        </is>
+      </c>
+      <c r="F1092" s="3" t="inlineStr">
+        <is>
+          <t>전반적인 공급망 취약성과 지연 가능성을 경고하며, 우리 물류 운영의 잠재적 위험을 상기시키므로 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G1092" s="3" t="inlineStr">
+        <is>
+          <t>공급망 가시성 강화 및 비상 계획 점검.</t>
+        </is>
+      </c>
+      <c r="H1092" s="3" t="inlineStr">
+        <is>
+          <t>Add-Vantage Bookkeeping</t>
+        </is>
+      </c>
+      <c r="I1092" s="3" t="inlineStr">
+        <is>
+          <t>https://addvantagebookkeeping.com/supply-chain-disruptions-and-operational-vulnerabilities</t>
+        </is>
+      </c>
+      <c r="J1092" s="3" t="inlineStr"/>
+    </row>
+    <row r="1093">
+      <c r="A1093" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B1093" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1093" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1093" s="3" t="inlineStr">
+        <is>
+          <t>How regional conflict is reshaping industrial investment</t>
+        </is>
+      </c>
+      <c r="E1093" s="3" t="inlineStr">
+        <is>
+          <t>지역 분쟁이 산업 투자 지형을 바꾸고 있으며, 기업들은 공급망, 물류 대안, 사업 연속성, 운영 유연성을 중점적으로 고려하고 있다. 이는 지정학적 리스크가 물류 전략에 미치는 영향을 강조한다.</t>
+        </is>
+      </c>
+      <c r="F1093" s="3" t="inlineStr">
+        <is>
+          <t>지정학적 리스크가 공급망 전략에 미치는 영향을 강조하며, 우리 회사의 물류 네트워크 및 투자 전략에 대한 재검토 필요성을 시사한다.</t>
+        </is>
+      </c>
+      <c r="G1093" s="3" t="inlineStr">
+        <is>
+          <t>잠재적 지정학적 리스크 지역의 물류 경로 및 대안 검토.</t>
+        </is>
+      </c>
+      <c r="H1093" s="3" t="inlineStr">
+        <is>
+          <t>Logistics Middle East</t>
+        </is>
+      </c>
+      <c r="I1093" s="3" t="inlineStr">
+        <is>
+          <t>https://www.logisticsmiddleeast.com/logistics/how-regional-conflict-is-reshaping-industrial-investment-across-the-uae</t>
+        </is>
+      </c>
+      <c r="J1093" s="3" t="inlineStr"/>
+    </row>
+    <row r="1094">
+      <c r="A1094" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B1094" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C1094" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1094" s="3" t="inlineStr">
+        <is>
+          <t>How exposed are we? Cyber risk, supply chains and the reality of grid resilience</t>
+        </is>
+      </c>
+      <c r="E1094" s="3" t="inlineStr">
+        <is>
+          <t>사이버 리스크와 공급망 취약성이 전력망 복원력에 미치는 영향을 다루며, 특히 PV 및 BESS(배터리 에너지 저장 시스템) 분야의 중요성을 강조한다. 이는 배터리 제조사에게 중요한 리스크 요인이다.</t>
+        </is>
+      </c>
+      <c r="F1094" s="3" t="inlineStr">
+        <is>
+          <t>사이버 공격이 공급망 및 전력망에 미칠 수 있는 잠재적 위험을 경고하며, 배터리 제조사로서 관련 리스크 관리가 중요함을 시사한다.</t>
+        </is>
+      </c>
+      <c r="G1094" s="3" t="inlineStr">
+        <is>
+          <t>IT/OT 보안 강화 및 공급망 파트너의 사이버 보안 수준 점검.</t>
+        </is>
+      </c>
+      <c r="H1094" s="3" t="inlineStr">
+        <is>
+          <t>PV-Tech</t>
+        </is>
+      </c>
+      <c r="I1094" s="3" t="inlineStr">
+        <is>
+          <t>https://pv-tech.org/how-exposed-are-we-cyber-risk-supply-chains-and-the-reality-of-grid-resilience</t>
+        </is>
+      </c>
+      <c r="J1094" s="3" t="inlineStr"/>
+    </row>
+    <row r="1095">
+      <c r="A1095" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B1095" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C1095" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1095" s="3" t="inlineStr">
+        <is>
+          <t>[논현논단-이덕환 칼럼] ‘리튬이온 배터리’ 상식이 필요한 까닭</t>
+        </is>
+      </c>
+      <c r="E1095" s="3" t="inlineStr">
+        <is>
+          <t>리튬이온 배터리의 분리막 파손 시 열폭주로 인한 화재 발생 위험을 경고하며, 소비자 자발적 안전 관리와 품질 관리 강화를 통한 불량품 차단이 중요하다고 강조한다. 이는 배터리 제조사의 책임과 직결된다.</t>
+        </is>
+      </c>
+      <c r="F1095" s="3" t="inlineStr">
+        <is>
+          <t>리튬이온 배터리의 화재 위험과 품질 관리의 중요성을 강조하며, 우리 회사의 제품 안전성 및 규제 준수에 대한 지속적인 관심과 점검이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G1095" s="3" t="inlineStr">
+        <is>
+          <t>제품 품질 관리 프로세스 및 안전 규정 준수 여부 재점검.</t>
+        </is>
+      </c>
+      <c r="H1095" s="3" t="inlineStr">
+        <is>
+          <t>이투데이</t>
+        </is>
+      </c>
+      <c r="I1095" s="3" t="inlineStr">
+        <is>
+          <t>https://etoday.co.kr/news/view/2608003</t>
+        </is>
+      </c>
+      <c r="J1095" s="3" t="inlineStr"/>
+    </row>
+    <row r="1096">
+      <c r="A1096" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B1096" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C1096" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1096" s="3" t="inlineStr">
+        <is>
+          <t>AI가 포장까지 바꾼다…'스마트 적정포장'이 여는 순환경제의 새 해법</t>
+        </is>
+      </c>
+      <c r="E1096" s="3" t="inlineStr">
+        <is>
+          <t>AI를 활용한 '스마트 적정포장'이 과대포장 및 포장 폐기물 문제를 해결하고 순환경제를 실현하는 새로운 해법으로 주목받고 있다. 이는 물류 포장 전략에 중요한 시사점을 제공한다.</t>
+        </is>
+      </c>
+      <c r="F1096" s="3" t="inlineStr">
+        <is>
+          <t>AI 기반 포장 최적화는 물류 비용 절감 및 환경 규제 대응에 기여할 수 있는 장기적 트렌드로, 우리 회사의 포장 전략에 대한 검토가 필요하다.</t>
+        </is>
+      </c>
+      <c r="G1096" s="3" t="inlineStr">
+        <is>
+          <t>AI 기반 포장 기술 동향 및 우리 회사 제품 포장 적용 가능성 검토.</t>
+        </is>
+      </c>
+      <c r="H1096" s="3" t="inlineStr">
+        <is>
+          <t>에너지데일리</t>
+        </is>
+      </c>
+      <c r="I1096" s="3" t="inlineStr">
+        <is>
+          <t>https://energydaily.co.kr/news/articleView.html?idxno=201749</t>
+        </is>
+      </c>
+      <c r="J1096" s="3" t="inlineStr"/>
+    </row>
+    <row r="1097">
+      <c r="A1097" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B1097" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C1097" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1097" s="3" t="inlineStr">
+        <is>
+          <t>'109시간 만에 진화' 인천 쿠팡 물류센터 화재, 내일 합동감식 | 뉴데일리</t>
+        </is>
+      </c>
+      <c r="E1097" s="3" t="inlineStr">
+        <is>
+          <t>인천 서해구 쿠팡 32물류센터에서 발생한 대형 화재가 109시간여 만에 진화되었으며, 경찰과 소방 당국이 28일 오전 10시부터 합동 감식에 나설 예정이다.</t>
+        </is>
+      </c>
+      <c r="F1097" s="3" t="inlineStr">
+        <is>
+          <t>대형 물류센터 화재는 창고 안전 규제 강화 논의로 이어질 수 있으며, 특히 배터리/전자부품은 위험물로 분류될 가능성이 있어 향후 보관 및 취급 규제 변화를 주시해야 한다.</t>
+        </is>
+      </c>
+      <c r="G1097" s="3" t="inlineStr">
+        <is>
+          <t>국내 물류센터 화재 관련 규제 동향 및 배터리/전자부품 보관 기준 변화 가능성 모니터링.</t>
+        </is>
+      </c>
+      <c r="H1097" s="3" t="inlineStr">
+        <is>
+          <t>뉴데일리</t>
+        </is>
+      </c>
+      <c r="I1097" s="3" t="inlineStr">
+        <is>
+          <t>https://www.newdaily.co.kr/site/data/html/2026/07/27/2026072700148.html</t>
+        </is>
+      </c>
+      <c r="J1097" s="3" t="inlineStr"/>
+    </row>
+    <row r="1098">
+      <c r="A1098" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B1098" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1098" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1098" s="3" t="inlineStr">
+        <is>
+          <t>쉬인 1분기 1448억 손실에 적자 전환...소액 소포 면세 폐지에 직격 | 서울경제</t>
+        </is>
+      </c>
+      <c r="E1098" s="3" t="inlineStr">
+        <is>
+          <t>중국 온라인 패션 기업 쉬인이 미국 정부의 소액 화물 면세 혜택 폐지 여파로 1분기 1448억 원의 손실을 기록하며 적자 전환했다.</t>
+        </is>
+      </c>
+      <c r="F1098" s="3" t="inlineStr">
+        <is>
+          <t>미국 정부의 소액 화물 면세 혜택 폐지는 중국발 이커머스 플랫폼에 대한 규제 강화의 일환으로, 향후 배터리/전자부품 등 다른 품목에도 유사한 관세 및 무역 정책 변화가 확대될 가능성을 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G1098" s="3" t="inlineStr">
+        <is>
+          <t>미-중 무역 정책 변화 및 관세 동향 지속 모니터링.</t>
+        </is>
+      </c>
+      <c r="H1098" s="3" t="inlineStr">
+        <is>
+          <t>서울경제</t>
+        </is>
+      </c>
+      <c r="I1098" s="3" t="inlineStr">
+        <is>
+          <t>https://sedaily.com/article/20072539</t>
+        </is>
+      </c>
+      <c r="J1098" s="3" t="inlineStr"/>
+    </row>
+    <row r="1099">
+      <c r="A1099" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B1099" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1099" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1099" s="3" t="inlineStr">
+        <is>
+          <t>中, 국산 DUV 양산 돌입…EUV 없이 HBM3E 길 열리나 &lt; 국제 &lt; 기사본문 - 이코노미트리뷴</t>
+        </is>
+      </c>
+      <c r="E1099" s="3" t="inlineStr">
+        <is>
+          <t>중국이 자국산 액침형 심자외선(DUV) 노광장비 양산에 돌입하며 미국의 반도체 장비 수출 통제에 대응하고 있어, 반도체 공급망 재편에 영향을 줄 것으로 예상된다.</t>
+        </is>
+      </c>
+      <c r="F1099" s="3" t="inlineStr">
+        <is>
+          <t>미-중 반도체 기술 경쟁 심화는 장기적으로 전자부품 공급망의 안정성 및 조달 비용에 영향을 미칠 수 있으며, 특정 부품의 수출입 규제 변화 가능성을 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G1099" s="3" t="inlineStr">
+        <is>
+          <t>반도체 관련 미-중 기술 및 무역 정책 동향을 주시하고, 잠재적인 공급망 변화에 대비.</t>
+        </is>
+      </c>
+      <c r="H1099" s="3" t="inlineStr">
+        <is>
+          <t>이코노미트리뷴</t>
+        </is>
+      </c>
+      <c r="I1099" s="3" t="inlineStr">
+        <is>
+          <t>https://economytribune.co.kr/news/articleView.html?idxno=3903454</t>
+        </is>
+      </c>
+      <c r="J1099" s="3" t="inlineStr"/>
+    </row>
+    <row r="1100">
+      <c r="A1100" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B1100" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1100" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1100" s="3" t="inlineStr">
+        <is>
+          <t>韓, 환율 방어에 280억弗 풀어…美재무부 "개입 규모 세계 3위" - 매일경제</t>
+        </is>
+      </c>
+      <c r="E1100" s="3" t="inlineStr">
+        <is>
+          <t>한국 정부가 원화 가치 하락을 방어하기 위해 280억 달러를 매도 개입했으며, 이는 미국 재무부 보고서에서 세계 3위 규모로 나타났다.</t>
+        </is>
+      </c>
+      <c r="F1100" s="3" t="inlineStr">
+        <is>
+          <t>정부의 환율 방어 개입은 원화 가치 변동성을 시사하며, 이는 국제 운임 및 해외 원자재 수입 비용에 간접적인 영향을 미칠 수 있어 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G1100" s="3" t="inlineStr">
+        <is>
+          <t>환율 변동 추이 모니터링 및 물류비용 예측에 반영.</t>
+        </is>
+      </c>
+      <c r="H1100" s="3" t="inlineStr">
+        <is>
+          <t>매일경제</t>
+        </is>
+      </c>
+      <c r="I1100" s="3" t="inlineStr">
+        <is>
+          <t>https://mk.co.kr/news/economy/12108688</t>
+        </is>
+      </c>
+      <c r="J1100" s="3" t="inlineStr"/>
+    </row>
+    <row r="1101">
+      <c r="A1101" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B1101" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1101" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1101" s="3" t="inlineStr">
+        <is>
+          <t>AI가 바꾼 제조업 지도…한은 "반도체·자동차 공급망 재편 가속" | 아주경제</t>
+        </is>
+      </c>
+      <c r="E1101" s="3" t="inlineStr">
+        <is>
+          <t>한국은행 보고서에 따르면 인공지능(AI) 확산, 미·중 갈등, 보호무역 강화 등의 영향으로 우리나라 제조업, 특히 반도체 및 자동차 산업의 생산과 공급망이 빠르게 재편되고 있다.</t>
+        </is>
+      </c>
+      <c r="F1101" s="3" t="inlineStr">
+        <is>
+          <t>반도체 및 전자부품 공급망 재편 가속화는 원자재 조달 및 생산 거점 전략에 장기적인 영향을 미칠 수 있으므로, 관련 동향을 지속적으로 모니터링하여 공급망 전략에 반영해야 한다.</t>
+        </is>
+      </c>
+      <c r="G1101" s="3" t="inlineStr">
+        <is>
+          <t>글로벌 공급망 재편 동향 분석 및 중장기 공급망 전략 수립에 참고.</t>
+        </is>
+      </c>
+      <c r="H1101" s="3" t="inlineStr">
+        <is>
+          <t>아주경제</t>
+        </is>
+      </c>
+      <c r="I1101" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ajunews.com/view/20260727101020819</t>
+        </is>
+      </c>
+      <c r="J1101" s="3" t="inlineStr"/>
+    </row>
+    <row r="1102">
+      <c r="A1102" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B1102" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C1102" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1102" s="3" t="inlineStr">
+        <is>
+          <t>산업부, 정유&amp;middot;해운업계와 원유 수급상황 점검회의</t>
+        </is>
+      </c>
+      <c r="E1102" s="3" t="inlineStr">
+        <is>
+          <t>산업통상부가 중동 지역 긴장 재고조와 홍해 통항 리스크 확대에 대응하여 정유 및 해운업계와 원유 수급상황 점검 회의를 개최했다.</t>
+        </is>
+      </c>
+      <c r="F1102" s="3" t="inlineStr">
+        <is>
+          <t>중동 및 홍해 리스크는 국제 유가 상승과 해상 운임 변동으로 이어질 수 있으며, 이는 우리 물류비용에 직접적인 영향을 미치므로 추이를 면밀히 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G1102" s="3" t="inlineStr">
+        <is>
+          <t>국제 유가 및 해상 운임 변동 추이 모니터링 강화, 비상시 대체 운송 경로 및 운송 수단 검토.</t>
+        </is>
+      </c>
+      <c r="H1102" s="3" t="inlineStr">
+        <is>
+          <t>베타뉴스</t>
+        </is>
+      </c>
+      <c r="I1102" s="3" t="inlineStr">
+        <is>
+          <t>https://betanews.net/article/view/beta202607270042</t>
+        </is>
+      </c>
+      <c r="J1102" s="3" t="inlineStr"/>
+    </row>
+    <row r="1103">
+      <c r="A1103" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B1103" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C1103" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1103" s="3" t="inlineStr">
+        <is>
+          <t>美이란 공습 중단에 국제유가 급락…브랜트유 90달러 밑으로 ‘뚝’ - 매일경제</t>
+        </is>
+      </c>
+      <c r="E1103" s="3" t="inlineStr">
+        <is>
+          <t>미국이 이란 공습을 중단하면서 국제 유가가 급락하여 9월 인도분 브렌트유 종가가 배럴당 88.36달러로 전장 대비 8.7% 하락했다.</t>
+        </is>
+      </c>
+      <c r="F1103" s="3" t="inlineStr">
+        <is>
+          <t>국제 유가 급락은 단기적으로 항공 및 해상 운임 하락 압력으로 작용하여 물류비용 절감에 긍정적일 수 있으나, 중동 정세의 불확실성으로 인해 유가 변동성이 클 수 있어 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G1103" s="3" t="inlineStr">
+        <is>
+          <t>유가 변동 추이 및 운임 시장 반응 모니터링, 물류비용 예측에 반영.</t>
+        </is>
+      </c>
+      <c r="H1103" s="3" t="inlineStr">
+        <is>
+          <t>매일경제</t>
+        </is>
+      </c>
+      <c r="I1103" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mk.co.kr/news/world/12109047</t>
+        </is>
+      </c>
+      <c r="J1103" s="3" t="inlineStr"/>
+    </row>
+    <row r="1104">
+      <c r="A1104" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B1104" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C1104" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1104" s="3" t="inlineStr">
+        <is>
+          <t>[속보] 국제유가, 급락...WTI 7.5% ↓</t>
+        </is>
+      </c>
+      <c r="E1104" s="3" t="inlineStr">
+        <is>
+          <t>국제유가(WTI)가 전 거래일 대비 7.5% 급락하여 배럴당 82.6달러를 기록했다.</t>
+        </is>
+      </c>
+      <c r="F1104" s="3" t="inlineStr">
+        <is>
+          <t>국제유가 급락은 해상, 항공, 육상 운송의 연료비 하락으로 이어져 향후 물류비용에 긍정적인 영향을 미칠 수 있으므로 추이를 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G1104" s="3" t="inlineStr">
+        <is>
+          <t>유가 변동 추이를 지속적으로 모니터링하고, 운송 파트너와의 계약 조건 및 연료 할증료(BAF/FAF) 조정 가능성을 검토해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H1104" s="3" t="inlineStr">
+        <is>
+          <t>이투데이</t>
+        </is>
+      </c>
+      <c r="I1104" s="3" t="inlineStr">
+        <is>
+          <t>https://www.etoday.co.kr/news/view/2608023</t>
+        </is>
+      </c>
+      <c r="J1104" s="3" t="inlineStr"/>
+    </row>
+    <row r="1105">
+      <c r="A1105" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B1105" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C1105" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D1105" s="4" t="inlineStr">
+        <is>
+          <t>CJ대한통운, 대신택배와 이형화물 협력</t>
+        </is>
+      </c>
+      <c r="E1105" s="4" t="inlineStr">
+        <is>
+          <t>CJ대한통운이 대신택배와 협력하여 대형·비규격 상품 배송 서비스를 확대하며 국내 물류 경쟁력을 강화한다.</t>
+        </is>
+      </c>
+      <c r="F1105" s="4" t="inlineStr">
+        <is>
+          <t>국내 택배사의 이형화물 배송 서비스 확대는 배터리/전자부품 제조기업의 주요 국제 운송 및 대량 물류 운영에 직접적인 영향이 미미하다.</t>
+        </is>
+      </c>
+      <c r="G1105" s="4" t="inlineStr"/>
+      <c r="H1105" s="4" t="inlineStr">
+        <is>
+          <t>cargonews</t>
+        </is>
+      </c>
+      <c r="I1105" s="4" t="inlineStr">
+        <is>
+          <t>https://www.cargonews.co.kr/news/articleView.html?idxno=60609</t>
+        </is>
+      </c>
+      <c r="J1105" s="4" t="inlineStr"/>
+    </row>
+    <row r="1106">
+      <c r="A1106" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B1106" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C1106" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D1106" s="4" t="inlineStr">
+        <is>
+          <t>Hapag-Lloyd Uses Shore Power in the Port of Hamburg</t>
+        </is>
+      </c>
+      <c r="E1106" s="4" t="inlineStr">
+        <is>
+          <t>하팍로이드가 함부르크 항만청과 협약을 맺고 함부르크 항에서 육상 전력(Shore Power) 사용을 확대하여 친환경 항만 운영에 기여한다.</t>
+        </is>
+      </c>
+      <c r="F1106" s="4" t="inlineStr">
+        <is>
+          <t>특정 선사의 특정 항만에서의 육상 전력 사용은 배터리/전자부품 제조기업의 글로벌 물류 운영에 직접적인 영향이 미미하다.</t>
+        </is>
+      </c>
+      <c r="G1106" s="4" t="inlineStr"/>
+      <c r="H1106" s="4" t="inlineStr">
+        <is>
+          <t>ksg</t>
+        </is>
+      </c>
+      <c r="I1106" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ksg.co.kr/news/main_newsView.jsp?pNum=147712</t>
+        </is>
+      </c>
+      <c r="J1106" s="4" t="inlineStr"/>
+    </row>
+    <row r="1107">
+      <c r="A1107" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B1107" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C1107" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D1107" s="4" t="inlineStr">
+        <is>
+          <t>Structural Contraction of Global Liner Networks (IMF projection)</t>
+        </is>
+      </c>
+      <c r="E1107" s="4" t="inlineStr">
+        <is>
+          <t>IMF의 2026년 세계 경제 전망에 따르면 글로벌 무역량 성장률이 2025년 5.0%에서 2026년 3.5%로 크게 둔화될 것으로 예상된다.</t>
+        </is>
+      </c>
+      <c r="F1107" s="4" t="inlineStr">
+        <is>
+          <t>글로벌 무역량 성장 둔화는 장기적인 해운 시장의 수요 감소로 이어질 수 있으나, 당사의 단기 물류 운영에 직접적인 영향은 낮다.</t>
+        </is>
+      </c>
+      <c r="G1107" s="4" t="n"/>
+      <c r="H1107" s="4" t="inlineStr">
+        <is>
+          <t>Sea-Intelligence</t>
+        </is>
+      </c>
+      <c r="I1107" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/398-structural-contraction-of-global-liner-network</t>
+        </is>
+      </c>
+      <c r="J1107" s="4" t="inlineStr"/>
+    </row>
+    <row r="1108">
+      <c r="A1108" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B1108" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C1108" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D1108" s="4" t="inlineStr">
+        <is>
+          <t>中, ‘6대 기반시설망’ 구축에 1500조 투자…AI·전력·물류 전국 연결</t>
+        </is>
+      </c>
+      <c r="E1108" s="4" t="inlineStr">
+        <is>
+          <t>중국이 1500조원 규모의 '6대 기반시설망' 프로젝트를 통해 AI, 전력, 물류망 등을 전국적으로 연결할 계획이다. 이는 장기적으로 중국 내 물류 효율성 개선에 기여할 수 있다.</t>
+        </is>
+      </c>
+      <c r="F1108" s="4" t="inlineStr">
+        <is>
+          <t>장기적인 인프라 투자로 당장 우리 물류 운영에 직접적인 영향은 없지만, 중국 내 물류 효율성 개선 추이를 모니터링할 필요가 있다.</t>
+        </is>
+      </c>
+      <c r="G1108" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H1108" s="4" t="inlineStr">
+        <is>
+          <t>헤럴드경제</t>
+        </is>
+      </c>
+      <c r="I1108" s="4" t="inlineStr">
+        <is>
+          <t>https://biz.heraldcorp.com/article/10821138</t>
+        </is>
+      </c>
+      <c r="J1108" s="4" t="inlineStr"/>
+    </row>
+    <row r="1109">
+      <c r="A1109" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B1109" s="4" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C1109" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D1109" s="4" t="inlineStr">
+        <is>
+          <t>중구, 화재 위험 높은 '폐배터리 전용 수거함' 169곳으로 대폭 확대</t>
+        </is>
+      </c>
+      <c r="E1109" s="4" t="inlineStr">
+        <is>
+          <t>서울 중구가 폐배터리로 인한 화재 사고를 예방하고 자원 재활용률을 높이기 위해 폐배터리 전용 수거함을 169곳으로 대폭 확대 운영한다. 이는 폐배터리 안전 관리의 중요성을 보여준다.</t>
+        </is>
+      </c>
+      <c r="F1109" s="4" t="inlineStr">
+        <is>
+          <t>폐배터리 수거 및 안전 관리 강화는 일반 소비자를 대상으로 한 조치로, 우리 회사의 생산/물류 운영에 직접적인 영향은 낮다.</t>
+        </is>
+      </c>
+      <c r="G1109" s="4" t="inlineStr">
+        <is>
+          <t>N/A (장기적으로 폐배터리 회수 및 재활용 정책 변화 추이 모니터링)</t>
+        </is>
+      </c>
+      <c r="H1109" s="4" t="inlineStr">
+        <is>
+          <t>시정일보</t>
+        </is>
+      </c>
+      <c r="I1109" s="4" t="inlineStr">
+        <is>
+          <t>https://sijung.co.kr/news/articleView.html?idxno=433889</t>
+        </is>
+      </c>
+      <c r="J1109" s="4" t="inlineStr"/>
+    </row>
+    <row r="1110">
+      <c r="A1110" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B1110" s="4" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1110" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D1110" s="4" t="inlineStr">
+        <is>
+          <t>복잡한 비특혜 원산지 판정, 더 쉽고 빨라진다</t>
+        </is>
+      </c>
+      <c r="E1110" s="4" t="inlineStr">
+        <is>
+          <t>관세청이 비특혜 원산지 판정 관련 정보를 FTA 포털에서 제공하여 수출입 기업의 원산지 판정 업무를 더 쉽고 빠르게 할 수 있도록 개선한다. 이는 무역 절차의 효율성을 높일 수 있다.</t>
+        </is>
+      </c>
+      <c r="F1110" s="4" t="inlineStr">
+        <is>
+          <t>원산지 판정 절차 간소화는 무역 업무 효율성을 높일 수 있으나, 우리 회사의 물류 운영에 즉각적인 영향은 미미하다.</t>
+        </is>
+      </c>
+      <c r="G1110" s="4" t="inlineStr">
+        <is>
+          <t>N/A (무역팀과 정보 공유 및 활용 방안 검토)</t>
+        </is>
+      </c>
+      <c r="H1110" s="4" t="inlineStr">
+        <is>
+          <t>한국세정신문</t>
+        </is>
+      </c>
+      <c r="I1110" s="4" t="inlineStr">
+        <is>
+          <t>https://taxtimes.co.kr/news/article.html?no=276137</t>
+        </is>
+      </c>
+      <c r="J1110" s="4" t="inlineStr"/>
+    </row>
+    <row r="1111">
+      <c r="A1111" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B1111" s="4" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1111" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D1111" s="4" t="inlineStr">
+        <is>
+          <t>李대통령 "브라질, 공급망 핵심축…韓-메르코수르 무역협정 중요" | 세계일보</t>
+        </is>
+      </c>
+      <c r="E1111" s="4" t="inlineStr">
+        <is>
+          <t>이재명 대통령이 브라질 국빈 방문 중 한국과 메르코수르 간 무역협정의 중요성을 강조하며, 통상 환경 불확실성 시대에 공급망 다변화의 필요성을 언급했다.</t>
+        </is>
+      </c>
+      <c r="F1111" s="4" t="inlineStr">
+        <is>
+          <t>한-메르코수르 무역협정은 장기적인 관점에서 남미 시장 접근성 및 공급망 다변화에 긍정적이나, 당장 우리 물류 운영에 직접적인 영향을 미치지는 않는다.</t>
+        </is>
+      </c>
+      <c r="G1111" s="4" t="n"/>
+      <c r="H1111" s="4" t="inlineStr">
+        <is>
+          <t>세계일보</t>
+        </is>
+      </c>
+      <c r="I1111" s="4" t="inlineStr">
+        <is>
+          <t>https://segye.com/newsView/20260728500647</t>
+        </is>
+      </c>
+      <c r="J1111" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -51330,7 +53114,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -52438,6 +54222,49 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>3062.95</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>-17 (-0.6%)</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>+1,330 (+76.7%)</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="n">
+        <v>4123</v>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>-81 (-1.9%)</t>
+        </is>
+      </c>
+      <c r="I27" s="5" t="inlineStr">
+        <is>
+          <t>+1,729 (+72.2%)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -52450,7 +54277,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I208"/>
+  <dimension ref="A1:I214"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -59756,6 +61583,216 @@
       </c>
       <c r="I208" s="6" t="inlineStr"/>
     </row>
+    <row r="209">
+      <c r="A209" s="6" t="inlineStr">
+        <is>
+          <t>RSK-208</t>
+        </is>
+      </c>
+      <c r="B209" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="C209" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D209" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E209" s="6" t="inlineStr">
+        <is>
+          <t>Section 301 Tariffs on Brazil Take Effect July 22, Stacking with Section 122 Duties; Strait of Hormuz Closure Restricts 200K TEU of Ocean Capacity</t>
+        </is>
+      </c>
+      <c r="F209" s="6" t="inlineStr"/>
+      <c r="G209" s="6" t="inlineStr"/>
+      <c r="H209" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈 해협 경유 노선 및 대체 운송 경로 검토, 중동발 원자재 재고 수준 점검, 브라질 및 러시아 관련 무역 동향 지속 모니터링 및 무역팀과 협의.</t>
+        </is>
+      </c>
+      <c r="I209" s="6" t="inlineStr"/>
+    </row>
+    <row r="210">
+      <c r="A210" s="6" t="inlineStr">
+        <is>
+          <t>RSK-209</t>
+        </is>
+      </c>
+      <c r="B210" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="C210" s="6" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="D210" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E210" s="6" t="inlineStr">
+        <is>
+          <t>미·이란, 공습·보복 이틀째 중단…'호르무즈 협상' 재개 분수령</t>
+        </is>
+      </c>
+      <c r="F210" s="6" t="inlineStr"/>
+      <c r="G210" s="6" t="inlineStr"/>
+      <c r="H210" s="6" t="inlineStr">
+        <is>
+          <t>중동 항로 이용 시 대체 경로 및 운송 수단 검토, 유가 변동에 따른 물류비 상승분 예측 및 대응 계획 수립.</t>
+        </is>
+      </c>
+      <c r="I210" s="6" t="inlineStr"/>
+    </row>
+    <row r="211">
+      <c r="A211" s="6" t="inlineStr">
+        <is>
+          <t>RSK-210</t>
+        </is>
+      </c>
+      <c r="B211" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="C211" s="6" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="D211" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E211" s="6" t="inlineStr">
+        <is>
+          <t>코트라, 중동 수출길 확보 총력 및 요르단서 'K-이니셔티브 판촉전' 개최</t>
+        </is>
+      </c>
+      <c r="F211" s="6" t="inlineStr"/>
+      <c r="G211" s="6" t="inlineStr"/>
+      <c r="H211" s="6" t="inlineStr">
+        <is>
+          <t>중동 지역 수출입 물량에 대한 운송 경로 및 리드타임 재검토, 현지 물류 파트너와 비상 계획 수립.</t>
+        </is>
+      </c>
+      <c r="I211" s="6" t="inlineStr"/>
+    </row>
+    <row r="212">
+      <c r="A212" s="6" t="inlineStr">
+        <is>
+          <t>RSK-211</t>
+        </is>
+      </c>
+      <c r="B212" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="C212" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D212" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E212" s="6" t="inlineStr">
+        <is>
+          <t>뛰는 유가에 물가 불안 우려…금리·관세·환율도 '경고등'</t>
+        </is>
+      </c>
+      <c r="F212" s="6" t="inlineStr"/>
+      <c r="G212" s="6" t="inlineStr"/>
+      <c r="H212" s="6" t="inlineStr">
+        <is>
+          <t>유가, 환율, 주요 관세 변동 추이 면밀히 모니터링, 물류비 및 원가 상승 시나리오별 대응 계획 수립, 헤징 전략 검토.</t>
+        </is>
+      </c>
+      <c r="I212" s="6" t="inlineStr"/>
+    </row>
+    <row r="213">
+      <c r="A213" s="6" t="inlineStr">
+        <is>
+          <t>RSK-212</t>
+        </is>
+      </c>
+      <c r="B213" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="C213" s="6" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="D213" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E213" s="6" t="inlineStr">
+        <is>
+          <t>호르무즈 긴장에도 운임 하락… 해운업계 시선은 홍해로</t>
+        </is>
+      </c>
+      <c r="F213" s="6" t="inlineStr"/>
+      <c r="G213" s="6" t="inlineStr"/>
+      <c r="H213" s="6" t="inlineStr">
+        <is>
+          <t>홍해 지역 지정학적 상황 및 해상 운임 변동 추이 면밀히 모니터링, 필요 시 대체 항로 및 운송 수단 검토.</t>
+        </is>
+      </c>
+      <c r="I213" s="6" t="inlineStr"/>
+    </row>
+    <row r="214">
+      <c r="A214" s="6" t="inlineStr">
+        <is>
+          <t>RSK-213</t>
+        </is>
+      </c>
+      <c r="B214" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="C214" s="6" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="D214" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E214" s="6" t="inlineStr">
+        <is>
+          <t>홍해 길목 지나는 화물선 하루 11척 불과...후티-사우디 충돌에 운항 '뚝'</t>
+        </is>
+      </c>
+      <c r="F214" s="6" t="inlineStr"/>
+      <c r="G214" s="6" t="inlineStr"/>
+      <c r="H214" s="6" t="inlineStr">
+        <is>
+          <t>홍해 항로 이용 시 대체 경로 및 운송 수단 검토, 중동/유럽향 물량의 운송 일정 재조정 및 고객사/협력사와의 소통 강화.</t>
+        </is>
+      </c>
+      <c r="I214" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
📰 뉴스 데이터 2026-07-29_09:02
</commit_message>
<xml_diff>
--- a/data/SCM_물류_브리핑.xlsx
+++ b/data/SCM_물류_브리핑.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1111"/>
+  <dimension ref="A1:J1147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -53102,6 +53102,1758 @@
       </c>
       <c r="J1111" s="4" t="inlineStr"/>
     </row>
+    <row r="1112">
+      <c r="A1112" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B1112" s="2" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C1112" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D1112" s="2" t="inlineStr">
+        <is>
+          <t>CBP Rejects Warehouse Entries on CAPE Declarations, Risking IEEPA Refunds; TPEB Rates Climb as Panama Canal Restrictions Tighten Capacity</t>
+        </is>
+      </c>
+      <c r="E1112" s="2" t="inlineStr">
+        <is>
+          <t>미국 CBP가 CAPE 신고에 대한 창고 입고를 거부하여 IEEPA 환급 위험을 초래하고 있으며, 파나마 운하의 통행 제한 강화로 태평양 횡단 동향 노선(TPEB) 운임이 상승하고 있다.</t>
+        </is>
+      </c>
+      <c r="F1112" s="2" t="inlineStr">
+        <is>
+          <t>파나마 운하 통행 제한 강화는 아시아-미국 동부 해상 운송의 지연 및 운임 상승을 유발하여 우리 회사의 물류 비용과 리드타임에 직접적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G1112" s="2" t="inlineStr">
+        <is>
+          <t>파나마 운하를 이용하는 노선의 운송 계획 및 비용을 재검토하고, 대체 경로(수에즈 운하, 미 서안 육상 운송 등) 또는 운송 수단(항공) 전환 가능성을 평가해야 한다. CBP의 CAPE 신고 관련 지침 변화를 확인하고 통관 절차에 미칠 영향을 분석해야 한다.</t>
+        </is>
+      </c>
+      <c r="H1112" s="2" t="inlineStr">
+        <is>
+          <t>flexport</t>
+        </is>
+      </c>
+      <c r="I1112" s="2" t="inlineStr">
+        <is>
+          <t>https://www.flexport.com/global-logistics-update/july-09-2026-GLU-Newsletter/</t>
+        </is>
+      </c>
+      <c r="J1112" s="2" t="inlineStr">
+        <is>
+          <t>RSK-214</t>
+        </is>
+      </c>
+    </row>
+    <row r="1113">
+      <c r="A1113" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B1113" s="2" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C1113" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D1113" s="2" t="inlineStr">
+        <is>
+          <t>Global Schedule Reliability drops to 62.6% in June 2026</t>
+        </is>
+      </c>
+      <c r="E1113" s="2" t="inlineStr">
+        <is>
+          <t>2026년 6월 전 세계 해상 운송 스케줄 정시성이 62.6%로 하락하여, 해상 운송의 지연 문제가 지속되고 있음을 나타낸다.</t>
+        </is>
+      </c>
+      <c r="F1113" s="2" t="inlineStr">
+        <is>
+          <t>해상 운송 스케줄 정시성 하락은 우리 회사의 해상 운송 리드타임 지연 및 생산 계획 차질로 이어질 수 있어 즉각적인 대응이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G1113" s="2" t="inlineStr">
+        <is>
+          <t>현재 해상 운송 중인 화물의 스케줄을 면밀히 추적하고, 주요 항로 및 선사의 정시성 데이터를 분석하여 잠재적 지연 위험을 평가해야 한다. 필요시 재고 수준 조정, 운송 모드 전환 또는 대체 선사/항로 검토를 고려해야 한다.</t>
+        </is>
+      </c>
+      <c r="H1113" s="2" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I1113" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/400-global-schedule-reliability-drops-to-62-6-in-june-2026</t>
+        </is>
+      </c>
+      <c r="J1113" s="2" t="inlineStr">
+        <is>
+          <t>RSK-215</t>
+        </is>
+      </c>
+    </row>
+    <row r="1114">
+      <c r="A1114" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B1114" s="2" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C1114" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D1114" s="2" t="inlineStr">
+        <is>
+          <t>미·이란, 공습·보복 이틀째 중단…'호르무즈 협상' 재개 분수령</t>
+        </is>
+      </c>
+      <c r="E1114" s="2" t="inlineStr">
+        <is>
+          <t>이란의 호르무즈 해협 사실상 봉쇄로 유조선·화물선 운항 차질이 발생하며 국제유가와 미국 휘발유 가격이 급등했습니다.</t>
+        </is>
+      </c>
+      <c r="F1114" s="2" t="inlineStr">
+        <is>
+          <t>호르무즈 해협은 주요 해상 운송로로, 봉쇄 시 유가 급등 및 해상 운송 차질이 발생하여 물류비 및 운송 계획에 직접적인 영향을 미칩니다.</t>
+        </is>
+      </c>
+      <c r="G1114" s="2" t="inlineStr">
+        <is>
+          <t>중동 정세 및 호르무즈 해협 운항 상황을 실시간으로 모니터링하고, 비상 운송 경로 및 재고 확보 계획을 검토해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H1114" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I1114" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260727-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J1114" s="2" t="inlineStr">
+        <is>
+          <t>RSK-216</t>
+        </is>
+      </c>
+    </row>
+    <row r="1115">
+      <c r="A1115" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B1115" s="2" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C1115" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D1115" s="2" t="inlineStr">
+        <is>
+          <t>코트라, 중동 수출길 확보 총력 및 요르단서 'K-이니셔티브 판촉전' 개최 - 중동 물류 혼란으로 항만 대기와 내륙 운송비 급증</t>
+        </is>
+      </c>
+      <c r="E1115" s="2" t="inlineStr">
+        <is>
+          <t>중동 물류 혼란으로 항만 대기와 내륙 운송비가 급증하며 최종 인도까지 추가로 한 달 이상 지연되는 사례가 늘고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F1115" s="2" t="inlineStr">
+        <is>
+          <t>중동향 물류의 지연 및 비용 증가는 우리 회사의 중동향 수출 계획 및 물류비에 즉각적인 영향을 미칩니다.</t>
+        </is>
+      </c>
+      <c r="G1115" s="2" t="inlineStr">
+        <is>
+          <t>중동향 수출 물량의 운송 경로 및 리드타임을 재검토하고, 대체 운송 수단 및 비용 효율화 방안을 모색해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H1115" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I1115" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260727-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J1115" s="2" t="inlineStr">
+        <is>
+          <t>RSK-217</t>
+        </is>
+      </c>
+    </row>
+    <row r="1116">
+      <c r="A1116" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B1116" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C1116" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D1116" s="2" t="inlineStr">
+        <is>
+          <t>현대글로비스 “유가 부담 600억 3분기 회수…하반기 해운... - 상하이컨테이너운임지수 상승과 유가 부담 회수 전망</t>
+        </is>
+      </c>
+      <c r="E1116" s="2" t="inlineStr">
+        <is>
+          <t>상하이컨테이너운임지수(SCFI) 상승과 유가 부담 회수 전망이 맞물리며 하반기 컨테이너 관련 매출과 물류 처리 실적에 영향이 예상됩니다.</t>
+        </is>
+      </c>
+      <c r="F1116" s="2" t="inlineStr">
+        <is>
+          <t>SCFI 상승 및 유가 부담 회수는 해상 운임 상승으로 이어져 우리 회사의 물류비에 직접적인 영향을 미칩니다.</t>
+        </is>
+      </c>
+      <c r="G1116" s="2" t="inlineStr">
+        <is>
+          <t>하반기 해상 운임 변동 추이를 면밀히 모니터링하고, 운송 계약 조건 재검토 및 비용 절감 방안을 모색해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H1116" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I1116" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260726-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J1116" s="2" t="inlineStr">
+        <is>
+          <t>RSK-218</t>
+        </is>
+      </c>
+    </row>
+    <row r="1117">
+      <c r="A1117" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B1117" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C1117" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D1117" s="2" t="inlineStr">
+        <is>
+          <t>뛰는 유가에 물가 불안 우려…금리·관세·환율도 '경고등'</t>
+        </is>
+      </c>
+      <c r="E1117" s="2" t="inlineStr">
+        <is>
+          <t>유가 급등에 더해 금리·관세·환율 변수까지 겹치며 물가와 대외무역 불확실성이 확대되고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F1117" s="2" t="inlineStr">
+        <is>
+          <t>유가, 관세, 환율 등 복합적인 요인이 물류비 및 대외 무역 불확실성을 높여 즉각적인 대응이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G1117" s="2" t="inlineStr">
+        <is>
+          <t>유가, 환율 변동성 및 주요국 관세 정책 변화를 모니터링하고, 물류비 상승에 대비한 예산 및 계약 조건 검토를 진행해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H1117" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I1117" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260726-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J1117" s="2" t="inlineStr">
+        <is>
+          <t>RSK-219</t>
+        </is>
+      </c>
+    </row>
+    <row r="1118">
+      <c r="A1118" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B1118" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1118" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D1118" s="2" t="inlineStr">
+        <is>
+          <t>미 301조 강제노동 관세 12.5% 매듭…과잉생산 관세는?</t>
+        </is>
+      </c>
+      <c r="E1118" s="2" t="inlineStr">
+        <is>
+          <t>미국의 무역법 301조 조사에서 강제노동 관련 관세가 먼저 확정되어 특정 지역/국가에서 생산된 부품/제품 수입 시 관세 부과 가능성이 커졌습니다.</t>
+        </is>
+      </c>
+      <c r="F1118" s="2" t="inlineStr">
+        <is>
+          <t>미국의 강제노동 관세는 특정 공급처로부터의 부품/제품 수입 비용을 증가시키거나 공급처 변경을 강제할 수 있어 즉각적인 대응이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G1118" s="2" t="inlineStr">
+        <is>
+          <t>강제노동 관련 관세 부과 대상 품목 및 지역을 확인하고, 해당 공급처와의 계약 조건 재검토 및 대체 공급처 발굴을 검토해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H1118" s="2" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I1118" s="2" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260725-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J1118" s="2" t="inlineStr">
+        <is>
+          <t>RSK-220</t>
+        </is>
+      </c>
+    </row>
+    <row r="1119">
+      <c r="A1119" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B1119" s="2" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C1119" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D1119" s="2" t="inlineStr">
+        <is>
+          <t>로테르담항 상반기 컨테이너 702만TEU…환적 20% 급감에 성장 정체</t>
+        </is>
+      </c>
+      <c r="E1119" s="2" t="inlineStr">
+        <is>
+          <t>로테르담항의 상반기 컨테이너 물동량이 환적 급감으로 성장 정체를 보였으며, 항만공사는 터미널 처리능력 부족을 주요 원인으로 지목했습니다.</t>
+        </is>
+      </c>
+      <c r="F1119" s="2" t="inlineStr">
+        <is>
+          <t>유럽향 수출/수입에 중요한 로테르담항의 컨테이너 처리 능력 부족 및 환적 적체는 유럽향 물류의 지연 및 비용 증가를 야기하여 즉각적인 대응이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G1119" s="2" t="inlineStr">
+        <is>
+          <t>유럽향 물량의 로테르담항 경유 여부를 확인하고, 대체 항만 또는 운송 경로를 검토하며, 리드타임 및 재고 계획을 조정해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H1119" s="2" t="inlineStr">
+        <is>
+          <t>해사신문</t>
+        </is>
+      </c>
+      <c r="I1119" s="2" t="inlineStr">
+        <is>
+          <t>https://haesanews.com/news/articleView.html?idxno=149702</t>
+        </is>
+      </c>
+      <c r="J1119" s="2" t="inlineStr">
+        <is>
+          <t>RSK-221</t>
+        </is>
+      </c>
+    </row>
+    <row r="1120">
+      <c r="A1120" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B1120" s="2" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C1120" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D1120" s="2" t="inlineStr">
+        <is>
+          <t>소방당국·경찰, 인천 쿠팡 물류센터 화재 원인 추정 배터리 수거</t>
+        </is>
+      </c>
+      <c r="E1120" s="2" t="inlineStr">
+        <is>
+          <t>인천 쿠팡 물류센터 화재 현장 감식에서 소방 당국과 경찰이 화재 원인으로 추정되는 배터리 등 생활용품들을 수거했다.</t>
+        </is>
+      </c>
+      <c r="F1120" s="2" t="inlineStr">
+        <is>
+          <t>배터리 화재는 물류센터 운영 안전 및 위험물 운송/보관 규제 강화로 이어질 수 있어 우리 제품의 물류 프로세스에 직접적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G1120" s="2" t="inlineStr">
+        <is>
+          <t>물류센터 내 배터리 보관 및 취급 안전 절차 재점검, 위험물 운송 규정 변화 모니터링, 잠재적 규제 강화에 대비.</t>
+        </is>
+      </c>
+      <c r="H1120" s="2" t="inlineStr">
+        <is>
+          <t>아시아경제</t>
+        </is>
+      </c>
+      <c r="I1120" s="2" t="inlineStr">
+        <is>
+          <t>https://asiae.co.kr/article/2026072816171197898</t>
+        </is>
+      </c>
+      <c r="J1120" s="2" t="inlineStr">
+        <is>
+          <t>RSK-222</t>
+        </is>
+      </c>
+    </row>
+    <row r="1121">
+      <c r="A1121" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B1121" s="2" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C1121" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D1121" s="2" t="inlineStr">
+        <is>
+          <t>충남소방, 28일 쿠팡풀필먼트서비스 천안 2·3센터 현장 점검</t>
+        </is>
+      </c>
+      <c r="E1121" s="2" t="inlineStr">
+        <is>
+          <t>충남소방본부가 최근 발생한 쿠팡 물류센터 화재를 계기로 쿠팡풀필먼트서비스 천안 2·3센터를 현장 점검하며 대형 물류센터 화재 예방을 강화했다.</t>
+        </is>
+      </c>
+      <c r="F1121" s="2" t="inlineStr">
+        <is>
+          <t>물류센터 화재 이후 유사 시설에 대한 안전 점검 강화는 우리 회사의 물류센터 운영 및 보관 규제에 직접적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G1121" s="2" t="inlineStr">
+        <is>
+          <t>우리 물류센터 및 협력사 물류센터의 화재 안전 점검 현황 확인, 배터리/위험물 보관 규정 준수 여부 재확인, 소방 점검 강화에 대비.</t>
+        </is>
+      </c>
+      <c r="H1121" s="2" t="inlineStr">
+        <is>
+          <t>일간투데이</t>
+        </is>
+      </c>
+      <c r="I1121" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dtoday.co.kr/news/articleView.html?idxno=783411</t>
+        </is>
+      </c>
+      <c r="J1121" s="2" t="inlineStr">
+        <is>
+          <t>RSK-223</t>
+        </is>
+      </c>
+    </row>
+    <row r="1122">
+      <c r="A1122" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B1122" s="2" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1122" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D1122" s="2" t="inlineStr">
+        <is>
+          <t>"중국산 우회수출 잡는다"…美세관당국, 베트남 내 중국계 공장 불시 점검</t>
+        </is>
+      </c>
+      <c r="E1122" s="2" t="inlineStr">
+        <is>
+          <t>미국 세관당국이 베트남 내 중국 연계 공장들을 불시 점검하여 중국산 우회 수출을 단속하고 있으며, 이는 베트남발 글로벌 공급망에 대한 추가 관세 부과 가능성을 시사한다.</t>
+        </is>
+      </c>
+      <c r="F1122" s="2" t="inlineStr">
+        <is>
+          <t>우리 회사가 베트남에서 부품이나 완제품을 조달하여 미국으로 수출하는 경우, 통관 지연, 추가 관세 부과 또는 공급망 재편 압박 등 직접적인 물류 및 공급망 리스크가 발생할 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G1122" s="2" t="inlineStr">
+        <is>
+          <t>베트남 공급망(특히 중국계 연관 공장) 현황 점검, 미국 수출 제품의 원산지 규정 준수 여부 재확인, 잠재적 관세 부과 시나리오에 대한 대응 계획 수립.</t>
+        </is>
+      </c>
+      <c r="H1122" s="2" t="inlineStr">
+        <is>
+          <t>뉴스핌</t>
+        </is>
+      </c>
+      <c r="I1122" s="2" t="inlineStr">
+        <is>
+          <t>https://www.newspim.com/news/view/20260728000812</t>
+        </is>
+      </c>
+      <c r="J1122" s="2" t="inlineStr">
+        <is>
+          <t>RSK-224</t>
+        </is>
+      </c>
+    </row>
+    <row r="1123">
+      <c r="A1123" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B1123" s="2" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C1123" s="2" t="inlineStr">
+        <is>
+          <t>🔴높음</t>
+        </is>
+      </c>
+      <c r="D1123" s="2" t="inlineStr">
+        <is>
+          <t>[초점] 중동 해상 리스크 다시 고조…정부, 정유·해운업계와 원유 공급망 비상점검 &lt; 초점 &lt; 분석 &lt; 기사본문 - 에너지데일리</t>
+        </is>
+      </c>
+      <c r="E1123" s="2" t="inlineStr">
+        <is>
+          <t>중동 정세 불안으로 홍해 해상 운송 리스크가 다시 고조되자 정부가 정유·해운업계와 함께 원유 공급망 비상 점검에 나섰다.</t>
+        </is>
+      </c>
+      <c r="F1123" s="2" t="inlineStr">
+        <is>
+          <t>중동 해상 운송 리스크는 홍해 항로를 이용하는 선박의 운항 지연 및 운임 상승을 유발할 수 있으며, 이는 우리 회사의 해상 운송 비용 및 리드타임에 직접적인 영향을 미칩니다.</t>
+        </is>
+      </c>
+      <c r="G1123" s="2" t="inlineStr">
+        <is>
+          <t>중동/홍해 항로 이용 현황 점검, 대체 항로 및 운송 방식(항공 등)의 비용/시간 분석, 비상 재고 확보 또는 운송 스케줄 조정 검토.</t>
+        </is>
+      </c>
+      <c r="H1123" s="2" t="inlineStr">
+        <is>
+          <t>에너지데일리</t>
+        </is>
+      </c>
+      <c r="I1123" s="2" t="inlineStr">
+        <is>
+          <t>https://energydaily.co.kr/news/articleView.html?idxno=201791</t>
+        </is>
+      </c>
+      <c r="J1123" s="2" t="inlineStr">
+        <is>
+          <t>RSK-225</t>
+        </is>
+      </c>
+    </row>
+    <row r="1124">
+      <c r="A1124" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B1124" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C1124" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1124" s="3" t="inlineStr">
+        <is>
+          <t>Statement on EU Commission Revision of the EU Emissions Trading System</t>
+        </is>
+      </c>
+      <c r="E1124" s="3" t="inlineStr">
+        <is>
+          <t>IATA는 EU ETS(배출권 거래 시스템)의 유럽 외 지역 확장 제안에 대해 깊은 우려를 표명하며, 이는 항공 운송 비용 증가로 이어질 수 있다고 경고했다.</t>
+        </is>
+      </c>
+      <c r="F1124" s="3" t="inlineStr">
+        <is>
+          <t>EU ETS의 확장은 항공 운송 비용을 증가시켜 유럽향 항공 화물 운임에 영향을 미칠 수 있으므로, 향후 규제 변화와 운임 추이를 지속적으로 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G1124" s="3" t="inlineStr">
+        <is>
+          <t>EU ETS 관련 규제 논의 진행 상황을 주시하고, 유럽향 항공 운송 비용 변화 가능성에 대비하여 운송 예산을 검토해야 한다.</t>
+        </is>
+      </c>
+      <c r="H1124" s="3" t="inlineStr">
+        <is>
+          <t>iata</t>
+        </is>
+      </c>
+      <c r="I1124" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iata.org/en/pressroom/2026-releases/07-17-statement-eu-commission-revision-emissions-trading-system/</t>
+        </is>
+      </c>
+      <c r="J1124" s="3" t="inlineStr"/>
+    </row>
+    <row r="1125">
+      <c r="A1125" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B1125" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1125" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1125" s="3" t="inlineStr">
+        <is>
+          <t>“EU 소액화물 관세 시행 직격탄” … WordlACD, 홍콩발 유럽행 항공화물 24% 급감</t>
+        </is>
+      </c>
+      <c r="E1125" s="3" t="inlineStr">
+        <is>
+          <t>EU의 소액 수입품 과세 강화로 홍콩/중국발 유럽행 항공화물 물동량이 24% 급감했으며, 이는 EU의 관세 정책이 항공 물류 흐름에 직접적인 영향을 미치고 있음을 보여준다.</t>
+        </is>
+      </c>
+      <c r="F1125" s="3" t="inlineStr">
+        <is>
+          <t>EU의 관세 정책 변화가 아시아발 유럽행 항공화물 물동량에 직접적인 영향을 미치고 있어, 우리 회사의 유럽향 소액 화물 운송 전략 및 비용에 잠재적 영향을 줄 수 있다.</t>
+        </is>
+      </c>
+      <c r="G1125" s="3" t="inlineStr">
+        <is>
+          <t>EU의 소액화물 관세 정책이 우리 회사의 유럽향 B2C 또는 소량 B2B 운송에 미치는 영향을 분석하고, 필요시 운송 전략 및 비용 구조를 재검토해야 한다.</t>
+        </is>
+      </c>
+      <c r="H1125" s="3" t="inlineStr">
+        <is>
+          <t>kita</t>
+        </is>
+      </c>
+      <c r="I1125" s="3" t="inlineStr">
+        <is>
+          <t>https://www.kita.net/shippers/board/newsView.do?morgueCode=2&amp;dataCls=C&amp;dataSeq=2862</t>
+        </is>
+      </c>
+      <c r="J1125" s="3" t="inlineStr"/>
+    </row>
+    <row r="1126">
+      <c r="A1126" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B1126" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C1126" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1126" s="3" t="inlineStr">
+        <is>
+          <t>Structural Shift in Blank Sailing Strategies</t>
+        </is>
+      </c>
+      <c r="E1126" s="3" t="inlineStr">
+        <is>
+          <t>2026년 상반기 주요 동서항로에서 선박 결항(Blank Sailing)으로 인한 용선 감소가 전체 용선 증가율보다 훨씬 빠르게 증가하고 있어, 선사들의 용선 전략에 구조적 변화가 있음을 시사한다.</t>
+        </is>
+      </c>
+      <c r="F1126" s="3" t="inlineStr">
+        <is>
+          <t>선사들의 Blank Sailing 전략 변화는 해상 운송 용선 공급에 영향을 미쳐 운임 상승 및 운송 지연을 유발할 수 있으므로, 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G1126" s="3" t="inlineStr">
+        <is>
+          <t>주요 항로의 Blank Sailing 추이를 지속적으로 모니터링하고, 선사와의 협의를 통해 안정적인 용선 확보 방안을 모색해야 한다.</t>
+        </is>
+      </c>
+      <c r="H1126" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I1126" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/399-structural-shift-in-blank-sailing-strategies</t>
+        </is>
+      </c>
+      <c r="J1126" s="3" t="inlineStr"/>
+    </row>
+    <row r="1127">
+      <c r="A1127" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B1127" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C1127" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1127" s="3" t="inlineStr">
+        <is>
+          <t>PLSCI Data Indicates Mega-Hub Retrenchment</t>
+        </is>
+      </c>
+      <c r="E1127" s="3" t="inlineStr">
+        <is>
+          <t>UNCTAD의 PLSCI(Port Liner Shipping Connectivity Index) 데이터 분석 결과, 최근 해운 네트워크 재조정이 메가 허브 항만의 연결성 축소로 이어지고 있음을 보여준다.</t>
+        </is>
+      </c>
+      <c r="F1127" s="3" t="inlineStr">
+        <is>
+          <t>메가 허브 항만의 연결성 축소는 특정 항만을 통한 운송 경로의 효율성 저하 또는 변경을 야기할 수 있으므로, 우리 회사의 주요 항만 이용 전략에 잠재적 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G1127" s="3" t="inlineStr">
+        <is>
+          <t>우리 회사가 주로 이용하는 메가 허브 항만의 연결성 변화를 주시하고, 필요시 대체 항만 또는 운송 경로를 검토해야 한다.</t>
+        </is>
+      </c>
+      <c r="H1127" s="3" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I1127" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/396-plsci-data-indicates-mega-hub-retrenchment</t>
+        </is>
+      </c>
+      <c r="J1127" s="3" t="inlineStr"/>
+    </row>
+    <row r="1128">
+      <c r="A1128" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B1128" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1128" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1128" s="3" t="inlineStr">
+        <is>
+          <t>한국·브라질 핵심광물 협정 체결…메르코수르 FTA 가속</t>
+        </is>
+      </c>
+      <c r="E1128" s="3" t="inlineStr">
+        <is>
+          <t>한국과 브라질이 핵심광물 협정을 체결하고 메르코수르 FTA 협상 가속에 합의하여, 배터리/전자부품의 핵심 원료 공급망 안정화에 긍정적인 영향을 줄 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="F1128" s="3" t="inlineStr">
+        <is>
+          <t>핵심광물 공급망 다변화 및 안정화에 장기적으로 긍정적이나, 즉각적인 물류 운영 영향은 낮아 추이를 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G1128" s="3" t="inlineStr">
+        <is>
+          <t>브라질과의 핵심광물 협정 및 메르코수르 FTA 진행 상황을 지속 모니터링하여 공급망 안정화 기회를 모색해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H1128" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I1128" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260728-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J1128" s="3" t="inlineStr"/>
+    </row>
+    <row r="1129">
+      <c r="A1129" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B1129" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1129" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1129" s="3" t="inlineStr">
+        <is>
+          <t>벤츠, 중국계 지분 리스크에 미국 현지화 승부수</t>
+        </is>
+      </c>
+      <c r="E1129" s="3" t="inlineStr">
+        <is>
+          <t>벤츠가 공급망 탈중국화와 북미 무역협정 재협상 등 지정학적 리스크에 대응하여 미국 현지 생산 확대를 추진하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="F1129" s="3" t="inlineStr">
+        <is>
+          <t>글로벌 기업의 공급망 재편 및 현지화 전략은 우리 회사의 공급망 전략 수립에 참고가 되며, 향후 무역 환경 변화 가능성을 시사합니다.</t>
+        </is>
+      </c>
+      <c r="G1129" s="3" t="inlineStr">
+        <is>
+          <t>주요 기업들의 공급망 재편 및 현지화 전략 동향을 지속 모니터링하여 우리 회사의 공급망 전략에 반영할 부분을 검토해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H1129" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I1129" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260729-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J1129" s="3" t="inlineStr"/>
+    </row>
+    <row r="1130">
+      <c r="A1130" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B1130" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1130" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1130" s="3" t="inlineStr">
+        <is>
+          <t>중, EU의 대러 제재에 보복… 라인메탈 등 유럽 기업 14곳 수출 통제</t>
+        </is>
+      </c>
+      <c r="E1130" s="3" t="inlineStr">
+        <is>
+          <t>중국과 유럽 간 무역 갈등이 격화되며 중국이 EU의 대러 제재에 대한 보복으로 유럽 기업 14곳에 수출 통제를 가했습니다.</t>
+        </is>
+      </c>
+      <c r="F1130" s="3" t="inlineStr">
+        <is>
+          <t>중국-EU 무역 갈등은 글로벌 공급망에 영향을 미칠 수 있으며, 우리 회사의 유럽향/중국향 부품 조달 및 수출에 간접적인 영향 가능성이 있습니다.</t>
+        </is>
+      </c>
+      <c r="G1130" s="3" t="inlineStr">
+        <is>
+          <t>중국-EU 무역 갈등 동향 및 수출 통제 대상 품목/기업 리스트를 지속 모니터링하여 잠재적 공급망 리스크를 평가해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H1130" s="3" t="inlineStr">
+        <is>
+          <t>surff</t>
+        </is>
+      </c>
+      <c r="I1130" s="3" t="inlineStr">
+        <is>
+          <t>https://surff.kr/ko/blog/detail/20260726-경제물류-주요뉴스</t>
+        </is>
+      </c>
+      <c r="J1130" s="3" t="inlineStr"/>
+    </row>
+    <row r="1131">
+      <c r="A1131" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B1131" s="3" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="C1131" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1131" s="3" t="inlineStr">
+        <is>
+          <t>벌크선대 노후화 가속…운임 강세에 스크랩 지연</t>
+        </is>
+      </c>
+      <c r="E1131" s="3" t="inlineStr">
+        <is>
+          <t>드라이벌크선 시장에서 노후선 증가와 운임 강세가 맞물려 노후선의 시장 퇴출이 지연되고 있어, 원자재 운송에 잠재적 지연 위험과 운임 상승 압력이 있습니다.</t>
+        </is>
+      </c>
+      <c r="F1131" s="3" t="inlineStr">
+        <is>
+          <t>벌크선 운임 강세 및 노후선 증가는 주요 원자재 수급 및 운송 비용에 영향을 줄 수 있으므로 추이를 모니터링하여 잠재적 리스크에 대비해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G1131" s="3" t="inlineStr">
+        <is>
+          <t>주요 원자재 운송에 사용되는 벌크선 시장 동향 및 운임 추이를 모니터링하고, 장기적인 원자재 공급망 안정화 방안을 검토해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H1131" s="3" t="inlineStr">
+        <is>
+          <t>해양통신</t>
+        </is>
+      </c>
+      <c r="I1131" s="3" t="inlineStr">
+        <is>
+          <t>https://oceanpress.co.kr/news/article.html?no=30754</t>
+        </is>
+      </c>
+      <c r="J1131" s="3" t="inlineStr"/>
+    </row>
+    <row r="1132">
+      <c r="A1132" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B1132" s="3" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C1132" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1132" s="3" t="inlineStr">
+        <is>
+          <t>[물류 혁신의 그늘] (상) 쿠팡 화재로 드러난 현장 안전 공백</t>
+        </is>
+      </c>
+      <c r="E1132" s="3" t="inlineStr">
+        <is>
+          <t>인천 쿠팡 물류센터 화재 사고는 첨단 물류시설의 현장 안전 공백을 드러냈으며, 이는 위험물로 분류될 수 있는 배터리/전자부품의 보관 및 운송 안전 규제 강화로 이어질 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="F1132" s="3" t="inlineStr">
+        <is>
+          <t>물류센터 화재는 위험물 보관 및 취급 규제 강화로 이어질 수 있으며, 우리 회사의 창고 운영 및 물류 파트너 선정에 영향을 줄 수 있으므로 추이 모니터링이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="G1132" s="3" t="inlineStr">
+        <is>
+          <t>물류센터 안전 규제 동향 및 위험물 보관/취급 기준 변화를 모니터링하고, 물류 파트너의 안전 관리 시스템을 점검하여 잠재적 리스크에 대비해야 합니다.</t>
+        </is>
+      </c>
+      <c r="H1132" s="3" t="inlineStr">
+        <is>
+          <t>인천일보</t>
+        </is>
+      </c>
+      <c r="I1132" s="3" t="inlineStr">
+        <is>
+          <t>https://www.incheonilbo.com/news/articleView.html?idxno=1328331</t>
+        </is>
+      </c>
+      <c r="J1132" s="3" t="inlineStr"/>
+    </row>
+    <row r="1133">
+      <c r="A1133" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B1133" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1133" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1133" s="3" t="inlineStr">
+        <is>
+          <t>나라마다 다른 인증, 고관세·물류비 부담…“중남미 진출, 정부 지원 뒷받침돼야”[라틴 홀린 K뷰티]</t>
+        </is>
+      </c>
+      <c r="E1133" s="3" t="inlineStr">
+        <is>
+          <t>중남미 시장 진출 시 국가별로 다른 인증, 높은 관세 및 물류비 부담이 커 정부 지원이 필요하다는 지적이 나왔다.</t>
+        </is>
+      </c>
+      <c r="F1133" s="3" t="inlineStr">
+        <is>
+          <t>중남미 시장 진출 시 발생할 수 있는 고관세 및 물류비 부담, 국가별 상이한 인증 규제는 우리 제품의 수출 전략 및 비용에 영향을 미칠 수 있으므로 지속적인 모니터링이 필요하다.</t>
+        </is>
+      </c>
+      <c r="G1133" s="3" t="inlineStr">
+        <is>
+          <t>중남미 시장 진출 계획 시 각국의 인증 및 관세, 물류비 관련 규제 사전 조사 및 대응 방안 마련.</t>
+        </is>
+      </c>
+      <c r="H1133" s="3" t="inlineStr">
+        <is>
+          <t>이투데이</t>
+        </is>
+      </c>
+      <c r="I1133" s="3" t="inlineStr">
+        <is>
+          <t>https://etoday.co.kr/news/view/2607340</t>
+        </is>
+      </c>
+      <c r="J1133" s="3" t="inlineStr"/>
+    </row>
+    <row r="1134">
+      <c r="A1134" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B1134" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1134" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1134" s="3" t="inlineStr">
+        <is>
+          <t>"중국에 더 센 관세 부과하라" 美, 멕시코에 무역장벽 압박</t>
+        </is>
+      </c>
+      <c r="E1134" s="3" t="inlineStr">
+        <is>
+          <t>미국이 멕시코에 중국산 제품에 대한 더 강력한 관세 부과를 압박하며, 이는 북중미 무역협정 협상을 빌미로 중국을 겨냥한 관세 전쟁에 동참을 요구하는 것으로 보인다.</t>
+        </is>
+      </c>
+      <c r="F1134" s="3" t="inlineStr">
+        <is>
+          <t>미국과 멕시코 간의 무역 장벽 압박은 글로벌 공급망 재편 및 관세 정책 변화로 이어질 수 있어, 우리 제품의 수출입 전략 및 비용에 간접적인 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G1134" s="3" t="inlineStr">
+        <is>
+          <t>미-중 무역 갈등 및 관련 국가들의 관세 정책 변화 추이 지속 모니터링, 잠재적 공급망 리스크 분석.</t>
+        </is>
+      </c>
+      <c r="H1134" s="3" t="inlineStr">
+        <is>
+          <t>매일경제</t>
+        </is>
+      </c>
+      <c r="I1134" s="3" t="inlineStr">
+        <is>
+          <t>https://mk.co.kr/news/world/12108665</t>
+        </is>
+      </c>
+      <c r="J1134" s="3" t="inlineStr"/>
+    </row>
+    <row r="1135">
+      <c r="A1135" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B1135" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1135" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1135" s="3" t="inlineStr">
+        <is>
+          <t>美관세장벽에 주춤…中 쉬인, 1분기 첫 적자전환</t>
+        </is>
+      </c>
+      <c r="E1135" s="3" t="inlineStr">
+        <is>
+          <t>중국 이커머스 플랫폼 쉬인이 미국 정부의 소액 화물 면세 혜택 폐지 여파로 1분기 첫 적자를 기록하며 미 관세 장벽의 영향을 받았다.</t>
+        </is>
+      </c>
+      <c r="F1135" s="3" t="inlineStr">
+        <is>
+          <t>미국 정부의 소액 화물 면세 혜택 폐지 등 관세 장벽 강화는 우리 회사의 대미 수출 전략 및 비용에 잠재적인 영향을 미칠 수 있으므로 추이를 모니터링해야 한다.</t>
+        </is>
+      </c>
+      <c r="G1135" s="3" t="inlineStr">
+        <is>
+          <t>미국 관세 정책 변화 동향 지속 모니터링, 소액 화물 수출 비중 및 관련 규제 변화에 대한 영향 분석.</t>
+        </is>
+      </c>
+      <c r="H1135" s="3" t="inlineStr">
+        <is>
+          <t>이데일리</t>
+        </is>
+      </c>
+      <c r="I1135" s="3" t="inlineStr">
+        <is>
+          <t>https://edaily.co.kr/News/Read?mediaCodeNo=257&amp;newsId=03972086645518784</t>
+        </is>
+      </c>
+      <c r="J1135" s="3" t="inlineStr"/>
+    </row>
+    <row r="1136">
+      <c r="A1136" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B1136" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1136" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1136" s="3" t="inlineStr">
+        <is>
+          <t>“60개국 추가관세, 미국 물가·금리 영향 없다”는 미 무역대표, 이번엔 ‘2차 관세’ 시사</t>
+        </is>
+      </c>
+      <c r="E1136" s="3" t="inlineStr">
+        <is>
+          <t>미 무역대표부(USTR) 대표가 60개국에 부과한 추가 관세가 미국 물가와 금리에 영향이 없다고 주장하며, 추가적인 '2차 관세' 부과 가능성을 시사했다.</t>
+        </is>
+      </c>
+      <c r="F1136" s="3" t="inlineStr">
+        <is>
+          <t>미국이 60개국에 추가 관세를 부과하고 2차 관세까지 시사하는 것은 글로벌 무역 환경의 불확실성을 높여 우리 회사의 수출입 전략 및 비용에 영향을 미칠 수 있다.</t>
+        </is>
+      </c>
+      <c r="G1136" s="3" t="inlineStr">
+        <is>
+          <t>미국 무역 정책 및 관세 부과 대상 국가 동향 지속 모니터링, 잠재적 관세 부과 리스크에 대한 공급망 및 비용 영향 분석.</t>
+        </is>
+      </c>
+      <c r="H1136" s="3" t="inlineStr">
+        <is>
+          <t>경향신문</t>
+        </is>
+      </c>
+      <c r="I1136" s="3" t="inlineStr">
+        <is>
+          <t>https://khan.co.kr/article/202607280946001</t>
+        </is>
+      </c>
+      <c r="J1136" s="3" t="inlineStr"/>
+    </row>
+    <row r="1137">
+      <c r="A1137" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B1137" s="3" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1137" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1137" s="3" t="inlineStr">
+        <is>
+          <t>日, 한국산 도금강판 덤핑 예비판정…내년 대일 철강 수출 ‘빨간불’ [안팎으로 갇힌 K-제조업]</t>
+        </is>
+      </c>
+      <c r="E1137" s="3" t="inlineStr">
+        <is>
+          <t>일본이 한국산 도금강판에 대한 덤핑 예비판정을 내리며 내년 대일 철강 수출에 관세 부과 가능성이 높아져 가격 경쟁력 및 수익성 압박이 예상된다.</t>
+        </is>
+      </c>
+      <c r="F1137" s="3" t="inlineStr">
+        <is>
+          <t>한국산 철강 제품에 대한 일본의 덤핑 관세 부과 가능성은 우리 회사의 원자재 공급망(철강 부품 사용 시) 및 전반적인 무역 환경에 간접적인 영향을 미칠 수 있어 추이를 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G1137" s="3" t="inlineStr">
+        <is>
+          <t>일본 시장으로의 철강 부품 조달 또는 수출 시 잠재적 영향 분석 및 대체 공급망/수출 전략 검토.</t>
+        </is>
+      </c>
+      <c r="H1137" s="3" t="inlineStr">
+        <is>
+          <t>이투데이</t>
+        </is>
+      </c>
+      <c r="I1137" s="3" t="inlineStr">
+        <is>
+          <t>https://etoday.co.kr/news/view/2608318</t>
+        </is>
+      </c>
+      <c r="J1137" s="3" t="inlineStr"/>
+    </row>
+    <row r="1138">
+      <c r="A1138" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B1138" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C1138" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1138" s="3" t="inlineStr">
+        <is>
+          <t>대한항공, 고유가·고환율 뚫었다…맞춤형 여객·화물 전략으로 수익성 방어</t>
+        </is>
+      </c>
+      <c r="E1138" s="3" t="inlineStr">
+        <is>
+          <t>대한항공이 고유가와 고환율이라는 악조건 속에서도 맞춤형 여객 및 화물 전략으로 매출 방어에 성공했으나, 여전히 높은 연료비 부담이 지속되고 있다.</t>
+        </is>
+      </c>
+      <c r="F1138" s="3" t="inlineStr">
+        <is>
+          <t>항공 운송 비용의 주요 요인인 유가와 환율의 높은 수준이 지속되고 있음을 보여주며, 이는 향후 우리 회사의 항공 운송 비용 상승 압력으로 작용할 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G1138" s="3" t="inlineStr">
+        <is>
+          <t>항공 운송 비용 추이 지속 모니터링, 환율 변동에 따른 비용 헤징 전략 검토.</t>
+        </is>
+      </c>
+      <c r="H1138" s="3" t="inlineStr">
+        <is>
+          <t>더밸류뉴스</t>
+        </is>
+      </c>
+      <c r="I1138" s="3" t="inlineStr">
+        <is>
+          <t>https://thevaluenews.co.kr/news/200313</t>
+        </is>
+      </c>
+      <c r="J1138" s="3" t="inlineStr"/>
+    </row>
+    <row r="1139">
+      <c r="A1139" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B1139" s="3" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C1139" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1139" s="3" t="inlineStr">
+        <is>
+          <t>물류 단기알바 몰렸다…일자리 1년 만에 74.9% 급증 | 한국경제</t>
+        </is>
+      </c>
+      <c r="E1139" s="3" t="inlineStr">
+        <is>
+          <t>물류 단기 아르바이트 일자리가 1년 만에 74.9% 급증했으며, 이는 물류 산업의 인력 수요 증가와 함께 운송·물류 임금 거래액 상승으로 이어지고 있다.</t>
+        </is>
+      </c>
+      <c r="F1139" s="3" t="inlineStr">
+        <is>
+          <t>물류 인력 수요 증가는 창고 운영 및 국내 운송 비용 상승 압력으로 작용할 수 있으며, 이는 우리 회사의 국내 물류 운영 효율성과 비용에 영향을 줄 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="G1139" s="3" t="inlineStr">
+        <is>
+          <t>국내 물류 파트너사의 인력 운영 현황 및 비용 구조 변화 모니터링, 계약 조건 재검토 필요성 확인.</t>
+        </is>
+      </c>
+      <c r="H1139" s="3" t="inlineStr">
+        <is>
+          <t>한국경제</t>
+        </is>
+      </c>
+      <c r="I1139" s="3" t="inlineStr">
+        <is>
+          <t>https://hankyung.com/article/202607279023g</t>
+        </is>
+      </c>
+      <c r="J1139" s="3" t="inlineStr"/>
+    </row>
+    <row r="1140">
+      <c r="A1140" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B1140" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C1140" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1140" s="3" t="inlineStr">
+        <is>
+          <t>이 대통령, 유가 안정 총력전…석유 최고가격제·유류세 인하 유지</t>
+        </is>
+      </c>
+      <c r="E1140" s="3" t="inlineStr">
+        <is>
+          <t>이재명 대통령이 중동 정세 불안에 따른 국제유가 상승 가능성에 대응하여 유가 안정 대책을 지속하고 석유 최고가격제 및 유류세 인하를 유지할 것을 주문했다.</t>
+        </is>
+      </c>
+      <c r="F1140" s="3" t="inlineStr">
+        <is>
+          <t>정부의 유가 안정화 정책은 국내 운송 비용 상승 압력을 완화하는 데 도움이 되지만, 국제 유가 변동성이 크므로 정책의 지속 여부와 효과를 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G1140" s="3" t="inlineStr">
+        <is>
+          <t>국내 운송 파트너사의 유류할증료 및 운송비 변동 추이 모니터링, 정부 정책 변화에 대한 정보 수집.</t>
+        </is>
+      </c>
+      <c r="H1140" s="3" t="inlineStr">
+        <is>
+          <t>경북일보</t>
+        </is>
+      </c>
+      <c r="I1140" s="3" t="inlineStr">
+        <is>
+          <t>https://kyongbuk.co.kr/news/articleView.html?idxno=4079492</t>
+        </is>
+      </c>
+      <c r="J1140" s="3" t="inlineStr"/>
+    </row>
+    <row r="1141">
+      <c r="A1141" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B1141" s="3" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="C1141" s="3" t="inlineStr">
+        <is>
+          <t>🟡모니터링</t>
+        </is>
+      </c>
+      <c r="D1141" s="3" t="inlineStr">
+        <is>
+          <t>美이란 공습 중단에 국제유가 급락…브랜트유 90달러 밑으로 ‘뚝’ - 매일경제</t>
+        </is>
+      </c>
+      <c r="E1141" s="3" t="inlineStr">
+        <is>
+          <t>미국이 이란 공습을 중단하면서 중동 긴장이 완화되어 국제 유가가 급락, 브렌트유가 배럴당 90달러 밑으로 떨어졌다.</t>
+        </is>
+      </c>
+      <c r="F1141" s="3" t="inlineStr">
+        <is>
+          <t>국제 유가 하락은 해상 및 항공 운임의 연료 할증료 인하로 이어질 수 있어 긍정적이나, 중동 정세의 불확실성이 여전하므로 추이를 지속적으로 모니터링해야 합니다.</t>
+        </is>
+      </c>
+      <c r="G1141" s="3" t="inlineStr">
+        <is>
+          <t>해상/항공 운임의 유류할증료 변동 추이 모니터링, 장기적인 유가 안정화 여부 주시.</t>
+        </is>
+      </c>
+      <c r="H1141" s="3" t="inlineStr">
+        <is>
+          <t>매일경제</t>
+        </is>
+      </c>
+      <c r="I1141" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mk.co.kr/news/world/12109047</t>
+        </is>
+      </c>
+      <c r="J1141" s="3" t="inlineStr"/>
+    </row>
+    <row r="1142">
+      <c r="A1142" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B1142" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C1142" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D1142" s="4" t="inlineStr">
+        <is>
+          <t>사우디카고×리야드카고, 인터라인 협정</t>
+        </is>
+      </c>
+      <c r="E1142" s="4" t="inlineStr">
+        <is>
+          <t>사우디항공과 리야드항공이 인터라인 협정을 체결하여 화물 부문 협력을 강화하고, 여객 노선 확대를 통해 벨리 화물 공급을 늘릴 계획이다.</t>
+        </is>
+      </c>
+      <c r="F1142" s="4" t="inlineStr">
+        <is>
+          <t>특정 항공사의 노선 확장 및 협력 강화 소식으로, 우리 회사의 전체 물류 운영에 직접적인 영향은 미미하다.</t>
+        </is>
+      </c>
+      <c r="G1142" s="4" t="n"/>
+      <c r="H1142" s="4" t="inlineStr">
+        <is>
+          <t>cargonews</t>
+        </is>
+      </c>
+      <c r="I1142" s="4" t="inlineStr">
+        <is>
+          <t>https://www.cargonews.co.kr/news/articleView.html?idxno=60617</t>
+        </is>
+      </c>
+      <c r="J1142" s="4" t="inlineStr"/>
+    </row>
+    <row r="1143">
+      <c r="A1143" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B1143" s="4" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1143" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D1143" s="4" t="inlineStr">
+        <is>
+          <t>러 유조선, 북극항로로 몰릴 조짐 보인다</t>
+        </is>
+      </c>
+      <c r="E1143" s="4" t="inlineStr">
+        <is>
+          <t>러시아가 유럽 해역에서의 선박 억류 위험과 중동 긴장 고조를 회피하기 위해 북극항로를 통한 유조선 운항을 확대하고 있으며, 이는 원유 수출 물류망 안정성 확보 전략의 일환이다.</t>
+        </is>
+      </c>
+      <c r="F1143" s="4" t="inlineStr">
+        <is>
+          <t>러시아 유조선의 북극항로 이용 확대는 주로 원유 운송에 해당하며, 우리 회사의 배터리/전자부품 운송에 직접적인 영향은 미미하다.</t>
+        </is>
+      </c>
+      <c r="G1143" s="4" t="n"/>
+      <c r="H1143" s="4" t="inlineStr">
+        <is>
+          <t>oceanpress</t>
+        </is>
+      </c>
+      <c r="I1143" s="4" t="inlineStr">
+        <is>
+          <t>https://www.oceanpress.co.kr/news/article.html?no=30764</t>
+        </is>
+      </c>
+      <c r="J1143" s="4" t="inlineStr"/>
+    </row>
+    <row r="1144">
+      <c r="A1144" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B1144" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C1144" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D1144" s="4" t="inlineStr">
+        <is>
+          <t>Structural Contraction of Global Liner Networks</t>
+        </is>
+      </c>
+      <c r="E1144" s="4" t="inlineStr">
+        <is>
+          <t>IMF의 최신 보고서에 따르면 2025년 5.0%에서 2026년 3.5%로 글로벌 무역량 성장률이 크게 둔화될 것으로 예상되며, 이는 해운 네트워크의 구조적 축소로 이어지고 있다.</t>
+        </is>
+      </c>
+      <c r="F1144" s="4" t="inlineStr">
+        <is>
+          <t>글로벌 무역량 성장 둔화는 장기적인 관점에서 해운 시장에 영향을 미치겠지만, 우리 회사의 단기적인 물류 운영에 직접적인 영향은 미미하다.</t>
+        </is>
+      </c>
+      <c r="G1144" s="4" t="n"/>
+      <c r="H1144" s="4" t="inlineStr">
+        <is>
+          <t>sea</t>
+        </is>
+      </c>
+      <c r="I1144" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sea-intelligence.com/press-room/398-structural-contraction-of-global-liner-network</t>
+        </is>
+      </c>
+      <c r="J1144" s="4" t="inlineStr"/>
+    </row>
+    <row r="1145">
+      <c r="A1145" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B1145" s="4" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="C1145" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D1145" s="4" t="inlineStr">
+        <is>
+          <t>"보조배터리 어디에 버리지?"…중구, 화재 막는 2차전지 전용 수거함 169곳 운영</t>
+        </is>
+      </c>
+      <c r="E1145" s="4" t="inlineStr">
+        <is>
+          <t>중구에서 2차전지 화재를 막기 위해 보조배터리 전용 수거함을 169곳에 운영하기 시작했다.</t>
+        </is>
+      </c>
+      <c r="F1145" s="4" t="inlineStr">
+        <is>
+          <t>주로 소비자 폐기물 관리에 대한 내용으로, 우리 회사의 생산 및 물류 운영에 직접적인 영향은 낮다.</t>
+        </is>
+      </c>
+      <c r="G1145" s="4" t="n"/>
+      <c r="H1145" s="4" t="inlineStr">
+        <is>
+          <t>연합뉴스</t>
+        </is>
+      </c>
+      <c r="I1145" s="4" t="inlineStr">
+        <is>
+          <t>https://yna.co.kr/view/RPR20260727002600353</t>
+        </is>
+      </c>
+      <c r="J1145" s="4" t="inlineStr"/>
+    </row>
+    <row r="1146">
+      <c r="A1146" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B1146" s="4" t="inlineStr">
+        <is>
+          <t>기타_물류</t>
+        </is>
+      </c>
+      <c r="C1146" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D1146" s="4" t="inlineStr">
+        <is>
+          <t>경기신문 - 기본에 충실한 경기·인천 지역 바른 신문</t>
+        </is>
+      </c>
+      <c r="E1146" s="4" t="inlineStr">
+        <is>
+          <t>인천해양경찰서가 대조기로 인한 해수면 상승으로 연안 안전사고 발생 가능성이 커짐에 따라 연안 안전사고 위험예보 '관심' 단계를 발령했다.</t>
+        </is>
+      </c>
+      <c r="F1146" s="4" t="inlineStr">
+        <is>
+          <t>연안 안전사고 위험예보 발령은 일반적인 해상 안전 조치로, 우리 회사의 주요 해상 운송이나 항만 운영에 직접적인 지연이나 영향은 없을 것으로 판단된다.</t>
+        </is>
+      </c>
+      <c r="G1146" s="4" t="n"/>
+      <c r="H1146" s="4" t="inlineStr">
+        <is>
+          <t>경기신문</t>
+        </is>
+      </c>
+      <c r="I1146" s="4" t="inlineStr">
+        <is>
+          <t>https://kgnews.co.kr/news/article.html?no=905571</t>
+        </is>
+      </c>
+      <c r="J1146" s="4" t="inlineStr"/>
+    </row>
+    <row r="1147">
+      <c r="A1147" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B1147" s="4" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="C1147" s="4" t="inlineStr">
+        <is>
+          <t>🟢낮음</t>
+        </is>
+      </c>
+      <c r="D1147" s="4" t="inlineStr">
+        <is>
+          <t>李대통령 "브라질, 공급망 핵심축…韓-메르코수르 무역협정 중요" | 연합뉴스</t>
+        </is>
+      </c>
+      <c r="E1147" s="4" t="inlineStr">
+        <is>
+          <t>이재명 대통령이 브라질을 공급망의 핵심 축으로 강조하며 한-메르코수르 무역협정의 중요성을 언급, 통상 환경 불확실성 시대에 공급망 다변화의 필요성을 시사했다.</t>
+        </is>
+      </c>
+      <c r="F1147" s="4" t="inlineStr">
+        <is>
+          <t>장기적인 공급망 다변화 및 통상 환경 개선에 긍정적이나, 당장 우리 회사의 물류 운영에 직접적인 영향을 미치지는 않습니다.</t>
+        </is>
+      </c>
+      <c r="G1147" s="4" t="n"/>
+      <c r="H1147" s="4" t="inlineStr">
+        <is>
+          <t>연합뉴스</t>
+        </is>
+      </c>
+      <c r="I1147" s="4" t="inlineStr">
+        <is>
+          <t>https://yna.co.kr/view/AKR20260727164600001</t>
+        </is>
+      </c>
+      <c r="J1147" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -53114,7 +54866,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -54265,6 +56017,49 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>3062.95</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>-17 (-0.6%)</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>+1,330 (+76.7%)</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="n">
+        <v>4123</v>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>-81 (-1.9%)</t>
+        </is>
+      </c>
+      <c r="I28" s="5" t="inlineStr">
+        <is>
+          <t>+1,729 (+72.2%)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -54277,7 +56072,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I214"/>
+  <dimension ref="A1:I226"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -61793,6 +63588,426 @@
       </c>
       <c r="I214" s="6" t="inlineStr"/>
     </row>
+    <row r="215">
+      <c r="A215" s="6" t="inlineStr">
+        <is>
+          <t>RSK-214</t>
+        </is>
+      </c>
+      <c r="B215" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="C215" s="6" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="D215" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E215" s="6" t="inlineStr">
+        <is>
+          <t>CBP Rejects Warehouse Entries on CAPE Declarations, Risking IEEPA Refunds; TPEB Rates Climb as Panama Canal Restrictions Tighten Capacity</t>
+        </is>
+      </c>
+      <c r="F215" s="6" t="inlineStr"/>
+      <c r="G215" s="6" t="inlineStr"/>
+      <c r="H215" s="6" t="inlineStr">
+        <is>
+          <t>파나마 운하를 이용하는 노선의 운송 계획 및 비용을 재검토하고, 대체 경로(수에즈 운하, 미 서안 육상 운송 등) 또는 운송 수단(항공) 전환 가능성을 평가해야 한다. CBP의 CAPE 신고 관련 지침 변화를 확인하고 통관 절차에 미칠 영향을 분석해야 한다.</t>
+        </is>
+      </c>
+      <c r="I215" s="6" t="inlineStr"/>
+    </row>
+    <row r="216">
+      <c r="A216" s="6" t="inlineStr">
+        <is>
+          <t>RSK-215</t>
+        </is>
+      </c>
+      <c r="B216" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="C216" s="6" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="D216" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E216" s="6" t="inlineStr">
+        <is>
+          <t>Global Schedule Reliability drops to 62.6% in June 2026</t>
+        </is>
+      </c>
+      <c r="F216" s="6" t="inlineStr"/>
+      <c r="G216" s="6" t="inlineStr"/>
+      <c r="H216" s="6" t="inlineStr">
+        <is>
+          <t>현재 해상 운송 중인 화물의 스케줄을 면밀히 추적하고, 주요 항로 및 선사의 정시성 데이터를 분석하여 잠재적 지연 위험을 평가해야 한다. 필요시 재고 수준 조정, 운송 모드 전환 또는 대체 선사/항로 검토를 고려해야 한다.</t>
+        </is>
+      </c>
+      <c r="I216" s="6" t="inlineStr"/>
+    </row>
+    <row r="217">
+      <c r="A217" s="6" t="inlineStr">
+        <is>
+          <t>RSK-216</t>
+        </is>
+      </c>
+      <c r="B217" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="C217" s="6" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="D217" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E217" s="6" t="inlineStr">
+        <is>
+          <t>미·이란, 공습·보복 이틀째 중단…'호르무즈 협상' 재개 분수령</t>
+        </is>
+      </c>
+      <c r="F217" s="6" t="inlineStr"/>
+      <c r="G217" s="6" t="inlineStr"/>
+      <c r="H217" s="6" t="inlineStr">
+        <is>
+          <t>중동 정세 및 호르무즈 해협 운항 상황을 실시간으로 모니터링하고, 비상 운송 경로 및 재고 확보 계획을 검토해야 합니다.</t>
+        </is>
+      </c>
+      <c r="I217" s="6" t="inlineStr"/>
+    </row>
+    <row r="218">
+      <c r="A218" s="6" t="inlineStr">
+        <is>
+          <t>RSK-217</t>
+        </is>
+      </c>
+      <c r="B218" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="C218" s="6" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="D218" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E218" s="6" t="inlineStr">
+        <is>
+          <t>코트라, 중동 수출길 확보 총력 및 요르단서 'K-이니셔티브 판촉전' 개최 - 중동 물류 혼란으로 항만 대기와 내륙 운송비 급증</t>
+        </is>
+      </c>
+      <c r="F218" s="6" t="inlineStr"/>
+      <c r="G218" s="6" t="inlineStr"/>
+      <c r="H218" s="6" t="inlineStr">
+        <is>
+          <t>중동향 수출 물량의 운송 경로 및 리드타임을 재검토하고, 대체 운송 수단 및 비용 효율화 방안을 모색해야 합니다.</t>
+        </is>
+      </c>
+      <c r="I218" s="6" t="inlineStr"/>
+    </row>
+    <row r="219">
+      <c r="A219" s="6" t="inlineStr">
+        <is>
+          <t>RSK-218</t>
+        </is>
+      </c>
+      <c r="B219" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="C219" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D219" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E219" s="6" t="inlineStr">
+        <is>
+          <t>현대글로비스 “유가 부담 600억 3분기 회수…하반기 해운... - 상하이컨테이너운임지수 상승과 유가 부담 회수 전망</t>
+        </is>
+      </c>
+      <c r="F219" s="6" t="inlineStr"/>
+      <c r="G219" s="6" t="inlineStr"/>
+      <c r="H219" s="6" t="inlineStr">
+        <is>
+          <t>하반기 해상 운임 변동 추이를 면밀히 모니터링하고, 운송 계약 조건 재검토 및 비용 절감 방안을 모색해야 합니다.</t>
+        </is>
+      </c>
+      <c r="I219" s="6" t="inlineStr"/>
+    </row>
+    <row r="220">
+      <c r="A220" s="6" t="inlineStr">
+        <is>
+          <t>RSK-219</t>
+        </is>
+      </c>
+      <c r="B220" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="C220" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D220" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E220" s="6" t="inlineStr">
+        <is>
+          <t>뛰는 유가에 물가 불안 우려…금리·관세·환율도 '경고등'</t>
+        </is>
+      </c>
+      <c r="F220" s="6" t="inlineStr"/>
+      <c r="G220" s="6" t="inlineStr"/>
+      <c r="H220" s="6" t="inlineStr">
+        <is>
+          <t>유가, 환율 변동성 및 주요국 관세 정책 변화를 모니터링하고, 물류비 상승에 대비한 예산 및 계약 조건 검토를 진행해야 합니다.</t>
+        </is>
+      </c>
+      <c r="I220" s="6" t="inlineStr"/>
+    </row>
+    <row r="221">
+      <c r="A221" s="6" t="inlineStr">
+        <is>
+          <t>RSK-220</t>
+        </is>
+      </c>
+      <c r="B221" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="C221" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D221" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E221" s="6" t="inlineStr">
+        <is>
+          <t>미 301조 강제노동 관세 12.5% 매듭…과잉생산 관세는?</t>
+        </is>
+      </c>
+      <c r="F221" s="6" t="inlineStr"/>
+      <c r="G221" s="6" t="inlineStr"/>
+      <c r="H221" s="6" t="inlineStr">
+        <is>
+          <t>강제노동 관련 관세 부과 대상 품목 및 지역을 확인하고, 해당 공급처와의 계약 조건 재검토 및 대체 공급처 발굴을 검토해야 합니다.</t>
+        </is>
+      </c>
+      <c r="I221" s="6" t="inlineStr"/>
+    </row>
+    <row r="222">
+      <c r="A222" s="6" t="inlineStr">
+        <is>
+          <t>RSK-221</t>
+        </is>
+      </c>
+      <c r="B222" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="C222" s="6" t="inlineStr">
+        <is>
+          <t>운송지연_항만적체</t>
+        </is>
+      </c>
+      <c r="D222" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E222" s="6" t="inlineStr">
+        <is>
+          <t>로테르담항 상반기 컨테이너 702만TEU…환적 20% 급감에 성장 정체</t>
+        </is>
+      </c>
+      <c r="F222" s="6" t="inlineStr"/>
+      <c r="G222" s="6" t="inlineStr"/>
+      <c r="H222" s="6" t="inlineStr">
+        <is>
+          <t>유럽향 물량의 로테르담항 경유 여부를 확인하고, 대체 항만 또는 운송 경로를 검토하며, 리드타임 및 재고 계획을 조정해야 합니다.</t>
+        </is>
+      </c>
+      <c r="I222" s="6" t="inlineStr"/>
+    </row>
+    <row r="223">
+      <c r="A223" s="6" t="inlineStr">
+        <is>
+          <t>RSK-222</t>
+        </is>
+      </c>
+      <c r="B223" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="C223" s="6" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="D223" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E223" s="6" t="inlineStr">
+        <is>
+          <t>소방당국·경찰, 인천 쿠팡 물류센터 화재 원인 추정 배터리 수거</t>
+        </is>
+      </c>
+      <c r="F223" s="6" t="inlineStr"/>
+      <c r="G223" s="6" t="inlineStr"/>
+      <c r="H223" s="6" t="inlineStr">
+        <is>
+          <t>물류센터 내 배터리 보관 및 취급 안전 절차 재점검, 위험물 운송 규정 변화 모니터링, 잠재적 규제 강화에 대비.</t>
+        </is>
+      </c>
+      <c r="I223" s="6" t="inlineStr"/>
+    </row>
+    <row r="224">
+      <c r="A224" s="6" t="inlineStr">
+        <is>
+          <t>RSK-223</t>
+        </is>
+      </c>
+      <c r="B224" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="C224" s="6" t="inlineStr">
+        <is>
+          <t>SHE_규제_위험물</t>
+        </is>
+      </c>
+      <c r="D224" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E224" s="6" t="inlineStr">
+        <is>
+          <t>충남소방, 28일 쿠팡풀필먼트서비스 천안 2·3센터 현장 점검</t>
+        </is>
+      </c>
+      <c r="F224" s="6" t="inlineStr"/>
+      <c r="G224" s="6" t="inlineStr"/>
+      <c r="H224" s="6" t="inlineStr">
+        <is>
+          <t>우리 물류센터 및 협력사 물류센터의 화재 안전 점검 현황 확인, 배터리/위험물 보관 규정 준수 여부 재확인, 소방 점검 강화에 대비.</t>
+        </is>
+      </c>
+      <c r="I224" s="6" t="inlineStr"/>
+    </row>
+    <row r="225">
+      <c r="A225" s="6" t="inlineStr">
+        <is>
+          <t>RSK-224</t>
+        </is>
+      </c>
+      <c r="B225" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="C225" s="6" t="inlineStr">
+        <is>
+          <t>지정학_리스크</t>
+        </is>
+      </c>
+      <c r="D225" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E225" s="6" t="inlineStr">
+        <is>
+          <t>"중국산 우회수출 잡는다"…美세관당국, 베트남 내 중국계 공장 불시 점검</t>
+        </is>
+      </c>
+      <c r="F225" s="6" t="inlineStr"/>
+      <c r="G225" s="6" t="inlineStr"/>
+      <c r="H225" s="6" t="inlineStr">
+        <is>
+          <t>베트남 공급망(특히 중국계 연관 공장) 현황 점검, 미국 수출 제품의 원산지 규정 준수 여부 재확인, 잠재적 관세 부과 시나리오에 대한 대응 계획 수립.</t>
+        </is>
+      </c>
+      <c r="I225" s="6" t="inlineStr"/>
+    </row>
+    <row r="226">
+      <c r="A226" s="6" t="inlineStr">
+        <is>
+          <t>RSK-225</t>
+        </is>
+      </c>
+      <c r="B226" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="C226" s="6" t="inlineStr">
+        <is>
+          <t>운임_유가</t>
+        </is>
+      </c>
+      <c r="D226" s="6" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="E226" s="6" t="inlineStr">
+        <is>
+          <t>[초점] 중동 해상 리스크 다시 고조…정부, 정유·해운업계와 원유 공급망 비상점검 &lt; 초점 &lt; 분석 &lt; 기사본문 - 에너지데일리</t>
+        </is>
+      </c>
+      <c r="F226" s="6" t="inlineStr"/>
+      <c r="G226" s="6" t="inlineStr"/>
+      <c r="H226" s="6" t="inlineStr">
+        <is>
+          <t>중동/홍해 항로 이용 현황 점검, 대체 항로 및 운송 방식(항공 등)의 비용/시간 분석, 비상 재고 확보 또는 운송 스케줄 조정 검토.</t>
+        </is>
+      </c>
+      <c r="I226" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>